<commit_message>
Actualización automatizada: historico_mallas.xlsx [2026-04-24 17:53]
</commit_message>
<xml_diff>
--- a/historico_mallas.xlsx
+++ b/historico_mallas.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
   <si>
     <t>Mes</t>
   </si>
@@ -34,13 +34,22 @@
     <t>Abril</t>
   </si>
   <si>
+    <t>Mayo</t>
+  </si>
+  <si>
     <t>Técnica</t>
   </si>
   <si>
     <t>24/04/2026 17:52</t>
   </si>
   <si>
+    <t>24/04/2026 17:53</t>
+  </si>
+  <si>
     <t>{"Grupo":{"0":"GRUPO 1","1":"GRUPO 1","2":"GRUPO 1","3":"GRUPO 1","4":"GRUPO 1","5":"GRUPO 1","6":"GRUPO 1","7":"GRUPO 1","8":"GRUPO 1","9":"GRUPO 1","10":"GRUPO 1","11":"GRUPO 1","12":"GRUPO 2","13":"GRUPO 2","14":"GRUPO 2","15":"GRUPO 2","16":"GRUPO 2","17":"GRUPO 2","18":"GRUPO 2","19":"GRUPO 2","20":"GRUPO 2","21":"GRUPO 2","22":"GRUPO 2","23":"GRUPO 2","24":"GRUPO 3","25":"GRUPO 3","26":"GRUPO 3","27":"GRUPO 3","28":"GRUPO 3","29":"GRUPO 3","30":"GRUPO 3","31":"GRUPO 3","32":"GRUPO 3","33":"GRUPO 3","34":"GRUPO 3","35":"GRUPO 3","36":"GRUPO 4","37":"GRUPO 4","38":"GRUPO 4","39":"GRUPO 4","40":"GRUPO 4","41":"GRUPO 4","42":"GRUPO 4","43":"GRUPO 4","44":"GRUPO 4","45":"GRUPO 4","46":"GRUPO 4","47":"GRUPO 4","48":"GRUPO 1","49":"GRUPO 1","50":"GRUPO 1","51":"GRUPO 1","52":"GRUPO 1","53":"GRUPO 1","54":"GRUPO 1","55":"GRUPO 1","56":"GRUPO 1","57":"GRUPO 1","58":"GRUPO 1","59":"GRUPO 1","60":"GRUPO 2","61":"GRUPO 2","62":"GRUPO 2","63":"GRUPO 2","64":"GRUPO 2","65":"GRUPO 2","66":"GRUPO 2","67":"GRUPO 2","68":"GRUPO 2","69":"GRUPO 2","70":"GRUPO 2","71":"GRUPO 2","72":"GRUPO 3","73":"GRUPO 3","74":"GRUPO 3","75":"GRUPO 3","76":"GRUPO 3","77":"GRUPO 3","78":"GRUPO 3","79":"GRUPO 3","80":"GRUPO 3","81":"GRUPO 3","82":"GRUPO 3","83":"GRUPO 3","84":"GRUPO 4","85":"GRUPO 4","86":"GRUPO 4","87":"GRUPO 4","88":"GRUPO 4","89":"GRUPO 4","90":"GRUPO 4","91":"GRUPO 4","92":"GRUPO 4","93":"GRUPO 4","94":"GRUPO 4","95":"GRUPO 4","96":"GRUPO 1","97":"GRUPO 1","98":"GRUPO 1","99":"GRUPO 1","100":"GRUPO 1","101":"GRUPO 1","102":"GRUPO 1","103":"GRUPO 1","104":"GRUPO 1","105":"GRUPO 1","106":"GRUPO 1","107":"GRUPO 1","108":"GRUPO 2","109":"GRUPO 2","110":"GRUPO 2","111":"GRUPO 2","112":"GRUPO 2","113":"GRUPO 2","114":"GRUPO 2","115":"GRUPO 2","116":"GRUPO 2","117":"GRUPO 2","118":"GRUPO 2","119":"GRUPO 2","120":"GRUPO 3","121":"GRUPO 3","122":"GRUPO 3","123":"GRUPO 3","124":"GRUPO 3","125":"GRUPO 3","126":"GRUPO 3","127":"GRUPO 3","128":"GRUPO 3","129":"GRUPO 3","130":"GRUPO 3","131":"GRUPO 3","132":"GRUPO 4","133":"GRUPO 4","134":"GRUPO 4","135":"GRUPO 4","136":"GRUPO 4","137":"GRUPO 4","138":"GRUPO 4","139":"GRUPO 4","140":"GRUPO 4","141":"GRUPO 4","142":"GRUPO 4","143":"GRUPO 4","144":"GRUPO 1","145":"GRUPO 1","146":"GRUPO 1","147":"GRUPO 1","148":"GRUPO 1","149":"GRUPO 1","150":"GRUPO 1","151":"GRUPO 1","152":"GRUPO 1","153":"GRUPO 1","154":"GRUPO 1","155":"GRUPO 1","156":"GRUPO 2","157":"GRUPO 2","158":"GRUPO 2","159":"GRUPO 2","160":"GRUPO 2","161":"GRUPO 2","162":"GRUPO 2","163":"GRUPO 2","164":"GRUPO 2","165":"GRUPO 2","166":"GRUPO 2","167":"GRUPO 2","168":"GRUPO 3","169":"GRUPO 3","170":"GRUPO 3","171":"GRUPO 3","172":"GRUPO 3","173":"GRUPO 3","174":"GRUPO 3","175":"GRUPO 3","176":"GRUPO 3","177":"GRUPO 3","178":"GRUPO 3","179":"GRUPO 3","180":"GRUPO 4","181":"GRUPO 4","182":"GRUPO 4","183":"GRUPO 4","184":"GRUPO 4","185":"GRUPO 4","186":"GRUPO 4","187":"GRUPO 4","188":"GRUPO 4","189":"GRUPO 4","190":"GRUPO 4","191":"GRUPO 4","192":"GRUPO 1","193":"GRUPO 1","194":"GRUPO 1","195":"GRUPO 1","196":"GRUPO 1","197":"GRUPO 1","198":"GRUPO 1","199":"GRUPO 1","200":"GRUPO 1","201":"GRUPO 1","202":"GRUPO 1","203":"GRUPO 1","204":"GRUPO 2","205":"GRUPO 2","206":"GRUPO 2","207":"GRUPO 2","208":"GRUPO 2","209":"GRUPO 2","210":"GRUPO 2","211":"GRUPO 2","212":"GRUPO 2","213":"GRUPO 2","214":"GRUPO 2","215":"GRUPO 2","216":"GRUPO 3","217":"GRUPO 3","218":"GRUPO 3","219":"GRUPO 3","220":"GRUPO 3","221":"GRUPO 3","222":"GRUPO 3","223":"GRUPO 3","224":"GRUPO 3","225":"GRUPO 3","226":"GRUPO 3","227":"GRUPO 3","228":"GRUPO 4","229":"GRUPO 4","230":"GRUPO 4","231":"GRUPO 4","232":"GRUPO 4","233":"GRUPO 4","234":"GRUPO 4","235":"GRUPO 4","236":"GRUPO 4","237":"GRUPO 4","238":"GRUPO 4","239":"GRUPO 4","240":"GRUPO 1","241":"GRUPO 1","242":"GRUPO 1","243":"GRUPO 1","244":"GRUPO 1","245":"GRUPO 1","246":"GRUPO 1","247":"GRUPO 1","248":"GRUPO 1","249":"GRUPO 1","250":"GRUPO 1","251":"GRUPO 1","252":"GRUPO 2","253":"GRUPO 2","254":"GRUPO 2","255":"GRUPO 2","256":"GRUPO 2","257":"GRUPO 2","258":"GRUPO 2","259":"GRUPO 2","260":"GRUPO 2","261":"GRUPO 2","262":"GRUPO 2","263":"GRUPO 2","264":"GRUPO 3","265":"GRUPO 3","266":"GRUPO 3","267":"GRUPO 3","268":"GRUPO 3","269":"GRUPO 3","270":"GRUPO 3","271":"GRUPO 3","272":"GRUPO 3","273":"GRUPO 3","274":"GRUPO 3","275":"GRUPO 3","276":"GRUPO 4","277":"GRUPO 4","278":"GRUPO 4","279":"GRUPO 4","280":"GRUPO 4","281":"GRUPO 4","282":"GRUPO 4","283":"GRUPO 4","284":"GRUPO 4","285":"GRUPO 4","286":"GRUPO 4","287":"GRUPO 4","288":"GRUPO 1","289":"GRUPO 1","290":"GRUPO 1","291":"GRUPO 1","292":"GRUPO 1","293":"GRUPO 1","294":"GRUPO 1","295":"GRUPO 1","296":"GRUPO 1","297":"GRUPO 1","298":"GRUPO 1","299":"GRUPO 1","300":"GRUPO 2","301":"GRUPO 2","302":"GRUPO 2","303":"GRUPO 2","304":"GRUPO 2","305":"GRUPO 2","306":"GRUPO 2","307":"GRUPO 2","308":"GRUPO 2","309":"GRUPO 2","310":"GRUPO 2","311":"GRUPO 2","312":"GRUPO 3","313":"GRUPO 3","314":"GRUPO 3","315":"GRUPO 3","316":"GRUPO 3","317":"GRUPO 3","318":"GRUPO 3","319":"GRUPO 3","320":"GRUPO 3","321":"GRUPO 3","322":"GRUPO 3","323":"GRUPO 3","324":"GRUPO 4","325":"GRUPO 4","326":"GRUPO 4","327":"GRUPO 4","328":"GRUPO 4","329":"GRUPO 4","330":"GRUPO 4","331":"GRUPO 4","332":"GRUPO 4","333":"GRUPO 4","334":"GRUPO 4","335":"GRUPO 4","336":"GRUPO 1","337":"GRUPO 1","338":"GRUPO 1","339":"GRUPO 1","340":"GRUPO 1","341":"GRUPO 1","342":"GRUPO 1","343":"GRUPO 1","344":"GRUPO 1","345":"GRUPO 1","346":"GRUPO 1","347":"GRUPO 1","348":"GRUPO 2","349":"GRUPO 2","350":"GRUPO 2","351":"GRUPO 2","352":"GRUPO 2","353":"GRUPO 2","354":"GRUPO 2","355":"GRUPO 2","356":"GRUPO 2","357":"GRUPO 2","358":"GRUPO 2","359":"GRUPO 2","360":"GRUPO 3","361":"GRUPO 3","362":"GRUPO 3","363":"GRUPO 3","364":"GRUPO 3","365":"GRUPO 3","366":"GRUPO 3","367":"GRUPO 3","368":"GRUPO 3","369":"GRUPO 3","370":"GRUPO 3","371":"GRUPO 3","372":"GRUPO 4","373":"GRUPO 4","374":"GRUPO 4","375":"GRUPO 4","376":"GRUPO 4","377":"GRUPO 4","378":"GRUPO 4","379":"GRUPO 4","380":"GRUPO 4","381":"GRUPO 4","382":"GRUPO 4","383":"GRUPO 4","384":"GRUPO 1","385":"GRUPO 1","386":"GRUPO 1","387":"GRUPO 1","388":"GRUPO 1","389":"GRUPO 1","390":"GRUPO 1","391":"GRUPO 1","392":"GRUPO 1","393":"GRUPO 1","394":"GRUPO 1","395":"GRUPO 1","396":"GRUPO 2","397":"GRUPO 2","398":"GRUPO 2","399":"GRUPO 2","400":"GRUPO 2","401":"GRUPO 2","402":"GRUPO 2","403":"GRUPO 2","404":"GRUPO 2","405":"GRUPO 2","406":"GRUPO 2","407":"GRUPO 2","408":"GRUPO 3","409":"GRUPO 3","410":"GRUPO 3","411":"GRUPO 3","412":"GRUPO 3","413":"GRUPO 3","414":"GRUPO 3","415":"GRUPO 3","416":"GRUPO 3","417":"GRUPO 3","418":"GRUPO 3","419":"GRUPO 3","420":"GRUPO 4","421":"GRUPO 4","422":"GRUPO 4","423":"GRUPO 4","424":"GRUPO 4","425":"GRUPO 4","426":"GRUPO 4","427":"GRUPO 4","428":"GRUPO 4","429":"GRUPO 4","430":"GRUPO 4","431":"GRUPO 4","432":"GRUPO 1","433":"GRUPO 1","434":"GRUPO 1","435":"GRUPO 1","436":"GRUPO 1","437":"GRUPO 1","438":"GRUPO 1","439":"GRUPO 1","440":"GRUPO 1","441":"GRUPO 1","442":"GRUPO 1","443":"GRUPO 1","444":"GRUPO 2","445":"GRUPO 2","446":"GRUPO 2","447":"GRUPO 2","448":"GRUPO 2","449":"GRUPO 2","450":"GRUPO 2","451":"GRUPO 2","452":"GRUPO 2","453":"GRUPO 2","454":"GRUPO 2","455":"GRUPO 2","456":"GRUPO 3","457":"GRUPO 3","458":"GRUPO 3","459":"GRUPO 3","460":"GRUPO 3","461":"GRUPO 3","462":"GRUPO 3","463":"GRUPO 3","464":"GRUPO 3","465":"GRUPO 3","466":"GRUPO 3","467":"GRUPO 3","468":"GRUPO 4","469":"GRUPO 4","470":"GRUPO 4","471":"GRUPO 4","472":"GRUPO 4","473":"GRUPO 4","474":"GRUPO 4","475":"GRUPO 4","476":"GRUPO 4","477":"GRUPO 4","478":"GRUPO 4","479":"GRUPO 4","480":"GRUPO 1","481":"GRUPO 1","482":"GRUPO 1","483":"GRUPO 1","484":"GRUPO 1","485":"GRUPO 1","486":"GRUPO 1","487":"GRUPO 1","488":"GRUPO 1","489":"GRUPO 1","490":"GRUPO 1","491":"GRUPO 1","492":"GRUPO 2","493":"GRUPO 2","494":"GRUPO 2","495":"GRUPO 2","496":"GRUPO 2","497":"GRUPO 2","498":"GRUPO 2","499":"GRUPO 2","500":"GRUPO 2","501":"GRUPO 2","502":"GRUPO 2","503":"GRUPO 2","504":"GRUPO 3","505":"GRUPO 3","506":"GRUPO 3","507":"GRUPO 3","508":"GRUPO 3","509":"GRUPO 3","510":"GRUPO 3","511":"GRUPO 3","512":"GRUPO 3","513":"GRUPO 3","514":"GRUPO 3","515":"GRUPO 3","516":"GRUPO 4","517":"GRUPO 4","518":"GRUPO 4","519":"GRUPO 4","520":"GRUPO 4","521":"GRUPO 4","522":"GRUPO 4","523":"GRUPO 4","524":"GRUPO 4","525":"GRUPO 4","526":"GRUPO 4","527":"GRUPO 4","528":"GRUPO 1","529":"GRUPO 1","530":"GRUPO 1","531":"GRUPO 1","532":"GRUPO 1","533":"GRUPO 1","534":"GRUPO 1","535":"GRUPO 1","536":"GRUPO 1","537":"GRUPO 1","538":"GRUPO 1","539":"GRUPO 1","540":"GRUPO 2","541":"GRUPO 2","542":"GRUPO 2","543":"GRUPO 2","544":"GRUPO 2","545":"GRUPO 2","546":"GRUPO 2","547":"GRUPO 2","548":"GRUPO 2","549":"GRUPO 2","550":"GRUPO 2","551":"GRUPO 2","552":"GRUPO 3","553":"GRUPO 3","554":"GRUPO 3","555":"GRUPO 3","556":"GRUPO 3","557":"GRUPO 3","558":"GRUPO 3","559":"GRUPO 3","560":"GRUPO 3","561":"GRUPO 3","562":"GRUPO 3","563":"GRUPO 3","564":"GRUPO 4","565":"GRUPO 4","566":"GRUPO 4","567":"GRUPO 4","568":"GRUPO 4","569":"GRUPO 4","570":"GRUPO 4","571":"GRUPO 4","572":"GRUPO 4","573":"GRUPO 4","574":"GRUPO 4","575":"GRUPO 4","576":"GRUPO 1","577":"GRUPO 1","578":"GRUPO 1","579":"GRUPO 1","580":"GRUPO 1","581":"GRUPO 1","582":"GRUPO 1","583":"GRUPO 1","584":"GRUPO 1","585":"GRUPO 1","586":"GRUPO 1","587":"GRUPO 1","588":"GRUPO 2","589":"GRUPO 2","590":"GRUPO 2","591":"GRUPO 2","592":"GRUPO 2","593":"GRUPO 2","594":"GRUPO 2","595":"GRUPO 2","596":"GRUPO 2","597":"GRUPO 2","598":"GRUPO 2","599":"GRUPO 2","600":"GRUPO 3","601":"GRUPO 3","602":"GRUPO 3","603":"GRUPO 3","604":"GRUPO 3","605":"GRUPO 3","606":"GRUPO 3","607":"GRUPO 3","608":"GRUPO 3","609":"GRUPO 3","610":"GRUPO 3","611":"GRUPO 3","612":"GRUPO 4","613":"GRUPO 4","614":"GRUPO 4","615":"GRUPO 4","616":"GRUPO 4","617":"GRUPO 4","618":"GRUPO 4","619":"GRUPO 4","620":"GRUPO 4","621":"GRUPO 4","622":"GRUPO 4","623":"GRUPO 4","624":"GRUPO 1","625":"GRUPO 1","626":"GRUPO 1","627":"GRUPO 1","628":"GRUPO 1","629":"GRUPO 1","630":"GRUPO 1","631":"GRUPO 1","632":"GRUPO 1","633":"GRUPO 1","634":"GRUPO 1","635":"GRUPO 1","636":"GRUPO 2","637":"GRUPO 2","638":"GRUPO 2","639":"GRUPO 2","640":"GRUPO 2","641":"GRUPO 2","642":"GRUPO 2","643":"GRUPO 2","644":"GRUPO 2","645":"GRUPO 2","646":"GRUPO 2","647":"GRUPO 2","648":"GRUPO 3","649":"GRUPO 3","650":"GRUPO 3","651":"GRUPO 3","652":"GRUPO 3","653":"GRUPO 3","654":"GRUPO 3","655":"GRUPO 3","656":"GRUPO 3","657":"GRUPO 3","658":"GRUPO 3","659":"GRUPO 3","660":"GRUPO 4","661":"GRUPO 4","662":"GRUPO 4","663":"GRUPO 4","664":"GRUPO 4","665":"GRUPO 4","666":"GRUPO 4","667":"GRUPO 4","668":"GRUPO 4","669":"GRUPO 4","670":"GRUPO 4","671":"GRUPO 4","672":"GRUPO 1","673":"GRUPO 1","674":"GRUPO 1","675":"GRUPO 1","676":"GRUPO 1","677":"GRUPO 1","678":"GRUPO 1","679":"GRUPO 1","680":"GRUPO 1","681":"GRUPO 1","682":"GRUPO 1","683":"GRUPO 1","684":"GRUPO 2","685":"GRUPO 2","686":"GRUPO 2","687":"GRUPO 2","688":"GRUPO 2","689":"GRUPO 2","690":"GRUPO 2","691":"GRUPO 2","692":"GRUPO 2","693":"GRUPO 2","694":"GRUPO 2","695":"GRUPO 2","696":"GRUPO 3","697":"GRUPO 3","698":"GRUPO 3","699":"GRUPO 3","700":"GRUPO 3","701":"GRUPO 3","702":"GRUPO 3","703":"GRUPO 3","704":"GRUPO 3","705":"GRUPO 3","706":"GRUPO 3","707":"GRUPO 3","708":"GRUPO 4","709":"GRUPO 4","710":"GRUPO 4","711":"GRUPO 4","712":"GRUPO 4","713":"GRUPO 4","714":"GRUPO 4","715":"GRUPO 4","716":"GRUPO 4","717":"GRUPO 4","718":"GRUPO 4","719":"GRUPO 4","720":"GRUPO 1","721":"GRUPO 1","722":"GRUPO 1","723":"GRUPO 1","724":"GRUPO 1","725":"GRUPO 1","726":"GRUPO 1","727":"GRUPO 1","728":"GRUPO 1","729":"GRUPO 1","730":"GRUPO 1","731":"GRUPO 1","732":"GRUPO 2","733":"GRUPO 2","734":"GRUPO 2","735":"GRUPO 2","736":"GRUPO 2","737":"GRUPO 2","738":"GRUPO 2","739":"GRUPO 2","740":"GRUPO 2","741":"GRUPO 2","742":"GRUPO 2","743":"GRUPO 2","744":"GRUPO 3","745":"GRUPO 3","746":"GRUPO 3","747":"GRUPO 3","748":"GRUPO 3","749":"GRUPO 3","750":"GRUPO 3","751":"GRUPO 3","752":"GRUPO 3","753":"GRUPO 3","754":"GRUPO 3","755":"GRUPO 3","756":"GRUPO 4","757":"GRUPO 4","758":"GRUPO 4","759":"GRUPO 4","760":"GRUPO 4","761":"GRUPO 4","762":"GRUPO 4","763":"GRUPO 4","764":"GRUPO 4","765":"GRUPO 4","766":"GRUPO 4","767":"GRUPO 4","768":"GRUPO 1","769":"GRUPO 1","770":"GRUPO 1","771":"GRUPO 1","772":"GRUPO 1","773":"GRUPO 1","774":"GRUPO 1","775":"GRUPO 1","776":"GRUPO 1","777":"GRUPO 1","778":"GRUPO 1","779":"GRUPO 1","780":"GRUPO 2","781":"GRUPO 2","782":"GRUPO 2","783":"GRUPO 2","784":"GRUPO 2","785":"GRUPO 2","786":"GRUPO 2","787":"GRUPO 2","788":"GRUPO 2","789":"GRUPO 2","790":"GRUPO 2","791":"GRUPO 2","792":"GRUPO 3","793":"GRUPO 3","794":"GRUPO 3","795":"GRUPO 3","796":"GRUPO 3","797":"GRUPO 3","798":"GRUPO 3","799":"GRUPO 3","800":"GRUPO 3","801":"GRUPO 3","802":"GRUPO 3","803":"GRUPO 3","804":"GRUPO 4","805":"GRUPO 4","806":"GRUPO 4","807":"GRUPO 4","808":"GRUPO 4","809":"GRUPO 4","810":"GRUPO 4","811":"GRUPO 4","812":"GRUPO 4","813":"GRUPO 4","814":"GRUPO 4","815":"GRUPO 4","816":"GRUPO 1","817":"GRUPO 1","818":"GRUPO 1","819":"GRUPO 1","820":"GRUPO 1","821":"GRUPO 1","822":"GRUPO 1","823":"GRUPO 1","824":"GRUPO 1","825":"GRUPO 1","826":"GRUPO 1","827":"GRUPO 1","828":"GRUPO 2","829":"GRUPO 2","830":"GRUPO 2","831":"GRUPO 2","832":"GRUPO 2","833":"GRUPO 2","834":"GRUPO 2","835":"GRUPO 2","836":"GRUPO 2","837":"GRUPO 2","838":"GRUPO 2","839":"GRUPO 2","840":"GRUPO 3","841":"GRUPO 3","842":"GRUPO 3","843":"GRUPO 3","844":"GRUPO 3","845":"GRUPO 3","846":"GRUPO 3","847":"GRUPO 3","848":"GRUPO 3","849":"GRUPO 3","850":"GRUPO 3","851":"GRUPO 3","852":"GRUPO 4","853":"GRUPO 4","854":"GRUPO 4","855":"GRUPO 4","856":"GRUPO 4","857":"GRUPO 4","858":"GRUPO 4","859":"GRUPO 4","860":"GRUPO 4","861":"GRUPO 4","862":"GRUPO 4","863":"GRUPO 4","864":"GRUPO 1","865":"GRUPO 1","866":"GRUPO 1","867":"GRUPO 1","868":"GRUPO 1","869":"GRUPO 1","870":"GRUPO 1","871":"GRUPO 1","872":"GRUPO 1","873":"GRUPO 1","874":"GRUPO 1","875":"GRUPO 1","876":"GRUPO 2","877":"GRUPO 2","878":"GRUPO 2","879":"GRUPO 2","880":"GRUPO 2","881":"GRUPO 2","882":"GRUPO 2","883":"GRUPO 2","884":"GRUPO 2","885":"GRUPO 2","886":"GRUPO 2","887":"GRUPO 2","888":"GRUPO 3","889":"GRUPO 3","890":"GRUPO 3","891":"GRUPO 3","892":"GRUPO 3","893":"GRUPO 3","894":"GRUPO 3","895":"GRUPO 3","896":"GRUPO 3","897":"GRUPO 3","898":"GRUPO 3","899":"GRUPO 3","900":"GRUPO 4","901":"GRUPO 4","902":"GRUPO 4","903":"GRUPO 4","904":"GRUPO 4","905":"GRUPO 4","906":"GRUPO 4","907":"GRUPO 4","908":"GRUPO 4","909":"GRUPO 4","910":"GRUPO 4","911":"GRUPO 4","912":"GRUPO 1","913":"GRUPO 1","914":"GRUPO 1","915":"GRUPO 1","916":"GRUPO 1","917":"GRUPO 1","918":"GRUPO 1","919":"GRUPO 1","920":"GRUPO 1","921":"GRUPO 1","922":"GRUPO 1","923":"GRUPO 1","924":"GRUPO 2","925":"GRUPO 2","926":"GRUPO 2","927":"GRUPO 2","928":"GRUPO 2","929":"GRUPO 2","930":"GRUPO 2","931":"GRUPO 2","932":"GRUPO 2","933":"GRUPO 2","934":"GRUPO 2","935":"GRUPO 2","936":"GRUPO 3","937":"GRUPO 3","938":"GRUPO 3","939":"GRUPO 3","940":"GRUPO 3","941":"GRUPO 3","942":"GRUPO 3","943":"GRUPO 3","944":"GRUPO 3","945":"GRUPO 3","946":"GRUPO 3","947":"GRUPO 3","948":"GRUPO 4","949":"GRUPO 4","950":"GRUPO 4","951":"GRUPO 4","952":"GRUPO 4","953":"GRUPO 4","954":"GRUPO 4","955":"GRUPO 4","956":"GRUPO 4","957":"GRUPO 4","958":"GRUPO 4","959":"GRUPO 4","960":"GRUPO 1","961":"GRUPO 1","962":"GRUPO 1","963":"GRUPO 1","964":"GRUPO 1","965":"GRUPO 1","966":"GRUPO 1","967":"GRUPO 1","968":"GRUPO 1","969":"GRUPO 1","970":"GRUPO 1","971":"GRUPO 1","972":"GRUPO 2","973":"GRUPO 2","974":"GRUPO 2","975":"GRUPO 2","976":"GRUPO 2","977":"GRUPO 2","978":"GRUPO 2","979":"GRUPO 2","980":"GRUPO 2","981":"GRUPO 2","982":"GRUPO 2","983":"GRUPO 2","984":"GRUPO 3","985":"GRUPO 3","986":"GRUPO 3","987":"GRUPO 3","988":"GRUPO 3","989":"GRUPO 3","990":"GRUPO 3","991":"GRUPO 3","992":"GRUPO 3","993":"GRUPO 3","994":"GRUPO 3","995":"GRUPO 3","996":"GRUPO 4","997":"GRUPO 4","998":"GRUPO 4","999":"GRUPO 4","1000":"GRUPO 4","1001":"GRUPO 4","1002":"GRUPO 4","1003":"GRUPO 4","1004":"GRUPO 4","1005":"GRUPO 4","1006":"GRUPO 4","1007":"GRUPO 4","1008":"GRUPO 1","1009":"GRUPO 1","1010":"GRUPO 1","1011":"GRUPO 1","1012":"GRUPO 1","1013":"GRUPO 1","1014":"GRUPO 1","1015":"GRUPO 1","1016":"GRUPO 1","1017":"GRUPO 1","1018":"GRUPO 1","1019":"GRUPO 1","1020":"GRUPO 2","1021":"GRUPO 2","1022":"GRUPO 2","1023":"GRUPO 2","1024":"GRUPO 2","1025":"GRUPO 2","1026":"GRUPO 2","1027":"GRUPO 2","1028":"GRUPO 2","1029":"GRUPO 2","1030":"GRUPO 2","1031":"GRUPO 2","1032":"GRUPO 3","1033":"GRUPO 3","1034":"GRUPO 3","1035":"GRUPO 3","1036":"GRUPO 3","1037":"GRUPO 3","1038":"GRUPO 3","1039":"GRUPO 3","1040":"GRUPO 3","1041":"GRUPO 3","1042":"GRUPO 3","1043":"GRUPO 3","1044":"GRUPO 4","1045":"GRUPO 4","1046":"GRUPO 4","1047":"GRUPO 4","1048":"GRUPO 4","1049":"GRUPO 4","1050":"GRUPO 4","1051":"GRUPO 4","1052":"GRUPO 4","1053":"GRUPO 4","1054":"GRUPO 4","1055":"GRUPO 4","1056":"GRUPO 1","1057":"GRUPO 1","1058":"GRUPO 1","1059":"GRUPO 1","1060":"GRUPO 1","1061":"GRUPO 1","1062":"GRUPO 1","1063":"GRUPO 1","1064":"GRUPO 1","1065":"GRUPO 1","1066":"GRUPO 1","1067":"GRUPO 1","1068":"GRUPO 2","1069":"GRUPO 2","1070":"GRUPO 2","1071":"GRUPO 2","1072":"GRUPO 2","1073":"GRUPO 2","1074":"GRUPO 2","1075":"GRUPO 2","1076":"GRUPO 2","1077":"GRUPO 2","1078":"GRUPO 2","1079":"GRUPO 2","1080":"GRUPO 3","1081":"GRUPO 3","1082":"GRUPO 3","1083":"GRUPO 3","1084":"GRUPO 3","1085":"GRUPO 3","1086":"GRUPO 3","1087":"GRUPO 3","1088":"GRUPO 3","1089":"GRUPO 3","1090":"GRUPO 3","1091":"GRUPO 3","1092":"GRUPO 4","1093":"GRUPO 4","1094":"GRUPO 4","1095":"GRUPO 4","1096":"GRUPO 4","1097":"GRUPO 4","1098":"GRUPO 4","1099":"GRUPO 4","1100":"GRUPO 4","1101":"GRUPO 4","1102":"GRUPO 4","1103":"GRUPO 4","1104":"GRUPO 1","1105":"GRUPO 1","1106":"GRUPO 1","1107":"GRUPO 1","1108":"GRUPO 1","1109":"GRUPO 1","1110":"GRUPO 1","1111":"GRUPO 1","1112":"GRUPO 1","1113":"GRUPO 1","1114":"GRUPO 1","1115":"GRUPO 1","1116":"GRUPO 2","1117":"GRUPO 2","1118":"GRUPO 2","1119":"GRUPO 2","1120":"GRUPO 2","1121":"GRUPO 2","1122":"GRUPO 2","1123":"GRUPO 2","1124":"GRUPO 2","1125":"GRUPO 2","1126":"GRUPO 2","1127":"GRUPO 2","1128":"GRUPO 3","1129":"GRUPO 3","1130":"GRUPO 3","1131":"GRUPO 3","1132":"GRUPO 3","1133":"GRUPO 3","1134":"GRUPO 3","1135":"GRUPO 3","1136":"GRUPO 3","1137":"GRUPO 3","1138":"GRUPO 3","1139":"GRUPO 3","1140":"GRUPO 4","1141":"GRUPO 4","1142":"GRUPO 4","1143":"GRUPO 4","1144":"GRUPO 4","1145":"GRUPO 4","1146":"GRUPO 4","1147":"GRUPO 4","1148":"GRUPO 4","1149":"GRUPO 4","1150":"GRUPO 4","1151":"GRUPO 4","1152":"GRUPO 1","1153":"GRUPO 1","1154":"GRUPO 1","1155":"GRUPO 1","1156":"GRUPO 1","1157":"GRUPO 1","1158":"GRUPO 1","1159":"GRUPO 1","1160":"GRUPO 1","1161":"GRUPO 1","1162":"GRUPO 1","1163":"GRUPO 1","1164":"GRUPO 2","1165":"GRUPO 2","1166":"GRUPO 2","1167":"GRUPO 2","1168":"GRUPO 2","1169":"GRUPO 2","1170":"GRUPO 2","1171":"GRUPO 2","1172":"GRUPO 2","1173":"GRUPO 2","1174":"GRUPO 2","1175":"GRUPO 2","1176":"GRUPO 3","1177":"GRUPO 3","1178":"GRUPO 3","1179":"GRUPO 3","1180":"GRUPO 3","1181":"GRUPO 3","1182":"GRUPO 3","1183":"GRUPO 3","1184":"GRUPO 3","1185":"GRUPO 3","1186":"GRUPO 3","1187":"GRUPO 3","1188":"GRUPO 4","1189":"GRUPO 4","1190":"GRUPO 4","1191":"GRUPO 4","1192":"GRUPO 4","1193":"GRUPO 4","1194":"GRUPO 4","1195":"GRUPO 4","1196":"GRUPO 4","1197":"GRUPO 4","1198":"GRUPO 4","1199":"GRUPO 4","1200":"GRUPO 1","1201":"GRUPO 1","1202":"GRUPO 1","1203":"GRUPO 1","1204":"GRUPO 1","1205":"GRUPO 1","1206":"GRUPO 1","1207":"GRUPO 1","1208":"GRUPO 1","1209":"GRUPO 1","1210":"GRUPO 1","1211":"GRUPO 1","1212":"GRUPO 2","1213":"GRUPO 2","1214":"GRUPO 2","1215":"GRUPO 2","1216":"GRUPO 2","1217":"GRUPO 2","1218":"GRUPO 2","1219":"GRUPO 2","1220":"GRUPO 2","1221":"GRUPO 2","1222":"GRUPO 2","1223":"GRUPO 2","1224":"GRUPO 3","1225":"GRUPO 3","1226":"GRUPO 3","1227":"GRUPO 3","1228":"GRUPO 3","1229":"GRUPO 3","1230":"GRUPO 3","1231":"GRUPO 3","1232":"GRUPO 3","1233":"GRUPO 3","1234":"GRUPO 3","1235":"GRUPO 3","1236":"GRUPO 4","1237":"GRUPO 4","1238":"GRUPO 4","1239":"GRUPO 4","1240":"GRUPO 4","1241":"GRUPO 4","1242":"GRUPO 4","1243":"GRUPO 4","1244":"GRUPO 4","1245":"GRUPO 4","1246":"GRUPO 4","1247":"GRUPO 4","1248":"GRUPO 1","1249":"GRUPO 1","1250":"GRUPO 1","1251":"GRUPO 1","1252":"GRUPO 1","1253":"GRUPO 1","1254":"GRUPO 1","1255":"GRUPO 1","1256":"GRUPO 1","1257":"GRUPO 1","1258":"GRUPO 1","1259":"GRUPO 1","1260":"GRUPO 2","1261":"GRUPO 2","1262":"GRUPO 2","1263":"GRUPO 2","1264":"GRUPO 2","1265":"GRUPO 2","1266":"GRUPO 2","1267":"GRUPO 2","1268":"GRUPO 2","1269":"GRUPO 2","1270":"GRUPO 2","1271":"GRUPO 2","1272":"GRUPO 3","1273":"GRUPO 3","1274":"GRUPO 3","1275":"GRUPO 3","1276":"GRUPO 3","1277":"GRUPO 3","1278":"GRUPO 3","1279":"GRUPO 3","1280":"GRUPO 3","1281":"GRUPO 3","1282":"GRUPO 3","1283":"GRUPO 3","1284":"GRUPO 4","1285":"GRUPO 4","1286":"GRUPO 4","1287":"GRUPO 4","1288":"GRUPO 4","1289":"GRUPO 4","1290":"GRUPO 4","1291":"GRUPO 4","1292":"GRUPO 4","1293":"GRUPO 4","1294":"GRUPO 4","1295":"GRUPO 4","1296":"GRUPO 1","1297":"GRUPO 1","1298":"GRUPO 1","1299":"GRUPO 1","1300":"GRUPO 1","1301":"GRUPO 1","1302":"GRUPO 1","1303":"GRUPO 1","1304":"GRUPO 1","1305":"GRUPO 1","1306":"GRUPO 1","1307":"GRUPO 1","1308":"GRUPO 2","1309":"GRUPO 2","1310":"GRUPO 2","1311":"GRUPO 2","1312":"GRUPO 2","1313":"GRUPO 2","1314":"GRUPO 2","1315":"GRUPO 2","1316":"GRUPO 2","1317":"GRUPO 2","1318":"GRUPO 2","1319":"GRUPO 2","1320":"GRUPO 3","1321":"GRUPO 3","1322":"GRUPO 3","1323":"GRUPO 3","1324":"GRUPO 3","1325":"GRUPO 3","1326":"GRUPO 3","1327":"GRUPO 3","1328":"GRUPO 3","1329":"GRUPO 3","1330":"GRUPO 3","1331":"GRUPO 3","1332":"GRUPO 4","1333":"GRUPO 4","1334":"GRUPO 4","1335":"GRUPO 4","1336":"GRUPO 4","1337":"GRUPO 4","1338":"GRUPO 4","1339":"GRUPO 4","1340":"GRUPO 4","1341":"GRUPO 4","1342":"GRUPO 4","1343":"GRUPO 4","1344":"GRUPO 1","1345":"GRUPO 1","1346":"GRUPO 1","1347":"GRUPO 1","1348":"GRUPO 1","1349":"GRUPO 1","1350":"GRUPO 1","1351":"GRUPO 1","1352":"GRUPO 1","1353":"GRUPO 1","1354":"GRUPO 1","1355":"GRUPO 1","1356":"GRUPO 2","1357":"GRUPO 2","1358":"GRUPO 2","1359":"GRUPO 2","1360":"GRUPO 2","1361":"GRUPO 2","1362":"GRUPO 2","1363":"GRUPO 2","1364":"GRUPO 2","1365":"GRUPO 2","1366":"GRUPO 2","1367":"GRUPO 2","1368":"GRUPO 3","1369":"GRUPO 3","1370":"GRUPO 3","1371":"GRUPO 3","1372":"GRUPO 3","1373":"GRUPO 3","1374":"GRUPO 3","1375":"GRUPO 3","1376":"GRUPO 3","1377":"GRUPO 3","1378":"GRUPO 3","1379":"GRUPO 3","1380":"GRUPO 4","1381":"GRUPO 4","1382":"GRUPO 4","1383":"GRUPO 4","1384":"GRUPO 4","1385":"GRUPO 4","1386":"GRUPO 4","1387":"GRUPO 4","1388":"GRUPO 4","1389":"GRUPO 4","1390":"GRUPO 4","1391":"GRUPO 4","1392":"GRUPO 1","1393":"GRUPO 1","1394":"GRUPO 1","1395":"GRUPO 1","1396":"GRUPO 1","1397":"GRUPO 1","1398":"GRUPO 1","1399":"GRUPO 1","1400":"GRUPO 1","1401":"GRUPO 1","1402":"GRUPO 1","1403":"GRUPO 1","1404":"GRUPO 2","1405":"GRUPO 2","1406":"GRUPO 2","1407":"GRUPO 2","1408":"GRUPO 2","1409":"GRUPO 2","1410":"GRUPO 2","1411":"GRUPO 2","1412":"GRUPO 2","1413":"GRUPO 2","1414":"GRUPO 2","1415":"GRUPO 2","1416":"GRUPO 3","1417":"GRUPO 3","1418":"GRUPO 3","1419":"GRUPO 3","1420":"GRUPO 3","1421":"GRUPO 3","1422":"GRUPO 3","1423":"GRUPO 3","1424":"GRUPO 3","1425":"GRUPO 3","1426":"GRUPO 3","1427":"GRUPO 3","1428":"GRUPO 4","1429":"GRUPO 4","1430":"GRUPO 4","1431":"GRUPO 4","1432":"GRUPO 4","1433":"GRUPO 4","1434":"GRUPO 4","1435":"GRUPO 4","1436":"GRUPO 4","1437":"GRUPO 4","1438":"GRUPO 4","1439":"GRUPO 4"},"Empleado":{"0":"BARON HERNANDEZ HAROLD ANTONIO","1":"CASTELLANOS CARVAJAL DEYVITH FABIAN","2":"AROCA TORRES JULIAN EDUARDO","3":"BERMUDEZ PARRA JENNIFER XIOMARA","4":"BERNAL BAQUERO JAMES RICARDO","5":"BURGOS ORTIZ JOSE HORACIO","6":"CANTOR PORRAS JUAN FERNEY","7":"CAPERA CAPERA JOSE GABRIEL","8":"CARDENAS LOTERO RICARDO ANDR\u00c9S","9":"RENDON OSPINA NELSON LEANDRO","10":"SARMIENTO URBINA MOISES DANIEL","11":"VELASCO VELASCO SEBASTI\u00c1N DAVID","12":"DELGADO DELGADO JOHAN DARIO","13":"FLOREZ SAUCESO KENIS ALBERTO","14":"CARDONA GARCIA OSCAR JAVIER","15":"CARVAJAL GARC\u00cdA HOVER MARCK","16":"CEPEDA PIRAQUIVE JUAN DAVID","17":"FAJARDO SAENZ OSCAR FERNANDO","18":"FLOREZ ESPITIA RONY ALBERTO","19":"GARCIA CUERVO EDWIN JAVIER","20":"GONZALEZ OCHOA JUAN CARLOS","21":"XXX1","22":"XXX2","23":"XXX3","24":"FONSECA RAY RICARDO","25":"GOMEZ BETANCUR JAIDER ANDRES","26":"GRANADA PATI\u00d1O CARLOS MARINO","27":"GRASS PLATA MIGUEL SNEIDER","28":"MANZANO CALVO JUAN SEBASTIAN","29":"MENDOZA GOITA MARIANSEL ZENAYDA","30":"MURILLO ARAQUE JAIVER GEOVANY","31":"NI\u00d1O ARENAS HECTOR GONZALO","32":"RAMIREZ CHAVERRA JHON EDISON","33":"XXX4","34":"XXX5","35":"XXX6","36":"RODRIGUEZ MOSQUERA LUIS FERNANDO","37":"PEPITO PEREZ","38":"RAMIREZ VARGAS MARCELA PAOLA","39":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","40":"TORO CISNEROS GARY JOSE","41":"USECHE CALDERON JADID ESTIVEN","42":"VASQUEZ NIETO CAMILO ANDRES","43":"JHONY CASTRO","44":"BERNAL JUAN DAVID","45":"XXX7","46":"XXX8","47":"XXX9","48":"BARON HERNANDEZ HAROLD ANTONIO","49":"CASTELLANOS CARVAJAL DEYVITH FABIAN","50":"AROCA TORRES JULIAN EDUARDO","51":"BERMUDEZ PARRA JENNIFER XIOMARA","52":"BERNAL BAQUERO JAMES RICARDO","53":"BURGOS ORTIZ JOSE HORACIO","54":"CANTOR PORRAS JUAN FERNEY","55":"CAPERA CAPERA JOSE GABRIEL","56":"CARDENAS LOTERO RICARDO ANDR\u00c9S","57":"RENDON OSPINA NELSON LEANDRO","58":"SARMIENTO URBINA MOISES DANIEL","59":"VELASCO VELASCO SEBASTI\u00c1N DAVID","60":"DELGADO DELGADO JOHAN DARIO","61":"FLOREZ SAUCESO KENIS ALBERTO","62":"CARDONA GARCIA OSCAR JAVIER","63":"CARVAJAL GARC\u00cdA HOVER MARCK","64":"CEPEDA PIRAQUIVE JUAN DAVID","65":"FAJARDO SAENZ OSCAR FERNANDO","66":"FLOREZ ESPITIA RONY ALBERTO","67":"GARCIA CUERVO EDWIN JAVIER","68":"GONZALEZ OCHOA JUAN CARLOS","69":"XXX1","70":"XXX2","71":"XXX3","72":"FONSECA RAY RICARDO","73":"GOMEZ BETANCUR JAIDER ANDRES","74":"GRANADA PATI\u00d1O CARLOS MARINO","75":"GRASS PLATA MIGUEL SNEIDER","76":"MANZANO CALVO JUAN SEBASTIAN","77":"MENDOZA GOITA MARIANSEL ZENAYDA","78":"MURILLO ARAQUE JAIVER GEOVANY","79":"NI\u00d1O ARENAS HECTOR GONZALO","80":"RAMIREZ CHAVERRA JHON EDISON","81":"XXX4","82":"XXX5","83":"XXX6","84":"RODRIGUEZ MOSQUERA LUIS FERNANDO","85":"PEPITO PEREZ","86":"RAMIREZ VARGAS MARCELA PAOLA","87":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","88":"TORO CISNEROS GARY JOSE","89":"USECHE CALDERON JADID ESTIVEN","90":"VASQUEZ NIETO CAMILO ANDRES","91":"JHONY CASTRO","92":"BERNAL JUAN DAVID","93":"XXX7","94":"XXX8","95":"XXX9","96":"BARON HERNANDEZ HAROLD ANTONIO","97":"CASTELLANOS CARVAJAL DEYVITH FABIAN","98":"AROCA TORRES JULIAN EDUARDO","99":"BERMUDEZ PARRA JENNIFER XIOMARA","100":"BERNAL BAQUERO JAMES RICARDO","101":"BURGOS ORTIZ JOSE HORACIO","102":"CANTOR PORRAS JUAN FERNEY","103":"CAPERA CAPERA JOSE GABRIEL","104":"CARDENAS LOTERO RICARDO ANDR\u00c9S","105":"RENDON OSPINA NELSON LEANDRO","106":"SARMIENTO URBINA MOISES DANIEL","107":"VELASCO VELASCO SEBASTI\u00c1N DAVID","108":"DELGADO DELGADO JOHAN DARIO","109":"FLOREZ SAUCESO KENIS ALBERTO","110":"CARDONA GARCIA OSCAR JAVIER","111":"CARVAJAL GARC\u00cdA HOVER MARCK","112":"CEPEDA PIRAQUIVE JUAN DAVID","113":"FAJARDO SAENZ OSCAR FERNANDO","114":"FLOREZ ESPITIA RONY ALBERTO","115":"GARCIA CUERVO EDWIN JAVIER","116":"GONZALEZ OCHOA JUAN CARLOS","117":"XXX1","118":"XXX2","119":"XXX3","120":"FONSECA RAY RICARDO","121":"GOMEZ BETANCUR JAIDER ANDRES","122":"GRANADA PATI\u00d1O CARLOS MARINO","123":"GRASS PLATA MIGUEL SNEIDER","124":"MANZANO CALVO JUAN SEBASTIAN","125":"MENDOZA GOITA MARIANSEL ZENAYDA","126":"MURILLO ARAQUE JAIVER GEOVANY","127":"NI\u00d1O ARENAS HECTOR GONZALO","128":"RAMIREZ CHAVERRA JHON EDISON","129":"XXX4","130":"XXX5","131":"XXX6","132":"RODRIGUEZ MOSQUERA LUIS FERNANDO","133":"PEPITO PEREZ","134":"RAMIREZ VARGAS MARCELA PAOLA","135":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","136":"TORO CISNEROS GARY JOSE","137":"USECHE CALDERON JADID ESTIVEN","138":"VASQUEZ NIETO CAMILO ANDRES","139":"JHONY CASTRO","140":"BERNAL JUAN DAVID","141":"XXX7","142":"XXX8","143":"XXX9","144":"BARON HERNANDEZ HAROLD ANTONIO","145":"CASTELLANOS CARVAJAL DEYVITH FABIAN","146":"AROCA TORRES JULIAN EDUARDO","147":"BERMUDEZ PARRA JENNIFER XIOMARA","148":"BERNAL BAQUERO JAMES RICARDO","149":"BURGOS ORTIZ JOSE HORACIO","150":"CANTOR PORRAS JUAN FERNEY","151":"CAPERA CAPERA JOSE GABRIEL","152":"CARDENAS LOTERO RICARDO ANDR\u00c9S","153":"RENDON OSPINA NELSON LEANDRO","154":"SARMIENTO URBINA MOISES DANIEL","155":"VELASCO VELASCO SEBASTI\u00c1N DAVID","156":"DELGADO DELGADO JOHAN DARIO","157":"FLOREZ SAUCESO KENIS ALBERTO","158":"CARDONA GARCIA OSCAR JAVIER","159":"CARVAJAL GARC\u00cdA HOVER MARCK","160":"CEPEDA PIRAQUIVE JUAN DAVID","161":"FAJARDO SAENZ OSCAR FERNANDO","162":"FLOREZ ESPITIA RONY ALBERTO","163":"GARCIA CUERVO EDWIN JAVIER","164":"GONZALEZ OCHOA JUAN CARLOS","165":"XXX1","166":"XXX2","167":"XXX3","168":"FONSECA RAY RICARDO","169":"GOMEZ BETANCUR JAIDER ANDRES","170":"GRANADA PATI\u00d1O CARLOS MARINO","171":"GRASS PLATA MIGUEL SNEIDER","172":"MANZANO CALVO JUAN SEBASTIAN","173":"MENDOZA GOITA MARIANSEL ZENAYDA","174":"MURILLO ARAQUE JAIVER GEOVANY","175":"NI\u00d1O ARENAS HECTOR GONZALO","176":"RAMIREZ CHAVERRA JHON EDISON","177":"XXX4","178":"XXX5","179":"XXX6","180":"RODRIGUEZ MOSQUERA LUIS FERNANDO","181":"PEPITO PEREZ","182":"RAMIREZ VARGAS MARCELA PAOLA","183":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","184":"TORO CISNEROS GARY JOSE","185":"USECHE CALDERON JADID ESTIVEN","186":"VASQUEZ NIETO CAMILO ANDRES","187":"JHONY CASTRO","188":"BERNAL JUAN DAVID","189":"XXX7","190":"XXX8","191":"XXX9","192":"BARON HERNANDEZ HAROLD ANTONIO","193":"CASTELLANOS CARVAJAL DEYVITH FABIAN","194":"AROCA TORRES JULIAN EDUARDO","195":"BERMUDEZ PARRA JENNIFER XIOMARA","196":"BERNAL BAQUERO JAMES RICARDO","197":"BURGOS ORTIZ JOSE HORACIO","198":"CANTOR PORRAS JUAN FERNEY","199":"CAPERA CAPERA JOSE GABRIEL","200":"CARDENAS LOTERO RICARDO ANDR\u00c9S","201":"RENDON OSPINA NELSON LEANDRO","202":"SARMIENTO URBINA MOISES DANIEL","203":"VELASCO VELASCO SEBASTI\u00c1N DAVID","204":"DELGADO DELGADO JOHAN DARIO","205":"FLOREZ SAUCESO KENIS ALBERTO","206":"CARDONA GARCIA OSCAR JAVIER","207":"CARVAJAL GARC\u00cdA HOVER MARCK","208":"CEPEDA PIRAQUIVE JUAN DAVID","209":"FAJARDO SAENZ OSCAR FERNANDO","210":"FLOREZ ESPITIA RONY ALBERTO","211":"GARCIA CUERVO EDWIN JAVIER","212":"GONZALEZ OCHOA JUAN CARLOS","213":"XXX1","214":"XXX2","215":"XXX3","216":"FONSECA RAY RICARDO","217":"GOMEZ BETANCUR JAIDER ANDRES","218":"GRANADA PATI\u00d1O CARLOS MARINO","219":"GRASS PLATA MIGUEL SNEIDER","220":"MANZANO CALVO JUAN SEBASTIAN","221":"MENDOZA GOITA MARIANSEL ZENAYDA","222":"MURILLO ARAQUE JAIVER GEOVANY","223":"NI\u00d1O ARENAS HECTOR GONZALO","224":"RAMIREZ CHAVERRA JHON EDISON","225":"XXX4","226":"XXX5","227":"XXX6","228":"RODRIGUEZ MOSQUERA LUIS FERNANDO","229":"PEPITO PEREZ","230":"RAMIREZ VARGAS MARCELA PAOLA","231":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","232":"TORO CISNEROS GARY JOSE","233":"USECHE CALDERON JADID ESTIVEN","234":"VASQUEZ NIETO CAMILO ANDRES","235":"JHONY CASTRO","236":"BERNAL JUAN DAVID","237":"XXX7","238":"XXX8","239":"XXX9","240":"BARON HERNANDEZ HAROLD ANTONIO","241":"CASTELLANOS CARVAJAL DEYVITH FABIAN","242":"AROCA TORRES JULIAN EDUARDO","243":"BERMUDEZ PARRA JENNIFER XIOMARA","244":"BERNAL BAQUERO JAMES RICARDO","245":"BURGOS ORTIZ JOSE HORACIO","246":"CANTOR PORRAS JUAN FERNEY","247":"CAPERA CAPERA JOSE GABRIEL","248":"CARDENAS LOTERO RICARDO ANDR\u00c9S","249":"RENDON OSPINA NELSON LEANDRO","250":"SARMIENTO URBINA MOISES DANIEL","251":"VELASCO VELASCO SEBASTI\u00c1N DAVID","252":"DELGADO DELGADO JOHAN DARIO","253":"FLOREZ SAUCESO KENIS ALBERTO","254":"CARDONA GARCIA OSCAR JAVIER","255":"CARVAJAL GARC\u00cdA HOVER MARCK","256":"CEPEDA PIRAQUIVE JUAN DAVID","257":"FAJARDO SAENZ OSCAR FERNANDO","258":"FLOREZ ESPITIA RONY ALBERTO","259":"GARCIA CUERVO EDWIN JAVIER","260":"GONZALEZ OCHOA JUAN CARLOS","261":"XXX1","262":"XXX2","263":"XXX3","264":"FONSECA RAY RICARDO","265":"GOMEZ BETANCUR JAIDER ANDRES","266":"GRANADA PATI\u00d1O CARLOS MARINO","267":"GRASS PLATA MIGUEL SNEIDER","268":"MANZANO CALVO JUAN SEBASTIAN","269":"MENDOZA GOITA MARIANSEL ZENAYDA","270":"MURILLO ARAQUE JAIVER GEOVANY","271":"NI\u00d1O ARENAS HECTOR GONZALO","272":"RAMIREZ CHAVERRA JHON EDISON","273":"XXX4","274":"XXX5","275":"XXX6","276":"RODRIGUEZ MOSQUERA LUIS FERNANDO","277":"PEPITO PEREZ","278":"RAMIREZ VARGAS MARCELA PAOLA","279":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","280":"TORO CISNEROS GARY JOSE","281":"USECHE CALDERON JADID ESTIVEN","282":"VASQUEZ NIETO CAMILO ANDRES","283":"JHONY CASTRO","284":"BERNAL JUAN DAVID","285":"XXX7","286":"XXX8","287":"XXX9","288":"BARON HERNANDEZ HAROLD ANTONIO","289":"CASTELLANOS CARVAJAL DEYVITH FABIAN","290":"AROCA TORRES JULIAN EDUARDO","291":"BERMUDEZ PARRA JENNIFER XIOMARA","292":"BERNAL BAQUERO JAMES RICARDO","293":"BURGOS ORTIZ JOSE</t>
+  </si>
+  <si>
+    <t>{"Grupo":{"0":"GRUPO 1","1":"GRUPO 1","2":"GRUPO 1","3":"GRUPO 1","4":"GRUPO 1","5":"GRUPO 1","6":"GRUPO 1","7":"GRUPO 1","8":"GRUPO 1","9":"GRUPO 1","10":"GRUPO 1","11":"GRUPO 1","12":"GRUPO 2","13":"GRUPO 2","14":"GRUPO 2","15":"GRUPO 2","16":"GRUPO 2","17":"GRUPO 2","18":"GRUPO 2","19":"GRUPO 2","20":"GRUPO 2","21":"GRUPO 2","22":"GRUPO 2","23":"GRUPO 2","24":"GRUPO 3","25":"GRUPO 3","26":"GRUPO 3","27":"GRUPO 3","28":"GRUPO 3","29":"GRUPO 3","30":"GRUPO 3","31":"GRUPO 3","32":"GRUPO 3","33":"GRUPO 3","34":"GRUPO 3","35":"GRUPO 3","36":"GRUPO 4","37":"GRUPO 4","38":"GRUPO 4","39":"GRUPO 4","40":"GRUPO 4","41":"GRUPO 4","42":"GRUPO 4","43":"GRUPO 4","44":"GRUPO 4","45":"GRUPO 4","46":"GRUPO 4","47":"GRUPO 4","48":"GRUPO 1","49":"GRUPO 1","50":"GRUPO 1","51":"GRUPO 1","52":"GRUPO 1","53":"GRUPO 1","54":"GRUPO 1","55":"GRUPO 1","56":"GRUPO 1","57":"GRUPO 1","58":"GRUPO 1","59":"GRUPO 1","60":"GRUPO 2","61":"GRUPO 2","62":"GRUPO 2","63":"GRUPO 2","64":"GRUPO 2","65":"GRUPO 2","66":"GRUPO 2","67":"GRUPO 2","68":"GRUPO 2","69":"GRUPO 2","70":"GRUPO 2","71":"GRUPO 2","72":"GRUPO 3","73":"GRUPO 3","74":"GRUPO 3","75":"GRUPO 3","76":"GRUPO 3","77":"GRUPO 3","78":"GRUPO 3","79":"GRUPO 3","80":"GRUPO 3","81":"GRUPO 3","82":"GRUPO 3","83":"GRUPO 3","84":"GRUPO 4","85":"GRUPO 4","86":"GRUPO 4","87":"GRUPO 4","88":"GRUPO 4","89":"GRUPO 4","90":"GRUPO 4","91":"GRUPO 4","92":"GRUPO 4","93":"GRUPO 4","94":"GRUPO 4","95":"GRUPO 4","96":"GRUPO 1","97":"GRUPO 1","98":"GRUPO 1","99":"GRUPO 1","100":"GRUPO 1","101":"GRUPO 1","102":"GRUPO 1","103":"GRUPO 1","104":"GRUPO 1","105":"GRUPO 1","106":"GRUPO 1","107":"GRUPO 1","108":"GRUPO 2","109":"GRUPO 2","110":"GRUPO 2","111":"GRUPO 2","112":"GRUPO 2","113":"GRUPO 2","114":"GRUPO 2","115":"GRUPO 2","116":"GRUPO 2","117":"GRUPO 2","118":"GRUPO 2","119":"GRUPO 2","120":"GRUPO 3","121":"GRUPO 3","122":"GRUPO 3","123":"GRUPO 3","124":"GRUPO 3","125":"GRUPO 3","126":"GRUPO 3","127":"GRUPO 3","128":"GRUPO 3","129":"GRUPO 3","130":"GRUPO 3","131":"GRUPO 3","132":"GRUPO 4","133":"GRUPO 4","134":"GRUPO 4","135":"GRUPO 4","136":"GRUPO 4","137":"GRUPO 4","138":"GRUPO 4","139":"GRUPO 4","140":"GRUPO 4","141":"GRUPO 4","142":"GRUPO 4","143":"GRUPO 4","144":"GRUPO 1","145":"GRUPO 1","146":"GRUPO 1","147":"GRUPO 1","148":"GRUPO 1","149":"GRUPO 1","150":"GRUPO 1","151":"GRUPO 1","152":"GRUPO 1","153":"GRUPO 1","154":"GRUPO 1","155":"GRUPO 1","156":"GRUPO 2","157":"GRUPO 2","158":"GRUPO 2","159":"GRUPO 2","160":"GRUPO 2","161":"GRUPO 2","162":"GRUPO 2","163":"GRUPO 2","164":"GRUPO 2","165":"GRUPO 2","166":"GRUPO 2","167":"GRUPO 2","168":"GRUPO 3","169":"GRUPO 3","170":"GRUPO 3","171":"GRUPO 3","172":"GRUPO 3","173":"GRUPO 3","174":"GRUPO 3","175":"GRUPO 3","176":"GRUPO 3","177":"GRUPO 3","178":"GRUPO 3","179":"GRUPO 3","180":"GRUPO 4","181":"GRUPO 4","182":"GRUPO 4","183":"GRUPO 4","184":"GRUPO 4","185":"GRUPO 4","186":"GRUPO 4","187":"GRUPO 4","188":"GRUPO 4","189":"GRUPO 4","190":"GRUPO 4","191":"GRUPO 4","192":"GRUPO 1","193":"GRUPO 1","194":"GRUPO 1","195":"GRUPO 1","196":"GRUPO 1","197":"GRUPO 1","198":"GRUPO 1","199":"GRUPO 1","200":"GRUPO 1","201":"GRUPO 1","202":"GRUPO 1","203":"GRUPO 1","204":"GRUPO 2","205":"GRUPO 2","206":"GRUPO 2","207":"GRUPO 2","208":"GRUPO 2","209":"GRUPO 2","210":"GRUPO 2","211":"GRUPO 2","212":"GRUPO 2","213":"GRUPO 2","214":"GRUPO 2","215":"GRUPO 2","216":"GRUPO 3","217":"GRUPO 3","218":"GRUPO 3","219":"GRUPO 3","220":"GRUPO 3","221":"GRUPO 3","222":"GRUPO 3","223":"GRUPO 3","224":"GRUPO 3","225":"GRUPO 3","226":"GRUPO 3","227":"GRUPO 3","228":"GRUPO 4","229":"GRUPO 4","230":"GRUPO 4","231":"GRUPO 4","232":"GRUPO 4","233":"GRUPO 4","234":"GRUPO 4","235":"GRUPO 4","236":"GRUPO 4","237":"GRUPO 4","238":"GRUPO 4","239":"GRUPO 4","240":"GRUPO 1","241":"GRUPO 1","242":"GRUPO 1","243":"GRUPO 1","244":"GRUPO 1","245":"GRUPO 1","246":"GRUPO 1","247":"GRUPO 1","248":"GRUPO 1","249":"GRUPO 1","250":"GRUPO 1","251":"GRUPO 1","252":"GRUPO 2","253":"GRUPO 2","254":"GRUPO 2","255":"GRUPO 2","256":"GRUPO 2","257":"GRUPO 2","258":"GRUPO 2","259":"GRUPO 2","260":"GRUPO 2","261":"GRUPO 2","262":"GRUPO 2","263":"GRUPO 2","264":"GRUPO 3","265":"GRUPO 3","266":"GRUPO 3","267":"GRUPO 3","268":"GRUPO 3","269":"GRUPO 3","270":"GRUPO 3","271":"GRUPO 3","272":"GRUPO 3","273":"GRUPO 3","274":"GRUPO 3","275":"GRUPO 3","276":"GRUPO 4","277":"GRUPO 4","278":"GRUPO 4","279":"GRUPO 4","280":"GRUPO 4","281":"GRUPO 4","282":"GRUPO 4","283":"GRUPO 4","284":"GRUPO 4","285":"GRUPO 4","286":"GRUPO 4","287":"GRUPO 4","288":"GRUPO 1","289":"GRUPO 1","290":"GRUPO 1","291":"GRUPO 1","292":"GRUPO 1","293":"GRUPO 1","294":"GRUPO 1","295":"GRUPO 1","296":"GRUPO 1","297":"GRUPO 1","298":"GRUPO 1","299":"GRUPO 1","300":"GRUPO 2","301":"GRUPO 2","302":"GRUPO 2","303":"GRUPO 2","304":"GRUPO 2","305":"GRUPO 2","306":"GRUPO 2","307":"GRUPO 2","308":"GRUPO 2","309":"GRUPO 2","310":"GRUPO 2","311":"GRUPO 2","312":"GRUPO 3","313":"GRUPO 3","314":"GRUPO 3","315":"GRUPO 3","316":"GRUPO 3","317":"GRUPO 3","318":"GRUPO 3","319":"GRUPO 3","320":"GRUPO 3","321":"GRUPO 3","322":"GRUPO 3","323":"GRUPO 3","324":"GRUPO 4","325":"GRUPO 4","326":"GRUPO 4","327":"GRUPO 4","328":"GRUPO 4","329":"GRUPO 4","330":"GRUPO 4","331":"GRUPO 4","332":"GRUPO 4","333":"GRUPO 4","334":"GRUPO 4","335":"GRUPO 4","336":"GRUPO 1","337":"GRUPO 1","338":"GRUPO 1","339":"GRUPO 1","340":"GRUPO 1","341":"GRUPO 1","342":"GRUPO 1","343":"GRUPO 1","344":"GRUPO 1","345":"GRUPO 1","346":"GRUPO 1","347":"GRUPO 1","348":"GRUPO 2","349":"GRUPO 2","350":"GRUPO 2","351":"GRUPO 2","352":"GRUPO 2","353":"GRUPO 2","354":"GRUPO 2","355":"GRUPO 2","356":"GRUPO 2","357":"GRUPO 2","358":"GRUPO 2","359":"GRUPO 2","360":"GRUPO 3","361":"GRUPO 3","362":"GRUPO 3","363":"GRUPO 3","364":"GRUPO 3","365":"GRUPO 3","366":"GRUPO 3","367":"GRUPO 3","368":"GRUPO 3","369":"GRUPO 3","370":"GRUPO 3","371":"GRUPO 3","372":"GRUPO 4","373":"GRUPO 4","374":"GRUPO 4","375":"GRUPO 4","376":"GRUPO 4","377":"GRUPO 4","378":"GRUPO 4","379":"GRUPO 4","380":"GRUPO 4","381":"GRUPO 4","382":"GRUPO 4","383":"GRUPO 4","384":"GRUPO 1","385":"GRUPO 1","386":"GRUPO 1","387":"GRUPO 1","388":"GRUPO 1","389":"GRUPO 1","390":"GRUPO 1","391":"GRUPO 1","392":"GRUPO 1","393":"GRUPO 1","394":"GRUPO 1","395":"GRUPO 1","396":"GRUPO 2","397":"GRUPO 2","398":"GRUPO 2","399":"GRUPO 2","400":"GRUPO 2","401":"GRUPO 2","402":"GRUPO 2","403":"GRUPO 2","404":"GRUPO 2","405":"GRUPO 2","406":"GRUPO 2","407":"GRUPO 2","408":"GRUPO 3","409":"GRUPO 3","410":"GRUPO 3","411":"GRUPO 3","412":"GRUPO 3","413":"GRUPO 3","414":"GRUPO 3","415":"GRUPO 3","416":"GRUPO 3","417":"GRUPO 3","418":"GRUPO 3","419":"GRUPO 3","420":"GRUPO 4","421":"GRUPO 4","422":"GRUPO 4","423":"GRUPO 4","424":"GRUPO 4","425":"GRUPO 4","426":"GRUPO 4","427":"GRUPO 4","428":"GRUPO 4","429":"GRUPO 4","430":"GRUPO 4","431":"GRUPO 4","432":"GRUPO 1","433":"GRUPO 1","434":"GRUPO 1","435":"GRUPO 1","436":"GRUPO 1","437":"GRUPO 1","438":"GRUPO 1","439":"GRUPO 1","440":"GRUPO 1","441":"GRUPO 1","442":"GRUPO 1","443":"GRUPO 1","444":"GRUPO 2","445":"GRUPO 2","446":"GRUPO 2","447":"GRUPO 2","448":"GRUPO 2","449":"GRUPO 2","450":"GRUPO 2","451":"GRUPO 2","452":"GRUPO 2","453":"GRUPO 2","454":"GRUPO 2","455":"GRUPO 2","456":"GRUPO 3","457":"GRUPO 3","458":"GRUPO 3","459":"GRUPO 3","460":"GRUPO 3","461":"GRUPO 3","462":"GRUPO 3","463":"GRUPO 3","464":"GRUPO 3","465":"GRUPO 3","466":"GRUPO 3","467":"GRUPO 3","468":"GRUPO 4","469":"GRUPO 4","470":"GRUPO 4","471":"GRUPO 4","472":"GRUPO 4","473":"GRUPO 4","474":"GRUPO 4","475":"GRUPO 4","476":"GRUPO 4","477":"GRUPO 4","478":"GRUPO 4","479":"GRUPO 4","480":"GRUPO 1","481":"GRUPO 1","482":"GRUPO 1","483":"GRUPO 1","484":"GRUPO 1","485":"GRUPO 1","486":"GRUPO 1","487":"GRUPO 1","488":"GRUPO 1","489":"GRUPO 1","490":"GRUPO 1","491":"GRUPO 1","492":"GRUPO 2","493":"GRUPO 2","494":"GRUPO 2","495":"GRUPO 2","496":"GRUPO 2","497":"GRUPO 2","498":"GRUPO 2","499":"GRUPO 2","500":"GRUPO 2","501":"GRUPO 2","502":"GRUPO 2","503":"GRUPO 2","504":"GRUPO 3","505":"GRUPO 3","506":"GRUPO 3","507":"GRUPO 3","508":"GRUPO 3","509":"GRUPO 3","510":"GRUPO 3","511":"GRUPO 3","512":"GRUPO 3","513":"GRUPO 3","514":"GRUPO 3","515":"GRUPO 3","516":"GRUPO 4","517":"GRUPO 4","518":"GRUPO 4","519":"GRUPO 4","520":"GRUPO 4","521":"GRUPO 4","522":"GRUPO 4","523":"GRUPO 4","524":"GRUPO 4","525":"GRUPO 4","526":"GRUPO 4","527":"GRUPO 4","528":"GRUPO 1","529":"GRUPO 1","530":"GRUPO 1","531":"GRUPO 1","532":"GRUPO 1","533":"GRUPO 1","534":"GRUPO 1","535":"GRUPO 1","536":"GRUPO 1","537":"GRUPO 1","538":"GRUPO 1","539":"GRUPO 1","540":"GRUPO 2","541":"GRUPO 2","542":"GRUPO 2","543":"GRUPO 2","544":"GRUPO 2","545":"GRUPO 2","546":"GRUPO 2","547":"GRUPO 2","548":"GRUPO 2","549":"GRUPO 2","550":"GRUPO 2","551":"GRUPO 2","552":"GRUPO 3","553":"GRUPO 3","554":"GRUPO 3","555":"GRUPO 3","556":"GRUPO 3","557":"GRUPO 3","558":"GRUPO 3","559":"GRUPO 3","560":"GRUPO 3","561":"GRUPO 3","562":"GRUPO 3","563":"GRUPO 3","564":"GRUPO 4","565":"GRUPO 4","566":"GRUPO 4","567":"GRUPO 4","568":"GRUPO 4","569":"GRUPO 4","570":"GRUPO 4","571":"GRUPO 4","572":"GRUPO 4","573":"GRUPO 4","574":"GRUPO 4","575":"GRUPO 4","576":"GRUPO 1","577":"GRUPO 1","578":"GRUPO 1","579":"GRUPO 1","580":"GRUPO 1","581":"GRUPO 1","582":"GRUPO 1","583":"GRUPO 1","584":"GRUPO 1","585":"GRUPO 1","586":"GRUPO 1","587":"GRUPO 1","588":"GRUPO 2","589":"GRUPO 2","590":"GRUPO 2","591":"GRUPO 2","592":"GRUPO 2","593":"GRUPO 2","594":"GRUPO 2","595":"GRUPO 2","596":"GRUPO 2","597":"GRUPO 2","598":"GRUPO 2","599":"GRUPO 2","600":"GRUPO 3","601":"GRUPO 3","602":"GRUPO 3","603":"GRUPO 3","604":"GRUPO 3","605":"GRUPO 3","606":"GRUPO 3","607":"GRUPO 3","608":"GRUPO 3","609":"GRUPO 3","610":"GRUPO 3","611":"GRUPO 3","612":"GRUPO 4","613":"GRUPO 4","614":"GRUPO 4","615":"GRUPO 4","616":"GRUPO 4","617":"GRUPO 4","618":"GRUPO 4","619":"GRUPO 4","620":"GRUPO 4","621":"GRUPO 4","622":"GRUPO 4","623":"GRUPO 4","624":"GRUPO 1","625":"GRUPO 1","626":"GRUPO 1","627":"GRUPO 1","628":"GRUPO 1","629":"GRUPO 1","630":"GRUPO 1","631":"GRUPO 1","632":"GRUPO 1","633":"GRUPO 1","634":"GRUPO 1","635":"GRUPO 1","636":"GRUPO 2","637":"GRUPO 2","638":"GRUPO 2","639":"GRUPO 2","640":"GRUPO 2","641":"GRUPO 2","642":"GRUPO 2","643":"GRUPO 2","644":"GRUPO 2","645":"GRUPO 2","646":"GRUPO 2","647":"GRUPO 2","648":"GRUPO 3","649":"GRUPO 3","650":"GRUPO 3","651":"GRUPO 3","652":"GRUPO 3","653":"GRUPO 3","654":"GRUPO 3","655":"GRUPO 3","656":"GRUPO 3","657":"GRUPO 3","658":"GRUPO 3","659":"GRUPO 3","660":"GRUPO 4","661":"GRUPO 4","662":"GRUPO 4","663":"GRUPO 4","664":"GRUPO 4","665":"GRUPO 4","666":"GRUPO 4","667":"GRUPO 4","668":"GRUPO 4","669":"GRUPO 4","670":"GRUPO 4","671":"GRUPO 4","672":"GRUPO 1","673":"GRUPO 1","674":"GRUPO 1","675":"GRUPO 1","676":"GRUPO 1","677":"GRUPO 1","678":"GRUPO 1","679":"GRUPO 1","680":"GRUPO 1","681":"GRUPO 1","682":"GRUPO 1","683":"GRUPO 1","684":"GRUPO 2","685":"GRUPO 2","686":"GRUPO 2","687":"GRUPO 2","688":"GRUPO 2","689":"GRUPO 2","690":"GRUPO 2","691":"GRUPO 2","692":"GRUPO 2","693":"GRUPO 2","694":"GRUPO 2","695":"GRUPO 2","696":"GRUPO 3","697":"GRUPO 3","698":"GRUPO 3","699":"GRUPO 3","700":"GRUPO 3","701":"GRUPO 3","702":"GRUPO 3","703":"GRUPO 3","704":"GRUPO 3","705":"GRUPO 3","706":"GRUPO 3","707":"GRUPO 3","708":"GRUPO 4","709":"GRUPO 4","710":"GRUPO 4","711":"GRUPO 4","712":"GRUPO 4","713":"GRUPO 4","714":"GRUPO 4","715":"GRUPO 4","716":"GRUPO 4","717":"GRUPO 4","718":"GRUPO 4","719":"GRUPO 4","720":"GRUPO 1","721":"GRUPO 1","722":"GRUPO 1","723":"GRUPO 1","724":"GRUPO 1","725":"GRUPO 1","726":"GRUPO 1","727":"GRUPO 1","728":"GRUPO 1","729":"GRUPO 1","730":"GRUPO 1","731":"GRUPO 1","732":"GRUPO 2","733":"GRUPO 2","734":"GRUPO 2","735":"GRUPO 2","736":"GRUPO 2","737":"GRUPO 2","738":"GRUPO 2","739":"GRUPO 2","740":"GRUPO 2","741":"GRUPO 2","742":"GRUPO 2","743":"GRUPO 2","744":"GRUPO 3","745":"GRUPO 3","746":"GRUPO 3","747":"GRUPO 3","748":"GRUPO 3","749":"GRUPO 3","750":"GRUPO 3","751":"GRUPO 3","752":"GRUPO 3","753":"GRUPO 3","754":"GRUPO 3","755":"GRUPO 3","756":"GRUPO 4","757":"GRUPO 4","758":"GRUPO 4","759":"GRUPO 4","760":"GRUPO 4","761":"GRUPO 4","762":"GRUPO 4","763":"GRUPO 4","764":"GRUPO 4","765":"GRUPO 4","766":"GRUPO 4","767":"GRUPO 4","768":"GRUPO 1","769":"GRUPO 1","770":"GRUPO 1","771":"GRUPO 1","772":"GRUPO 1","773":"GRUPO 1","774":"GRUPO 1","775":"GRUPO 1","776":"GRUPO 1","777":"GRUPO 1","778":"GRUPO 1","779":"GRUPO 1","780":"GRUPO 2","781":"GRUPO 2","782":"GRUPO 2","783":"GRUPO 2","784":"GRUPO 2","785":"GRUPO 2","786":"GRUPO 2","787":"GRUPO 2","788":"GRUPO 2","789":"GRUPO 2","790":"GRUPO 2","791":"GRUPO 2","792":"GRUPO 3","793":"GRUPO 3","794":"GRUPO 3","795":"GRUPO 3","796":"GRUPO 3","797":"GRUPO 3","798":"GRUPO 3","799":"GRUPO 3","800":"GRUPO 3","801":"GRUPO 3","802":"GRUPO 3","803":"GRUPO 3","804":"GRUPO 4","805":"GRUPO 4","806":"GRUPO 4","807":"GRUPO 4","808":"GRUPO 4","809":"GRUPO 4","810":"GRUPO 4","811":"GRUPO 4","812":"GRUPO 4","813":"GRUPO 4","814":"GRUPO 4","815":"GRUPO 4","816":"GRUPO 1","817":"GRUPO 1","818":"GRUPO 1","819":"GRUPO 1","820":"GRUPO 1","821":"GRUPO 1","822":"GRUPO 1","823":"GRUPO 1","824":"GRUPO 1","825":"GRUPO 1","826":"GRUPO 1","827":"GRUPO 1","828":"GRUPO 2","829":"GRUPO 2","830":"GRUPO 2","831":"GRUPO 2","832":"GRUPO 2","833":"GRUPO 2","834":"GRUPO 2","835":"GRUPO 2","836":"GRUPO 2","837":"GRUPO 2","838":"GRUPO 2","839":"GRUPO 2","840":"GRUPO 3","841":"GRUPO 3","842":"GRUPO 3","843":"GRUPO 3","844":"GRUPO 3","845":"GRUPO 3","846":"GRUPO 3","847":"GRUPO 3","848":"GRUPO 3","849":"GRUPO 3","850":"GRUPO 3","851":"GRUPO 3","852":"GRUPO 4","853":"GRUPO 4","854":"GRUPO 4","855":"GRUPO 4","856":"GRUPO 4","857":"GRUPO 4","858":"GRUPO 4","859":"GRUPO 4","860":"GRUPO 4","861":"GRUPO 4","862":"GRUPO 4","863":"GRUPO 4","864":"GRUPO 1","865":"GRUPO 1","866":"GRUPO 1","867":"GRUPO 1","868":"GRUPO 1","869":"GRUPO 1","870":"GRUPO 1","871":"GRUPO 1","872":"GRUPO 1","873":"GRUPO 1","874":"GRUPO 1","875":"GRUPO 1","876":"GRUPO 2","877":"GRUPO 2","878":"GRUPO 2","879":"GRUPO 2","880":"GRUPO 2","881":"GRUPO 2","882":"GRUPO 2","883":"GRUPO 2","884":"GRUPO 2","885":"GRUPO 2","886":"GRUPO 2","887":"GRUPO 2","888":"GRUPO 3","889":"GRUPO 3","890":"GRUPO 3","891":"GRUPO 3","892":"GRUPO 3","893":"GRUPO 3","894":"GRUPO 3","895":"GRUPO 3","896":"GRUPO 3","897":"GRUPO 3","898":"GRUPO 3","899":"GRUPO 3","900":"GRUPO 4","901":"GRUPO 4","902":"GRUPO 4","903":"GRUPO 4","904":"GRUPO 4","905":"GRUPO 4","906":"GRUPO 4","907":"GRUPO 4","908":"GRUPO 4","909":"GRUPO 4","910":"GRUPO 4","911":"GRUPO 4","912":"GRUPO 1","913":"GRUPO 1","914":"GRUPO 1","915":"GRUPO 1","916":"GRUPO 1","917":"GRUPO 1","918":"GRUPO 1","919":"GRUPO 1","920":"GRUPO 1","921":"GRUPO 1","922":"GRUPO 1","923":"GRUPO 1","924":"GRUPO 2","925":"GRUPO 2","926":"GRUPO 2","927":"GRUPO 2","928":"GRUPO 2","929":"GRUPO 2","930":"GRUPO 2","931":"GRUPO 2","932":"GRUPO 2","933":"GRUPO 2","934":"GRUPO 2","935":"GRUPO 2","936":"GRUPO 3","937":"GRUPO 3","938":"GRUPO 3","939":"GRUPO 3","940":"GRUPO 3","941":"GRUPO 3","942":"GRUPO 3","943":"GRUPO 3","944":"GRUPO 3","945":"GRUPO 3","946":"GRUPO 3","947":"GRUPO 3","948":"GRUPO 4","949":"GRUPO 4","950":"GRUPO 4","951":"GRUPO 4","952":"GRUPO 4","953":"GRUPO 4","954":"GRUPO 4","955":"GRUPO 4","956":"GRUPO 4","957":"GRUPO 4","958":"GRUPO 4","959":"GRUPO 4","960":"GRUPO 1","961":"GRUPO 1","962":"GRUPO 1","963":"GRUPO 1","964":"GRUPO 1","965":"GRUPO 1","966":"GRUPO 1","967":"GRUPO 1","968":"GRUPO 1","969":"GRUPO 1","970":"GRUPO 1","971":"GRUPO 1","972":"GRUPO 2","973":"GRUPO 2","974":"GRUPO 2","975":"GRUPO 2","976":"GRUPO 2","977":"GRUPO 2","978":"GRUPO 2","979":"GRUPO 2","980":"GRUPO 2","981":"GRUPO 2","982":"GRUPO 2","983":"GRUPO 2","984":"GRUPO 3","985":"GRUPO 3","986":"GRUPO 3","987":"GRUPO 3","988":"GRUPO 3","989":"GRUPO 3","990":"GRUPO 3","991":"GRUPO 3","992":"GRUPO 3","993":"GRUPO 3","994":"GRUPO 3","995":"GRUPO 3","996":"GRUPO 4","997":"GRUPO 4","998":"GRUPO 4","999":"GRUPO 4","1000":"GRUPO 4","1001":"GRUPO 4","1002":"GRUPO 4","1003":"GRUPO 4","1004":"GRUPO 4","1005":"GRUPO 4","1006":"GRUPO 4","1007":"GRUPO 4","1008":"GRUPO 1","1009":"GRUPO 1","1010":"GRUPO 1","1011":"GRUPO 1","1012":"GRUPO 1","1013":"GRUPO 1","1014":"GRUPO 1","1015":"GRUPO 1","1016":"GRUPO 1","1017":"GRUPO 1","1018":"GRUPO 1","1019":"GRUPO 1","1020":"GRUPO 2","1021":"GRUPO 2","1022":"GRUPO 2","1023":"GRUPO 2","1024":"GRUPO 2","1025":"GRUPO 2","1026":"GRUPO 2","1027":"GRUPO 2","1028":"GRUPO 2","1029":"GRUPO 2","1030":"GRUPO 2","1031":"GRUPO 2","1032":"GRUPO 3","1033":"GRUPO 3","1034":"GRUPO 3","1035":"GRUPO 3","1036":"GRUPO 3","1037":"GRUPO 3","1038":"GRUPO 3","1039":"GRUPO 3","1040":"GRUPO 3","1041":"GRUPO 3","1042":"GRUPO 3","1043":"GRUPO 3","1044":"GRUPO 4","1045":"GRUPO 4","1046":"GRUPO 4","1047":"GRUPO 4","1048":"GRUPO 4","1049":"GRUPO 4","1050":"GRUPO 4","1051":"GRUPO 4","1052":"GRUPO 4","1053":"GRUPO 4","1054":"GRUPO 4","1055":"GRUPO 4","1056":"GRUPO 1","1057":"GRUPO 1","1058":"GRUPO 1","1059":"GRUPO 1","1060":"GRUPO 1","1061":"GRUPO 1","1062":"GRUPO 1","1063":"GRUPO 1","1064":"GRUPO 1","1065":"GRUPO 1","1066":"GRUPO 1","1067":"GRUPO 1","1068":"GRUPO 2","1069":"GRUPO 2","1070":"GRUPO 2","1071":"GRUPO 2","1072":"GRUPO 2","1073":"GRUPO 2","1074":"GRUPO 2","1075":"GRUPO 2","1076":"GRUPO 2","1077":"GRUPO 2","1078":"GRUPO 2","1079":"GRUPO 2","1080":"GRUPO 3","1081":"GRUPO 3","1082":"GRUPO 3","1083":"GRUPO 3","1084":"GRUPO 3","1085":"GRUPO 3","1086":"GRUPO 3","1087":"GRUPO 3","1088":"GRUPO 3","1089":"GRUPO 3","1090":"GRUPO 3","1091":"GRUPO 3","1092":"GRUPO 4","1093":"GRUPO 4","1094":"GRUPO 4","1095":"GRUPO 4","1096":"GRUPO 4","1097":"GRUPO 4","1098":"GRUPO 4","1099":"GRUPO 4","1100":"GRUPO 4","1101":"GRUPO 4","1102":"GRUPO 4","1103":"GRUPO 4","1104":"GRUPO 1","1105":"GRUPO 1","1106":"GRUPO 1","1107":"GRUPO 1","1108":"GRUPO 1","1109":"GRUPO 1","1110":"GRUPO 1","1111":"GRUPO 1","1112":"GRUPO 1","1113":"GRUPO 1","1114":"GRUPO 1","1115":"GRUPO 1","1116":"GRUPO 2","1117":"GRUPO 2","1118":"GRUPO 2","1119":"GRUPO 2","1120":"GRUPO 2","1121":"GRUPO 2","1122":"GRUPO 2","1123":"GRUPO 2","1124":"GRUPO 2","1125":"GRUPO 2","1126":"GRUPO 2","1127":"GRUPO 2","1128":"GRUPO 3","1129":"GRUPO 3","1130":"GRUPO 3","1131":"GRUPO 3","1132":"GRUPO 3","1133":"GRUPO 3","1134":"GRUPO 3","1135":"GRUPO 3","1136":"GRUPO 3","1137":"GRUPO 3","1138":"GRUPO 3","1139":"GRUPO 3","1140":"GRUPO 4","1141":"GRUPO 4","1142":"GRUPO 4","1143":"GRUPO 4","1144":"GRUPO 4","1145":"GRUPO 4","1146":"GRUPO 4","1147":"GRUPO 4","1148":"GRUPO 4","1149":"GRUPO 4","1150":"GRUPO 4","1151":"GRUPO 4","1152":"GRUPO 1","1153":"GRUPO 1","1154":"GRUPO 1","1155":"GRUPO 1","1156":"GRUPO 1","1157":"GRUPO 1","1158":"GRUPO 1","1159":"GRUPO 1","1160":"GRUPO 1","1161":"GRUPO 1","1162":"GRUPO 1","1163":"GRUPO 1","1164":"GRUPO 2","1165":"GRUPO 2","1166":"GRUPO 2","1167":"GRUPO 2","1168":"GRUPO 2","1169":"GRUPO 2","1170":"GRUPO 2","1171":"GRUPO 2","1172":"GRUPO 2","1173":"GRUPO 2","1174":"GRUPO 2","1175":"GRUPO 2","1176":"GRUPO 3","1177":"GRUPO 3","1178":"GRUPO 3","1179":"GRUPO 3","1180":"GRUPO 3","1181":"GRUPO 3","1182":"GRUPO 3","1183":"GRUPO 3","1184":"GRUPO 3","1185":"GRUPO 3","1186":"GRUPO 3","1187":"GRUPO 3","1188":"GRUPO 4","1189":"GRUPO 4","1190":"GRUPO 4","1191":"GRUPO 4","1192":"GRUPO 4","1193":"GRUPO 4","1194":"GRUPO 4","1195":"GRUPO 4","1196":"GRUPO 4","1197":"GRUPO 4","1198":"GRUPO 4","1199":"GRUPO 4","1200":"GRUPO 1","1201":"GRUPO 1","1202":"GRUPO 1","1203":"GRUPO 1","1204":"GRUPO 1","1205":"GRUPO 1","1206":"GRUPO 1","1207":"GRUPO 1","1208":"GRUPO 1","1209":"GRUPO 1","1210":"GRUPO 1","1211":"GRUPO 1","1212":"GRUPO 2","1213":"GRUPO 2","1214":"GRUPO 2","1215":"GRUPO 2","1216":"GRUPO 2","1217":"GRUPO 2","1218":"GRUPO 2","1219":"GRUPO 2","1220":"GRUPO 2","1221":"GRUPO 2","1222":"GRUPO 2","1223":"GRUPO 2","1224":"GRUPO 3","1225":"GRUPO 3","1226":"GRUPO 3","1227":"GRUPO 3","1228":"GRUPO 3","1229":"GRUPO 3","1230":"GRUPO 3","1231":"GRUPO 3","1232":"GRUPO 3","1233":"GRUPO 3","1234":"GRUPO 3","1235":"GRUPO 3","1236":"GRUPO 4","1237":"GRUPO 4","1238":"GRUPO 4","1239":"GRUPO 4","1240":"GRUPO 4","1241":"GRUPO 4","1242":"GRUPO 4","1243":"GRUPO 4","1244":"GRUPO 4","1245":"GRUPO 4","1246":"GRUPO 4","1247":"GRUPO 4","1248":"GRUPO 1","1249":"GRUPO 1","1250":"GRUPO 1","1251":"GRUPO 1","1252":"GRUPO 1","1253":"GRUPO 1","1254":"GRUPO 1","1255":"GRUPO 1","1256":"GRUPO 1","1257":"GRUPO 1","1258":"GRUPO 1","1259":"GRUPO 1","1260":"GRUPO 2","1261":"GRUPO 2","1262":"GRUPO 2","1263":"GRUPO 2","1264":"GRUPO 2","1265":"GRUPO 2","1266":"GRUPO 2","1267":"GRUPO 2","1268":"GRUPO 2","1269":"GRUPO 2","1270":"GRUPO 2","1271":"GRUPO 2","1272":"GRUPO 3","1273":"GRUPO 3","1274":"GRUPO 3","1275":"GRUPO 3","1276":"GRUPO 3","1277":"GRUPO 3","1278":"GRUPO 3","1279":"GRUPO 3","1280":"GRUPO 3","1281":"GRUPO 3","1282":"GRUPO 3","1283":"GRUPO 3","1284":"GRUPO 4","1285":"GRUPO 4","1286":"GRUPO 4","1287":"GRUPO 4","1288":"GRUPO 4","1289":"GRUPO 4","1290":"GRUPO 4","1291":"GRUPO 4","1292":"GRUPO 4","1293":"GRUPO 4","1294":"GRUPO 4","1295":"GRUPO 4","1296":"GRUPO 1","1297":"GRUPO 1","1298":"GRUPO 1","1299":"GRUPO 1","1300":"GRUPO 1","1301":"GRUPO 1","1302":"GRUPO 1","1303":"GRUPO 1","1304":"GRUPO 1","1305":"GRUPO 1","1306":"GRUPO 1","1307":"GRUPO 1","1308":"GRUPO 2","1309":"GRUPO 2","1310":"GRUPO 2","1311":"GRUPO 2","1312":"GRUPO 2","1313":"GRUPO 2","1314":"GRUPO 2","1315":"GRUPO 2","1316":"GRUPO 2","1317":"GRUPO 2","1318":"GRUPO 2","1319":"GRUPO 2","1320":"GRUPO 3","1321":"GRUPO 3","1322":"GRUPO 3","1323":"GRUPO 3","1324":"GRUPO 3","1325":"GRUPO 3","1326":"GRUPO 3","1327":"GRUPO 3","1328":"GRUPO 3","1329":"GRUPO 3","1330":"GRUPO 3","1331":"GRUPO 3","1332":"GRUPO 4","1333":"GRUPO 4","1334":"GRUPO 4","1335":"GRUPO 4","1336":"GRUPO 4","1337":"GRUPO 4","1338":"GRUPO 4","1339":"GRUPO 4","1340":"GRUPO 4","1341":"GRUPO 4","1342":"GRUPO 4","1343":"GRUPO 4","1344":"GRUPO 1","1345":"GRUPO 1","1346":"GRUPO 1","1347":"GRUPO 1","1348":"GRUPO 1","1349":"GRUPO 1","1350":"GRUPO 1","1351":"GRUPO 1","1352":"GRUPO 1","1353":"GRUPO 1","1354":"GRUPO 1","1355":"GRUPO 1","1356":"GRUPO 2","1357":"GRUPO 2","1358":"GRUPO 2","1359":"GRUPO 2","1360":"GRUPO 2","1361":"GRUPO 2","1362":"GRUPO 2","1363":"GRUPO 2","1364":"GRUPO 2","1365":"GRUPO 2","1366":"GRUPO 2","1367":"GRUPO 2","1368":"GRUPO 3","1369":"GRUPO 3","1370":"GRUPO 3","1371":"GRUPO 3","1372":"GRUPO 3","1373":"GRUPO 3","1374":"GRUPO 3","1375":"GRUPO 3","1376":"GRUPO 3","1377":"GRUPO 3","1378":"GRUPO 3","1379":"GRUPO 3","1380":"GRUPO 4","1381":"GRUPO 4","1382":"GRUPO 4","1383":"GRUPO 4","1384":"GRUPO 4","1385":"GRUPO 4","1386":"GRUPO 4","1387":"GRUPO 4","1388":"GRUPO 4","1389":"GRUPO 4","1390":"GRUPO 4","1391":"GRUPO 4","1392":"GRUPO 1","1393":"GRUPO 1","1394":"GRUPO 1","1395":"GRUPO 1","1396":"GRUPO 1","1397":"GRUPO 1","1398":"GRUPO 1","1399":"GRUPO 1","1400":"GRUPO 1","1401":"GRUPO 1","1402":"GRUPO 1","1403":"GRUPO 1","1404":"GRUPO 2","1405":"GRUPO 2","1406":"GRUPO 2","1407":"GRUPO 2","1408":"GRUPO 2","1409":"GRUPO 2","1410":"GRUPO 2","1411":"GRUPO 2","1412":"GRUPO 2","1413":"GRUPO 2","1414":"GRUPO 2","1415":"GRUPO 2","1416":"GRUPO 3","1417":"GRUPO 3","1418":"GRUPO 3","1419":"GRUPO 3","1420":"GRUPO 3","1421":"GRUPO 3","1422":"GRUPO 3","1423":"GRUPO 3","1424":"GRUPO 3","1425":"GRUPO 3","1426":"GRUPO 3","1427":"GRUPO 3","1428":"GRUPO 4","1429":"GRUPO 4","1430":"GRUPO 4","1431":"GRUPO 4","1432":"GRUPO 4","1433":"GRUPO 4","1434":"GRUPO 4","1435":"GRUPO 4","1436":"GRUPO 4","1437":"GRUPO 4","1438":"GRUPO 4","1439":"GRUPO 4","1440":"GRUPO 1","1441":"GRUPO 1","1442":"GRUPO 1","1443":"GRUPO 1","1444":"GRUPO 1","1445":"GRUPO 1","1446":"GRUPO 1","1447":"GRUPO 1","1448":"GRUPO 1","1449":"GRUPO 1","1450":"GRUPO 1","1451":"GRUPO 1","1452":"GRUPO 2","1453":"GRUPO 2","1454":"GRUPO 2","1455":"GRUPO 2","1456":"GRUPO 2","1457":"GRUPO 2","1458":"GRUPO 2","1459":"GRUPO 2","1460":"GRUPO 2","1461":"GRUPO 2","1462":"GRUPO 2","1463":"GRUPO 2","1464":"GRUPO 3","1465":"GRUPO 3","1466":"GRUPO 3","1467":"GRUPO 3","1468":"GRUPO 3","1469":"GRUPO 3","1470":"GRUPO 3","1471":"GRUPO 3","1472":"GRUPO 3","1473":"GRUPO 3","1474":"GRUPO 3","1475":"GRUPO 3","1476":"GRUPO 4","1477":"GRUPO 4","1478":"GRUPO 4","1479":"GRUPO 4","1480":"GRUPO 4","1481":"GRUPO 4","1482":"GRUPO 4","1483":"GRUPO 4","1484":"GRUPO 4","1485":"GRUPO 4","1486":"GRUPO 4","1487":"GRUPO 4"},"Empleado":{"0":"BARON HERNANDEZ HAROLD ANTONIO","1":"CASTELLANOS CARVAJAL DEYVITH FABIAN","2":"AROCA TORRES JULIAN EDUARDO","3":"BERMUDEZ PARRA JENNIFER XIOMARA","4":"BERNAL BAQUERO JAMES RICARDO","5":"BURGOS ORTIZ JOSE HORACIO","6":"CANTOR PORRAS JUAN FERNEY","7":"CAPERA CAPERA JOSE GABRIEL","8":"CARDENAS LOTERO RICARDO ANDR\u00c9S","9":"RENDON OSPINA NELSON LEANDRO","10":"SARMIENTO URBINA MOISES DANIEL","11":"VELASCO VELASCO SEBASTI\u00c1N DAVID","12":"DELGADO DELGADO JOHAN DARIO","13":"FLOREZ SAUCESO KENIS ALBERTO","14":"CARDONA GARCIA OSCAR JAVIER","15":"CARVAJAL GARC\u00cdA HOVER MARCK","16":"CEPEDA PIRAQUIVE JUAN DAVID","17":"FAJARDO SAENZ OSCAR FERNANDO","18":"FLOREZ ESPITIA RONY ALBERTO","19":"GARCIA CUERVO EDWIN JAVIER","20":"GONZALEZ OCHOA JUAN CARLOS","21":"XXX1","22":"XXX2","23":"XXX3","24":"FONSECA RAY RICARDO","25":"GOMEZ BETANCUR JAIDER ANDRES","26":"GRANADA PATI\u00d1O CARLOS MARINO","27":"GRASS PLATA MIGUEL SNEIDER","28":"MANZANO CALVO JUAN SEBASTIAN","29":"MENDOZA GOITA MARIANSEL ZENAYDA","30":"MURILLO ARAQUE JAIVER GEOVANY","31":"NI\u00d1O ARENAS HECTOR GONZALO","32":"RAMIREZ CHAVERRA JHON EDISON","33":"XXX4","34":"XXX5","35":"XXX6","36":"RODRIGUEZ MOSQUERA LUIS FERNANDO","37":"PEPITO PEREZ","38":"RAMIREZ VARGAS MARCELA PAOLA","39":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","40":"TORO CISNEROS GARY JOSE","41":"USECHE CALDERON JADID ESTIVEN","42":"VASQUEZ NIETO CAMILO ANDRES","43":"JHONY CASTRO","44":"BERNAL JUAN DAVID","45":"XXX7","46":"XXX8","47":"XXX9","48":"BARON HERNANDEZ HAROLD ANTONIO","49":"CASTELLANOS CARVAJAL DEYVITH FABIAN","50":"AROCA TORRES JULIAN EDUARDO","51":"BERMUDEZ PARRA JENNIFER XIOMARA","52":"BERNAL BAQUERO JAMES RICARDO","53":"BURGOS ORTIZ JOSE HORACIO","54":"CANTOR PORRAS JUAN FERNEY","55":"CAPERA CAPERA JOSE GABRIEL","56":"CARDENAS LOTERO RICARDO ANDR\u00c9S","57":"RENDON OSPINA NELSON LEANDRO","58":"SARMIENTO URBINA MOISES DANIEL","59":"VELASCO VELASCO SEBASTI\u00c1N DAVID","60":"DELGADO DELGADO JOHAN DARIO","61":"FLOREZ SAUCESO KENIS ALBERTO","62":"CARDONA GARCIA OSCAR JAVIER","63":"CARVAJAL GARC\u00cdA HOVER MARCK","64":"CEPEDA PIRAQUIVE JUAN DAVID","65":"FAJARDO SAENZ OSCAR FERNANDO","66":"FLOREZ ESPITIA RONY ALBERTO","67":"GARCIA CUERVO EDWIN JAVIER","68":"GONZALEZ OCHOA JUAN CARLOS","69":"XXX1","70":"XXX2","71":"XXX3","72":"FONSECA RAY RICARDO","73":"GOMEZ BETANCUR JAIDER ANDRES","74":"GRANADA PATI\u00d1O CARLOS MARINO","75":"GRASS PLATA MIGUEL SNEIDER","76":"MANZANO CALVO JUAN SEBASTIAN","77":"MENDOZA GOITA MARIANSEL ZENAYDA","78":"MURILLO ARAQUE JAIVER GEOVANY","79":"NI\u00d1O ARENAS HECTOR GONZALO","80":"RAMIREZ CHAVERRA JHON EDISON","81":"XXX4","82":"XXX5","83":"XXX6","84":"RODRIGUEZ MOSQUERA LUIS FERNANDO","85":"PEPITO PEREZ","86":"RAMIREZ VARGAS MARCELA PAOLA","87":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","88":"TORO CISNEROS GARY JOSE","89":"USECHE CALDERON JADID ESTIVEN","90":"VASQUEZ NIETO CAMILO ANDRES","91":"JHONY CASTRO","92":"BERNAL JUAN DAVID","93":"XXX7","94":"XXX8","95":"XXX9","96":"BARON HERNANDEZ HAROLD ANTONIO","97":"CASTELLANOS CARVAJAL DEYVITH FABIAN","98":"AROCA TORRES JULIAN EDUARDO","99":"BERMUDEZ PARRA JENNIFER XIOMARA","100":"BERNAL BAQUERO JAMES RICARDO","101":"BURGOS ORTIZ JOSE HORACIO","102":"CANTOR PORRAS JUAN FERNEY","103":"CAPERA CAPERA JOSE GABRIEL","104":"CARDENAS LOTERO RICARDO ANDR\u00c9S","105":"RENDON OSPINA NELSON LEANDRO","106":"SARMIENTO URBINA MOISES DANIEL","107":"VELASCO VELASCO SEBASTI\u00c1N DAVID","108":"DELGADO DELGADO JOHAN DARIO","109":"FLOREZ SAUCESO KENIS ALBERTO","110":"CARDONA GARCIA OSCAR JAVIER","111":"CARVAJAL GARC\u00cdA HOVER MARCK","112":"CEPEDA PIRAQUIVE JUAN DAVID","113":"FAJARDO SAENZ OSCAR FERNANDO","114":"FLOREZ ESPITIA RONY ALBERTO","115":"GARCIA CUERVO EDWIN JAVIER","116":"GONZALEZ OCHOA JUAN CARLOS","117":"XXX1","118":"XXX2","119":"XXX3","120":"FONSECA RAY RICARDO","121":"GOMEZ BETANCUR JAIDER ANDRES","122":"GRANADA PATI\u00d1O CARLOS MARINO","123":"GRASS PLATA MIGUEL SNEIDER","124":"MANZANO CALVO JUAN SEBASTIAN","125":"MENDOZA GOITA MARIANSEL ZENAYDA","126":"MURILLO ARAQUE JAIVER GEOVANY","127":"NI\u00d1O ARENAS HECTOR GONZALO","128":"RAMIREZ CHAVERRA JHON EDISON","129":"XXX4","130":"XXX5","131":"XXX6","132":"RODRIGUEZ MOSQUERA LUIS FERNANDO","133":"PEPITO PEREZ","134":"RAMIREZ VARGAS MARCELA PAOLA","135":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","136":"TORO CISNEROS GARY JOSE","137":"USECHE CALDERON JADID ESTIVEN","138":"VASQUEZ NIETO CAMILO ANDRES","139":"JHONY CASTRO","140":"BERNAL JUAN DAVID","141":"XXX7","142":"XXX8","143":"XXX9","144":"BARON HERNANDEZ HAROLD ANTONIO","145":"CASTELLANOS CARVAJAL DEYVITH FABIAN","146":"AROCA TORRES JULIAN EDUARDO","147":"BERMUDEZ PARRA JENNIFER XIOMARA","148":"BERNAL BAQUERO JAMES RICARDO","149":"BURGOS ORTIZ JOSE HORACIO","150":"CANTOR PORRAS JUAN FERNEY","151":"CAPERA CAPERA JOSE GABRIEL","152":"CARDENAS LOTERO RICARDO ANDR\u00c9S","153":"RENDON OSPINA NELSON LEANDRO","154":"SARMIENTO URBINA MOISES DANIEL","155":"VELASCO VELASCO SEBASTI\u00c1N DAVID","156":"DELGADO DELGADO JOHAN DARIO","157":"FLOREZ SAUCESO KENIS ALBERTO","158":"CARDONA GARCIA OSCAR JAVIER","159":"CARVAJAL GARC\u00cdA HOVER MARCK","160":"CEPEDA PIRAQUIVE JUAN DAVID","161":"FAJARDO SAENZ OSCAR FERNANDO","162":"FLOREZ ESPITIA RONY ALBERTO","163":"GARCIA CUERVO EDWIN JAVIER","164":"GONZALEZ OCHOA JUAN CARLOS","165":"XXX1","166":"XXX2","167":"XXX3","168":"FONSECA RAY RICARDO","169":"GOMEZ BETANCUR JAIDER ANDRES","170":"GRANADA PATI\u00d1O CARLOS MARINO","171":"GRASS PLATA MIGUEL SNEIDER","172":"MANZANO CALVO JUAN SEBASTIAN","173":"MENDOZA GOITA MARIANSEL ZENAYDA","174":"MURILLO ARAQUE JAIVER GEOVANY","175":"NI\u00d1O ARENAS HECTOR GONZALO","176":"RAMIREZ CHAVERRA JHON EDISON","177":"XXX4","178":"XXX5","179":"XXX6","180":"RODRIGUEZ MOSQUERA LUIS FERNANDO","181":"PEPITO PEREZ","182":"RAMIREZ VARGAS MARCELA PAOLA","183":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","184":"TORO CISNEROS GARY JOSE","185":"USECHE CALDERON JADID ESTIVEN","186":"VASQUEZ NIETO CAMILO ANDRES","187":"JHONY CASTRO","188":"BERNAL JUAN DAVID","189":"XXX7","190":"XXX8","191":"XXX9","192":"BARON HERNANDEZ HAROLD ANTONIO","193":"CASTELLANOS CARVAJAL DEYVITH FABIAN","194":"AROCA TORRES JULIAN EDUARDO","195":"BERMUDEZ PARRA JENNIFER XIOMARA","196":"BERNAL BAQUERO JAMES RICARDO","197":"BURGOS ORTIZ JOSE HORACIO","198":"CANTOR PORRAS JUAN FERNEY","199":"CAPERA CAPERA JOSE GABRIEL","200":"CARDENAS LOTERO RICARDO ANDR\u00c9S","201":"RENDON OSPINA NELSON LEANDRO","202":"SARMIENTO URBINA MOISES DANIEL","203":"VELASCO VELASCO SEBASTI\u00c1N DAVID","204":"DELGADO DELGADO JOHAN DARIO","205":"FLOREZ SAUCESO KENIS ALBERTO","206":"CARDONA GARCIA OSCAR JAVIER","207":"CARVAJAL GARC\u00cdA HOVER MARCK","208":"CEPEDA PIRAQUIVE JUAN DAVID","209":"FAJARDO SAENZ OSCAR FERNANDO","210":"FLOREZ ESPITIA RONY ALBERTO","211":"GARCIA CUERVO EDWIN JAVIER","212":"GONZALEZ OCHOA JUAN CARLOS","213":"XXX1","214":"XXX2","215":"XXX3","216":"FONSECA RAY RICARDO","217":"GOMEZ BETANCUR JAIDER ANDRES","218":"GRANADA PATI\u00d1O CARLOS MARINO","219":"GRASS PLATA MIGUEL SNEIDER","220":"MANZANO CALVO JUAN SEBASTIAN","221":"MENDOZA GOITA MARIANSEL ZENAYDA","222":"MURILLO ARAQUE JAIVER GEOVANY","223":"NI\u00d1O ARENAS HECTOR GONZALO","224":"RAMIREZ CHAVERRA JHON EDISON","225":"XXX4","226":"XXX5","227":"XXX6","228":"RODRIGUEZ MOSQUERA LUIS FERNANDO","229":"PEPITO PEREZ","230":"RAMIREZ VARGAS MARCELA PAOLA","231":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","232":"TORO CISNEROS GARY JOSE","233":"USECHE CALDERON JADID ESTIVEN","234":"VASQUEZ NIETO CAMILO ANDRES","235":"JHONY CASTRO","236":"BERNAL JUAN DAVID","237":"XXX7","238":"XXX8","239":"XXX9","240":"BARON HERNANDEZ HAROLD ANTONIO","241":"CASTELLANOS CARVAJAL DEYVITH FABIAN","242":"AROCA TORRES JULIAN EDUARDO","243":"BERMUDEZ PARRA JENNIFER XIOMARA","244":"BERNAL BAQUERO JAMES RICARDO","245":"BURGOS ORTIZ JOSE HORACIO","246":"CANTOR PORRAS JUAN FERNEY","247":"CAPERA CAPERA JOSE GABRIEL","248":"CARDENAS LOTERO RICARDO ANDR\u00c9S","249":"RENDON OSPINA NELSON LEANDRO","250":"SARMIENTO URBINA MOISES DANIEL","251":"VELASCO VELASCO SEBASTI\u00c1N DAVID","252":"DELGADO DELGADO JOHAN DARIO","253":"FLOREZ SAUCESO KENIS ALBERTO","254":"CARDONA GARCIA OSCAR JAVIER","255":"CARVAJAL GARC\u00cdA HOVER MARCK","256":"CEPEDA PIRAQUIVE JUAN DAVID","257":"FAJARDO SAENZ OSCAR FERNANDO","258":"FLOREZ ESPITIA RONY ALBERTO","259":"GARCIA CUERVO EDWIN JAVIER","260":"GONZALEZ OCHOA JUAN CARLOS","261":"XXX1","262":"XXX2","263":"XXX3","264":"FONSECA RAY RICARDO","265":"GOMEZ BETANCUR JAIDER ANDRES","266":"GRANADA PATI\u00d1O CARLOS MARINO","267":"GR</t>
   </si>
 </sst>
 </file>
@@ -372,7 +381,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -400,13 +409,30 @@
         <v>2026</v>
       </c>
       <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" t="s">
         <v>6</v>
       </c>
-      <c r="D2" t="s">
+      <c r="B3">
+        <v>2026</v>
+      </c>
+      <c r="C3" t="s">
         <v>7</v>
       </c>
-      <c r="E2" t="s">
-        <v>8</v>
+      <c r="D3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automatizada: historico_mallas.xlsx [2026-04-24 17:56]
</commit_message>
<xml_diff>
--- a/historico_mallas.xlsx
+++ b/historico_mallas.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="14">
   <si>
     <t>Mes</t>
   </si>
@@ -37,6 +37,9 @@
     <t>Mayo</t>
   </si>
   <si>
+    <t>Junio</t>
+  </si>
+  <si>
     <t>Técnica</t>
   </si>
   <si>
@@ -44,6 +47,9 @@
   </si>
   <si>
     <t>24/04/2026 17:55</t>
+  </si>
+  <si>
+    <t>24/04/2026 17:56</t>
   </si>
   <si>
     <t>{"Grupo":{"0":"GRUPO 1","1":"GRUPO 1","2":"GRUPO 1","3":"GRUPO 1","4":"GRUPO 1","5":"GRUPO 1","6":"GRUPO 1","7":"GRUPO 1","8":"GRUPO 1","9":"GRUPO 1","10":"GRUPO 1","11":"GRUPO 1","12":"GRUPO 2","13":"GRUPO 2","14":"GRUPO 2","15":"GRUPO 2","16":"GRUPO 2","17":"GRUPO 2","18":"GRUPO 2","19":"GRUPO 2","20":"GRUPO 2","21":"GRUPO 2","22":"GRUPO 2","23":"GRUPO 2","24":"GRUPO 3","25":"GRUPO 3","26":"GRUPO 3","27":"GRUPO 3","28":"GRUPO 3","29":"GRUPO 3","30":"GRUPO 3","31":"GRUPO 3","32":"GRUPO 3","33":"GRUPO 3","34":"GRUPO 3","35":"GRUPO 3","36":"GRUPO 4","37":"GRUPO 4","38":"GRUPO 4","39":"GRUPO 4","40":"GRUPO 4","41":"GRUPO 4","42":"GRUPO 4","43":"GRUPO 4","44":"GRUPO 4","45":"GRUPO 4","46":"GRUPO 4","47":"GRUPO 4","48":"GRUPO 1","49":"GRUPO 1","50":"GRUPO 1","51":"GRUPO 1","52":"GRUPO 1","53":"GRUPO 1","54":"GRUPO 1","55":"GRUPO 1","56":"GRUPO 1","57":"GRUPO 1","58":"GRUPO 1","59":"GRUPO 1","60":"GRUPO 2","61":"GRUPO 2","62":"GRUPO 2","63":"GRUPO 2","64":"GRUPO 2","65":"GRUPO 2","66":"GRUPO 2","67":"GRUPO 2","68":"GRUPO 2","69":"GRUPO 2","70":"GRUPO 2","71":"GRUPO 2","72":"GRUPO 3","73":"GRUPO 3","74":"GRUPO 3","75":"GRUPO 3","76":"GRUPO 3","77":"GRUPO 3","78":"GRUPO 3","79":"GRUPO 3","80":"GRUPO 3","81":"GRUPO 3","82":"GRUPO 3","83":"GRUPO 3","84":"GRUPO 4","85":"GRUPO 4","86":"GRUPO 4","87":"GRUPO 4","88":"GRUPO 4","89":"GRUPO 4","90":"GRUPO 4","91":"GRUPO 4","92":"GRUPO 4","93":"GRUPO 4","94":"GRUPO 4","95":"GRUPO 4","96":"GRUPO 1","97":"GRUPO 1","98":"GRUPO 1","99":"GRUPO 1","100":"GRUPO 1","101":"GRUPO 1","102":"GRUPO 1","103":"GRUPO 1","104":"GRUPO 1","105":"GRUPO 1","106":"GRUPO 1","107":"GRUPO 1","108":"GRUPO 2","109":"GRUPO 2","110":"GRUPO 2","111":"GRUPO 2","112":"GRUPO 2","113":"GRUPO 2","114":"GRUPO 2","115":"GRUPO 2","116":"GRUPO 2","117":"GRUPO 2","118":"GRUPO 2","119":"GRUPO 2","120":"GRUPO 3","121":"GRUPO 3","122":"GRUPO 3","123":"GRUPO 3","124":"GRUPO 3","125":"GRUPO 3","126":"GRUPO 3","127":"GRUPO 3","128":"GRUPO 3","129":"GRUPO 3","130":"GRUPO 3","131":"GRUPO 3","132":"GRUPO 4","133":"GRUPO 4","134":"GRUPO 4","135":"GRUPO 4","136":"GRUPO 4","137":"GRUPO 4","138":"GRUPO 4","139":"GRUPO 4","140":"GRUPO 4","141":"GRUPO 4","142":"GRUPO 4","143":"GRUPO 4","144":"GRUPO 1","145":"GRUPO 1","146":"GRUPO 1","147":"GRUPO 1","148":"GRUPO 1","149":"GRUPO 1","150":"GRUPO 1","151":"GRUPO 1","152":"GRUPO 1","153":"GRUPO 1","154":"GRUPO 1","155":"GRUPO 1","156":"GRUPO 2","157":"GRUPO 2","158":"GRUPO 2","159":"GRUPO 2","160":"GRUPO 2","161":"GRUPO 2","162":"GRUPO 2","163":"GRUPO 2","164":"GRUPO 2","165":"GRUPO 2","166":"GRUPO 2","167":"GRUPO 2","168":"GRUPO 3","169":"GRUPO 3","170":"GRUPO 3","171":"GRUPO 3","172":"GRUPO 3","173":"GRUPO 3","174":"GRUPO 3","175":"GRUPO 3","176":"GRUPO 3","177":"GRUPO 3","178":"GRUPO 3","179":"GRUPO 3","180":"GRUPO 4","181":"GRUPO 4","182":"GRUPO 4","183":"GRUPO 4","184":"GRUPO 4","185":"GRUPO 4","186":"GRUPO 4","187":"GRUPO 4","188":"GRUPO 4","189":"GRUPO 4","190":"GRUPO 4","191":"GRUPO 4","192":"GRUPO 1","193":"GRUPO 1","194":"GRUPO 1","195":"GRUPO 1","196":"GRUPO 1","197":"GRUPO 1","198":"GRUPO 1","199":"GRUPO 1","200":"GRUPO 1","201":"GRUPO 1","202":"GRUPO 1","203":"GRUPO 1","204":"GRUPO 2","205":"GRUPO 2","206":"GRUPO 2","207":"GRUPO 2","208":"GRUPO 2","209":"GRUPO 2","210":"GRUPO 2","211":"GRUPO 2","212":"GRUPO 2","213":"GRUPO 2","214":"GRUPO 2","215":"GRUPO 2","216":"GRUPO 3","217":"GRUPO 3","218":"GRUPO 3","219":"GRUPO 3","220":"GRUPO 3","221":"GRUPO 3","222":"GRUPO 3","223":"GRUPO 3","224":"GRUPO 3","225":"GRUPO 3","226":"GRUPO 3","227":"GRUPO 3","228":"GRUPO 4","229":"GRUPO 4","230":"GRUPO 4","231":"GRUPO 4","232":"GRUPO 4","233":"GRUPO 4","234":"GRUPO 4","235":"GRUPO 4","236":"GRUPO 4","237":"GRUPO 4","238":"GRUPO 4","239":"GRUPO 4","240":"GRUPO 1","241":"GRUPO 1","242":"GRUPO 1","243":"GRUPO 1","244":"GRUPO 1","245":"GRUPO 1","246":"GRUPO 1","247":"GRUPO 1","248":"GRUPO 1","249":"GRUPO 1","250":"GRUPO 1","251":"GRUPO 1","252":"GRUPO 2","253":"GRUPO 2","254":"GRUPO 2","255":"GRUPO 2","256":"GRUPO 2","257":"GRUPO 2","258":"GRUPO 2","259":"GRUPO 2","260":"GRUPO 2","261":"GRUPO 2","262":"GRUPO 2","263":"GRUPO 2","264":"GRUPO 3","265":"GRUPO 3","266":"GRUPO 3","267":"GRUPO 3","268":"GRUPO 3","269":"GRUPO 3","270":"GRUPO 3","271":"GRUPO 3","272":"GRUPO 3","273":"GRUPO 3","274":"GRUPO 3","275":"GRUPO 3","276":"GRUPO 4","277":"GRUPO 4","278":"GRUPO 4","279":"GRUPO 4","280":"GRUPO 4","281":"GRUPO 4","282":"GRUPO 4","283":"GRUPO 4","284":"GRUPO 4","285":"GRUPO 4","286":"GRUPO 4","287":"GRUPO 4","288":"GRUPO 1","289":"GRUPO 1","290":"GRUPO 1","291":"GRUPO 1","292":"GRUPO 1","293":"GRUPO 1","294":"GRUPO 1","295":"GRUPO 1","296":"GRUPO 1","297":"GRUPO 1","298":"GRUPO 1","299":"GRUPO 1","300":"GRUPO 2","301":"GRUPO 2","302":"GRUPO 2","303":"GRUPO 2","304":"GRUPO 2","305":"GRUPO 2","306":"GRUPO 2","307":"GRUPO 2","308":"GRUPO 2","309":"GRUPO 2","310":"GRUPO 2","311":"GRUPO 2","312":"GRUPO 3","313":"GRUPO 3","314":"GRUPO 3","315":"GRUPO 3","316":"GRUPO 3","317":"GRUPO 3","318":"GRUPO 3","319":"GRUPO 3","320":"GRUPO 3","321":"GRUPO 3","322":"GRUPO 3","323":"GRUPO 3","324":"GRUPO 4","325":"GRUPO 4","326":"GRUPO 4","327":"GRUPO 4","328":"GRUPO 4","329":"GRUPO 4","330":"GRUPO 4","331":"GRUPO 4","332":"GRUPO 4","333":"GRUPO 4","334":"GRUPO 4","335":"GRUPO 4","336":"GRUPO 1","337":"GRUPO 1","338":"GRUPO 1","339":"GRUPO 1","340":"GRUPO 1","341":"GRUPO 1","342":"GRUPO 1","343":"GRUPO 1","344":"GRUPO 1","345":"GRUPO 1","346":"GRUPO 1","347":"GRUPO 1","348":"GRUPO 2","349":"GRUPO 2","350":"GRUPO 2","351":"GRUPO 2","352":"GRUPO 2","353":"GRUPO 2","354":"GRUPO 2","355":"GRUPO 2","356":"GRUPO 2","357":"GRUPO 2","358":"GRUPO 2","359":"GRUPO 2","360":"GRUPO 3","361":"GRUPO 3","362":"GRUPO 3","363":"GRUPO 3","364":"GRUPO 3","365":"GRUPO 3","366":"GRUPO 3","367":"GRUPO 3","368":"GRUPO 3","369":"GRUPO 3","370":"GRUPO 3","371":"GRUPO 3","372":"GRUPO 4","373":"GRUPO 4","374":"GRUPO 4","375":"GRUPO 4","376":"GRUPO 4","377":"GRUPO 4","378":"GRUPO 4","379":"GRUPO 4","380":"GRUPO 4","381":"GRUPO 4","382":"GRUPO 4","383":"GRUPO 4","384":"GRUPO 1","385":"GRUPO 1","386":"GRUPO 1","387":"GRUPO 1","388":"GRUPO 1","389":"GRUPO 1","390":"GRUPO 1","391":"GRUPO 1","392":"GRUPO 1","393":"GRUPO 1","394":"GRUPO 1","395":"GRUPO 1","396":"GRUPO 2","397":"GRUPO 2","398":"GRUPO 2","399":"GRUPO 2","400":"GRUPO 2","401":"GRUPO 2","402":"GRUPO 2","403":"GRUPO 2","404":"GRUPO 2","405":"GRUPO 2","406":"GRUPO 2","407":"GRUPO 2","408":"GRUPO 3","409":"GRUPO 3","410":"GRUPO 3","411":"GRUPO 3","412":"GRUPO 3","413":"GRUPO 3","414":"GRUPO 3","415":"GRUPO 3","416":"GRUPO 3","417":"GRUPO 3","418":"GRUPO 3","419":"GRUPO 3","420":"GRUPO 4","421":"GRUPO 4","422":"GRUPO 4","423":"GRUPO 4","424":"GRUPO 4","425":"GRUPO 4","426":"GRUPO 4","427":"GRUPO 4","428":"GRUPO 4","429":"GRUPO 4","430":"GRUPO 4","431":"GRUPO 4","432":"GRUPO 1","433":"GRUPO 1","434":"GRUPO 1","435":"GRUPO 1","436":"GRUPO 1","437":"GRUPO 1","438":"GRUPO 1","439":"GRUPO 1","440":"GRUPO 1","441":"GRUPO 1","442":"GRUPO 1","443":"GRUPO 1","444":"GRUPO 2","445":"GRUPO 2","446":"GRUPO 2","447":"GRUPO 2","448":"GRUPO 2","449":"GRUPO 2","450":"GRUPO 2","451":"GRUPO 2","452":"GRUPO 2","453":"GRUPO 2","454":"GRUPO 2","455":"GRUPO 2","456":"GRUPO 3","457":"GRUPO 3","458":"GRUPO 3","459":"GRUPO 3","460":"GRUPO 3","461":"GRUPO 3","462":"GRUPO 3","463":"GRUPO 3","464":"GRUPO 3","465":"GRUPO 3","466":"GRUPO 3","467":"GRUPO 3","468":"GRUPO 4","469":"GRUPO 4","470":"GRUPO 4","471":"GRUPO 4","472":"GRUPO 4","473":"GRUPO 4","474":"GRUPO 4","475":"GRUPO 4","476":"GRUPO 4","477":"GRUPO 4","478":"GRUPO 4","479":"GRUPO 4","480":"GRUPO 1","481":"GRUPO 1","482":"GRUPO 1","483":"GRUPO 1","484":"GRUPO 1","485":"GRUPO 1","486":"GRUPO 1","487":"GRUPO 1","488":"GRUPO 1","489":"GRUPO 1","490":"GRUPO 1","491":"GRUPO 1","492":"GRUPO 2","493":"GRUPO 2","494":"GRUPO 2","495":"GRUPO 2","496":"GRUPO 2","497":"GRUPO 2","498":"GRUPO 2","499":"GRUPO 2","500":"GRUPO 2","501":"GRUPO 2","502":"GRUPO 2","503":"GRUPO 2","504":"GRUPO 3","505":"GRUPO 3","506":"GRUPO 3","507":"GRUPO 3","508":"GRUPO 3","509":"GRUPO 3","510":"GRUPO 3","511":"GRUPO 3","512":"GRUPO 3","513":"GRUPO 3","514":"GRUPO 3","515":"GRUPO 3","516":"GRUPO 4","517":"GRUPO 4","518":"GRUPO 4","519":"GRUPO 4","520":"GRUPO 4","521":"GRUPO 4","522":"GRUPO 4","523":"GRUPO 4","524":"GRUPO 4","525":"GRUPO 4","526":"GRUPO 4","527":"GRUPO 4","528":"GRUPO 1","529":"GRUPO 1","530":"GRUPO 1","531":"GRUPO 1","532":"GRUPO 1","533":"GRUPO 1","534":"GRUPO 1","535":"GRUPO 1","536":"GRUPO 1","537":"GRUPO 1","538":"GRUPO 1","539":"GRUPO 1","540":"GRUPO 2","541":"GRUPO 2","542":"GRUPO 2","543":"GRUPO 2","544":"GRUPO 2","545":"GRUPO 2","546":"GRUPO 2","547":"GRUPO 2","548":"GRUPO 2","549":"GRUPO 2","550":"GRUPO 2","551":"GRUPO 2","552":"GRUPO 3","553":"GRUPO 3","554":"GRUPO 3","555":"GRUPO 3","556":"GRUPO 3","557":"GRUPO 3","558":"GRUPO 3","559":"GRUPO 3","560":"GRUPO 3","561":"GRUPO 3","562":"GRUPO 3","563":"GRUPO 3","564":"GRUPO 4","565":"GRUPO 4","566":"GRUPO 4","567":"GRUPO 4","568":"GRUPO 4","569":"GRUPO 4","570":"GRUPO 4","571":"GRUPO 4","572":"GRUPO 4","573":"GRUPO 4","574":"GRUPO 4","575":"GRUPO 4","576":"GRUPO 1","577":"GRUPO 1","578":"GRUPO 1","579":"GRUPO 1","580":"GRUPO 1","581":"GRUPO 1","582":"GRUPO 1","583":"GRUPO 1","584":"GRUPO 1","585":"GRUPO 1","586":"GRUPO 1","587":"GRUPO 1","588":"GRUPO 2","589":"GRUPO 2","590":"GRUPO 2","591":"GRUPO 2","592":"GRUPO 2","593":"GRUPO 2","594":"GRUPO 2","595":"GRUPO 2","596":"GRUPO 2","597":"GRUPO 2","598":"GRUPO 2","599":"GRUPO 2","600":"GRUPO 3","601":"GRUPO 3","602":"GRUPO 3","603":"GRUPO 3","604":"GRUPO 3","605":"GRUPO 3","606":"GRUPO 3","607":"GRUPO 3","608":"GRUPO 3","609":"GRUPO 3","610":"GRUPO 3","611":"GRUPO 3","612":"GRUPO 4","613":"GRUPO 4","614":"GRUPO 4","615":"GRUPO 4","616":"GRUPO 4","617":"GRUPO 4","618":"GRUPO 4","619":"GRUPO 4","620":"GRUPO 4","621":"GRUPO 4","622":"GRUPO 4","623":"GRUPO 4","624":"GRUPO 1","625":"GRUPO 1","626":"GRUPO 1","627":"GRUPO 1","628":"GRUPO 1","629":"GRUPO 1","630":"GRUPO 1","631":"GRUPO 1","632":"GRUPO 1","633":"GRUPO 1","634":"GRUPO 1","635":"GRUPO 1","636":"GRUPO 2","637":"GRUPO 2","638":"GRUPO 2","639":"GRUPO 2","640":"GRUPO 2","641":"GRUPO 2","642":"GRUPO 2","643":"GRUPO 2","644":"GRUPO 2","645":"GRUPO 2","646":"GRUPO 2","647":"GRUPO 2","648":"GRUPO 3","649":"GRUPO 3","650":"GRUPO 3","651":"GRUPO 3","652":"GRUPO 3","653":"GRUPO 3","654":"GRUPO 3","655":"GRUPO 3","656":"GRUPO 3","657":"GRUPO 3","658":"GRUPO 3","659":"GRUPO 3","660":"GRUPO 4","661":"GRUPO 4","662":"GRUPO 4","663":"GRUPO 4","664":"GRUPO 4","665":"GRUPO 4","666":"GRUPO 4","667":"GRUPO 4","668":"GRUPO 4","669":"GRUPO 4","670":"GRUPO 4","671":"GRUPO 4","672":"GRUPO 1","673":"GRUPO 1","674":"GRUPO 1","675":"GRUPO 1","676":"GRUPO 1","677":"GRUPO 1","678":"GRUPO 1","679":"GRUPO 1","680":"GRUPO 1","681":"GRUPO 1","682":"GRUPO 1","683":"GRUPO 1","684":"GRUPO 2","685":"GRUPO 2","686":"GRUPO 2","687":"GRUPO 2","688":"GRUPO 2","689":"GRUPO 2","690":"GRUPO 2","691":"GRUPO 2","692":"GRUPO 2","693":"GRUPO 2","694":"GRUPO 2","695":"GRUPO 2","696":"GRUPO 3","697":"GRUPO 3","698":"GRUPO 3","699":"GRUPO 3","700":"GRUPO 3","701":"GRUPO 3","702":"GRUPO 3","703":"GRUPO 3","704":"GRUPO 3","705":"GRUPO 3","706":"GRUPO 3","707":"GRUPO 3","708":"GRUPO 4","709":"GRUPO 4","710":"GRUPO 4","711":"GRUPO 4","712":"GRUPO 4","713":"GRUPO 4","714":"GRUPO 4","715":"GRUPO 4","716":"GRUPO 4","717":"GRUPO 4","718":"GRUPO 4","719":"GRUPO 4","720":"GRUPO 1","721":"GRUPO 1","722":"GRUPO 1","723":"GRUPO 1","724":"GRUPO 1","725":"GRUPO 1","726":"GRUPO 1","727":"GRUPO 1","728":"GRUPO 1","729":"GRUPO 1","730":"GRUPO 1","731":"GRUPO 1","732":"GRUPO 2","733":"GRUPO 2","734":"GRUPO 2","735":"GRUPO 2","736":"GRUPO 2","737":"GRUPO 2","738":"GRUPO 2","739":"GRUPO 2","740":"GRUPO 2","741":"GRUPO 2","742":"GRUPO 2","743":"GRUPO 2","744":"GRUPO 3","745":"GRUPO 3","746":"GRUPO 3","747":"GRUPO 3","748":"GRUPO 3","749":"GRUPO 3","750":"GRUPO 3","751":"GRUPO 3","752":"GRUPO 3","753":"GRUPO 3","754":"GRUPO 3","755":"GRUPO 3","756":"GRUPO 4","757":"GRUPO 4","758":"GRUPO 4","759":"GRUPO 4","760":"GRUPO 4","761":"GRUPO 4","762":"GRUPO 4","763":"GRUPO 4","764":"GRUPO 4","765":"GRUPO 4","766":"GRUPO 4","767":"GRUPO 4","768":"GRUPO 1","769":"GRUPO 1","770":"GRUPO 1","771":"GRUPO 1","772":"GRUPO 1","773":"GRUPO 1","774":"GRUPO 1","775":"GRUPO 1","776":"GRUPO 1","777":"GRUPO 1","778":"GRUPO 1","779":"GRUPO 1","780":"GRUPO 2","781":"GRUPO 2","782":"GRUPO 2","783":"GRUPO 2","784":"GRUPO 2","785":"GRUPO 2","786":"GRUPO 2","787":"GRUPO 2","788":"GRUPO 2","789":"GRUPO 2","790":"GRUPO 2","791":"GRUPO 2","792":"GRUPO 3","793":"GRUPO 3","794":"GRUPO 3","795":"GRUPO 3","796":"GRUPO 3","797":"GRUPO 3","798":"GRUPO 3","799":"GRUPO 3","800":"GRUPO 3","801":"GRUPO 3","802":"GRUPO 3","803":"GRUPO 3","804":"GRUPO 4","805":"GRUPO 4","806":"GRUPO 4","807":"GRUPO 4","808":"GRUPO 4","809":"GRUPO 4","810":"GRUPO 4","811":"GRUPO 4","812":"GRUPO 4","813":"GRUPO 4","814":"GRUPO 4","815":"GRUPO 4","816":"GRUPO 1","817":"GRUPO 1","818":"GRUPO 1","819":"GRUPO 1","820":"GRUPO 1","821":"GRUPO 1","822":"GRUPO 1","823":"GRUPO 1","824":"GRUPO 1","825":"GRUPO 1","826":"GRUPO 1","827":"GRUPO 1","828":"GRUPO 2","829":"GRUPO 2","830":"GRUPO 2","831":"GRUPO 2","832":"GRUPO 2","833":"GRUPO 2","834":"GRUPO 2","835":"GRUPO 2","836":"GRUPO 2","837":"GRUPO 2","838":"GRUPO 2","839":"GRUPO 2","840":"GRUPO 3","841":"GRUPO 3","842":"GRUPO 3","843":"GRUPO 3","844":"GRUPO 3","845":"GRUPO 3","846":"GRUPO 3","847":"GRUPO 3","848":"GRUPO 3","849":"GRUPO 3","850":"GRUPO 3","851":"GRUPO 3","852":"GRUPO 4","853":"GRUPO 4","854":"GRUPO 4","855":"GRUPO 4","856":"GRUPO 4","857":"GRUPO 4","858":"GRUPO 4","859":"GRUPO 4","860":"GRUPO 4","861":"GRUPO 4","862":"GRUPO 4","863":"GRUPO 4","864":"GRUPO 1","865":"GRUPO 1","866":"GRUPO 1","867":"GRUPO 1","868":"GRUPO 1","869":"GRUPO 1","870":"GRUPO 1","871":"GRUPO 1","872":"GRUPO 1","873":"GRUPO 1","874":"GRUPO 1","875":"GRUPO 1","876":"GRUPO 2","877":"GRUPO 2","878":"GRUPO 2","879":"GRUPO 2","880":"GRUPO 2","881":"GRUPO 2","882":"GRUPO 2","883":"GRUPO 2","884":"GRUPO 2","885":"GRUPO 2","886":"GRUPO 2","887":"GRUPO 2","888":"GRUPO 3","889":"GRUPO 3","890":"GRUPO 3","891":"GRUPO 3","892":"GRUPO 3","893":"GRUPO 3","894":"GRUPO 3","895":"GRUPO 3","896":"GRUPO 3","897":"GRUPO 3","898":"GRUPO 3","899":"GRUPO 3","900":"GRUPO 4","901":"GRUPO 4","902":"GRUPO 4","903":"GRUPO 4","904":"GRUPO 4","905":"GRUPO 4","906":"GRUPO 4","907":"GRUPO 4","908":"GRUPO 4","909":"GRUPO 4","910":"GRUPO 4","911":"GRUPO 4","912":"GRUPO 1","913":"GRUPO 1","914":"GRUPO 1","915":"GRUPO 1","916":"GRUPO 1","917":"GRUPO 1","918":"GRUPO 1","919":"GRUPO 1","920":"GRUPO 1","921":"GRUPO 1","922":"GRUPO 1","923":"GRUPO 1","924":"GRUPO 2","925":"GRUPO 2","926":"GRUPO 2","927":"GRUPO 2","928":"GRUPO 2","929":"GRUPO 2","930":"GRUPO 2","931":"GRUPO 2","932":"GRUPO 2","933":"GRUPO 2","934":"GRUPO 2","935":"GRUPO 2","936":"GRUPO 3","937":"GRUPO 3","938":"GRUPO 3","939":"GRUPO 3","940":"GRUPO 3","941":"GRUPO 3","942":"GRUPO 3","943":"GRUPO 3","944":"GRUPO 3","945":"GRUPO 3","946":"GRUPO 3","947":"GRUPO 3","948":"GRUPO 4","949":"GRUPO 4","950":"GRUPO 4","951":"GRUPO 4","952":"GRUPO 4","953":"GRUPO 4","954":"GRUPO 4","955":"GRUPO 4","956":"GRUPO 4","957":"GRUPO 4","958":"GRUPO 4","959":"GRUPO 4","960":"GRUPO 1","961":"GRUPO 1","962":"GRUPO 1","963":"GRUPO 1","964":"GRUPO 1","965":"GRUPO 1","966":"GRUPO 1","967":"GRUPO 1","968":"GRUPO 1","969":"GRUPO 1","970":"GRUPO 1","971":"GRUPO 1","972":"GRUPO 2","973":"GRUPO 2","974":"GRUPO 2","975":"GRUPO 2","976":"GRUPO 2","977":"GRUPO 2","978":"GRUPO 2","979":"GRUPO 2","980":"GRUPO 2","981":"GRUPO 2","982":"GRUPO 2","983":"GRUPO 2","984":"GRUPO 3","985":"GRUPO 3","986":"GRUPO 3","987":"GRUPO 3","988":"GRUPO 3","989":"GRUPO 3","990":"GRUPO 3","991":"GRUPO 3","992":"GRUPO 3","993":"GRUPO 3","994":"GRUPO 3","995":"GRUPO 3","996":"GRUPO 4","997":"GRUPO 4","998":"GRUPO 4","999":"GRUPO 4","1000":"GRUPO 4","1001":"GRUPO 4","1002":"GRUPO 4","1003":"GRUPO 4","1004":"GRUPO 4","1005":"GRUPO 4","1006":"GRUPO 4","1007":"GRUPO 4","1008":"GRUPO 1","1009":"GRUPO 1","1010":"GRUPO 1","1011":"GRUPO 1","1012":"GRUPO 1","1013":"GRUPO 1","1014":"GRUPO 1","1015":"GRUPO 1","1016":"GRUPO 1","1017":"GRUPO 1","1018":"GRUPO 1","1019":"GRUPO 1","1020":"GRUPO 2","1021":"GRUPO 2","1022":"GRUPO 2","1023":"GRUPO 2","1024":"GRUPO 2","1025":"GRUPO 2","1026":"GRUPO 2","1027":"GRUPO 2","1028":"GRUPO 2","1029":"GRUPO 2","1030":"GRUPO 2","1031":"GRUPO 2","1032":"GRUPO 3","1033":"GRUPO 3","1034":"GRUPO 3","1035":"GRUPO 3","1036":"GRUPO 3","1037":"GRUPO 3","1038":"GRUPO 3","1039":"GRUPO 3","1040":"GRUPO 3","1041":"GRUPO 3","1042":"GRUPO 3","1043":"GRUPO 3","1044":"GRUPO 4","1045":"GRUPO 4","1046":"GRUPO 4","1047":"GRUPO 4","1048":"GRUPO 4","1049":"GRUPO 4","1050":"GRUPO 4","1051":"GRUPO 4","1052":"GRUPO 4","1053":"GRUPO 4","1054":"GRUPO 4","1055":"GRUPO 4","1056":"GRUPO 1","1057":"GRUPO 1","1058":"GRUPO 1","1059":"GRUPO 1","1060":"GRUPO 1","1061":"GRUPO 1","1062":"GRUPO 1","1063":"GRUPO 1","1064":"GRUPO 1","1065":"GRUPO 1","1066":"GRUPO 1","1067":"GRUPO 1","1068":"GRUPO 2","1069":"GRUPO 2","1070":"GRUPO 2","1071":"GRUPO 2","1072":"GRUPO 2","1073":"GRUPO 2","1074":"GRUPO 2","1075":"GRUPO 2","1076":"GRUPO 2","1077":"GRUPO 2","1078":"GRUPO 2","1079":"GRUPO 2","1080":"GRUPO 3","1081":"GRUPO 3","1082":"GRUPO 3","1083":"GRUPO 3","1084":"GRUPO 3","1085":"GRUPO 3","1086":"GRUPO 3","1087":"GRUPO 3","1088":"GRUPO 3","1089":"GRUPO 3","1090":"GRUPO 3","1091":"GRUPO 3","1092":"GRUPO 4","1093":"GRUPO 4","1094":"GRUPO 4","1095":"GRUPO 4","1096":"GRUPO 4","1097":"GRUPO 4","1098":"GRUPO 4","1099":"GRUPO 4","1100":"GRUPO 4","1101":"GRUPO 4","1102":"GRUPO 4","1103":"GRUPO 4","1104":"GRUPO 1","1105":"GRUPO 1","1106":"GRUPO 1","1107":"GRUPO 1","1108":"GRUPO 1","1109":"GRUPO 1","1110":"GRUPO 1","1111":"GRUPO 1","1112":"GRUPO 1","1113":"GRUPO 1","1114":"GRUPO 1","1115":"GRUPO 1","1116":"GRUPO 2","1117":"GRUPO 2","1118":"GRUPO 2","1119":"GRUPO 2","1120":"GRUPO 2","1121":"GRUPO 2","1122":"GRUPO 2","1123":"GRUPO 2","1124":"GRUPO 2","1125":"GRUPO 2","1126":"GRUPO 2","1127":"GRUPO 2","1128":"GRUPO 3","1129":"GRUPO 3","1130":"GRUPO 3","1131":"GRUPO 3","1132":"GRUPO 3","1133":"GRUPO 3","1134":"GRUPO 3","1135":"GRUPO 3","1136":"GRUPO 3","1137":"GRUPO 3","1138":"GRUPO 3","1139":"GRUPO 3","1140":"GRUPO 4","1141":"GRUPO 4","1142":"GRUPO 4","1143":"GRUPO 4","1144":"GRUPO 4","1145":"GRUPO 4","1146":"GRUPO 4","1147":"GRUPO 4","1148":"GRUPO 4","1149":"GRUPO 4","1150":"GRUPO 4","1151":"GRUPO 4","1152":"GRUPO 1","1153":"GRUPO 1","1154":"GRUPO 1","1155":"GRUPO 1","1156":"GRUPO 1","1157":"GRUPO 1","1158":"GRUPO 1","1159":"GRUPO 1","1160":"GRUPO 1","1161":"GRUPO 1","1162":"GRUPO 1","1163":"GRUPO 1","1164":"GRUPO 2","1165":"GRUPO 2","1166":"GRUPO 2","1167":"GRUPO 2","1168":"GRUPO 2","1169":"GRUPO 2","1170":"GRUPO 2","1171":"GRUPO 2","1172":"GRUPO 2","1173":"GRUPO 2","1174":"GRUPO 2","1175":"GRUPO 2","1176":"GRUPO 3","1177":"GRUPO 3","1178":"GRUPO 3","1179":"GRUPO 3","1180":"GRUPO 3","1181":"GRUPO 3","1182":"GRUPO 3","1183":"GRUPO 3","1184":"GRUPO 3","1185":"GRUPO 3","1186":"GRUPO 3","1187":"GRUPO 3","1188":"GRUPO 4","1189":"GRUPO 4","1190":"GRUPO 4","1191":"GRUPO 4","1192":"GRUPO 4","1193":"GRUPO 4","1194":"GRUPO 4","1195":"GRUPO 4","1196":"GRUPO 4","1197":"GRUPO 4","1198":"GRUPO 4","1199":"GRUPO 4","1200":"GRUPO 1","1201":"GRUPO 1","1202":"GRUPO 1","1203":"GRUPO 1","1204":"GRUPO 1","1205":"GRUPO 1","1206":"GRUPO 1","1207":"GRUPO 1","1208":"GRUPO 1","1209":"GRUPO 1","1210":"GRUPO 1","1211":"GRUPO 1","1212":"GRUPO 2","1213":"GRUPO 2","1214":"GRUPO 2","1215":"GRUPO 2","1216":"GRUPO 2","1217":"GRUPO 2","1218":"GRUPO 2","1219":"GRUPO 2","1220":"GRUPO 2","1221":"GRUPO 2","1222":"GRUPO 2","1223":"GRUPO 2","1224":"GRUPO 3","1225":"GRUPO 3","1226":"GRUPO 3","1227":"GRUPO 3","1228":"GRUPO 3","1229":"GRUPO 3","1230":"GRUPO 3","1231":"GRUPO 3","1232":"GRUPO 3","1233":"GRUPO 3","1234":"GRUPO 3","1235":"GRUPO 3","1236":"GRUPO 4","1237":"GRUPO 4","1238":"GRUPO 4","1239":"GRUPO 4","1240":"GRUPO 4","1241":"GRUPO 4","1242":"GRUPO 4","1243":"GRUPO 4","1244":"GRUPO 4","1245":"GRUPO 4","1246":"GRUPO 4","1247":"GRUPO 4","1248":"GRUPO 1","1249":"GRUPO 1","1250":"GRUPO 1","1251":"GRUPO 1","1252":"GRUPO 1","1253":"GRUPO 1","1254":"GRUPO 1","1255":"GRUPO 1","1256":"GRUPO 1","1257":"GRUPO 1","1258":"GRUPO 1","1259":"GRUPO 1","1260":"GRUPO 2","1261":"GRUPO 2","1262":"GRUPO 2","1263":"GRUPO 2","1264":"GRUPO 2","1265":"GRUPO 2","1266":"GRUPO 2","1267":"GRUPO 2","1268":"GRUPO 2","1269":"GRUPO 2","1270":"GRUPO 2","1271":"GRUPO 2","1272":"GRUPO 3","1273":"GRUPO 3","1274":"GRUPO 3","1275":"GRUPO 3","1276":"GRUPO 3","1277":"GRUPO 3","1278":"GRUPO 3","1279":"GRUPO 3","1280":"GRUPO 3","1281":"GRUPO 3","1282":"GRUPO 3","1283":"GRUPO 3","1284":"GRUPO 4","1285":"GRUPO 4","1286":"GRUPO 4","1287":"GRUPO 4","1288":"GRUPO 4","1289":"GRUPO 4","1290":"GRUPO 4","1291":"GRUPO 4","1292":"GRUPO 4","1293":"GRUPO 4","1294":"GRUPO 4","1295":"GRUPO 4","1296":"GRUPO 1","1297":"GRUPO 1","1298":"GRUPO 1","1299":"GRUPO 1","1300":"GRUPO 1","1301":"GRUPO 1","1302":"GRUPO 1","1303":"GRUPO 1","1304":"GRUPO 1","1305":"GRUPO 1","1306":"GRUPO 1","1307":"GRUPO 1","1308":"GRUPO 2","1309":"GRUPO 2","1310":"GRUPO 2","1311":"GRUPO 2","1312":"GRUPO 2","1313":"GRUPO 2","1314":"GRUPO 2","1315":"GRUPO 2","1316":"GRUPO 2","1317":"GRUPO 2","1318":"GRUPO 2","1319":"GRUPO 2","1320":"GRUPO 3","1321":"GRUPO 3","1322":"GRUPO 3","1323":"GRUPO 3","1324":"GRUPO 3","1325":"GRUPO 3","1326":"GRUPO 3","1327":"GRUPO 3","1328":"GRUPO 3","1329":"GRUPO 3","1330":"GRUPO 3","1331":"GRUPO 3","1332":"GRUPO 4","1333":"GRUPO 4","1334":"GRUPO 4","1335":"GRUPO 4","1336":"GRUPO 4","1337":"GRUPO 4","1338":"GRUPO 4","1339":"GRUPO 4","1340":"GRUPO 4","1341":"GRUPO 4","1342":"GRUPO 4","1343":"GRUPO 4","1344":"GRUPO 1","1345":"GRUPO 1","1346":"GRUPO 1","1347":"GRUPO 1","1348":"GRUPO 1","1349":"GRUPO 1","1350":"GRUPO 1","1351":"GRUPO 1","1352":"GRUPO 1","1353":"GRUPO 1","1354":"GRUPO 1","1355":"GRUPO 1","1356":"GRUPO 2","1357":"GRUPO 2","1358":"GRUPO 2","1359":"GRUPO 2","1360":"GRUPO 2","1361":"GRUPO 2","1362":"GRUPO 2","1363":"GRUPO 2","1364":"GRUPO 2","1365":"GRUPO 2","1366":"GRUPO 2","1367":"GRUPO 2","1368":"GRUPO 3","1369":"GRUPO 3","1370":"GRUPO 3","1371":"GRUPO 3","1372":"GRUPO 3","1373":"GRUPO 3","1374":"GRUPO 3","1375":"GRUPO 3","1376":"GRUPO 3","1377":"GRUPO 3","1378":"GRUPO 3","1379":"GRUPO 3","1380":"GRUPO 4","1381":"GRUPO 4","1382":"GRUPO 4","1383":"GRUPO 4","1384":"GRUPO 4","1385":"GRUPO 4","1386":"GRUPO 4","1387":"GRUPO 4","1388":"GRUPO 4","1389":"GRUPO 4","1390":"GRUPO 4","1391":"GRUPO 4","1392":"GRUPO 1","1393":"GRUPO 1","1394":"GRUPO 1","1395":"GRUPO 1","1396":"GRUPO 1","1397":"GRUPO 1","1398":"GRUPO 1","1399":"GRUPO 1","1400":"GRUPO 1","1401":"GRUPO 1","1402":"GRUPO 1","1403":"GRUPO 1","1404":"GRUPO 2","1405":"GRUPO 2","1406":"GRUPO 2","1407":"GRUPO 2","1408":"GRUPO 2","1409":"GRUPO 2","1410":"GRUPO 2","1411":"GRUPO 2","1412":"GRUPO 2","1413":"GRUPO 2","1414":"GRUPO 2","1415":"GRUPO 2","1416":"GRUPO 3","1417":"GRUPO 3","1418":"GRUPO 3","1419":"GRUPO 3","1420":"GRUPO 3","1421":"GRUPO 3","1422":"GRUPO 3","1423":"GRUPO 3","1424":"GRUPO 3","1425":"GRUPO 3","1426":"GRUPO 3","1427":"GRUPO 3","1428":"GRUPO 4","1429":"GRUPO 4","1430":"GRUPO 4","1431":"GRUPO 4","1432":"GRUPO 4","1433":"GRUPO 4","1434":"GRUPO 4","1435":"GRUPO 4","1436":"GRUPO 4","1437":"GRUPO 4","1438":"GRUPO 4","1439":"GRUPO 4"},"Empleado":{"0":"BARON HERNANDEZ HAROLD ANTONIO","1":"CASTELLANOS CARVAJAL DEYVITH FABIAN","2":"AROCA TORRES JULIAN EDUARDO","3":"BERMUDEZ PARRA JENNIFER XIOMARA","4":"BERNAL BAQUERO JAMES RICARDO","5":"BURGOS ORTIZ JOSE HORACIO","6":"CANTOR PORRAS JUAN FERNEY","7":"CAPERA CAPERA JOSE GABRIEL","8":"CARDENAS LOTERO RICARDO ANDR\u00c9S","9":"RENDON OSPINA NELSON LEANDRO","10":"SARMIENTO URBINA MOISES DANIEL","11":"VELASCO VELASCO SEBASTI\u00c1N DAVID","12":"DELGADO DELGADO JOHAN DARIO","13":"FLOREZ SAUCESO KENIS ALBERTO","14":"CARDONA GARCIA OSCAR JAVIER","15":"CARVAJAL GARC\u00cdA HOVER MARCK","16":"CEPEDA PIRAQUIVE JUAN DAVID","17":"FAJARDO SAENZ OSCAR FERNANDO","18":"FLOREZ ESPITIA RONY ALBERTO","19":"GARCIA CUERVO EDWIN JAVIER","20":"GONZALEZ OCHOA JUAN CARLOS","21":"XXX1","22":"XXX2","23":"XXX3","24":"FONSECA RAY RICARDO","25":"GOMEZ BETANCUR JAIDER ANDRES","26":"GRANADA PATI\u00d1O CARLOS MARINO","27":"GRASS PLATA MIGUEL SNEIDER","28":"MANZANO CALVO JUAN SEBASTIAN","29":"MENDOZA GOITA MARIANSEL ZENAYDA","30":"MURILLO ARAQUE JAIVER GEOVANY","31":"NI\u00d1O ARENAS HECTOR GONZALO","32":"RAMIREZ CHAVERRA JHON EDISON","33":"XXX4","34":"XXX5","35":"XXX6","36":"RODRIGUEZ MOSQUERA LUIS FERNANDO","37":"PEPITO PEREZ","38":"RAMIREZ VARGAS MARCELA PAOLA","39":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","40":"TORO CISNEROS GARY JOSE","41":"USECHE CALDERON JADID ESTIVEN","42":"VASQUEZ NIETO CAMILO ANDRES","43":"JHONY CASTRO","44":"BERNAL JUAN DAVID","45":"XXX7","46":"XXX8","47":"XXX9","48":"BARON HERNANDEZ HAROLD ANTONIO","49":"CASTELLANOS CARVAJAL DEYVITH FABIAN","50":"AROCA TORRES JULIAN EDUARDO","51":"BERMUDEZ PARRA JENNIFER XIOMARA","52":"BERNAL BAQUERO JAMES RICARDO","53":"BURGOS ORTIZ JOSE HORACIO","54":"CANTOR PORRAS JUAN FERNEY","55":"CAPERA CAPERA JOSE GABRIEL","56":"CARDENAS LOTERO RICARDO ANDR\u00c9S","57":"RENDON OSPINA NELSON LEANDRO","58":"SARMIENTO URBINA MOISES DANIEL","59":"VELASCO VELASCO SEBASTI\u00c1N DAVID","60":"DELGADO DELGADO JOHAN DARIO","61":"FLOREZ SAUCESO KENIS ALBERTO","62":"CARDONA GARCIA OSCAR JAVIER","63":"CARVAJAL GARC\u00cdA HOVER MARCK","64":"CEPEDA PIRAQUIVE JUAN DAVID","65":"FAJARDO SAENZ OSCAR FERNANDO","66":"FLOREZ ESPITIA RONY ALBERTO","67":"GARCIA CUERVO EDWIN JAVIER","68":"GONZALEZ OCHOA JUAN CARLOS","69":"XXX1","70":"XXX2","71":"XXX3","72":"FONSECA RAY RICARDO","73":"GOMEZ BETANCUR JAIDER ANDRES","74":"GRANADA PATI\u00d1O CARLOS MARINO","75":"GRASS PLATA MIGUEL SNEIDER","76":"MANZANO CALVO JUAN SEBASTIAN","77":"MENDOZA GOITA MARIANSEL ZENAYDA","78":"MURILLO ARAQUE JAIVER GEOVANY","79":"NI\u00d1O ARENAS HECTOR GONZALO","80":"RAMIREZ CHAVERRA JHON EDISON","81":"XXX4","82":"XXX5","83":"XXX6","84":"RODRIGUEZ MOSQUERA LUIS FERNANDO","85":"PEPITO PEREZ","86":"RAMIREZ VARGAS MARCELA PAOLA","87":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","88":"TORO CISNEROS GARY JOSE","89":"USECHE CALDERON JADID ESTIVEN","90":"VASQUEZ NIETO CAMILO ANDRES","91":"JHONY CASTRO","92":"BERNAL JUAN DAVID","93":"XXX7","94":"XXX8","95":"XXX9","96":"BARON HERNANDEZ HAROLD ANTONIO","97":"CASTELLANOS CARVAJAL DEYVITH FABIAN","98":"AROCA TORRES JULIAN EDUARDO","99":"BERMUDEZ PARRA JENNIFER XIOMARA","100":"BERNAL BAQUERO JAMES RICARDO","101":"BURGOS ORTIZ JOSE HORACIO","102":"CANTOR PORRAS JUAN FERNEY","103":"CAPERA CAPERA JOSE GABRIEL","104":"CARDENAS LOTERO RICARDO ANDR\u00c9S","105":"RENDON OSPINA NELSON LEANDRO","106":"SARMIENTO URBINA MOISES DANIEL","107":"VELASCO VELASCO SEBASTI\u00c1N DAVID","108":"DELGADO DELGADO JOHAN DARIO","109":"FLOREZ SAUCESO KENIS ALBERTO","110":"CARDONA GARCIA OSCAR JAVIER","111":"CARVAJAL GARC\u00cdA HOVER MARCK","112":"CEPEDA PIRAQUIVE JUAN DAVID","113":"FAJARDO SAENZ OSCAR FERNANDO","114":"FLOREZ ESPITIA RONY ALBERTO","115":"GARCIA CUERVO EDWIN JAVIER","116":"GONZALEZ OCHOA JUAN CARLOS","117":"XXX1","118":"XXX2","119":"XXX3","120":"FONSECA RAY RICARDO","121":"GOMEZ BETANCUR JAIDER ANDRES","122":"GRANADA PATI\u00d1O CARLOS MARINO","123":"GRASS PLATA MIGUEL SNEIDER","124":"MANZANO CALVO JUAN SEBASTIAN","125":"MENDOZA GOITA MARIANSEL ZENAYDA","126":"MURILLO ARAQUE JAIVER GEOVANY","127":"NI\u00d1O ARENAS HECTOR GONZALO","128":"RAMIREZ CHAVERRA JHON EDISON","129":"XXX4","130":"XXX5","131":"XXX6","132":"RODRIGUEZ MOSQUERA LUIS FERNANDO","133":"PEPITO PEREZ","134":"RAMIREZ VARGAS MARCELA PAOLA","135":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","136":"TORO CISNEROS GARY JOSE","137":"USECHE CALDERON JADID ESTIVEN","138":"VASQUEZ NIETO CAMILO ANDRES","139":"JHONY CASTRO","140":"BERNAL JUAN DAVID","141":"XXX7","142":"XXX8","143":"XXX9","144":"BARON HERNANDEZ HAROLD ANTONIO","145":"CASTELLANOS CARVAJAL DEYVITH FABIAN","146":"AROCA TORRES JULIAN EDUARDO","147":"BERMUDEZ PARRA JENNIFER XIOMARA","148":"BERNAL BAQUERO JAMES RICARDO","149":"BURGOS ORTIZ JOSE HORACIO","150":"CANTOR PORRAS JUAN FERNEY","151":"CAPERA CAPERA JOSE GABRIEL","152":"CARDENAS LOTERO RICARDO ANDR\u00c9S","153":"RENDON OSPINA NELSON LEANDRO","154":"SARMIENTO URBINA MOISES DANIEL","155":"VELASCO VELASCO SEBASTI\u00c1N DAVID","156":"DELGADO DELGADO JOHAN DARIO","157":"FLOREZ SAUCESO KENIS ALBERTO","158":"CARDONA GARCIA OSCAR JAVIER","159":"CARVAJAL GARC\u00cdA HOVER MARCK","160":"CEPEDA PIRAQUIVE JUAN DAVID","161":"FAJARDO SAENZ OSCAR FERNANDO","162":"FLOREZ ESPITIA RONY ALBERTO","163":"GARCIA CUERVO EDWIN JAVIER","164":"GONZALEZ OCHOA JUAN CARLOS","165":"XXX1","166":"XXX2","167":"XXX3","168":"FONSECA RAY RICARDO","169":"GOMEZ BETANCUR JAIDER ANDRES","170":"GRANADA PATI\u00d1O CARLOS MARINO","171":"GRASS PLATA MIGUEL SNEIDER","172":"MANZANO CALVO JUAN SEBASTIAN","173":"MENDOZA GOITA MARIANSEL ZENAYDA","174":"MURILLO ARAQUE JAIVER GEOVANY","175":"NI\u00d1O ARENAS HECTOR GONZALO","176":"RAMIREZ CHAVERRA JHON EDISON","177":"XXX4","178":"XXX5","179":"XXX6","180":"RODRIGUEZ MOSQUERA LUIS FERNANDO","181":"PEPITO PEREZ","182":"RAMIREZ VARGAS MARCELA PAOLA","183":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","184":"TORO CISNEROS GARY JOSE","185":"USECHE CALDERON JADID ESTIVEN","186":"VASQUEZ NIETO CAMILO ANDRES","187":"JHONY CASTRO","188":"BERNAL JUAN DAVID","189":"XXX7","190":"XXX8","191":"XXX9","192":"BARON HERNANDEZ HAROLD ANTONIO","193":"CASTELLANOS CARVAJAL DEYVITH FABIAN","194":"AROCA TORRES JULIAN EDUARDO","195":"BERMUDEZ PARRA JENNIFER XIOMARA","196":"BERNAL BAQUERO JAMES RICARDO","197":"BURGOS ORTIZ JOSE HORACIO","198":"CANTOR PORRAS JUAN FERNEY","199":"CAPERA CAPERA JOSE GABRIEL","200":"CARDENAS LOTERO RICARDO ANDR\u00c9S","201":"RENDON OSPINA NELSON LEANDRO","202":"SARMIENTO URBINA MOISES DANIEL","203":"VELASCO VELASCO SEBASTI\u00c1N DAVID","204":"DELGADO DELGADO JOHAN DARIO","205":"FLOREZ SAUCESO KENIS ALBERTO","206":"CARDONA GARCIA OSCAR JAVIER","207":"CARVAJAL GARC\u00cdA HOVER MARCK","208":"CEPEDA PIRAQUIVE JUAN DAVID","209":"FAJARDO SAENZ OSCAR FERNANDO","210":"FLOREZ ESPITIA RONY ALBERTO","211":"GARCIA CUERVO EDWIN JAVIER","212":"GONZALEZ OCHOA JUAN CARLOS","213":"XXX1","214":"XXX2","215":"XXX3","216":"FONSECA RAY RICARDO","217":"GOMEZ BETANCUR JAIDER ANDRES","218":"GRANADA PATI\u00d1O CARLOS MARINO","219":"GRASS PLATA MIGUEL SNEIDER","220":"MANZANO CALVO JUAN SEBASTIAN","221":"MENDOZA GOITA MARIANSEL ZENAYDA","222":"MURILLO ARAQUE JAIVER GEOVANY","223":"NI\u00d1O ARENAS HECTOR GONZALO","224":"RAMIREZ CHAVERRA JHON EDISON","225":"XXX4","226":"XXX5","227":"XXX6","228":"RODRIGUEZ MOSQUERA LUIS FERNANDO","229":"PEPITO PEREZ","230":"RAMIREZ VARGAS MARCELA PAOLA","231":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","232":"TORO CISNEROS GARY JOSE","233":"USECHE CALDERON JADID ESTIVEN","234":"VASQUEZ NIETO CAMILO ANDRES","235":"JHONY CASTRO","236":"BERNAL JUAN DAVID","237":"XXX7","238":"XXX8","239":"XXX9","240":"BARON HERNANDEZ HAROLD ANTONIO","241":"CASTELLANOS CARVAJAL DEYVITH FABIAN","242":"AROCA TORRES JULIAN EDUARDO","243":"BERMUDEZ PARRA JENNIFER XIOMARA","244":"BERNAL BAQUERO JAMES RICARDO","245":"BURGOS ORTIZ JOSE HORACIO","246":"CANTOR PORRAS JUAN FERNEY","247":"CAPERA CAPERA JOSE GABRIEL","248":"CARDENAS LOTERO RICARDO ANDR\u00c9S","249":"RENDON OSPINA NELSON LEANDRO","250":"SARMIENTO URBINA MOISES DANIEL","251":"VELASCO VELASCO SEBASTI\u00c1N DAVID","252":"DELGADO DELGADO JOHAN DARIO","253":"FLOREZ SAUCESO KENIS ALBERTO","254":"CARDONA GARCIA OSCAR JAVIER","255":"CARVAJAL GARC\u00cdA HOVER MARCK","256":"CEPEDA PIRAQUIVE JUAN DAVID","257":"FAJARDO SAENZ OSCAR FERNANDO","258":"FLOREZ ESPITIA RONY ALBERTO","259":"GARCIA CUERVO EDWIN JAVIER","260":"GONZALEZ OCHOA JUAN CARLOS","261":"XXX1","262":"XXX2","263":"XXX3","264":"FONSECA RAY RICARDO","265":"GOMEZ BETANCUR JAIDER ANDRES","266":"GRANADA PATI\u00d1O CARLOS MARINO","267":"GRASS PLATA MIGUEL SNEIDER","268":"MANZANO CALVO JUAN SEBASTIAN","269":"MENDOZA GOITA MARIANSEL ZENAYDA","270":"MURILLO ARAQUE JAIVER GEOVANY","271":"NI\u00d1O ARENAS HECTOR GONZALO","272":"RAMIREZ CHAVERRA JHON EDISON","273":"XXX4","274":"XXX5","275":"XXX6","276":"RODRIGUEZ MOSQUERA LUIS FERNANDO","277":"PEPITO PEREZ","278":"RAMIREZ VARGAS MARCELA PAOLA","279":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","280":"TORO CISNEROS GARY JOSE","281":"USECHE CALDERON JADID ESTIVEN","282":"VASQUEZ NIETO CAMILO ANDRES","283":"JHONY CASTRO","284":"BERNAL JUAN DAVID","285":"XXX7","286":"XXX8","287":"XXX9","288":"BARON HERNANDEZ HAROLD ANTONIO","289":"CASTELLANOS CARVAJAL DEYVITH FABIAN","290":"AROCA TORRES JULIAN EDUARDO","291":"BERMUDEZ PARRA JENNIFER XIOMARA","292":"BERNAL BAQUERO JAMES RICARDO","293":"BURGOS ORTIZ JOSE</t>
@@ -381,7 +387,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -409,13 +415,13 @@
         <v>2026</v>
       </c>
       <c r="C2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -426,13 +432,30 @@
         <v>2026</v>
       </c>
       <c r="C3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" t="s">
         <v>7</v>
       </c>
-      <c r="D3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E3" t="s">
+      <c r="B4">
+        <v>2026</v>
+      </c>
+      <c r="C4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" t="s">
         <v>11</v>
+      </c>
+      <c r="E4" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update historico_mallas.xlsx 2026-04-24 18:15:47.930720
</commit_message>
<xml_diff>
--- a/historico_mallas.xlsx
+++ b/historico_mallas.xlsx
@@ -31,31 +31,31 @@
     <t>Datos_JSON</t>
   </si>
   <si>
+    <t>Mayo</t>
+  </si>
+  <si>
+    <t>Junio</t>
+  </si>
+  <si>
     <t>Abril</t>
   </si>
   <si>
-    <t>Mayo</t>
-  </si>
-  <si>
-    <t>Junio</t>
-  </si>
-  <si>
     <t>Técnica</t>
   </si>
   <si>
-    <t>24/04/2026 17:52</t>
-  </si>
-  <si>
     <t>24/04/2026 17:55</t>
   </si>
   <si>
     <t>24/04/2026 17:56</t>
   </si>
   <si>
+    <t>2026-04-24 18:15</t>
+  </si>
+  <si>
+    <t>{"Grupo":{"0":"GRUPO 1","1":"GRUPO 1","2":"GRUPO 1","3":"GRUPO 1","4":"GRUPO 1","5":"GRUPO 1","6":"GRUPO 1","7":"GRUPO 1","8":"GRUPO 1","9":"GRUPO 1","10":"GRUPO 1","11":"GRUPO 1","12":"GRUPO 2","13":"GRUPO 2","14":"GRUPO 2","15":"GRUPO 2","16":"GRUPO 2","17":"GRUPO 2","18":"GRUPO 2","19":"GRUPO 2","20":"GRUPO 2","21":"GRUPO 2","22":"GRUPO 2","23":"GRUPO 2","24":"GRUPO 3","25":"GRUPO 3","26":"GRUPO 3","27":"GRUPO 3","28":"GRUPO 3","29":"GRUPO 3","30":"GRUPO 3","31":"GRUPO 3","32":"GRUPO 3","33":"GRUPO 3","34":"GRUPO 3","35":"GRUPO 3","36":"GRUPO 4","37":"GRUPO 4","38":"GRUPO 4","39":"GRUPO 4","40":"GRUPO 4","41":"GRUPO 4","42":"GRUPO 4","43":"GRUPO 4","44":"GRUPO 4","45":"GRUPO 4","46":"GRUPO 4","47":"GRUPO 4","48":"GRUPO 1","49":"GRUPO 1","50":"GRUPO 1","51":"GRUPO 1","52":"GRUPO 1","53":"GRUPO 1","54":"GRUPO 1","55":"GRUPO 1","56":"GRUPO 1","57":"GRUPO 1","58":"GRUPO 1","59":"GRUPO 1","60":"GRUPO 2","61":"GRUPO 2","62":"GRUPO 2","63":"GRUPO 2","64":"GRUPO 2","65":"GRUPO 2","66":"GRUPO 2","67":"GRUPO 2","68":"GRUPO 2","69":"GRUPO 2","70":"GRUPO 2","71":"GRUPO 2","72":"GRUPO 3","73":"GRUPO 3","74":"GRUPO 3","75":"GRUPO 3","76":"GRUPO 3","77":"GRUPO 3","78":"GRUPO 3","79":"GRUPO 3","80":"GRUPO 3","81":"GRUPO 3","82":"GRUPO 3","83":"GRUPO 3","84":"GRUPO 4","85":"GRUPO 4","86":"GRUPO 4","87":"GRUPO 4","88":"GRUPO 4","89":"GRUPO 4","90":"GRUPO 4","91":"GRUPO 4","92":"GRUPO 4","93":"GRUPO 4","94":"GRUPO 4","95":"GRUPO 4","96":"GRUPO 1","97":"GRUPO 1","98":"GRUPO 1","99":"GRUPO 1","100":"GRUPO 1","101":"GRUPO 1","102":"GRUPO 1","103":"GRUPO 1","104":"GRUPO 1","105":"GRUPO 1","106":"GRUPO 1","107":"GRUPO 1","108":"GRUPO 2","109":"GRUPO 2","110":"GRUPO 2","111":"GRUPO 2","112":"GRUPO 2","113":"GRUPO 2","114":"GRUPO 2","115":"GRUPO 2","116":"GRUPO 2","117":"GRUPO 2","118":"GRUPO 2","119":"GRUPO 2","120":"GRUPO 3","121":"GRUPO 3","122":"GRUPO 3","123":"GRUPO 3","124":"GRUPO 3","125":"GRUPO 3","126":"GRUPO 3","127":"GRUPO 3","128":"GRUPO 3","129":"GRUPO 3","130":"GRUPO 3","131":"GRUPO 3","132":"GRUPO 4","133":"GRUPO 4","134":"GRUPO 4","135":"GRUPO 4","136":"GRUPO 4","137":"GRUPO 4","138":"GRUPO 4","139":"GRUPO 4","140":"GRUPO 4","141":"GRUPO 4","142":"GRUPO 4","143":"GRUPO 4","144":"GRUPO 1","145":"GRUPO 1","146":"GRUPO 1","147":"GRUPO 1","148":"GRUPO 1","149":"GRUPO 1","150":"GRUPO 1","151":"GRUPO 1","152":"GRUPO 1","153":"GRUPO 1","154":"GRUPO 1","155":"GRUPO 1","156":"GRUPO 2","157":"GRUPO 2","158":"GRUPO 2","159":"GRUPO 2","160":"GRUPO 2","161":"GRUPO 2","162":"GRUPO 2","163":"GRUPO 2","164":"GRUPO 2","165":"GRUPO 2","166":"GRUPO 2","167":"GRUPO 2","168":"GRUPO 3","169":"GRUPO 3","170":"GRUPO 3","171":"GRUPO 3","172":"GRUPO 3","173":"GRUPO 3","174":"GRUPO 3","175":"GRUPO 3","176":"GRUPO 3","177":"GRUPO 3","178":"GRUPO 3","179":"GRUPO 3","180":"GRUPO 4","181":"GRUPO 4","182":"GRUPO 4","183":"GRUPO 4","184":"GRUPO 4","185":"GRUPO 4","186":"GRUPO 4","187":"GRUPO 4","188":"GRUPO 4","189":"GRUPO 4","190":"GRUPO 4","191":"GRUPO 4","192":"GRUPO 1","193":"GRUPO 1","194":"GRUPO 1","195":"GRUPO 1","196":"GRUPO 1","197":"GRUPO 1","198":"GRUPO 1","199":"GRUPO 1","200":"GRUPO 1","201":"GRUPO 1","202":"GRUPO 1","203":"GRUPO 1","204":"GRUPO 2","205":"GRUPO 2","206":"GRUPO 2","207":"GRUPO 2","208":"GRUPO 2","209":"GRUPO 2","210":"GRUPO 2","211":"GRUPO 2","212":"GRUPO 2","213":"GRUPO 2","214":"GRUPO 2","215":"GRUPO 2","216":"GRUPO 3","217":"GRUPO 3","218":"GRUPO 3","219":"GRUPO 3","220":"GRUPO 3","221":"GRUPO 3","222":"GRUPO 3","223":"GRUPO 3","224":"GRUPO 3","225":"GRUPO 3","226":"GRUPO 3","227":"GRUPO 3","228":"GRUPO 4","229":"GRUPO 4","230":"GRUPO 4","231":"GRUPO 4","232":"GRUPO 4","233":"GRUPO 4","234":"GRUPO 4","235":"GRUPO 4","236":"GRUPO 4","237":"GRUPO 4","238":"GRUPO 4","239":"GRUPO 4","240":"GRUPO 1","241":"GRUPO 1","242":"GRUPO 1","243":"GRUPO 1","244":"GRUPO 1","245":"GRUPO 1","246":"GRUPO 1","247":"GRUPO 1","248":"GRUPO 1","249":"GRUPO 1","250":"GRUPO 1","251":"GRUPO 1","252":"GRUPO 2","253":"GRUPO 2","254":"GRUPO 2","255":"GRUPO 2","256":"GRUPO 2","257":"GRUPO 2","258":"GRUPO 2","259":"GRUPO 2","260":"GRUPO 2","261":"GRUPO 2","262":"GRUPO 2","263":"GRUPO 2","264":"GRUPO 3","265":"GRUPO 3","266":"GRUPO 3","267":"GRUPO 3","268":"GRUPO 3","269":"GRUPO 3","270":"GRUPO 3","271":"GRUPO 3","272":"GRUPO 3","273":"GRUPO 3","274":"GRUPO 3","275":"GRUPO 3","276":"GRUPO 4","277":"GRUPO 4","278":"GRUPO 4","279":"GRUPO 4","280":"GRUPO 4","281":"GRUPO 4","282":"GRUPO 4","283":"GRUPO 4","284":"GRUPO 4","285":"GRUPO 4","286":"GRUPO 4","287":"GRUPO 4","288":"GRUPO 1","289":"GRUPO 1","290":"GRUPO 1","291":"GRUPO 1","292":"GRUPO 1","293":"GRUPO 1","294":"GRUPO 1","295":"GRUPO 1","296":"GRUPO 1","297":"GRUPO 1","298":"GRUPO 1","299":"GRUPO 1","300":"GRUPO 2","301":"GRUPO 2","302":"GRUPO 2","303":"GRUPO 2","304":"GRUPO 2","305":"GRUPO 2","306":"GRUPO 2","307":"GRUPO 2","308":"GRUPO 2","309":"GRUPO 2","310":"GRUPO 2","311":"GRUPO 2","312":"GRUPO 3","313":"GRUPO 3","314":"GRUPO 3","315":"GRUPO 3","316":"GRUPO 3","317":"GRUPO 3","318":"GRUPO 3","319":"GRUPO 3","320":"GRUPO 3","321":"GRUPO 3","322":"GRUPO 3","323":"GRUPO 3","324":"GRUPO 4","325":"GRUPO 4","326":"GRUPO 4","327":"GRUPO 4","328":"GRUPO 4","329":"GRUPO 4","330":"GRUPO 4","331":"GRUPO 4","332":"GRUPO 4","333":"GRUPO 4","334":"GRUPO 4","335":"GRUPO 4","336":"GRUPO 1","337":"GRUPO 1","338":"GRUPO 1","339":"GRUPO 1","340":"GRUPO 1","341":"GRUPO 1","342":"GRUPO 1","343":"GRUPO 1","344":"GRUPO 1","345":"GRUPO 1","346":"GRUPO 1","347":"GRUPO 1","348":"GRUPO 2","349":"GRUPO 2","350":"GRUPO 2","351":"GRUPO 2","352":"GRUPO 2","353":"GRUPO 2","354":"GRUPO 2","355":"GRUPO 2","356":"GRUPO 2","357":"GRUPO 2","358":"GRUPO 2","359":"GRUPO 2","360":"GRUPO 3","361":"GRUPO 3","362":"GRUPO 3","363":"GRUPO 3","364":"GRUPO 3","365":"GRUPO 3","366":"GRUPO 3","367":"GRUPO 3","368":"GRUPO 3","369":"GRUPO 3","370":"GRUPO 3","371":"GRUPO 3","372":"GRUPO 4","373":"GRUPO 4","374":"GRUPO 4","375":"GRUPO 4","376":"GRUPO 4","377":"GRUPO 4","378":"GRUPO 4","379":"GRUPO 4","380":"GRUPO 4","381":"GRUPO 4","382":"GRUPO 4","383":"GRUPO 4","384":"GRUPO 1","385":"GRUPO 1","386":"GRUPO 1","387":"GRUPO 1","388":"GRUPO 1","389":"GRUPO 1","390":"GRUPO 1","391":"GRUPO 1","392":"GRUPO 1","393":"GRUPO 1","394":"GRUPO 1","395":"GRUPO 1","396":"GRUPO 2","397":"GRUPO 2","398":"GRUPO 2","399":"GRUPO 2","400":"GRUPO 2","401":"GRUPO 2","402":"GRUPO 2","403":"GRUPO 2","404":"GRUPO 2","405":"GRUPO 2","406":"GRUPO 2","407":"GRUPO 2","408":"GRUPO 3","409":"GRUPO 3","410":"GRUPO 3","411":"GRUPO 3","412":"GRUPO 3","413":"GRUPO 3","414":"GRUPO 3","415":"GRUPO 3","416":"GRUPO 3","417":"GRUPO 3","418":"GRUPO 3","419":"GRUPO 3","420":"GRUPO 4","421":"GRUPO 4","422":"GRUPO 4","423":"GRUPO 4","424":"GRUPO 4","425":"GRUPO 4","426":"GRUPO 4","427":"GRUPO 4","428":"GRUPO 4","429":"GRUPO 4","430":"GRUPO 4","431":"GRUPO 4","432":"GRUPO 1","433":"GRUPO 1","434":"GRUPO 1","435":"GRUPO 1","436":"GRUPO 1","437":"GRUPO 1","438":"GRUPO 1","439":"GRUPO 1","440":"GRUPO 1","441":"GRUPO 1","442":"GRUPO 1","443":"GRUPO 1","444":"GRUPO 2","445":"GRUPO 2","446":"GRUPO 2","447":"GRUPO 2","448":"GRUPO 2","449":"GRUPO 2","450":"GRUPO 2","451":"GRUPO 2","452":"GRUPO 2","453":"GRUPO 2","454":"GRUPO 2","455":"GRUPO 2","456":"GRUPO 3","457":"GRUPO 3","458":"GRUPO 3","459":"GRUPO 3","460":"GRUPO 3","461":"GRUPO 3","462":"GRUPO 3","463":"GRUPO 3","464":"GRUPO 3","465":"GRUPO 3","466":"GRUPO 3","467":"GRUPO 3","468":"GRUPO 4","469":"GRUPO 4","470":"GRUPO 4","471":"GRUPO 4","472":"GRUPO 4","473":"GRUPO 4","474":"GRUPO 4","475":"GRUPO 4","476":"GRUPO 4","477":"GRUPO 4","478":"GRUPO 4","479":"GRUPO 4","480":"GRUPO 1","481":"GRUPO 1","482":"GRUPO 1","483":"GRUPO 1","484":"GRUPO 1","485":"GRUPO 1","486":"GRUPO 1","487":"GRUPO 1","488":"GRUPO 1","489":"GRUPO 1","490":"GRUPO 1","491":"GRUPO 1","492":"GRUPO 2","493":"GRUPO 2","494":"GRUPO 2","495":"GRUPO 2","496":"GRUPO 2","497":"GRUPO 2","498":"GRUPO 2","499":"GRUPO 2","500":"GRUPO 2","501":"GRUPO 2","502":"GRUPO 2","503":"GRUPO 2","504":"GRUPO 3","505":"GRUPO 3","506":"GRUPO 3","507":"GRUPO 3","508":"GRUPO 3","509":"GRUPO 3","510":"GRUPO 3","511":"GRUPO 3","512":"GRUPO 3","513":"GRUPO 3","514":"GRUPO 3","515":"GRUPO 3","516":"GRUPO 4","517":"GRUPO 4","518":"GRUPO 4","519":"GRUPO 4","520":"GRUPO 4","521":"GRUPO 4","522":"GRUPO 4","523":"GRUPO 4","524":"GRUPO 4","525":"GRUPO 4","526":"GRUPO 4","527":"GRUPO 4","528":"GRUPO 1","529":"GRUPO 1","530":"GRUPO 1","531":"GRUPO 1","532":"GRUPO 1","533":"GRUPO 1","534":"GRUPO 1","535":"GRUPO 1","536":"GRUPO 1","537":"GRUPO 1","538":"GRUPO 1","539":"GRUPO 1","540":"GRUPO 2","541":"GRUPO 2","542":"GRUPO 2","543":"GRUPO 2","544":"GRUPO 2","545":"GRUPO 2","546":"GRUPO 2","547":"GRUPO 2","548":"GRUPO 2","549":"GRUPO 2","550":"GRUPO 2","551":"GRUPO 2","552":"GRUPO 3","553":"GRUPO 3","554":"GRUPO 3","555":"GRUPO 3","556":"GRUPO 3","557":"GRUPO 3","558":"GRUPO 3","559":"GRUPO 3","560":"GRUPO 3","561":"GRUPO 3","562":"GRUPO 3","563":"GRUPO 3","564":"GRUPO 4","565":"GRUPO 4","566":"GRUPO 4","567":"GRUPO 4","568":"GRUPO 4","569":"GRUPO 4","570":"GRUPO 4","571":"GRUPO 4","572":"GRUPO 4","573":"GRUPO 4","574":"GRUPO 4","575":"GRUPO 4","576":"GRUPO 1","577":"GRUPO 1","578":"GRUPO 1","579":"GRUPO 1","580":"GRUPO 1","581":"GRUPO 1","582":"GRUPO 1","583":"GRUPO 1","584":"GRUPO 1","585":"GRUPO 1","586":"GRUPO 1","587":"GRUPO 1","588":"GRUPO 2","589":"GRUPO 2","590":"GRUPO 2","591":"GRUPO 2","592":"GRUPO 2","593":"GRUPO 2","594":"GRUPO 2","595":"GRUPO 2","596":"GRUPO 2","597":"GRUPO 2","598":"GRUPO 2","599":"GRUPO 2","600":"GRUPO 3","601":"GRUPO 3","602":"GRUPO 3","603":"GRUPO 3","604":"GRUPO 3","605":"GRUPO 3","606":"GRUPO 3","607":"GRUPO 3","608":"GRUPO 3","609":"GRUPO 3","610":"GRUPO 3","611":"GRUPO 3","612":"GRUPO 4","613":"GRUPO 4","614":"GRUPO 4","615":"GRUPO 4","616":"GRUPO 4","617":"GRUPO 4","618":"GRUPO 4","619":"GRUPO 4","620":"GRUPO 4","621":"GRUPO 4","622":"GRUPO 4","623":"GRUPO 4","624":"GRUPO 1","625":"GRUPO 1","626":"GRUPO 1","627":"GRUPO 1","628":"GRUPO 1","629":"GRUPO 1","630":"GRUPO 1","631":"GRUPO 1","632":"GRUPO 1","633":"GRUPO 1","634":"GRUPO 1","635":"GRUPO 1","636":"GRUPO 2","637":"GRUPO 2","638":"GRUPO 2","639":"GRUPO 2","640":"GRUPO 2","641":"GRUPO 2","642":"GRUPO 2","643":"GRUPO 2","644":"GRUPO 2","645":"GRUPO 2","646":"GRUPO 2","647":"GRUPO 2","648":"GRUPO 3","649":"GRUPO 3","650":"GRUPO 3","651":"GRUPO 3","652":"GRUPO 3","653":"GRUPO 3","654":"GRUPO 3","655":"GRUPO 3","656":"GRUPO 3","657":"GRUPO 3","658":"GRUPO 3","659":"GRUPO 3","660":"GRUPO 4","661":"GRUPO 4","662":"GRUPO 4","663":"GRUPO 4","664":"GRUPO 4","665":"GRUPO 4","666":"GRUPO 4","667":"GRUPO 4","668":"GRUPO 4","669":"GRUPO 4","670":"GRUPO 4","671":"GRUPO 4","672":"GRUPO 1","673":"GRUPO 1","674":"GRUPO 1","675":"GRUPO 1","676":"GRUPO 1","677":"GRUPO 1","678":"GRUPO 1","679":"GRUPO 1","680":"GRUPO 1","681":"GRUPO 1","682":"GRUPO 1","683":"GRUPO 1","684":"GRUPO 2","685":"GRUPO 2","686":"GRUPO 2","687":"GRUPO 2","688":"GRUPO 2","689":"GRUPO 2","690":"GRUPO 2","691":"GRUPO 2","692":"GRUPO 2","693":"GRUPO 2","694":"GRUPO 2","695":"GRUPO 2","696":"GRUPO 3","697":"GRUPO 3","698":"GRUPO 3","699":"GRUPO 3","700":"GRUPO 3","701":"GRUPO 3","702":"GRUPO 3","703":"GRUPO 3","704":"GRUPO 3","705":"GRUPO 3","706":"GRUPO 3","707":"GRUPO 3","708":"GRUPO 4","709":"GRUPO 4","710":"GRUPO 4","711":"GRUPO 4","712":"GRUPO 4","713":"GRUPO 4","714":"GRUPO 4","715":"GRUPO 4","716":"GRUPO 4","717":"GRUPO 4","718":"GRUPO 4","719":"GRUPO 4","720":"GRUPO 1","721":"GRUPO 1","722":"GRUPO 1","723":"GRUPO 1","724":"GRUPO 1","725":"GRUPO 1","726":"GRUPO 1","727":"GRUPO 1","728":"GRUPO 1","729":"GRUPO 1","730":"GRUPO 1","731":"GRUPO 1","732":"GRUPO 2","733":"GRUPO 2","734":"GRUPO 2","735":"GRUPO 2","736":"GRUPO 2","737":"GRUPO 2","738":"GRUPO 2","739":"GRUPO 2","740":"GRUPO 2","741":"GRUPO 2","742":"GRUPO 2","743":"GRUPO 2","744":"GRUPO 3","745":"GRUPO 3","746":"GRUPO 3","747":"GRUPO 3","748":"GRUPO 3","749":"GRUPO 3","750":"GRUPO 3","751":"GRUPO 3","752":"GRUPO 3","753":"GRUPO 3","754":"GRUPO 3","755":"GRUPO 3","756":"GRUPO 4","757":"GRUPO 4","758":"GRUPO 4","759":"GRUPO 4","760":"GRUPO 4","761":"GRUPO 4","762":"GRUPO 4","763":"GRUPO 4","764":"GRUPO 4","765":"GRUPO 4","766":"GRUPO 4","767":"GRUPO 4","768":"GRUPO 1","769":"GRUPO 1","770":"GRUPO 1","771":"GRUPO 1","772":"GRUPO 1","773":"GRUPO 1","774":"GRUPO 1","775":"GRUPO 1","776":"GRUPO 1","777":"GRUPO 1","778":"GRUPO 1","779":"GRUPO 1","780":"GRUPO 2","781":"GRUPO 2","782":"GRUPO 2","783":"GRUPO 2","784":"GRUPO 2","785":"GRUPO 2","786":"GRUPO 2","787":"GRUPO 2","788":"GRUPO 2","789":"GRUPO 2","790":"GRUPO 2","791":"GRUPO 2","792":"GRUPO 3","793":"GRUPO 3","794":"GRUPO 3","795":"GRUPO 3","796":"GRUPO 3","797":"GRUPO 3","798":"GRUPO 3","799":"GRUPO 3","800":"GRUPO 3","801":"GRUPO 3","802":"GRUPO 3","803":"GRUPO 3","804":"GRUPO 4","805":"GRUPO 4","806":"GRUPO 4","807":"GRUPO 4","808":"GRUPO 4","809":"GRUPO 4","810":"GRUPO 4","811":"GRUPO 4","812":"GRUPO 4","813":"GRUPO 4","814":"GRUPO 4","815":"GRUPO 4","816":"GRUPO 1","817":"GRUPO 1","818":"GRUPO 1","819":"GRUPO 1","820":"GRUPO 1","821":"GRUPO 1","822":"GRUPO 1","823":"GRUPO 1","824":"GRUPO 1","825":"GRUPO 1","826":"GRUPO 1","827":"GRUPO 1","828":"GRUPO 2","829":"GRUPO 2","830":"GRUPO 2","831":"GRUPO 2","832":"GRUPO 2","833":"GRUPO 2","834":"GRUPO 2","835":"GRUPO 2","836":"GRUPO 2","837":"GRUPO 2","838":"GRUPO 2","839":"GRUPO 2","840":"GRUPO 3","841":"GRUPO 3","842":"GRUPO 3","843":"GRUPO 3","844":"GRUPO 3","845":"GRUPO 3","846":"GRUPO 3","847":"GRUPO 3","848":"GRUPO 3","849":"GRUPO 3","850":"GRUPO 3","851":"GRUPO 3","852":"GRUPO 4","853":"GRUPO 4","854":"GRUPO 4","855":"GRUPO 4","856":"GRUPO 4","857":"GRUPO 4","858":"GRUPO 4","859":"GRUPO 4","860":"GRUPO 4","861":"GRUPO 4","862":"GRUPO 4","863":"GRUPO 4","864":"GRUPO 1","865":"GRUPO 1","866":"GRUPO 1","867":"GRUPO 1","868":"GRUPO 1","869":"GRUPO 1","870":"GRUPO 1","871":"GRUPO 1","872":"GRUPO 1","873":"GRUPO 1","874":"GRUPO 1","875":"GRUPO 1","876":"GRUPO 2","877":"GRUPO 2","878":"GRUPO 2","879":"GRUPO 2","880":"GRUPO 2","881":"GRUPO 2","882":"GRUPO 2","883":"GRUPO 2","884":"GRUPO 2","885":"GRUPO 2","886":"GRUPO 2","887":"GRUPO 2","888":"GRUPO 3","889":"GRUPO 3","890":"GRUPO 3","891":"GRUPO 3","892":"GRUPO 3","893":"GRUPO 3","894":"GRUPO 3","895":"GRUPO 3","896":"GRUPO 3","897":"GRUPO 3","898":"GRUPO 3","899":"GRUPO 3","900":"GRUPO 4","901":"GRUPO 4","902":"GRUPO 4","903":"GRUPO 4","904":"GRUPO 4","905":"GRUPO 4","906":"GRUPO 4","907":"GRUPO 4","908":"GRUPO 4","909":"GRUPO 4","910":"GRUPO 4","911":"GRUPO 4","912":"GRUPO 1","913":"GRUPO 1","914":"GRUPO 1","915":"GRUPO 1","916":"GRUPO 1","917":"GRUPO 1","918":"GRUPO 1","919":"GRUPO 1","920":"GRUPO 1","921":"GRUPO 1","922":"GRUPO 1","923":"GRUPO 1","924":"GRUPO 2","925":"GRUPO 2","926":"GRUPO 2","927":"GRUPO 2","928":"GRUPO 2","929":"GRUPO 2","930":"GRUPO 2","931":"GRUPO 2","932":"GRUPO 2","933":"GRUPO 2","934":"GRUPO 2","935":"GRUPO 2","936":"GRUPO 3","937":"GRUPO 3","938":"GRUPO 3","939":"GRUPO 3","940":"GRUPO 3","941":"GRUPO 3","942":"GRUPO 3","943":"GRUPO 3","944":"GRUPO 3","945":"GRUPO 3","946":"GRUPO 3","947":"GRUPO 3","948":"GRUPO 4","949":"GRUPO 4","950":"GRUPO 4","951":"GRUPO 4","952":"GRUPO 4","953":"GRUPO 4","954":"GRUPO 4","955":"GRUPO 4","956":"GRUPO 4","957":"GRUPO 4","958":"GRUPO 4","959":"GRUPO 4","960":"GRUPO 1","961":"GRUPO 1","962":"GRUPO 1","963":"GRUPO 1","964":"GRUPO 1","965":"GRUPO 1","966":"GRUPO 1","967":"GRUPO 1","968":"GRUPO 1","969":"GRUPO 1","970":"GRUPO 1","971":"GRUPO 1","972":"GRUPO 2","973":"GRUPO 2","974":"GRUPO 2","975":"GRUPO 2","976":"GRUPO 2","977":"GRUPO 2","978":"GRUPO 2","979":"GRUPO 2","980":"GRUPO 2","981":"GRUPO 2","982":"GRUPO 2","983":"GRUPO 2","984":"GRUPO 3","985":"GRUPO 3","986":"GRUPO 3","987":"GRUPO 3","988":"GRUPO 3","989":"GRUPO 3","990":"GRUPO 3","991":"GRUPO 3","992":"GRUPO 3","993":"GRUPO 3","994":"GRUPO 3","995":"GRUPO 3","996":"GRUPO 4","997":"GRUPO 4","998":"GRUPO 4","999":"GRUPO 4","1000":"GRUPO 4","1001":"GRUPO 4","1002":"GRUPO 4","1003":"GRUPO 4","1004":"GRUPO 4","1005":"GRUPO 4","1006":"GRUPO 4","1007":"GRUPO 4","1008":"GRUPO 1","1009":"GRUPO 1","1010":"GRUPO 1","1011":"GRUPO 1","1012":"GRUPO 1","1013":"GRUPO 1","1014":"GRUPO 1","1015":"GRUPO 1","1016":"GRUPO 1","1017":"GRUPO 1","1018":"GRUPO 1","1019":"GRUPO 1","1020":"GRUPO 2","1021":"GRUPO 2","1022":"GRUPO 2","1023":"GRUPO 2","1024":"GRUPO 2","1025":"GRUPO 2","1026":"GRUPO 2","1027":"GRUPO 2","1028":"GRUPO 2","1029":"GRUPO 2","1030":"GRUPO 2","1031":"GRUPO 2","1032":"GRUPO 3","1033":"GRUPO 3","1034":"GRUPO 3","1035":"GRUPO 3","1036":"GRUPO 3","1037":"GRUPO 3","1038":"GRUPO 3","1039":"GRUPO 3","1040":"GRUPO 3","1041":"GRUPO 3","1042":"GRUPO 3","1043":"GRUPO 3","1044":"GRUPO 4","1045":"GRUPO 4","1046":"GRUPO 4","1047":"GRUPO 4","1048":"GRUPO 4","1049":"GRUPO 4","1050":"GRUPO 4","1051":"GRUPO 4","1052":"GRUPO 4","1053":"GRUPO 4","1054":"GRUPO 4","1055":"GRUPO 4","1056":"GRUPO 1","1057":"GRUPO 1","1058":"GRUPO 1","1059":"GRUPO 1","1060":"GRUPO 1","1061":"GRUPO 1","1062":"GRUPO 1","1063":"GRUPO 1","1064":"GRUPO 1","1065":"GRUPO 1","1066":"GRUPO 1","1067":"GRUPO 1","1068":"GRUPO 2","1069":"GRUPO 2","1070":"GRUPO 2","1071":"GRUPO 2","1072":"GRUPO 2","1073":"GRUPO 2","1074":"GRUPO 2","1075":"GRUPO 2","1076":"GRUPO 2","1077":"GRUPO 2","1078":"GRUPO 2","1079":"GRUPO 2","1080":"GRUPO 3","1081":"GRUPO 3","1082":"GRUPO 3","1083":"GRUPO 3","1084":"GRUPO 3","1085":"GRUPO 3","1086":"GRUPO 3","1087":"GRUPO 3","1088":"GRUPO 3","1089":"GRUPO 3","1090":"GRUPO 3","1091":"GRUPO 3","1092":"GRUPO 4","1093":"GRUPO 4","1094":"GRUPO 4","1095":"GRUPO 4","1096":"GRUPO 4","1097":"GRUPO 4","1098":"GRUPO 4","1099":"GRUPO 4","1100":"GRUPO 4","1101":"GRUPO 4","1102":"GRUPO 4","1103":"GRUPO 4","1104":"GRUPO 1","1105":"GRUPO 1","1106":"GRUPO 1","1107":"GRUPO 1","1108":"GRUPO 1","1109":"GRUPO 1","1110":"GRUPO 1","1111":"GRUPO 1","1112":"GRUPO 1","1113":"GRUPO 1","1114":"GRUPO 1","1115":"GRUPO 1","1116":"GRUPO 2","1117":"GRUPO 2","1118":"GRUPO 2","1119":"GRUPO 2","1120":"GRUPO 2","1121":"GRUPO 2","1122":"GRUPO 2","1123":"GRUPO 2","1124":"GRUPO 2","1125":"GRUPO 2","1126":"GRUPO 2","1127":"GRUPO 2","1128":"GRUPO 3","1129":"GRUPO 3","1130":"GRUPO 3","1131":"GRUPO 3","1132":"GRUPO 3","1133":"GRUPO 3","1134":"GRUPO 3","1135":"GRUPO 3","1136":"GRUPO 3","1137":"GRUPO 3","1138":"GRUPO 3","1139":"GRUPO 3","1140":"GRUPO 4","1141":"GRUPO 4","1142":"GRUPO 4","1143":"GRUPO 4","1144":"GRUPO 4","1145":"GRUPO 4","1146":"GRUPO 4","1147":"GRUPO 4","1148":"GRUPO 4","1149":"GRUPO 4","1150":"GRUPO 4","1151":"GRUPO 4","1152":"GRUPO 1","1153":"GRUPO 1","1154":"GRUPO 1","1155":"GRUPO 1","1156":"GRUPO 1","1157":"GRUPO 1","1158":"GRUPO 1","1159":"GRUPO 1","1160":"GRUPO 1","1161":"GRUPO 1","1162":"GRUPO 1","1163":"GRUPO 1","1164":"GRUPO 2","1165":"GRUPO 2","1166":"GRUPO 2","1167":"GRUPO 2","1168":"GRUPO 2","1169":"GRUPO 2","1170":"GRUPO 2","1171":"GRUPO 2","1172":"GRUPO 2","1173":"GRUPO 2","1174":"GRUPO 2","1175":"GRUPO 2","1176":"GRUPO 3","1177":"GRUPO 3","1178":"GRUPO 3","1179":"GRUPO 3","1180":"GRUPO 3","1181":"GRUPO 3","1182":"GRUPO 3","1183":"GRUPO 3","1184":"GRUPO 3","1185":"GRUPO 3","1186":"GRUPO 3","1187":"GRUPO 3","1188":"GRUPO 4","1189":"GRUPO 4","1190":"GRUPO 4","1191":"GRUPO 4","1192":"GRUPO 4","1193":"GRUPO 4","1194":"GRUPO 4","1195":"GRUPO 4","1196":"GRUPO 4","1197":"GRUPO 4","1198":"GRUPO 4","1199":"GRUPO 4","1200":"GRUPO 1","1201":"GRUPO 1","1202":"GRUPO 1","1203":"GRUPO 1","1204":"GRUPO 1","1205":"GRUPO 1","1206":"GRUPO 1","1207":"GRUPO 1","1208":"GRUPO 1","1209":"GRUPO 1","1210":"GRUPO 1","1211":"GRUPO 1","1212":"GRUPO 2","1213":"GRUPO 2","1214":"GRUPO 2","1215":"GRUPO 2","1216":"GRUPO 2","1217":"GRUPO 2","1218":"GRUPO 2","1219":"GRUPO 2","1220":"GRUPO 2","1221":"GRUPO 2","1222":"GRUPO 2","1223":"GRUPO 2","1224":"GRUPO 3","1225":"GRUPO 3","1226":"GRUPO 3","1227":"GRUPO 3","1228":"GRUPO 3","1229":"GRUPO 3","1230":"GRUPO 3","1231":"GRUPO 3","1232":"GRUPO 3","1233":"GRUPO 3","1234":"GRUPO 3","1235":"GRUPO 3","1236":"GRUPO 4","1237":"GRUPO 4","1238":"GRUPO 4","1239":"GRUPO 4","1240":"GRUPO 4","1241":"GRUPO 4","1242":"GRUPO 4","1243":"GRUPO 4","1244":"GRUPO 4","1245":"GRUPO 4","1246":"GRUPO 4","1247":"GRUPO 4","1248":"GRUPO 1","1249":"GRUPO 1","1250":"GRUPO 1","1251":"GRUPO 1","1252":"GRUPO 1","1253":"GRUPO 1","1254":"GRUPO 1","1255":"GRUPO 1","1256":"GRUPO 1","1257":"GRUPO 1","1258":"GRUPO 1","1259":"GRUPO 1","1260":"GRUPO 2","1261":"GRUPO 2","1262":"GRUPO 2","1263":"GRUPO 2","1264":"GRUPO 2","1265":"GRUPO 2","1266":"GRUPO 2","1267":"GRUPO 2","1268":"GRUPO 2","1269":"GRUPO 2","1270":"GRUPO 2","1271":"GRUPO 2","1272":"GRUPO 3","1273":"GRUPO 3","1274":"GRUPO 3","1275":"GRUPO 3","1276":"GRUPO 3","1277":"GRUPO 3","1278":"GRUPO 3","1279":"GRUPO 3","1280":"GRUPO 3","1281":"GRUPO 3","1282":"GRUPO 3","1283":"GRUPO 3","1284":"GRUPO 4","1285":"GRUPO 4","1286":"GRUPO 4","1287":"GRUPO 4","1288":"GRUPO 4","1289":"GRUPO 4","1290":"GRUPO 4","1291":"GRUPO 4","1292":"GRUPO 4","1293":"GRUPO 4","1294":"GRUPO 4","1295":"GRUPO 4","1296":"GRUPO 1","1297":"GRUPO 1","1298":"GRUPO 1","1299":"GRUPO 1","1300":"GRUPO 1","1301":"GRUPO 1","1302":"GRUPO 1","1303":"GRUPO 1","1304":"GRUPO 1","1305":"GRUPO 1","1306":"GRUPO 1","1307":"GRUPO 1","1308":"GRUPO 2","1309":"GRUPO 2","1310":"GRUPO 2","1311":"GRUPO 2","1312":"GRUPO 2","1313":"GRUPO 2","1314":"GRUPO 2","1315":"GRUPO 2","1316":"GRUPO 2","1317":"GRUPO 2","1318":"GRUPO 2","1319":"GRUPO 2","1320":"GRUPO 3","1321":"GRUPO 3","1322":"GRUPO 3","1323":"GRUPO 3","1324":"GRUPO 3","1325":"GRUPO 3","1326":"GRUPO 3","1327":"GRUPO 3","1328":"GRUPO 3","1329":"GRUPO 3","1330":"GRUPO 3","1331":"GRUPO 3","1332":"GRUPO 4","1333":"GRUPO 4","1334":"GRUPO 4","1335":"GRUPO 4","1336":"GRUPO 4","1337":"GRUPO 4","1338":"GRUPO 4","1339":"GRUPO 4","1340":"GRUPO 4","1341":"GRUPO 4","1342":"GRUPO 4","1343":"GRUPO 4","1344":"GRUPO 1","1345":"GRUPO 1","1346":"GRUPO 1","1347":"GRUPO 1","1348":"GRUPO 1","1349":"GRUPO 1","1350":"GRUPO 1","1351":"GRUPO 1","1352":"GRUPO 1","1353":"GRUPO 1","1354":"GRUPO 1","1355":"GRUPO 1","1356":"GRUPO 2","1357":"GRUPO 2","1358":"GRUPO 2","1359":"GRUPO 2","1360":"GRUPO 2","1361":"GRUPO 2","1362":"GRUPO 2","1363":"GRUPO 2","1364":"GRUPO 2","1365":"GRUPO 2","1366":"GRUPO 2","1367":"GRUPO 2","1368":"GRUPO 3","1369":"GRUPO 3","1370":"GRUPO 3","1371":"GRUPO 3","1372":"GRUPO 3","1373":"GRUPO 3","1374":"GRUPO 3","1375":"GRUPO 3","1376":"GRUPO 3","1377":"GRUPO 3","1378":"GRUPO 3","1379":"GRUPO 3","1380":"GRUPO 4","1381":"GRUPO 4","1382":"GRUPO 4","1383":"GRUPO 4","1384":"GRUPO 4","1385":"GRUPO 4","1386":"GRUPO 4","1387":"GRUPO 4","1388":"GRUPO 4","1389":"GRUPO 4","1390":"GRUPO 4","1391":"GRUPO 4","1392":"GRUPO 1","1393":"GRUPO 1","1394":"GRUPO 1","1395":"GRUPO 1","1396":"GRUPO 1","1397":"GRUPO 1","1398":"GRUPO 1","1399":"GRUPO 1","1400":"GRUPO 1","1401":"GRUPO 1","1402":"GRUPO 1","1403":"GRUPO 1","1404":"GRUPO 2","1405":"GRUPO 2","1406":"GRUPO 2","1407":"GRUPO 2","1408":"GRUPO 2","1409":"GRUPO 2","1410":"GRUPO 2","1411":"GRUPO 2","1412":"GRUPO 2","1413":"GRUPO 2","1414":"GRUPO 2","1415":"GRUPO 2","1416":"GRUPO 3","1417":"GRUPO 3","1418":"GRUPO 3","1419":"GRUPO 3","1420":"GRUPO 3","1421":"GRUPO 3","1422":"GRUPO 3","1423":"GRUPO 3","1424":"GRUPO 3","1425":"GRUPO 3","1426":"GRUPO 3","1427":"GRUPO 3","1428":"GRUPO 4","1429":"GRUPO 4","1430":"GRUPO 4","1431":"GRUPO 4","1432":"GRUPO 4","1433":"GRUPO 4","1434":"GRUPO 4","1435":"GRUPO 4","1436":"GRUPO 4","1437":"GRUPO 4","1438":"GRUPO 4","1439":"GRUPO 4","1440":"GRUPO 1","1441":"GRUPO 1","1442":"GRUPO 1","1443":"GRUPO 1","1444":"GRUPO 1","1445":"GRUPO 1","1446":"GRUPO 1","1447":"GRUPO 1","1448":"GRUPO 1","1449":"GRUPO 1","1450":"GRUPO 1","1451":"GRUPO 1","1452":"GRUPO 2","1453":"GRUPO 2","1454":"GRUPO 2","1455":"GRUPO 2","1456":"GRUPO 2","1457":"GRUPO 2","1458":"GRUPO 2","1459":"GRUPO 2","1460":"GRUPO 2","1461":"GRUPO 2","1462":"GRUPO 2","1463":"GRUPO 2","1464":"GRUPO 3","1465":"GRUPO 3","1466":"GRUPO 3","1467":"GRUPO 3","1468":"GRUPO 3","1469":"GRUPO 3","1470":"GRUPO 3","1471":"GRUPO 3","1472":"GRUPO 3","1473":"GRUPO 3","1474":"GRUPO 3","1475":"GRUPO 3","1476":"GRUPO 4","1477":"GRUPO 4","1478":"GRUPO 4","1479":"GRUPO 4","1480":"GRUPO 4","1481":"GRUPO 4","1482":"GRUPO 4","1483":"GRUPO 4","1484":"GRUPO 4","1485":"GRUPO 4","1486":"GRUPO 4","1487":"GRUPO 4"},"Empleado":{"0":"BARON HERNANDEZ HAROLD ANTONIO","1":"CASTELLANOS CARVAJAL DEYVITH FABIAN","2":"AROCA TORRES JULIAN EDUARDO","3":"BERMUDEZ PARRA JENNIFER XIOMARA","4":"BERNAL BAQUERO JAMES RICARDO","5":"BURGOS ORTIZ JOSE HORACIO","6":"CANTOR PORRAS JUAN FERNEY","7":"CAPERA CAPERA JOSE GABRIEL","8":"CARDENAS LOTERO RICARDO ANDR\u00c9S","9":"RENDON OSPINA NELSON LEANDRO","10":"SARMIENTO URBINA MOISES DANIEL","11":"VELASCO VELASCO SEBASTI\u00c1N DAVID","12":"DELGADO DELGADO JOHAN DARIO","13":"FLOREZ SAUCESO KENIS ALBERTO","14":"CARDONA GARCIA OSCAR JAVIER","15":"CARVAJAL GARC\u00cdA HOVER MARCK","16":"CEPEDA PIRAQUIVE JUAN DAVID","17":"FAJARDO SAENZ OSCAR FERNANDO","18":"FLOREZ ESPITIA RONY ALBERTO","19":"GARCIA CUERVO EDWIN JAVIER","20":"GONZALEZ OCHOA JUAN CARLOS","21":"XXX1","22":"XXX2","23":"XXX3","24":"FONSECA RAY RICARDO","25":"GOMEZ BETANCUR JAIDER ANDRES","26":"GRANADA PATI\u00d1O CARLOS MARINO","27":"GRASS PLATA MIGUEL SNEIDER","28":"MANZANO CALVO JUAN SEBASTIAN","29":"MENDOZA GOITA MARIANSEL ZENAYDA","30":"MURILLO ARAQUE JAIVER GEOVANY","31":"NI\u00d1O ARENAS HECTOR GONZALO","32":"RAMIREZ CHAVERRA JHON EDISON","33":"XXX4","34":"XXX5","35":"XXX6","36":"RODRIGUEZ MOSQUERA LUIS FERNANDO","37":"PEPITO PEREZ","38":"RAMIREZ VARGAS MARCELA PAOLA","39":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","40":"TORO CISNEROS GARY JOSE","41":"USECHE CALDERON JADID ESTIVEN","42":"VASQUEZ NIETO CAMILO ANDRES","43":"JHONY CASTRO","44":"BERNAL JUAN DAVID","45":"XXX7","46":"XXX8","47":"XXX9","48":"BARON HERNANDEZ HAROLD ANTONIO","49":"CASTELLANOS CARVAJAL DEYVITH FABIAN","50":"AROCA TORRES JULIAN EDUARDO","51":"BERMUDEZ PARRA JENNIFER XIOMARA","52":"BERNAL BAQUERO JAMES RICARDO","53":"BURGOS ORTIZ JOSE HORACIO","54":"CANTOR PORRAS JUAN FERNEY","55":"CAPERA CAPERA JOSE GABRIEL","56":"CARDENAS LOTERO RICARDO ANDR\u00c9S","57":"RENDON OSPINA NELSON LEANDRO","58":"SARMIENTO URBINA MOISES DANIEL","59":"VELASCO VELASCO SEBASTI\u00c1N DAVID","60":"DELGADO DELGADO JOHAN DARIO","61":"FLOREZ SAUCESO KENIS ALBERTO","62":"CARDONA GARCIA OSCAR JAVIER","63":"CARVAJAL GARC\u00cdA HOVER MARCK","64":"CEPEDA PIRAQUIVE JUAN DAVID","65":"FAJARDO SAENZ OSCAR FERNANDO","66":"FLOREZ ESPITIA RONY ALBERTO","67":"GARCIA CUERVO EDWIN JAVIER","68":"GONZALEZ OCHOA JUAN CARLOS","69":"XXX1","70":"XXX2","71":"XXX3","72":"FONSECA RAY RICARDO","73":"GOMEZ BETANCUR JAIDER ANDRES","74":"GRANADA PATI\u00d1O CARLOS MARINO","75":"GRASS PLATA MIGUEL SNEIDER","76":"MANZANO CALVO JUAN SEBASTIAN","77":"MENDOZA GOITA MARIANSEL ZENAYDA","78":"MURILLO ARAQUE JAIVER GEOVANY","79":"NI\u00d1O ARENAS HECTOR GONZALO","80":"RAMIREZ CHAVERRA JHON EDISON","81":"XXX4","82":"XXX5","83":"XXX6","84":"RODRIGUEZ MOSQUERA LUIS FERNANDO","85":"PEPITO PEREZ","86":"RAMIREZ VARGAS MARCELA PAOLA","87":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","88":"TORO CISNEROS GARY JOSE","89":"USECHE CALDERON JADID ESTIVEN","90":"VASQUEZ NIETO CAMILO ANDRES","91":"JHONY CASTRO","92":"BERNAL JUAN DAVID","93":"XXX7","94":"XXX8","95":"XXX9","96":"BARON HERNANDEZ HAROLD ANTONIO","97":"CASTELLANOS CARVAJAL DEYVITH FABIAN","98":"AROCA TORRES JULIAN EDUARDO","99":"BERMUDEZ PARRA JENNIFER XIOMARA","100":"BERNAL BAQUERO JAMES RICARDO","101":"BURGOS ORTIZ JOSE HORACIO","102":"CANTOR PORRAS JUAN FERNEY","103":"CAPERA CAPERA JOSE GABRIEL","104":"CARDENAS LOTERO RICARDO ANDR\u00c9S","105":"RENDON OSPINA NELSON LEANDRO","106":"SARMIENTO URBINA MOISES DANIEL","107":"VELASCO VELASCO SEBASTI\u00c1N DAVID","108":"DELGADO DELGADO JOHAN DARIO","109":"FLOREZ SAUCESO KENIS ALBERTO","110":"CARDONA GARCIA OSCAR JAVIER","111":"CARVAJAL GARC\u00cdA HOVER MARCK","112":"CEPEDA PIRAQUIVE JUAN DAVID","113":"FAJARDO SAENZ OSCAR FERNANDO","114":"FLOREZ ESPITIA RONY ALBERTO","115":"GARCIA CUERVO EDWIN JAVIER","116":"GONZALEZ OCHOA JUAN CARLOS","117":"XXX1","118":"XXX2","119":"XXX3","120":"FONSECA RAY RICARDO","121":"GOMEZ BETANCUR JAIDER ANDRES","122":"GRANADA PATI\u00d1O CARLOS MARINO","123":"GRASS PLATA MIGUEL SNEIDER","124":"MANZANO CALVO JUAN SEBASTIAN","125":"MENDOZA GOITA MARIANSEL ZENAYDA","126":"MURILLO ARAQUE JAIVER GEOVANY","127":"NI\u00d1O ARENAS HECTOR GONZALO","128":"RAMIREZ CHAVERRA JHON EDISON","129":"XXX4","130":"XXX5","131":"XXX6","132":"RODRIGUEZ MOSQUERA LUIS FERNANDO","133":"PEPITO PEREZ","134":"RAMIREZ VARGAS MARCELA PAOLA","135":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","136":"TORO CISNEROS GARY JOSE","137":"USECHE CALDERON JADID ESTIVEN","138":"VASQUEZ NIETO CAMILO ANDRES","139":"JHONY CASTRO","140":"BERNAL JUAN DAVID","141":"XXX7","142":"XXX8","143":"XXX9","144":"BARON HERNANDEZ HAROLD ANTONIO","145":"CASTELLANOS CARVAJAL DEYVITH FABIAN","146":"AROCA TORRES JULIAN EDUARDO","147":"BERMUDEZ PARRA JENNIFER XIOMARA","148":"BERNAL BAQUERO JAMES RICARDO","149":"BURGOS ORTIZ JOSE HORACIO","150":"CANTOR PORRAS JUAN FERNEY","151":"CAPERA CAPERA JOSE GABRIEL","152":"CARDENAS LOTERO RICARDO ANDR\u00c9S","153":"RENDON OSPINA NELSON LEANDRO","154":"SARMIENTO URBINA MOISES DANIEL","155":"VELASCO VELASCO SEBASTI\u00c1N DAVID","156":"DELGADO DELGADO JOHAN DARIO","157":"FLOREZ SAUCESO KENIS ALBERTO","158":"CARDONA GARCIA OSCAR JAVIER","159":"CARVAJAL GARC\u00cdA HOVER MARCK","160":"CEPEDA PIRAQUIVE JUAN DAVID","161":"FAJARDO SAENZ OSCAR FERNANDO","162":"FLOREZ ESPITIA RONY ALBERTO","163":"GARCIA CUERVO EDWIN JAVIER","164":"GONZALEZ OCHOA JUAN CARLOS","165":"XXX1","166":"XXX2","167":"XXX3","168":"FONSECA RAY RICARDO","169":"GOMEZ BETANCUR JAIDER ANDRES","170":"GRANADA PATI\u00d1O CARLOS MARINO","171":"GRASS PLATA MIGUEL SNEIDER","172":"MANZANO CALVO JUAN SEBASTIAN","173":"MENDOZA GOITA MARIANSEL ZENAYDA","174":"MURILLO ARAQUE JAIVER GEOVANY","175":"NI\u00d1O ARENAS HECTOR GONZALO","176":"RAMIREZ CHAVERRA JHON EDISON","177":"XXX4","178":"XXX5","179":"XXX6","180":"RODRIGUEZ MOSQUERA LUIS FERNANDO","181":"PEPITO PEREZ","182":"RAMIREZ VARGAS MARCELA PAOLA","183":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","184":"TORO CISNEROS GARY JOSE","185":"USECHE CALDERON JADID ESTIVEN","186":"VASQUEZ NIETO CAMILO ANDRES","187":"JHONY CASTRO","188":"BERNAL JUAN DAVID","189":"XXX7","190":"XXX8","191":"XXX9","192":"BARON HERNANDEZ HAROLD ANTONIO","193":"CASTELLANOS CARVAJAL DEYVITH FABIAN","194":"AROCA TORRES JULIAN EDUARDO","195":"BERMUDEZ PARRA JENNIFER XIOMARA","196":"BERNAL BAQUERO JAMES RICARDO","197":"BURGOS ORTIZ JOSE HORACIO","198":"CANTOR PORRAS JUAN FERNEY","199":"CAPERA CAPERA JOSE GABRIEL","200":"CARDENAS LOTERO RICARDO ANDR\u00c9S","201":"RENDON OSPINA NELSON LEANDRO","202":"SARMIENTO URBINA MOISES DANIEL","203":"VELASCO VELASCO SEBASTI\u00c1N DAVID","204":"DELGADO DELGADO JOHAN DARIO","205":"FLOREZ SAUCESO KENIS ALBERTO","206":"CARDONA GARCIA OSCAR JAVIER","207":"CARVAJAL GARC\u00cdA HOVER MARCK","208":"CEPEDA PIRAQUIVE JUAN DAVID","209":"FAJARDO SAENZ OSCAR FERNANDO","210":"FLOREZ ESPITIA RONY ALBERTO","211":"GARCIA CUERVO EDWIN JAVIER","212":"GONZALEZ OCHOA JUAN CARLOS","213":"XXX1","214":"XXX2","215":"XXX3","216":"FONSECA RAY RICARDO","217":"GOMEZ BETANCUR JAIDER ANDRES","218":"GRANADA PATI\u00d1O CARLOS MARINO","219":"GRASS PLATA MIGUEL SNEIDER","220":"MANZANO CALVO JUAN SEBASTIAN","221":"MENDOZA GOITA MARIANSEL ZENAYDA","222":"MURILLO ARAQUE JAIVER GEOVANY","223":"NI\u00d1O ARENAS HECTOR GONZALO","224":"RAMIREZ CHAVERRA JHON EDISON","225":"XXX4","226":"XXX5","227":"XXX6","228":"RODRIGUEZ MOSQUERA LUIS FERNANDO","229":"PEPITO PEREZ","230":"RAMIREZ VARGAS MARCELA PAOLA","231":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","232":"TORO CISNEROS GARY JOSE","233":"USECHE CALDERON JADID ESTIVEN","234":"VASQUEZ NIETO CAMILO ANDRES","235":"JHONY CASTRO","236":"BERNAL JUAN DAVID","237":"XXX7","238":"XXX8","239":"XXX9","240":"BARON HERNANDEZ HAROLD ANTONIO","241":"CASTELLANOS CARVAJAL DEYVITH FABIAN","242":"AROCA TORRES JULIAN EDUARDO","243":"BERMUDEZ PARRA JENNIFER XIOMARA","244":"BERNAL BAQUERO JAMES RICARDO","245":"BURGOS ORTIZ JOSE HORACIO","246":"CANTOR PORRAS JUAN FERNEY","247":"CAPERA CAPERA JOSE GABRIEL","248":"CARDENAS LOTERO RICARDO ANDR\u00c9S","249":"RENDON OSPINA NELSON LEANDRO","250":"SARMIENTO URBINA MOISES DANIEL","251":"VELASCO VELASCO SEBASTI\u00c1N DAVID","252":"DELGADO DELGADO JOHAN DARIO","253":"FLOREZ SAUCESO KENIS ALBERTO","254":"CARDONA GARCIA OSCAR JAVIER","255":"CARVAJAL GARC\u00cdA HOVER MARCK","256":"CEPEDA PIRAQUIVE JUAN DAVID","257":"FAJARDO SAENZ OSCAR FERNANDO","258":"FLOREZ ESPITIA RONY ALBERTO","259":"GARCIA CUERVO EDWIN JAVIER","260":"GONZALEZ OCHOA JUAN CARLOS","261":"XXX1","262":"XXX2","263":"XXX3","264":"FONSECA RAY RICARDO","265":"GOMEZ BETANCUR JAIDER ANDRES","266":"GRANADA PATI\u00d1O CARLOS MARINO","267":"GR</t>
+  </si>
+  <si>
     <t>{"Grupo":{"0":"GRUPO 1","1":"GRUPO 1","2":"GRUPO 1","3":"GRUPO 1","4":"GRUPO 1","5":"GRUPO 1","6":"GRUPO 1","7":"GRUPO 1","8":"GRUPO 1","9":"GRUPO 1","10":"GRUPO 1","11":"GRUPO 1","12":"GRUPO 2","13":"GRUPO 2","14":"GRUPO 2","15":"GRUPO 2","16":"GRUPO 2","17":"GRUPO 2","18":"GRUPO 2","19":"GRUPO 2","20":"GRUPO 2","21":"GRUPO 2","22":"GRUPO 2","23":"GRUPO 2","24":"GRUPO 3","25":"GRUPO 3","26":"GRUPO 3","27":"GRUPO 3","28":"GRUPO 3","29":"GRUPO 3","30":"GRUPO 3","31":"GRUPO 3","32":"GRUPO 3","33":"GRUPO 3","34":"GRUPO 3","35":"GRUPO 3","36":"GRUPO 4","37":"GRUPO 4","38":"GRUPO 4","39":"GRUPO 4","40":"GRUPO 4","41":"GRUPO 4","42":"GRUPO 4","43":"GRUPO 4","44":"GRUPO 4","45":"GRUPO 4","46":"GRUPO 4","47":"GRUPO 4","48":"GRUPO 1","49":"GRUPO 1","50":"GRUPO 1","51":"GRUPO 1","52":"GRUPO 1","53":"GRUPO 1","54":"GRUPO 1","55":"GRUPO 1","56":"GRUPO 1","57":"GRUPO 1","58":"GRUPO 1","59":"GRUPO 1","60":"GRUPO 2","61":"GRUPO 2","62":"GRUPO 2","63":"GRUPO 2","64":"GRUPO 2","65":"GRUPO 2","66":"GRUPO 2","67":"GRUPO 2","68":"GRUPO 2","69":"GRUPO 2","70":"GRUPO 2","71":"GRUPO 2","72":"GRUPO 3","73":"GRUPO 3","74":"GRUPO 3","75":"GRUPO 3","76":"GRUPO 3","77":"GRUPO 3","78":"GRUPO 3","79":"GRUPO 3","80":"GRUPO 3","81":"GRUPO 3","82":"GRUPO 3","83":"GRUPO 3","84":"GRUPO 4","85":"GRUPO 4","86":"GRUPO 4","87":"GRUPO 4","88":"GRUPO 4","89":"GRUPO 4","90":"GRUPO 4","91":"GRUPO 4","92":"GRUPO 4","93":"GRUPO 4","94":"GRUPO 4","95":"GRUPO 4","96":"GRUPO 1","97":"GRUPO 1","98":"GRUPO 1","99":"GRUPO 1","100":"GRUPO 1","101":"GRUPO 1","102":"GRUPO 1","103":"GRUPO 1","104":"GRUPO 1","105":"GRUPO 1","106":"GRUPO 1","107":"GRUPO 1","108":"GRUPO 2","109":"GRUPO 2","110":"GRUPO 2","111":"GRUPO 2","112":"GRUPO 2","113":"GRUPO 2","114":"GRUPO 2","115":"GRUPO 2","116":"GRUPO 2","117":"GRUPO 2","118":"GRUPO 2","119":"GRUPO 2","120":"GRUPO 3","121":"GRUPO 3","122":"GRUPO 3","123":"GRUPO 3","124":"GRUPO 3","125":"GRUPO 3","126":"GRUPO 3","127":"GRUPO 3","128":"GRUPO 3","129":"GRUPO 3","130":"GRUPO 3","131":"GRUPO 3","132":"GRUPO 4","133":"GRUPO 4","134":"GRUPO 4","135":"GRUPO 4","136":"GRUPO 4","137":"GRUPO 4","138":"GRUPO 4","139":"GRUPO 4","140":"GRUPO 4","141":"GRUPO 4","142":"GRUPO 4","143":"GRUPO 4","144":"GRUPO 1","145":"GRUPO 1","146":"GRUPO 1","147":"GRUPO 1","148":"GRUPO 1","149":"GRUPO 1","150":"GRUPO 1","151":"GRUPO 1","152":"GRUPO 1","153":"GRUPO 1","154":"GRUPO 1","155":"GRUPO 1","156":"GRUPO 2","157":"GRUPO 2","158":"GRUPO 2","159":"GRUPO 2","160":"GRUPO 2","161":"GRUPO 2","162":"GRUPO 2","163":"GRUPO 2","164":"GRUPO 2","165":"GRUPO 2","166":"GRUPO 2","167":"GRUPO 2","168":"GRUPO 3","169":"GRUPO 3","170":"GRUPO 3","171":"GRUPO 3","172":"GRUPO 3","173":"GRUPO 3","174":"GRUPO 3","175":"GRUPO 3","176":"GRUPO 3","177":"GRUPO 3","178":"GRUPO 3","179":"GRUPO 3","180":"GRUPO 4","181":"GRUPO 4","182":"GRUPO 4","183":"GRUPO 4","184":"GRUPO 4","185":"GRUPO 4","186":"GRUPO 4","187":"GRUPO 4","188":"GRUPO 4","189":"GRUPO 4","190":"GRUPO 4","191":"GRUPO 4","192":"GRUPO 1","193":"GRUPO 1","194":"GRUPO 1","195":"GRUPO 1","196":"GRUPO 1","197":"GRUPO 1","198":"GRUPO 1","199":"GRUPO 1","200":"GRUPO 1","201":"GRUPO 1","202":"GRUPO 1","203":"GRUPO 1","204":"GRUPO 2","205":"GRUPO 2","206":"GRUPO 2","207":"GRUPO 2","208":"GRUPO 2","209":"GRUPO 2","210":"GRUPO 2","211":"GRUPO 2","212":"GRUPO 2","213":"GRUPO 2","214":"GRUPO 2","215":"GRUPO 2","216":"GRUPO 3","217":"GRUPO 3","218":"GRUPO 3","219":"GRUPO 3","220":"GRUPO 3","221":"GRUPO 3","222":"GRUPO 3","223":"GRUPO 3","224":"GRUPO 3","225":"GRUPO 3","226":"GRUPO 3","227":"GRUPO 3","228":"GRUPO 4","229":"GRUPO 4","230":"GRUPO 4","231":"GRUPO 4","232":"GRUPO 4","233":"GRUPO 4","234":"GRUPO 4","235":"GRUPO 4","236":"GRUPO 4","237":"GRUPO 4","238":"GRUPO 4","239":"GRUPO 4","240":"GRUPO 1","241":"GRUPO 1","242":"GRUPO 1","243":"GRUPO 1","244":"GRUPO 1","245":"GRUPO 1","246":"GRUPO 1","247":"GRUPO 1","248":"GRUPO 1","249":"GRUPO 1","250":"GRUPO 1","251":"GRUPO 1","252":"GRUPO 2","253":"GRUPO 2","254":"GRUPO 2","255":"GRUPO 2","256":"GRUPO 2","257":"GRUPO 2","258":"GRUPO 2","259":"GRUPO 2","260":"GRUPO 2","261":"GRUPO 2","262":"GRUPO 2","263":"GRUPO 2","264":"GRUPO 3","265":"GRUPO 3","266":"GRUPO 3","267":"GRUPO 3","268":"GRUPO 3","269":"GRUPO 3","270":"GRUPO 3","271":"GRUPO 3","272":"GRUPO 3","273":"GRUPO 3","274":"GRUPO 3","275":"GRUPO 3","276":"GRUPO 4","277":"GRUPO 4","278":"GRUPO 4","279":"GRUPO 4","280":"GRUPO 4","281":"GRUPO 4","282":"GRUPO 4","283":"GRUPO 4","284":"GRUPO 4","285":"GRUPO 4","286":"GRUPO 4","287":"GRUPO 4","288":"GRUPO 1","289":"GRUPO 1","290":"GRUPO 1","291":"GRUPO 1","292":"GRUPO 1","293":"GRUPO 1","294":"GRUPO 1","295":"GRUPO 1","296":"GRUPO 1","297":"GRUPO 1","298":"GRUPO 1","299":"GRUPO 1","300":"GRUPO 2","301":"GRUPO 2","302":"GRUPO 2","303":"GRUPO 2","304":"GRUPO 2","305":"GRUPO 2","306":"GRUPO 2","307":"GRUPO 2","308":"GRUPO 2","309":"GRUPO 2","310":"GRUPO 2","311":"GRUPO 2","312":"GRUPO 3","313":"GRUPO 3","314":"GRUPO 3","315":"GRUPO 3","316":"GRUPO 3","317":"GRUPO 3","318":"GRUPO 3","319":"GRUPO 3","320":"GRUPO 3","321":"GRUPO 3","322":"GRUPO 3","323":"GRUPO 3","324":"GRUPO 4","325":"GRUPO 4","326":"GRUPO 4","327":"GRUPO 4","328":"GRUPO 4","329":"GRUPO 4","330":"GRUPO 4","331":"GRUPO 4","332":"GRUPO 4","333":"GRUPO 4","334":"GRUPO 4","335":"GRUPO 4","336":"GRUPO 1","337":"GRUPO 1","338":"GRUPO 1","339":"GRUPO 1","340":"GRUPO 1","341":"GRUPO 1","342":"GRUPO 1","343":"GRUPO 1","344":"GRUPO 1","345":"GRUPO 1","346":"GRUPO 1","347":"GRUPO 1","348":"GRUPO 2","349":"GRUPO 2","350":"GRUPO 2","351":"GRUPO 2","352":"GRUPO 2","353":"GRUPO 2","354":"GRUPO 2","355":"GRUPO 2","356":"GRUPO 2","357":"GRUPO 2","358":"GRUPO 2","359":"GRUPO 2","360":"GRUPO 3","361":"GRUPO 3","362":"GRUPO 3","363":"GRUPO 3","364":"GRUPO 3","365":"GRUPO 3","366":"GRUPO 3","367":"GRUPO 3","368":"GRUPO 3","369":"GRUPO 3","370":"GRUPO 3","371":"GRUPO 3","372":"GRUPO 4","373":"GRUPO 4","374":"GRUPO 4","375":"GRUPO 4","376":"GRUPO 4","377":"GRUPO 4","378":"GRUPO 4","379":"GRUPO 4","380":"GRUPO 4","381":"GRUPO 4","382":"GRUPO 4","383":"GRUPO 4","384":"GRUPO 1","385":"GRUPO 1","386":"GRUPO 1","387":"GRUPO 1","388":"GRUPO 1","389":"GRUPO 1","390":"GRUPO 1","391":"GRUPO 1","392":"GRUPO 1","393":"GRUPO 1","394":"GRUPO 1","395":"GRUPO 1","396":"GRUPO 2","397":"GRUPO 2","398":"GRUPO 2","399":"GRUPO 2","400":"GRUPO 2","401":"GRUPO 2","402":"GRUPO 2","403":"GRUPO 2","404":"GRUPO 2","405":"GRUPO 2","406":"GRUPO 2","407":"GRUPO 2","408":"GRUPO 3","409":"GRUPO 3","410":"GRUPO 3","411":"GRUPO 3","412":"GRUPO 3","413":"GRUPO 3","414":"GRUPO 3","415":"GRUPO 3","416":"GRUPO 3","417":"GRUPO 3","418":"GRUPO 3","419":"GRUPO 3","420":"GRUPO 4","421":"GRUPO 4","422":"GRUPO 4","423":"GRUPO 4","424":"GRUPO 4","425":"GRUPO 4","426":"GRUPO 4","427":"GRUPO 4","428":"GRUPO 4","429":"GRUPO 4","430":"GRUPO 4","431":"GRUPO 4","432":"GRUPO 1","433":"GRUPO 1","434":"GRUPO 1","435":"GRUPO 1","436":"GRUPO 1","437":"GRUPO 1","438":"GRUPO 1","439":"GRUPO 1","440":"GRUPO 1","441":"GRUPO 1","442":"GRUPO 1","443":"GRUPO 1","444":"GRUPO 2","445":"GRUPO 2","446":"GRUPO 2","447":"GRUPO 2","448":"GRUPO 2","449":"GRUPO 2","450":"GRUPO 2","451":"GRUPO 2","452":"GRUPO 2","453":"GRUPO 2","454":"GRUPO 2","455":"GRUPO 2","456":"GRUPO 3","457":"GRUPO 3","458":"GRUPO 3","459":"GRUPO 3","460":"GRUPO 3","461":"GRUPO 3","462":"GRUPO 3","463":"GRUPO 3","464":"GRUPO 3","465":"GRUPO 3","466":"GRUPO 3","467":"GRUPO 3","468":"GRUPO 4","469":"GRUPO 4","470":"GRUPO 4","471":"GRUPO 4","472":"GRUPO 4","473":"GRUPO 4","474":"GRUPO 4","475":"GRUPO 4","476":"GRUPO 4","477":"GRUPO 4","478":"GRUPO 4","479":"GRUPO 4","480":"GRUPO 1","481":"GRUPO 1","482":"GRUPO 1","483":"GRUPO 1","484":"GRUPO 1","485":"GRUPO 1","486":"GRUPO 1","487":"GRUPO 1","488":"GRUPO 1","489":"GRUPO 1","490":"GRUPO 1","491":"GRUPO 1","492":"GRUPO 2","493":"GRUPO 2","494":"GRUPO 2","495":"GRUPO 2","496":"GRUPO 2","497":"GRUPO 2","498":"GRUPO 2","499":"GRUPO 2","500":"GRUPO 2","501":"GRUPO 2","502":"GRUPO 2","503":"GRUPO 2","504":"GRUPO 3","505":"GRUPO 3","506":"GRUPO 3","507":"GRUPO 3","508":"GRUPO 3","509":"GRUPO 3","510":"GRUPO 3","511":"GRUPO 3","512":"GRUPO 3","513":"GRUPO 3","514":"GRUPO 3","515":"GRUPO 3","516":"GRUPO 4","517":"GRUPO 4","518":"GRUPO 4","519":"GRUPO 4","520":"GRUPO 4","521":"GRUPO 4","522":"GRUPO 4","523":"GRUPO 4","524":"GRUPO 4","525":"GRUPO 4","526":"GRUPO 4","527":"GRUPO 4","528":"GRUPO 1","529":"GRUPO 1","530":"GRUPO 1","531":"GRUPO 1","532":"GRUPO 1","533":"GRUPO 1","534":"GRUPO 1","535":"GRUPO 1","536":"GRUPO 1","537":"GRUPO 1","538":"GRUPO 1","539":"GRUPO 1","540":"GRUPO 2","541":"GRUPO 2","542":"GRUPO 2","543":"GRUPO 2","544":"GRUPO 2","545":"GRUPO 2","546":"GRUPO 2","547":"GRUPO 2","548":"GRUPO 2","549":"GRUPO 2","550":"GRUPO 2","551":"GRUPO 2","552":"GRUPO 3","553":"GRUPO 3","554":"GRUPO 3","555":"GRUPO 3","556":"GRUPO 3","557":"GRUPO 3","558":"GRUPO 3","559":"GRUPO 3","560":"GRUPO 3","561":"GRUPO 3","562":"GRUPO 3","563":"GRUPO 3","564":"GRUPO 4","565":"GRUPO 4","566":"GRUPO 4","567":"GRUPO 4","568":"GRUPO 4","569":"GRUPO 4","570":"GRUPO 4","571":"GRUPO 4","572":"GRUPO 4","573":"GRUPO 4","574":"GRUPO 4","575":"GRUPO 4","576":"GRUPO 1","577":"GRUPO 1","578":"GRUPO 1","579":"GRUPO 1","580":"GRUPO 1","581":"GRUPO 1","582":"GRUPO 1","583":"GRUPO 1","584":"GRUPO 1","585":"GRUPO 1","586":"GRUPO 1","587":"GRUPO 1","588":"GRUPO 2","589":"GRUPO 2","590":"GRUPO 2","591":"GRUPO 2","592":"GRUPO 2","593":"GRUPO 2","594":"GRUPO 2","595":"GRUPO 2","596":"GRUPO 2","597":"GRUPO 2","598":"GRUPO 2","599":"GRUPO 2","600":"GRUPO 3","601":"GRUPO 3","602":"GRUPO 3","603":"GRUPO 3","604":"GRUPO 3","605":"GRUPO 3","606":"GRUPO 3","607":"GRUPO 3","608":"GRUPO 3","609":"GRUPO 3","610":"GRUPO 3","611":"GRUPO 3","612":"GRUPO 4","613":"GRUPO 4","614":"GRUPO 4","615":"GRUPO 4","616":"GRUPO 4","617":"GRUPO 4","618":"GRUPO 4","619":"GRUPO 4","620":"GRUPO 4","621":"GRUPO 4","622":"GRUPO 4","623":"GRUPO 4","624":"GRUPO 1","625":"GRUPO 1","626":"GRUPO 1","627":"GRUPO 1","628":"GRUPO 1","629":"GRUPO 1","630":"GRUPO 1","631":"GRUPO 1","632":"GRUPO 1","633":"GRUPO 1","634":"GRUPO 1","635":"GRUPO 1","636":"GRUPO 2","637":"GRUPO 2","638":"GRUPO 2","639":"GRUPO 2","640":"GRUPO 2","641":"GRUPO 2","642":"GRUPO 2","643":"GRUPO 2","644":"GRUPO 2","645":"GRUPO 2","646":"GRUPO 2","647":"GRUPO 2","648":"GRUPO 3","649":"GRUPO 3","650":"GRUPO 3","651":"GRUPO 3","652":"GRUPO 3","653":"GRUPO 3","654":"GRUPO 3","655":"GRUPO 3","656":"GRUPO 3","657":"GRUPO 3","658":"GRUPO 3","659":"GRUPO 3","660":"GRUPO 4","661":"GRUPO 4","662":"GRUPO 4","663":"GRUPO 4","664":"GRUPO 4","665":"GRUPO 4","666":"GRUPO 4","667":"GRUPO 4","668":"GRUPO 4","669":"GRUPO 4","670":"GRUPO 4","671":"GRUPO 4","672":"GRUPO 1","673":"GRUPO 1","674":"GRUPO 1","675":"GRUPO 1","676":"GRUPO 1","677":"GRUPO 1","678":"GRUPO 1","679":"GRUPO 1","680":"GRUPO 1","681":"GRUPO 1","682":"GRUPO 1","683":"GRUPO 1","684":"GRUPO 2","685":"GRUPO 2","686":"GRUPO 2","687":"GRUPO 2","688":"GRUPO 2","689":"GRUPO 2","690":"GRUPO 2","691":"GRUPO 2","692":"GRUPO 2","693":"GRUPO 2","694":"GRUPO 2","695":"GRUPO 2","696":"GRUPO 3","697":"GRUPO 3","698":"GRUPO 3","699":"GRUPO 3","700":"GRUPO 3","701":"GRUPO 3","702":"GRUPO 3","703":"GRUPO 3","704":"GRUPO 3","705":"GRUPO 3","706":"GRUPO 3","707":"GRUPO 3","708":"GRUPO 4","709":"GRUPO 4","710":"GRUPO 4","711":"GRUPO 4","712":"GRUPO 4","713":"GRUPO 4","714":"GRUPO 4","715":"GRUPO 4","716":"GRUPO 4","717":"GRUPO 4","718":"GRUPO 4","719":"GRUPO 4","720":"GRUPO 1","721":"GRUPO 1","722":"GRUPO 1","723":"GRUPO 1","724":"GRUPO 1","725":"GRUPO 1","726":"GRUPO 1","727":"GRUPO 1","728":"GRUPO 1","729":"GRUPO 1","730":"GRUPO 1","731":"GRUPO 1","732":"GRUPO 2","733":"GRUPO 2","734":"GRUPO 2","735":"GRUPO 2","736":"GRUPO 2","737":"GRUPO 2","738":"GRUPO 2","739":"GRUPO 2","740":"GRUPO 2","741":"GRUPO 2","742":"GRUPO 2","743":"GRUPO 2","744":"GRUPO 3","745":"GRUPO 3","746":"GRUPO 3","747":"GRUPO 3","748":"GRUPO 3","749":"GRUPO 3","750":"GRUPO 3","751":"GRUPO 3","752":"GRUPO 3","753":"GRUPO 3","754":"GRUPO 3","755":"GRUPO 3","756":"GRUPO 4","757":"GRUPO 4","758":"GRUPO 4","759":"GRUPO 4","760":"GRUPO 4","761":"GRUPO 4","762":"GRUPO 4","763":"GRUPO 4","764":"GRUPO 4","765":"GRUPO 4","766":"GRUPO 4","767":"GRUPO 4","768":"GRUPO 1","769":"GRUPO 1","770":"GRUPO 1","771":"GRUPO 1","772":"GRUPO 1","773":"GRUPO 1","774":"GRUPO 1","775":"GRUPO 1","776":"GRUPO 1","777":"GRUPO 1","778":"GRUPO 1","779":"GRUPO 1","780":"GRUPO 2","781":"GRUPO 2","782":"GRUPO 2","783":"GRUPO 2","784":"GRUPO 2","785":"GRUPO 2","786":"GRUPO 2","787":"GRUPO 2","788":"GRUPO 2","789":"GRUPO 2","790":"GRUPO 2","791":"GRUPO 2","792":"GRUPO 3","793":"GRUPO 3","794":"GRUPO 3","795":"GRUPO 3","796":"GRUPO 3","797":"GRUPO 3","798":"GRUPO 3","799":"GRUPO 3","800":"GRUPO 3","801":"GRUPO 3","802":"GRUPO 3","803":"GRUPO 3","804":"GRUPO 4","805":"GRUPO 4","806":"GRUPO 4","807":"GRUPO 4","808":"GRUPO 4","809":"GRUPO 4","810":"GRUPO 4","811":"GRUPO 4","812":"GRUPO 4","813":"GRUPO 4","814":"GRUPO 4","815":"GRUPO 4","816":"GRUPO 1","817":"GRUPO 1","818":"GRUPO 1","819":"GRUPO 1","820":"GRUPO 1","821":"GRUPO 1","822":"GRUPO 1","823":"GRUPO 1","824":"GRUPO 1","825":"GRUPO 1","826":"GRUPO 1","827":"GRUPO 1","828":"GRUPO 2","829":"GRUPO 2","830":"GRUPO 2","831":"GRUPO 2","832":"GRUPO 2","833":"GRUPO 2","834":"GRUPO 2","835":"GRUPO 2","836":"GRUPO 2","837":"GRUPO 2","838":"GRUPO 2","839":"GRUPO 2","840":"GRUPO 3","841":"GRUPO 3","842":"GRUPO 3","843":"GRUPO 3","844":"GRUPO 3","845":"GRUPO 3","846":"GRUPO 3","847":"GRUPO 3","848":"GRUPO 3","849":"GRUPO 3","850":"GRUPO 3","851":"GRUPO 3","852":"GRUPO 4","853":"GRUPO 4","854":"GRUPO 4","855":"GRUPO 4","856":"GRUPO 4","857":"GRUPO 4","858":"GRUPO 4","859":"GRUPO 4","860":"GRUPO 4","861":"GRUPO 4","862":"GRUPO 4","863":"GRUPO 4","864":"GRUPO 1","865":"GRUPO 1","866":"GRUPO 1","867":"GRUPO 1","868":"GRUPO 1","869":"GRUPO 1","870":"GRUPO 1","871":"GRUPO 1","872":"GRUPO 1","873":"GRUPO 1","874":"GRUPO 1","875":"GRUPO 1","876":"GRUPO 2","877":"GRUPO 2","878":"GRUPO 2","879":"GRUPO 2","880":"GRUPO 2","881":"GRUPO 2","882":"GRUPO 2","883":"GRUPO 2","884":"GRUPO 2","885":"GRUPO 2","886":"GRUPO 2","887":"GRUPO 2","888":"GRUPO 3","889":"GRUPO 3","890":"GRUPO 3","891":"GRUPO 3","892":"GRUPO 3","893":"GRUPO 3","894":"GRUPO 3","895":"GRUPO 3","896":"GRUPO 3","897":"GRUPO 3","898":"GRUPO 3","899":"GRUPO 3","900":"GRUPO 4","901":"GRUPO 4","902":"GRUPO 4","903":"GRUPO 4","904":"GRUPO 4","905":"GRUPO 4","906":"GRUPO 4","907":"GRUPO 4","908":"GRUPO 4","909":"GRUPO 4","910":"GRUPO 4","911":"GRUPO 4","912":"GRUPO 1","913":"GRUPO 1","914":"GRUPO 1","915":"GRUPO 1","916":"GRUPO 1","917":"GRUPO 1","918":"GRUPO 1","919":"GRUPO 1","920":"GRUPO 1","921":"GRUPO 1","922":"GRUPO 1","923":"GRUPO 1","924":"GRUPO 2","925":"GRUPO 2","926":"GRUPO 2","927":"GRUPO 2","928":"GRUPO 2","929":"GRUPO 2","930":"GRUPO 2","931":"GRUPO 2","932":"GRUPO 2","933":"GRUPO 2","934":"GRUPO 2","935":"GRUPO 2","936":"GRUPO 3","937":"GRUPO 3","938":"GRUPO 3","939":"GRUPO 3","940":"GRUPO 3","941":"GRUPO 3","942":"GRUPO 3","943":"GRUPO 3","944":"GRUPO 3","945":"GRUPO 3","946":"GRUPO 3","947":"GRUPO 3","948":"GRUPO 4","949":"GRUPO 4","950":"GRUPO 4","951":"GRUPO 4","952":"GRUPO 4","953":"GRUPO 4","954":"GRUPO 4","955":"GRUPO 4","956":"GRUPO 4","957":"GRUPO 4","958":"GRUPO 4","959":"GRUPO 4","960":"GRUPO 1","961":"GRUPO 1","962":"GRUPO 1","963":"GRUPO 1","964":"GRUPO 1","965":"GRUPO 1","966":"GRUPO 1","967":"GRUPO 1","968":"GRUPO 1","969":"GRUPO 1","970":"GRUPO 1","971":"GRUPO 1","972":"GRUPO 2","973":"GRUPO 2","974":"GRUPO 2","975":"GRUPO 2","976":"GRUPO 2","977":"GRUPO 2","978":"GRUPO 2","979":"GRUPO 2","980":"GRUPO 2","981":"GRUPO 2","982":"GRUPO 2","983":"GRUPO 2","984":"GRUPO 3","985":"GRUPO 3","986":"GRUPO 3","987":"GRUPO 3","988":"GRUPO 3","989":"GRUPO 3","990":"GRUPO 3","991":"GRUPO 3","992":"GRUPO 3","993":"GRUPO 3","994":"GRUPO 3","995":"GRUPO 3","996":"GRUPO 4","997":"GRUPO 4","998":"GRUPO 4","999":"GRUPO 4","1000":"GRUPO 4","1001":"GRUPO 4","1002":"GRUPO 4","1003":"GRUPO 4","1004":"GRUPO 4","1005":"GRUPO 4","1006":"GRUPO 4","1007":"GRUPO 4","1008":"GRUPO 1","1009":"GRUPO 1","1010":"GRUPO 1","1011":"GRUPO 1","1012":"GRUPO 1","1013":"GRUPO 1","1014":"GRUPO 1","1015":"GRUPO 1","1016":"GRUPO 1","1017":"GRUPO 1","1018":"GRUPO 1","1019":"GRUPO 1","1020":"GRUPO 2","1021":"GRUPO 2","1022":"GRUPO 2","1023":"GRUPO 2","1024":"GRUPO 2","1025":"GRUPO 2","1026":"GRUPO 2","1027":"GRUPO 2","1028":"GRUPO 2","1029":"GRUPO 2","1030":"GRUPO 2","1031":"GRUPO 2","1032":"GRUPO 3","1033":"GRUPO 3","1034":"GRUPO 3","1035":"GRUPO 3","1036":"GRUPO 3","1037":"GRUPO 3","1038":"GRUPO 3","1039":"GRUPO 3","1040":"GRUPO 3","1041":"GRUPO 3","1042":"GRUPO 3","1043":"GRUPO 3","1044":"GRUPO 4","1045":"GRUPO 4","1046":"GRUPO 4","1047":"GRUPO 4","1048":"GRUPO 4","1049":"GRUPO 4","1050":"GRUPO 4","1051":"GRUPO 4","1052":"GRUPO 4","1053":"GRUPO 4","1054":"GRUPO 4","1055":"GRUPO 4","1056":"GRUPO 1","1057":"GRUPO 1","1058":"GRUPO 1","1059":"GRUPO 1","1060":"GRUPO 1","1061":"GRUPO 1","1062":"GRUPO 1","1063":"GRUPO 1","1064":"GRUPO 1","1065":"GRUPO 1","1066":"GRUPO 1","1067":"GRUPO 1","1068":"GRUPO 2","1069":"GRUPO 2","1070":"GRUPO 2","1071":"GRUPO 2","1072":"GRUPO 2","1073":"GRUPO 2","1074":"GRUPO 2","1075":"GRUPO 2","1076":"GRUPO 2","1077":"GRUPO 2","1078":"GRUPO 2","1079":"GRUPO 2","1080":"GRUPO 3","1081":"GRUPO 3","1082":"GRUPO 3","1083":"GRUPO 3","1084":"GRUPO 3","1085":"GRUPO 3","1086":"GRUPO 3","1087":"GRUPO 3","1088":"GRUPO 3","1089":"GRUPO 3","1090":"GRUPO 3","1091":"GRUPO 3","1092":"GRUPO 4","1093":"GRUPO 4","1094":"GRUPO 4","1095":"GRUPO 4","1096":"GRUPO 4","1097":"GRUPO 4","1098":"GRUPO 4","1099":"GRUPO 4","1100":"GRUPO 4","1101":"GRUPO 4","1102":"GRUPO 4","1103":"GRUPO 4","1104":"GRUPO 1","1105":"GRUPO 1","1106":"GRUPO 1","1107":"GRUPO 1","1108":"GRUPO 1","1109":"GRUPO 1","1110":"GRUPO 1","1111":"GRUPO 1","1112":"GRUPO 1","1113":"GRUPO 1","1114":"GRUPO 1","1115":"GRUPO 1","1116":"GRUPO 2","1117":"GRUPO 2","1118":"GRUPO 2","1119":"GRUPO 2","1120":"GRUPO 2","1121":"GRUPO 2","1122":"GRUPO 2","1123":"GRUPO 2","1124":"GRUPO 2","1125":"GRUPO 2","1126":"GRUPO 2","1127":"GRUPO 2","1128":"GRUPO 3","1129":"GRUPO 3","1130":"GRUPO 3","1131":"GRUPO 3","1132":"GRUPO 3","1133":"GRUPO 3","1134":"GRUPO 3","1135":"GRUPO 3","1136":"GRUPO 3","1137":"GRUPO 3","1138":"GRUPO 3","1139":"GRUPO 3","1140":"GRUPO 4","1141":"GRUPO 4","1142":"GRUPO 4","1143":"GRUPO 4","1144":"GRUPO 4","1145":"GRUPO 4","1146":"GRUPO 4","1147":"GRUPO 4","1148":"GRUPO 4","1149":"GRUPO 4","1150":"GRUPO 4","1151":"GRUPO 4","1152":"GRUPO 1","1153":"GRUPO 1","1154":"GRUPO 1","1155":"GRUPO 1","1156":"GRUPO 1","1157":"GRUPO 1","1158":"GRUPO 1","1159":"GRUPO 1","1160":"GRUPO 1","1161":"GRUPO 1","1162":"GRUPO 1","1163":"GRUPO 1","1164":"GRUPO 2","1165":"GRUPO 2","1166":"GRUPO 2","1167":"GRUPO 2","1168":"GRUPO 2","1169":"GRUPO 2","1170":"GRUPO 2","1171":"GRUPO 2","1172":"GRUPO 2","1173":"GRUPO 2","1174":"GRUPO 2","1175":"GRUPO 2","1176":"GRUPO 3","1177":"GRUPO 3","1178":"GRUPO 3","1179":"GRUPO 3","1180":"GRUPO 3","1181":"GRUPO 3","1182":"GRUPO 3","1183":"GRUPO 3","1184":"GRUPO 3","1185":"GRUPO 3","1186":"GRUPO 3","1187":"GRUPO 3","1188":"GRUPO 4","1189":"GRUPO 4","1190":"GRUPO 4","1191":"GRUPO 4","1192":"GRUPO 4","1193":"GRUPO 4","1194":"GRUPO 4","1195":"GRUPO 4","1196":"GRUPO 4","1197":"GRUPO 4","1198":"GRUPO 4","1199":"GRUPO 4","1200":"GRUPO 1","1201":"GRUPO 1","1202":"GRUPO 1","1203":"GRUPO 1","1204":"GRUPO 1","1205":"GRUPO 1","1206":"GRUPO 1","1207":"GRUPO 1","1208":"GRUPO 1","1209":"GRUPO 1","1210":"GRUPO 1","1211":"GRUPO 1","1212":"GRUPO 2","1213":"GRUPO 2","1214":"GRUPO 2","1215":"GRUPO 2","1216":"GRUPO 2","1217":"GRUPO 2","1218":"GRUPO 2","1219":"GRUPO 2","1220":"GRUPO 2","1221":"GRUPO 2","1222":"GRUPO 2","1223":"GRUPO 2","1224":"GRUPO 3","1225":"GRUPO 3","1226":"GRUPO 3","1227":"GRUPO 3","1228":"GRUPO 3","1229":"GRUPO 3","1230":"GRUPO 3","1231":"GRUPO 3","1232":"GRUPO 3","1233":"GRUPO 3","1234":"GRUPO 3","1235":"GRUPO 3","1236":"GRUPO 4","1237":"GRUPO 4","1238":"GRUPO 4","1239":"GRUPO 4","1240":"GRUPO 4","1241":"GRUPO 4","1242":"GRUPO 4","1243":"GRUPO 4","1244":"GRUPO 4","1245":"GRUPO 4","1246":"GRUPO 4","1247":"GRUPO 4","1248":"GRUPO 1","1249":"GRUPO 1","1250":"GRUPO 1","1251":"GRUPO 1","1252":"GRUPO 1","1253":"GRUPO 1","1254":"GRUPO 1","1255":"GRUPO 1","1256":"GRUPO 1","1257":"GRUPO 1","1258":"GRUPO 1","1259":"GRUPO 1","1260":"GRUPO 2","1261":"GRUPO 2","1262":"GRUPO 2","1263":"GRUPO 2","1264":"GRUPO 2","1265":"GRUPO 2","1266":"GRUPO 2","1267":"GRUPO 2","1268":"GRUPO 2","1269":"GRUPO 2","1270":"GRUPO 2","1271":"GRUPO 2","1272":"GRUPO 3","1273":"GRUPO 3","1274":"GRUPO 3","1275":"GRUPO 3","1276":"GRUPO 3","1277":"GRUPO 3","1278":"GRUPO 3","1279":"GRUPO 3","1280":"GRUPO 3","1281":"GRUPO 3","1282":"GRUPO 3","1283":"GRUPO 3","1284":"GRUPO 4","1285":"GRUPO 4","1286":"GRUPO 4","1287":"GRUPO 4","1288":"GRUPO 4","1289":"GRUPO 4","1290":"GRUPO 4","1291":"GRUPO 4","1292":"GRUPO 4","1293":"GRUPO 4","1294":"GRUPO 4","1295":"GRUPO 4","1296":"GRUPO 1","1297":"GRUPO 1","1298":"GRUPO 1","1299":"GRUPO 1","1300":"GRUPO 1","1301":"GRUPO 1","1302":"GRUPO 1","1303":"GRUPO 1","1304":"GRUPO 1","1305":"GRUPO 1","1306":"GRUPO 1","1307":"GRUPO 1","1308":"GRUPO 2","1309":"GRUPO 2","1310":"GRUPO 2","1311":"GRUPO 2","1312":"GRUPO 2","1313":"GRUPO 2","1314":"GRUPO 2","1315":"GRUPO 2","1316":"GRUPO 2","1317":"GRUPO 2","1318":"GRUPO 2","1319":"GRUPO 2","1320":"GRUPO 3","1321":"GRUPO 3","1322":"GRUPO 3","1323":"GRUPO 3","1324":"GRUPO 3","1325":"GRUPO 3","1326":"GRUPO 3","1327":"GRUPO 3","1328":"GRUPO 3","1329":"GRUPO 3","1330":"GRUPO 3","1331":"GRUPO 3","1332":"GRUPO 4","1333":"GRUPO 4","1334":"GRUPO 4","1335":"GRUPO 4","1336":"GRUPO 4","1337":"GRUPO 4","1338":"GRUPO 4","1339":"GRUPO 4","1340":"GRUPO 4","1341":"GRUPO 4","1342":"GRUPO 4","1343":"GRUPO 4","1344":"GRUPO 1","1345":"GRUPO 1","1346":"GRUPO 1","1347":"GRUPO 1","1348":"GRUPO 1","1349":"GRUPO 1","1350":"GRUPO 1","1351":"GRUPO 1","1352":"GRUPO 1","1353":"GRUPO 1","1354":"GRUPO 1","1355":"GRUPO 1","1356":"GRUPO 2","1357":"GRUPO 2","1358":"GRUPO 2","1359":"GRUPO 2","1360":"GRUPO 2","1361":"GRUPO 2","1362":"GRUPO 2","1363":"GRUPO 2","1364":"GRUPO 2","1365":"GRUPO 2","1366":"GRUPO 2","1367":"GRUPO 2","1368":"GRUPO 3","1369":"GRUPO 3","1370":"GRUPO 3","1371":"GRUPO 3","1372":"GRUPO 3","1373":"GRUPO 3","1374":"GRUPO 3","1375":"GRUPO 3","1376":"GRUPO 3","1377":"GRUPO 3","1378":"GRUPO 3","1379":"GRUPO 3","1380":"GRUPO 4","1381":"GRUPO 4","1382":"GRUPO 4","1383":"GRUPO 4","1384":"GRUPO 4","1385":"GRUPO 4","1386":"GRUPO 4","1387":"GRUPO 4","1388":"GRUPO 4","1389":"GRUPO 4","1390":"GRUPO 4","1391":"GRUPO 4","1392":"GRUPO 1","1393":"GRUPO 1","1394":"GRUPO 1","1395":"GRUPO 1","1396":"GRUPO 1","1397":"GRUPO 1","1398":"GRUPO 1","1399":"GRUPO 1","1400":"GRUPO 1","1401":"GRUPO 1","1402":"GRUPO 1","1403":"GRUPO 1","1404":"GRUPO 2","1405":"GRUPO 2","1406":"GRUPO 2","1407":"GRUPO 2","1408":"GRUPO 2","1409":"GRUPO 2","1410":"GRUPO 2","1411":"GRUPO 2","1412":"GRUPO 2","1413":"GRUPO 2","1414":"GRUPO 2","1415":"GRUPO 2","1416":"GRUPO 3","1417":"GRUPO 3","1418":"GRUPO 3","1419":"GRUPO 3","1420":"GRUPO 3","1421":"GRUPO 3","1422":"GRUPO 3","1423":"GRUPO 3","1424":"GRUPO 3","1425":"GRUPO 3","1426":"GRUPO 3","1427":"GRUPO 3","1428":"GRUPO 4","1429":"GRUPO 4","1430":"GRUPO 4","1431":"GRUPO 4","1432":"GRUPO 4","1433":"GRUPO 4","1434":"GRUPO 4","1435":"GRUPO 4","1436":"GRUPO 4","1437":"GRUPO 4","1438":"GRUPO 4","1439":"GRUPO 4"},"Empleado":{"0":"BARON HERNANDEZ HAROLD ANTONIO","1":"CASTELLANOS CARVAJAL DEYVITH FABIAN","2":"AROCA TORRES JULIAN EDUARDO","3":"BERMUDEZ PARRA JENNIFER XIOMARA","4":"BERNAL BAQUERO JAMES RICARDO","5":"BURGOS ORTIZ JOSE HORACIO","6":"CANTOR PORRAS JUAN FERNEY","7":"CAPERA CAPERA JOSE GABRIEL","8":"CARDENAS LOTERO RICARDO ANDR\u00c9S","9":"RENDON OSPINA NELSON LEANDRO","10":"SARMIENTO URBINA MOISES DANIEL","11":"VELASCO VELASCO SEBASTI\u00c1N DAVID","12":"DELGADO DELGADO JOHAN DARIO","13":"FLOREZ SAUCESO KENIS ALBERTO","14":"CARDONA GARCIA OSCAR JAVIER","15":"CARVAJAL GARC\u00cdA HOVER MARCK","16":"CEPEDA PIRAQUIVE JUAN DAVID","17":"FAJARDO SAENZ OSCAR FERNANDO","18":"FLOREZ ESPITIA RONY ALBERTO","19":"GARCIA CUERVO EDWIN JAVIER","20":"GONZALEZ OCHOA JUAN CARLOS","21":"XXX1","22":"XXX2","23":"XXX3","24":"FONSECA RAY RICARDO","25":"GOMEZ BETANCUR JAIDER ANDRES","26":"GRANADA PATI\u00d1O CARLOS MARINO","27":"GRASS PLATA MIGUEL SNEIDER","28":"MANZANO CALVO JUAN SEBASTIAN","29":"MENDOZA GOITA MARIANSEL ZENAYDA","30":"MURILLO ARAQUE JAIVER GEOVANY","31":"NI\u00d1O ARENAS HECTOR GONZALO","32":"RAMIREZ CHAVERRA JHON EDISON","33":"XXX4","34":"XXX5","35":"XXX6","36":"RODRIGUEZ MOSQUERA LUIS FERNANDO","37":"PEPITO PEREZ","38":"RAMIREZ VARGAS MARCELA PAOLA","39":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","40":"TORO CISNEROS GARY JOSE","41":"USECHE CALDERON JADID ESTIVEN","42":"VASQUEZ NIETO CAMILO ANDRES","43":"JHONY CASTRO","44":"BERNAL JUAN DAVID","45":"XXX7","46":"XXX8","47":"XXX9","48":"BARON HERNANDEZ HAROLD ANTONIO","49":"CASTELLANOS CARVAJAL DEYVITH FABIAN","50":"AROCA TORRES JULIAN EDUARDO","51":"BERMUDEZ PARRA JENNIFER XIOMARA","52":"BERNAL BAQUERO JAMES RICARDO","53":"BURGOS ORTIZ JOSE HORACIO","54":"CANTOR PORRAS JUAN FERNEY","55":"CAPERA CAPERA JOSE GABRIEL","56":"CARDENAS LOTERO RICARDO ANDR\u00c9S","57":"RENDON OSPINA NELSON LEANDRO","58":"SARMIENTO URBINA MOISES DANIEL","59":"VELASCO VELASCO SEBASTI\u00c1N DAVID","60":"DELGADO DELGADO JOHAN DARIO","61":"FLOREZ SAUCESO KENIS ALBERTO","62":"CARDONA GARCIA OSCAR JAVIER","63":"CARVAJAL GARC\u00cdA HOVER MARCK","64":"CEPEDA PIRAQUIVE JUAN DAVID","65":"FAJARDO SAENZ OSCAR FERNANDO","66":"FLOREZ ESPITIA RONY ALBERTO","67":"GARCIA CUERVO EDWIN JAVIER","68":"GONZALEZ OCHOA JUAN CARLOS","69":"XXX1","70":"XXX2","71":"XXX3","72":"FONSECA RAY RICARDO","73":"GOMEZ BETANCUR JAIDER ANDRES","74":"GRANADA PATI\u00d1O CARLOS MARINO","75":"GRASS PLATA MIGUEL SNEIDER","76":"MANZANO CALVO JUAN SEBASTIAN","77":"MENDOZA GOITA MARIANSEL ZENAYDA","78":"MURILLO ARAQUE JAIVER GEOVANY","79":"NI\u00d1O ARENAS HECTOR GONZALO","80":"RAMIREZ CHAVERRA JHON EDISON","81":"XXX4","82":"XXX5","83":"XXX6","84":"RODRIGUEZ MOSQUERA LUIS FERNANDO","85":"PEPITO PEREZ","86":"RAMIREZ VARGAS MARCELA PAOLA","87":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","88":"TORO CISNEROS GARY JOSE","89":"USECHE CALDERON JADID ESTIVEN","90":"VASQUEZ NIETO CAMILO ANDRES","91":"JHONY CASTRO","92":"BERNAL JUAN DAVID","93":"XXX7","94":"XXX8","95":"XXX9","96":"BARON HERNANDEZ HAROLD ANTONIO","97":"CASTELLANOS CARVAJAL DEYVITH FABIAN","98":"AROCA TORRES JULIAN EDUARDO","99":"BERMUDEZ PARRA JENNIFER XIOMARA","100":"BERNAL BAQUERO JAMES RICARDO","101":"BURGOS ORTIZ JOSE HORACIO","102":"CANTOR PORRAS JUAN FERNEY","103":"CAPERA CAPERA JOSE GABRIEL","104":"CARDENAS LOTERO RICARDO ANDR\u00c9S","105":"RENDON OSPINA NELSON LEANDRO","106":"SARMIENTO URBINA MOISES DANIEL","107":"VELASCO VELASCO SEBASTI\u00c1N DAVID","108":"DELGADO DELGADO JOHAN DARIO","109":"FLOREZ SAUCESO KENIS ALBERTO","110":"CARDONA GARCIA OSCAR JAVIER","111":"CARVAJAL GARC\u00cdA HOVER MARCK","112":"CEPEDA PIRAQUIVE JUAN DAVID","113":"FAJARDO SAENZ OSCAR FERNANDO","114":"FLOREZ ESPITIA RONY ALBERTO","115":"GARCIA CUERVO EDWIN JAVIER","116":"GONZALEZ OCHOA JUAN CARLOS","117":"XXX1","118":"XXX2","119":"XXX3","120":"FONSECA RAY RICARDO","121":"GOMEZ BETANCUR JAIDER ANDRES","122":"GRANADA PATI\u00d1O CARLOS MARINO","123":"GRASS PLATA MIGUEL SNEIDER","124":"MANZANO CALVO JUAN SEBASTIAN","125":"MENDOZA GOITA MARIANSEL ZENAYDA","126":"MURILLO ARAQUE JAIVER GEOVANY","127":"NI\u00d1O ARENAS HECTOR GONZALO","128":"RAMIREZ CHAVERRA JHON EDISON","129":"XXX4","130":"XXX5","131":"XXX6","132":"RODRIGUEZ MOSQUERA LUIS FERNANDO","133":"PEPITO PEREZ","134":"RAMIREZ VARGAS MARCELA PAOLA","135":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","136":"TORO CISNEROS GARY JOSE","137":"USECHE CALDERON JADID ESTIVEN","138":"VASQUEZ NIETO CAMILO ANDRES","139":"JHONY CASTRO","140":"BERNAL JUAN DAVID","141":"XXX7","142":"XXX8","143":"XXX9","144":"BARON HERNANDEZ HAROLD ANTONIO","145":"CASTELLANOS CARVAJAL DEYVITH FABIAN","146":"AROCA TORRES JULIAN EDUARDO","147":"BERMUDEZ PARRA JENNIFER XIOMARA","148":"BERNAL BAQUERO JAMES RICARDO","149":"BURGOS ORTIZ JOSE HORACIO","150":"CANTOR PORRAS JUAN FERNEY","151":"CAPERA CAPERA JOSE GABRIEL","152":"CARDENAS LOTERO RICARDO ANDR\u00c9S","153":"RENDON OSPINA NELSON LEANDRO","154":"SARMIENTO URBINA MOISES DANIEL","155":"VELASCO VELASCO SEBASTI\u00c1N DAVID","156":"DELGADO DELGADO JOHAN DARIO","157":"FLOREZ SAUCESO KENIS ALBERTO","158":"CARDONA GARCIA OSCAR JAVIER","159":"CARVAJAL GARC\u00cdA HOVER MARCK","160":"CEPEDA PIRAQUIVE JUAN DAVID","161":"FAJARDO SAENZ OSCAR FERNANDO","162":"FLOREZ ESPITIA RONY ALBERTO","163":"GARCIA CUERVO EDWIN JAVIER","164":"GONZALEZ OCHOA JUAN CARLOS","165":"XXX1","166":"XXX2","167":"XXX3","168":"FONSECA RAY RICARDO","169":"GOMEZ BETANCUR JAIDER ANDRES","170":"GRANADA PATI\u00d1O CARLOS MARINO","171":"GRASS PLATA MIGUEL SNEIDER","172":"MANZANO CALVO JUAN SEBASTIAN","173":"MENDOZA GOITA MARIANSEL ZENAYDA","174":"MURILLO ARAQUE JAIVER GEOVANY","175":"NI\u00d1O ARENAS HECTOR GONZALO","176":"RAMIREZ CHAVERRA JHON EDISON","177":"XXX4","178":"XXX5","179":"XXX6","180":"RODRIGUEZ MOSQUERA LUIS FERNANDO","181":"PEPITO PEREZ","182":"RAMIREZ VARGAS MARCELA PAOLA","183":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","184":"TORO CISNEROS GARY JOSE","185":"USECHE CALDERON JADID ESTIVEN","186":"VASQUEZ NIETO CAMILO ANDRES","187":"JHONY CASTRO","188":"BERNAL JUAN DAVID","189":"XXX7","190":"XXX8","191":"XXX9","192":"BARON HERNANDEZ HAROLD ANTONIO","193":"CASTELLANOS CARVAJAL DEYVITH FABIAN","194":"AROCA TORRES JULIAN EDUARDO","195":"BERMUDEZ PARRA JENNIFER XIOMARA","196":"BERNAL BAQUERO JAMES RICARDO","197":"BURGOS ORTIZ JOSE HORACIO","198":"CANTOR PORRAS JUAN FERNEY","199":"CAPERA CAPERA JOSE GABRIEL","200":"CARDENAS LOTERO RICARDO ANDR\u00c9S","201":"RENDON OSPINA NELSON LEANDRO","202":"SARMIENTO URBINA MOISES DANIEL","203":"VELASCO VELASCO SEBASTI\u00c1N DAVID","204":"DELGADO DELGADO JOHAN DARIO","205":"FLOREZ SAUCESO KENIS ALBERTO","206":"CARDONA GARCIA OSCAR JAVIER","207":"CARVAJAL GARC\u00cdA HOVER MARCK","208":"CEPEDA PIRAQUIVE JUAN DAVID","209":"FAJARDO SAENZ OSCAR FERNANDO","210":"FLOREZ ESPITIA RONY ALBERTO","211":"GARCIA CUERVO EDWIN JAVIER","212":"GONZALEZ OCHOA JUAN CARLOS","213":"XXX1","214":"XXX2","215":"XXX3","216":"FONSECA RAY RICARDO","217":"GOMEZ BETANCUR JAIDER ANDRES","218":"GRANADA PATI\u00d1O CARLOS MARINO","219":"GRASS PLATA MIGUEL SNEIDER","220":"MANZANO CALVO JUAN SEBASTIAN","221":"MENDOZA GOITA MARIANSEL ZENAYDA","222":"MURILLO ARAQUE JAIVER GEOVANY","223":"NI\u00d1O ARENAS HECTOR GONZALO","224":"RAMIREZ CHAVERRA JHON EDISON","225":"XXX4","226":"XXX5","227":"XXX6","228":"RODRIGUEZ MOSQUERA LUIS FERNANDO","229":"PEPITO PEREZ","230":"RAMIREZ VARGAS MARCELA PAOLA","231":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","232":"TORO CISNEROS GARY JOSE","233":"USECHE CALDERON JADID ESTIVEN","234":"VASQUEZ NIETO CAMILO ANDRES","235":"JHONY CASTRO","236":"BERNAL JUAN DAVID","237":"XXX7","238":"XXX8","239":"XXX9","240":"BARON HERNANDEZ HAROLD ANTONIO","241":"CASTELLANOS CARVAJAL DEYVITH FABIAN","242":"AROCA TORRES JULIAN EDUARDO","243":"BERMUDEZ PARRA JENNIFER XIOMARA","244":"BERNAL BAQUERO JAMES RICARDO","245":"BURGOS ORTIZ JOSE HORACIO","246":"CANTOR PORRAS JUAN FERNEY","247":"CAPERA CAPERA JOSE GABRIEL","248":"CARDENAS LOTERO RICARDO ANDR\u00c9S","249":"RENDON OSPINA NELSON LEANDRO","250":"SARMIENTO URBINA MOISES DANIEL","251":"VELASCO VELASCO SEBASTI\u00c1N DAVID","252":"DELGADO DELGADO JOHAN DARIO","253":"FLOREZ SAUCESO KENIS ALBERTO","254":"CARDONA GARCIA OSCAR JAVIER","255":"CARVAJAL GARC\u00cdA HOVER MARCK","256":"CEPEDA PIRAQUIVE JUAN DAVID","257":"FAJARDO SAENZ OSCAR FERNANDO","258":"FLOREZ ESPITIA RONY ALBERTO","259":"GARCIA CUERVO EDWIN JAVIER","260":"GONZALEZ OCHOA JUAN CARLOS","261":"XXX1","262":"XXX2","263":"XXX3","264":"FONSECA RAY RICARDO","265":"GOMEZ BETANCUR JAIDER ANDRES","266":"GRANADA PATI\u00d1O CARLOS MARINO","267":"GRASS PLATA MIGUEL SNEIDER","268":"MANZANO CALVO JUAN SEBASTIAN","269":"MENDOZA GOITA MARIANSEL ZENAYDA","270":"MURILLO ARAQUE JAIVER GEOVANY","271":"NI\u00d1O ARENAS HECTOR GONZALO","272":"RAMIREZ CHAVERRA JHON EDISON","273":"XXX4","274":"XXX5","275":"XXX6","276":"RODRIGUEZ MOSQUERA LUIS FERNANDO","277":"PEPITO PEREZ","278":"RAMIREZ VARGAS MARCELA PAOLA","279":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","280":"TORO CISNEROS GARY JOSE","281":"USECHE CALDERON JADID ESTIVEN","282":"VASQUEZ NIETO CAMILO ANDRES","283":"JHONY CASTRO","284":"BERNAL JUAN DAVID","285":"XXX7","286":"XXX8","287":"XXX9","288":"BARON HERNANDEZ HAROLD ANTONIO","289":"CASTELLANOS CARVAJAL DEYVITH FABIAN","290":"AROCA TORRES JULIAN EDUARDO","291":"BERMUDEZ PARRA JENNIFER XIOMARA","292":"BERNAL BAQUERO JAMES RICARDO","293":"BURGOS ORTIZ JOSE</t>
-  </si>
-  <si>
-    <t>{"Grupo":{"0":"GRUPO 1","1":"GRUPO 1","2":"GRUPO 1","3":"GRUPO 1","4":"GRUPO 1","5":"GRUPO 1","6":"GRUPO 1","7":"GRUPO 1","8":"GRUPO 1","9":"GRUPO 1","10":"GRUPO 1","11":"GRUPO 1","12":"GRUPO 2","13":"GRUPO 2","14":"GRUPO 2","15":"GRUPO 2","16":"GRUPO 2","17":"GRUPO 2","18":"GRUPO 2","19":"GRUPO 2","20":"GRUPO 2","21":"GRUPO 2","22":"GRUPO 2","23":"GRUPO 2","24":"GRUPO 3","25":"GRUPO 3","26":"GRUPO 3","27":"GRUPO 3","28":"GRUPO 3","29":"GRUPO 3","30":"GRUPO 3","31":"GRUPO 3","32":"GRUPO 3","33":"GRUPO 3","34":"GRUPO 3","35":"GRUPO 3","36":"GRUPO 4","37":"GRUPO 4","38":"GRUPO 4","39":"GRUPO 4","40":"GRUPO 4","41":"GRUPO 4","42":"GRUPO 4","43":"GRUPO 4","44":"GRUPO 4","45":"GRUPO 4","46":"GRUPO 4","47":"GRUPO 4","48":"GRUPO 1","49":"GRUPO 1","50":"GRUPO 1","51":"GRUPO 1","52":"GRUPO 1","53":"GRUPO 1","54":"GRUPO 1","55":"GRUPO 1","56":"GRUPO 1","57":"GRUPO 1","58":"GRUPO 1","59":"GRUPO 1","60":"GRUPO 2","61":"GRUPO 2","62":"GRUPO 2","63":"GRUPO 2","64":"GRUPO 2","65":"GRUPO 2","66":"GRUPO 2","67":"GRUPO 2","68":"GRUPO 2","69":"GRUPO 2","70":"GRUPO 2","71":"GRUPO 2","72":"GRUPO 3","73":"GRUPO 3","74":"GRUPO 3","75":"GRUPO 3","76":"GRUPO 3","77":"GRUPO 3","78":"GRUPO 3","79":"GRUPO 3","80":"GRUPO 3","81":"GRUPO 3","82":"GRUPO 3","83":"GRUPO 3","84":"GRUPO 4","85":"GRUPO 4","86":"GRUPO 4","87":"GRUPO 4","88":"GRUPO 4","89":"GRUPO 4","90":"GRUPO 4","91":"GRUPO 4","92":"GRUPO 4","93":"GRUPO 4","94":"GRUPO 4","95":"GRUPO 4","96":"GRUPO 1","97":"GRUPO 1","98":"GRUPO 1","99":"GRUPO 1","100":"GRUPO 1","101":"GRUPO 1","102":"GRUPO 1","103":"GRUPO 1","104":"GRUPO 1","105":"GRUPO 1","106":"GRUPO 1","107":"GRUPO 1","108":"GRUPO 2","109":"GRUPO 2","110":"GRUPO 2","111":"GRUPO 2","112":"GRUPO 2","113":"GRUPO 2","114":"GRUPO 2","115":"GRUPO 2","116":"GRUPO 2","117":"GRUPO 2","118":"GRUPO 2","119":"GRUPO 2","120":"GRUPO 3","121":"GRUPO 3","122":"GRUPO 3","123":"GRUPO 3","124":"GRUPO 3","125":"GRUPO 3","126":"GRUPO 3","127":"GRUPO 3","128":"GRUPO 3","129":"GRUPO 3","130":"GRUPO 3","131":"GRUPO 3","132":"GRUPO 4","133":"GRUPO 4","134":"GRUPO 4","135":"GRUPO 4","136":"GRUPO 4","137":"GRUPO 4","138":"GRUPO 4","139":"GRUPO 4","140":"GRUPO 4","141":"GRUPO 4","142":"GRUPO 4","143":"GRUPO 4","144":"GRUPO 1","145":"GRUPO 1","146":"GRUPO 1","147":"GRUPO 1","148":"GRUPO 1","149":"GRUPO 1","150":"GRUPO 1","151":"GRUPO 1","152":"GRUPO 1","153":"GRUPO 1","154":"GRUPO 1","155":"GRUPO 1","156":"GRUPO 2","157":"GRUPO 2","158":"GRUPO 2","159":"GRUPO 2","160":"GRUPO 2","161":"GRUPO 2","162":"GRUPO 2","163":"GRUPO 2","164":"GRUPO 2","165":"GRUPO 2","166":"GRUPO 2","167":"GRUPO 2","168":"GRUPO 3","169":"GRUPO 3","170":"GRUPO 3","171":"GRUPO 3","172":"GRUPO 3","173":"GRUPO 3","174":"GRUPO 3","175":"GRUPO 3","176":"GRUPO 3","177":"GRUPO 3","178":"GRUPO 3","179":"GRUPO 3","180":"GRUPO 4","181":"GRUPO 4","182":"GRUPO 4","183":"GRUPO 4","184":"GRUPO 4","185":"GRUPO 4","186":"GRUPO 4","187":"GRUPO 4","188":"GRUPO 4","189":"GRUPO 4","190":"GRUPO 4","191":"GRUPO 4","192":"GRUPO 1","193":"GRUPO 1","194":"GRUPO 1","195":"GRUPO 1","196":"GRUPO 1","197":"GRUPO 1","198":"GRUPO 1","199":"GRUPO 1","200":"GRUPO 1","201":"GRUPO 1","202":"GRUPO 1","203":"GRUPO 1","204":"GRUPO 2","205":"GRUPO 2","206":"GRUPO 2","207":"GRUPO 2","208":"GRUPO 2","209":"GRUPO 2","210":"GRUPO 2","211":"GRUPO 2","212":"GRUPO 2","213":"GRUPO 2","214":"GRUPO 2","215":"GRUPO 2","216":"GRUPO 3","217":"GRUPO 3","218":"GRUPO 3","219":"GRUPO 3","220":"GRUPO 3","221":"GRUPO 3","222":"GRUPO 3","223":"GRUPO 3","224":"GRUPO 3","225":"GRUPO 3","226":"GRUPO 3","227":"GRUPO 3","228":"GRUPO 4","229":"GRUPO 4","230":"GRUPO 4","231":"GRUPO 4","232":"GRUPO 4","233":"GRUPO 4","234":"GRUPO 4","235":"GRUPO 4","236":"GRUPO 4","237":"GRUPO 4","238":"GRUPO 4","239":"GRUPO 4","240":"GRUPO 1","241":"GRUPO 1","242":"GRUPO 1","243":"GRUPO 1","244":"GRUPO 1","245":"GRUPO 1","246":"GRUPO 1","247":"GRUPO 1","248":"GRUPO 1","249":"GRUPO 1","250":"GRUPO 1","251":"GRUPO 1","252":"GRUPO 2","253":"GRUPO 2","254":"GRUPO 2","255":"GRUPO 2","256":"GRUPO 2","257":"GRUPO 2","258":"GRUPO 2","259":"GRUPO 2","260":"GRUPO 2","261":"GRUPO 2","262":"GRUPO 2","263":"GRUPO 2","264":"GRUPO 3","265":"GRUPO 3","266":"GRUPO 3","267":"GRUPO 3","268":"GRUPO 3","269":"GRUPO 3","270":"GRUPO 3","271":"GRUPO 3","272":"GRUPO 3","273":"GRUPO 3","274":"GRUPO 3","275":"GRUPO 3","276":"GRUPO 4","277":"GRUPO 4","278":"GRUPO 4","279":"GRUPO 4","280":"GRUPO 4","281":"GRUPO 4","282":"GRUPO 4","283":"GRUPO 4","284":"GRUPO 4","285":"GRUPO 4","286":"GRUPO 4","287":"GRUPO 4","288":"GRUPO 1","289":"GRUPO 1","290":"GRUPO 1","291":"GRUPO 1","292":"GRUPO 1","293":"GRUPO 1","294":"GRUPO 1","295":"GRUPO 1","296":"GRUPO 1","297":"GRUPO 1","298":"GRUPO 1","299":"GRUPO 1","300":"GRUPO 2","301":"GRUPO 2","302":"GRUPO 2","303":"GRUPO 2","304":"GRUPO 2","305":"GRUPO 2","306":"GRUPO 2","307":"GRUPO 2","308":"GRUPO 2","309":"GRUPO 2","310":"GRUPO 2","311":"GRUPO 2","312":"GRUPO 3","313":"GRUPO 3","314":"GRUPO 3","315":"GRUPO 3","316":"GRUPO 3","317":"GRUPO 3","318":"GRUPO 3","319":"GRUPO 3","320":"GRUPO 3","321":"GRUPO 3","322":"GRUPO 3","323":"GRUPO 3","324":"GRUPO 4","325":"GRUPO 4","326":"GRUPO 4","327":"GRUPO 4","328":"GRUPO 4","329":"GRUPO 4","330":"GRUPO 4","331":"GRUPO 4","332":"GRUPO 4","333":"GRUPO 4","334":"GRUPO 4","335":"GRUPO 4","336":"GRUPO 1","337":"GRUPO 1","338":"GRUPO 1","339":"GRUPO 1","340":"GRUPO 1","341":"GRUPO 1","342":"GRUPO 1","343":"GRUPO 1","344":"GRUPO 1","345":"GRUPO 1","346":"GRUPO 1","347":"GRUPO 1","348":"GRUPO 2","349":"GRUPO 2","350":"GRUPO 2","351":"GRUPO 2","352":"GRUPO 2","353":"GRUPO 2","354":"GRUPO 2","355":"GRUPO 2","356":"GRUPO 2","357":"GRUPO 2","358":"GRUPO 2","359":"GRUPO 2","360":"GRUPO 3","361":"GRUPO 3","362":"GRUPO 3","363":"GRUPO 3","364":"GRUPO 3","365":"GRUPO 3","366":"GRUPO 3","367":"GRUPO 3","368":"GRUPO 3","369":"GRUPO 3","370":"GRUPO 3","371":"GRUPO 3","372":"GRUPO 4","373":"GRUPO 4","374":"GRUPO 4","375":"GRUPO 4","376":"GRUPO 4","377":"GRUPO 4","378":"GRUPO 4","379":"GRUPO 4","380":"GRUPO 4","381":"GRUPO 4","382":"GRUPO 4","383":"GRUPO 4","384":"GRUPO 1","385":"GRUPO 1","386":"GRUPO 1","387":"GRUPO 1","388":"GRUPO 1","389":"GRUPO 1","390":"GRUPO 1","391":"GRUPO 1","392":"GRUPO 1","393":"GRUPO 1","394":"GRUPO 1","395":"GRUPO 1","396":"GRUPO 2","397":"GRUPO 2","398":"GRUPO 2","399":"GRUPO 2","400":"GRUPO 2","401":"GRUPO 2","402":"GRUPO 2","403":"GRUPO 2","404":"GRUPO 2","405":"GRUPO 2","406":"GRUPO 2","407":"GRUPO 2","408":"GRUPO 3","409":"GRUPO 3","410":"GRUPO 3","411":"GRUPO 3","412":"GRUPO 3","413":"GRUPO 3","414":"GRUPO 3","415":"GRUPO 3","416":"GRUPO 3","417":"GRUPO 3","418":"GRUPO 3","419":"GRUPO 3","420":"GRUPO 4","421":"GRUPO 4","422":"GRUPO 4","423":"GRUPO 4","424":"GRUPO 4","425":"GRUPO 4","426":"GRUPO 4","427":"GRUPO 4","428":"GRUPO 4","429":"GRUPO 4","430":"GRUPO 4","431":"GRUPO 4","432":"GRUPO 1","433":"GRUPO 1","434":"GRUPO 1","435":"GRUPO 1","436":"GRUPO 1","437":"GRUPO 1","438":"GRUPO 1","439":"GRUPO 1","440":"GRUPO 1","441":"GRUPO 1","442":"GRUPO 1","443":"GRUPO 1","444":"GRUPO 2","445":"GRUPO 2","446":"GRUPO 2","447":"GRUPO 2","448":"GRUPO 2","449":"GRUPO 2","450":"GRUPO 2","451":"GRUPO 2","452":"GRUPO 2","453":"GRUPO 2","454":"GRUPO 2","455":"GRUPO 2","456":"GRUPO 3","457":"GRUPO 3","458":"GRUPO 3","459":"GRUPO 3","460":"GRUPO 3","461":"GRUPO 3","462":"GRUPO 3","463":"GRUPO 3","464":"GRUPO 3","465":"GRUPO 3","466":"GRUPO 3","467":"GRUPO 3","468":"GRUPO 4","469":"GRUPO 4","470":"GRUPO 4","471":"GRUPO 4","472":"GRUPO 4","473":"GRUPO 4","474":"GRUPO 4","475":"GRUPO 4","476":"GRUPO 4","477":"GRUPO 4","478":"GRUPO 4","479":"GRUPO 4","480":"GRUPO 1","481":"GRUPO 1","482":"GRUPO 1","483":"GRUPO 1","484":"GRUPO 1","485":"GRUPO 1","486":"GRUPO 1","487":"GRUPO 1","488":"GRUPO 1","489":"GRUPO 1","490":"GRUPO 1","491":"GRUPO 1","492":"GRUPO 2","493":"GRUPO 2","494":"GRUPO 2","495":"GRUPO 2","496":"GRUPO 2","497":"GRUPO 2","498":"GRUPO 2","499":"GRUPO 2","500":"GRUPO 2","501":"GRUPO 2","502":"GRUPO 2","503":"GRUPO 2","504":"GRUPO 3","505":"GRUPO 3","506":"GRUPO 3","507":"GRUPO 3","508":"GRUPO 3","509":"GRUPO 3","510":"GRUPO 3","511":"GRUPO 3","512":"GRUPO 3","513":"GRUPO 3","514":"GRUPO 3","515":"GRUPO 3","516":"GRUPO 4","517":"GRUPO 4","518":"GRUPO 4","519":"GRUPO 4","520":"GRUPO 4","521":"GRUPO 4","522":"GRUPO 4","523":"GRUPO 4","524":"GRUPO 4","525":"GRUPO 4","526":"GRUPO 4","527":"GRUPO 4","528":"GRUPO 1","529":"GRUPO 1","530":"GRUPO 1","531":"GRUPO 1","532":"GRUPO 1","533":"GRUPO 1","534":"GRUPO 1","535":"GRUPO 1","536":"GRUPO 1","537":"GRUPO 1","538":"GRUPO 1","539":"GRUPO 1","540":"GRUPO 2","541":"GRUPO 2","542":"GRUPO 2","543":"GRUPO 2","544":"GRUPO 2","545":"GRUPO 2","546":"GRUPO 2","547":"GRUPO 2","548":"GRUPO 2","549":"GRUPO 2","550":"GRUPO 2","551":"GRUPO 2","552":"GRUPO 3","553":"GRUPO 3","554":"GRUPO 3","555":"GRUPO 3","556":"GRUPO 3","557":"GRUPO 3","558":"GRUPO 3","559":"GRUPO 3","560":"GRUPO 3","561":"GRUPO 3","562":"GRUPO 3","563":"GRUPO 3","564":"GRUPO 4","565":"GRUPO 4","566":"GRUPO 4","567":"GRUPO 4","568":"GRUPO 4","569":"GRUPO 4","570":"GRUPO 4","571":"GRUPO 4","572":"GRUPO 4","573":"GRUPO 4","574":"GRUPO 4","575":"GRUPO 4","576":"GRUPO 1","577":"GRUPO 1","578":"GRUPO 1","579":"GRUPO 1","580":"GRUPO 1","581":"GRUPO 1","582":"GRUPO 1","583":"GRUPO 1","584":"GRUPO 1","585":"GRUPO 1","586":"GRUPO 1","587":"GRUPO 1","588":"GRUPO 2","589":"GRUPO 2","590":"GRUPO 2","591":"GRUPO 2","592":"GRUPO 2","593":"GRUPO 2","594":"GRUPO 2","595":"GRUPO 2","596":"GRUPO 2","597":"GRUPO 2","598":"GRUPO 2","599":"GRUPO 2","600":"GRUPO 3","601":"GRUPO 3","602":"GRUPO 3","603":"GRUPO 3","604":"GRUPO 3","605":"GRUPO 3","606":"GRUPO 3","607":"GRUPO 3","608":"GRUPO 3","609":"GRUPO 3","610":"GRUPO 3","611":"GRUPO 3","612":"GRUPO 4","613":"GRUPO 4","614":"GRUPO 4","615":"GRUPO 4","616":"GRUPO 4","617":"GRUPO 4","618":"GRUPO 4","619":"GRUPO 4","620":"GRUPO 4","621":"GRUPO 4","622":"GRUPO 4","623":"GRUPO 4","624":"GRUPO 1","625":"GRUPO 1","626":"GRUPO 1","627":"GRUPO 1","628":"GRUPO 1","629":"GRUPO 1","630":"GRUPO 1","631":"GRUPO 1","632":"GRUPO 1","633":"GRUPO 1","634":"GRUPO 1","635":"GRUPO 1","636":"GRUPO 2","637":"GRUPO 2","638":"GRUPO 2","639":"GRUPO 2","640":"GRUPO 2","641":"GRUPO 2","642":"GRUPO 2","643":"GRUPO 2","644":"GRUPO 2","645":"GRUPO 2","646":"GRUPO 2","647":"GRUPO 2","648":"GRUPO 3","649":"GRUPO 3","650":"GRUPO 3","651":"GRUPO 3","652":"GRUPO 3","653":"GRUPO 3","654":"GRUPO 3","655":"GRUPO 3","656":"GRUPO 3","657":"GRUPO 3","658":"GRUPO 3","659":"GRUPO 3","660":"GRUPO 4","661":"GRUPO 4","662":"GRUPO 4","663":"GRUPO 4","664":"GRUPO 4","665":"GRUPO 4","666":"GRUPO 4","667":"GRUPO 4","668":"GRUPO 4","669":"GRUPO 4","670":"GRUPO 4","671":"GRUPO 4","672":"GRUPO 1","673":"GRUPO 1","674":"GRUPO 1","675":"GRUPO 1","676":"GRUPO 1","677":"GRUPO 1","678":"GRUPO 1","679":"GRUPO 1","680":"GRUPO 1","681":"GRUPO 1","682":"GRUPO 1","683":"GRUPO 1","684":"GRUPO 2","685":"GRUPO 2","686":"GRUPO 2","687":"GRUPO 2","688":"GRUPO 2","689":"GRUPO 2","690":"GRUPO 2","691":"GRUPO 2","692":"GRUPO 2","693":"GRUPO 2","694":"GRUPO 2","695":"GRUPO 2","696":"GRUPO 3","697":"GRUPO 3","698":"GRUPO 3","699":"GRUPO 3","700":"GRUPO 3","701":"GRUPO 3","702":"GRUPO 3","703":"GRUPO 3","704":"GRUPO 3","705":"GRUPO 3","706":"GRUPO 3","707":"GRUPO 3","708":"GRUPO 4","709":"GRUPO 4","710":"GRUPO 4","711":"GRUPO 4","712":"GRUPO 4","713":"GRUPO 4","714":"GRUPO 4","715":"GRUPO 4","716":"GRUPO 4","717":"GRUPO 4","718":"GRUPO 4","719":"GRUPO 4","720":"GRUPO 1","721":"GRUPO 1","722":"GRUPO 1","723":"GRUPO 1","724":"GRUPO 1","725":"GRUPO 1","726":"GRUPO 1","727":"GRUPO 1","728":"GRUPO 1","729":"GRUPO 1","730":"GRUPO 1","731":"GRUPO 1","732":"GRUPO 2","733":"GRUPO 2","734":"GRUPO 2","735":"GRUPO 2","736":"GRUPO 2","737":"GRUPO 2","738":"GRUPO 2","739":"GRUPO 2","740":"GRUPO 2","741":"GRUPO 2","742":"GRUPO 2","743":"GRUPO 2","744":"GRUPO 3","745":"GRUPO 3","746":"GRUPO 3","747":"GRUPO 3","748":"GRUPO 3","749":"GRUPO 3","750":"GRUPO 3","751":"GRUPO 3","752":"GRUPO 3","753":"GRUPO 3","754":"GRUPO 3","755":"GRUPO 3","756":"GRUPO 4","757":"GRUPO 4","758":"GRUPO 4","759":"GRUPO 4","760":"GRUPO 4","761":"GRUPO 4","762":"GRUPO 4","763":"GRUPO 4","764":"GRUPO 4","765":"GRUPO 4","766":"GRUPO 4","767":"GRUPO 4","768":"GRUPO 1","769":"GRUPO 1","770":"GRUPO 1","771":"GRUPO 1","772":"GRUPO 1","773":"GRUPO 1","774":"GRUPO 1","775":"GRUPO 1","776":"GRUPO 1","777":"GRUPO 1","778":"GRUPO 1","779":"GRUPO 1","780":"GRUPO 2","781":"GRUPO 2","782":"GRUPO 2","783":"GRUPO 2","784":"GRUPO 2","785":"GRUPO 2","786":"GRUPO 2","787":"GRUPO 2","788":"GRUPO 2","789":"GRUPO 2","790":"GRUPO 2","791":"GRUPO 2","792":"GRUPO 3","793":"GRUPO 3","794":"GRUPO 3","795":"GRUPO 3","796":"GRUPO 3","797":"GRUPO 3","798":"GRUPO 3","799":"GRUPO 3","800":"GRUPO 3","801":"GRUPO 3","802":"GRUPO 3","803":"GRUPO 3","804":"GRUPO 4","805":"GRUPO 4","806":"GRUPO 4","807":"GRUPO 4","808":"GRUPO 4","809":"GRUPO 4","810":"GRUPO 4","811":"GRUPO 4","812":"GRUPO 4","813":"GRUPO 4","814":"GRUPO 4","815":"GRUPO 4","816":"GRUPO 1","817":"GRUPO 1","818":"GRUPO 1","819":"GRUPO 1","820":"GRUPO 1","821":"GRUPO 1","822":"GRUPO 1","823":"GRUPO 1","824":"GRUPO 1","825":"GRUPO 1","826":"GRUPO 1","827":"GRUPO 1","828":"GRUPO 2","829":"GRUPO 2","830":"GRUPO 2","831":"GRUPO 2","832":"GRUPO 2","833":"GRUPO 2","834":"GRUPO 2","835":"GRUPO 2","836":"GRUPO 2","837":"GRUPO 2","838":"GRUPO 2","839":"GRUPO 2","840":"GRUPO 3","841":"GRUPO 3","842":"GRUPO 3","843":"GRUPO 3","844":"GRUPO 3","845":"GRUPO 3","846":"GRUPO 3","847":"GRUPO 3","848":"GRUPO 3","849":"GRUPO 3","850":"GRUPO 3","851":"GRUPO 3","852":"GRUPO 4","853":"GRUPO 4","854":"GRUPO 4","855":"GRUPO 4","856":"GRUPO 4","857":"GRUPO 4","858":"GRUPO 4","859":"GRUPO 4","860":"GRUPO 4","861":"GRUPO 4","862":"GRUPO 4","863":"GRUPO 4","864":"GRUPO 1","865":"GRUPO 1","866":"GRUPO 1","867":"GRUPO 1","868":"GRUPO 1","869":"GRUPO 1","870":"GRUPO 1","871":"GRUPO 1","872":"GRUPO 1","873":"GRUPO 1","874":"GRUPO 1","875":"GRUPO 1","876":"GRUPO 2","877":"GRUPO 2","878":"GRUPO 2","879":"GRUPO 2","880":"GRUPO 2","881":"GRUPO 2","882":"GRUPO 2","883":"GRUPO 2","884":"GRUPO 2","885":"GRUPO 2","886":"GRUPO 2","887":"GRUPO 2","888":"GRUPO 3","889":"GRUPO 3","890":"GRUPO 3","891":"GRUPO 3","892":"GRUPO 3","893":"GRUPO 3","894":"GRUPO 3","895":"GRUPO 3","896":"GRUPO 3","897":"GRUPO 3","898":"GRUPO 3","899":"GRUPO 3","900":"GRUPO 4","901":"GRUPO 4","902":"GRUPO 4","903":"GRUPO 4","904":"GRUPO 4","905":"GRUPO 4","906":"GRUPO 4","907":"GRUPO 4","908":"GRUPO 4","909":"GRUPO 4","910":"GRUPO 4","911":"GRUPO 4","912":"GRUPO 1","913":"GRUPO 1","914":"GRUPO 1","915":"GRUPO 1","916":"GRUPO 1","917":"GRUPO 1","918":"GRUPO 1","919":"GRUPO 1","920":"GRUPO 1","921":"GRUPO 1","922":"GRUPO 1","923":"GRUPO 1","924":"GRUPO 2","925":"GRUPO 2","926":"GRUPO 2","927":"GRUPO 2","928":"GRUPO 2","929":"GRUPO 2","930":"GRUPO 2","931":"GRUPO 2","932":"GRUPO 2","933":"GRUPO 2","934":"GRUPO 2","935":"GRUPO 2","936":"GRUPO 3","937":"GRUPO 3","938":"GRUPO 3","939":"GRUPO 3","940":"GRUPO 3","941":"GRUPO 3","942":"GRUPO 3","943":"GRUPO 3","944":"GRUPO 3","945":"GRUPO 3","946":"GRUPO 3","947":"GRUPO 3","948":"GRUPO 4","949":"GRUPO 4","950":"GRUPO 4","951":"GRUPO 4","952":"GRUPO 4","953":"GRUPO 4","954":"GRUPO 4","955":"GRUPO 4","956":"GRUPO 4","957":"GRUPO 4","958":"GRUPO 4","959":"GRUPO 4","960":"GRUPO 1","961":"GRUPO 1","962":"GRUPO 1","963":"GRUPO 1","964":"GRUPO 1","965":"GRUPO 1","966":"GRUPO 1","967":"GRUPO 1","968":"GRUPO 1","969":"GRUPO 1","970":"GRUPO 1","971":"GRUPO 1","972":"GRUPO 2","973":"GRUPO 2","974":"GRUPO 2","975":"GRUPO 2","976":"GRUPO 2","977":"GRUPO 2","978":"GRUPO 2","979":"GRUPO 2","980":"GRUPO 2","981":"GRUPO 2","982":"GRUPO 2","983":"GRUPO 2","984":"GRUPO 3","985":"GRUPO 3","986":"GRUPO 3","987":"GRUPO 3","988":"GRUPO 3","989":"GRUPO 3","990":"GRUPO 3","991":"GRUPO 3","992":"GRUPO 3","993":"GRUPO 3","994":"GRUPO 3","995":"GRUPO 3","996":"GRUPO 4","997":"GRUPO 4","998":"GRUPO 4","999":"GRUPO 4","1000":"GRUPO 4","1001":"GRUPO 4","1002":"GRUPO 4","1003":"GRUPO 4","1004":"GRUPO 4","1005":"GRUPO 4","1006":"GRUPO 4","1007":"GRUPO 4","1008":"GRUPO 1","1009":"GRUPO 1","1010":"GRUPO 1","1011":"GRUPO 1","1012":"GRUPO 1","1013":"GRUPO 1","1014":"GRUPO 1","1015":"GRUPO 1","1016":"GRUPO 1","1017":"GRUPO 1","1018":"GRUPO 1","1019":"GRUPO 1","1020":"GRUPO 2","1021":"GRUPO 2","1022":"GRUPO 2","1023":"GRUPO 2","1024":"GRUPO 2","1025":"GRUPO 2","1026":"GRUPO 2","1027":"GRUPO 2","1028":"GRUPO 2","1029":"GRUPO 2","1030":"GRUPO 2","1031":"GRUPO 2","1032":"GRUPO 3","1033":"GRUPO 3","1034":"GRUPO 3","1035":"GRUPO 3","1036":"GRUPO 3","1037":"GRUPO 3","1038":"GRUPO 3","1039":"GRUPO 3","1040":"GRUPO 3","1041":"GRUPO 3","1042":"GRUPO 3","1043":"GRUPO 3","1044":"GRUPO 4","1045":"GRUPO 4","1046":"GRUPO 4","1047":"GRUPO 4","1048":"GRUPO 4","1049":"GRUPO 4","1050":"GRUPO 4","1051":"GRUPO 4","1052":"GRUPO 4","1053":"GRUPO 4","1054":"GRUPO 4","1055":"GRUPO 4","1056":"GRUPO 1","1057":"GRUPO 1","1058":"GRUPO 1","1059":"GRUPO 1","1060":"GRUPO 1","1061":"GRUPO 1","1062":"GRUPO 1","1063":"GRUPO 1","1064":"GRUPO 1","1065":"GRUPO 1","1066":"GRUPO 1","1067":"GRUPO 1","1068":"GRUPO 2","1069":"GRUPO 2","1070":"GRUPO 2","1071":"GRUPO 2","1072":"GRUPO 2","1073":"GRUPO 2","1074":"GRUPO 2","1075":"GRUPO 2","1076":"GRUPO 2","1077":"GRUPO 2","1078":"GRUPO 2","1079":"GRUPO 2","1080":"GRUPO 3","1081":"GRUPO 3","1082":"GRUPO 3","1083":"GRUPO 3","1084":"GRUPO 3","1085":"GRUPO 3","1086":"GRUPO 3","1087":"GRUPO 3","1088":"GRUPO 3","1089":"GRUPO 3","1090":"GRUPO 3","1091":"GRUPO 3","1092":"GRUPO 4","1093":"GRUPO 4","1094":"GRUPO 4","1095":"GRUPO 4","1096":"GRUPO 4","1097":"GRUPO 4","1098":"GRUPO 4","1099":"GRUPO 4","1100":"GRUPO 4","1101":"GRUPO 4","1102":"GRUPO 4","1103":"GRUPO 4","1104":"GRUPO 1","1105":"GRUPO 1","1106":"GRUPO 1","1107":"GRUPO 1","1108":"GRUPO 1","1109":"GRUPO 1","1110":"GRUPO 1","1111":"GRUPO 1","1112":"GRUPO 1","1113":"GRUPO 1","1114":"GRUPO 1","1115":"GRUPO 1","1116":"GRUPO 2","1117":"GRUPO 2","1118":"GRUPO 2","1119":"GRUPO 2","1120":"GRUPO 2","1121":"GRUPO 2","1122":"GRUPO 2","1123":"GRUPO 2","1124":"GRUPO 2","1125":"GRUPO 2","1126":"GRUPO 2","1127":"GRUPO 2","1128":"GRUPO 3","1129":"GRUPO 3","1130":"GRUPO 3","1131":"GRUPO 3","1132":"GRUPO 3","1133":"GRUPO 3","1134":"GRUPO 3","1135":"GRUPO 3","1136":"GRUPO 3","1137":"GRUPO 3","1138":"GRUPO 3","1139":"GRUPO 3","1140":"GRUPO 4","1141":"GRUPO 4","1142":"GRUPO 4","1143":"GRUPO 4","1144":"GRUPO 4","1145":"GRUPO 4","1146":"GRUPO 4","1147":"GRUPO 4","1148":"GRUPO 4","1149":"GRUPO 4","1150":"GRUPO 4","1151":"GRUPO 4","1152":"GRUPO 1","1153":"GRUPO 1","1154":"GRUPO 1","1155":"GRUPO 1","1156":"GRUPO 1","1157":"GRUPO 1","1158":"GRUPO 1","1159":"GRUPO 1","1160":"GRUPO 1","1161":"GRUPO 1","1162":"GRUPO 1","1163":"GRUPO 1","1164":"GRUPO 2","1165":"GRUPO 2","1166":"GRUPO 2","1167":"GRUPO 2","1168":"GRUPO 2","1169":"GRUPO 2","1170":"GRUPO 2","1171":"GRUPO 2","1172":"GRUPO 2","1173":"GRUPO 2","1174":"GRUPO 2","1175":"GRUPO 2","1176":"GRUPO 3","1177":"GRUPO 3","1178":"GRUPO 3","1179":"GRUPO 3","1180":"GRUPO 3","1181":"GRUPO 3","1182":"GRUPO 3","1183":"GRUPO 3","1184":"GRUPO 3","1185":"GRUPO 3","1186":"GRUPO 3","1187":"GRUPO 3","1188":"GRUPO 4","1189":"GRUPO 4","1190":"GRUPO 4","1191":"GRUPO 4","1192":"GRUPO 4","1193":"GRUPO 4","1194":"GRUPO 4","1195":"GRUPO 4","1196":"GRUPO 4","1197":"GRUPO 4","1198":"GRUPO 4","1199":"GRUPO 4","1200":"GRUPO 1","1201":"GRUPO 1","1202":"GRUPO 1","1203":"GRUPO 1","1204":"GRUPO 1","1205":"GRUPO 1","1206":"GRUPO 1","1207":"GRUPO 1","1208":"GRUPO 1","1209":"GRUPO 1","1210":"GRUPO 1","1211":"GRUPO 1","1212":"GRUPO 2","1213":"GRUPO 2","1214":"GRUPO 2","1215":"GRUPO 2","1216":"GRUPO 2","1217":"GRUPO 2","1218":"GRUPO 2","1219":"GRUPO 2","1220":"GRUPO 2","1221":"GRUPO 2","1222":"GRUPO 2","1223":"GRUPO 2","1224":"GRUPO 3","1225":"GRUPO 3","1226":"GRUPO 3","1227":"GRUPO 3","1228":"GRUPO 3","1229":"GRUPO 3","1230":"GRUPO 3","1231":"GRUPO 3","1232":"GRUPO 3","1233":"GRUPO 3","1234":"GRUPO 3","1235":"GRUPO 3","1236":"GRUPO 4","1237":"GRUPO 4","1238":"GRUPO 4","1239":"GRUPO 4","1240":"GRUPO 4","1241":"GRUPO 4","1242":"GRUPO 4","1243":"GRUPO 4","1244":"GRUPO 4","1245":"GRUPO 4","1246":"GRUPO 4","1247":"GRUPO 4","1248":"GRUPO 1","1249":"GRUPO 1","1250":"GRUPO 1","1251":"GRUPO 1","1252":"GRUPO 1","1253":"GRUPO 1","1254":"GRUPO 1","1255":"GRUPO 1","1256":"GRUPO 1","1257":"GRUPO 1","1258":"GRUPO 1","1259":"GRUPO 1","1260":"GRUPO 2","1261":"GRUPO 2","1262":"GRUPO 2","1263":"GRUPO 2","1264":"GRUPO 2","1265":"GRUPO 2","1266":"GRUPO 2","1267":"GRUPO 2","1268":"GRUPO 2","1269":"GRUPO 2","1270":"GRUPO 2","1271":"GRUPO 2","1272":"GRUPO 3","1273":"GRUPO 3","1274":"GRUPO 3","1275":"GRUPO 3","1276":"GRUPO 3","1277":"GRUPO 3","1278":"GRUPO 3","1279":"GRUPO 3","1280":"GRUPO 3","1281":"GRUPO 3","1282":"GRUPO 3","1283":"GRUPO 3","1284":"GRUPO 4","1285":"GRUPO 4","1286":"GRUPO 4","1287":"GRUPO 4","1288":"GRUPO 4","1289":"GRUPO 4","1290":"GRUPO 4","1291":"GRUPO 4","1292":"GRUPO 4","1293":"GRUPO 4","1294":"GRUPO 4","1295":"GRUPO 4","1296":"GRUPO 1","1297":"GRUPO 1","1298":"GRUPO 1","1299":"GRUPO 1","1300":"GRUPO 1","1301":"GRUPO 1","1302":"GRUPO 1","1303":"GRUPO 1","1304":"GRUPO 1","1305":"GRUPO 1","1306":"GRUPO 1","1307":"GRUPO 1","1308":"GRUPO 2","1309":"GRUPO 2","1310":"GRUPO 2","1311":"GRUPO 2","1312":"GRUPO 2","1313":"GRUPO 2","1314":"GRUPO 2","1315":"GRUPO 2","1316":"GRUPO 2","1317":"GRUPO 2","1318":"GRUPO 2","1319":"GRUPO 2","1320":"GRUPO 3","1321":"GRUPO 3","1322":"GRUPO 3","1323":"GRUPO 3","1324":"GRUPO 3","1325":"GRUPO 3","1326":"GRUPO 3","1327":"GRUPO 3","1328":"GRUPO 3","1329":"GRUPO 3","1330":"GRUPO 3","1331":"GRUPO 3","1332":"GRUPO 4","1333":"GRUPO 4","1334":"GRUPO 4","1335":"GRUPO 4","1336":"GRUPO 4","1337":"GRUPO 4","1338":"GRUPO 4","1339":"GRUPO 4","1340":"GRUPO 4","1341":"GRUPO 4","1342":"GRUPO 4","1343":"GRUPO 4","1344":"GRUPO 1","1345":"GRUPO 1","1346":"GRUPO 1","1347":"GRUPO 1","1348":"GRUPO 1","1349":"GRUPO 1","1350":"GRUPO 1","1351":"GRUPO 1","1352":"GRUPO 1","1353":"GRUPO 1","1354":"GRUPO 1","1355":"GRUPO 1","1356":"GRUPO 2","1357":"GRUPO 2","1358":"GRUPO 2","1359":"GRUPO 2","1360":"GRUPO 2","1361":"GRUPO 2","1362":"GRUPO 2","1363":"GRUPO 2","1364":"GRUPO 2","1365":"GRUPO 2","1366":"GRUPO 2","1367":"GRUPO 2","1368":"GRUPO 3","1369":"GRUPO 3","1370":"GRUPO 3","1371":"GRUPO 3","1372":"GRUPO 3","1373":"GRUPO 3","1374":"GRUPO 3","1375":"GRUPO 3","1376":"GRUPO 3","1377":"GRUPO 3","1378":"GRUPO 3","1379":"GRUPO 3","1380":"GRUPO 4","1381":"GRUPO 4","1382":"GRUPO 4","1383":"GRUPO 4","1384":"GRUPO 4","1385":"GRUPO 4","1386":"GRUPO 4","1387":"GRUPO 4","1388":"GRUPO 4","1389":"GRUPO 4","1390":"GRUPO 4","1391":"GRUPO 4","1392":"GRUPO 1","1393":"GRUPO 1","1394":"GRUPO 1","1395":"GRUPO 1","1396":"GRUPO 1","1397":"GRUPO 1","1398":"GRUPO 1","1399":"GRUPO 1","1400":"GRUPO 1","1401":"GRUPO 1","1402":"GRUPO 1","1403":"GRUPO 1","1404":"GRUPO 2","1405":"GRUPO 2","1406":"GRUPO 2","1407":"GRUPO 2","1408":"GRUPO 2","1409":"GRUPO 2","1410":"GRUPO 2","1411":"GRUPO 2","1412":"GRUPO 2","1413":"GRUPO 2","1414":"GRUPO 2","1415":"GRUPO 2","1416":"GRUPO 3","1417":"GRUPO 3","1418":"GRUPO 3","1419":"GRUPO 3","1420":"GRUPO 3","1421":"GRUPO 3","1422":"GRUPO 3","1423":"GRUPO 3","1424":"GRUPO 3","1425":"GRUPO 3","1426":"GRUPO 3","1427":"GRUPO 3","1428":"GRUPO 4","1429":"GRUPO 4","1430":"GRUPO 4","1431":"GRUPO 4","1432":"GRUPO 4","1433":"GRUPO 4","1434":"GRUPO 4","1435":"GRUPO 4","1436":"GRUPO 4","1437":"GRUPO 4","1438":"GRUPO 4","1439":"GRUPO 4","1440":"GRUPO 1","1441":"GRUPO 1","1442":"GRUPO 1","1443":"GRUPO 1","1444":"GRUPO 1","1445":"GRUPO 1","1446":"GRUPO 1","1447":"GRUPO 1","1448":"GRUPO 1","1449":"GRUPO 1","1450":"GRUPO 1","1451":"GRUPO 1","1452":"GRUPO 2","1453":"GRUPO 2","1454":"GRUPO 2","1455":"GRUPO 2","1456":"GRUPO 2","1457":"GRUPO 2","1458":"GRUPO 2","1459":"GRUPO 2","1460":"GRUPO 2","1461":"GRUPO 2","1462":"GRUPO 2","1463":"GRUPO 2","1464":"GRUPO 3","1465":"GRUPO 3","1466":"GRUPO 3","1467":"GRUPO 3","1468":"GRUPO 3","1469":"GRUPO 3","1470":"GRUPO 3","1471":"GRUPO 3","1472":"GRUPO 3","1473":"GRUPO 3","1474":"GRUPO 3","1475":"GRUPO 3","1476":"GRUPO 4","1477":"GRUPO 4","1478":"GRUPO 4","1479":"GRUPO 4","1480":"GRUPO 4","1481":"GRUPO 4","1482":"GRUPO 4","1483":"GRUPO 4","1484":"GRUPO 4","1485":"GRUPO 4","1486":"GRUPO 4","1487":"GRUPO 4"},"Empleado":{"0":"BARON HERNANDEZ HAROLD ANTONIO","1":"CASTELLANOS CARVAJAL DEYVITH FABIAN","2":"AROCA TORRES JULIAN EDUARDO","3":"BERMUDEZ PARRA JENNIFER XIOMARA","4":"BERNAL BAQUERO JAMES RICARDO","5":"BURGOS ORTIZ JOSE HORACIO","6":"CANTOR PORRAS JUAN FERNEY","7":"CAPERA CAPERA JOSE GABRIEL","8":"CARDENAS LOTERO RICARDO ANDR\u00c9S","9":"RENDON OSPINA NELSON LEANDRO","10":"SARMIENTO URBINA MOISES DANIEL","11":"VELASCO VELASCO SEBASTI\u00c1N DAVID","12":"DELGADO DELGADO JOHAN DARIO","13":"FLOREZ SAUCESO KENIS ALBERTO","14":"CARDONA GARCIA OSCAR JAVIER","15":"CARVAJAL GARC\u00cdA HOVER MARCK","16":"CEPEDA PIRAQUIVE JUAN DAVID","17":"FAJARDO SAENZ OSCAR FERNANDO","18":"FLOREZ ESPITIA RONY ALBERTO","19":"GARCIA CUERVO EDWIN JAVIER","20":"GONZALEZ OCHOA JUAN CARLOS","21":"XXX1","22":"XXX2","23":"XXX3","24":"FONSECA RAY RICARDO","25":"GOMEZ BETANCUR JAIDER ANDRES","26":"GRANADA PATI\u00d1O CARLOS MARINO","27":"GRASS PLATA MIGUEL SNEIDER","28":"MANZANO CALVO JUAN SEBASTIAN","29":"MENDOZA GOITA MARIANSEL ZENAYDA","30":"MURILLO ARAQUE JAIVER GEOVANY","31":"NI\u00d1O ARENAS HECTOR GONZALO","32":"RAMIREZ CHAVERRA JHON EDISON","33":"XXX4","34":"XXX5","35":"XXX6","36":"RODRIGUEZ MOSQUERA LUIS FERNANDO","37":"PEPITO PEREZ","38":"RAMIREZ VARGAS MARCELA PAOLA","39":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","40":"TORO CISNEROS GARY JOSE","41":"USECHE CALDERON JADID ESTIVEN","42":"VASQUEZ NIETO CAMILO ANDRES","43":"JHONY CASTRO","44":"BERNAL JUAN DAVID","45":"XXX7","46":"XXX8","47":"XXX9","48":"BARON HERNANDEZ HAROLD ANTONIO","49":"CASTELLANOS CARVAJAL DEYVITH FABIAN","50":"AROCA TORRES JULIAN EDUARDO","51":"BERMUDEZ PARRA JENNIFER XIOMARA","52":"BERNAL BAQUERO JAMES RICARDO","53":"BURGOS ORTIZ JOSE HORACIO","54":"CANTOR PORRAS JUAN FERNEY","55":"CAPERA CAPERA JOSE GABRIEL","56":"CARDENAS LOTERO RICARDO ANDR\u00c9S","57":"RENDON OSPINA NELSON LEANDRO","58":"SARMIENTO URBINA MOISES DANIEL","59":"VELASCO VELASCO SEBASTI\u00c1N DAVID","60":"DELGADO DELGADO JOHAN DARIO","61":"FLOREZ SAUCESO KENIS ALBERTO","62":"CARDONA GARCIA OSCAR JAVIER","63":"CARVAJAL GARC\u00cdA HOVER MARCK","64":"CEPEDA PIRAQUIVE JUAN DAVID","65":"FAJARDO SAENZ OSCAR FERNANDO","66":"FLOREZ ESPITIA RONY ALBERTO","67":"GARCIA CUERVO EDWIN JAVIER","68":"GONZALEZ OCHOA JUAN CARLOS","69":"XXX1","70":"XXX2","71":"XXX3","72":"FONSECA RAY RICARDO","73":"GOMEZ BETANCUR JAIDER ANDRES","74":"GRANADA PATI\u00d1O CARLOS MARINO","75":"GRASS PLATA MIGUEL SNEIDER","76":"MANZANO CALVO JUAN SEBASTIAN","77":"MENDOZA GOITA MARIANSEL ZENAYDA","78":"MURILLO ARAQUE JAIVER GEOVANY","79":"NI\u00d1O ARENAS HECTOR GONZALO","80":"RAMIREZ CHAVERRA JHON EDISON","81":"XXX4","82":"XXX5","83":"XXX6","84":"RODRIGUEZ MOSQUERA LUIS FERNANDO","85":"PEPITO PEREZ","86":"RAMIREZ VARGAS MARCELA PAOLA","87":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","88":"TORO CISNEROS GARY JOSE","89":"USECHE CALDERON JADID ESTIVEN","90":"VASQUEZ NIETO CAMILO ANDRES","91":"JHONY CASTRO","92":"BERNAL JUAN DAVID","93":"XXX7","94":"XXX8","95":"XXX9","96":"BARON HERNANDEZ HAROLD ANTONIO","97":"CASTELLANOS CARVAJAL DEYVITH FABIAN","98":"AROCA TORRES JULIAN EDUARDO","99":"BERMUDEZ PARRA JENNIFER XIOMARA","100":"BERNAL BAQUERO JAMES RICARDO","101":"BURGOS ORTIZ JOSE HORACIO","102":"CANTOR PORRAS JUAN FERNEY","103":"CAPERA CAPERA JOSE GABRIEL","104":"CARDENAS LOTERO RICARDO ANDR\u00c9S","105":"RENDON OSPINA NELSON LEANDRO","106":"SARMIENTO URBINA MOISES DANIEL","107":"VELASCO VELASCO SEBASTI\u00c1N DAVID","108":"DELGADO DELGADO JOHAN DARIO","109":"FLOREZ SAUCESO KENIS ALBERTO","110":"CARDONA GARCIA OSCAR JAVIER","111":"CARVAJAL GARC\u00cdA HOVER MARCK","112":"CEPEDA PIRAQUIVE JUAN DAVID","113":"FAJARDO SAENZ OSCAR FERNANDO","114":"FLOREZ ESPITIA RONY ALBERTO","115":"GARCIA CUERVO EDWIN JAVIER","116":"GONZALEZ OCHOA JUAN CARLOS","117":"XXX1","118":"XXX2","119":"XXX3","120":"FONSECA RAY RICARDO","121":"GOMEZ BETANCUR JAIDER ANDRES","122":"GRANADA PATI\u00d1O CARLOS MARINO","123":"GRASS PLATA MIGUEL SNEIDER","124":"MANZANO CALVO JUAN SEBASTIAN","125":"MENDOZA GOITA MARIANSEL ZENAYDA","126":"MURILLO ARAQUE JAIVER GEOVANY","127":"NI\u00d1O ARENAS HECTOR GONZALO","128":"RAMIREZ CHAVERRA JHON EDISON","129":"XXX4","130":"XXX5","131":"XXX6","132":"RODRIGUEZ MOSQUERA LUIS FERNANDO","133":"PEPITO PEREZ","134":"RAMIREZ VARGAS MARCELA PAOLA","135":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","136":"TORO CISNEROS GARY JOSE","137":"USECHE CALDERON JADID ESTIVEN","138":"VASQUEZ NIETO CAMILO ANDRES","139":"JHONY CASTRO","140":"BERNAL JUAN DAVID","141":"XXX7","142":"XXX8","143":"XXX9","144":"BARON HERNANDEZ HAROLD ANTONIO","145":"CASTELLANOS CARVAJAL DEYVITH FABIAN","146":"AROCA TORRES JULIAN EDUARDO","147":"BERMUDEZ PARRA JENNIFER XIOMARA","148":"BERNAL BAQUERO JAMES RICARDO","149":"BURGOS ORTIZ JOSE HORACIO","150":"CANTOR PORRAS JUAN FERNEY","151":"CAPERA CAPERA JOSE GABRIEL","152":"CARDENAS LOTERO RICARDO ANDR\u00c9S","153":"RENDON OSPINA NELSON LEANDRO","154":"SARMIENTO URBINA MOISES DANIEL","155":"VELASCO VELASCO SEBASTI\u00c1N DAVID","156":"DELGADO DELGADO JOHAN DARIO","157":"FLOREZ SAUCESO KENIS ALBERTO","158":"CARDONA GARCIA OSCAR JAVIER","159":"CARVAJAL GARC\u00cdA HOVER MARCK","160":"CEPEDA PIRAQUIVE JUAN DAVID","161":"FAJARDO SAENZ OSCAR FERNANDO","162":"FLOREZ ESPITIA RONY ALBERTO","163":"GARCIA CUERVO EDWIN JAVIER","164":"GONZALEZ OCHOA JUAN CARLOS","165":"XXX1","166":"XXX2","167":"XXX3","168":"FONSECA RAY RICARDO","169":"GOMEZ BETANCUR JAIDER ANDRES","170":"GRANADA PATI\u00d1O CARLOS MARINO","171":"GRASS PLATA MIGUEL SNEIDER","172":"MANZANO CALVO JUAN SEBASTIAN","173":"MENDOZA GOITA MARIANSEL ZENAYDA","174":"MURILLO ARAQUE JAIVER GEOVANY","175":"NI\u00d1O ARENAS HECTOR GONZALO","176":"RAMIREZ CHAVERRA JHON EDISON","177":"XXX4","178":"XXX5","179":"XXX6","180":"RODRIGUEZ MOSQUERA LUIS FERNANDO","181":"PEPITO PEREZ","182":"RAMIREZ VARGAS MARCELA PAOLA","183":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","184":"TORO CISNEROS GARY JOSE","185":"USECHE CALDERON JADID ESTIVEN","186":"VASQUEZ NIETO CAMILO ANDRES","187":"JHONY CASTRO","188":"BERNAL JUAN DAVID","189":"XXX7","190":"XXX8","191":"XXX9","192":"BARON HERNANDEZ HAROLD ANTONIO","193":"CASTELLANOS CARVAJAL DEYVITH FABIAN","194":"AROCA TORRES JULIAN EDUARDO","195":"BERMUDEZ PARRA JENNIFER XIOMARA","196":"BERNAL BAQUERO JAMES RICARDO","197":"BURGOS ORTIZ JOSE HORACIO","198":"CANTOR PORRAS JUAN FERNEY","199":"CAPERA CAPERA JOSE GABRIEL","200":"CARDENAS LOTERO RICARDO ANDR\u00c9S","201":"RENDON OSPINA NELSON LEANDRO","202":"SARMIENTO URBINA MOISES DANIEL","203":"VELASCO VELASCO SEBASTI\u00c1N DAVID","204":"DELGADO DELGADO JOHAN DARIO","205":"FLOREZ SAUCESO KENIS ALBERTO","206":"CARDONA GARCIA OSCAR JAVIER","207":"CARVAJAL GARC\u00cdA HOVER MARCK","208":"CEPEDA PIRAQUIVE JUAN DAVID","209":"FAJARDO SAENZ OSCAR FERNANDO","210":"FLOREZ ESPITIA RONY ALBERTO","211":"GARCIA CUERVO EDWIN JAVIER","212":"GONZALEZ OCHOA JUAN CARLOS","213":"XXX1","214":"XXX2","215":"XXX3","216":"FONSECA RAY RICARDO","217":"GOMEZ BETANCUR JAIDER ANDRES","218":"GRANADA PATI\u00d1O CARLOS MARINO","219":"GRASS PLATA MIGUEL SNEIDER","220":"MANZANO CALVO JUAN SEBASTIAN","221":"MENDOZA GOITA MARIANSEL ZENAYDA","222":"MURILLO ARAQUE JAIVER GEOVANY","223":"NI\u00d1O ARENAS HECTOR GONZALO","224":"RAMIREZ CHAVERRA JHON EDISON","225":"XXX4","226":"XXX5","227":"XXX6","228":"RODRIGUEZ MOSQUERA LUIS FERNANDO","229":"PEPITO PEREZ","230":"RAMIREZ VARGAS MARCELA PAOLA","231":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","232":"TORO CISNEROS GARY JOSE","233":"USECHE CALDERON JADID ESTIVEN","234":"VASQUEZ NIETO CAMILO ANDRES","235":"JHONY CASTRO","236":"BERNAL JUAN DAVID","237":"XXX7","238":"XXX8","239":"XXX9","240":"BARON HERNANDEZ HAROLD ANTONIO","241":"CASTELLANOS CARVAJAL DEYVITH FABIAN","242":"AROCA TORRES JULIAN EDUARDO","243":"BERMUDEZ PARRA JENNIFER XIOMARA","244":"BERNAL BAQUERO JAMES RICARDO","245":"BURGOS ORTIZ JOSE HORACIO","246":"CANTOR PORRAS JUAN FERNEY","247":"CAPERA CAPERA JOSE GABRIEL","248":"CARDENAS LOTERO RICARDO ANDR\u00c9S","249":"RENDON OSPINA NELSON LEANDRO","250":"SARMIENTO URBINA MOISES DANIEL","251":"VELASCO VELASCO SEBASTI\u00c1N DAVID","252":"DELGADO DELGADO JOHAN DARIO","253":"FLOREZ SAUCESO KENIS ALBERTO","254":"CARDONA GARCIA OSCAR JAVIER","255":"CARVAJAL GARC\u00cdA HOVER MARCK","256":"CEPEDA PIRAQUIVE JUAN DAVID","257":"FAJARDO SAENZ OSCAR FERNANDO","258":"FLOREZ ESPITIA RONY ALBERTO","259":"GARCIA CUERVO EDWIN JAVIER","260":"GONZALEZ OCHOA JUAN CARLOS","261":"XXX1","262":"XXX2","263":"XXX3","264":"FONSECA RAY RICARDO","265":"GOMEZ BETANCUR JAIDER ANDRES","266":"GRANADA PATI\u00d1O CARLOS MARINO","267":"GR</t>
   </si>
 </sst>
 </file>
@@ -455,7 +455,7 @@
         <v>11</v>
       </c>
       <c r="E4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update historico_mallas.xlsx 2026-04-24 18:19:22.647392
</commit_message>
<xml_diff>
--- a/historico_mallas.xlsx
+++ b/historico_mallas.xlsx
@@ -34,22 +34,22 @@
     <t>Mayo</t>
   </si>
   <si>
+    <t>Abril</t>
+  </si>
+  <si>
     <t>Junio</t>
   </si>
   <si>
-    <t>Abril</t>
-  </si>
-  <si>
     <t>Técnica</t>
   </si>
   <si>
     <t>24/04/2026 17:55</t>
   </si>
   <si>
-    <t>24/04/2026 17:56</t>
-  </si>
-  <si>
     <t>2026-04-24 18:15</t>
+  </si>
+  <si>
+    <t>2026-04-24 18:19</t>
   </si>
   <si>
     <t>{"Grupo":{"0":"GRUPO 1","1":"GRUPO 1","2":"GRUPO 1","3":"GRUPO 1","4":"GRUPO 1","5":"GRUPO 1","6":"GRUPO 1","7":"GRUPO 1","8":"GRUPO 1","9":"GRUPO 1","10":"GRUPO 1","11":"GRUPO 1","12":"GRUPO 2","13":"GRUPO 2","14":"GRUPO 2","15":"GRUPO 2","16":"GRUPO 2","17":"GRUPO 2","18":"GRUPO 2","19":"GRUPO 2","20":"GRUPO 2","21":"GRUPO 2","22":"GRUPO 2","23":"GRUPO 2","24":"GRUPO 3","25":"GRUPO 3","26":"GRUPO 3","27":"GRUPO 3","28":"GRUPO 3","29":"GRUPO 3","30":"GRUPO 3","31":"GRUPO 3","32":"GRUPO 3","33":"GRUPO 3","34":"GRUPO 3","35":"GRUPO 3","36":"GRUPO 4","37":"GRUPO 4","38":"GRUPO 4","39":"GRUPO 4","40":"GRUPO 4","41":"GRUPO 4","42":"GRUPO 4","43":"GRUPO 4","44":"GRUPO 4","45":"GRUPO 4","46":"GRUPO 4","47":"GRUPO 4","48":"GRUPO 1","49":"GRUPO 1","50":"GRUPO 1","51":"GRUPO 1","52":"GRUPO 1","53":"GRUPO 1","54":"GRUPO 1","55":"GRUPO 1","56":"GRUPO 1","57":"GRUPO 1","58":"GRUPO 1","59":"GRUPO 1","60":"GRUPO 2","61":"GRUPO 2","62":"GRUPO 2","63":"GRUPO 2","64":"GRUPO 2","65":"GRUPO 2","66":"GRUPO 2","67":"GRUPO 2","68":"GRUPO 2","69":"GRUPO 2","70":"GRUPO 2","71":"GRUPO 2","72":"GRUPO 3","73":"GRUPO 3","74":"GRUPO 3","75":"GRUPO 3","76":"GRUPO 3","77":"GRUPO 3","78":"GRUPO 3","79":"GRUPO 3","80":"GRUPO 3","81":"GRUPO 3","82":"GRUPO 3","83":"GRUPO 3","84":"GRUPO 4","85":"GRUPO 4","86":"GRUPO 4","87":"GRUPO 4","88":"GRUPO 4","89":"GRUPO 4","90":"GRUPO 4","91":"GRUPO 4","92":"GRUPO 4","93":"GRUPO 4","94":"GRUPO 4","95":"GRUPO 4","96":"GRUPO 1","97":"GRUPO 1","98":"GRUPO 1","99":"GRUPO 1","100":"GRUPO 1","101":"GRUPO 1","102":"GRUPO 1","103":"GRUPO 1","104":"GRUPO 1","105":"GRUPO 1","106":"GRUPO 1","107":"GRUPO 1","108":"GRUPO 2","109":"GRUPO 2","110":"GRUPO 2","111":"GRUPO 2","112":"GRUPO 2","113":"GRUPO 2","114":"GRUPO 2","115":"GRUPO 2","116":"GRUPO 2","117":"GRUPO 2","118":"GRUPO 2","119":"GRUPO 2","120":"GRUPO 3","121":"GRUPO 3","122":"GRUPO 3","123":"GRUPO 3","124":"GRUPO 3","125":"GRUPO 3","126":"GRUPO 3","127":"GRUPO 3","128":"GRUPO 3","129":"GRUPO 3","130":"GRUPO 3","131":"GRUPO 3","132":"GRUPO 4","133":"GRUPO 4","134":"GRUPO 4","135":"GRUPO 4","136":"GRUPO 4","137":"GRUPO 4","138":"GRUPO 4","139":"GRUPO 4","140":"GRUPO 4","141":"GRUPO 4","142":"GRUPO 4","143":"GRUPO 4","144":"GRUPO 1","145":"GRUPO 1","146":"GRUPO 1","147":"GRUPO 1","148":"GRUPO 1","149":"GRUPO 1","150":"GRUPO 1","151":"GRUPO 1","152":"GRUPO 1","153":"GRUPO 1","154":"GRUPO 1","155":"GRUPO 1","156":"GRUPO 2","157":"GRUPO 2","158":"GRUPO 2","159":"GRUPO 2","160":"GRUPO 2","161":"GRUPO 2","162":"GRUPO 2","163":"GRUPO 2","164":"GRUPO 2","165":"GRUPO 2","166":"GRUPO 2","167":"GRUPO 2","168":"GRUPO 3","169":"GRUPO 3","170":"GRUPO 3","171":"GRUPO 3","172":"GRUPO 3","173":"GRUPO 3","174":"GRUPO 3","175":"GRUPO 3","176":"GRUPO 3","177":"GRUPO 3","178":"GRUPO 3","179":"GRUPO 3","180":"GRUPO 4","181":"GRUPO 4","182":"GRUPO 4","183":"GRUPO 4","184":"GRUPO 4","185":"GRUPO 4","186":"GRUPO 4","187":"GRUPO 4","188":"GRUPO 4","189":"GRUPO 4","190":"GRUPO 4","191":"GRUPO 4","192":"GRUPO 1","193":"GRUPO 1","194":"GRUPO 1","195":"GRUPO 1","196":"GRUPO 1","197":"GRUPO 1","198":"GRUPO 1","199":"GRUPO 1","200":"GRUPO 1","201":"GRUPO 1","202":"GRUPO 1","203":"GRUPO 1","204":"GRUPO 2","205":"GRUPO 2","206":"GRUPO 2","207":"GRUPO 2","208":"GRUPO 2","209":"GRUPO 2","210":"GRUPO 2","211":"GRUPO 2","212":"GRUPO 2","213":"GRUPO 2","214":"GRUPO 2","215":"GRUPO 2","216":"GRUPO 3","217":"GRUPO 3","218":"GRUPO 3","219":"GRUPO 3","220":"GRUPO 3","221":"GRUPO 3","222":"GRUPO 3","223":"GRUPO 3","224":"GRUPO 3","225":"GRUPO 3","226":"GRUPO 3","227":"GRUPO 3","228":"GRUPO 4","229":"GRUPO 4","230":"GRUPO 4","231":"GRUPO 4","232":"GRUPO 4","233":"GRUPO 4","234":"GRUPO 4","235":"GRUPO 4","236":"GRUPO 4","237":"GRUPO 4","238":"GRUPO 4","239":"GRUPO 4","240":"GRUPO 1","241":"GRUPO 1","242":"GRUPO 1","243":"GRUPO 1","244":"GRUPO 1","245":"GRUPO 1","246":"GRUPO 1","247":"GRUPO 1","248":"GRUPO 1","249":"GRUPO 1","250":"GRUPO 1","251":"GRUPO 1","252":"GRUPO 2","253":"GRUPO 2","254":"GRUPO 2","255":"GRUPO 2","256":"GRUPO 2","257":"GRUPO 2","258":"GRUPO 2","259":"GRUPO 2","260":"GRUPO 2","261":"GRUPO 2","262":"GRUPO 2","263":"GRUPO 2","264":"GRUPO 3","265":"GRUPO 3","266":"GRUPO 3","267":"GRUPO 3","268":"GRUPO 3","269":"GRUPO 3","270":"GRUPO 3","271":"GRUPO 3","272":"GRUPO 3","273":"GRUPO 3","274":"GRUPO 3","275":"GRUPO 3","276":"GRUPO 4","277":"GRUPO 4","278":"GRUPO 4","279":"GRUPO 4","280":"GRUPO 4","281":"GRUPO 4","282":"GRUPO 4","283":"GRUPO 4","284":"GRUPO 4","285":"GRUPO 4","286":"GRUPO 4","287":"GRUPO 4","288":"GRUPO 1","289":"GRUPO 1","290":"GRUPO 1","291":"GRUPO 1","292":"GRUPO 1","293":"GRUPO 1","294":"GRUPO 1","295":"GRUPO 1","296":"GRUPO 1","297":"GRUPO 1","298":"GRUPO 1","299":"GRUPO 1","300":"GRUPO 2","301":"GRUPO 2","302":"GRUPO 2","303":"GRUPO 2","304":"GRUPO 2","305":"GRUPO 2","306":"GRUPO 2","307":"GRUPO 2","308":"GRUPO 2","309":"GRUPO 2","310":"GRUPO 2","311":"GRUPO 2","312":"GRUPO 3","313":"GRUPO 3","314":"GRUPO 3","315":"GRUPO 3","316":"GRUPO 3","317":"GRUPO 3","318":"GRUPO 3","319":"GRUPO 3","320":"GRUPO 3","321":"GRUPO 3","322":"GRUPO 3","323":"GRUPO 3","324":"GRUPO 4","325":"GRUPO 4","326":"GRUPO 4","327":"GRUPO 4","328":"GRUPO 4","329":"GRUPO 4","330":"GRUPO 4","331":"GRUPO 4","332":"GRUPO 4","333":"GRUPO 4","334":"GRUPO 4","335":"GRUPO 4","336":"GRUPO 1","337":"GRUPO 1","338":"GRUPO 1","339":"GRUPO 1","340":"GRUPO 1","341":"GRUPO 1","342":"GRUPO 1","343":"GRUPO 1","344":"GRUPO 1","345":"GRUPO 1","346":"GRUPO 1","347":"GRUPO 1","348":"GRUPO 2","349":"GRUPO 2","350":"GRUPO 2","351":"GRUPO 2","352":"GRUPO 2","353":"GRUPO 2","354":"GRUPO 2","355":"GRUPO 2","356":"GRUPO 2","357":"GRUPO 2","358":"GRUPO 2","359":"GRUPO 2","360":"GRUPO 3","361":"GRUPO 3","362":"GRUPO 3","363":"GRUPO 3","364":"GRUPO 3","365":"GRUPO 3","366":"GRUPO 3","367":"GRUPO 3","368":"GRUPO 3","369":"GRUPO 3","370":"GRUPO 3","371":"GRUPO 3","372":"GRUPO 4","373":"GRUPO 4","374":"GRUPO 4","375":"GRUPO 4","376":"GRUPO 4","377":"GRUPO 4","378":"GRUPO 4","379":"GRUPO 4","380":"GRUPO 4","381":"GRUPO 4","382":"GRUPO 4","383":"GRUPO 4","384":"GRUPO 1","385":"GRUPO 1","386":"GRUPO 1","387":"GRUPO 1","388":"GRUPO 1","389":"GRUPO 1","390":"GRUPO 1","391":"GRUPO 1","392":"GRUPO 1","393":"GRUPO 1","394":"GRUPO 1","395":"GRUPO 1","396":"GRUPO 2","397":"GRUPO 2","398":"GRUPO 2","399":"GRUPO 2","400":"GRUPO 2","401":"GRUPO 2","402":"GRUPO 2","403":"GRUPO 2","404":"GRUPO 2","405":"GRUPO 2","406":"GRUPO 2","407":"GRUPO 2","408":"GRUPO 3","409":"GRUPO 3","410":"GRUPO 3","411":"GRUPO 3","412":"GRUPO 3","413":"GRUPO 3","414":"GRUPO 3","415":"GRUPO 3","416":"GRUPO 3","417":"GRUPO 3","418":"GRUPO 3","419":"GRUPO 3","420":"GRUPO 4","421":"GRUPO 4","422":"GRUPO 4","423":"GRUPO 4","424":"GRUPO 4","425":"GRUPO 4","426":"GRUPO 4","427":"GRUPO 4","428":"GRUPO 4","429":"GRUPO 4","430":"GRUPO 4","431":"GRUPO 4","432":"GRUPO 1","433":"GRUPO 1","434":"GRUPO 1","435":"GRUPO 1","436":"GRUPO 1","437":"GRUPO 1","438":"GRUPO 1","439":"GRUPO 1","440":"GRUPO 1","441":"GRUPO 1","442":"GRUPO 1","443":"GRUPO 1","444":"GRUPO 2","445":"GRUPO 2","446":"GRUPO 2","447":"GRUPO 2","448":"GRUPO 2","449":"GRUPO 2","450":"GRUPO 2","451":"GRUPO 2","452":"GRUPO 2","453":"GRUPO 2","454":"GRUPO 2","455":"GRUPO 2","456":"GRUPO 3","457":"GRUPO 3","458":"GRUPO 3","459":"GRUPO 3","460":"GRUPO 3","461":"GRUPO 3","462":"GRUPO 3","463":"GRUPO 3","464":"GRUPO 3","465":"GRUPO 3","466":"GRUPO 3","467":"GRUPO 3","468":"GRUPO 4","469":"GRUPO 4","470":"GRUPO 4","471":"GRUPO 4","472":"GRUPO 4","473":"GRUPO 4","474":"GRUPO 4","475":"GRUPO 4","476":"GRUPO 4","477":"GRUPO 4","478":"GRUPO 4","479":"GRUPO 4","480":"GRUPO 1","481":"GRUPO 1","482":"GRUPO 1","483":"GRUPO 1","484":"GRUPO 1","485":"GRUPO 1","486":"GRUPO 1","487":"GRUPO 1","488":"GRUPO 1","489":"GRUPO 1","490":"GRUPO 1","491":"GRUPO 1","492":"GRUPO 2","493":"GRUPO 2","494":"GRUPO 2","495":"GRUPO 2","496":"GRUPO 2","497":"GRUPO 2","498":"GRUPO 2","499":"GRUPO 2","500":"GRUPO 2","501":"GRUPO 2","502":"GRUPO 2","503":"GRUPO 2","504":"GRUPO 3","505":"GRUPO 3","506":"GRUPO 3","507":"GRUPO 3","508":"GRUPO 3","509":"GRUPO 3","510":"GRUPO 3","511":"GRUPO 3","512":"GRUPO 3","513":"GRUPO 3","514":"GRUPO 3","515":"GRUPO 3","516":"GRUPO 4","517":"GRUPO 4","518":"GRUPO 4","519":"GRUPO 4","520":"GRUPO 4","521":"GRUPO 4","522":"GRUPO 4","523":"GRUPO 4","524":"GRUPO 4","525":"GRUPO 4","526":"GRUPO 4","527":"GRUPO 4","528":"GRUPO 1","529":"GRUPO 1","530":"GRUPO 1","531":"GRUPO 1","532":"GRUPO 1","533":"GRUPO 1","534":"GRUPO 1","535":"GRUPO 1","536":"GRUPO 1","537":"GRUPO 1","538":"GRUPO 1","539":"GRUPO 1","540":"GRUPO 2","541":"GRUPO 2","542":"GRUPO 2","543":"GRUPO 2","544":"GRUPO 2","545":"GRUPO 2","546":"GRUPO 2","547":"GRUPO 2","548":"GRUPO 2","549":"GRUPO 2","550":"GRUPO 2","551":"GRUPO 2","552":"GRUPO 3","553":"GRUPO 3","554":"GRUPO 3","555":"GRUPO 3","556":"GRUPO 3","557":"GRUPO 3","558":"GRUPO 3","559":"GRUPO 3","560":"GRUPO 3","561":"GRUPO 3","562":"GRUPO 3","563":"GRUPO 3","564":"GRUPO 4","565":"GRUPO 4","566":"GRUPO 4","567":"GRUPO 4","568":"GRUPO 4","569":"GRUPO 4","570":"GRUPO 4","571":"GRUPO 4","572":"GRUPO 4","573":"GRUPO 4","574":"GRUPO 4","575":"GRUPO 4","576":"GRUPO 1","577":"GRUPO 1","578":"GRUPO 1","579":"GRUPO 1","580":"GRUPO 1","581":"GRUPO 1","582":"GRUPO 1","583":"GRUPO 1","584":"GRUPO 1","585":"GRUPO 1","586":"GRUPO 1","587":"GRUPO 1","588":"GRUPO 2","589":"GRUPO 2","590":"GRUPO 2","591":"GRUPO 2","592":"GRUPO 2","593":"GRUPO 2","594":"GRUPO 2","595":"GRUPO 2","596":"GRUPO 2","597":"GRUPO 2","598":"GRUPO 2","599":"GRUPO 2","600":"GRUPO 3","601":"GRUPO 3","602":"GRUPO 3","603":"GRUPO 3","604":"GRUPO 3","605":"GRUPO 3","606":"GRUPO 3","607":"GRUPO 3","608":"GRUPO 3","609":"GRUPO 3","610":"GRUPO 3","611":"GRUPO 3","612":"GRUPO 4","613":"GRUPO 4","614":"GRUPO 4","615":"GRUPO 4","616":"GRUPO 4","617":"GRUPO 4","618":"GRUPO 4","619":"GRUPO 4","620":"GRUPO 4","621":"GRUPO 4","622":"GRUPO 4","623":"GRUPO 4","624":"GRUPO 1","625":"GRUPO 1","626":"GRUPO 1","627":"GRUPO 1","628":"GRUPO 1","629":"GRUPO 1","630":"GRUPO 1","631":"GRUPO 1","632":"GRUPO 1","633":"GRUPO 1","634":"GRUPO 1","635":"GRUPO 1","636":"GRUPO 2","637":"GRUPO 2","638":"GRUPO 2","639":"GRUPO 2","640":"GRUPO 2","641":"GRUPO 2","642":"GRUPO 2","643":"GRUPO 2","644":"GRUPO 2","645":"GRUPO 2","646":"GRUPO 2","647":"GRUPO 2","648":"GRUPO 3","649":"GRUPO 3","650":"GRUPO 3","651":"GRUPO 3","652":"GRUPO 3","653":"GRUPO 3","654":"GRUPO 3","655":"GRUPO 3","656":"GRUPO 3","657":"GRUPO 3","658":"GRUPO 3","659":"GRUPO 3","660":"GRUPO 4","661":"GRUPO 4","662":"GRUPO 4","663":"GRUPO 4","664":"GRUPO 4","665":"GRUPO 4","666":"GRUPO 4","667":"GRUPO 4","668":"GRUPO 4","669":"GRUPO 4","670":"GRUPO 4","671":"GRUPO 4","672":"GRUPO 1","673":"GRUPO 1","674":"GRUPO 1","675":"GRUPO 1","676":"GRUPO 1","677":"GRUPO 1","678":"GRUPO 1","679":"GRUPO 1","680":"GRUPO 1","681":"GRUPO 1","682":"GRUPO 1","683":"GRUPO 1","684":"GRUPO 2","685":"GRUPO 2","686":"GRUPO 2","687":"GRUPO 2","688":"GRUPO 2","689":"GRUPO 2","690":"GRUPO 2","691":"GRUPO 2","692":"GRUPO 2","693":"GRUPO 2","694":"GRUPO 2","695":"GRUPO 2","696":"GRUPO 3","697":"GRUPO 3","698":"GRUPO 3","699":"GRUPO 3","700":"GRUPO 3","701":"GRUPO 3","702":"GRUPO 3","703":"GRUPO 3","704":"GRUPO 3","705":"GRUPO 3","706":"GRUPO 3","707":"GRUPO 3","708":"GRUPO 4","709":"GRUPO 4","710":"GRUPO 4","711":"GRUPO 4","712":"GRUPO 4","713":"GRUPO 4","714":"GRUPO 4","715":"GRUPO 4","716":"GRUPO 4","717":"GRUPO 4","718":"GRUPO 4","719":"GRUPO 4","720":"GRUPO 1","721":"GRUPO 1","722":"GRUPO 1","723":"GRUPO 1","724":"GRUPO 1","725":"GRUPO 1","726":"GRUPO 1","727":"GRUPO 1","728":"GRUPO 1","729":"GRUPO 1","730":"GRUPO 1","731":"GRUPO 1","732":"GRUPO 2","733":"GRUPO 2","734":"GRUPO 2","735":"GRUPO 2","736":"GRUPO 2","737":"GRUPO 2","738":"GRUPO 2","739":"GRUPO 2","740":"GRUPO 2","741":"GRUPO 2","742":"GRUPO 2","743":"GRUPO 2","744":"GRUPO 3","745":"GRUPO 3","746":"GRUPO 3","747":"GRUPO 3","748":"GRUPO 3","749":"GRUPO 3","750":"GRUPO 3","751":"GRUPO 3","752":"GRUPO 3","753":"GRUPO 3","754":"GRUPO 3","755":"GRUPO 3","756":"GRUPO 4","757":"GRUPO 4","758":"GRUPO 4","759":"GRUPO 4","760":"GRUPO 4","761":"GRUPO 4","762":"GRUPO 4","763":"GRUPO 4","764":"GRUPO 4","765":"GRUPO 4","766":"GRUPO 4","767":"GRUPO 4","768":"GRUPO 1","769":"GRUPO 1","770":"GRUPO 1","771":"GRUPO 1","772":"GRUPO 1","773":"GRUPO 1","774":"GRUPO 1","775":"GRUPO 1","776":"GRUPO 1","777":"GRUPO 1","778":"GRUPO 1","779":"GRUPO 1","780":"GRUPO 2","781":"GRUPO 2","782":"GRUPO 2","783":"GRUPO 2","784":"GRUPO 2","785":"GRUPO 2","786":"GRUPO 2","787":"GRUPO 2","788":"GRUPO 2","789":"GRUPO 2","790":"GRUPO 2","791":"GRUPO 2","792":"GRUPO 3","793":"GRUPO 3","794":"GRUPO 3","795":"GRUPO 3","796":"GRUPO 3","797":"GRUPO 3","798":"GRUPO 3","799":"GRUPO 3","800":"GRUPO 3","801":"GRUPO 3","802":"GRUPO 3","803":"GRUPO 3","804":"GRUPO 4","805":"GRUPO 4","806":"GRUPO 4","807":"GRUPO 4","808":"GRUPO 4","809":"GRUPO 4","810":"GRUPO 4","811":"GRUPO 4","812":"GRUPO 4","813":"GRUPO 4","814":"GRUPO 4","815":"GRUPO 4","816":"GRUPO 1","817":"GRUPO 1","818":"GRUPO 1","819":"GRUPO 1","820":"GRUPO 1","821":"GRUPO 1","822":"GRUPO 1","823":"GRUPO 1","824":"GRUPO 1","825":"GRUPO 1","826":"GRUPO 1","827":"GRUPO 1","828":"GRUPO 2","829":"GRUPO 2","830":"GRUPO 2","831":"GRUPO 2","832":"GRUPO 2","833":"GRUPO 2","834":"GRUPO 2","835":"GRUPO 2","836":"GRUPO 2","837":"GRUPO 2","838":"GRUPO 2","839":"GRUPO 2","840":"GRUPO 3","841":"GRUPO 3","842":"GRUPO 3","843":"GRUPO 3","844":"GRUPO 3","845":"GRUPO 3","846":"GRUPO 3","847":"GRUPO 3","848":"GRUPO 3","849":"GRUPO 3","850":"GRUPO 3","851":"GRUPO 3","852":"GRUPO 4","853":"GRUPO 4","854":"GRUPO 4","855":"GRUPO 4","856":"GRUPO 4","857":"GRUPO 4","858":"GRUPO 4","859":"GRUPO 4","860":"GRUPO 4","861":"GRUPO 4","862":"GRUPO 4","863":"GRUPO 4","864":"GRUPO 1","865":"GRUPO 1","866":"GRUPO 1","867":"GRUPO 1","868":"GRUPO 1","869":"GRUPO 1","870":"GRUPO 1","871":"GRUPO 1","872":"GRUPO 1","873":"GRUPO 1","874":"GRUPO 1","875":"GRUPO 1","876":"GRUPO 2","877":"GRUPO 2","878":"GRUPO 2","879":"GRUPO 2","880":"GRUPO 2","881":"GRUPO 2","882":"GRUPO 2","883":"GRUPO 2","884":"GRUPO 2","885":"GRUPO 2","886":"GRUPO 2","887":"GRUPO 2","888":"GRUPO 3","889":"GRUPO 3","890":"GRUPO 3","891":"GRUPO 3","892":"GRUPO 3","893":"GRUPO 3","894":"GRUPO 3","895":"GRUPO 3","896":"GRUPO 3","897":"GRUPO 3","898":"GRUPO 3","899":"GRUPO 3","900":"GRUPO 4","901":"GRUPO 4","902":"GRUPO 4","903":"GRUPO 4","904":"GRUPO 4","905":"GRUPO 4","906":"GRUPO 4","907":"GRUPO 4","908":"GRUPO 4","909":"GRUPO 4","910":"GRUPO 4","911":"GRUPO 4","912":"GRUPO 1","913":"GRUPO 1","914":"GRUPO 1","915":"GRUPO 1","916":"GRUPO 1","917":"GRUPO 1","918":"GRUPO 1","919":"GRUPO 1","920":"GRUPO 1","921":"GRUPO 1","922":"GRUPO 1","923":"GRUPO 1","924":"GRUPO 2","925":"GRUPO 2","926":"GRUPO 2","927":"GRUPO 2","928":"GRUPO 2","929":"GRUPO 2","930":"GRUPO 2","931":"GRUPO 2","932":"GRUPO 2","933":"GRUPO 2","934":"GRUPO 2","935":"GRUPO 2","936":"GRUPO 3","937":"GRUPO 3","938":"GRUPO 3","939":"GRUPO 3","940":"GRUPO 3","941":"GRUPO 3","942":"GRUPO 3","943":"GRUPO 3","944":"GRUPO 3","945":"GRUPO 3","946":"GRUPO 3","947":"GRUPO 3","948":"GRUPO 4","949":"GRUPO 4","950":"GRUPO 4","951":"GRUPO 4","952":"GRUPO 4","953":"GRUPO 4","954":"GRUPO 4","955":"GRUPO 4","956":"GRUPO 4","957":"GRUPO 4","958":"GRUPO 4","959":"GRUPO 4","960":"GRUPO 1","961":"GRUPO 1","962":"GRUPO 1","963":"GRUPO 1","964":"GRUPO 1","965":"GRUPO 1","966":"GRUPO 1","967":"GRUPO 1","968":"GRUPO 1","969":"GRUPO 1","970":"GRUPO 1","971":"GRUPO 1","972":"GRUPO 2","973":"GRUPO 2","974":"GRUPO 2","975":"GRUPO 2","976":"GRUPO 2","977":"GRUPO 2","978":"GRUPO 2","979":"GRUPO 2","980":"GRUPO 2","981":"GRUPO 2","982":"GRUPO 2","983":"GRUPO 2","984":"GRUPO 3","985":"GRUPO 3","986":"GRUPO 3","987":"GRUPO 3","988":"GRUPO 3","989":"GRUPO 3","990":"GRUPO 3","991":"GRUPO 3","992":"GRUPO 3","993":"GRUPO 3","994":"GRUPO 3","995":"GRUPO 3","996":"GRUPO 4","997":"GRUPO 4","998":"GRUPO 4","999":"GRUPO 4","1000":"GRUPO 4","1001":"GRUPO 4","1002":"GRUPO 4","1003":"GRUPO 4","1004":"GRUPO 4","1005":"GRUPO 4","1006":"GRUPO 4","1007":"GRUPO 4","1008":"GRUPO 1","1009":"GRUPO 1","1010":"GRUPO 1","1011":"GRUPO 1","1012":"GRUPO 1","1013":"GRUPO 1","1014":"GRUPO 1","1015":"GRUPO 1","1016":"GRUPO 1","1017":"GRUPO 1","1018":"GRUPO 1","1019":"GRUPO 1","1020":"GRUPO 2","1021":"GRUPO 2","1022":"GRUPO 2","1023":"GRUPO 2","1024":"GRUPO 2","1025":"GRUPO 2","1026":"GRUPO 2","1027":"GRUPO 2","1028":"GRUPO 2","1029":"GRUPO 2","1030":"GRUPO 2","1031":"GRUPO 2","1032":"GRUPO 3","1033":"GRUPO 3","1034":"GRUPO 3","1035":"GRUPO 3","1036":"GRUPO 3","1037":"GRUPO 3","1038":"GRUPO 3","1039":"GRUPO 3","1040":"GRUPO 3","1041":"GRUPO 3","1042":"GRUPO 3","1043":"GRUPO 3","1044":"GRUPO 4","1045":"GRUPO 4","1046":"GRUPO 4","1047":"GRUPO 4","1048":"GRUPO 4","1049":"GRUPO 4","1050":"GRUPO 4","1051":"GRUPO 4","1052":"GRUPO 4","1053":"GRUPO 4","1054":"GRUPO 4","1055":"GRUPO 4","1056":"GRUPO 1","1057":"GRUPO 1","1058":"GRUPO 1","1059":"GRUPO 1","1060":"GRUPO 1","1061":"GRUPO 1","1062":"GRUPO 1","1063":"GRUPO 1","1064":"GRUPO 1","1065":"GRUPO 1","1066":"GRUPO 1","1067":"GRUPO 1","1068":"GRUPO 2","1069":"GRUPO 2","1070":"GRUPO 2","1071":"GRUPO 2","1072":"GRUPO 2","1073":"GRUPO 2","1074":"GRUPO 2","1075":"GRUPO 2","1076":"GRUPO 2","1077":"GRUPO 2","1078":"GRUPO 2","1079":"GRUPO 2","1080":"GRUPO 3","1081":"GRUPO 3","1082":"GRUPO 3","1083":"GRUPO 3","1084":"GRUPO 3","1085":"GRUPO 3","1086":"GRUPO 3","1087":"GRUPO 3","1088":"GRUPO 3","1089":"GRUPO 3","1090":"GRUPO 3","1091":"GRUPO 3","1092":"GRUPO 4","1093":"GRUPO 4","1094":"GRUPO 4","1095":"GRUPO 4","1096":"GRUPO 4","1097":"GRUPO 4","1098":"GRUPO 4","1099":"GRUPO 4","1100":"GRUPO 4","1101":"GRUPO 4","1102":"GRUPO 4","1103":"GRUPO 4","1104":"GRUPO 1","1105":"GRUPO 1","1106":"GRUPO 1","1107":"GRUPO 1","1108":"GRUPO 1","1109":"GRUPO 1","1110":"GRUPO 1","1111":"GRUPO 1","1112":"GRUPO 1","1113":"GRUPO 1","1114":"GRUPO 1","1115":"GRUPO 1","1116":"GRUPO 2","1117":"GRUPO 2","1118":"GRUPO 2","1119":"GRUPO 2","1120":"GRUPO 2","1121":"GRUPO 2","1122":"GRUPO 2","1123":"GRUPO 2","1124":"GRUPO 2","1125":"GRUPO 2","1126":"GRUPO 2","1127":"GRUPO 2","1128":"GRUPO 3","1129":"GRUPO 3","1130":"GRUPO 3","1131":"GRUPO 3","1132":"GRUPO 3","1133":"GRUPO 3","1134":"GRUPO 3","1135":"GRUPO 3","1136":"GRUPO 3","1137":"GRUPO 3","1138":"GRUPO 3","1139":"GRUPO 3","1140":"GRUPO 4","1141":"GRUPO 4","1142":"GRUPO 4","1143":"GRUPO 4","1144":"GRUPO 4","1145":"GRUPO 4","1146":"GRUPO 4","1147":"GRUPO 4","1148":"GRUPO 4","1149":"GRUPO 4","1150":"GRUPO 4","1151":"GRUPO 4","1152":"GRUPO 1","1153":"GRUPO 1","1154":"GRUPO 1","1155":"GRUPO 1","1156":"GRUPO 1","1157":"GRUPO 1","1158":"GRUPO 1","1159":"GRUPO 1","1160":"GRUPO 1","1161":"GRUPO 1","1162":"GRUPO 1","1163":"GRUPO 1","1164":"GRUPO 2","1165":"GRUPO 2","1166":"GRUPO 2","1167":"GRUPO 2","1168":"GRUPO 2","1169":"GRUPO 2","1170":"GRUPO 2","1171":"GRUPO 2","1172":"GRUPO 2","1173":"GRUPO 2","1174":"GRUPO 2","1175":"GRUPO 2","1176":"GRUPO 3","1177":"GRUPO 3","1178":"GRUPO 3","1179":"GRUPO 3","1180":"GRUPO 3","1181":"GRUPO 3","1182":"GRUPO 3","1183":"GRUPO 3","1184":"GRUPO 3","1185":"GRUPO 3","1186":"GRUPO 3","1187":"GRUPO 3","1188":"GRUPO 4","1189":"GRUPO 4","1190":"GRUPO 4","1191":"GRUPO 4","1192":"GRUPO 4","1193":"GRUPO 4","1194":"GRUPO 4","1195":"GRUPO 4","1196":"GRUPO 4","1197":"GRUPO 4","1198":"GRUPO 4","1199":"GRUPO 4","1200":"GRUPO 1","1201":"GRUPO 1","1202":"GRUPO 1","1203":"GRUPO 1","1204":"GRUPO 1","1205":"GRUPO 1","1206":"GRUPO 1","1207":"GRUPO 1","1208":"GRUPO 1","1209":"GRUPO 1","1210":"GRUPO 1","1211":"GRUPO 1","1212":"GRUPO 2","1213":"GRUPO 2","1214":"GRUPO 2","1215":"GRUPO 2","1216":"GRUPO 2","1217":"GRUPO 2","1218":"GRUPO 2","1219":"GRUPO 2","1220":"GRUPO 2","1221":"GRUPO 2","1222":"GRUPO 2","1223":"GRUPO 2","1224":"GRUPO 3","1225":"GRUPO 3","1226":"GRUPO 3","1227":"GRUPO 3","1228":"GRUPO 3","1229":"GRUPO 3","1230":"GRUPO 3","1231":"GRUPO 3","1232":"GRUPO 3","1233":"GRUPO 3","1234":"GRUPO 3","1235":"GRUPO 3","1236":"GRUPO 4","1237":"GRUPO 4","1238":"GRUPO 4","1239":"GRUPO 4","1240":"GRUPO 4","1241":"GRUPO 4","1242":"GRUPO 4","1243":"GRUPO 4","1244":"GRUPO 4","1245":"GRUPO 4","1246":"GRUPO 4","1247":"GRUPO 4","1248":"GRUPO 1","1249":"GRUPO 1","1250":"GRUPO 1","1251":"GRUPO 1","1252":"GRUPO 1","1253":"GRUPO 1","1254":"GRUPO 1","1255":"GRUPO 1","1256":"GRUPO 1","1257":"GRUPO 1","1258":"GRUPO 1","1259":"GRUPO 1","1260":"GRUPO 2","1261":"GRUPO 2","1262":"GRUPO 2","1263":"GRUPO 2","1264":"GRUPO 2","1265":"GRUPO 2","1266":"GRUPO 2","1267":"GRUPO 2","1268":"GRUPO 2","1269":"GRUPO 2","1270":"GRUPO 2","1271":"GRUPO 2","1272":"GRUPO 3","1273":"GRUPO 3","1274":"GRUPO 3","1275":"GRUPO 3","1276":"GRUPO 3","1277":"GRUPO 3","1278":"GRUPO 3","1279":"GRUPO 3","1280":"GRUPO 3","1281":"GRUPO 3","1282":"GRUPO 3","1283":"GRUPO 3","1284":"GRUPO 4","1285":"GRUPO 4","1286":"GRUPO 4","1287":"GRUPO 4","1288":"GRUPO 4","1289":"GRUPO 4","1290":"GRUPO 4","1291":"GRUPO 4","1292":"GRUPO 4","1293":"GRUPO 4","1294":"GRUPO 4","1295":"GRUPO 4","1296":"GRUPO 1","1297":"GRUPO 1","1298":"GRUPO 1","1299":"GRUPO 1","1300":"GRUPO 1","1301":"GRUPO 1","1302":"GRUPO 1","1303":"GRUPO 1","1304":"GRUPO 1","1305":"GRUPO 1","1306":"GRUPO 1","1307":"GRUPO 1","1308":"GRUPO 2","1309":"GRUPO 2","1310":"GRUPO 2","1311":"GRUPO 2","1312":"GRUPO 2","1313":"GRUPO 2","1314":"GRUPO 2","1315":"GRUPO 2","1316":"GRUPO 2","1317":"GRUPO 2","1318":"GRUPO 2","1319":"GRUPO 2","1320":"GRUPO 3","1321":"GRUPO 3","1322":"GRUPO 3","1323":"GRUPO 3","1324":"GRUPO 3","1325":"GRUPO 3","1326":"GRUPO 3","1327":"GRUPO 3","1328":"GRUPO 3","1329":"GRUPO 3","1330":"GRUPO 3","1331":"GRUPO 3","1332":"GRUPO 4","1333":"GRUPO 4","1334":"GRUPO 4","1335":"GRUPO 4","1336":"GRUPO 4","1337":"GRUPO 4","1338":"GRUPO 4","1339":"GRUPO 4","1340":"GRUPO 4","1341":"GRUPO 4","1342":"GRUPO 4","1343":"GRUPO 4","1344":"GRUPO 1","1345":"GRUPO 1","1346":"GRUPO 1","1347":"GRUPO 1","1348":"GRUPO 1","1349":"GRUPO 1","1350":"GRUPO 1","1351":"GRUPO 1","1352":"GRUPO 1","1353":"GRUPO 1","1354":"GRUPO 1","1355":"GRUPO 1","1356":"GRUPO 2","1357":"GRUPO 2","1358":"GRUPO 2","1359":"GRUPO 2","1360":"GRUPO 2","1361":"GRUPO 2","1362":"GRUPO 2","1363":"GRUPO 2","1364":"GRUPO 2","1365":"GRUPO 2","1366":"GRUPO 2","1367":"GRUPO 2","1368":"GRUPO 3","1369":"GRUPO 3","1370":"GRUPO 3","1371":"GRUPO 3","1372":"GRUPO 3","1373":"GRUPO 3","1374":"GRUPO 3","1375":"GRUPO 3","1376":"GRUPO 3","1377":"GRUPO 3","1378":"GRUPO 3","1379":"GRUPO 3","1380":"GRUPO 4","1381":"GRUPO 4","1382":"GRUPO 4","1383":"GRUPO 4","1384":"GRUPO 4","1385":"GRUPO 4","1386":"GRUPO 4","1387":"GRUPO 4","1388":"GRUPO 4","1389":"GRUPO 4","1390":"GRUPO 4","1391":"GRUPO 4","1392":"GRUPO 1","1393":"GRUPO 1","1394":"GRUPO 1","1395":"GRUPO 1","1396":"GRUPO 1","1397":"GRUPO 1","1398":"GRUPO 1","1399":"GRUPO 1","1400":"GRUPO 1","1401":"GRUPO 1","1402":"GRUPO 1","1403":"GRUPO 1","1404":"GRUPO 2","1405":"GRUPO 2","1406":"GRUPO 2","1407":"GRUPO 2","1408":"GRUPO 2","1409":"GRUPO 2","1410":"GRUPO 2","1411":"GRUPO 2","1412":"GRUPO 2","1413":"GRUPO 2","1414":"GRUPO 2","1415":"GRUPO 2","1416":"GRUPO 3","1417":"GRUPO 3","1418":"GRUPO 3","1419":"GRUPO 3","1420":"GRUPO 3","1421":"GRUPO 3","1422":"GRUPO 3","1423":"GRUPO 3","1424":"GRUPO 3","1425":"GRUPO 3","1426":"GRUPO 3","1427":"GRUPO 3","1428":"GRUPO 4","1429":"GRUPO 4","1430":"GRUPO 4","1431":"GRUPO 4","1432":"GRUPO 4","1433":"GRUPO 4","1434":"GRUPO 4","1435":"GRUPO 4","1436":"GRUPO 4","1437":"GRUPO 4","1438":"GRUPO 4","1439":"GRUPO 4","1440":"GRUPO 1","1441":"GRUPO 1","1442":"GRUPO 1","1443":"GRUPO 1","1444":"GRUPO 1","1445":"GRUPO 1","1446":"GRUPO 1","1447":"GRUPO 1","1448":"GRUPO 1","1449":"GRUPO 1","1450":"GRUPO 1","1451":"GRUPO 1","1452":"GRUPO 2","1453":"GRUPO 2","1454":"GRUPO 2","1455":"GRUPO 2","1456":"GRUPO 2","1457":"GRUPO 2","1458":"GRUPO 2","1459":"GRUPO 2","1460":"GRUPO 2","1461":"GRUPO 2","1462":"GRUPO 2","1463":"GRUPO 2","1464":"GRUPO 3","1465":"GRUPO 3","1466":"GRUPO 3","1467":"GRUPO 3","1468":"GRUPO 3","1469":"GRUPO 3","1470":"GRUPO 3","1471":"GRUPO 3","1472":"GRUPO 3","1473":"GRUPO 3","1474":"GRUPO 3","1475":"GRUPO 3","1476":"GRUPO 4","1477":"GRUPO 4","1478":"GRUPO 4","1479":"GRUPO 4","1480":"GRUPO 4","1481":"GRUPO 4","1482":"GRUPO 4","1483":"GRUPO 4","1484":"GRUPO 4","1485":"GRUPO 4","1486":"GRUPO 4","1487":"GRUPO 4"},"Empleado":{"0":"BARON HERNANDEZ HAROLD ANTONIO","1":"CASTELLANOS CARVAJAL DEYVITH FABIAN","2":"AROCA TORRES JULIAN EDUARDO","3":"BERMUDEZ PARRA JENNIFER XIOMARA","4":"BERNAL BAQUERO JAMES RICARDO","5":"BURGOS ORTIZ JOSE HORACIO","6":"CANTOR PORRAS JUAN FERNEY","7":"CAPERA CAPERA JOSE GABRIEL","8":"CARDENAS LOTERO RICARDO ANDR\u00c9S","9":"RENDON OSPINA NELSON LEANDRO","10":"SARMIENTO URBINA MOISES DANIEL","11":"VELASCO VELASCO SEBASTI\u00c1N DAVID","12":"DELGADO DELGADO JOHAN DARIO","13":"FLOREZ SAUCESO KENIS ALBERTO","14":"CARDONA GARCIA OSCAR JAVIER","15":"CARVAJAL GARC\u00cdA HOVER MARCK","16":"CEPEDA PIRAQUIVE JUAN DAVID","17":"FAJARDO SAENZ OSCAR FERNANDO","18":"FLOREZ ESPITIA RONY ALBERTO","19":"GARCIA CUERVO EDWIN JAVIER","20":"GONZALEZ OCHOA JUAN CARLOS","21":"XXX1","22":"XXX2","23":"XXX3","24":"FONSECA RAY RICARDO","25":"GOMEZ BETANCUR JAIDER ANDRES","26":"GRANADA PATI\u00d1O CARLOS MARINO","27":"GRASS PLATA MIGUEL SNEIDER","28":"MANZANO CALVO JUAN SEBASTIAN","29":"MENDOZA GOITA MARIANSEL ZENAYDA","30":"MURILLO ARAQUE JAIVER GEOVANY","31":"NI\u00d1O ARENAS HECTOR GONZALO","32":"RAMIREZ CHAVERRA JHON EDISON","33":"XXX4","34":"XXX5","35":"XXX6","36":"RODRIGUEZ MOSQUERA LUIS FERNANDO","37":"PEPITO PEREZ","38":"RAMIREZ VARGAS MARCELA PAOLA","39":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","40":"TORO CISNEROS GARY JOSE","41":"USECHE CALDERON JADID ESTIVEN","42":"VASQUEZ NIETO CAMILO ANDRES","43":"JHONY CASTRO","44":"BERNAL JUAN DAVID","45":"XXX7","46":"XXX8","47":"XXX9","48":"BARON HERNANDEZ HAROLD ANTONIO","49":"CASTELLANOS CARVAJAL DEYVITH FABIAN","50":"AROCA TORRES JULIAN EDUARDO","51":"BERMUDEZ PARRA JENNIFER XIOMARA","52":"BERNAL BAQUERO JAMES RICARDO","53":"BURGOS ORTIZ JOSE HORACIO","54":"CANTOR PORRAS JUAN FERNEY","55":"CAPERA CAPERA JOSE GABRIEL","56":"CARDENAS LOTERO RICARDO ANDR\u00c9S","57":"RENDON OSPINA NELSON LEANDRO","58":"SARMIENTO URBINA MOISES DANIEL","59":"VELASCO VELASCO SEBASTI\u00c1N DAVID","60":"DELGADO DELGADO JOHAN DARIO","61":"FLOREZ SAUCESO KENIS ALBERTO","62":"CARDONA GARCIA OSCAR JAVIER","63":"CARVAJAL GARC\u00cdA HOVER MARCK","64":"CEPEDA PIRAQUIVE JUAN DAVID","65":"FAJARDO SAENZ OSCAR FERNANDO","66":"FLOREZ ESPITIA RONY ALBERTO","67":"GARCIA CUERVO EDWIN JAVIER","68":"GONZALEZ OCHOA JUAN CARLOS","69":"XXX1","70":"XXX2","71":"XXX3","72":"FONSECA RAY RICARDO","73":"GOMEZ BETANCUR JAIDER ANDRES","74":"GRANADA PATI\u00d1O CARLOS MARINO","75":"GRASS PLATA MIGUEL SNEIDER","76":"MANZANO CALVO JUAN SEBASTIAN","77":"MENDOZA GOITA MARIANSEL ZENAYDA","78":"MURILLO ARAQUE JAIVER GEOVANY","79":"NI\u00d1O ARENAS HECTOR GONZALO","80":"RAMIREZ CHAVERRA JHON EDISON","81":"XXX4","82":"XXX5","83":"XXX6","84":"RODRIGUEZ MOSQUERA LUIS FERNANDO","85":"PEPITO PEREZ","86":"RAMIREZ VARGAS MARCELA PAOLA","87":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","88":"TORO CISNEROS GARY JOSE","89":"USECHE CALDERON JADID ESTIVEN","90":"VASQUEZ NIETO CAMILO ANDRES","91":"JHONY CASTRO","92":"BERNAL JUAN DAVID","93":"XXX7","94":"XXX8","95":"XXX9","96":"BARON HERNANDEZ HAROLD ANTONIO","97":"CASTELLANOS CARVAJAL DEYVITH FABIAN","98":"AROCA TORRES JULIAN EDUARDO","99":"BERMUDEZ PARRA JENNIFER XIOMARA","100":"BERNAL BAQUERO JAMES RICARDO","101":"BURGOS ORTIZ JOSE HORACIO","102":"CANTOR PORRAS JUAN FERNEY","103":"CAPERA CAPERA JOSE GABRIEL","104":"CARDENAS LOTERO RICARDO ANDR\u00c9S","105":"RENDON OSPINA NELSON LEANDRO","106":"SARMIENTO URBINA MOISES DANIEL","107":"VELASCO VELASCO SEBASTI\u00c1N DAVID","108":"DELGADO DELGADO JOHAN DARIO","109":"FLOREZ SAUCESO KENIS ALBERTO","110":"CARDONA GARCIA OSCAR JAVIER","111":"CARVAJAL GARC\u00cdA HOVER MARCK","112":"CEPEDA PIRAQUIVE JUAN DAVID","113":"FAJARDO SAENZ OSCAR FERNANDO","114":"FLOREZ ESPITIA RONY ALBERTO","115":"GARCIA CUERVO EDWIN JAVIER","116":"GONZALEZ OCHOA JUAN CARLOS","117":"XXX1","118":"XXX2","119":"XXX3","120":"FONSECA RAY RICARDO","121":"GOMEZ BETANCUR JAIDER ANDRES","122":"GRANADA PATI\u00d1O CARLOS MARINO","123":"GRASS PLATA MIGUEL SNEIDER","124":"MANZANO CALVO JUAN SEBASTIAN","125":"MENDOZA GOITA MARIANSEL ZENAYDA","126":"MURILLO ARAQUE JAIVER GEOVANY","127":"NI\u00d1O ARENAS HECTOR GONZALO","128":"RAMIREZ CHAVERRA JHON EDISON","129":"XXX4","130":"XXX5","131":"XXX6","132":"RODRIGUEZ MOSQUERA LUIS FERNANDO","133":"PEPITO PEREZ","134":"RAMIREZ VARGAS MARCELA PAOLA","135":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","136":"TORO CISNEROS GARY JOSE","137":"USECHE CALDERON JADID ESTIVEN","138":"VASQUEZ NIETO CAMILO ANDRES","139":"JHONY CASTRO","140":"BERNAL JUAN DAVID","141":"XXX7","142":"XXX8","143":"XXX9","144":"BARON HERNANDEZ HAROLD ANTONIO","145":"CASTELLANOS CARVAJAL DEYVITH FABIAN","146":"AROCA TORRES JULIAN EDUARDO","147":"BERMUDEZ PARRA JENNIFER XIOMARA","148":"BERNAL BAQUERO JAMES RICARDO","149":"BURGOS ORTIZ JOSE HORACIO","150":"CANTOR PORRAS JUAN FERNEY","151":"CAPERA CAPERA JOSE GABRIEL","152":"CARDENAS LOTERO RICARDO ANDR\u00c9S","153":"RENDON OSPINA NELSON LEANDRO","154":"SARMIENTO URBINA MOISES DANIEL","155":"VELASCO VELASCO SEBASTI\u00c1N DAVID","156":"DELGADO DELGADO JOHAN DARIO","157":"FLOREZ SAUCESO KENIS ALBERTO","158":"CARDONA GARCIA OSCAR JAVIER","159":"CARVAJAL GARC\u00cdA HOVER MARCK","160":"CEPEDA PIRAQUIVE JUAN DAVID","161":"FAJARDO SAENZ OSCAR FERNANDO","162":"FLOREZ ESPITIA RONY ALBERTO","163":"GARCIA CUERVO EDWIN JAVIER","164":"GONZALEZ OCHOA JUAN CARLOS","165":"XXX1","166":"XXX2","167":"XXX3","168":"FONSECA RAY RICARDO","169":"GOMEZ BETANCUR JAIDER ANDRES","170":"GRANADA PATI\u00d1O CARLOS MARINO","171":"GRASS PLATA MIGUEL SNEIDER","172":"MANZANO CALVO JUAN SEBASTIAN","173":"MENDOZA GOITA MARIANSEL ZENAYDA","174":"MURILLO ARAQUE JAIVER GEOVANY","175":"NI\u00d1O ARENAS HECTOR GONZALO","176":"RAMIREZ CHAVERRA JHON EDISON","177":"XXX4","178":"XXX5","179":"XXX6","180":"RODRIGUEZ MOSQUERA LUIS FERNANDO","181":"PEPITO PEREZ","182":"RAMIREZ VARGAS MARCELA PAOLA","183":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","184":"TORO CISNEROS GARY JOSE","185":"USECHE CALDERON JADID ESTIVEN","186":"VASQUEZ NIETO CAMILO ANDRES","187":"JHONY CASTRO","188":"BERNAL JUAN DAVID","189":"XXX7","190":"XXX8","191":"XXX9","192":"BARON HERNANDEZ HAROLD ANTONIO","193":"CASTELLANOS CARVAJAL DEYVITH FABIAN","194":"AROCA TORRES JULIAN EDUARDO","195":"BERMUDEZ PARRA JENNIFER XIOMARA","196":"BERNAL BAQUERO JAMES RICARDO","197":"BURGOS ORTIZ JOSE HORACIO","198":"CANTOR PORRAS JUAN FERNEY","199":"CAPERA CAPERA JOSE GABRIEL","200":"CARDENAS LOTERO RICARDO ANDR\u00c9S","201":"RENDON OSPINA NELSON LEANDRO","202":"SARMIENTO URBINA MOISES DANIEL","203":"VELASCO VELASCO SEBASTI\u00c1N DAVID","204":"DELGADO DELGADO JOHAN DARIO","205":"FLOREZ SAUCESO KENIS ALBERTO","206":"CARDONA GARCIA OSCAR JAVIER","207":"CARVAJAL GARC\u00cdA HOVER MARCK","208":"CEPEDA PIRAQUIVE JUAN DAVID","209":"FAJARDO SAENZ OSCAR FERNANDO","210":"FLOREZ ESPITIA RONY ALBERTO","211":"GARCIA CUERVO EDWIN JAVIER","212":"GONZALEZ OCHOA JUAN CARLOS","213":"XXX1","214":"XXX2","215":"XXX3","216":"FONSECA RAY RICARDO","217":"GOMEZ BETANCUR JAIDER ANDRES","218":"GRANADA PATI\u00d1O CARLOS MARINO","219":"GRASS PLATA MIGUEL SNEIDER","220":"MANZANO CALVO JUAN SEBASTIAN","221":"MENDOZA GOITA MARIANSEL ZENAYDA","222":"MURILLO ARAQUE JAIVER GEOVANY","223":"NI\u00d1O ARENAS HECTOR GONZALO","224":"RAMIREZ CHAVERRA JHON EDISON","225":"XXX4","226":"XXX5","227":"XXX6","228":"RODRIGUEZ MOSQUERA LUIS FERNANDO","229":"PEPITO PEREZ","230":"RAMIREZ VARGAS MARCELA PAOLA","231":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","232":"TORO CISNEROS GARY JOSE","233":"USECHE CALDERON JADID ESTIVEN","234":"VASQUEZ NIETO CAMILO ANDRES","235":"JHONY CASTRO","236":"BERNAL JUAN DAVID","237":"XXX7","238":"XXX8","239":"XXX9","240":"BARON HERNANDEZ HAROLD ANTONIO","241":"CASTELLANOS CARVAJAL DEYVITH FABIAN","242":"AROCA TORRES JULIAN EDUARDO","243":"BERMUDEZ PARRA JENNIFER XIOMARA","244":"BERNAL BAQUERO JAMES RICARDO","245":"BURGOS ORTIZ JOSE HORACIO","246":"CANTOR PORRAS JUAN FERNEY","247":"CAPERA CAPERA JOSE GABRIEL","248":"CARDENAS LOTERO RICARDO ANDR\u00c9S","249":"RENDON OSPINA NELSON LEANDRO","250":"SARMIENTO URBINA MOISES DANIEL","251":"VELASCO VELASCO SEBASTI\u00c1N DAVID","252":"DELGADO DELGADO JOHAN DARIO","253":"FLOREZ SAUCESO KENIS ALBERTO","254":"CARDONA GARCIA OSCAR JAVIER","255":"CARVAJAL GARC\u00cdA HOVER MARCK","256":"CEPEDA PIRAQUIVE JUAN DAVID","257":"FAJARDO SAENZ OSCAR FERNANDO","258":"FLOREZ ESPITIA RONY ALBERTO","259":"GARCIA CUERVO EDWIN JAVIER","260":"GONZALEZ OCHOA JUAN CARLOS","261":"XXX1","262":"XXX2","263":"XXX3","264":"FONSECA RAY RICARDO","265":"GOMEZ BETANCUR JAIDER ANDRES","266":"GRANADA PATI\u00d1O CARLOS MARINO","267":"GR</t>

</xml_diff>

<commit_message>
Update historico_mallas.xlsx 2026-04-24 18:24:56.744201
</commit_message>
<xml_diff>
--- a/historico_mallas.xlsx
+++ b/historico_mallas.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="15">
   <si>
     <t>Mes</t>
   </si>
@@ -49,13 +49,16 @@
     <t>2026-04-24 18:15</t>
   </si>
   <si>
-    <t>2026-04-24 18:19</t>
+    <t>2026-04-24 18:24</t>
   </si>
   <si>
     <t>{"Grupo":{"0":"GRUPO 1","1":"GRUPO 1","2":"GRUPO 1","3":"GRUPO 1","4":"GRUPO 1","5":"GRUPO 1","6":"GRUPO 1","7":"GRUPO 1","8":"GRUPO 1","9":"GRUPO 1","10":"GRUPO 1","11":"GRUPO 1","12":"GRUPO 2","13":"GRUPO 2","14":"GRUPO 2","15":"GRUPO 2","16":"GRUPO 2","17":"GRUPO 2","18":"GRUPO 2","19":"GRUPO 2","20":"GRUPO 2","21":"GRUPO 2","22":"GRUPO 2","23":"GRUPO 2","24":"GRUPO 3","25":"GRUPO 3","26":"GRUPO 3","27":"GRUPO 3","28":"GRUPO 3","29":"GRUPO 3","30":"GRUPO 3","31":"GRUPO 3","32":"GRUPO 3","33":"GRUPO 3","34":"GRUPO 3","35":"GRUPO 3","36":"GRUPO 4","37":"GRUPO 4","38":"GRUPO 4","39":"GRUPO 4","40":"GRUPO 4","41":"GRUPO 4","42":"GRUPO 4","43":"GRUPO 4","44":"GRUPO 4","45":"GRUPO 4","46":"GRUPO 4","47":"GRUPO 4","48":"GRUPO 1","49":"GRUPO 1","50":"GRUPO 1","51":"GRUPO 1","52":"GRUPO 1","53":"GRUPO 1","54":"GRUPO 1","55":"GRUPO 1","56":"GRUPO 1","57":"GRUPO 1","58":"GRUPO 1","59":"GRUPO 1","60":"GRUPO 2","61":"GRUPO 2","62":"GRUPO 2","63":"GRUPO 2","64":"GRUPO 2","65":"GRUPO 2","66":"GRUPO 2","67":"GRUPO 2","68":"GRUPO 2","69":"GRUPO 2","70":"GRUPO 2","71":"GRUPO 2","72":"GRUPO 3","73":"GRUPO 3","74":"GRUPO 3","75":"GRUPO 3","76":"GRUPO 3","77":"GRUPO 3","78":"GRUPO 3","79":"GRUPO 3","80":"GRUPO 3","81":"GRUPO 3","82":"GRUPO 3","83":"GRUPO 3","84":"GRUPO 4","85":"GRUPO 4","86":"GRUPO 4","87":"GRUPO 4","88":"GRUPO 4","89":"GRUPO 4","90":"GRUPO 4","91":"GRUPO 4","92":"GRUPO 4","93":"GRUPO 4","94":"GRUPO 4","95":"GRUPO 4","96":"GRUPO 1","97":"GRUPO 1","98":"GRUPO 1","99":"GRUPO 1","100":"GRUPO 1","101":"GRUPO 1","102":"GRUPO 1","103":"GRUPO 1","104":"GRUPO 1","105":"GRUPO 1","106":"GRUPO 1","107":"GRUPO 1","108":"GRUPO 2","109":"GRUPO 2","110":"GRUPO 2","111":"GRUPO 2","112":"GRUPO 2","113":"GRUPO 2","114":"GRUPO 2","115":"GRUPO 2","116":"GRUPO 2","117":"GRUPO 2","118":"GRUPO 2","119":"GRUPO 2","120":"GRUPO 3","121":"GRUPO 3","122":"GRUPO 3","123":"GRUPO 3","124":"GRUPO 3","125":"GRUPO 3","126":"GRUPO 3","127":"GRUPO 3","128":"GRUPO 3","129":"GRUPO 3","130":"GRUPO 3","131":"GRUPO 3","132":"GRUPO 4","133":"GRUPO 4","134":"GRUPO 4","135":"GRUPO 4","136":"GRUPO 4","137":"GRUPO 4","138":"GRUPO 4","139":"GRUPO 4","140":"GRUPO 4","141":"GRUPO 4","142":"GRUPO 4","143":"GRUPO 4","144":"GRUPO 1","145":"GRUPO 1","146":"GRUPO 1","147":"GRUPO 1","148":"GRUPO 1","149":"GRUPO 1","150":"GRUPO 1","151":"GRUPO 1","152":"GRUPO 1","153":"GRUPO 1","154":"GRUPO 1","155":"GRUPO 1","156":"GRUPO 2","157":"GRUPO 2","158":"GRUPO 2","159":"GRUPO 2","160":"GRUPO 2","161":"GRUPO 2","162":"GRUPO 2","163":"GRUPO 2","164":"GRUPO 2","165":"GRUPO 2","166":"GRUPO 2","167":"GRUPO 2","168":"GRUPO 3","169":"GRUPO 3","170":"GRUPO 3","171":"GRUPO 3","172":"GRUPO 3","173":"GRUPO 3","174":"GRUPO 3","175":"GRUPO 3","176":"GRUPO 3","177":"GRUPO 3","178":"GRUPO 3","179":"GRUPO 3","180":"GRUPO 4","181":"GRUPO 4","182":"GRUPO 4","183":"GRUPO 4","184":"GRUPO 4","185":"GRUPO 4","186":"GRUPO 4","187":"GRUPO 4","188":"GRUPO 4","189":"GRUPO 4","190":"GRUPO 4","191":"GRUPO 4","192":"GRUPO 1","193":"GRUPO 1","194":"GRUPO 1","195":"GRUPO 1","196":"GRUPO 1","197":"GRUPO 1","198":"GRUPO 1","199":"GRUPO 1","200":"GRUPO 1","201":"GRUPO 1","202":"GRUPO 1","203":"GRUPO 1","204":"GRUPO 2","205":"GRUPO 2","206":"GRUPO 2","207":"GRUPO 2","208":"GRUPO 2","209":"GRUPO 2","210":"GRUPO 2","211":"GRUPO 2","212":"GRUPO 2","213":"GRUPO 2","214":"GRUPO 2","215":"GRUPO 2","216":"GRUPO 3","217":"GRUPO 3","218":"GRUPO 3","219":"GRUPO 3","220":"GRUPO 3","221":"GRUPO 3","222":"GRUPO 3","223":"GRUPO 3","224":"GRUPO 3","225":"GRUPO 3","226":"GRUPO 3","227":"GRUPO 3","228":"GRUPO 4","229":"GRUPO 4","230":"GRUPO 4","231":"GRUPO 4","232":"GRUPO 4","233":"GRUPO 4","234":"GRUPO 4","235":"GRUPO 4","236":"GRUPO 4","237":"GRUPO 4","238":"GRUPO 4","239":"GRUPO 4","240":"GRUPO 1","241":"GRUPO 1","242":"GRUPO 1","243":"GRUPO 1","244":"GRUPO 1","245":"GRUPO 1","246":"GRUPO 1","247":"GRUPO 1","248":"GRUPO 1","249":"GRUPO 1","250":"GRUPO 1","251":"GRUPO 1","252":"GRUPO 2","253":"GRUPO 2","254":"GRUPO 2","255":"GRUPO 2","256":"GRUPO 2","257":"GRUPO 2","258":"GRUPO 2","259":"GRUPO 2","260":"GRUPO 2","261":"GRUPO 2","262":"GRUPO 2","263":"GRUPO 2","264":"GRUPO 3","265":"GRUPO 3","266":"GRUPO 3","267":"GRUPO 3","268":"GRUPO 3","269":"GRUPO 3","270":"GRUPO 3","271":"GRUPO 3","272":"GRUPO 3","273":"GRUPO 3","274":"GRUPO 3","275":"GRUPO 3","276":"GRUPO 4","277":"GRUPO 4","278":"GRUPO 4","279":"GRUPO 4","280":"GRUPO 4","281":"GRUPO 4","282":"GRUPO 4","283":"GRUPO 4","284":"GRUPO 4","285":"GRUPO 4","286":"GRUPO 4","287":"GRUPO 4","288":"GRUPO 1","289":"GRUPO 1","290":"GRUPO 1","291":"GRUPO 1","292":"GRUPO 1","293":"GRUPO 1","294":"GRUPO 1","295":"GRUPO 1","296":"GRUPO 1","297":"GRUPO 1","298":"GRUPO 1","299":"GRUPO 1","300":"GRUPO 2","301":"GRUPO 2","302":"GRUPO 2","303":"GRUPO 2","304":"GRUPO 2","305":"GRUPO 2","306":"GRUPO 2","307":"GRUPO 2","308":"GRUPO 2","309":"GRUPO 2","310":"GRUPO 2","311":"GRUPO 2","312":"GRUPO 3","313":"GRUPO 3","314":"GRUPO 3","315":"GRUPO 3","316":"GRUPO 3","317":"GRUPO 3","318":"GRUPO 3","319":"GRUPO 3","320":"GRUPO 3","321":"GRUPO 3","322":"GRUPO 3","323":"GRUPO 3","324":"GRUPO 4","325":"GRUPO 4","326":"GRUPO 4","327":"GRUPO 4","328":"GRUPO 4","329":"GRUPO 4","330":"GRUPO 4","331":"GRUPO 4","332":"GRUPO 4","333":"GRUPO 4","334":"GRUPO 4","335":"GRUPO 4","336":"GRUPO 1","337":"GRUPO 1","338":"GRUPO 1","339":"GRUPO 1","340":"GRUPO 1","341":"GRUPO 1","342":"GRUPO 1","343":"GRUPO 1","344":"GRUPO 1","345":"GRUPO 1","346":"GRUPO 1","347":"GRUPO 1","348":"GRUPO 2","349":"GRUPO 2","350":"GRUPO 2","351":"GRUPO 2","352":"GRUPO 2","353":"GRUPO 2","354":"GRUPO 2","355":"GRUPO 2","356":"GRUPO 2","357":"GRUPO 2","358":"GRUPO 2","359":"GRUPO 2","360":"GRUPO 3","361":"GRUPO 3","362":"GRUPO 3","363":"GRUPO 3","364":"GRUPO 3","365":"GRUPO 3","366":"GRUPO 3","367":"GRUPO 3","368":"GRUPO 3","369":"GRUPO 3","370":"GRUPO 3","371":"GRUPO 3","372":"GRUPO 4","373":"GRUPO 4","374":"GRUPO 4","375":"GRUPO 4","376":"GRUPO 4","377":"GRUPO 4","378":"GRUPO 4","379":"GRUPO 4","380":"GRUPO 4","381":"GRUPO 4","382":"GRUPO 4","383":"GRUPO 4","384":"GRUPO 1","385":"GRUPO 1","386":"GRUPO 1","387":"GRUPO 1","388":"GRUPO 1","389":"GRUPO 1","390":"GRUPO 1","391":"GRUPO 1","392":"GRUPO 1","393":"GRUPO 1","394":"GRUPO 1","395":"GRUPO 1","396":"GRUPO 2","397":"GRUPO 2","398":"GRUPO 2","399":"GRUPO 2","400":"GRUPO 2","401":"GRUPO 2","402":"GRUPO 2","403":"GRUPO 2","404":"GRUPO 2","405":"GRUPO 2","406":"GRUPO 2","407":"GRUPO 2","408":"GRUPO 3","409":"GRUPO 3","410":"GRUPO 3","411":"GRUPO 3","412":"GRUPO 3","413":"GRUPO 3","414":"GRUPO 3","415":"GRUPO 3","416":"GRUPO 3","417":"GRUPO 3","418":"GRUPO 3","419":"GRUPO 3","420":"GRUPO 4","421":"GRUPO 4","422":"GRUPO 4","423":"GRUPO 4","424":"GRUPO 4","425":"GRUPO 4","426":"GRUPO 4","427":"GRUPO 4","428":"GRUPO 4","429":"GRUPO 4","430":"GRUPO 4","431":"GRUPO 4","432":"GRUPO 1","433":"GRUPO 1","434":"GRUPO 1","435":"GRUPO 1","436":"GRUPO 1","437":"GRUPO 1","438":"GRUPO 1","439":"GRUPO 1","440":"GRUPO 1","441":"GRUPO 1","442":"GRUPO 1","443":"GRUPO 1","444":"GRUPO 2","445":"GRUPO 2","446":"GRUPO 2","447":"GRUPO 2","448":"GRUPO 2","449":"GRUPO 2","450":"GRUPO 2","451":"GRUPO 2","452":"GRUPO 2","453":"GRUPO 2","454":"GRUPO 2","455":"GRUPO 2","456":"GRUPO 3","457":"GRUPO 3","458":"GRUPO 3","459":"GRUPO 3","460":"GRUPO 3","461":"GRUPO 3","462":"GRUPO 3","463":"GRUPO 3","464":"GRUPO 3","465":"GRUPO 3","466":"GRUPO 3","467":"GRUPO 3","468":"GRUPO 4","469":"GRUPO 4","470":"GRUPO 4","471":"GRUPO 4","472":"GRUPO 4","473":"GRUPO 4","474":"GRUPO 4","475":"GRUPO 4","476":"GRUPO 4","477":"GRUPO 4","478":"GRUPO 4","479":"GRUPO 4","480":"GRUPO 1","481":"GRUPO 1","482":"GRUPO 1","483":"GRUPO 1","484":"GRUPO 1","485":"GRUPO 1","486":"GRUPO 1","487":"GRUPO 1","488":"GRUPO 1","489":"GRUPO 1","490":"GRUPO 1","491":"GRUPO 1","492":"GRUPO 2","493":"GRUPO 2","494":"GRUPO 2","495":"GRUPO 2","496":"GRUPO 2","497":"GRUPO 2","498":"GRUPO 2","499":"GRUPO 2","500":"GRUPO 2","501":"GRUPO 2","502":"GRUPO 2","503":"GRUPO 2","504":"GRUPO 3","505":"GRUPO 3","506":"GRUPO 3","507":"GRUPO 3","508":"GRUPO 3","509":"GRUPO 3","510":"GRUPO 3","511":"GRUPO 3","512":"GRUPO 3","513":"GRUPO 3","514":"GRUPO 3","515":"GRUPO 3","516":"GRUPO 4","517":"GRUPO 4","518":"GRUPO 4","519":"GRUPO 4","520":"GRUPO 4","521":"GRUPO 4","522":"GRUPO 4","523":"GRUPO 4","524":"GRUPO 4","525":"GRUPO 4","526":"GRUPO 4","527":"GRUPO 4","528":"GRUPO 1","529":"GRUPO 1","530":"GRUPO 1","531":"GRUPO 1","532":"GRUPO 1","533":"GRUPO 1","534":"GRUPO 1","535":"GRUPO 1","536":"GRUPO 1","537":"GRUPO 1","538":"GRUPO 1","539":"GRUPO 1","540":"GRUPO 2","541":"GRUPO 2","542":"GRUPO 2","543":"GRUPO 2","544":"GRUPO 2","545":"GRUPO 2","546":"GRUPO 2","547":"GRUPO 2","548":"GRUPO 2","549":"GRUPO 2","550":"GRUPO 2","551":"GRUPO 2","552":"GRUPO 3","553":"GRUPO 3","554":"GRUPO 3","555":"GRUPO 3","556":"GRUPO 3","557":"GRUPO 3","558":"GRUPO 3","559":"GRUPO 3","560":"GRUPO 3","561":"GRUPO 3","562":"GRUPO 3","563":"GRUPO 3","564":"GRUPO 4","565":"GRUPO 4","566":"GRUPO 4","567":"GRUPO 4","568":"GRUPO 4","569":"GRUPO 4","570":"GRUPO 4","571":"GRUPO 4","572":"GRUPO 4","573":"GRUPO 4","574":"GRUPO 4","575":"GRUPO 4","576":"GRUPO 1","577":"GRUPO 1","578":"GRUPO 1","579":"GRUPO 1","580":"GRUPO 1","581":"GRUPO 1","582":"GRUPO 1","583":"GRUPO 1","584":"GRUPO 1","585":"GRUPO 1","586":"GRUPO 1","587":"GRUPO 1","588":"GRUPO 2","589":"GRUPO 2","590":"GRUPO 2","591":"GRUPO 2","592":"GRUPO 2","593":"GRUPO 2","594":"GRUPO 2","595":"GRUPO 2","596":"GRUPO 2","597":"GRUPO 2","598":"GRUPO 2","599":"GRUPO 2","600":"GRUPO 3","601":"GRUPO 3","602":"GRUPO 3","603":"GRUPO 3","604":"GRUPO 3","605":"GRUPO 3","606":"GRUPO 3","607":"GRUPO 3","608":"GRUPO 3","609":"GRUPO 3","610":"GRUPO 3","611":"GRUPO 3","612":"GRUPO 4","613":"GRUPO 4","614":"GRUPO 4","615":"GRUPO 4","616":"GRUPO 4","617":"GRUPO 4","618":"GRUPO 4","619":"GRUPO 4","620":"GRUPO 4","621":"GRUPO 4","622":"GRUPO 4","623":"GRUPO 4","624":"GRUPO 1","625":"GRUPO 1","626":"GRUPO 1","627":"GRUPO 1","628":"GRUPO 1","629":"GRUPO 1","630":"GRUPO 1","631":"GRUPO 1","632":"GRUPO 1","633":"GRUPO 1","634":"GRUPO 1","635":"GRUPO 1","636":"GRUPO 2","637":"GRUPO 2","638":"GRUPO 2","639":"GRUPO 2","640":"GRUPO 2","641":"GRUPO 2","642":"GRUPO 2","643":"GRUPO 2","644":"GRUPO 2","645":"GRUPO 2","646":"GRUPO 2","647":"GRUPO 2","648":"GRUPO 3","649":"GRUPO 3","650":"GRUPO 3","651":"GRUPO 3","652":"GRUPO 3","653":"GRUPO 3","654":"GRUPO 3","655":"GRUPO 3","656":"GRUPO 3","657":"GRUPO 3","658":"GRUPO 3","659":"GRUPO 3","660":"GRUPO 4","661":"GRUPO 4","662":"GRUPO 4","663":"GRUPO 4","664":"GRUPO 4","665":"GRUPO 4","666":"GRUPO 4","667":"GRUPO 4","668":"GRUPO 4","669":"GRUPO 4","670":"GRUPO 4","671":"GRUPO 4","672":"GRUPO 1","673":"GRUPO 1","674":"GRUPO 1","675":"GRUPO 1","676":"GRUPO 1","677":"GRUPO 1","678":"GRUPO 1","679":"GRUPO 1","680":"GRUPO 1","681":"GRUPO 1","682":"GRUPO 1","683":"GRUPO 1","684":"GRUPO 2","685":"GRUPO 2","686":"GRUPO 2","687":"GRUPO 2","688":"GRUPO 2","689":"GRUPO 2","690":"GRUPO 2","691":"GRUPO 2","692":"GRUPO 2","693":"GRUPO 2","694":"GRUPO 2","695":"GRUPO 2","696":"GRUPO 3","697":"GRUPO 3","698":"GRUPO 3","699":"GRUPO 3","700":"GRUPO 3","701":"GRUPO 3","702":"GRUPO 3","703":"GRUPO 3","704":"GRUPO 3","705":"GRUPO 3","706":"GRUPO 3","707":"GRUPO 3","708":"GRUPO 4","709":"GRUPO 4","710":"GRUPO 4","711":"GRUPO 4","712":"GRUPO 4","713":"GRUPO 4","714":"GRUPO 4","715":"GRUPO 4","716":"GRUPO 4","717":"GRUPO 4","718":"GRUPO 4","719":"GRUPO 4","720":"GRUPO 1","721":"GRUPO 1","722":"GRUPO 1","723":"GRUPO 1","724":"GRUPO 1","725":"GRUPO 1","726":"GRUPO 1","727":"GRUPO 1","728":"GRUPO 1","729":"GRUPO 1","730":"GRUPO 1","731":"GRUPO 1","732":"GRUPO 2","733":"GRUPO 2","734":"GRUPO 2","735":"GRUPO 2","736":"GRUPO 2","737":"GRUPO 2","738":"GRUPO 2","739":"GRUPO 2","740":"GRUPO 2","741":"GRUPO 2","742":"GRUPO 2","743":"GRUPO 2","744":"GRUPO 3","745":"GRUPO 3","746":"GRUPO 3","747":"GRUPO 3","748":"GRUPO 3","749":"GRUPO 3","750":"GRUPO 3","751":"GRUPO 3","752":"GRUPO 3","753":"GRUPO 3","754":"GRUPO 3","755":"GRUPO 3","756":"GRUPO 4","757":"GRUPO 4","758":"GRUPO 4","759":"GRUPO 4","760":"GRUPO 4","761":"GRUPO 4","762":"GRUPO 4","763":"GRUPO 4","764":"GRUPO 4","765":"GRUPO 4","766":"GRUPO 4","767":"GRUPO 4","768":"GRUPO 1","769":"GRUPO 1","770":"GRUPO 1","771":"GRUPO 1","772":"GRUPO 1","773":"GRUPO 1","774":"GRUPO 1","775":"GRUPO 1","776":"GRUPO 1","777":"GRUPO 1","778":"GRUPO 1","779":"GRUPO 1","780":"GRUPO 2","781":"GRUPO 2","782":"GRUPO 2","783":"GRUPO 2","784":"GRUPO 2","785":"GRUPO 2","786":"GRUPO 2","787":"GRUPO 2","788":"GRUPO 2","789":"GRUPO 2","790":"GRUPO 2","791":"GRUPO 2","792":"GRUPO 3","793":"GRUPO 3","794":"GRUPO 3","795":"GRUPO 3","796":"GRUPO 3","797":"GRUPO 3","798":"GRUPO 3","799":"GRUPO 3","800":"GRUPO 3","801":"GRUPO 3","802":"GRUPO 3","803":"GRUPO 3","804":"GRUPO 4","805":"GRUPO 4","806":"GRUPO 4","807":"GRUPO 4","808":"GRUPO 4","809":"GRUPO 4","810":"GRUPO 4","811":"GRUPO 4","812":"GRUPO 4","813":"GRUPO 4","814":"GRUPO 4","815":"GRUPO 4","816":"GRUPO 1","817":"GRUPO 1","818":"GRUPO 1","819":"GRUPO 1","820":"GRUPO 1","821":"GRUPO 1","822":"GRUPO 1","823":"GRUPO 1","824":"GRUPO 1","825":"GRUPO 1","826":"GRUPO 1","827":"GRUPO 1","828":"GRUPO 2","829":"GRUPO 2","830":"GRUPO 2","831":"GRUPO 2","832":"GRUPO 2","833":"GRUPO 2","834":"GRUPO 2","835":"GRUPO 2","836":"GRUPO 2","837":"GRUPO 2","838":"GRUPO 2","839":"GRUPO 2","840":"GRUPO 3","841":"GRUPO 3","842":"GRUPO 3","843":"GRUPO 3","844":"GRUPO 3","845":"GRUPO 3","846":"GRUPO 3","847":"GRUPO 3","848":"GRUPO 3","849":"GRUPO 3","850":"GRUPO 3","851":"GRUPO 3","852":"GRUPO 4","853":"GRUPO 4","854":"GRUPO 4","855":"GRUPO 4","856":"GRUPO 4","857":"GRUPO 4","858":"GRUPO 4","859":"GRUPO 4","860":"GRUPO 4","861":"GRUPO 4","862":"GRUPO 4","863":"GRUPO 4","864":"GRUPO 1","865":"GRUPO 1","866":"GRUPO 1","867":"GRUPO 1","868":"GRUPO 1","869":"GRUPO 1","870":"GRUPO 1","871":"GRUPO 1","872":"GRUPO 1","873":"GRUPO 1","874":"GRUPO 1","875":"GRUPO 1","876":"GRUPO 2","877":"GRUPO 2","878":"GRUPO 2","879":"GRUPO 2","880":"GRUPO 2","881":"GRUPO 2","882":"GRUPO 2","883":"GRUPO 2","884":"GRUPO 2","885":"GRUPO 2","886":"GRUPO 2","887":"GRUPO 2","888":"GRUPO 3","889":"GRUPO 3","890":"GRUPO 3","891":"GRUPO 3","892":"GRUPO 3","893":"GRUPO 3","894":"GRUPO 3","895":"GRUPO 3","896":"GRUPO 3","897":"GRUPO 3","898":"GRUPO 3","899":"GRUPO 3","900":"GRUPO 4","901":"GRUPO 4","902":"GRUPO 4","903":"GRUPO 4","904":"GRUPO 4","905":"GRUPO 4","906":"GRUPO 4","907":"GRUPO 4","908":"GRUPO 4","909":"GRUPO 4","910":"GRUPO 4","911":"GRUPO 4","912":"GRUPO 1","913":"GRUPO 1","914":"GRUPO 1","915":"GRUPO 1","916":"GRUPO 1","917":"GRUPO 1","918":"GRUPO 1","919":"GRUPO 1","920":"GRUPO 1","921":"GRUPO 1","922":"GRUPO 1","923":"GRUPO 1","924":"GRUPO 2","925":"GRUPO 2","926":"GRUPO 2","927":"GRUPO 2","928":"GRUPO 2","929":"GRUPO 2","930":"GRUPO 2","931":"GRUPO 2","932":"GRUPO 2","933":"GRUPO 2","934":"GRUPO 2","935":"GRUPO 2","936":"GRUPO 3","937":"GRUPO 3","938":"GRUPO 3","939":"GRUPO 3","940":"GRUPO 3","941":"GRUPO 3","942":"GRUPO 3","943":"GRUPO 3","944":"GRUPO 3","945":"GRUPO 3","946":"GRUPO 3","947":"GRUPO 3","948":"GRUPO 4","949":"GRUPO 4","950":"GRUPO 4","951":"GRUPO 4","952":"GRUPO 4","953":"GRUPO 4","954":"GRUPO 4","955":"GRUPO 4","956":"GRUPO 4","957":"GRUPO 4","958":"GRUPO 4","959":"GRUPO 4","960":"GRUPO 1","961":"GRUPO 1","962":"GRUPO 1","963":"GRUPO 1","964":"GRUPO 1","965":"GRUPO 1","966":"GRUPO 1","967":"GRUPO 1","968":"GRUPO 1","969":"GRUPO 1","970":"GRUPO 1","971":"GRUPO 1","972":"GRUPO 2","973":"GRUPO 2","974":"GRUPO 2","975":"GRUPO 2","976":"GRUPO 2","977":"GRUPO 2","978":"GRUPO 2","979":"GRUPO 2","980":"GRUPO 2","981":"GRUPO 2","982":"GRUPO 2","983":"GRUPO 2","984":"GRUPO 3","985":"GRUPO 3","986":"GRUPO 3","987":"GRUPO 3","988":"GRUPO 3","989":"GRUPO 3","990":"GRUPO 3","991":"GRUPO 3","992":"GRUPO 3","993":"GRUPO 3","994":"GRUPO 3","995":"GRUPO 3","996":"GRUPO 4","997":"GRUPO 4","998":"GRUPO 4","999":"GRUPO 4","1000":"GRUPO 4","1001":"GRUPO 4","1002":"GRUPO 4","1003":"GRUPO 4","1004":"GRUPO 4","1005":"GRUPO 4","1006":"GRUPO 4","1007":"GRUPO 4","1008":"GRUPO 1","1009":"GRUPO 1","1010":"GRUPO 1","1011":"GRUPO 1","1012":"GRUPO 1","1013":"GRUPO 1","1014":"GRUPO 1","1015":"GRUPO 1","1016":"GRUPO 1","1017":"GRUPO 1","1018":"GRUPO 1","1019":"GRUPO 1","1020":"GRUPO 2","1021":"GRUPO 2","1022":"GRUPO 2","1023":"GRUPO 2","1024":"GRUPO 2","1025":"GRUPO 2","1026":"GRUPO 2","1027":"GRUPO 2","1028":"GRUPO 2","1029":"GRUPO 2","1030":"GRUPO 2","1031":"GRUPO 2","1032":"GRUPO 3","1033":"GRUPO 3","1034":"GRUPO 3","1035":"GRUPO 3","1036":"GRUPO 3","1037":"GRUPO 3","1038":"GRUPO 3","1039":"GRUPO 3","1040":"GRUPO 3","1041":"GRUPO 3","1042":"GRUPO 3","1043":"GRUPO 3","1044":"GRUPO 4","1045":"GRUPO 4","1046":"GRUPO 4","1047":"GRUPO 4","1048":"GRUPO 4","1049":"GRUPO 4","1050":"GRUPO 4","1051":"GRUPO 4","1052":"GRUPO 4","1053":"GRUPO 4","1054":"GRUPO 4","1055":"GRUPO 4","1056":"GRUPO 1","1057":"GRUPO 1","1058":"GRUPO 1","1059":"GRUPO 1","1060":"GRUPO 1","1061":"GRUPO 1","1062":"GRUPO 1","1063":"GRUPO 1","1064":"GRUPO 1","1065":"GRUPO 1","1066":"GRUPO 1","1067":"GRUPO 1","1068":"GRUPO 2","1069":"GRUPO 2","1070":"GRUPO 2","1071":"GRUPO 2","1072":"GRUPO 2","1073":"GRUPO 2","1074":"GRUPO 2","1075":"GRUPO 2","1076":"GRUPO 2","1077":"GRUPO 2","1078":"GRUPO 2","1079":"GRUPO 2","1080":"GRUPO 3","1081":"GRUPO 3","1082":"GRUPO 3","1083":"GRUPO 3","1084":"GRUPO 3","1085":"GRUPO 3","1086":"GRUPO 3","1087":"GRUPO 3","1088":"GRUPO 3","1089":"GRUPO 3","1090":"GRUPO 3","1091":"GRUPO 3","1092":"GRUPO 4","1093":"GRUPO 4","1094":"GRUPO 4","1095":"GRUPO 4","1096":"GRUPO 4","1097":"GRUPO 4","1098":"GRUPO 4","1099":"GRUPO 4","1100":"GRUPO 4","1101":"GRUPO 4","1102":"GRUPO 4","1103":"GRUPO 4","1104":"GRUPO 1","1105":"GRUPO 1","1106":"GRUPO 1","1107":"GRUPO 1","1108":"GRUPO 1","1109":"GRUPO 1","1110":"GRUPO 1","1111":"GRUPO 1","1112":"GRUPO 1","1113":"GRUPO 1","1114":"GRUPO 1","1115":"GRUPO 1","1116":"GRUPO 2","1117":"GRUPO 2","1118":"GRUPO 2","1119":"GRUPO 2","1120":"GRUPO 2","1121":"GRUPO 2","1122":"GRUPO 2","1123":"GRUPO 2","1124":"GRUPO 2","1125":"GRUPO 2","1126":"GRUPO 2","1127":"GRUPO 2","1128":"GRUPO 3","1129":"GRUPO 3","1130":"GRUPO 3","1131":"GRUPO 3","1132":"GRUPO 3","1133":"GRUPO 3","1134":"GRUPO 3","1135":"GRUPO 3","1136":"GRUPO 3","1137":"GRUPO 3","1138":"GRUPO 3","1139":"GRUPO 3","1140":"GRUPO 4","1141":"GRUPO 4","1142":"GRUPO 4","1143":"GRUPO 4","1144":"GRUPO 4","1145":"GRUPO 4","1146":"GRUPO 4","1147":"GRUPO 4","1148":"GRUPO 4","1149":"GRUPO 4","1150":"GRUPO 4","1151":"GRUPO 4","1152":"GRUPO 1","1153":"GRUPO 1","1154":"GRUPO 1","1155":"GRUPO 1","1156":"GRUPO 1","1157":"GRUPO 1","1158":"GRUPO 1","1159":"GRUPO 1","1160":"GRUPO 1","1161":"GRUPO 1","1162":"GRUPO 1","1163":"GRUPO 1","1164":"GRUPO 2","1165":"GRUPO 2","1166":"GRUPO 2","1167":"GRUPO 2","1168":"GRUPO 2","1169":"GRUPO 2","1170":"GRUPO 2","1171":"GRUPO 2","1172":"GRUPO 2","1173":"GRUPO 2","1174":"GRUPO 2","1175":"GRUPO 2","1176":"GRUPO 3","1177":"GRUPO 3","1178":"GRUPO 3","1179":"GRUPO 3","1180":"GRUPO 3","1181":"GRUPO 3","1182":"GRUPO 3","1183":"GRUPO 3","1184":"GRUPO 3","1185":"GRUPO 3","1186":"GRUPO 3","1187":"GRUPO 3","1188":"GRUPO 4","1189":"GRUPO 4","1190":"GRUPO 4","1191":"GRUPO 4","1192":"GRUPO 4","1193":"GRUPO 4","1194":"GRUPO 4","1195":"GRUPO 4","1196":"GRUPO 4","1197":"GRUPO 4","1198":"GRUPO 4","1199":"GRUPO 4","1200":"GRUPO 1","1201":"GRUPO 1","1202":"GRUPO 1","1203":"GRUPO 1","1204":"GRUPO 1","1205":"GRUPO 1","1206":"GRUPO 1","1207":"GRUPO 1","1208":"GRUPO 1","1209":"GRUPO 1","1210":"GRUPO 1","1211":"GRUPO 1","1212":"GRUPO 2","1213":"GRUPO 2","1214":"GRUPO 2","1215":"GRUPO 2","1216":"GRUPO 2","1217":"GRUPO 2","1218":"GRUPO 2","1219":"GRUPO 2","1220":"GRUPO 2","1221":"GRUPO 2","1222":"GRUPO 2","1223":"GRUPO 2","1224":"GRUPO 3","1225":"GRUPO 3","1226":"GRUPO 3","1227":"GRUPO 3","1228":"GRUPO 3","1229":"GRUPO 3","1230":"GRUPO 3","1231":"GRUPO 3","1232":"GRUPO 3","1233":"GRUPO 3","1234":"GRUPO 3","1235":"GRUPO 3","1236":"GRUPO 4","1237":"GRUPO 4","1238":"GRUPO 4","1239":"GRUPO 4","1240":"GRUPO 4","1241":"GRUPO 4","1242":"GRUPO 4","1243":"GRUPO 4","1244":"GRUPO 4","1245":"GRUPO 4","1246":"GRUPO 4","1247":"GRUPO 4","1248":"GRUPO 1","1249":"GRUPO 1","1250":"GRUPO 1","1251":"GRUPO 1","1252":"GRUPO 1","1253":"GRUPO 1","1254":"GRUPO 1","1255":"GRUPO 1","1256":"GRUPO 1","1257":"GRUPO 1","1258":"GRUPO 1","1259":"GRUPO 1","1260":"GRUPO 2","1261":"GRUPO 2","1262":"GRUPO 2","1263":"GRUPO 2","1264":"GRUPO 2","1265":"GRUPO 2","1266":"GRUPO 2","1267":"GRUPO 2","1268":"GRUPO 2","1269":"GRUPO 2","1270":"GRUPO 2","1271":"GRUPO 2","1272":"GRUPO 3","1273":"GRUPO 3","1274":"GRUPO 3","1275":"GRUPO 3","1276":"GRUPO 3","1277":"GRUPO 3","1278":"GRUPO 3","1279":"GRUPO 3","1280":"GRUPO 3","1281":"GRUPO 3","1282":"GRUPO 3","1283":"GRUPO 3","1284":"GRUPO 4","1285":"GRUPO 4","1286":"GRUPO 4","1287":"GRUPO 4","1288":"GRUPO 4","1289":"GRUPO 4","1290":"GRUPO 4","1291":"GRUPO 4","1292":"GRUPO 4","1293":"GRUPO 4","1294":"GRUPO 4","1295":"GRUPO 4","1296":"GRUPO 1","1297":"GRUPO 1","1298":"GRUPO 1","1299":"GRUPO 1","1300":"GRUPO 1","1301":"GRUPO 1","1302":"GRUPO 1","1303":"GRUPO 1","1304":"GRUPO 1","1305":"GRUPO 1","1306":"GRUPO 1","1307":"GRUPO 1","1308":"GRUPO 2","1309":"GRUPO 2","1310":"GRUPO 2","1311":"GRUPO 2","1312":"GRUPO 2","1313":"GRUPO 2","1314":"GRUPO 2","1315":"GRUPO 2","1316":"GRUPO 2","1317":"GRUPO 2","1318":"GRUPO 2","1319":"GRUPO 2","1320":"GRUPO 3","1321":"GRUPO 3","1322":"GRUPO 3","1323":"GRUPO 3","1324":"GRUPO 3","1325":"GRUPO 3","1326":"GRUPO 3","1327":"GRUPO 3","1328":"GRUPO 3","1329":"GRUPO 3","1330":"GRUPO 3","1331":"GRUPO 3","1332":"GRUPO 4","1333":"GRUPO 4","1334":"GRUPO 4","1335":"GRUPO 4","1336":"GRUPO 4","1337":"GRUPO 4","1338":"GRUPO 4","1339":"GRUPO 4","1340":"GRUPO 4","1341":"GRUPO 4","1342":"GRUPO 4","1343":"GRUPO 4","1344":"GRUPO 1","1345":"GRUPO 1","1346":"GRUPO 1","1347":"GRUPO 1","1348":"GRUPO 1","1349":"GRUPO 1","1350":"GRUPO 1","1351":"GRUPO 1","1352":"GRUPO 1","1353":"GRUPO 1","1354":"GRUPO 1","1355":"GRUPO 1","1356":"GRUPO 2","1357":"GRUPO 2","1358":"GRUPO 2","1359":"GRUPO 2","1360":"GRUPO 2","1361":"GRUPO 2","1362":"GRUPO 2","1363":"GRUPO 2","1364":"GRUPO 2","1365":"GRUPO 2","1366":"GRUPO 2","1367":"GRUPO 2","1368":"GRUPO 3","1369":"GRUPO 3","1370":"GRUPO 3","1371":"GRUPO 3","1372":"GRUPO 3","1373":"GRUPO 3","1374":"GRUPO 3","1375":"GRUPO 3","1376":"GRUPO 3","1377":"GRUPO 3","1378":"GRUPO 3","1379":"GRUPO 3","1380":"GRUPO 4","1381":"GRUPO 4","1382":"GRUPO 4","1383":"GRUPO 4","1384":"GRUPO 4","1385":"GRUPO 4","1386":"GRUPO 4","1387":"GRUPO 4","1388":"GRUPO 4","1389":"GRUPO 4","1390":"GRUPO 4","1391":"GRUPO 4","1392":"GRUPO 1","1393":"GRUPO 1","1394":"GRUPO 1","1395":"GRUPO 1","1396":"GRUPO 1","1397":"GRUPO 1","1398":"GRUPO 1","1399":"GRUPO 1","1400":"GRUPO 1","1401":"GRUPO 1","1402":"GRUPO 1","1403":"GRUPO 1","1404":"GRUPO 2","1405":"GRUPO 2","1406":"GRUPO 2","1407":"GRUPO 2","1408":"GRUPO 2","1409":"GRUPO 2","1410":"GRUPO 2","1411":"GRUPO 2","1412":"GRUPO 2","1413":"GRUPO 2","1414":"GRUPO 2","1415":"GRUPO 2","1416":"GRUPO 3","1417":"GRUPO 3","1418":"GRUPO 3","1419":"GRUPO 3","1420":"GRUPO 3","1421":"GRUPO 3","1422":"GRUPO 3","1423":"GRUPO 3","1424":"GRUPO 3","1425":"GRUPO 3","1426":"GRUPO 3","1427":"GRUPO 3","1428":"GRUPO 4","1429":"GRUPO 4","1430":"GRUPO 4","1431":"GRUPO 4","1432":"GRUPO 4","1433":"GRUPO 4","1434":"GRUPO 4","1435":"GRUPO 4","1436":"GRUPO 4","1437":"GRUPO 4","1438":"GRUPO 4","1439":"GRUPO 4","1440":"GRUPO 1","1441":"GRUPO 1","1442":"GRUPO 1","1443":"GRUPO 1","1444":"GRUPO 1","1445":"GRUPO 1","1446":"GRUPO 1","1447":"GRUPO 1","1448":"GRUPO 1","1449":"GRUPO 1","1450":"GRUPO 1","1451":"GRUPO 1","1452":"GRUPO 2","1453":"GRUPO 2","1454":"GRUPO 2","1455":"GRUPO 2","1456":"GRUPO 2","1457":"GRUPO 2","1458":"GRUPO 2","1459":"GRUPO 2","1460":"GRUPO 2","1461":"GRUPO 2","1462":"GRUPO 2","1463":"GRUPO 2","1464":"GRUPO 3","1465":"GRUPO 3","1466":"GRUPO 3","1467":"GRUPO 3","1468":"GRUPO 3","1469":"GRUPO 3","1470":"GRUPO 3","1471":"GRUPO 3","1472":"GRUPO 3","1473":"GRUPO 3","1474":"GRUPO 3","1475":"GRUPO 3","1476":"GRUPO 4","1477":"GRUPO 4","1478":"GRUPO 4","1479":"GRUPO 4","1480":"GRUPO 4","1481":"GRUPO 4","1482":"GRUPO 4","1483":"GRUPO 4","1484":"GRUPO 4","1485":"GRUPO 4","1486":"GRUPO 4","1487":"GRUPO 4"},"Empleado":{"0":"BARON HERNANDEZ HAROLD ANTONIO","1":"CASTELLANOS CARVAJAL DEYVITH FABIAN","2":"AROCA TORRES JULIAN EDUARDO","3":"BERMUDEZ PARRA JENNIFER XIOMARA","4":"BERNAL BAQUERO JAMES RICARDO","5":"BURGOS ORTIZ JOSE HORACIO","6":"CANTOR PORRAS JUAN FERNEY","7":"CAPERA CAPERA JOSE GABRIEL","8":"CARDENAS LOTERO RICARDO ANDR\u00c9S","9":"RENDON OSPINA NELSON LEANDRO","10":"SARMIENTO URBINA MOISES DANIEL","11":"VELASCO VELASCO SEBASTI\u00c1N DAVID","12":"DELGADO DELGADO JOHAN DARIO","13":"FLOREZ SAUCESO KENIS ALBERTO","14":"CARDONA GARCIA OSCAR JAVIER","15":"CARVAJAL GARC\u00cdA HOVER MARCK","16":"CEPEDA PIRAQUIVE JUAN DAVID","17":"FAJARDO SAENZ OSCAR FERNANDO","18":"FLOREZ ESPITIA RONY ALBERTO","19":"GARCIA CUERVO EDWIN JAVIER","20":"GONZALEZ OCHOA JUAN CARLOS","21":"XXX1","22":"XXX2","23":"XXX3","24":"FONSECA RAY RICARDO","25":"GOMEZ BETANCUR JAIDER ANDRES","26":"GRANADA PATI\u00d1O CARLOS MARINO","27":"GRASS PLATA MIGUEL SNEIDER","28":"MANZANO CALVO JUAN SEBASTIAN","29":"MENDOZA GOITA MARIANSEL ZENAYDA","30":"MURILLO ARAQUE JAIVER GEOVANY","31":"NI\u00d1O ARENAS HECTOR GONZALO","32":"RAMIREZ CHAVERRA JHON EDISON","33":"XXX4","34":"XXX5","35":"XXX6","36":"RODRIGUEZ MOSQUERA LUIS FERNANDO","37":"PEPITO PEREZ","38":"RAMIREZ VARGAS MARCELA PAOLA","39":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","40":"TORO CISNEROS GARY JOSE","41":"USECHE CALDERON JADID ESTIVEN","42":"VASQUEZ NIETO CAMILO ANDRES","43":"JHONY CASTRO","44":"BERNAL JUAN DAVID","45":"XXX7","46":"XXX8","47":"XXX9","48":"BARON HERNANDEZ HAROLD ANTONIO","49":"CASTELLANOS CARVAJAL DEYVITH FABIAN","50":"AROCA TORRES JULIAN EDUARDO","51":"BERMUDEZ PARRA JENNIFER XIOMARA","52":"BERNAL BAQUERO JAMES RICARDO","53":"BURGOS ORTIZ JOSE HORACIO","54":"CANTOR PORRAS JUAN FERNEY","55":"CAPERA CAPERA JOSE GABRIEL","56":"CARDENAS LOTERO RICARDO ANDR\u00c9S","57":"RENDON OSPINA NELSON LEANDRO","58":"SARMIENTO URBINA MOISES DANIEL","59":"VELASCO VELASCO SEBASTI\u00c1N DAVID","60":"DELGADO DELGADO JOHAN DARIO","61":"FLOREZ SAUCESO KENIS ALBERTO","62":"CARDONA GARCIA OSCAR JAVIER","63":"CARVAJAL GARC\u00cdA HOVER MARCK","64":"CEPEDA PIRAQUIVE JUAN DAVID","65":"FAJARDO SAENZ OSCAR FERNANDO","66":"FLOREZ ESPITIA RONY ALBERTO","67":"GARCIA CUERVO EDWIN JAVIER","68":"GONZALEZ OCHOA JUAN CARLOS","69":"XXX1","70":"XXX2","71":"XXX3","72":"FONSECA RAY RICARDO","73":"GOMEZ BETANCUR JAIDER ANDRES","74":"GRANADA PATI\u00d1O CARLOS MARINO","75":"GRASS PLATA MIGUEL SNEIDER","76":"MANZANO CALVO JUAN SEBASTIAN","77":"MENDOZA GOITA MARIANSEL ZENAYDA","78":"MURILLO ARAQUE JAIVER GEOVANY","79":"NI\u00d1O ARENAS HECTOR GONZALO","80":"RAMIREZ CHAVERRA JHON EDISON","81":"XXX4","82":"XXX5","83":"XXX6","84":"RODRIGUEZ MOSQUERA LUIS FERNANDO","85":"PEPITO PEREZ","86":"RAMIREZ VARGAS MARCELA PAOLA","87":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","88":"TORO CISNEROS GARY JOSE","89":"USECHE CALDERON JADID ESTIVEN","90":"VASQUEZ NIETO CAMILO ANDRES","91":"JHONY CASTRO","92":"BERNAL JUAN DAVID","93":"XXX7","94":"XXX8","95":"XXX9","96":"BARON HERNANDEZ HAROLD ANTONIO","97":"CASTELLANOS CARVAJAL DEYVITH FABIAN","98":"AROCA TORRES JULIAN EDUARDO","99":"BERMUDEZ PARRA JENNIFER XIOMARA","100":"BERNAL BAQUERO JAMES RICARDO","101":"BURGOS ORTIZ JOSE HORACIO","102":"CANTOR PORRAS JUAN FERNEY","103":"CAPERA CAPERA JOSE GABRIEL","104":"CARDENAS LOTERO RICARDO ANDR\u00c9S","105":"RENDON OSPINA NELSON LEANDRO","106":"SARMIENTO URBINA MOISES DANIEL","107":"VELASCO VELASCO SEBASTI\u00c1N DAVID","108":"DELGADO DELGADO JOHAN DARIO","109":"FLOREZ SAUCESO KENIS ALBERTO","110":"CARDONA GARCIA OSCAR JAVIER","111":"CARVAJAL GARC\u00cdA HOVER MARCK","112":"CEPEDA PIRAQUIVE JUAN DAVID","113":"FAJARDO SAENZ OSCAR FERNANDO","114":"FLOREZ ESPITIA RONY ALBERTO","115":"GARCIA CUERVO EDWIN JAVIER","116":"GONZALEZ OCHOA JUAN CARLOS","117":"XXX1","118":"XXX2","119":"XXX3","120":"FONSECA RAY RICARDO","121":"GOMEZ BETANCUR JAIDER ANDRES","122":"GRANADA PATI\u00d1O CARLOS MARINO","123":"GRASS PLATA MIGUEL SNEIDER","124":"MANZANO CALVO JUAN SEBASTIAN","125":"MENDOZA GOITA MARIANSEL ZENAYDA","126":"MURILLO ARAQUE JAIVER GEOVANY","127":"NI\u00d1O ARENAS HECTOR GONZALO","128":"RAMIREZ CHAVERRA JHON EDISON","129":"XXX4","130":"XXX5","131":"XXX6","132":"RODRIGUEZ MOSQUERA LUIS FERNANDO","133":"PEPITO PEREZ","134":"RAMIREZ VARGAS MARCELA PAOLA","135":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","136":"TORO CISNEROS GARY JOSE","137":"USECHE CALDERON JADID ESTIVEN","138":"VASQUEZ NIETO CAMILO ANDRES","139":"JHONY CASTRO","140":"BERNAL JUAN DAVID","141":"XXX7","142":"XXX8","143":"XXX9","144":"BARON HERNANDEZ HAROLD ANTONIO","145":"CASTELLANOS CARVAJAL DEYVITH FABIAN","146":"AROCA TORRES JULIAN EDUARDO","147":"BERMUDEZ PARRA JENNIFER XIOMARA","148":"BERNAL BAQUERO JAMES RICARDO","149":"BURGOS ORTIZ JOSE HORACIO","150":"CANTOR PORRAS JUAN FERNEY","151":"CAPERA CAPERA JOSE GABRIEL","152":"CARDENAS LOTERO RICARDO ANDR\u00c9S","153":"RENDON OSPINA NELSON LEANDRO","154":"SARMIENTO URBINA MOISES DANIEL","155":"VELASCO VELASCO SEBASTI\u00c1N DAVID","156":"DELGADO DELGADO JOHAN DARIO","157":"FLOREZ SAUCESO KENIS ALBERTO","158":"CARDONA GARCIA OSCAR JAVIER","159":"CARVAJAL GARC\u00cdA HOVER MARCK","160":"CEPEDA PIRAQUIVE JUAN DAVID","161":"FAJARDO SAENZ OSCAR FERNANDO","162":"FLOREZ ESPITIA RONY ALBERTO","163":"GARCIA CUERVO EDWIN JAVIER","164":"GONZALEZ OCHOA JUAN CARLOS","165":"XXX1","166":"XXX2","167":"XXX3","168":"FONSECA RAY RICARDO","169":"GOMEZ BETANCUR JAIDER ANDRES","170":"GRANADA PATI\u00d1O CARLOS MARINO","171":"GRASS PLATA MIGUEL SNEIDER","172":"MANZANO CALVO JUAN SEBASTIAN","173":"MENDOZA GOITA MARIANSEL ZENAYDA","174":"MURILLO ARAQUE JAIVER GEOVANY","175":"NI\u00d1O ARENAS HECTOR GONZALO","176":"RAMIREZ CHAVERRA JHON EDISON","177":"XXX4","178":"XXX5","179":"XXX6","180":"RODRIGUEZ MOSQUERA LUIS FERNANDO","181":"PEPITO PEREZ","182":"RAMIREZ VARGAS MARCELA PAOLA","183":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","184":"TORO CISNEROS GARY JOSE","185":"USECHE CALDERON JADID ESTIVEN","186":"VASQUEZ NIETO CAMILO ANDRES","187":"JHONY CASTRO","188":"BERNAL JUAN DAVID","189":"XXX7","190":"XXX8","191":"XXX9","192":"BARON HERNANDEZ HAROLD ANTONIO","193":"CASTELLANOS CARVAJAL DEYVITH FABIAN","194":"AROCA TORRES JULIAN EDUARDO","195":"BERMUDEZ PARRA JENNIFER XIOMARA","196":"BERNAL BAQUERO JAMES RICARDO","197":"BURGOS ORTIZ JOSE HORACIO","198":"CANTOR PORRAS JUAN FERNEY","199":"CAPERA CAPERA JOSE GABRIEL","200":"CARDENAS LOTERO RICARDO ANDR\u00c9S","201":"RENDON OSPINA NELSON LEANDRO","202":"SARMIENTO URBINA MOISES DANIEL","203":"VELASCO VELASCO SEBASTI\u00c1N DAVID","204":"DELGADO DELGADO JOHAN DARIO","205":"FLOREZ SAUCESO KENIS ALBERTO","206":"CARDONA GARCIA OSCAR JAVIER","207":"CARVAJAL GARC\u00cdA HOVER MARCK","208":"CEPEDA PIRAQUIVE JUAN DAVID","209":"FAJARDO SAENZ OSCAR FERNANDO","210":"FLOREZ ESPITIA RONY ALBERTO","211":"GARCIA CUERVO EDWIN JAVIER","212":"GONZALEZ OCHOA JUAN CARLOS","213":"XXX1","214":"XXX2","215":"XXX3","216":"FONSECA RAY RICARDO","217":"GOMEZ BETANCUR JAIDER ANDRES","218":"GRANADA PATI\u00d1O CARLOS MARINO","219":"GRASS PLATA MIGUEL SNEIDER","220":"MANZANO CALVO JUAN SEBASTIAN","221":"MENDOZA GOITA MARIANSEL ZENAYDA","222":"MURILLO ARAQUE JAIVER GEOVANY","223":"NI\u00d1O ARENAS HECTOR GONZALO","224":"RAMIREZ CHAVERRA JHON EDISON","225":"XXX4","226":"XXX5","227":"XXX6","228":"RODRIGUEZ MOSQUERA LUIS FERNANDO","229":"PEPITO PEREZ","230":"RAMIREZ VARGAS MARCELA PAOLA","231":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","232":"TORO CISNEROS GARY JOSE","233":"USECHE CALDERON JADID ESTIVEN","234":"VASQUEZ NIETO CAMILO ANDRES","235":"JHONY CASTRO","236":"BERNAL JUAN DAVID","237":"XXX7","238":"XXX8","239":"XXX9","240":"BARON HERNANDEZ HAROLD ANTONIO","241":"CASTELLANOS CARVAJAL DEYVITH FABIAN","242":"AROCA TORRES JULIAN EDUARDO","243":"BERMUDEZ PARRA JENNIFER XIOMARA","244":"BERNAL BAQUERO JAMES RICARDO","245":"BURGOS ORTIZ JOSE HORACIO","246":"CANTOR PORRAS JUAN FERNEY","247":"CAPERA CAPERA JOSE GABRIEL","248":"CARDENAS LOTERO RICARDO ANDR\u00c9S","249":"RENDON OSPINA NELSON LEANDRO","250":"SARMIENTO URBINA MOISES DANIEL","251":"VELASCO VELASCO SEBASTI\u00c1N DAVID","252":"DELGADO DELGADO JOHAN DARIO","253":"FLOREZ SAUCESO KENIS ALBERTO","254":"CARDONA GARCIA OSCAR JAVIER","255":"CARVAJAL GARC\u00cdA HOVER MARCK","256":"CEPEDA PIRAQUIVE JUAN DAVID","257":"FAJARDO SAENZ OSCAR FERNANDO","258":"FLOREZ ESPITIA RONY ALBERTO","259":"GARCIA CUERVO EDWIN JAVIER","260":"GONZALEZ OCHOA JUAN CARLOS","261":"XXX1","262":"XXX2","263":"XXX3","264":"FONSECA RAY RICARDO","265":"GOMEZ BETANCUR JAIDER ANDRES","266":"GRANADA PATI\u00d1O CARLOS MARINO","267":"GR</t>
   </si>
   <si>
     <t>{"Grupo":{"0":"GRUPO 1","1":"GRUPO 1","2":"GRUPO 1","3":"GRUPO 1","4":"GRUPO 1","5":"GRUPO 1","6":"GRUPO 1","7":"GRUPO 1","8":"GRUPO 1","9":"GRUPO 1","10":"GRUPO 1","11":"GRUPO 1","12":"GRUPO 2","13":"GRUPO 2","14":"GRUPO 2","15":"GRUPO 2","16":"GRUPO 2","17":"GRUPO 2","18":"GRUPO 2","19":"GRUPO 2","20":"GRUPO 2","21":"GRUPO 2","22":"GRUPO 2","23":"GRUPO 2","24":"GRUPO 3","25":"GRUPO 3","26":"GRUPO 3","27":"GRUPO 3","28":"GRUPO 3","29":"GRUPO 3","30":"GRUPO 3","31":"GRUPO 3","32":"GRUPO 3","33":"GRUPO 3","34":"GRUPO 3","35":"GRUPO 3","36":"GRUPO 4","37":"GRUPO 4","38":"GRUPO 4","39":"GRUPO 4","40":"GRUPO 4","41":"GRUPO 4","42":"GRUPO 4","43":"GRUPO 4","44":"GRUPO 4","45":"GRUPO 4","46":"GRUPO 4","47":"GRUPO 4","48":"GRUPO 1","49":"GRUPO 1","50":"GRUPO 1","51":"GRUPO 1","52":"GRUPO 1","53":"GRUPO 1","54":"GRUPO 1","55":"GRUPO 1","56":"GRUPO 1","57":"GRUPO 1","58":"GRUPO 1","59":"GRUPO 1","60":"GRUPO 2","61":"GRUPO 2","62":"GRUPO 2","63":"GRUPO 2","64":"GRUPO 2","65":"GRUPO 2","66":"GRUPO 2","67":"GRUPO 2","68":"GRUPO 2","69":"GRUPO 2","70":"GRUPO 2","71":"GRUPO 2","72":"GRUPO 3","73":"GRUPO 3","74":"GRUPO 3","75":"GRUPO 3","76":"GRUPO 3","77":"GRUPO 3","78":"GRUPO 3","79":"GRUPO 3","80":"GRUPO 3","81":"GRUPO 3","82":"GRUPO 3","83":"GRUPO 3","84":"GRUPO 4","85":"GRUPO 4","86":"GRUPO 4","87":"GRUPO 4","88":"GRUPO 4","89":"GRUPO 4","90":"GRUPO 4","91":"GRUPO 4","92":"GRUPO 4","93":"GRUPO 4","94":"GRUPO 4","95":"GRUPO 4","96":"GRUPO 1","97":"GRUPO 1","98":"GRUPO 1","99":"GRUPO 1","100":"GRUPO 1","101":"GRUPO 1","102":"GRUPO 1","103":"GRUPO 1","104":"GRUPO 1","105":"GRUPO 1","106":"GRUPO 1","107":"GRUPO 1","108":"GRUPO 2","109":"GRUPO 2","110":"GRUPO 2","111":"GRUPO 2","112":"GRUPO 2","113":"GRUPO 2","114":"GRUPO 2","115":"GRUPO 2","116":"GRUPO 2","117":"GRUPO 2","118":"GRUPO 2","119":"GRUPO 2","120":"GRUPO 3","121":"GRUPO 3","122":"GRUPO 3","123":"GRUPO 3","124":"GRUPO 3","125":"GRUPO 3","126":"GRUPO 3","127":"GRUPO 3","128":"GRUPO 3","129":"GRUPO 3","130":"GRUPO 3","131":"GRUPO 3","132":"GRUPO 4","133":"GRUPO 4","134":"GRUPO 4","135":"GRUPO 4","136":"GRUPO 4","137":"GRUPO 4","138":"GRUPO 4","139":"GRUPO 4","140":"GRUPO 4","141":"GRUPO 4","142":"GRUPO 4","143":"GRUPO 4","144":"GRUPO 1","145":"GRUPO 1","146":"GRUPO 1","147":"GRUPO 1","148":"GRUPO 1","149":"GRUPO 1","150":"GRUPO 1","151":"GRUPO 1","152":"GRUPO 1","153":"GRUPO 1","154":"GRUPO 1","155":"GRUPO 1","156":"GRUPO 2","157":"GRUPO 2","158":"GRUPO 2","159":"GRUPO 2","160":"GRUPO 2","161":"GRUPO 2","162":"GRUPO 2","163":"GRUPO 2","164":"GRUPO 2","165":"GRUPO 2","166":"GRUPO 2","167":"GRUPO 2","168":"GRUPO 3","169":"GRUPO 3","170":"GRUPO 3","171":"GRUPO 3","172":"GRUPO 3","173":"GRUPO 3","174":"GRUPO 3","175":"GRUPO 3","176":"GRUPO 3","177":"GRUPO 3","178":"GRUPO 3","179":"GRUPO 3","180":"GRUPO 4","181":"GRUPO 4","182":"GRUPO 4","183":"GRUPO 4","184":"GRUPO 4","185":"GRUPO 4","186":"GRUPO 4","187":"GRUPO 4","188":"GRUPO 4","189":"GRUPO 4","190":"GRUPO 4","191":"GRUPO 4","192":"GRUPO 1","193":"GRUPO 1","194":"GRUPO 1","195":"GRUPO 1","196":"GRUPO 1","197":"GRUPO 1","198":"GRUPO 1","199":"GRUPO 1","200":"GRUPO 1","201":"GRUPO 1","202":"GRUPO 1","203":"GRUPO 1","204":"GRUPO 2","205":"GRUPO 2","206":"GRUPO 2","207":"GRUPO 2","208":"GRUPO 2","209":"GRUPO 2","210":"GRUPO 2","211":"GRUPO 2","212":"GRUPO 2","213":"GRUPO 2","214":"GRUPO 2","215":"GRUPO 2","216":"GRUPO 3","217":"GRUPO 3","218":"GRUPO 3","219":"GRUPO 3","220":"GRUPO 3","221":"GRUPO 3","222":"GRUPO 3","223":"GRUPO 3","224":"GRUPO 3","225":"GRUPO 3","226":"GRUPO 3","227":"GRUPO 3","228":"GRUPO 4","229":"GRUPO 4","230":"GRUPO 4","231":"GRUPO 4","232":"GRUPO 4","233":"GRUPO 4","234":"GRUPO 4","235":"GRUPO 4","236":"GRUPO 4","237":"GRUPO 4","238":"GRUPO 4","239":"GRUPO 4","240":"GRUPO 1","241":"GRUPO 1","242":"GRUPO 1","243":"GRUPO 1","244":"GRUPO 1","245":"GRUPO 1","246":"GRUPO 1","247":"GRUPO 1","248":"GRUPO 1","249":"GRUPO 1","250":"GRUPO 1","251":"GRUPO 1","252":"GRUPO 2","253":"GRUPO 2","254":"GRUPO 2","255":"GRUPO 2","256":"GRUPO 2","257":"GRUPO 2","258":"GRUPO 2","259":"GRUPO 2","260":"GRUPO 2","261":"GRUPO 2","262":"GRUPO 2","263":"GRUPO 2","264":"GRUPO 3","265":"GRUPO 3","266":"GRUPO 3","267":"GRUPO 3","268":"GRUPO 3","269":"GRUPO 3","270":"GRUPO 3","271":"GRUPO 3","272":"GRUPO 3","273":"GRUPO 3","274":"GRUPO 3","275":"GRUPO 3","276":"GRUPO 4","277":"GRUPO 4","278":"GRUPO 4","279":"GRUPO 4","280":"GRUPO 4","281":"GRUPO 4","282":"GRUPO 4","283":"GRUPO 4","284":"GRUPO 4","285":"GRUPO 4","286":"GRUPO 4","287":"GRUPO 4","288":"GRUPO 1","289":"GRUPO 1","290":"GRUPO 1","291":"GRUPO 1","292":"GRUPO 1","293":"GRUPO 1","294":"GRUPO 1","295":"GRUPO 1","296":"GRUPO 1","297":"GRUPO 1","298":"GRUPO 1","299":"GRUPO 1","300":"GRUPO 2","301":"GRUPO 2","302":"GRUPO 2","303":"GRUPO 2","304":"GRUPO 2","305":"GRUPO 2","306":"GRUPO 2","307":"GRUPO 2","308":"GRUPO 2","309":"GRUPO 2","310":"GRUPO 2","311":"GRUPO 2","312":"GRUPO 3","313":"GRUPO 3","314":"GRUPO 3","315":"GRUPO 3","316":"GRUPO 3","317":"GRUPO 3","318":"GRUPO 3","319":"GRUPO 3","320":"GRUPO 3","321":"GRUPO 3","322":"GRUPO 3","323":"GRUPO 3","324":"GRUPO 4","325":"GRUPO 4","326":"GRUPO 4","327":"GRUPO 4","328":"GRUPO 4","329":"GRUPO 4","330":"GRUPO 4","331":"GRUPO 4","332":"GRUPO 4","333":"GRUPO 4","334":"GRUPO 4","335":"GRUPO 4","336":"GRUPO 1","337":"GRUPO 1","338":"GRUPO 1","339":"GRUPO 1","340":"GRUPO 1","341":"GRUPO 1","342":"GRUPO 1","343":"GRUPO 1","344":"GRUPO 1","345":"GRUPO 1","346":"GRUPO 1","347":"GRUPO 1","348":"GRUPO 2","349":"GRUPO 2","350":"GRUPO 2","351":"GRUPO 2","352":"GRUPO 2","353":"GRUPO 2","354":"GRUPO 2","355":"GRUPO 2","356":"GRUPO 2","357":"GRUPO 2","358":"GRUPO 2","359":"GRUPO 2","360":"GRUPO 3","361":"GRUPO 3","362":"GRUPO 3","363":"GRUPO 3","364":"GRUPO 3","365":"GRUPO 3","366":"GRUPO 3","367":"GRUPO 3","368":"GRUPO 3","369":"GRUPO 3","370":"GRUPO 3","371":"GRUPO 3","372":"GRUPO 4","373":"GRUPO 4","374":"GRUPO 4","375":"GRUPO 4","376":"GRUPO 4","377":"GRUPO 4","378":"GRUPO 4","379":"GRUPO 4","380":"GRUPO 4","381":"GRUPO 4","382":"GRUPO 4","383":"GRUPO 4","384":"GRUPO 1","385":"GRUPO 1","386":"GRUPO 1","387":"GRUPO 1","388":"GRUPO 1","389":"GRUPO 1","390":"GRUPO 1","391":"GRUPO 1","392":"GRUPO 1","393":"GRUPO 1","394":"GRUPO 1","395":"GRUPO 1","396":"GRUPO 2","397":"GRUPO 2","398":"GRUPO 2","399":"GRUPO 2","400":"GRUPO 2","401":"GRUPO 2","402":"GRUPO 2","403":"GRUPO 2","404":"GRUPO 2","405":"GRUPO 2","406":"GRUPO 2","407":"GRUPO 2","408":"GRUPO 3","409":"GRUPO 3","410":"GRUPO 3","411":"GRUPO 3","412":"GRUPO 3","413":"GRUPO 3","414":"GRUPO 3","415":"GRUPO 3","416":"GRUPO 3","417":"GRUPO 3","418":"GRUPO 3","419":"GRUPO 3","420":"GRUPO 4","421":"GRUPO 4","422":"GRUPO 4","423":"GRUPO 4","424":"GRUPO 4","425":"GRUPO 4","426":"GRUPO 4","427":"GRUPO 4","428":"GRUPO 4","429":"GRUPO 4","430":"GRUPO 4","431":"GRUPO 4","432":"GRUPO 1","433":"GRUPO 1","434":"GRUPO 1","435":"GRUPO 1","436":"GRUPO 1","437":"GRUPO 1","438":"GRUPO 1","439":"GRUPO 1","440":"GRUPO 1","441":"GRUPO 1","442":"GRUPO 1","443":"GRUPO 1","444":"GRUPO 2","445":"GRUPO 2","446":"GRUPO 2","447":"GRUPO 2","448":"GRUPO 2","449":"GRUPO 2","450":"GRUPO 2","451":"GRUPO 2","452":"GRUPO 2","453":"GRUPO 2","454":"GRUPO 2","455":"GRUPO 2","456":"GRUPO 3","457":"GRUPO 3","458":"GRUPO 3","459":"GRUPO 3","460":"GRUPO 3","461":"GRUPO 3","462":"GRUPO 3","463":"GRUPO 3","464":"GRUPO 3","465":"GRUPO 3","466":"GRUPO 3","467":"GRUPO 3","468":"GRUPO 4","469":"GRUPO 4","470":"GRUPO 4","471":"GRUPO 4","472":"GRUPO 4","473":"GRUPO 4","474":"GRUPO 4","475":"GRUPO 4","476":"GRUPO 4","477":"GRUPO 4","478":"GRUPO 4","479":"GRUPO 4","480":"GRUPO 1","481":"GRUPO 1","482":"GRUPO 1","483":"GRUPO 1","484":"GRUPO 1","485":"GRUPO 1","486":"GRUPO 1","487":"GRUPO 1","488":"GRUPO 1","489":"GRUPO 1","490":"GRUPO 1","491":"GRUPO 1","492":"GRUPO 2","493":"GRUPO 2","494":"GRUPO 2","495":"GRUPO 2","496":"GRUPO 2","497":"GRUPO 2","498":"GRUPO 2","499":"GRUPO 2","500":"GRUPO 2","501":"GRUPO 2","502":"GRUPO 2","503":"GRUPO 2","504":"GRUPO 3","505":"GRUPO 3","506":"GRUPO 3","507":"GRUPO 3","508":"GRUPO 3","509":"GRUPO 3","510":"GRUPO 3","511":"GRUPO 3","512":"GRUPO 3","513":"GRUPO 3","514":"GRUPO 3","515":"GRUPO 3","516":"GRUPO 4","517":"GRUPO 4","518":"GRUPO 4","519":"GRUPO 4","520":"GRUPO 4","521":"GRUPO 4","522":"GRUPO 4","523":"GRUPO 4","524":"GRUPO 4","525":"GRUPO 4","526":"GRUPO 4","527":"GRUPO 4","528":"GRUPO 1","529":"GRUPO 1","530":"GRUPO 1","531":"GRUPO 1","532":"GRUPO 1","533":"GRUPO 1","534":"GRUPO 1","535":"GRUPO 1","536":"GRUPO 1","537":"GRUPO 1","538":"GRUPO 1","539":"GRUPO 1","540":"GRUPO 2","541":"GRUPO 2","542":"GRUPO 2","543":"GRUPO 2","544":"GRUPO 2","545":"GRUPO 2","546":"GRUPO 2","547":"GRUPO 2","548":"GRUPO 2","549":"GRUPO 2","550":"GRUPO 2","551":"GRUPO 2","552":"GRUPO 3","553":"GRUPO 3","554":"GRUPO 3","555":"GRUPO 3","556":"GRUPO 3","557":"GRUPO 3","558":"GRUPO 3","559":"GRUPO 3","560":"GRUPO 3","561":"GRUPO 3","562":"GRUPO 3","563":"GRUPO 3","564":"GRUPO 4","565":"GRUPO 4","566":"GRUPO 4","567":"GRUPO 4","568":"GRUPO 4","569":"GRUPO 4","570":"GRUPO 4","571":"GRUPO 4","572":"GRUPO 4","573":"GRUPO 4","574":"GRUPO 4","575":"GRUPO 4","576":"GRUPO 1","577":"GRUPO 1","578":"GRUPO 1","579":"GRUPO 1","580":"GRUPO 1","581":"GRUPO 1","582":"GRUPO 1","583":"GRUPO 1","584":"GRUPO 1","585":"GRUPO 1","586":"GRUPO 1","587":"GRUPO 1","588":"GRUPO 2","589":"GRUPO 2","590":"GRUPO 2","591":"GRUPO 2","592":"GRUPO 2","593":"GRUPO 2","594":"GRUPO 2","595":"GRUPO 2","596":"GRUPO 2","597":"GRUPO 2","598":"GRUPO 2","599":"GRUPO 2","600":"GRUPO 3","601":"GRUPO 3","602":"GRUPO 3","603":"GRUPO 3","604":"GRUPO 3","605":"GRUPO 3","606":"GRUPO 3","607":"GRUPO 3","608":"GRUPO 3","609":"GRUPO 3","610":"GRUPO 3","611":"GRUPO 3","612":"GRUPO 4","613":"GRUPO 4","614":"GRUPO 4","615":"GRUPO 4","616":"GRUPO 4","617":"GRUPO 4","618":"GRUPO 4","619":"GRUPO 4","620":"GRUPO 4","621":"GRUPO 4","622":"GRUPO 4","623":"GRUPO 4","624":"GRUPO 1","625":"GRUPO 1","626":"GRUPO 1","627":"GRUPO 1","628":"GRUPO 1","629":"GRUPO 1","630":"GRUPO 1","631":"GRUPO 1","632":"GRUPO 1","633":"GRUPO 1","634":"GRUPO 1","635":"GRUPO 1","636":"GRUPO 2","637":"GRUPO 2","638":"GRUPO 2","639":"GRUPO 2","640":"GRUPO 2","641":"GRUPO 2","642":"GRUPO 2","643":"GRUPO 2","644":"GRUPO 2","645":"GRUPO 2","646":"GRUPO 2","647":"GRUPO 2","648":"GRUPO 3","649":"GRUPO 3","650":"GRUPO 3","651":"GRUPO 3","652":"GRUPO 3","653":"GRUPO 3","654":"GRUPO 3","655":"GRUPO 3","656":"GRUPO 3","657":"GRUPO 3","658":"GRUPO 3","659":"GRUPO 3","660":"GRUPO 4","661":"GRUPO 4","662":"GRUPO 4","663":"GRUPO 4","664":"GRUPO 4","665":"GRUPO 4","666":"GRUPO 4","667":"GRUPO 4","668":"GRUPO 4","669":"GRUPO 4","670":"GRUPO 4","671":"GRUPO 4","672":"GRUPO 1","673":"GRUPO 1","674":"GRUPO 1","675":"GRUPO 1","676":"GRUPO 1","677":"GRUPO 1","678":"GRUPO 1","679":"GRUPO 1","680":"GRUPO 1","681":"GRUPO 1","682":"GRUPO 1","683":"GRUPO 1","684":"GRUPO 2","685":"GRUPO 2","686":"GRUPO 2","687":"GRUPO 2","688":"GRUPO 2","689":"GRUPO 2","690":"GRUPO 2","691":"GRUPO 2","692":"GRUPO 2","693":"GRUPO 2","694":"GRUPO 2","695":"GRUPO 2","696":"GRUPO 3","697":"GRUPO 3","698":"GRUPO 3","699":"GRUPO 3","700":"GRUPO 3","701":"GRUPO 3","702":"GRUPO 3","703":"GRUPO 3","704":"GRUPO 3","705":"GRUPO 3","706":"GRUPO 3","707":"GRUPO 3","708":"GRUPO 4","709":"GRUPO 4","710":"GRUPO 4","711":"GRUPO 4","712":"GRUPO 4","713":"GRUPO 4","714":"GRUPO 4","715":"GRUPO 4","716":"GRUPO 4","717":"GRUPO 4","718":"GRUPO 4","719":"GRUPO 4","720":"GRUPO 1","721":"GRUPO 1","722":"GRUPO 1","723":"GRUPO 1","724":"GRUPO 1","725":"GRUPO 1","726":"GRUPO 1","727":"GRUPO 1","728":"GRUPO 1","729":"GRUPO 1","730":"GRUPO 1","731":"GRUPO 1","732":"GRUPO 2","733":"GRUPO 2","734":"GRUPO 2","735":"GRUPO 2","736":"GRUPO 2","737":"GRUPO 2","738":"GRUPO 2","739":"GRUPO 2","740":"GRUPO 2","741":"GRUPO 2","742":"GRUPO 2","743":"GRUPO 2","744":"GRUPO 3","745":"GRUPO 3","746":"GRUPO 3","747":"GRUPO 3","748":"GRUPO 3","749":"GRUPO 3","750":"GRUPO 3","751":"GRUPO 3","752":"GRUPO 3","753":"GRUPO 3","754":"GRUPO 3","755":"GRUPO 3","756":"GRUPO 4","757":"GRUPO 4","758":"GRUPO 4","759":"GRUPO 4","760":"GRUPO 4","761":"GRUPO 4","762":"GRUPO 4","763":"GRUPO 4","764":"GRUPO 4","765":"GRUPO 4","766":"GRUPO 4","767":"GRUPO 4","768":"GRUPO 1","769":"GRUPO 1","770":"GRUPO 1","771":"GRUPO 1","772":"GRUPO 1","773":"GRUPO 1","774":"GRUPO 1","775":"GRUPO 1","776":"GRUPO 1","777":"GRUPO 1","778":"GRUPO 1","779":"GRUPO 1","780":"GRUPO 2","781":"GRUPO 2","782":"GRUPO 2","783":"GRUPO 2","784":"GRUPO 2","785":"GRUPO 2","786":"GRUPO 2","787":"GRUPO 2","788":"GRUPO 2","789":"GRUPO 2","790":"GRUPO 2","791":"GRUPO 2","792":"GRUPO 3","793":"GRUPO 3","794":"GRUPO 3","795":"GRUPO 3","796":"GRUPO 3","797":"GRUPO 3","798":"GRUPO 3","799":"GRUPO 3","800":"GRUPO 3","801":"GRUPO 3","802":"GRUPO 3","803":"GRUPO 3","804":"GRUPO 4","805":"GRUPO 4","806":"GRUPO 4","807":"GRUPO 4","808":"GRUPO 4","809":"GRUPO 4","810":"GRUPO 4","811":"GRUPO 4","812":"GRUPO 4","813":"GRUPO 4","814":"GRUPO 4","815":"GRUPO 4","816":"GRUPO 1","817":"GRUPO 1","818":"GRUPO 1","819":"GRUPO 1","820":"GRUPO 1","821":"GRUPO 1","822":"GRUPO 1","823":"GRUPO 1","824":"GRUPO 1","825":"GRUPO 1","826":"GRUPO 1","827":"GRUPO 1","828":"GRUPO 2","829":"GRUPO 2","830":"GRUPO 2","831":"GRUPO 2","832":"GRUPO 2","833":"GRUPO 2","834":"GRUPO 2","835":"GRUPO 2","836":"GRUPO 2","837":"GRUPO 2","838":"GRUPO 2","839":"GRUPO 2","840":"GRUPO 3","841":"GRUPO 3","842":"GRUPO 3","843":"GRUPO 3","844":"GRUPO 3","845":"GRUPO 3","846":"GRUPO 3","847":"GRUPO 3","848":"GRUPO 3","849":"GRUPO 3","850":"GRUPO 3","851":"GRUPO 3","852":"GRUPO 4","853":"GRUPO 4","854":"GRUPO 4","855":"GRUPO 4","856":"GRUPO 4","857":"GRUPO 4","858":"GRUPO 4","859":"GRUPO 4","860":"GRUPO 4","861":"GRUPO 4","862":"GRUPO 4","863":"GRUPO 4","864":"GRUPO 1","865":"GRUPO 1","866":"GRUPO 1","867":"GRUPO 1","868":"GRUPO 1","869":"GRUPO 1","870":"GRUPO 1","871":"GRUPO 1","872":"GRUPO 1","873":"GRUPO 1","874":"GRUPO 1","875":"GRUPO 1","876":"GRUPO 2","877":"GRUPO 2","878":"GRUPO 2","879":"GRUPO 2","880":"GRUPO 2","881":"GRUPO 2","882":"GRUPO 2","883":"GRUPO 2","884":"GRUPO 2","885":"GRUPO 2","886":"GRUPO 2","887":"GRUPO 2","888":"GRUPO 3","889":"GRUPO 3","890":"GRUPO 3","891":"GRUPO 3","892":"GRUPO 3","893":"GRUPO 3","894":"GRUPO 3","895":"GRUPO 3","896":"GRUPO 3","897":"GRUPO 3","898":"GRUPO 3","899":"GRUPO 3","900":"GRUPO 4","901":"GRUPO 4","902":"GRUPO 4","903":"GRUPO 4","904":"GRUPO 4","905":"GRUPO 4","906":"GRUPO 4","907":"GRUPO 4","908":"GRUPO 4","909":"GRUPO 4","910":"GRUPO 4","911":"GRUPO 4","912":"GRUPO 1","913":"GRUPO 1","914":"GRUPO 1","915":"GRUPO 1","916":"GRUPO 1","917":"GRUPO 1","918":"GRUPO 1","919":"GRUPO 1","920":"GRUPO 1","921":"GRUPO 1","922":"GRUPO 1","923":"GRUPO 1","924":"GRUPO 2","925":"GRUPO 2","926":"GRUPO 2","927":"GRUPO 2","928":"GRUPO 2","929":"GRUPO 2","930":"GRUPO 2","931":"GRUPO 2","932":"GRUPO 2","933":"GRUPO 2","934":"GRUPO 2","935":"GRUPO 2","936":"GRUPO 3","937":"GRUPO 3","938":"GRUPO 3","939":"GRUPO 3","940":"GRUPO 3","941":"GRUPO 3","942":"GRUPO 3","943":"GRUPO 3","944":"GRUPO 3","945":"GRUPO 3","946":"GRUPO 3","947":"GRUPO 3","948":"GRUPO 4","949":"GRUPO 4","950":"GRUPO 4","951":"GRUPO 4","952":"GRUPO 4","953":"GRUPO 4","954":"GRUPO 4","955":"GRUPO 4","956":"GRUPO 4","957":"GRUPO 4","958":"GRUPO 4","959":"GRUPO 4","960":"GRUPO 1","961":"GRUPO 1","962":"GRUPO 1","963":"GRUPO 1","964":"GRUPO 1","965":"GRUPO 1","966":"GRUPO 1","967":"GRUPO 1","968":"GRUPO 1","969":"GRUPO 1","970":"GRUPO 1","971":"GRUPO 1","972":"GRUPO 2","973":"GRUPO 2","974":"GRUPO 2","975":"GRUPO 2","976":"GRUPO 2","977":"GRUPO 2","978":"GRUPO 2","979":"GRUPO 2","980":"GRUPO 2","981":"GRUPO 2","982":"GRUPO 2","983":"GRUPO 2","984":"GRUPO 3","985":"GRUPO 3","986":"GRUPO 3","987":"GRUPO 3","988":"GRUPO 3","989":"GRUPO 3","990":"GRUPO 3","991":"GRUPO 3","992":"GRUPO 3","993":"GRUPO 3","994":"GRUPO 3","995":"GRUPO 3","996":"GRUPO 4","997":"GRUPO 4","998":"GRUPO 4","999":"GRUPO 4","1000":"GRUPO 4","1001":"GRUPO 4","1002":"GRUPO 4","1003":"GRUPO 4","1004":"GRUPO 4","1005":"GRUPO 4","1006":"GRUPO 4","1007":"GRUPO 4","1008":"GRUPO 1","1009":"GRUPO 1","1010":"GRUPO 1","1011":"GRUPO 1","1012":"GRUPO 1","1013":"GRUPO 1","1014":"GRUPO 1","1015":"GRUPO 1","1016":"GRUPO 1","1017":"GRUPO 1","1018":"GRUPO 1","1019":"GRUPO 1","1020":"GRUPO 2","1021":"GRUPO 2","1022":"GRUPO 2","1023":"GRUPO 2","1024":"GRUPO 2","1025":"GRUPO 2","1026":"GRUPO 2","1027":"GRUPO 2","1028":"GRUPO 2","1029":"GRUPO 2","1030":"GRUPO 2","1031":"GRUPO 2","1032":"GRUPO 3","1033":"GRUPO 3","1034":"GRUPO 3","1035":"GRUPO 3","1036":"GRUPO 3","1037":"GRUPO 3","1038":"GRUPO 3","1039":"GRUPO 3","1040":"GRUPO 3","1041":"GRUPO 3","1042":"GRUPO 3","1043":"GRUPO 3","1044":"GRUPO 4","1045":"GRUPO 4","1046":"GRUPO 4","1047":"GRUPO 4","1048":"GRUPO 4","1049":"GRUPO 4","1050":"GRUPO 4","1051":"GRUPO 4","1052":"GRUPO 4","1053":"GRUPO 4","1054":"GRUPO 4","1055":"GRUPO 4","1056":"GRUPO 1","1057":"GRUPO 1","1058":"GRUPO 1","1059":"GRUPO 1","1060":"GRUPO 1","1061":"GRUPO 1","1062":"GRUPO 1","1063":"GRUPO 1","1064":"GRUPO 1","1065":"GRUPO 1","1066":"GRUPO 1","1067":"GRUPO 1","1068":"GRUPO 2","1069":"GRUPO 2","1070":"GRUPO 2","1071":"GRUPO 2","1072":"GRUPO 2","1073":"GRUPO 2","1074":"GRUPO 2","1075":"GRUPO 2","1076":"GRUPO 2","1077":"GRUPO 2","1078":"GRUPO 2","1079":"GRUPO 2","1080":"GRUPO 3","1081":"GRUPO 3","1082":"GRUPO 3","1083":"GRUPO 3","1084":"GRUPO 3","1085":"GRUPO 3","1086":"GRUPO 3","1087":"GRUPO 3","1088":"GRUPO 3","1089":"GRUPO 3","1090":"GRUPO 3","1091":"GRUPO 3","1092":"GRUPO 4","1093":"GRUPO 4","1094":"GRUPO 4","1095":"GRUPO 4","1096":"GRUPO 4","1097":"GRUPO 4","1098":"GRUPO 4","1099":"GRUPO 4","1100":"GRUPO 4","1101":"GRUPO 4","1102":"GRUPO 4","1103":"GRUPO 4","1104":"GRUPO 1","1105":"GRUPO 1","1106":"GRUPO 1","1107":"GRUPO 1","1108":"GRUPO 1","1109":"GRUPO 1","1110":"GRUPO 1","1111":"GRUPO 1","1112":"GRUPO 1","1113":"GRUPO 1","1114":"GRUPO 1","1115":"GRUPO 1","1116":"GRUPO 2","1117":"GRUPO 2","1118":"GRUPO 2","1119":"GRUPO 2","1120":"GRUPO 2","1121":"GRUPO 2","1122":"GRUPO 2","1123":"GRUPO 2","1124":"GRUPO 2","1125":"GRUPO 2","1126":"GRUPO 2","1127":"GRUPO 2","1128":"GRUPO 3","1129":"GRUPO 3","1130":"GRUPO 3","1131":"GRUPO 3","1132":"GRUPO 3","1133":"GRUPO 3","1134":"GRUPO 3","1135":"GRUPO 3","1136":"GRUPO 3","1137":"GRUPO 3","1138":"GRUPO 3","1139":"GRUPO 3","1140":"GRUPO 4","1141":"GRUPO 4","1142":"GRUPO 4","1143":"GRUPO 4","1144":"GRUPO 4","1145":"GRUPO 4","1146":"GRUPO 4","1147":"GRUPO 4","1148":"GRUPO 4","1149":"GRUPO 4","1150":"GRUPO 4","1151":"GRUPO 4","1152":"GRUPO 1","1153":"GRUPO 1","1154":"GRUPO 1","1155":"GRUPO 1","1156":"GRUPO 1","1157":"GRUPO 1","1158":"GRUPO 1","1159":"GRUPO 1","1160":"GRUPO 1","1161":"GRUPO 1","1162":"GRUPO 1","1163":"GRUPO 1","1164":"GRUPO 2","1165":"GRUPO 2","1166":"GRUPO 2","1167":"GRUPO 2","1168":"GRUPO 2","1169":"GRUPO 2","1170":"GRUPO 2","1171":"GRUPO 2","1172":"GRUPO 2","1173":"GRUPO 2","1174":"GRUPO 2","1175":"GRUPO 2","1176":"GRUPO 3","1177":"GRUPO 3","1178":"GRUPO 3","1179":"GRUPO 3","1180":"GRUPO 3","1181":"GRUPO 3","1182":"GRUPO 3","1183":"GRUPO 3","1184":"GRUPO 3","1185":"GRUPO 3","1186":"GRUPO 3","1187":"GRUPO 3","1188":"GRUPO 4","1189":"GRUPO 4","1190":"GRUPO 4","1191":"GRUPO 4","1192":"GRUPO 4","1193":"GRUPO 4","1194":"GRUPO 4","1195":"GRUPO 4","1196":"GRUPO 4","1197":"GRUPO 4","1198":"GRUPO 4","1199":"GRUPO 4","1200":"GRUPO 1","1201":"GRUPO 1","1202":"GRUPO 1","1203":"GRUPO 1","1204":"GRUPO 1","1205":"GRUPO 1","1206":"GRUPO 1","1207":"GRUPO 1","1208":"GRUPO 1","1209":"GRUPO 1","1210":"GRUPO 1","1211":"GRUPO 1","1212":"GRUPO 2","1213":"GRUPO 2","1214":"GRUPO 2","1215":"GRUPO 2","1216":"GRUPO 2","1217":"GRUPO 2","1218":"GRUPO 2","1219":"GRUPO 2","1220":"GRUPO 2","1221":"GRUPO 2","1222":"GRUPO 2","1223":"GRUPO 2","1224":"GRUPO 3","1225":"GRUPO 3","1226":"GRUPO 3","1227":"GRUPO 3","1228":"GRUPO 3","1229":"GRUPO 3","1230":"GRUPO 3","1231":"GRUPO 3","1232":"GRUPO 3","1233":"GRUPO 3","1234":"GRUPO 3","1235":"GRUPO 3","1236":"GRUPO 4","1237":"GRUPO 4","1238":"GRUPO 4","1239":"GRUPO 4","1240":"GRUPO 4","1241":"GRUPO 4","1242":"GRUPO 4","1243":"GRUPO 4","1244":"GRUPO 4","1245":"GRUPO 4","1246":"GRUPO 4","1247":"GRUPO 4","1248":"GRUPO 1","1249":"GRUPO 1","1250":"GRUPO 1","1251":"GRUPO 1","1252":"GRUPO 1","1253":"GRUPO 1","1254":"GRUPO 1","1255":"GRUPO 1","1256":"GRUPO 1","1257":"GRUPO 1","1258":"GRUPO 1","1259":"GRUPO 1","1260":"GRUPO 2","1261":"GRUPO 2","1262":"GRUPO 2","1263":"GRUPO 2","1264":"GRUPO 2","1265":"GRUPO 2","1266":"GRUPO 2","1267":"GRUPO 2","1268":"GRUPO 2","1269":"GRUPO 2","1270":"GRUPO 2","1271":"GRUPO 2","1272":"GRUPO 3","1273":"GRUPO 3","1274":"GRUPO 3","1275":"GRUPO 3","1276":"GRUPO 3","1277":"GRUPO 3","1278":"GRUPO 3","1279":"GRUPO 3","1280":"GRUPO 3","1281":"GRUPO 3","1282":"GRUPO 3","1283":"GRUPO 3","1284":"GRUPO 4","1285":"GRUPO 4","1286":"GRUPO 4","1287":"GRUPO 4","1288":"GRUPO 4","1289":"GRUPO 4","1290":"GRUPO 4","1291":"GRUPO 4","1292":"GRUPO 4","1293":"GRUPO 4","1294":"GRUPO 4","1295":"GRUPO 4","1296":"GRUPO 1","1297":"GRUPO 1","1298":"GRUPO 1","1299":"GRUPO 1","1300":"GRUPO 1","1301":"GRUPO 1","1302":"GRUPO 1","1303":"GRUPO 1","1304":"GRUPO 1","1305":"GRUPO 1","1306":"GRUPO 1","1307":"GRUPO 1","1308":"GRUPO 2","1309":"GRUPO 2","1310":"GRUPO 2","1311":"GRUPO 2","1312":"GRUPO 2","1313":"GRUPO 2","1314":"GRUPO 2","1315":"GRUPO 2","1316":"GRUPO 2","1317":"GRUPO 2","1318":"GRUPO 2","1319":"GRUPO 2","1320":"GRUPO 3","1321":"GRUPO 3","1322":"GRUPO 3","1323":"GRUPO 3","1324":"GRUPO 3","1325":"GRUPO 3","1326":"GRUPO 3","1327":"GRUPO 3","1328":"GRUPO 3","1329":"GRUPO 3","1330":"GRUPO 3","1331":"GRUPO 3","1332":"GRUPO 4","1333":"GRUPO 4","1334":"GRUPO 4","1335":"GRUPO 4","1336":"GRUPO 4","1337":"GRUPO 4","1338":"GRUPO 4","1339":"GRUPO 4","1340":"GRUPO 4","1341":"GRUPO 4","1342":"GRUPO 4","1343":"GRUPO 4","1344":"GRUPO 1","1345":"GRUPO 1","1346":"GRUPO 1","1347":"GRUPO 1","1348":"GRUPO 1","1349":"GRUPO 1","1350":"GRUPO 1","1351":"GRUPO 1","1352":"GRUPO 1","1353":"GRUPO 1","1354":"GRUPO 1","1355":"GRUPO 1","1356":"GRUPO 2","1357":"GRUPO 2","1358":"GRUPO 2","1359":"GRUPO 2","1360":"GRUPO 2","1361":"GRUPO 2","1362":"GRUPO 2","1363":"GRUPO 2","1364":"GRUPO 2","1365":"GRUPO 2","1366":"GRUPO 2","1367":"GRUPO 2","1368":"GRUPO 3","1369":"GRUPO 3","1370":"GRUPO 3","1371":"GRUPO 3","1372":"GRUPO 3","1373":"GRUPO 3","1374":"GRUPO 3","1375":"GRUPO 3","1376":"GRUPO 3","1377":"GRUPO 3","1378":"GRUPO 3","1379":"GRUPO 3","1380":"GRUPO 4","1381":"GRUPO 4","1382":"GRUPO 4","1383":"GRUPO 4","1384":"GRUPO 4","1385":"GRUPO 4","1386":"GRUPO 4","1387":"GRUPO 4","1388":"GRUPO 4","1389":"GRUPO 4","1390":"GRUPO 4","1391":"GRUPO 4","1392":"GRUPO 1","1393":"GRUPO 1","1394":"GRUPO 1","1395":"GRUPO 1","1396":"GRUPO 1","1397":"GRUPO 1","1398":"GRUPO 1","1399":"GRUPO 1","1400":"GRUPO 1","1401":"GRUPO 1","1402":"GRUPO 1","1403":"GRUPO 1","1404":"GRUPO 2","1405":"GRUPO 2","1406":"GRUPO 2","1407":"GRUPO 2","1408":"GRUPO 2","1409":"GRUPO 2","1410":"GRUPO 2","1411":"GRUPO 2","1412":"GRUPO 2","1413":"GRUPO 2","1414":"GRUPO 2","1415":"GRUPO 2","1416":"GRUPO 3","1417":"GRUPO 3","1418":"GRUPO 3","1419":"GRUPO 3","1420":"GRUPO 3","1421":"GRUPO 3","1422":"GRUPO 3","1423":"GRUPO 3","1424":"GRUPO 3","1425":"GRUPO 3","1426":"GRUPO 3","1427":"GRUPO 3","1428":"GRUPO 4","1429":"GRUPO 4","1430":"GRUPO 4","1431":"GRUPO 4","1432":"GRUPO 4","1433":"GRUPO 4","1434":"GRUPO 4","1435":"GRUPO 4","1436":"GRUPO 4","1437":"GRUPO 4","1438":"GRUPO 4","1439":"GRUPO 4"},"Empleado":{"0":"BARON HERNANDEZ HAROLD ANTONIO","1":"CASTELLANOS CARVAJAL DEYVITH FABIAN","2":"AROCA TORRES JULIAN EDUARDO","3":"BERMUDEZ PARRA JENNIFER XIOMARA","4":"BERNAL BAQUERO JAMES RICARDO","5":"BURGOS ORTIZ JOSE HORACIO","6":"CANTOR PORRAS JUAN FERNEY","7":"CAPERA CAPERA JOSE GABRIEL","8":"CARDENAS LOTERO RICARDO ANDR\u00c9S","9":"RENDON OSPINA NELSON LEANDRO","10":"SARMIENTO URBINA MOISES DANIEL","11":"VELASCO VELASCO SEBASTI\u00c1N DAVID","12":"DELGADO DELGADO JOHAN DARIO","13":"FLOREZ SAUCESO KENIS ALBERTO","14":"CARDONA GARCIA OSCAR JAVIER","15":"CARVAJAL GARC\u00cdA HOVER MARCK","16":"CEPEDA PIRAQUIVE JUAN DAVID","17":"FAJARDO SAENZ OSCAR FERNANDO","18":"FLOREZ ESPITIA RONY ALBERTO","19":"GARCIA CUERVO EDWIN JAVIER","20":"GONZALEZ OCHOA JUAN CARLOS","21":"XXX1","22":"XXX2","23":"XXX3","24":"FONSECA RAY RICARDO","25":"GOMEZ BETANCUR JAIDER ANDRES","26":"GRANADA PATI\u00d1O CARLOS MARINO","27":"GRASS PLATA MIGUEL SNEIDER","28":"MANZANO CALVO JUAN SEBASTIAN","29":"MENDOZA GOITA MARIANSEL ZENAYDA","30":"MURILLO ARAQUE JAIVER GEOVANY","31":"NI\u00d1O ARENAS HECTOR GONZALO","32":"RAMIREZ CHAVERRA JHON EDISON","33":"XXX4","34":"XXX5","35":"XXX6","36":"RODRIGUEZ MOSQUERA LUIS FERNANDO","37":"PEPITO PEREZ","38":"RAMIREZ VARGAS MARCELA PAOLA","39":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","40":"TORO CISNEROS GARY JOSE","41":"USECHE CALDERON JADID ESTIVEN","42":"VASQUEZ NIETO CAMILO ANDRES","43":"JHONY CASTRO","44":"BERNAL JUAN DAVID","45":"XXX7","46":"XXX8","47":"XXX9","48":"BARON HERNANDEZ HAROLD ANTONIO","49":"CASTELLANOS CARVAJAL DEYVITH FABIAN","50":"AROCA TORRES JULIAN EDUARDO","51":"BERMUDEZ PARRA JENNIFER XIOMARA","52":"BERNAL BAQUERO JAMES RICARDO","53":"BURGOS ORTIZ JOSE HORACIO","54":"CANTOR PORRAS JUAN FERNEY","55":"CAPERA CAPERA JOSE GABRIEL","56":"CARDENAS LOTERO RICARDO ANDR\u00c9S","57":"RENDON OSPINA NELSON LEANDRO","58":"SARMIENTO URBINA MOISES DANIEL","59":"VELASCO VELASCO SEBASTI\u00c1N DAVID","60":"DELGADO DELGADO JOHAN DARIO","61":"FLOREZ SAUCESO KENIS ALBERTO","62":"CARDONA GARCIA OSCAR JAVIER","63":"CARVAJAL GARC\u00cdA HOVER MARCK","64":"CEPEDA PIRAQUIVE JUAN DAVID","65":"FAJARDO SAENZ OSCAR FERNANDO","66":"FLOREZ ESPITIA RONY ALBERTO","67":"GARCIA CUERVO EDWIN JAVIER","68":"GONZALEZ OCHOA JUAN CARLOS","69":"XXX1","70":"XXX2","71":"XXX3","72":"FONSECA RAY RICARDO","73":"GOMEZ BETANCUR JAIDER ANDRES","74":"GRANADA PATI\u00d1O CARLOS MARINO","75":"GRASS PLATA MIGUEL SNEIDER","76":"MANZANO CALVO JUAN SEBASTIAN","77":"MENDOZA GOITA MARIANSEL ZENAYDA","78":"MURILLO ARAQUE JAIVER GEOVANY","79":"NI\u00d1O ARENAS HECTOR GONZALO","80":"RAMIREZ CHAVERRA JHON EDISON","81":"XXX4","82":"XXX5","83":"XXX6","84":"RODRIGUEZ MOSQUERA LUIS FERNANDO","85":"PEPITO PEREZ","86":"RAMIREZ VARGAS MARCELA PAOLA","87":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","88":"TORO CISNEROS GARY JOSE","89":"USECHE CALDERON JADID ESTIVEN","90":"VASQUEZ NIETO CAMILO ANDRES","91":"JHONY CASTRO","92":"BERNAL JUAN DAVID","93":"XXX7","94":"XXX8","95":"XXX9","96":"BARON HERNANDEZ HAROLD ANTONIO","97":"CASTELLANOS CARVAJAL DEYVITH FABIAN","98":"AROCA TORRES JULIAN EDUARDO","99":"BERMUDEZ PARRA JENNIFER XIOMARA","100":"BERNAL BAQUERO JAMES RICARDO","101":"BURGOS ORTIZ JOSE HORACIO","102":"CANTOR PORRAS JUAN FERNEY","103":"CAPERA CAPERA JOSE GABRIEL","104":"CARDENAS LOTERO RICARDO ANDR\u00c9S","105":"RENDON OSPINA NELSON LEANDRO","106":"SARMIENTO URBINA MOISES DANIEL","107":"VELASCO VELASCO SEBASTI\u00c1N DAVID","108":"DELGADO DELGADO JOHAN DARIO","109":"FLOREZ SAUCESO KENIS ALBERTO","110":"CARDONA GARCIA OSCAR JAVIER","111":"CARVAJAL GARC\u00cdA HOVER MARCK","112":"CEPEDA PIRAQUIVE JUAN DAVID","113":"FAJARDO SAENZ OSCAR FERNANDO","114":"FLOREZ ESPITIA RONY ALBERTO","115":"GARCIA CUERVO EDWIN JAVIER","116":"GONZALEZ OCHOA JUAN CARLOS","117":"XXX1","118":"XXX2","119":"XXX3","120":"FONSECA RAY RICARDO","121":"GOMEZ BETANCUR JAIDER ANDRES","122":"GRANADA PATI\u00d1O CARLOS MARINO","123":"GRASS PLATA MIGUEL SNEIDER","124":"MANZANO CALVO JUAN SEBASTIAN","125":"MENDOZA GOITA MARIANSEL ZENAYDA","126":"MURILLO ARAQUE JAIVER GEOVANY","127":"NI\u00d1O ARENAS HECTOR GONZALO","128":"RAMIREZ CHAVERRA JHON EDISON","129":"XXX4","130":"XXX5","131":"XXX6","132":"RODRIGUEZ MOSQUERA LUIS FERNANDO","133":"PEPITO PEREZ","134":"RAMIREZ VARGAS MARCELA PAOLA","135":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","136":"TORO CISNEROS GARY JOSE","137":"USECHE CALDERON JADID ESTIVEN","138":"VASQUEZ NIETO CAMILO ANDRES","139":"JHONY CASTRO","140":"BERNAL JUAN DAVID","141":"XXX7","142":"XXX8","143":"XXX9","144":"BARON HERNANDEZ HAROLD ANTONIO","145":"CASTELLANOS CARVAJAL DEYVITH FABIAN","146":"AROCA TORRES JULIAN EDUARDO","147":"BERMUDEZ PARRA JENNIFER XIOMARA","148":"BERNAL BAQUERO JAMES RICARDO","149":"BURGOS ORTIZ JOSE HORACIO","150":"CANTOR PORRAS JUAN FERNEY","151":"CAPERA CAPERA JOSE GABRIEL","152":"CARDENAS LOTERO RICARDO ANDR\u00c9S","153":"RENDON OSPINA NELSON LEANDRO","154":"SARMIENTO URBINA MOISES DANIEL","155":"VELASCO VELASCO SEBASTI\u00c1N DAVID","156":"DELGADO DELGADO JOHAN DARIO","157":"FLOREZ SAUCESO KENIS ALBERTO","158":"CARDONA GARCIA OSCAR JAVIER","159":"CARVAJAL GARC\u00cdA HOVER MARCK","160":"CEPEDA PIRAQUIVE JUAN DAVID","161":"FAJARDO SAENZ OSCAR FERNANDO","162":"FLOREZ ESPITIA RONY ALBERTO","163":"GARCIA CUERVO EDWIN JAVIER","164":"GONZALEZ OCHOA JUAN CARLOS","165":"XXX1","166":"XXX2","167":"XXX3","168":"FONSECA RAY RICARDO","169":"GOMEZ BETANCUR JAIDER ANDRES","170":"GRANADA PATI\u00d1O CARLOS MARINO","171":"GRASS PLATA MIGUEL SNEIDER","172":"MANZANO CALVO JUAN SEBASTIAN","173":"MENDOZA GOITA MARIANSEL ZENAYDA","174":"MURILLO ARAQUE JAIVER GEOVANY","175":"NI\u00d1O ARENAS HECTOR GONZALO","176":"RAMIREZ CHAVERRA JHON EDISON","177":"XXX4","178":"XXX5","179":"XXX6","180":"RODRIGUEZ MOSQUERA LUIS FERNANDO","181":"PEPITO PEREZ","182":"RAMIREZ VARGAS MARCELA PAOLA","183":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","184":"TORO CISNEROS GARY JOSE","185":"USECHE CALDERON JADID ESTIVEN","186":"VASQUEZ NIETO CAMILO ANDRES","187":"JHONY CASTRO","188":"BERNAL JUAN DAVID","189":"XXX7","190":"XXX8","191":"XXX9","192":"BARON HERNANDEZ HAROLD ANTONIO","193":"CASTELLANOS CARVAJAL DEYVITH FABIAN","194":"AROCA TORRES JULIAN EDUARDO","195":"BERMUDEZ PARRA JENNIFER XIOMARA","196":"BERNAL BAQUERO JAMES RICARDO","197":"BURGOS ORTIZ JOSE HORACIO","198":"CANTOR PORRAS JUAN FERNEY","199":"CAPERA CAPERA JOSE GABRIEL","200":"CARDENAS LOTERO RICARDO ANDR\u00c9S","201":"RENDON OSPINA NELSON LEANDRO","202":"SARMIENTO URBINA MOISES DANIEL","203":"VELASCO VELASCO SEBASTI\u00c1N DAVID","204":"DELGADO DELGADO JOHAN DARIO","205":"FLOREZ SAUCESO KENIS ALBERTO","206":"CARDONA GARCIA OSCAR JAVIER","207":"CARVAJAL GARC\u00cdA HOVER MARCK","208":"CEPEDA PIRAQUIVE JUAN DAVID","209":"FAJARDO SAENZ OSCAR FERNANDO","210":"FLOREZ ESPITIA RONY ALBERTO","211":"GARCIA CUERVO EDWIN JAVIER","212":"GONZALEZ OCHOA JUAN CARLOS","213":"XXX1","214":"XXX2","215":"XXX3","216":"FONSECA RAY RICARDO","217":"GOMEZ BETANCUR JAIDER ANDRES","218":"GRANADA PATI\u00d1O CARLOS MARINO","219":"GRASS PLATA MIGUEL SNEIDER","220":"MANZANO CALVO JUAN SEBASTIAN","221":"MENDOZA GOITA MARIANSEL ZENAYDA","222":"MURILLO ARAQUE JAIVER GEOVANY","223":"NI\u00d1O ARENAS HECTOR GONZALO","224":"RAMIREZ CHAVERRA JHON EDISON","225":"XXX4","226":"XXX5","227":"XXX6","228":"RODRIGUEZ MOSQUERA LUIS FERNANDO","229":"PEPITO PEREZ","230":"RAMIREZ VARGAS MARCELA PAOLA","231":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","232":"TORO CISNEROS GARY JOSE","233":"USECHE CALDERON JADID ESTIVEN","234":"VASQUEZ NIETO CAMILO ANDRES","235":"JHONY CASTRO","236":"BERNAL JUAN DAVID","237":"XXX7","238":"XXX8","239":"XXX9","240":"BARON HERNANDEZ HAROLD ANTONIO","241":"CASTELLANOS CARVAJAL DEYVITH FABIAN","242":"AROCA TORRES JULIAN EDUARDO","243":"BERMUDEZ PARRA JENNIFER XIOMARA","244":"BERNAL BAQUERO JAMES RICARDO","245":"BURGOS ORTIZ JOSE HORACIO","246":"CANTOR PORRAS JUAN FERNEY","247":"CAPERA CAPERA JOSE GABRIEL","248":"CARDENAS LOTERO RICARDO ANDR\u00c9S","249":"RENDON OSPINA NELSON LEANDRO","250":"SARMIENTO URBINA MOISES DANIEL","251":"VELASCO VELASCO SEBASTI\u00c1N DAVID","252":"DELGADO DELGADO JOHAN DARIO","253":"FLOREZ SAUCESO KENIS ALBERTO","254":"CARDONA GARCIA OSCAR JAVIER","255":"CARVAJAL GARC\u00cdA HOVER MARCK","256":"CEPEDA PIRAQUIVE JUAN DAVID","257":"FAJARDO SAENZ OSCAR FERNANDO","258":"FLOREZ ESPITIA RONY ALBERTO","259":"GARCIA CUERVO EDWIN JAVIER","260":"GONZALEZ OCHOA JUAN CARLOS","261":"XXX1","262":"XXX2","263":"XXX3","264":"FONSECA RAY RICARDO","265":"GOMEZ BETANCUR JAIDER ANDRES","266":"GRANADA PATI\u00d1O CARLOS MARINO","267":"GRASS PLATA MIGUEL SNEIDER","268":"MANZANO CALVO JUAN SEBASTIAN","269":"MENDOZA GOITA MARIANSEL ZENAYDA","270":"MURILLO ARAQUE JAIVER GEOVANY","271":"NI\u00d1O ARENAS HECTOR GONZALO","272":"RAMIREZ CHAVERRA JHON EDISON","273":"XXX4","274":"XXX5","275":"XXX6","276":"RODRIGUEZ MOSQUERA LUIS FERNANDO","277":"PEPITO PEREZ","278":"RAMIREZ VARGAS MARCELA PAOLA","279":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","280":"TORO CISNEROS GARY JOSE","281":"USECHE CALDERON JADID ESTIVEN","282":"VASQUEZ NIETO CAMILO ANDRES","283":"JHONY CASTRO","284":"BERNAL JUAN DAVID","285":"XXX7","286":"XXX8","287":"XXX9","288":"BARON HERNANDEZ HAROLD ANTONIO","289":"CASTELLANOS CARVAJAL DEYVITH FABIAN","290":"AROCA TORRES JULIAN EDUARDO","291":"BERMUDEZ PARRA JENNIFER XIOMARA","292":"BERNAL BAQUERO JAMES RICARDO","293":"BURGOS ORTIZ JOSE</t>
+  </si>
+  <si>
+    <t>[{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"01-Mie","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"01-Mie","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"01-Mie","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"01-Mie","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"01-Mie","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"01-Mie","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"01-Mie","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"01-Mie","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"01-Mie","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"01-Mie","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"01-Mie","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"01-Mie","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"06-Lun","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"06-Lun","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"06-Lun","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"06-Lun","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"06-Lun","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"06-Lun","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"06-Lun","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"06-Lun","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"06-Lun","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"06-Lun","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"06-Lun","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"06-Lun","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VA</t>
   </si>
 </sst>
 </file>
@@ -455,7 +458,7 @@
         <v>11</v>
       </c>
       <c r="E4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update historico_mallas.xlsx 2026-04-24 18:26:56.253790
</commit_message>
<xml_diff>
--- a/historico_mallas.xlsx
+++ b/historico_mallas.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="17">
   <si>
     <t>Mes</t>
   </si>
@@ -40,6 +40,9 @@
     <t>Junio</t>
   </si>
   <si>
+    <t>Julio</t>
+  </si>
+  <si>
     <t>Técnica</t>
   </si>
   <si>
@@ -50,6 +53,9 @@
   </si>
   <si>
     <t>2026-04-24 18:24</t>
+  </si>
+  <si>
+    <t>2026-04-24 18:26</t>
   </si>
   <si>
     <t>{"Grupo":{"0":"GRUPO 1","1":"GRUPO 1","2":"GRUPO 1","3":"GRUPO 1","4":"GRUPO 1","5":"GRUPO 1","6":"GRUPO 1","7":"GRUPO 1","8":"GRUPO 1","9":"GRUPO 1","10":"GRUPO 1","11":"GRUPO 1","12":"GRUPO 2","13":"GRUPO 2","14":"GRUPO 2","15":"GRUPO 2","16":"GRUPO 2","17":"GRUPO 2","18":"GRUPO 2","19":"GRUPO 2","20":"GRUPO 2","21":"GRUPO 2","22":"GRUPO 2","23":"GRUPO 2","24":"GRUPO 3","25":"GRUPO 3","26":"GRUPO 3","27":"GRUPO 3","28":"GRUPO 3","29":"GRUPO 3","30":"GRUPO 3","31":"GRUPO 3","32":"GRUPO 3","33":"GRUPO 3","34":"GRUPO 3","35":"GRUPO 3","36":"GRUPO 4","37":"GRUPO 4","38":"GRUPO 4","39":"GRUPO 4","40":"GRUPO 4","41":"GRUPO 4","42":"GRUPO 4","43":"GRUPO 4","44":"GRUPO 4","45":"GRUPO 4","46":"GRUPO 4","47":"GRUPO 4","48":"GRUPO 1","49":"GRUPO 1","50":"GRUPO 1","51":"GRUPO 1","52":"GRUPO 1","53":"GRUPO 1","54":"GRUPO 1","55":"GRUPO 1","56":"GRUPO 1","57":"GRUPO 1","58":"GRUPO 1","59":"GRUPO 1","60":"GRUPO 2","61":"GRUPO 2","62":"GRUPO 2","63":"GRUPO 2","64":"GRUPO 2","65":"GRUPO 2","66":"GRUPO 2","67":"GRUPO 2","68":"GRUPO 2","69":"GRUPO 2","70":"GRUPO 2","71":"GRUPO 2","72":"GRUPO 3","73":"GRUPO 3","74":"GRUPO 3","75":"GRUPO 3","76":"GRUPO 3","77":"GRUPO 3","78":"GRUPO 3","79":"GRUPO 3","80":"GRUPO 3","81":"GRUPO 3","82":"GRUPO 3","83":"GRUPO 3","84":"GRUPO 4","85":"GRUPO 4","86":"GRUPO 4","87":"GRUPO 4","88":"GRUPO 4","89":"GRUPO 4","90":"GRUPO 4","91":"GRUPO 4","92":"GRUPO 4","93":"GRUPO 4","94":"GRUPO 4","95":"GRUPO 4","96":"GRUPO 1","97":"GRUPO 1","98":"GRUPO 1","99":"GRUPO 1","100":"GRUPO 1","101":"GRUPO 1","102":"GRUPO 1","103":"GRUPO 1","104":"GRUPO 1","105":"GRUPO 1","106":"GRUPO 1","107":"GRUPO 1","108":"GRUPO 2","109":"GRUPO 2","110":"GRUPO 2","111":"GRUPO 2","112":"GRUPO 2","113":"GRUPO 2","114":"GRUPO 2","115":"GRUPO 2","116":"GRUPO 2","117":"GRUPO 2","118":"GRUPO 2","119":"GRUPO 2","120":"GRUPO 3","121":"GRUPO 3","122":"GRUPO 3","123":"GRUPO 3","124":"GRUPO 3","125":"GRUPO 3","126":"GRUPO 3","127":"GRUPO 3","128":"GRUPO 3","129":"GRUPO 3","130":"GRUPO 3","131":"GRUPO 3","132":"GRUPO 4","133":"GRUPO 4","134":"GRUPO 4","135":"GRUPO 4","136":"GRUPO 4","137":"GRUPO 4","138":"GRUPO 4","139":"GRUPO 4","140":"GRUPO 4","141":"GRUPO 4","142":"GRUPO 4","143":"GRUPO 4","144":"GRUPO 1","145":"GRUPO 1","146":"GRUPO 1","147":"GRUPO 1","148":"GRUPO 1","149":"GRUPO 1","150":"GRUPO 1","151":"GRUPO 1","152":"GRUPO 1","153":"GRUPO 1","154":"GRUPO 1","155":"GRUPO 1","156":"GRUPO 2","157":"GRUPO 2","158":"GRUPO 2","159":"GRUPO 2","160":"GRUPO 2","161":"GRUPO 2","162":"GRUPO 2","163":"GRUPO 2","164":"GRUPO 2","165":"GRUPO 2","166":"GRUPO 2","167":"GRUPO 2","168":"GRUPO 3","169":"GRUPO 3","170":"GRUPO 3","171":"GRUPO 3","172":"GRUPO 3","173":"GRUPO 3","174":"GRUPO 3","175":"GRUPO 3","176":"GRUPO 3","177":"GRUPO 3","178":"GRUPO 3","179":"GRUPO 3","180":"GRUPO 4","181":"GRUPO 4","182":"GRUPO 4","183":"GRUPO 4","184":"GRUPO 4","185":"GRUPO 4","186":"GRUPO 4","187":"GRUPO 4","188":"GRUPO 4","189":"GRUPO 4","190":"GRUPO 4","191":"GRUPO 4","192":"GRUPO 1","193":"GRUPO 1","194":"GRUPO 1","195":"GRUPO 1","196":"GRUPO 1","197":"GRUPO 1","198":"GRUPO 1","199":"GRUPO 1","200":"GRUPO 1","201":"GRUPO 1","202":"GRUPO 1","203":"GRUPO 1","204":"GRUPO 2","205":"GRUPO 2","206":"GRUPO 2","207":"GRUPO 2","208":"GRUPO 2","209":"GRUPO 2","210":"GRUPO 2","211":"GRUPO 2","212":"GRUPO 2","213":"GRUPO 2","214":"GRUPO 2","215":"GRUPO 2","216":"GRUPO 3","217":"GRUPO 3","218":"GRUPO 3","219":"GRUPO 3","220":"GRUPO 3","221":"GRUPO 3","222":"GRUPO 3","223":"GRUPO 3","224":"GRUPO 3","225":"GRUPO 3","226":"GRUPO 3","227":"GRUPO 3","228":"GRUPO 4","229":"GRUPO 4","230":"GRUPO 4","231":"GRUPO 4","232":"GRUPO 4","233":"GRUPO 4","234":"GRUPO 4","235":"GRUPO 4","236":"GRUPO 4","237":"GRUPO 4","238":"GRUPO 4","239":"GRUPO 4","240":"GRUPO 1","241":"GRUPO 1","242":"GRUPO 1","243":"GRUPO 1","244":"GRUPO 1","245":"GRUPO 1","246":"GRUPO 1","247":"GRUPO 1","248":"GRUPO 1","249":"GRUPO 1","250":"GRUPO 1","251":"GRUPO 1","252":"GRUPO 2","253":"GRUPO 2","254":"GRUPO 2","255":"GRUPO 2","256":"GRUPO 2","257":"GRUPO 2","258":"GRUPO 2","259":"GRUPO 2","260":"GRUPO 2","261":"GRUPO 2","262":"GRUPO 2","263":"GRUPO 2","264":"GRUPO 3","265":"GRUPO 3","266":"GRUPO 3","267":"GRUPO 3","268":"GRUPO 3","269":"GRUPO 3","270":"GRUPO 3","271":"GRUPO 3","272":"GRUPO 3","273":"GRUPO 3","274":"GRUPO 3","275":"GRUPO 3","276":"GRUPO 4","277":"GRUPO 4","278":"GRUPO 4","279":"GRUPO 4","280":"GRUPO 4","281":"GRUPO 4","282":"GRUPO 4","283":"GRUPO 4","284":"GRUPO 4","285":"GRUPO 4","286":"GRUPO 4","287":"GRUPO 4","288":"GRUPO 1","289":"GRUPO 1","290":"GRUPO 1","291":"GRUPO 1","292":"GRUPO 1","293":"GRUPO 1","294":"GRUPO 1","295":"GRUPO 1","296":"GRUPO 1","297":"GRUPO 1","298":"GRUPO 1","299":"GRUPO 1","300":"GRUPO 2","301":"GRUPO 2","302":"GRUPO 2","303":"GRUPO 2","304":"GRUPO 2","305":"GRUPO 2","306":"GRUPO 2","307":"GRUPO 2","308":"GRUPO 2","309":"GRUPO 2","310":"GRUPO 2","311":"GRUPO 2","312":"GRUPO 3","313":"GRUPO 3","314":"GRUPO 3","315":"GRUPO 3","316":"GRUPO 3","317":"GRUPO 3","318":"GRUPO 3","319":"GRUPO 3","320":"GRUPO 3","321":"GRUPO 3","322":"GRUPO 3","323":"GRUPO 3","324":"GRUPO 4","325":"GRUPO 4","326":"GRUPO 4","327":"GRUPO 4","328":"GRUPO 4","329":"GRUPO 4","330":"GRUPO 4","331":"GRUPO 4","332":"GRUPO 4","333":"GRUPO 4","334":"GRUPO 4","335":"GRUPO 4","336":"GRUPO 1","337":"GRUPO 1","338":"GRUPO 1","339":"GRUPO 1","340":"GRUPO 1","341":"GRUPO 1","342":"GRUPO 1","343":"GRUPO 1","344":"GRUPO 1","345":"GRUPO 1","346":"GRUPO 1","347":"GRUPO 1","348":"GRUPO 2","349":"GRUPO 2","350":"GRUPO 2","351":"GRUPO 2","352":"GRUPO 2","353":"GRUPO 2","354":"GRUPO 2","355":"GRUPO 2","356":"GRUPO 2","357":"GRUPO 2","358":"GRUPO 2","359":"GRUPO 2","360":"GRUPO 3","361":"GRUPO 3","362":"GRUPO 3","363":"GRUPO 3","364":"GRUPO 3","365":"GRUPO 3","366":"GRUPO 3","367":"GRUPO 3","368":"GRUPO 3","369":"GRUPO 3","370":"GRUPO 3","371":"GRUPO 3","372":"GRUPO 4","373":"GRUPO 4","374":"GRUPO 4","375":"GRUPO 4","376":"GRUPO 4","377":"GRUPO 4","378":"GRUPO 4","379":"GRUPO 4","380":"GRUPO 4","381":"GRUPO 4","382":"GRUPO 4","383":"GRUPO 4","384":"GRUPO 1","385":"GRUPO 1","386":"GRUPO 1","387":"GRUPO 1","388":"GRUPO 1","389":"GRUPO 1","390":"GRUPO 1","391":"GRUPO 1","392":"GRUPO 1","393":"GRUPO 1","394":"GRUPO 1","395":"GRUPO 1","396":"GRUPO 2","397":"GRUPO 2","398":"GRUPO 2","399":"GRUPO 2","400":"GRUPO 2","401":"GRUPO 2","402":"GRUPO 2","403":"GRUPO 2","404":"GRUPO 2","405":"GRUPO 2","406":"GRUPO 2","407":"GRUPO 2","408":"GRUPO 3","409":"GRUPO 3","410":"GRUPO 3","411":"GRUPO 3","412":"GRUPO 3","413":"GRUPO 3","414":"GRUPO 3","415":"GRUPO 3","416":"GRUPO 3","417":"GRUPO 3","418":"GRUPO 3","419":"GRUPO 3","420":"GRUPO 4","421":"GRUPO 4","422":"GRUPO 4","423":"GRUPO 4","424":"GRUPO 4","425":"GRUPO 4","426":"GRUPO 4","427":"GRUPO 4","428":"GRUPO 4","429":"GRUPO 4","430":"GRUPO 4","431":"GRUPO 4","432":"GRUPO 1","433":"GRUPO 1","434":"GRUPO 1","435":"GRUPO 1","436":"GRUPO 1","437":"GRUPO 1","438":"GRUPO 1","439":"GRUPO 1","440":"GRUPO 1","441":"GRUPO 1","442":"GRUPO 1","443":"GRUPO 1","444":"GRUPO 2","445":"GRUPO 2","446":"GRUPO 2","447":"GRUPO 2","448":"GRUPO 2","449":"GRUPO 2","450":"GRUPO 2","451":"GRUPO 2","452":"GRUPO 2","453":"GRUPO 2","454":"GRUPO 2","455":"GRUPO 2","456":"GRUPO 3","457":"GRUPO 3","458":"GRUPO 3","459":"GRUPO 3","460":"GRUPO 3","461":"GRUPO 3","462":"GRUPO 3","463":"GRUPO 3","464":"GRUPO 3","465":"GRUPO 3","466":"GRUPO 3","467":"GRUPO 3","468":"GRUPO 4","469":"GRUPO 4","470":"GRUPO 4","471":"GRUPO 4","472":"GRUPO 4","473":"GRUPO 4","474":"GRUPO 4","475":"GRUPO 4","476":"GRUPO 4","477":"GRUPO 4","478":"GRUPO 4","479":"GRUPO 4","480":"GRUPO 1","481":"GRUPO 1","482":"GRUPO 1","483":"GRUPO 1","484":"GRUPO 1","485":"GRUPO 1","486":"GRUPO 1","487":"GRUPO 1","488":"GRUPO 1","489":"GRUPO 1","490":"GRUPO 1","491":"GRUPO 1","492":"GRUPO 2","493":"GRUPO 2","494":"GRUPO 2","495":"GRUPO 2","496":"GRUPO 2","497":"GRUPO 2","498":"GRUPO 2","499":"GRUPO 2","500":"GRUPO 2","501":"GRUPO 2","502":"GRUPO 2","503":"GRUPO 2","504":"GRUPO 3","505":"GRUPO 3","506":"GRUPO 3","507":"GRUPO 3","508":"GRUPO 3","509":"GRUPO 3","510":"GRUPO 3","511":"GRUPO 3","512":"GRUPO 3","513":"GRUPO 3","514":"GRUPO 3","515":"GRUPO 3","516":"GRUPO 4","517":"GRUPO 4","518":"GRUPO 4","519":"GRUPO 4","520":"GRUPO 4","521":"GRUPO 4","522":"GRUPO 4","523":"GRUPO 4","524":"GRUPO 4","525":"GRUPO 4","526":"GRUPO 4","527":"GRUPO 4","528":"GRUPO 1","529":"GRUPO 1","530":"GRUPO 1","531":"GRUPO 1","532":"GRUPO 1","533":"GRUPO 1","534":"GRUPO 1","535":"GRUPO 1","536":"GRUPO 1","537":"GRUPO 1","538":"GRUPO 1","539":"GRUPO 1","540":"GRUPO 2","541":"GRUPO 2","542":"GRUPO 2","543":"GRUPO 2","544":"GRUPO 2","545":"GRUPO 2","546":"GRUPO 2","547":"GRUPO 2","548":"GRUPO 2","549":"GRUPO 2","550":"GRUPO 2","551":"GRUPO 2","552":"GRUPO 3","553":"GRUPO 3","554":"GRUPO 3","555":"GRUPO 3","556":"GRUPO 3","557":"GRUPO 3","558":"GRUPO 3","559":"GRUPO 3","560":"GRUPO 3","561":"GRUPO 3","562":"GRUPO 3","563":"GRUPO 3","564":"GRUPO 4","565":"GRUPO 4","566":"GRUPO 4","567":"GRUPO 4","568":"GRUPO 4","569":"GRUPO 4","570":"GRUPO 4","571":"GRUPO 4","572":"GRUPO 4","573":"GRUPO 4","574":"GRUPO 4","575":"GRUPO 4","576":"GRUPO 1","577":"GRUPO 1","578":"GRUPO 1","579":"GRUPO 1","580":"GRUPO 1","581":"GRUPO 1","582":"GRUPO 1","583":"GRUPO 1","584":"GRUPO 1","585":"GRUPO 1","586":"GRUPO 1","587":"GRUPO 1","588":"GRUPO 2","589":"GRUPO 2","590":"GRUPO 2","591":"GRUPO 2","592":"GRUPO 2","593":"GRUPO 2","594":"GRUPO 2","595":"GRUPO 2","596":"GRUPO 2","597":"GRUPO 2","598":"GRUPO 2","599":"GRUPO 2","600":"GRUPO 3","601":"GRUPO 3","602":"GRUPO 3","603":"GRUPO 3","604":"GRUPO 3","605":"GRUPO 3","606":"GRUPO 3","607":"GRUPO 3","608":"GRUPO 3","609":"GRUPO 3","610":"GRUPO 3","611":"GRUPO 3","612":"GRUPO 4","613":"GRUPO 4","614":"GRUPO 4","615":"GRUPO 4","616":"GRUPO 4","617":"GRUPO 4","618":"GRUPO 4","619":"GRUPO 4","620":"GRUPO 4","621":"GRUPO 4","622":"GRUPO 4","623":"GRUPO 4","624":"GRUPO 1","625":"GRUPO 1","626":"GRUPO 1","627":"GRUPO 1","628":"GRUPO 1","629":"GRUPO 1","630":"GRUPO 1","631":"GRUPO 1","632":"GRUPO 1","633":"GRUPO 1","634":"GRUPO 1","635":"GRUPO 1","636":"GRUPO 2","637":"GRUPO 2","638":"GRUPO 2","639":"GRUPO 2","640":"GRUPO 2","641":"GRUPO 2","642":"GRUPO 2","643":"GRUPO 2","644":"GRUPO 2","645":"GRUPO 2","646":"GRUPO 2","647":"GRUPO 2","648":"GRUPO 3","649":"GRUPO 3","650":"GRUPO 3","651":"GRUPO 3","652":"GRUPO 3","653":"GRUPO 3","654":"GRUPO 3","655":"GRUPO 3","656":"GRUPO 3","657":"GRUPO 3","658":"GRUPO 3","659":"GRUPO 3","660":"GRUPO 4","661":"GRUPO 4","662":"GRUPO 4","663":"GRUPO 4","664":"GRUPO 4","665":"GRUPO 4","666":"GRUPO 4","667":"GRUPO 4","668":"GRUPO 4","669":"GRUPO 4","670":"GRUPO 4","671":"GRUPO 4","672":"GRUPO 1","673":"GRUPO 1","674":"GRUPO 1","675":"GRUPO 1","676":"GRUPO 1","677":"GRUPO 1","678":"GRUPO 1","679":"GRUPO 1","680":"GRUPO 1","681":"GRUPO 1","682":"GRUPO 1","683":"GRUPO 1","684":"GRUPO 2","685":"GRUPO 2","686":"GRUPO 2","687":"GRUPO 2","688":"GRUPO 2","689":"GRUPO 2","690":"GRUPO 2","691":"GRUPO 2","692":"GRUPO 2","693":"GRUPO 2","694":"GRUPO 2","695":"GRUPO 2","696":"GRUPO 3","697":"GRUPO 3","698":"GRUPO 3","699":"GRUPO 3","700":"GRUPO 3","701":"GRUPO 3","702":"GRUPO 3","703":"GRUPO 3","704":"GRUPO 3","705":"GRUPO 3","706":"GRUPO 3","707":"GRUPO 3","708":"GRUPO 4","709":"GRUPO 4","710":"GRUPO 4","711":"GRUPO 4","712":"GRUPO 4","713":"GRUPO 4","714":"GRUPO 4","715":"GRUPO 4","716":"GRUPO 4","717":"GRUPO 4","718":"GRUPO 4","719":"GRUPO 4","720":"GRUPO 1","721":"GRUPO 1","722":"GRUPO 1","723":"GRUPO 1","724":"GRUPO 1","725":"GRUPO 1","726":"GRUPO 1","727":"GRUPO 1","728":"GRUPO 1","729":"GRUPO 1","730":"GRUPO 1","731":"GRUPO 1","732":"GRUPO 2","733":"GRUPO 2","734":"GRUPO 2","735":"GRUPO 2","736":"GRUPO 2","737":"GRUPO 2","738":"GRUPO 2","739":"GRUPO 2","740":"GRUPO 2","741":"GRUPO 2","742":"GRUPO 2","743":"GRUPO 2","744":"GRUPO 3","745":"GRUPO 3","746":"GRUPO 3","747":"GRUPO 3","748":"GRUPO 3","749":"GRUPO 3","750":"GRUPO 3","751":"GRUPO 3","752":"GRUPO 3","753":"GRUPO 3","754":"GRUPO 3","755":"GRUPO 3","756":"GRUPO 4","757":"GRUPO 4","758":"GRUPO 4","759":"GRUPO 4","760":"GRUPO 4","761":"GRUPO 4","762":"GRUPO 4","763":"GRUPO 4","764":"GRUPO 4","765":"GRUPO 4","766":"GRUPO 4","767":"GRUPO 4","768":"GRUPO 1","769":"GRUPO 1","770":"GRUPO 1","771":"GRUPO 1","772":"GRUPO 1","773":"GRUPO 1","774":"GRUPO 1","775":"GRUPO 1","776":"GRUPO 1","777":"GRUPO 1","778":"GRUPO 1","779":"GRUPO 1","780":"GRUPO 2","781":"GRUPO 2","782":"GRUPO 2","783":"GRUPO 2","784":"GRUPO 2","785":"GRUPO 2","786":"GRUPO 2","787":"GRUPO 2","788":"GRUPO 2","789":"GRUPO 2","790":"GRUPO 2","791":"GRUPO 2","792":"GRUPO 3","793":"GRUPO 3","794":"GRUPO 3","795":"GRUPO 3","796":"GRUPO 3","797":"GRUPO 3","798":"GRUPO 3","799":"GRUPO 3","800":"GRUPO 3","801":"GRUPO 3","802":"GRUPO 3","803":"GRUPO 3","804":"GRUPO 4","805":"GRUPO 4","806":"GRUPO 4","807":"GRUPO 4","808":"GRUPO 4","809":"GRUPO 4","810":"GRUPO 4","811":"GRUPO 4","812":"GRUPO 4","813":"GRUPO 4","814":"GRUPO 4","815":"GRUPO 4","816":"GRUPO 1","817":"GRUPO 1","818":"GRUPO 1","819":"GRUPO 1","820":"GRUPO 1","821":"GRUPO 1","822":"GRUPO 1","823":"GRUPO 1","824":"GRUPO 1","825":"GRUPO 1","826":"GRUPO 1","827":"GRUPO 1","828":"GRUPO 2","829":"GRUPO 2","830":"GRUPO 2","831":"GRUPO 2","832":"GRUPO 2","833":"GRUPO 2","834":"GRUPO 2","835":"GRUPO 2","836":"GRUPO 2","837":"GRUPO 2","838":"GRUPO 2","839":"GRUPO 2","840":"GRUPO 3","841":"GRUPO 3","842":"GRUPO 3","843":"GRUPO 3","844":"GRUPO 3","845":"GRUPO 3","846":"GRUPO 3","847":"GRUPO 3","848":"GRUPO 3","849":"GRUPO 3","850":"GRUPO 3","851":"GRUPO 3","852":"GRUPO 4","853":"GRUPO 4","854":"GRUPO 4","855":"GRUPO 4","856":"GRUPO 4","857":"GRUPO 4","858":"GRUPO 4","859":"GRUPO 4","860":"GRUPO 4","861":"GRUPO 4","862":"GRUPO 4","863":"GRUPO 4","864":"GRUPO 1","865":"GRUPO 1","866":"GRUPO 1","867":"GRUPO 1","868":"GRUPO 1","869":"GRUPO 1","870":"GRUPO 1","871":"GRUPO 1","872":"GRUPO 1","873":"GRUPO 1","874":"GRUPO 1","875":"GRUPO 1","876":"GRUPO 2","877":"GRUPO 2","878":"GRUPO 2","879":"GRUPO 2","880":"GRUPO 2","881":"GRUPO 2","882":"GRUPO 2","883":"GRUPO 2","884":"GRUPO 2","885":"GRUPO 2","886":"GRUPO 2","887":"GRUPO 2","888":"GRUPO 3","889":"GRUPO 3","890":"GRUPO 3","891":"GRUPO 3","892":"GRUPO 3","893":"GRUPO 3","894":"GRUPO 3","895":"GRUPO 3","896":"GRUPO 3","897":"GRUPO 3","898":"GRUPO 3","899":"GRUPO 3","900":"GRUPO 4","901":"GRUPO 4","902":"GRUPO 4","903":"GRUPO 4","904":"GRUPO 4","905":"GRUPO 4","906":"GRUPO 4","907":"GRUPO 4","908":"GRUPO 4","909":"GRUPO 4","910":"GRUPO 4","911":"GRUPO 4","912":"GRUPO 1","913":"GRUPO 1","914":"GRUPO 1","915":"GRUPO 1","916":"GRUPO 1","917":"GRUPO 1","918":"GRUPO 1","919":"GRUPO 1","920":"GRUPO 1","921":"GRUPO 1","922":"GRUPO 1","923":"GRUPO 1","924":"GRUPO 2","925":"GRUPO 2","926":"GRUPO 2","927":"GRUPO 2","928":"GRUPO 2","929":"GRUPO 2","930":"GRUPO 2","931":"GRUPO 2","932":"GRUPO 2","933":"GRUPO 2","934":"GRUPO 2","935":"GRUPO 2","936":"GRUPO 3","937":"GRUPO 3","938":"GRUPO 3","939":"GRUPO 3","940":"GRUPO 3","941":"GRUPO 3","942":"GRUPO 3","943":"GRUPO 3","944":"GRUPO 3","945":"GRUPO 3","946":"GRUPO 3","947":"GRUPO 3","948":"GRUPO 4","949":"GRUPO 4","950":"GRUPO 4","951":"GRUPO 4","952":"GRUPO 4","953":"GRUPO 4","954":"GRUPO 4","955":"GRUPO 4","956":"GRUPO 4","957":"GRUPO 4","958":"GRUPO 4","959":"GRUPO 4","960":"GRUPO 1","961":"GRUPO 1","962":"GRUPO 1","963":"GRUPO 1","964":"GRUPO 1","965":"GRUPO 1","966":"GRUPO 1","967":"GRUPO 1","968":"GRUPO 1","969":"GRUPO 1","970":"GRUPO 1","971":"GRUPO 1","972":"GRUPO 2","973":"GRUPO 2","974":"GRUPO 2","975":"GRUPO 2","976":"GRUPO 2","977":"GRUPO 2","978":"GRUPO 2","979":"GRUPO 2","980":"GRUPO 2","981":"GRUPO 2","982":"GRUPO 2","983":"GRUPO 2","984":"GRUPO 3","985":"GRUPO 3","986":"GRUPO 3","987":"GRUPO 3","988":"GRUPO 3","989":"GRUPO 3","990":"GRUPO 3","991":"GRUPO 3","992":"GRUPO 3","993":"GRUPO 3","994":"GRUPO 3","995":"GRUPO 3","996":"GRUPO 4","997":"GRUPO 4","998":"GRUPO 4","999":"GRUPO 4","1000":"GRUPO 4","1001":"GRUPO 4","1002":"GRUPO 4","1003":"GRUPO 4","1004":"GRUPO 4","1005":"GRUPO 4","1006":"GRUPO 4","1007":"GRUPO 4","1008":"GRUPO 1","1009":"GRUPO 1","1010":"GRUPO 1","1011":"GRUPO 1","1012":"GRUPO 1","1013":"GRUPO 1","1014":"GRUPO 1","1015":"GRUPO 1","1016":"GRUPO 1","1017":"GRUPO 1","1018":"GRUPO 1","1019":"GRUPO 1","1020":"GRUPO 2","1021":"GRUPO 2","1022":"GRUPO 2","1023":"GRUPO 2","1024":"GRUPO 2","1025":"GRUPO 2","1026":"GRUPO 2","1027":"GRUPO 2","1028":"GRUPO 2","1029":"GRUPO 2","1030":"GRUPO 2","1031":"GRUPO 2","1032":"GRUPO 3","1033":"GRUPO 3","1034":"GRUPO 3","1035":"GRUPO 3","1036":"GRUPO 3","1037":"GRUPO 3","1038":"GRUPO 3","1039":"GRUPO 3","1040":"GRUPO 3","1041":"GRUPO 3","1042":"GRUPO 3","1043":"GRUPO 3","1044":"GRUPO 4","1045":"GRUPO 4","1046":"GRUPO 4","1047":"GRUPO 4","1048":"GRUPO 4","1049":"GRUPO 4","1050":"GRUPO 4","1051":"GRUPO 4","1052":"GRUPO 4","1053":"GRUPO 4","1054":"GRUPO 4","1055":"GRUPO 4","1056":"GRUPO 1","1057":"GRUPO 1","1058":"GRUPO 1","1059":"GRUPO 1","1060":"GRUPO 1","1061":"GRUPO 1","1062":"GRUPO 1","1063":"GRUPO 1","1064":"GRUPO 1","1065":"GRUPO 1","1066":"GRUPO 1","1067":"GRUPO 1","1068":"GRUPO 2","1069":"GRUPO 2","1070":"GRUPO 2","1071":"GRUPO 2","1072":"GRUPO 2","1073":"GRUPO 2","1074":"GRUPO 2","1075":"GRUPO 2","1076":"GRUPO 2","1077":"GRUPO 2","1078":"GRUPO 2","1079":"GRUPO 2","1080":"GRUPO 3","1081":"GRUPO 3","1082":"GRUPO 3","1083":"GRUPO 3","1084":"GRUPO 3","1085":"GRUPO 3","1086":"GRUPO 3","1087":"GRUPO 3","1088":"GRUPO 3","1089":"GRUPO 3","1090":"GRUPO 3","1091":"GRUPO 3","1092":"GRUPO 4","1093":"GRUPO 4","1094":"GRUPO 4","1095":"GRUPO 4","1096":"GRUPO 4","1097":"GRUPO 4","1098":"GRUPO 4","1099":"GRUPO 4","1100":"GRUPO 4","1101":"GRUPO 4","1102":"GRUPO 4","1103":"GRUPO 4","1104":"GRUPO 1","1105":"GRUPO 1","1106":"GRUPO 1","1107":"GRUPO 1","1108":"GRUPO 1","1109":"GRUPO 1","1110":"GRUPO 1","1111":"GRUPO 1","1112":"GRUPO 1","1113":"GRUPO 1","1114":"GRUPO 1","1115":"GRUPO 1","1116":"GRUPO 2","1117":"GRUPO 2","1118":"GRUPO 2","1119":"GRUPO 2","1120":"GRUPO 2","1121":"GRUPO 2","1122":"GRUPO 2","1123":"GRUPO 2","1124":"GRUPO 2","1125":"GRUPO 2","1126":"GRUPO 2","1127":"GRUPO 2","1128":"GRUPO 3","1129":"GRUPO 3","1130":"GRUPO 3","1131":"GRUPO 3","1132":"GRUPO 3","1133":"GRUPO 3","1134":"GRUPO 3","1135":"GRUPO 3","1136":"GRUPO 3","1137":"GRUPO 3","1138":"GRUPO 3","1139":"GRUPO 3","1140":"GRUPO 4","1141":"GRUPO 4","1142":"GRUPO 4","1143":"GRUPO 4","1144":"GRUPO 4","1145":"GRUPO 4","1146":"GRUPO 4","1147":"GRUPO 4","1148":"GRUPO 4","1149":"GRUPO 4","1150":"GRUPO 4","1151":"GRUPO 4","1152":"GRUPO 1","1153":"GRUPO 1","1154":"GRUPO 1","1155":"GRUPO 1","1156":"GRUPO 1","1157":"GRUPO 1","1158":"GRUPO 1","1159":"GRUPO 1","1160":"GRUPO 1","1161":"GRUPO 1","1162":"GRUPO 1","1163":"GRUPO 1","1164":"GRUPO 2","1165":"GRUPO 2","1166":"GRUPO 2","1167":"GRUPO 2","1168":"GRUPO 2","1169":"GRUPO 2","1170":"GRUPO 2","1171":"GRUPO 2","1172":"GRUPO 2","1173":"GRUPO 2","1174":"GRUPO 2","1175":"GRUPO 2","1176":"GRUPO 3","1177":"GRUPO 3","1178":"GRUPO 3","1179":"GRUPO 3","1180":"GRUPO 3","1181":"GRUPO 3","1182":"GRUPO 3","1183":"GRUPO 3","1184":"GRUPO 3","1185":"GRUPO 3","1186":"GRUPO 3","1187":"GRUPO 3","1188":"GRUPO 4","1189":"GRUPO 4","1190":"GRUPO 4","1191":"GRUPO 4","1192":"GRUPO 4","1193":"GRUPO 4","1194":"GRUPO 4","1195":"GRUPO 4","1196":"GRUPO 4","1197":"GRUPO 4","1198":"GRUPO 4","1199":"GRUPO 4","1200":"GRUPO 1","1201":"GRUPO 1","1202":"GRUPO 1","1203":"GRUPO 1","1204":"GRUPO 1","1205":"GRUPO 1","1206":"GRUPO 1","1207":"GRUPO 1","1208":"GRUPO 1","1209":"GRUPO 1","1210":"GRUPO 1","1211":"GRUPO 1","1212":"GRUPO 2","1213":"GRUPO 2","1214":"GRUPO 2","1215":"GRUPO 2","1216":"GRUPO 2","1217":"GRUPO 2","1218":"GRUPO 2","1219":"GRUPO 2","1220":"GRUPO 2","1221":"GRUPO 2","1222":"GRUPO 2","1223":"GRUPO 2","1224":"GRUPO 3","1225":"GRUPO 3","1226":"GRUPO 3","1227":"GRUPO 3","1228":"GRUPO 3","1229":"GRUPO 3","1230":"GRUPO 3","1231":"GRUPO 3","1232":"GRUPO 3","1233":"GRUPO 3","1234":"GRUPO 3","1235":"GRUPO 3","1236":"GRUPO 4","1237":"GRUPO 4","1238":"GRUPO 4","1239":"GRUPO 4","1240":"GRUPO 4","1241":"GRUPO 4","1242":"GRUPO 4","1243":"GRUPO 4","1244":"GRUPO 4","1245":"GRUPO 4","1246":"GRUPO 4","1247":"GRUPO 4","1248":"GRUPO 1","1249":"GRUPO 1","1250":"GRUPO 1","1251":"GRUPO 1","1252":"GRUPO 1","1253":"GRUPO 1","1254":"GRUPO 1","1255":"GRUPO 1","1256":"GRUPO 1","1257":"GRUPO 1","1258":"GRUPO 1","1259":"GRUPO 1","1260":"GRUPO 2","1261":"GRUPO 2","1262":"GRUPO 2","1263":"GRUPO 2","1264":"GRUPO 2","1265":"GRUPO 2","1266":"GRUPO 2","1267":"GRUPO 2","1268":"GRUPO 2","1269":"GRUPO 2","1270":"GRUPO 2","1271":"GRUPO 2","1272":"GRUPO 3","1273":"GRUPO 3","1274":"GRUPO 3","1275":"GRUPO 3","1276":"GRUPO 3","1277":"GRUPO 3","1278":"GRUPO 3","1279":"GRUPO 3","1280":"GRUPO 3","1281":"GRUPO 3","1282":"GRUPO 3","1283":"GRUPO 3","1284":"GRUPO 4","1285":"GRUPO 4","1286":"GRUPO 4","1287":"GRUPO 4","1288":"GRUPO 4","1289":"GRUPO 4","1290":"GRUPO 4","1291":"GRUPO 4","1292":"GRUPO 4","1293":"GRUPO 4","1294":"GRUPO 4","1295":"GRUPO 4","1296":"GRUPO 1","1297":"GRUPO 1","1298":"GRUPO 1","1299":"GRUPO 1","1300":"GRUPO 1","1301":"GRUPO 1","1302":"GRUPO 1","1303":"GRUPO 1","1304":"GRUPO 1","1305":"GRUPO 1","1306":"GRUPO 1","1307":"GRUPO 1","1308":"GRUPO 2","1309":"GRUPO 2","1310":"GRUPO 2","1311":"GRUPO 2","1312":"GRUPO 2","1313":"GRUPO 2","1314":"GRUPO 2","1315":"GRUPO 2","1316":"GRUPO 2","1317":"GRUPO 2","1318":"GRUPO 2","1319":"GRUPO 2","1320":"GRUPO 3","1321":"GRUPO 3","1322":"GRUPO 3","1323":"GRUPO 3","1324":"GRUPO 3","1325":"GRUPO 3","1326":"GRUPO 3","1327":"GRUPO 3","1328":"GRUPO 3","1329":"GRUPO 3","1330":"GRUPO 3","1331":"GRUPO 3","1332":"GRUPO 4","1333":"GRUPO 4","1334":"GRUPO 4","1335":"GRUPO 4","1336":"GRUPO 4","1337":"GRUPO 4","1338":"GRUPO 4","1339":"GRUPO 4","1340":"GRUPO 4","1341":"GRUPO 4","1342":"GRUPO 4","1343":"GRUPO 4","1344":"GRUPO 1","1345":"GRUPO 1","1346":"GRUPO 1","1347":"GRUPO 1","1348":"GRUPO 1","1349":"GRUPO 1","1350":"GRUPO 1","1351":"GRUPO 1","1352":"GRUPO 1","1353":"GRUPO 1","1354":"GRUPO 1","1355":"GRUPO 1","1356":"GRUPO 2","1357":"GRUPO 2","1358":"GRUPO 2","1359":"GRUPO 2","1360":"GRUPO 2","1361":"GRUPO 2","1362":"GRUPO 2","1363":"GRUPO 2","1364":"GRUPO 2","1365":"GRUPO 2","1366":"GRUPO 2","1367":"GRUPO 2","1368":"GRUPO 3","1369":"GRUPO 3","1370":"GRUPO 3","1371":"GRUPO 3","1372":"GRUPO 3","1373":"GRUPO 3","1374":"GRUPO 3","1375":"GRUPO 3","1376":"GRUPO 3","1377":"GRUPO 3","1378":"GRUPO 3","1379":"GRUPO 3","1380":"GRUPO 4","1381":"GRUPO 4","1382":"GRUPO 4","1383":"GRUPO 4","1384":"GRUPO 4","1385":"GRUPO 4","1386":"GRUPO 4","1387":"GRUPO 4","1388":"GRUPO 4","1389":"GRUPO 4","1390":"GRUPO 4","1391":"GRUPO 4","1392":"GRUPO 1","1393":"GRUPO 1","1394":"GRUPO 1","1395":"GRUPO 1","1396":"GRUPO 1","1397":"GRUPO 1","1398":"GRUPO 1","1399":"GRUPO 1","1400":"GRUPO 1","1401":"GRUPO 1","1402":"GRUPO 1","1403":"GRUPO 1","1404":"GRUPO 2","1405":"GRUPO 2","1406":"GRUPO 2","1407":"GRUPO 2","1408":"GRUPO 2","1409":"GRUPO 2","1410":"GRUPO 2","1411":"GRUPO 2","1412":"GRUPO 2","1413":"GRUPO 2","1414":"GRUPO 2","1415":"GRUPO 2","1416":"GRUPO 3","1417":"GRUPO 3","1418":"GRUPO 3","1419":"GRUPO 3","1420":"GRUPO 3","1421":"GRUPO 3","1422":"GRUPO 3","1423":"GRUPO 3","1424":"GRUPO 3","1425":"GRUPO 3","1426":"GRUPO 3","1427":"GRUPO 3","1428":"GRUPO 4","1429":"GRUPO 4","1430":"GRUPO 4","1431":"GRUPO 4","1432":"GRUPO 4","1433":"GRUPO 4","1434":"GRUPO 4","1435":"GRUPO 4","1436":"GRUPO 4","1437":"GRUPO 4","1438":"GRUPO 4","1439":"GRUPO 4","1440":"GRUPO 1","1441":"GRUPO 1","1442":"GRUPO 1","1443":"GRUPO 1","1444":"GRUPO 1","1445":"GRUPO 1","1446":"GRUPO 1","1447":"GRUPO 1","1448":"GRUPO 1","1449":"GRUPO 1","1450":"GRUPO 1","1451":"GRUPO 1","1452":"GRUPO 2","1453":"GRUPO 2","1454":"GRUPO 2","1455":"GRUPO 2","1456":"GRUPO 2","1457":"GRUPO 2","1458":"GRUPO 2","1459":"GRUPO 2","1460":"GRUPO 2","1461":"GRUPO 2","1462":"GRUPO 2","1463":"GRUPO 2","1464":"GRUPO 3","1465":"GRUPO 3","1466":"GRUPO 3","1467":"GRUPO 3","1468":"GRUPO 3","1469":"GRUPO 3","1470":"GRUPO 3","1471":"GRUPO 3","1472":"GRUPO 3","1473":"GRUPO 3","1474":"GRUPO 3","1475":"GRUPO 3","1476":"GRUPO 4","1477":"GRUPO 4","1478":"GRUPO 4","1479":"GRUPO 4","1480":"GRUPO 4","1481":"GRUPO 4","1482":"GRUPO 4","1483":"GRUPO 4","1484":"GRUPO 4","1485":"GRUPO 4","1486":"GRUPO 4","1487":"GRUPO 4"},"Empleado":{"0":"BARON HERNANDEZ HAROLD ANTONIO","1":"CASTELLANOS CARVAJAL DEYVITH FABIAN","2":"AROCA TORRES JULIAN EDUARDO","3":"BERMUDEZ PARRA JENNIFER XIOMARA","4":"BERNAL BAQUERO JAMES RICARDO","5":"BURGOS ORTIZ JOSE HORACIO","6":"CANTOR PORRAS JUAN FERNEY","7":"CAPERA CAPERA JOSE GABRIEL","8":"CARDENAS LOTERO RICARDO ANDR\u00c9S","9":"RENDON OSPINA NELSON LEANDRO","10":"SARMIENTO URBINA MOISES DANIEL","11":"VELASCO VELASCO SEBASTI\u00c1N DAVID","12":"DELGADO DELGADO JOHAN DARIO","13":"FLOREZ SAUCESO KENIS ALBERTO","14":"CARDONA GARCIA OSCAR JAVIER","15":"CARVAJAL GARC\u00cdA HOVER MARCK","16":"CEPEDA PIRAQUIVE JUAN DAVID","17":"FAJARDO SAENZ OSCAR FERNANDO","18":"FLOREZ ESPITIA RONY ALBERTO","19":"GARCIA CUERVO EDWIN JAVIER","20":"GONZALEZ OCHOA JUAN CARLOS","21":"XXX1","22":"XXX2","23":"XXX3","24":"FONSECA RAY RICARDO","25":"GOMEZ BETANCUR JAIDER ANDRES","26":"GRANADA PATI\u00d1O CARLOS MARINO","27":"GRASS PLATA MIGUEL SNEIDER","28":"MANZANO CALVO JUAN SEBASTIAN","29":"MENDOZA GOITA MARIANSEL ZENAYDA","30":"MURILLO ARAQUE JAIVER GEOVANY","31":"NI\u00d1O ARENAS HECTOR GONZALO","32":"RAMIREZ CHAVERRA JHON EDISON","33":"XXX4","34":"XXX5","35":"XXX6","36":"RODRIGUEZ MOSQUERA LUIS FERNANDO","37":"PEPITO PEREZ","38":"RAMIREZ VARGAS MARCELA PAOLA","39":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","40":"TORO CISNEROS GARY JOSE","41":"USECHE CALDERON JADID ESTIVEN","42":"VASQUEZ NIETO CAMILO ANDRES","43":"JHONY CASTRO","44":"BERNAL JUAN DAVID","45":"XXX7","46":"XXX8","47":"XXX9","48":"BARON HERNANDEZ HAROLD ANTONIO","49":"CASTELLANOS CARVAJAL DEYVITH FABIAN","50":"AROCA TORRES JULIAN EDUARDO","51":"BERMUDEZ PARRA JENNIFER XIOMARA","52":"BERNAL BAQUERO JAMES RICARDO","53":"BURGOS ORTIZ JOSE HORACIO","54":"CANTOR PORRAS JUAN FERNEY","55":"CAPERA CAPERA JOSE GABRIEL","56":"CARDENAS LOTERO RICARDO ANDR\u00c9S","57":"RENDON OSPINA NELSON LEANDRO","58":"SARMIENTO URBINA MOISES DANIEL","59":"VELASCO VELASCO SEBASTI\u00c1N DAVID","60":"DELGADO DELGADO JOHAN DARIO","61":"FLOREZ SAUCESO KENIS ALBERTO","62":"CARDONA GARCIA OSCAR JAVIER","63":"CARVAJAL GARC\u00cdA HOVER MARCK","64":"CEPEDA PIRAQUIVE JUAN DAVID","65":"FAJARDO SAENZ OSCAR FERNANDO","66":"FLOREZ ESPITIA RONY ALBERTO","67":"GARCIA CUERVO EDWIN JAVIER","68":"GONZALEZ OCHOA JUAN CARLOS","69":"XXX1","70":"XXX2","71":"XXX3","72":"FONSECA RAY RICARDO","73":"GOMEZ BETANCUR JAIDER ANDRES","74":"GRANADA PATI\u00d1O CARLOS MARINO","75":"GRASS PLATA MIGUEL SNEIDER","76":"MANZANO CALVO JUAN SEBASTIAN","77":"MENDOZA GOITA MARIANSEL ZENAYDA","78":"MURILLO ARAQUE JAIVER GEOVANY","79":"NI\u00d1O ARENAS HECTOR GONZALO","80":"RAMIREZ CHAVERRA JHON EDISON","81":"XXX4","82":"XXX5","83":"XXX6","84":"RODRIGUEZ MOSQUERA LUIS FERNANDO","85":"PEPITO PEREZ","86":"RAMIREZ VARGAS MARCELA PAOLA","87":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","88":"TORO CISNEROS GARY JOSE","89":"USECHE CALDERON JADID ESTIVEN","90":"VASQUEZ NIETO CAMILO ANDRES","91":"JHONY CASTRO","92":"BERNAL JUAN DAVID","93":"XXX7","94":"XXX8","95":"XXX9","96":"BARON HERNANDEZ HAROLD ANTONIO","97":"CASTELLANOS CARVAJAL DEYVITH FABIAN","98":"AROCA TORRES JULIAN EDUARDO","99":"BERMUDEZ PARRA JENNIFER XIOMARA","100":"BERNAL BAQUERO JAMES RICARDO","101":"BURGOS ORTIZ JOSE HORACIO","102":"CANTOR PORRAS JUAN FERNEY","103":"CAPERA CAPERA JOSE GABRIEL","104":"CARDENAS LOTERO RICARDO ANDR\u00c9S","105":"RENDON OSPINA NELSON LEANDRO","106":"SARMIENTO URBINA MOISES DANIEL","107":"VELASCO VELASCO SEBASTI\u00c1N DAVID","108":"DELGADO DELGADO JOHAN DARIO","109":"FLOREZ SAUCESO KENIS ALBERTO","110":"CARDONA GARCIA OSCAR JAVIER","111":"CARVAJAL GARC\u00cdA HOVER MARCK","112":"CEPEDA PIRAQUIVE JUAN DAVID","113":"FAJARDO SAENZ OSCAR FERNANDO","114":"FLOREZ ESPITIA RONY ALBERTO","115":"GARCIA CUERVO EDWIN JAVIER","116":"GONZALEZ OCHOA JUAN CARLOS","117":"XXX1","118":"XXX2","119":"XXX3","120":"FONSECA RAY RICARDO","121":"GOMEZ BETANCUR JAIDER ANDRES","122":"GRANADA PATI\u00d1O CARLOS MARINO","123":"GRASS PLATA MIGUEL SNEIDER","124":"MANZANO CALVO JUAN SEBASTIAN","125":"MENDOZA GOITA MARIANSEL ZENAYDA","126":"MURILLO ARAQUE JAIVER GEOVANY","127":"NI\u00d1O ARENAS HECTOR GONZALO","128":"RAMIREZ CHAVERRA JHON EDISON","129":"XXX4","130":"XXX5","131":"XXX6","132":"RODRIGUEZ MOSQUERA LUIS FERNANDO","133":"PEPITO PEREZ","134":"RAMIREZ VARGAS MARCELA PAOLA","135":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","136":"TORO CISNEROS GARY JOSE","137":"USECHE CALDERON JADID ESTIVEN","138":"VASQUEZ NIETO CAMILO ANDRES","139":"JHONY CASTRO","140":"BERNAL JUAN DAVID","141":"XXX7","142":"XXX8","143":"XXX9","144":"BARON HERNANDEZ HAROLD ANTONIO","145":"CASTELLANOS CARVAJAL DEYVITH FABIAN","146":"AROCA TORRES JULIAN EDUARDO","147":"BERMUDEZ PARRA JENNIFER XIOMARA","148":"BERNAL BAQUERO JAMES RICARDO","149":"BURGOS ORTIZ JOSE HORACIO","150":"CANTOR PORRAS JUAN FERNEY","151":"CAPERA CAPERA JOSE GABRIEL","152":"CARDENAS LOTERO RICARDO ANDR\u00c9S","153":"RENDON OSPINA NELSON LEANDRO","154":"SARMIENTO URBINA MOISES DANIEL","155":"VELASCO VELASCO SEBASTI\u00c1N DAVID","156":"DELGADO DELGADO JOHAN DARIO","157":"FLOREZ SAUCESO KENIS ALBERTO","158":"CARDONA GARCIA OSCAR JAVIER","159":"CARVAJAL GARC\u00cdA HOVER MARCK","160":"CEPEDA PIRAQUIVE JUAN DAVID","161":"FAJARDO SAENZ OSCAR FERNANDO","162":"FLOREZ ESPITIA RONY ALBERTO","163":"GARCIA CUERVO EDWIN JAVIER","164":"GONZALEZ OCHOA JUAN CARLOS","165":"XXX1","166":"XXX2","167":"XXX3","168":"FONSECA RAY RICARDO","169":"GOMEZ BETANCUR JAIDER ANDRES","170":"GRANADA PATI\u00d1O CARLOS MARINO","171":"GRASS PLATA MIGUEL SNEIDER","172":"MANZANO CALVO JUAN SEBASTIAN","173":"MENDOZA GOITA MARIANSEL ZENAYDA","174":"MURILLO ARAQUE JAIVER GEOVANY","175":"NI\u00d1O ARENAS HECTOR GONZALO","176":"RAMIREZ CHAVERRA JHON EDISON","177":"XXX4","178":"XXX5","179":"XXX6","180":"RODRIGUEZ MOSQUERA LUIS FERNANDO","181":"PEPITO PEREZ","182":"RAMIREZ VARGAS MARCELA PAOLA","183":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","184":"TORO CISNEROS GARY JOSE","185":"USECHE CALDERON JADID ESTIVEN","186":"VASQUEZ NIETO CAMILO ANDRES","187":"JHONY CASTRO","188":"BERNAL JUAN DAVID","189":"XXX7","190":"XXX8","191":"XXX9","192":"BARON HERNANDEZ HAROLD ANTONIO","193":"CASTELLANOS CARVAJAL DEYVITH FABIAN","194":"AROCA TORRES JULIAN EDUARDO","195":"BERMUDEZ PARRA JENNIFER XIOMARA","196":"BERNAL BAQUERO JAMES RICARDO","197":"BURGOS ORTIZ JOSE HORACIO","198":"CANTOR PORRAS JUAN FERNEY","199":"CAPERA CAPERA JOSE GABRIEL","200":"CARDENAS LOTERO RICARDO ANDR\u00c9S","201":"RENDON OSPINA NELSON LEANDRO","202":"SARMIENTO URBINA MOISES DANIEL","203":"VELASCO VELASCO SEBASTI\u00c1N DAVID","204":"DELGADO DELGADO JOHAN DARIO","205":"FLOREZ SAUCESO KENIS ALBERTO","206":"CARDONA GARCIA OSCAR JAVIER","207":"CARVAJAL GARC\u00cdA HOVER MARCK","208":"CEPEDA PIRAQUIVE JUAN DAVID","209":"FAJARDO SAENZ OSCAR FERNANDO","210":"FLOREZ ESPITIA RONY ALBERTO","211":"GARCIA CUERVO EDWIN JAVIER","212":"GONZALEZ OCHOA JUAN CARLOS","213":"XXX1","214":"XXX2","215":"XXX3","216":"FONSECA RAY RICARDO","217":"GOMEZ BETANCUR JAIDER ANDRES","218":"GRANADA PATI\u00d1O CARLOS MARINO","219":"GRASS PLATA MIGUEL SNEIDER","220":"MANZANO CALVO JUAN SEBASTIAN","221":"MENDOZA GOITA MARIANSEL ZENAYDA","222":"MURILLO ARAQUE JAIVER GEOVANY","223":"NI\u00d1O ARENAS HECTOR GONZALO","224":"RAMIREZ CHAVERRA JHON EDISON","225":"XXX4","226":"XXX5","227":"XXX6","228":"RODRIGUEZ MOSQUERA LUIS FERNANDO","229":"PEPITO PEREZ","230":"RAMIREZ VARGAS MARCELA PAOLA","231":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","232":"TORO CISNEROS GARY JOSE","233":"USECHE CALDERON JADID ESTIVEN","234":"VASQUEZ NIETO CAMILO ANDRES","235":"JHONY CASTRO","236":"BERNAL JUAN DAVID","237":"XXX7","238":"XXX8","239":"XXX9","240":"BARON HERNANDEZ HAROLD ANTONIO","241":"CASTELLANOS CARVAJAL DEYVITH FABIAN","242":"AROCA TORRES JULIAN EDUARDO","243":"BERMUDEZ PARRA JENNIFER XIOMARA","244":"BERNAL BAQUERO JAMES RICARDO","245":"BURGOS ORTIZ JOSE HORACIO","246":"CANTOR PORRAS JUAN FERNEY","247":"CAPERA CAPERA JOSE GABRIEL","248":"CARDENAS LOTERO RICARDO ANDR\u00c9S","249":"RENDON OSPINA NELSON LEANDRO","250":"SARMIENTO URBINA MOISES DANIEL","251":"VELASCO VELASCO SEBASTI\u00c1N DAVID","252":"DELGADO DELGADO JOHAN DARIO","253":"FLOREZ SAUCESO KENIS ALBERTO","254":"CARDONA GARCIA OSCAR JAVIER","255":"CARVAJAL GARC\u00cdA HOVER MARCK","256":"CEPEDA PIRAQUIVE JUAN DAVID","257":"FAJARDO SAENZ OSCAR FERNANDO","258":"FLOREZ ESPITIA RONY ALBERTO","259":"GARCIA CUERVO EDWIN JAVIER","260":"GONZALEZ OCHOA JUAN CARLOS","261":"XXX1","262":"XXX2","263":"XXX3","264":"FONSECA RAY RICARDO","265":"GOMEZ BETANCUR JAIDER ANDRES","266":"GRANADA PATI\u00d1O CARLOS MARINO","267":"GR</t>
@@ -390,7 +396,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -418,13 +424,13 @@
         <v>2026</v>
       </c>
       <c r="C2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -435,13 +441,13 @@
         <v>2026</v>
       </c>
       <c r="C3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -452,13 +458,30 @@
         <v>2026</v>
       </c>
       <c r="C4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" t="s">
         <v>8</v>
       </c>
-      <c r="D4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E4" t="s">
-        <v>14</v>
+      <c r="B5">
+        <v>2026</v>
+      </c>
+      <c r="C5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update historico_mallas.xlsx 2026-04-24 18:27:42.933440
</commit_message>
<xml_diff>
--- a/historico_mallas.xlsx
+++ b/historico_mallas.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="18">
   <si>
     <t>Mes</t>
   </si>
@@ -55,7 +55,7 @@
     <t>2026-04-24 18:24</t>
   </si>
   <si>
-    <t>2026-04-24 18:26</t>
+    <t>2026-04-24 18:27</t>
   </si>
   <si>
     <t>{"Grupo":{"0":"GRUPO 1","1":"GRUPO 1","2":"GRUPO 1","3":"GRUPO 1","4":"GRUPO 1","5":"GRUPO 1","6":"GRUPO 1","7":"GRUPO 1","8":"GRUPO 1","9":"GRUPO 1","10":"GRUPO 1","11":"GRUPO 1","12":"GRUPO 2","13":"GRUPO 2","14":"GRUPO 2","15":"GRUPO 2","16":"GRUPO 2","17":"GRUPO 2","18":"GRUPO 2","19":"GRUPO 2","20":"GRUPO 2","21":"GRUPO 2","22":"GRUPO 2","23":"GRUPO 2","24":"GRUPO 3","25":"GRUPO 3","26":"GRUPO 3","27":"GRUPO 3","28":"GRUPO 3","29":"GRUPO 3","30":"GRUPO 3","31":"GRUPO 3","32":"GRUPO 3","33":"GRUPO 3","34":"GRUPO 3","35":"GRUPO 3","36":"GRUPO 4","37":"GRUPO 4","38":"GRUPO 4","39":"GRUPO 4","40":"GRUPO 4","41":"GRUPO 4","42":"GRUPO 4","43":"GRUPO 4","44":"GRUPO 4","45":"GRUPO 4","46":"GRUPO 4","47":"GRUPO 4","48":"GRUPO 1","49":"GRUPO 1","50":"GRUPO 1","51":"GRUPO 1","52":"GRUPO 1","53":"GRUPO 1","54":"GRUPO 1","55":"GRUPO 1","56":"GRUPO 1","57":"GRUPO 1","58":"GRUPO 1","59":"GRUPO 1","60":"GRUPO 2","61":"GRUPO 2","62":"GRUPO 2","63":"GRUPO 2","64":"GRUPO 2","65":"GRUPO 2","66":"GRUPO 2","67":"GRUPO 2","68":"GRUPO 2","69":"GRUPO 2","70":"GRUPO 2","71":"GRUPO 2","72":"GRUPO 3","73":"GRUPO 3","74":"GRUPO 3","75":"GRUPO 3","76":"GRUPO 3","77":"GRUPO 3","78":"GRUPO 3","79":"GRUPO 3","80":"GRUPO 3","81":"GRUPO 3","82":"GRUPO 3","83":"GRUPO 3","84":"GRUPO 4","85":"GRUPO 4","86":"GRUPO 4","87":"GRUPO 4","88":"GRUPO 4","89":"GRUPO 4","90":"GRUPO 4","91":"GRUPO 4","92":"GRUPO 4","93":"GRUPO 4","94":"GRUPO 4","95":"GRUPO 4","96":"GRUPO 1","97":"GRUPO 1","98":"GRUPO 1","99":"GRUPO 1","100":"GRUPO 1","101":"GRUPO 1","102":"GRUPO 1","103":"GRUPO 1","104":"GRUPO 1","105":"GRUPO 1","106":"GRUPO 1","107":"GRUPO 1","108":"GRUPO 2","109":"GRUPO 2","110":"GRUPO 2","111":"GRUPO 2","112":"GRUPO 2","113":"GRUPO 2","114":"GRUPO 2","115":"GRUPO 2","116":"GRUPO 2","117":"GRUPO 2","118":"GRUPO 2","119":"GRUPO 2","120":"GRUPO 3","121":"GRUPO 3","122":"GRUPO 3","123":"GRUPO 3","124":"GRUPO 3","125":"GRUPO 3","126":"GRUPO 3","127":"GRUPO 3","128":"GRUPO 3","129":"GRUPO 3","130":"GRUPO 3","131":"GRUPO 3","132":"GRUPO 4","133":"GRUPO 4","134":"GRUPO 4","135":"GRUPO 4","136":"GRUPO 4","137":"GRUPO 4","138":"GRUPO 4","139":"GRUPO 4","140":"GRUPO 4","141":"GRUPO 4","142":"GRUPO 4","143":"GRUPO 4","144":"GRUPO 1","145":"GRUPO 1","146":"GRUPO 1","147":"GRUPO 1","148":"GRUPO 1","149":"GRUPO 1","150":"GRUPO 1","151":"GRUPO 1","152":"GRUPO 1","153":"GRUPO 1","154":"GRUPO 1","155":"GRUPO 1","156":"GRUPO 2","157":"GRUPO 2","158":"GRUPO 2","159":"GRUPO 2","160":"GRUPO 2","161":"GRUPO 2","162":"GRUPO 2","163":"GRUPO 2","164":"GRUPO 2","165":"GRUPO 2","166":"GRUPO 2","167":"GRUPO 2","168":"GRUPO 3","169":"GRUPO 3","170":"GRUPO 3","171":"GRUPO 3","172":"GRUPO 3","173":"GRUPO 3","174":"GRUPO 3","175":"GRUPO 3","176":"GRUPO 3","177":"GRUPO 3","178":"GRUPO 3","179":"GRUPO 3","180":"GRUPO 4","181":"GRUPO 4","182":"GRUPO 4","183":"GRUPO 4","184":"GRUPO 4","185":"GRUPO 4","186":"GRUPO 4","187":"GRUPO 4","188":"GRUPO 4","189":"GRUPO 4","190":"GRUPO 4","191":"GRUPO 4","192":"GRUPO 1","193":"GRUPO 1","194":"GRUPO 1","195":"GRUPO 1","196":"GRUPO 1","197":"GRUPO 1","198":"GRUPO 1","199":"GRUPO 1","200":"GRUPO 1","201":"GRUPO 1","202":"GRUPO 1","203":"GRUPO 1","204":"GRUPO 2","205":"GRUPO 2","206":"GRUPO 2","207":"GRUPO 2","208":"GRUPO 2","209":"GRUPO 2","210":"GRUPO 2","211":"GRUPO 2","212":"GRUPO 2","213":"GRUPO 2","214":"GRUPO 2","215":"GRUPO 2","216":"GRUPO 3","217":"GRUPO 3","218":"GRUPO 3","219":"GRUPO 3","220":"GRUPO 3","221":"GRUPO 3","222":"GRUPO 3","223":"GRUPO 3","224":"GRUPO 3","225":"GRUPO 3","226":"GRUPO 3","227":"GRUPO 3","228":"GRUPO 4","229":"GRUPO 4","230":"GRUPO 4","231":"GRUPO 4","232":"GRUPO 4","233":"GRUPO 4","234":"GRUPO 4","235":"GRUPO 4","236":"GRUPO 4","237":"GRUPO 4","238":"GRUPO 4","239":"GRUPO 4","240":"GRUPO 1","241":"GRUPO 1","242":"GRUPO 1","243":"GRUPO 1","244":"GRUPO 1","245":"GRUPO 1","246":"GRUPO 1","247":"GRUPO 1","248":"GRUPO 1","249":"GRUPO 1","250":"GRUPO 1","251":"GRUPO 1","252":"GRUPO 2","253":"GRUPO 2","254":"GRUPO 2","255":"GRUPO 2","256":"GRUPO 2","257":"GRUPO 2","258":"GRUPO 2","259":"GRUPO 2","260":"GRUPO 2","261":"GRUPO 2","262":"GRUPO 2","263":"GRUPO 2","264":"GRUPO 3","265":"GRUPO 3","266":"GRUPO 3","267":"GRUPO 3","268":"GRUPO 3","269":"GRUPO 3","270":"GRUPO 3","271":"GRUPO 3","272":"GRUPO 3","273":"GRUPO 3","274":"GRUPO 3","275":"GRUPO 3","276":"GRUPO 4","277":"GRUPO 4","278":"GRUPO 4","279":"GRUPO 4","280":"GRUPO 4","281":"GRUPO 4","282":"GRUPO 4","283":"GRUPO 4","284":"GRUPO 4","285":"GRUPO 4","286":"GRUPO 4","287":"GRUPO 4","288":"GRUPO 1","289":"GRUPO 1","290":"GRUPO 1","291":"GRUPO 1","292":"GRUPO 1","293":"GRUPO 1","294":"GRUPO 1","295":"GRUPO 1","296":"GRUPO 1","297":"GRUPO 1","298":"GRUPO 1","299":"GRUPO 1","300":"GRUPO 2","301":"GRUPO 2","302":"GRUPO 2","303":"GRUPO 2","304":"GRUPO 2","305":"GRUPO 2","306":"GRUPO 2","307":"GRUPO 2","308":"GRUPO 2","309":"GRUPO 2","310":"GRUPO 2","311":"GRUPO 2","312":"GRUPO 3","313":"GRUPO 3","314":"GRUPO 3","315":"GRUPO 3","316":"GRUPO 3","317":"GRUPO 3","318":"GRUPO 3","319":"GRUPO 3","320":"GRUPO 3","321":"GRUPO 3","322":"GRUPO 3","323":"GRUPO 3","324":"GRUPO 4","325":"GRUPO 4","326":"GRUPO 4","327":"GRUPO 4","328":"GRUPO 4","329":"GRUPO 4","330":"GRUPO 4","331":"GRUPO 4","332":"GRUPO 4","333":"GRUPO 4","334":"GRUPO 4","335":"GRUPO 4","336":"GRUPO 1","337":"GRUPO 1","338":"GRUPO 1","339":"GRUPO 1","340":"GRUPO 1","341":"GRUPO 1","342":"GRUPO 1","343":"GRUPO 1","344":"GRUPO 1","345":"GRUPO 1","346":"GRUPO 1","347":"GRUPO 1","348":"GRUPO 2","349":"GRUPO 2","350":"GRUPO 2","351":"GRUPO 2","352":"GRUPO 2","353":"GRUPO 2","354":"GRUPO 2","355":"GRUPO 2","356":"GRUPO 2","357":"GRUPO 2","358":"GRUPO 2","359":"GRUPO 2","360":"GRUPO 3","361":"GRUPO 3","362":"GRUPO 3","363":"GRUPO 3","364":"GRUPO 3","365":"GRUPO 3","366":"GRUPO 3","367":"GRUPO 3","368":"GRUPO 3","369":"GRUPO 3","370":"GRUPO 3","371":"GRUPO 3","372":"GRUPO 4","373":"GRUPO 4","374":"GRUPO 4","375":"GRUPO 4","376":"GRUPO 4","377":"GRUPO 4","378":"GRUPO 4","379":"GRUPO 4","380":"GRUPO 4","381":"GRUPO 4","382":"GRUPO 4","383":"GRUPO 4","384":"GRUPO 1","385":"GRUPO 1","386":"GRUPO 1","387":"GRUPO 1","388":"GRUPO 1","389":"GRUPO 1","390":"GRUPO 1","391":"GRUPO 1","392":"GRUPO 1","393":"GRUPO 1","394":"GRUPO 1","395":"GRUPO 1","396":"GRUPO 2","397":"GRUPO 2","398":"GRUPO 2","399":"GRUPO 2","400":"GRUPO 2","401":"GRUPO 2","402":"GRUPO 2","403":"GRUPO 2","404":"GRUPO 2","405":"GRUPO 2","406":"GRUPO 2","407":"GRUPO 2","408":"GRUPO 3","409":"GRUPO 3","410":"GRUPO 3","411":"GRUPO 3","412":"GRUPO 3","413":"GRUPO 3","414":"GRUPO 3","415":"GRUPO 3","416":"GRUPO 3","417":"GRUPO 3","418":"GRUPO 3","419":"GRUPO 3","420":"GRUPO 4","421":"GRUPO 4","422":"GRUPO 4","423":"GRUPO 4","424":"GRUPO 4","425":"GRUPO 4","426":"GRUPO 4","427":"GRUPO 4","428":"GRUPO 4","429":"GRUPO 4","430":"GRUPO 4","431":"GRUPO 4","432":"GRUPO 1","433":"GRUPO 1","434":"GRUPO 1","435":"GRUPO 1","436":"GRUPO 1","437":"GRUPO 1","438":"GRUPO 1","439":"GRUPO 1","440":"GRUPO 1","441":"GRUPO 1","442":"GRUPO 1","443":"GRUPO 1","444":"GRUPO 2","445":"GRUPO 2","446":"GRUPO 2","447":"GRUPO 2","448":"GRUPO 2","449":"GRUPO 2","450":"GRUPO 2","451":"GRUPO 2","452":"GRUPO 2","453":"GRUPO 2","454":"GRUPO 2","455":"GRUPO 2","456":"GRUPO 3","457":"GRUPO 3","458":"GRUPO 3","459":"GRUPO 3","460":"GRUPO 3","461":"GRUPO 3","462":"GRUPO 3","463":"GRUPO 3","464":"GRUPO 3","465":"GRUPO 3","466":"GRUPO 3","467":"GRUPO 3","468":"GRUPO 4","469":"GRUPO 4","470":"GRUPO 4","471":"GRUPO 4","472":"GRUPO 4","473":"GRUPO 4","474":"GRUPO 4","475":"GRUPO 4","476":"GRUPO 4","477":"GRUPO 4","478":"GRUPO 4","479":"GRUPO 4","480":"GRUPO 1","481":"GRUPO 1","482":"GRUPO 1","483":"GRUPO 1","484":"GRUPO 1","485":"GRUPO 1","486":"GRUPO 1","487":"GRUPO 1","488":"GRUPO 1","489":"GRUPO 1","490":"GRUPO 1","491":"GRUPO 1","492":"GRUPO 2","493":"GRUPO 2","494":"GRUPO 2","495":"GRUPO 2","496":"GRUPO 2","497":"GRUPO 2","498":"GRUPO 2","499":"GRUPO 2","500":"GRUPO 2","501":"GRUPO 2","502":"GRUPO 2","503":"GRUPO 2","504":"GRUPO 3","505":"GRUPO 3","506":"GRUPO 3","507":"GRUPO 3","508":"GRUPO 3","509":"GRUPO 3","510":"GRUPO 3","511":"GRUPO 3","512":"GRUPO 3","513":"GRUPO 3","514":"GRUPO 3","515":"GRUPO 3","516":"GRUPO 4","517":"GRUPO 4","518":"GRUPO 4","519":"GRUPO 4","520":"GRUPO 4","521":"GRUPO 4","522":"GRUPO 4","523":"GRUPO 4","524":"GRUPO 4","525":"GRUPO 4","526":"GRUPO 4","527":"GRUPO 4","528":"GRUPO 1","529":"GRUPO 1","530":"GRUPO 1","531":"GRUPO 1","532":"GRUPO 1","533":"GRUPO 1","534":"GRUPO 1","535":"GRUPO 1","536":"GRUPO 1","537":"GRUPO 1","538":"GRUPO 1","539":"GRUPO 1","540":"GRUPO 2","541":"GRUPO 2","542":"GRUPO 2","543":"GRUPO 2","544":"GRUPO 2","545":"GRUPO 2","546":"GRUPO 2","547":"GRUPO 2","548":"GRUPO 2","549":"GRUPO 2","550":"GRUPO 2","551":"GRUPO 2","552":"GRUPO 3","553":"GRUPO 3","554":"GRUPO 3","555":"GRUPO 3","556":"GRUPO 3","557":"GRUPO 3","558":"GRUPO 3","559":"GRUPO 3","560":"GRUPO 3","561":"GRUPO 3","562":"GRUPO 3","563":"GRUPO 3","564":"GRUPO 4","565":"GRUPO 4","566":"GRUPO 4","567":"GRUPO 4","568":"GRUPO 4","569":"GRUPO 4","570":"GRUPO 4","571":"GRUPO 4","572":"GRUPO 4","573":"GRUPO 4","574":"GRUPO 4","575":"GRUPO 4","576":"GRUPO 1","577":"GRUPO 1","578":"GRUPO 1","579":"GRUPO 1","580":"GRUPO 1","581":"GRUPO 1","582":"GRUPO 1","583":"GRUPO 1","584":"GRUPO 1","585":"GRUPO 1","586":"GRUPO 1","587":"GRUPO 1","588":"GRUPO 2","589":"GRUPO 2","590":"GRUPO 2","591":"GRUPO 2","592":"GRUPO 2","593":"GRUPO 2","594":"GRUPO 2","595":"GRUPO 2","596":"GRUPO 2","597":"GRUPO 2","598":"GRUPO 2","599":"GRUPO 2","600":"GRUPO 3","601":"GRUPO 3","602":"GRUPO 3","603":"GRUPO 3","604":"GRUPO 3","605":"GRUPO 3","606":"GRUPO 3","607":"GRUPO 3","608":"GRUPO 3","609":"GRUPO 3","610":"GRUPO 3","611":"GRUPO 3","612":"GRUPO 4","613":"GRUPO 4","614":"GRUPO 4","615":"GRUPO 4","616":"GRUPO 4","617":"GRUPO 4","618":"GRUPO 4","619":"GRUPO 4","620":"GRUPO 4","621":"GRUPO 4","622":"GRUPO 4","623":"GRUPO 4","624":"GRUPO 1","625":"GRUPO 1","626":"GRUPO 1","627":"GRUPO 1","628":"GRUPO 1","629":"GRUPO 1","630":"GRUPO 1","631":"GRUPO 1","632":"GRUPO 1","633":"GRUPO 1","634":"GRUPO 1","635":"GRUPO 1","636":"GRUPO 2","637":"GRUPO 2","638":"GRUPO 2","639":"GRUPO 2","640":"GRUPO 2","641":"GRUPO 2","642":"GRUPO 2","643":"GRUPO 2","644":"GRUPO 2","645":"GRUPO 2","646":"GRUPO 2","647":"GRUPO 2","648":"GRUPO 3","649":"GRUPO 3","650":"GRUPO 3","651":"GRUPO 3","652":"GRUPO 3","653":"GRUPO 3","654":"GRUPO 3","655":"GRUPO 3","656":"GRUPO 3","657":"GRUPO 3","658":"GRUPO 3","659":"GRUPO 3","660":"GRUPO 4","661":"GRUPO 4","662":"GRUPO 4","663":"GRUPO 4","664":"GRUPO 4","665":"GRUPO 4","666":"GRUPO 4","667":"GRUPO 4","668":"GRUPO 4","669":"GRUPO 4","670":"GRUPO 4","671":"GRUPO 4","672":"GRUPO 1","673":"GRUPO 1","674":"GRUPO 1","675":"GRUPO 1","676":"GRUPO 1","677":"GRUPO 1","678":"GRUPO 1","679":"GRUPO 1","680":"GRUPO 1","681":"GRUPO 1","682":"GRUPO 1","683":"GRUPO 1","684":"GRUPO 2","685":"GRUPO 2","686":"GRUPO 2","687":"GRUPO 2","688":"GRUPO 2","689":"GRUPO 2","690":"GRUPO 2","691":"GRUPO 2","692":"GRUPO 2","693":"GRUPO 2","694":"GRUPO 2","695":"GRUPO 2","696":"GRUPO 3","697":"GRUPO 3","698":"GRUPO 3","699":"GRUPO 3","700":"GRUPO 3","701":"GRUPO 3","702":"GRUPO 3","703":"GRUPO 3","704":"GRUPO 3","705":"GRUPO 3","706":"GRUPO 3","707":"GRUPO 3","708":"GRUPO 4","709":"GRUPO 4","710":"GRUPO 4","711":"GRUPO 4","712":"GRUPO 4","713":"GRUPO 4","714":"GRUPO 4","715":"GRUPO 4","716":"GRUPO 4","717":"GRUPO 4","718":"GRUPO 4","719":"GRUPO 4","720":"GRUPO 1","721":"GRUPO 1","722":"GRUPO 1","723":"GRUPO 1","724":"GRUPO 1","725":"GRUPO 1","726":"GRUPO 1","727":"GRUPO 1","728":"GRUPO 1","729":"GRUPO 1","730":"GRUPO 1","731":"GRUPO 1","732":"GRUPO 2","733":"GRUPO 2","734":"GRUPO 2","735":"GRUPO 2","736":"GRUPO 2","737":"GRUPO 2","738":"GRUPO 2","739":"GRUPO 2","740":"GRUPO 2","741":"GRUPO 2","742":"GRUPO 2","743":"GRUPO 2","744":"GRUPO 3","745":"GRUPO 3","746":"GRUPO 3","747":"GRUPO 3","748":"GRUPO 3","749":"GRUPO 3","750":"GRUPO 3","751":"GRUPO 3","752":"GRUPO 3","753":"GRUPO 3","754":"GRUPO 3","755":"GRUPO 3","756":"GRUPO 4","757":"GRUPO 4","758":"GRUPO 4","759":"GRUPO 4","760":"GRUPO 4","761":"GRUPO 4","762":"GRUPO 4","763":"GRUPO 4","764":"GRUPO 4","765":"GRUPO 4","766":"GRUPO 4","767":"GRUPO 4","768":"GRUPO 1","769":"GRUPO 1","770":"GRUPO 1","771":"GRUPO 1","772":"GRUPO 1","773":"GRUPO 1","774":"GRUPO 1","775":"GRUPO 1","776":"GRUPO 1","777":"GRUPO 1","778":"GRUPO 1","779":"GRUPO 1","780":"GRUPO 2","781":"GRUPO 2","782":"GRUPO 2","783":"GRUPO 2","784":"GRUPO 2","785":"GRUPO 2","786":"GRUPO 2","787":"GRUPO 2","788":"GRUPO 2","789":"GRUPO 2","790":"GRUPO 2","791":"GRUPO 2","792":"GRUPO 3","793":"GRUPO 3","794":"GRUPO 3","795":"GRUPO 3","796":"GRUPO 3","797":"GRUPO 3","798":"GRUPO 3","799":"GRUPO 3","800":"GRUPO 3","801":"GRUPO 3","802":"GRUPO 3","803":"GRUPO 3","804":"GRUPO 4","805":"GRUPO 4","806":"GRUPO 4","807":"GRUPO 4","808":"GRUPO 4","809":"GRUPO 4","810":"GRUPO 4","811":"GRUPO 4","812":"GRUPO 4","813":"GRUPO 4","814":"GRUPO 4","815":"GRUPO 4","816":"GRUPO 1","817":"GRUPO 1","818":"GRUPO 1","819":"GRUPO 1","820":"GRUPO 1","821":"GRUPO 1","822":"GRUPO 1","823":"GRUPO 1","824":"GRUPO 1","825":"GRUPO 1","826":"GRUPO 1","827":"GRUPO 1","828":"GRUPO 2","829":"GRUPO 2","830":"GRUPO 2","831":"GRUPO 2","832":"GRUPO 2","833":"GRUPO 2","834":"GRUPO 2","835":"GRUPO 2","836":"GRUPO 2","837":"GRUPO 2","838":"GRUPO 2","839":"GRUPO 2","840":"GRUPO 3","841":"GRUPO 3","842":"GRUPO 3","843":"GRUPO 3","844":"GRUPO 3","845":"GRUPO 3","846":"GRUPO 3","847":"GRUPO 3","848":"GRUPO 3","849":"GRUPO 3","850":"GRUPO 3","851":"GRUPO 3","852":"GRUPO 4","853":"GRUPO 4","854":"GRUPO 4","855":"GRUPO 4","856":"GRUPO 4","857":"GRUPO 4","858":"GRUPO 4","859":"GRUPO 4","860":"GRUPO 4","861":"GRUPO 4","862":"GRUPO 4","863":"GRUPO 4","864":"GRUPO 1","865":"GRUPO 1","866":"GRUPO 1","867":"GRUPO 1","868":"GRUPO 1","869":"GRUPO 1","870":"GRUPO 1","871":"GRUPO 1","872":"GRUPO 1","873":"GRUPO 1","874":"GRUPO 1","875":"GRUPO 1","876":"GRUPO 2","877":"GRUPO 2","878":"GRUPO 2","879":"GRUPO 2","880":"GRUPO 2","881":"GRUPO 2","882":"GRUPO 2","883":"GRUPO 2","884":"GRUPO 2","885":"GRUPO 2","886":"GRUPO 2","887":"GRUPO 2","888":"GRUPO 3","889":"GRUPO 3","890":"GRUPO 3","891":"GRUPO 3","892":"GRUPO 3","893":"GRUPO 3","894":"GRUPO 3","895":"GRUPO 3","896":"GRUPO 3","897":"GRUPO 3","898":"GRUPO 3","899":"GRUPO 3","900":"GRUPO 4","901":"GRUPO 4","902":"GRUPO 4","903":"GRUPO 4","904":"GRUPO 4","905":"GRUPO 4","906":"GRUPO 4","907":"GRUPO 4","908":"GRUPO 4","909":"GRUPO 4","910":"GRUPO 4","911":"GRUPO 4","912":"GRUPO 1","913":"GRUPO 1","914":"GRUPO 1","915":"GRUPO 1","916":"GRUPO 1","917":"GRUPO 1","918":"GRUPO 1","919":"GRUPO 1","920":"GRUPO 1","921":"GRUPO 1","922":"GRUPO 1","923":"GRUPO 1","924":"GRUPO 2","925":"GRUPO 2","926":"GRUPO 2","927":"GRUPO 2","928":"GRUPO 2","929":"GRUPO 2","930":"GRUPO 2","931":"GRUPO 2","932":"GRUPO 2","933":"GRUPO 2","934":"GRUPO 2","935":"GRUPO 2","936":"GRUPO 3","937":"GRUPO 3","938":"GRUPO 3","939":"GRUPO 3","940":"GRUPO 3","941":"GRUPO 3","942":"GRUPO 3","943":"GRUPO 3","944":"GRUPO 3","945":"GRUPO 3","946":"GRUPO 3","947":"GRUPO 3","948":"GRUPO 4","949":"GRUPO 4","950":"GRUPO 4","951":"GRUPO 4","952":"GRUPO 4","953":"GRUPO 4","954":"GRUPO 4","955":"GRUPO 4","956":"GRUPO 4","957":"GRUPO 4","958":"GRUPO 4","959":"GRUPO 4","960":"GRUPO 1","961":"GRUPO 1","962":"GRUPO 1","963":"GRUPO 1","964":"GRUPO 1","965":"GRUPO 1","966":"GRUPO 1","967":"GRUPO 1","968":"GRUPO 1","969":"GRUPO 1","970":"GRUPO 1","971":"GRUPO 1","972":"GRUPO 2","973":"GRUPO 2","974":"GRUPO 2","975":"GRUPO 2","976":"GRUPO 2","977":"GRUPO 2","978":"GRUPO 2","979":"GRUPO 2","980":"GRUPO 2","981":"GRUPO 2","982":"GRUPO 2","983":"GRUPO 2","984":"GRUPO 3","985":"GRUPO 3","986":"GRUPO 3","987":"GRUPO 3","988":"GRUPO 3","989":"GRUPO 3","990":"GRUPO 3","991":"GRUPO 3","992":"GRUPO 3","993":"GRUPO 3","994":"GRUPO 3","995":"GRUPO 3","996":"GRUPO 4","997":"GRUPO 4","998":"GRUPO 4","999":"GRUPO 4","1000":"GRUPO 4","1001":"GRUPO 4","1002":"GRUPO 4","1003":"GRUPO 4","1004":"GRUPO 4","1005":"GRUPO 4","1006":"GRUPO 4","1007":"GRUPO 4","1008":"GRUPO 1","1009":"GRUPO 1","1010":"GRUPO 1","1011":"GRUPO 1","1012":"GRUPO 1","1013":"GRUPO 1","1014":"GRUPO 1","1015":"GRUPO 1","1016":"GRUPO 1","1017":"GRUPO 1","1018":"GRUPO 1","1019":"GRUPO 1","1020":"GRUPO 2","1021":"GRUPO 2","1022":"GRUPO 2","1023":"GRUPO 2","1024":"GRUPO 2","1025":"GRUPO 2","1026":"GRUPO 2","1027":"GRUPO 2","1028":"GRUPO 2","1029":"GRUPO 2","1030":"GRUPO 2","1031":"GRUPO 2","1032":"GRUPO 3","1033":"GRUPO 3","1034":"GRUPO 3","1035":"GRUPO 3","1036":"GRUPO 3","1037":"GRUPO 3","1038":"GRUPO 3","1039":"GRUPO 3","1040":"GRUPO 3","1041":"GRUPO 3","1042":"GRUPO 3","1043":"GRUPO 3","1044":"GRUPO 4","1045":"GRUPO 4","1046":"GRUPO 4","1047":"GRUPO 4","1048":"GRUPO 4","1049":"GRUPO 4","1050":"GRUPO 4","1051":"GRUPO 4","1052":"GRUPO 4","1053":"GRUPO 4","1054":"GRUPO 4","1055":"GRUPO 4","1056":"GRUPO 1","1057":"GRUPO 1","1058":"GRUPO 1","1059":"GRUPO 1","1060":"GRUPO 1","1061":"GRUPO 1","1062":"GRUPO 1","1063":"GRUPO 1","1064":"GRUPO 1","1065":"GRUPO 1","1066":"GRUPO 1","1067":"GRUPO 1","1068":"GRUPO 2","1069":"GRUPO 2","1070":"GRUPO 2","1071":"GRUPO 2","1072":"GRUPO 2","1073":"GRUPO 2","1074":"GRUPO 2","1075":"GRUPO 2","1076":"GRUPO 2","1077":"GRUPO 2","1078":"GRUPO 2","1079":"GRUPO 2","1080":"GRUPO 3","1081":"GRUPO 3","1082":"GRUPO 3","1083":"GRUPO 3","1084":"GRUPO 3","1085":"GRUPO 3","1086":"GRUPO 3","1087":"GRUPO 3","1088":"GRUPO 3","1089":"GRUPO 3","1090":"GRUPO 3","1091":"GRUPO 3","1092":"GRUPO 4","1093":"GRUPO 4","1094":"GRUPO 4","1095":"GRUPO 4","1096":"GRUPO 4","1097":"GRUPO 4","1098":"GRUPO 4","1099":"GRUPO 4","1100":"GRUPO 4","1101":"GRUPO 4","1102":"GRUPO 4","1103":"GRUPO 4","1104":"GRUPO 1","1105":"GRUPO 1","1106":"GRUPO 1","1107":"GRUPO 1","1108":"GRUPO 1","1109":"GRUPO 1","1110":"GRUPO 1","1111":"GRUPO 1","1112":"GRUPO 1","1113":"GRUPO 1","1114":"GRUPO 1","1115":"GRUPO 1","1116":"GRUPO 2","1117":"GRUPO 2","1118":"GRUPO 2","1119":"GRUPO 2","1120":"GRUPO 2","1121":"GRUPO 2","1122":"GRUPO 2","1123":"GRUPO 2","1124":"GRUPO 2","1125":"GRUPO 2","1126":"GRUPO 2","1127":"GRUPO 2","1128":"GRUPO 3","1129":"GRUPO 3","1130":"GRUPO 3","1131":"GRUPO 3","1132":"GRUPO 3","1133":"GRUPO 3","1134":"GRUPO 3","1135":"GRUPO 3","1136":"GRUPO 3","1137":"GRUPO 3","1138":"GRUPO 3","1139":"GRUPO 3","1140":"GRUPO 4","1141":"GRUPO 4","1142":"GRUPO 4","1143":"GRUPO 4","1144":"GRUPO 4","1145":"GRUPO 4","1146":"GRUPO 4","1147":"GRUPO 4","1148":"GRUPO 4","1149":"GRUPO 4","1150":"GRUPO 4","1151":"GRUPO 4","1152":"GRUPO 1","1153":"GRUPO 1","1154":"GRUPO 1","1155":"GRUPO 1","1156":"GRUPO 1","1157":"GRUPO 1","1158":"GRUPO 1","1159":"GRUPO 1","1160":"GRUPO 1","1161":"GRUPO 1","1162":"GRUPO 1","1163":"GRUPO 1","1164":"GRUPO 2","1165":"GRUPO 2","1166":"GRUPO 2","1167":"GRUPO 2","1168":"GRUPO 2","1169":"GRUPO 2","1170":"GRUPO 2","1171":"GRUPO 2","1172":"GRUPO 2","1173":"GRUPO 2","1174":"GRUPO 2","1175":"GRUPO 2","1176":"GRUPO 3","1177":"GRUPO 3","1178":"GRUPO 3","1179":"GRUPO 3","1180":"GRUPO 3","1181":"GRUPO 3","1182":"GRUPO 3","1183":"GRUPO 3","1184":"GRUPO 3","1185":"GRUPO 3","1186":"GRUPO 3","1187":"GRUPO 3","1188":"GRUPO 4","1189":"GRUPO 4","1190":"GRUPO 4","1191":"GRUPO 4","1192":"GRUPO 4","1193":"GRUPO 4","1194":"GRUPO 4","1195":"GRUPO 4","1196":"GRUPO 4","1197":"GRUPO 4","1198":"GRUPO 4","1199":"GRUPO 4","1200":"GRUPO 1","1201":"GRUPO 1","1202":"GRUPO 1","1203":"GRUPO 1","1204":"GRUPO 1","1205":"GRUPO 1","1206":"GRUPO 1","1207":"GRUPO 1","1208":"GRUPO 1","1209":"GRUPO 1","1210":"GRUPO 1","1211":"GRUPO 1","1212":"GRUPO 2","1213":"GRUPO 2","1214":"GRUPO 2","1215":"GRUPO 2","1216":"GRUPO 2","1217":"GRUPO 2","1218":"GRUPO 2","1219":"GRUPO 2","1220":"GRUPO 2","1221":"GRUPO 2","1222":"GRUPO 2","1223":"GRUPO 2","1224":"GRUPO 3","1225":"GRUPO 3","1226":"GRUPO 3","1227":"GRUPO 3","1228":"GRUPO 3","1229":"GRUPO 3","1230":"GRUPO 3","1231":"GRUPO 3","1232":"GRUPO 3","1233":"GRUPO 3","1234":"GRUPO 3","1235":"GRUPO 3","1236":"GRUPO 4","1237":"GRUPO 4","1238":"GRUPO 4","1239":"GRUPO 4","1240":"GRUPO 4","1241":"GRUPO 4","1242":"GRUPO 4","1243":"GRUPO 4","1244":"GRUPO 4","1245":"GRUPO 4","1246":"GRUPO 4","1247":"GRUPO 4","1248":"GRUPO 1","1249":"GRUPO 1","1250":"GRUPO 1","1251":"GRUPO 1","1252":"GRUPO 1","1253":"GRUPO 1","1254":"GRUPO 1","1255":"GRUPO 1","1256":"GRUPO 1","1257":"GRUPO 1","1258":"GRUPO 1","1259":"GRUPO 1","1260":"GRUPO 2","1261":"GRUPO 2","1262":"GRUPO 2","1263":"GRUPO 2","1264":"GRUPO 2","1265":"GRUPO 2","1266":"GRUPO 2","1267":"GRUPO 2","1268":"GRUPO 2","1269":"GRUPO 2","1270":"GRUPO 2","1271":"GRUPO 2","1272":"GRUPO 3","1273":"GRUPO 3","1274":"GRUPO 3","1275":"GRUPO 3","1276":"GRUPO 3","1277":"GRUPO 3","1278":"GRUPO 3","1279":"GRUPO 3","1280":"GRUPO 3","1281":"GRUPO 3","1282":"GRUPO 3","1283":"GRUPO 3","1284":"GRUPO 4","1285":"GRUPO 4","1286":"GRUPO 4","1287":"GRUPO 4","1288":"GRUPO 4","1289":"GRUPO 4","1290":"GRUPO 4","1291":"GRUPO 4","1292":"GRUPO 4","1293":"GRUPO 4","1294":"GRUPO 4","1295":"GRUPO 4","1296":"GRUPO 1","1297":"GRUPO 1","1298":"GRUPO 1","1299":"GRUPO 1","1300":"GRUPO 1","1301":"GRUPO 1","1302":"GRUPO 1","1303":"GRUPO 1","1304":"GRUPO 1","1305":"GRUPO 1","1306":"GRUPO 1","1307":"GRUPO 1","1308":"GRUPO 2","1309":"GRUPO 2","1310":"GRUPO 2","1311":"GRUPO 2","1312":"GRUPO 2","1313":"GRUPO 2","1314":"GRUPO 2","1315":"GRUPO 2","1316":"GRUPO 2","1317":"GRUPO 2","1318":"GRUPO 2","1319":"GRUPO 2","1320":"GRUPO 3","1321":"GRUPO 3","1322":"GRUPO 3","1323":"GRUPO 3","1324":"GRUPO 3","1325":"GRUPO 3","1326":"GRUPO 3","1327":"GRUPO 3","1328":"GRUPO 3","1329":"GRUPO 3","1330":"GRUPO 3","1331":"GRUPO 3","1332":"GRUPO 4","1333":"GRUPO 4","1334":"GRUPO 4","1335":"GRUPO 4","1336":"GRUPO 4","1337":"GRUPO 4","1338":"GRUPO 4","1339":"GRUPO 4","1340":"GRUPO 4","1341":"GRUPO 4","1342":"GRUPO 4","1343":"GRUPO 4","1344":"GRUPO 1","1345":"GRUPO 1","1346":"GRUPO 1","1347":"GRUPO 1","1348":"GRUPO 1","1349":"GRUPO 1","1350":"GRUPO 1","1351":"GRUPO 1","1352":"GRUPO 1","1353":"GRUPO 1","1354":"GRUPO 1","1355":"GRUPO 1","1356":"GRUPO 2","1357":"GRUPO 2","1358":"GRUPO 2","1359":"GRUPO 2","1360":"GRUPO 2","1361":"GRUPO 2","1362":"GRUPO 2","1363":"GRUPO 2","1364":"GRUPO 2","1365":"GRUPO 2","1366":"GRUPO 2","1367":"GRUPO 2","1368":"GRUPO 3","1369":"GRUPO 3","1370":"GRUPO 3","1371":"GRUPO 3","1372":"GRUPO 3","1373":"GRUPO 3","1374":"GRUPO 3","1375":"GRUPO 3","1376":"GRUPO 3","1377":"GRUPO 3","1378":"GRUPO 3","1379":"GRUPO 3","1380":"GRUPO 4","1381":"GRUPO 4","1382":"GRUPO 4","1383":"GRUPO 4","1384":"GRUPO 4","1385":"GRUPO 4","1386":"GRUPO 4","1387":"GRUPO 4","1388":"GRUPO 4","1389":"GRUPO 4","1390":"GRUPO 4","1391":"GRUPO 4","1392":"GRUPO 1","1393":"GRUPO 1","1394":"GRUPO 1","1395":"GRUPO 1","1396":"GRUPO 1","1397":"GRUPO 1","1398":"GRUPO 1","1399":"GRUPO 1","1400":"GRUPO 1","1401":"GRUPO 1","1402":"GRUPO 1","1403":"GRUPO 1","1404":"GRUPO 2","1405":"GRUPO 2","1406":"GRUPO 2","1407":"GRUPO 2","1408":"GRUPO 2","1409":"GRUPO 2","1410":"GRUPO 2","1411":"GRUPO 2","1412":"GRUPO 2","1413":"GRUPO 2","1414":"GRUPO 2","1415":"GRUPO 2","1416":"GRUPO 3","1417":"GRUPO 3","1418":"GRUPO 3","1419":"GRUPO 3","1420":"GRUPO 3","1421":"GRUPO 3","1422":"GRUPO 3","1423":"GRUPO 3","1424":"GRUPO 3","1425":"GRUPO 3","1426":"GRUPO 3","1427":"GRUPO 3","1428":"GRUPO 4","1429":"GRUPO 4","1430":"GRUPO 4","1431":"GRUPO 4","1432":"GRUPO 4","1433":"GRUPO 4","1434":"GRUPO 4","1435":"GRUPO 4","1436":"GRUPO 4","1437":"GRUPO 4","1438":"GRUPO 4","1439":"GRUPO 4","1440":"GRUPO 1","1441":"GRUPO 1","1442":"GRUPO 1","1443":"GRUPO 1","1444":"GRUPO 1","1445":"GRUPO 1","1446":"GRUPO 1","1447":"GRUPO 1","1448":"GRUPO 1","1449":"GRUPO 1","1450":"GRUPO 1","1451":"GRUPO 1","1452":"GRUPO 2","1453":"GRUPO 2","1454":"GRUPO 2","1455":"GRUPO 2","1456":"GRUPO 2","1457":"GRUPO 2","1458":"GRUPO 2","1459":"GRUPO 2","1460":"GRUPO 2","1461":"GRUPO 2","1462":"GRUPO 2","1463":"GRUPO 2","1464":"GRUPO 3","1465":"GRUPO 3","1466":"GRUPO 3","1467":"GRUPO 3","1468":"GRUPO 3","1469":"GRUPO 3","1470":"GRUPO 3","1471":"GRUPO 3","1472":"GRUPO 3","1473":"GRUPO 3","1474":"GRUPO 3","1475":"GRUPO 3","1476":"GRUPO 4","1477":"GRUPO 4","1478":"GRUPO 4","1479":"GRUPO 4","1480":"GRUPO 4","1481":"GRUPO 4","1482":"GRUPO 4","1483":"GRUPO 4","1484":"GRUPO 4","1485":"GRUPO 4","1486":"GRUPO 4","1487":"GRUPO 4"},"Empleado":{"0":"BARON HERNANDEZ HAROLD ANTONIO","1":"CASTELLANOS CARVAJAL DEYVITH FABIAN","2":"AROCA TORRES JULIAN EDUARDO","3":"BERMUDEZ PARRA JENNIFER XIOMARA","4":"BERNAL BAQUERO JAMES RICARDO","5":"BURGOS ORTIZ JOSE HORACIO","6":"CANTOR PORRAS JUAN FERNEY","7":"CAPERA CAPERA JOSE GABRIEL","8":"CARDENAS LOTERO RICARDO ANDR\u00c9S","9":"RENDON OSPINA NELSON LEANDRO","10":"SARMIENTO URBINA MOISES DANIEL","11":"VELASCO VELASCO SEBASTI\u00c1N DAVID","12":"DELGADO DELGADO JOHAN DARIO","13":"FLOREZ SAUCESO KENIS ALBERTO","14":"CARDONA GARCIA OSCAR JAVIER","15":"CARVAJAL GARC\u00cdA HOVER MARCK","16":"CEPEDA PIRAQUIVE JUAN DAVID","17":"FAJARDO SAENZ OSCAR FERNANDO","18":"FLOREZ ESPITIA RONY ALBERTO","19":"GARCIA CUERVO EDWIN JAVIER","20":"GONZALEZ OCHOA JUAN CARLOS","21":"XXX1","22":"XXX2","23":"XXX3","24":"FONSECA RAY RICARDO","25":"GOMEZ BETANCUR JAIDER ANDRES","26":"GRANADA PATI\u00d1O CARLOS MARINO","27":"GRASS PLATA MIGUEL SNEIDER","28":"MANZANO CALVO JUAN SEBASTIAN","29":"MENDOZA GOITA MARIANSEL ZENAYDA","30":"MURILLO ARAQUE JAIVER GEOVANY","31":"NI\u00d1O ARENAS HECTOR GONZALO","32":"RAMIREZ CHAVERRA JHON EDISON","33":"XXX4","34":"XXX5","35":"XXX6","36":"RODRIGUEZ MOSQUERA LUIS FERNANDO","37":"PEPITO PEREZ","38":"RAMIREZ VARGAS MARCELA PAOLA","39":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","40":"TORO CISNEROS GARY JOSE","41":"USECHE CALDERON JADID ESTIVEN","42":"VASQUEZ NIETO CAMILO ANDRES","43":"JHONY CASTRO","44":"BERNAL JUAN DAVID","45":"XXX7","46":"XXX8","47":"XXX9","48":"BARON HERNANDEZ HAROLD ANTONIO","49":"CASTELLANOS CARVAJAL DEYVITH FABIAN","50":"AROCA TORRES JULIAN EDUARDO","51":"BERMUDEZ PARRA JENNIFER XIOMARA","52":"BERNAL BAQUERO JAMES RICARDO","53":"BURGOS ORTIZ JOSE HORACIO","54":"CANTOR PORRAS JUAN FERNEY","55":"CAPERA CAPERA JOSE GABRIEL","56":"CARDENAS LOTERO RICARDO ANDR\u00c9S","57":"RENDON OSPINA NELSON LEANDRO","58":"SARMIENTO URBINA MOISES DANIEL","59":"VELASCO VELASCO SEBASTI\u00c1N DAVID","60":"DELGADO DELGADO JOHAN DARIO","61":"FLOREZ SAUCESO KENIS ALBERTO","62":"CARDONA GARCIA OSCAR JAVIER","63":"CARVAJAL GARC\u00cdA HOVER MARCK","64":"CEPEDA PIRAQUIVE JUAN DAVID","65":"FAJARDO SAENZ OSCAR FERNANDO","66":"FLOREZ ESPITIA RONY ALBERTO","67":"GARCIA CUERVO EDWIN JAVIER","68":"GONZALEZ OCHOA JUAN CARLOS","69":"XXX1","70":"XXX2","71":"XXX3","72":"FONSECA RAY RICARDO","73":"GOMEZ BETANCUR JAIDER ANDRES","74":"GRANADA PATI\u00d1O CARLOS MARINO","75":"GRASS PLATA MIGUEL SNEIDER","76":"MANZANO CALVO JUAN SEBASTIAN","77":"MENDOZA GOITA MARIANSEL ZENAYDA","78":"MURILLO ARAQUE JAIVER GEOVANY","79":"NI\u00d1O ARENAS HECTOR GONZALO","80":"RAMIREZ CHAVERRA JHON EDISON","81":"XXX4","82":"XXX5","83":"XXX6","84":"RODRIGUEZ MOSQUERA LUIS FERNANDO","85":"PEPITO PEREZ","86":"RAMIREZ VARGAS MARCELA PAOLA","87":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","88":"TORO CISNEROS GARY JOSE","89":"USECHE CALDERON JADID ESTIVEN","90":"VASQUEZ NIETO CAMILO ANDRES","91":"JHONY CASTRO","92":"BERNAL JUAN DAVID","93":"XXX7","94":"XXX8","95":"XXX9","96":"BARON HERNANDEZ HAROLD ANTONIO","97":"CASTELLANOS CARVAJAL DEYVITH FABIAN","98":"AROCA TORRES JULIAN EDUARDO","99":"BERMUDEZ PARRA JENNIFER XIOMARA","100":"BERNAL BAQUERO JAMES RICARDO","101":"BURGOS ORTIZ JOSE HORACIO","102":"CANTOR PORRAS JUAN FERNEY","103":"CAPERA CAPERA JOSE GABRIEL","104":"CARDENAS LOTERO RICARDO ANDR\u00c9S","105":"RENDON OSPINA NELSON LEANDRO","106":"SARMIENTO URBINA MOISES DANIEL","107":"VELASCO VELASCO SEBASTI\u00c1N DAVID","108":"DELGADO DELGADO JOHAN DARIO","109":"FLOREZ SAUCESO KENIS ALBERTO","110":"CARDONA GARCIA OSCAR JAVIER","111":"CARVAJAL GARC\u00cdA HOVER MARCK","112":"CEPEDA PIRAQUIVE JUAN DAVID","113":"FAJARDO SAENZ OSCAR FERNANDO","114":"FLOREZ ESPITIA RONY ALBERTO","115":"GARCIA CUERVO EDWIN JAVIER","116":"GONZALEZ OCHOA JUAN CARLOS","117":"XXX1","118":"XXX2","119":"XXX3","120":"FONSECA RAY RICARDO","121":"GOMEZ BETANCUR JAIDER ANDRES","122":"GRANADA PATI\u00d1O CARLOS MARINO","123":"GRASS PLATA MIGUEL SNEIDER","124":"MANZANO CALVO JUAN SEBASTIAN","125":"MENDOZA GOITA MARIANSEL ZENAYDA","126":"MURILLO ARAQUE JAIVER GEOVANY","127":"NI\u00d1O ARENAS HECTOR GONZALO","128":"RAMIREZ CHAVERRA JHON EDISON","129":"XXX4","130":"XXX5","131":"XXX6","132":"RODRIGUEZ MOSQUERA LUIS FERNANDO","133":"PEPITO PEREZ","134":"RAMIREZ VARGAS MARCELA PAOLA","135":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","136":"TORO CISNEROS GARY JOSE","137":"USECHE CALDERON JADID ESTIVEN","138":"VASQUEZ NIETO CAMILO ANDRES","139":"JHONY CASTRO","140":"BERNAL JUAN DAVID","141":"XXX7","142":"XXX8","143":"XXX9","144":"BARON HERNANDEZ HAROLD ANTONIO","145":"CASTELLANOS CARVAJAL DEYVITH FABIAN","146":"AROCA TORRES JULIAN EDUARDO","147":"BERMUDEZ PARRA JENNIFER XIOMARA","148":"BERNAL BAQUERO JAMES RICARDO","149":"BURGOS ORTIZ JOSE HORACIO","150":"CANTOR PORRAS JUAN FERNEY","151":"CAPERA CAPERA JOSE GABRIEL","152":"CARDENAS LOTERO RICARDO ANDR\u00c9S","153":"RENDON OSPINA NELSON LEANDRO","154":"SARMIENTO URBINA MOISES DANIEL","155":"VELASCO VELASCO SEBASTI\u00c1N DAVID","156":"DELGADO DELGADO JOHAN DARIO","157":"FLOREZ SAUCESO KENIS ALBERTO","158":"CARDONA GARCIA OSCAR JAVIER","159":"CARVAJAL GARC\u00cdA HOVER MARCK","160":"CEPEDA PIRAQUIVE JUAN DAVID","161":"FAJARDO SAENZ OSCAR FERNANDO","162":"FLOREZ ESPITIA RONY ALBERTO","163":"GARCIA CUERVO EDWIN JAVIER","164":"GONZALEZ OCHOA JUAN CARLOS","165":"XXX1","166":"XXX2","167":"XXX3","168":"FONSECA RAY RICARDO","169":"GOMEZ BETANCUR JAIDER ANDRES","170":"GRANADA PATI\u00d1O CARLOS MARINO","171":"GRASS PLATA MIGUEL SNEIDER","172":"MANZANO CALVO JUAN SEBASTIAN","173":"MENDOZA GOITA MARIANSEL ZENAYDA","174":"MURILLO ARAQUE JAIVER GEOVANY","175":"NI\u00d1O ARENAS HECTOR GONZALO","176":"RAMIREZ CHAVERRA JHON EDISON","177":"XXX4","178":"XXX5","179":"XXX6","180":"RODRIGUEZ MOSQUERA LUIS FERNANDO","181":"PEPITO PEREZ","182":"RAMIREZ VARGAS MARCELA PAOLA","183":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","184":"TORO CISNEROS GARY JOSE","185":"USECHE CALDERON JADID ESTIVEN","186":"VASQUEZ NIETO CAMILO ANDRES","187":"JHONY CASTRO","188":"BERNAL JUAN DAVID","189":"XXX7","190":"XXX8","191":"XXX9","192":"BARON HERNANDEZ HAROLD ANTONIO","193":"CASTELLANOS CARVAJAL DEYVITH FABIAN","194":"AROCA TORRES JULIAN EDUARDO","195":"BERMUDEZ PARRA JENNIFER XIOMARA","196":"BERNAL BAQUERO JAMES RICARDO","197":"BURGOS ORTIZ JOSE HORACIO","198":"CANTOR PORRAS JUAN FERNEY","199":"CAPERA CAPERA JOSE GABRIEL","200":"CARDENAS LOTERO RICARDO ANDR\u00c9S","201":"RENDON OSPINA NELSON LEANDRO","202":"SARMIENTO URBINA MOISES DANIEL","203":"VELASCO VELASCO SEBASTI\u00c1N DAVID","204":"DELGADO DELGADO JOHAN DARIO","205":"FLOREZ SAUCESO KENIS ALBERTO","206":"CARDONA GARCIA OSCAR JAVIER","207":"CARVAJAL GARC\u00cdA HOVER MARCK","208":"CEPEDA PIRAQUIVE JUAN DAVID","209":"FAJARDO SAENZ OSCAR FERNANDO","210":"FLOREZ ESPITIA RONY ALBERTO","211":"GARCIA CUERVO EDWIN JAVIER","212":"GONZALEZ OCHOA JUAN CARLOS","213":"XXX1","214":"XXX2","215":"XXX3","216":"FONSECA RAY RICARDO","217":"GOMEZ BETANCUR JAIDER ANDRES","218":"GRANADA PATI\u00d1O CARLOS MARINO","219":"GRASS PLATA MIGUEL SNEIDER","220":"MANZANO CALVO JUAN SEBASTIAN","221":"MENDOZA GOITA MARIANSEL ZENAYDA","222":"MURILLO ARAQUE JAIVER GEOVANY","223":"NI\u00d1O ARENAS HECTOR GONZALO","224":"RAMIREZ CHAVERRA JHON EDISON","225":"XXX4","226":"XXX5","227":"XXX6","228":"RODRIGUEZ MOSQUERA LUIS FERNANDO","229":"PEPITO PEREZ","230":"RAMIREZ VARGAS MARCELA PAOLA","231":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","232":"TORO CISNEROS GARY JOSE","233":"USECHE CALDERON JADID ESTIVEN","234":"VASQUEZ NIETO CAMILO ANDRES","235":"JHONY CASTRO","236":"BERNAL JUAN DAVID","237":"XXX7","238":"XXX8","239":"XXX9","240":"BARON HERNANDEZ HAROLD ANTONIO","241":"CASTELLANOS CARVAJAL DEYVITH FABIAN","242":"AROCA TORRES JULIAN EDUARDO","243":"BERMUDEZ PARRA JENNIFER XIOMARA","244":"BERNAL BAQUERO JAMES RICARDO","245":"BURGOS ORTIZ JOSE HORACIO","246":"CANTOR PORRAS JUAN FERNEY","247":"CAPERA CAPERA JOSE GABRIEL","248":"CARDENAS LOTERO RICARDO ANDR\u00c9S","249":"RENDON OSPINA NELSON LEANDRO","250":"SARMIENTO URBINA MOISES DANIEL","251":"VELASCO VELASCO SEBASTI\u00c1N DAVID","252":"DELGADO DELGADO JOHAN DARIO","253":"FLOREZ SAUCESO KENIS ALBERTO","254":"CARDONA GARCIA OSCAR JAVIER","255":"CARVAJAL GARC\u00cdA HOVER MARCK","256":"CEPEDA PIRAQUIVE JUAN DAVID","257":"FAJARDO SAENZ OSCAR FERNANDO","258":"FLOREZ ESPITIA RONY ALBERTO","259":"GARCIA CUERVO EDWIN JAVIER","260":"GONZALEZ OCHOA JUAN CARLOS","261":"XXX1","262":"XXX2","263":"XXX3","264":"FONSECA RAY RICARDO","265":"GOMEZ BETANCUR JAIDER ANDRES","266":"GRANADA PATI\u00d1O CARLOS MARINO","267":"GR</t>
@@ -65,6 +65,9 @@
   </si>
   <si>
     <t>[{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"01-Mie","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"01-Mie","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"01-Mie","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"01-Mie","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"01-Mie","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"01-Mie","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"01-Mie","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"01-Mie","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"01-Mie","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"01-Mie","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"01-Mie","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"01-Mie","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"06-Lun","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"06-Lun","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"06-Lun","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"06-Lun","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"06-Lun","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"06-Lun","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"06-Lun","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"06-Lun","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"06-Lun","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"06-Lun","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"06-Lun","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"06-Lun","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VA</t>
+  </si>
+  <si>
+    <t>[{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master</t>
   </si>
 </sst>
 </file>
@@ -481,7 +484,7 @@
         <v>13</v>
       </c>
       <c r="E5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update historico_mallas.xlsx 2026-04-24 18:28:09.055025
</commit_message>
<xml_diff>
--- a/historico_mallas.xlsx
+++ b/historico_mallas.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
   <si>
     <t>Mes</t>
   </si>
@@ -43,6 +43,9 @@
     <t>Julio</t>
   </si>
   <si>
+    <t>Agosto</t>
+  </si>
+  <si>
     <t>Técnica</t>
   </si>
   <si>
@@ -58,6 +61,9 @@
     <t>2026-04-24 18:27</t>
   </si>
   <si>
+    <t>2026-04-24 18:28</t>
+  </si>
+  <si>
     <t>{"Grupo":{"0":"GRUPO 1","1":"GRUPO 1","2":"GRUPO 1","3":"GRUPO 1","4":"GRUPO 1","5":"GRUPO 1","6":"GRUPO 1","7":"GRUPO 1","8":"GRUPO 1","9":"GRUPO 1","10":"GRUPO 1","11":"GRUPO 1","12":"GRUPO 2","13":"GRUPO 2","14":"GRUPO 2","15":"GRUPO 2","16":"GRUPO 2","17":"GRUPO 2","18":"GRUPO 2","19":"GRUPO 2","20":"GRUPO 2","21":"GRUPO 2","22":"GRUPO 2","23":"GRUPO 2","24":"GRUPO 3","25":"GRUPO 3","26":"GRUPO 3","27":"GRUPO 3","28":"GRUPO 3","29":"GRUPO 3","30":"GRUPO 3","31":"GRUPO 3","32":"GRUPO 3","33":"GRUPO 3","34":"GRUPO 3","35":"GRUPO 3","36":"GRUPO 4","37":"GRUPO 4","38":"GRUPO 4","39":"GRUPO 4","40":"GRUPO 4","41":"GRUPO 4","42":"GRUPO 4","43":"GRUPO 4","44":"GRUPO 4","45":"GRUPO 4","46":"GRUPO 4","47":"GRUPO 4","48":"GRUPO 1","49":"GRUPO 1","50":"GRUPO 1","51":"GRUPO 1","52":"GRUPO 1","53":"GRUPO 1","54":"GRUPO 1","55":"GRUPO 1","56":"GRUPO 1","57":"GRUPO 1","58":"GRUPO 1","59":"GRUPO 1","60":"GRUPO 2","61":"GRUPO 2","62":"GRUPO 2","63":"GRUPO 2","64":"GRUPO 2","65":"GRUPO 2","66":"GRUPO 2","67":"GRUPO 2","68":"GRUPO 2","69":"GRUPO 2","70":"GRUPO 2","71":"GRUPO 2","72":"GRUPO 3","73":"GRUPO 3","74":"GRUPO 3","75":"GRUPO 3","76":"GRUPO 3","77":"GRUPO 3","78":"GRUPO 3","79":"GRUPO 3","80":"GRUPO 3","81":"GRUPO 3","82":"GRUPO 3","83":"GRUPO 3","84":"GRUPO 4","85":"GRUPO 4","86":"GRUPO 4","87":"GRUPO 4","88":"GRUPO 4","89":"GRUPO 4","90":"GRUPO 4","91":"GRUPO 4","92":"GRUPO 4","93":"GRUPO 4","94":"GRUPO 4","95":"GRUPO 4","96":"GRUPO 1","97":"GRUPO 1","98":"GRUPO 1","99":"GRUPO 1","100":"GRUPO 1","101":"GRUPO 1","102":"GRUPO 1","103":"GRUPO 1","104":"GRUPO 1","105":"GRUPO 1","106":"GRUPO 1","107":"GRUPO 1","108":"GRUPO 2","109":"GRUPO 2","110":"GRUPO 2","111":"GRUPO 2","112":"GRUPO 2","113":"GRUPO 2","114":"GRUPO 2","115":"GRUPO 2","116":"GRUPO 2","117":"GRUPO 2","118":"GRUPO 2","119":"GRUPO 2","120":"GRUPO 3","121":"GRUPO 3","122":"GRUPO 3","123":"GRUPO 3","124":"GRUPO 3","125":"GRUPO 3","126":"GRUPO 3","127":"GRUPO 3","128":"GRUPO 3","129":"GRUPO 3","130":"GRUPO 3","131":"GRUPO 3","132":"GRUPO 4","133":"GRUPO 4","134":"GRUPO 4","135":"GRUPO 4","136":"GRUPO 4","137":"GRUPO 4","138":"GRUPO 4","139":"GRUPO 4","140":"GRUPO 4","141":"GRUPO 4","142":"GRUPO 4","143":"GRUPO 4","144":"GRUPO 1","145":"GRUPO 1","146":"GRUPO 1","147":"GRUPO 1","148":"GRUPO 1","149":"GRUPO 1","150":"GRUPO 1","151":"GRUPO 1","152":"GRUPO 1","153":"GRUPO 1","154":"GRUPO 1","155":"GRUPO 1","156":"GRUPO 2","157":"GRUPO 2","158":"GRUPO 2","159":"GRUPO 2","160":"GRUPO 2","161":"GRUPO 2","162":"GRUPO 2","163":"GRUPO 2","164":"GRUPO 2","165":"GRUPO 2","166":"GRUPO 2","167":"GRUPO 2","168":"GRUPO 3","169":"GRUPO 3","170":"GRUPO 3","171":"GRUPO 3","172":"GRUPO 3","173":"GRUPO 3","174":"GRUPO 3","175":"GRUPO 3","176":"GRUPO 3","177":"GRUPO 3","178":"GRUPO 3","179":"GRUPO 3","180":"GRUPO 4","181":"GRUPO 4","182":"GRUPO 4","183":"GRUPO 4","184":"GRUPO 4","185":"GRUPO 4","186":"GRUPO 4","187":"GRUPO 4","188":"GRUPO 4","189":"GRUPO 4","190":"GRUPO 4","191":"GRUPO 4","192":"GRUPO 1","193":"GRUPO 1","194":"GRUPO 1","195":"GRUPO 1","196":"GRUPO 1","197":"GRUPO 1","198":"GRUPO 1","199":"GRUPO 1","200":"GRUPO 1","201":"GRUPO 1","202":"GRUPO 1","203":"GRUPO 1","204":"GRUPO 2","205":"GRUPO 2","206":"GRUPO 2","207":"GRUPO 2","208":"GRUPO 2","209":"GRUPO 2","210":"GRUPO 2","211":"GRUPO 2","212":"GRUPO 2","213":"GRUPO 2","214":"GRUPO 2","215":"GRUPO 2","216":"GRUPO 3","217":"GRUPO 3","218":"GRUPO 3","219":"GRUPO 3","220":"GRUPO 3","221":"GRUPO 3","222":"GRUPO 3","223":"GRUPO 3","224":"GRUPO 3","225":"GRUPO 3","226":"GRUPO 3","227":"GRUPO 3","228":"GRUPO 4","229":"GRUPO 4","230":"GRUPO 4","231":"GRUPO 4","232":"GRUPO 4","233":"GRUPO 4","234":"GRUPO 4","235":"GRUPO 4","236":"GRUPO 4","237":"GRUPO 4","238":"GRUPO 4","239":"GRUPO 4","240":"GRUPO 1","241":"GRUPO 1","242":"GRUPO 1","243":"GRUPO 1","244":"GRUPO 1","245":"GRUPO 1","246":"GRUPO 1","247":"GRUPO 1","248":"GRUPO 1","249":"GRUPO 1","250":"GRUPO 1","251":"GRUPO 1","252":"GRUPO 2","253":"GRUPO 2","254":"GRUPO 2","255":"GRUPO 2","256":"GRUPO 2","257":"GRUPO 2","258":"GRUPO 2","259":"GRUPO 2","260":"GRUPO 2","261":"GRUPO 2","262":"GRUPO 2","263":"GRUPO 2","264":"GRUPO 3","265":"GRUPO 3","266":"GRUPO 3","267":"GRUPO 3","268":"GRUPO 3","269":"GRUPO 3","270":"GRUPO 3","271":"GRUPO 3","272":"GRUPO 3","273":"GRUPO 3","274":"GRUPO 3","275":"GRUPO 3","276":"GRUPO 4","277":"GRUPO 4","278":"GRUPO 4","279":"GRUPO 4","280":"GRUPO 4","281":"GRUPO 4","282":"GRUPO 4","283":"GRUPO 4","284":"GRUPO 4","285":"GRUPO 4","286":"GRUPO 4","287":"GRUPO 4","288":"GRUPO 1","289":"GRUPO 1","290":"GRUPO 1","291":"GRUPO 1","292":"GRUPO 1","293":"GRUPO 1","294":"GRUPO 1","295":"GRUPO 1","296":"GRUPO 1","297":"GRUPO 1","298":"GRUPO 1","299":"GRUPO 1","300":"GRUPO 2","301":"GRUPO 2","302":"GRUPO 2","303":"GRUPO 2","304":"GRUPO 2","305":"GRUPO 2","306":"GRUPO 2","307":"GRUPO 2","308":"GRUPO 2","309":"GRUPO 2","310":"GRUPO 2","311":"GRUPO 2","312":"GRUPO 3","313":"GRUPO 3","314":"GRUPO 3","315":"GRUPO 3","316":"GRUPO 3","317":"GRUPO 3","318":"GRUPO 3","319":"GRUPO 3","320":"GRUPO 3","321":"GRUPO 3","322":"GRUPO 3","323":"GRUPO 3","324":"GRUPO 4","325":"GRUPO 4","326":"GRUPO 4","327":"GRUPO 4","328":"GRUPO 4","329":"GRUPO 4","330":"GRUPO 4","331":"GRUPO 4","332":"GRUPO 4","333":"GRUPO 4","334":"GRUPO 4","335":"GRUPO 4","336":"GRUPO 1","337":"GRUPO 1","338":"GRUPO 1","339":"GRUPO 1","340":"GRUPO 1","341":"GRUPO 1","342":"GRUPO 1","343":"GRUPO 1","344":"GRUPO 1","345":"GRUPO 1","346":"GRUPO 1","347":"GRUPO 1","348":"GRUPO 2","349":"GRUPO 2","350":"GRUPO 2","351":"GRUPO 2","352":"GRUPO 2","353":"GRUPO 2","354":"GRUPO 2","355":"GRUPO 2","356":"GRUPO 2","357":"GRUPO 2","358":"GRUPO 2","359":"GRUPO 2","360":"GRUPO 3","361":"GRUPO 3","362":"GRUPO 3","363":"GRUPO 3","364":"GRUPO 3","365":"GRUPO 3","366":"GRUPO 3","367":"GRUPO 3","368":"GRUPO 3","369":"GRUPO 3","370":"GRUPO 3","371":"GRUPO 3","372":"GRUPO 4","373":"GRUPO 4","374":"GRUPO 4","375":"GRUPO 4","376":"GRUPO 4","377":"GRUPO 4","378":"GRUPO 4","379":"GRUPO 4","380":"GRUPO 4","381":"GRUPO 4","382":"GRUPO 4","383":"GRUPO 4","384":"GRUPO 1","385":"GRUPO 1","386":"GRUPO 1","387":"GRUPO 1","388":"GRUPO 1","389":"GRUPO 1","390":"GRUPO 1","391":"GRUPO 1","392":"GRUPO 1","393":"GRUPO 1","394":"GRUPO 1","395":"GRUPO 1","396":"GRUPO 2","397":"GRUPO 2","398":"GRUPO 2","399":"GRUPO 2","400":"GRUPO 2","401":"GRUPO 2","402":"GRUPO 2","403":"GRUPO 2","404":"GRUPO 2","405":"GRUPO 2","406":"GRUPO 2","407":"GRUPO 2","408":"GRUPO 3","409":"GRUPO 3","410":"GRUPO 3","411":"GRUPO 3","412":"GRUPO 3","413":"GRUPO 3","414":"GRUPO 3","415":"GRUPO 3","416":"GRUPO 3","417":"GRUPO 3","418":"GRUPO 3","419":"GRUPO 3","420":"GRUPO 4","421":"GRUPO 4","422":"GRUPO 4","423":"GRUPO 4","424":"GRUPO 4","425":"GRUPO 4","426":"GRUPO 4","427":"GRUPO 4","428":"GRUPO 4","429":"GRUPO 4","430":"GRUPO 4","431":"GRUPO 4","432":"GRUPO 1","433":"GRUPO 1","434":"GRUPO 1","435":"GRUPO 1","436":"GRUPO 1","437":"GRUPO 1","438":"GRUPO 1","439":"GRUPO 1","440":"GRUPO 1","441":"GRUPO 1","442":"GRUPO 1","443":"GRUPO 1","444":"GRUPO 2","445":"GRUPO 2","446":"GRUPO 2","447":"GRUPO 2","448":"GRUPO 2","449":"GRUPO 2","450":"GRUPO 2","451":"GRUPO 2","452":"GRUPO 2","453":"GRUPO 2","454":"GRUPO 2","455":"GRUPO 2","456":"GRUPO 3","457":"GRUPO 3","458":"GRUPO 3","459":"GRUPO 3","460":"GRUPO 3","461":"GRUPO 3","462":"GRUPO 3","463":"GRUPO 3","464":"GRUPO 3","465":"GRUPO 3","466":"GRUPO 3","467":"GRUPO 3","468":"GRUPO 4","469":"GRUPO 4","470":"GRUPO 4","471":"GRUPO 4","472":"GRUPO 4","473":"GRUPO 4","474":"GRUPO 4","475":"GRUPO 4","476":"GRUPO 4","477":"GRUPO 4","478":"GRUPO 4","479":"GRUPO 4","480":"GRUPO 1","481":"GRUPO 1","482":"GRUPO 1","483":"GRUPO 1","484":"GRUPO 1","485":"GRUPO 1","486":"GRUPO 1","487":"GRUPO 1","488":"GRUPO 1","489":"GRUPO 1","490":"GRUPO 1","491":"GRUPO 1","492":"GRUPO 2","493":"GRUPO 2","494":"GRUPO 2","495":"GRUPO 2","496":"GRUPO 2","497":"GRUPO 2","498":"GRUPO 2","499":"GRUPO 2","500":"GRUPO 2","501":"GRUPO 2","502":"GRUPO 2","503":"GRUPO 2","504":"GRUPO 3","505":"GRUPO 3","506":"GRUPO 3","507":"GRUPO 3","508":"GRUPO 3","509":"GRUPO 3","510":"GRUPO 3","511":"GRUPO 3","512":"GRUPO 3","513":"GRUPO 3","514":"GRUPO 3","515":"GRUPO 3","516":"GRUPO 4","517":"GRUPO 4","518":"GRUPO 4","519":"GRUPO 4","520":"GRUPO 4","521":"GRUPO 4","522":"GRUPO 4","523":"GRUPO 4","524":"GRUPO 4","525":"GRUPO 4","526":"GRUPO 4","527":"GRUPO 4","528":"GRUPO 1","529":"GRUPO 1","530":"GRUPO 1","531":"GRUPO 1","532":"GRUPO 1","533":"GRUPO 1","534":"GRUPO 1","535":"GRUPO 1","536":"GRUPO 1","537":"GRUPO 1","538":"GRUPO 1","539":"GRUPO 1","540":"GRUPO 2","541":"GRUPO 2","542":"GRUPO 2","543":"GRUPO 2","544":"GRUPO 2","545":"GRUPO 2","546":"GRUPO 2","547":"GRUPO 2","548":"GRUPO 2","549":"GRUPO 2","550":"GRUPO 2","551":"GRUPO 2","552":"GRUPO 3","553":"GRUPO 3","554":"GRUPO 3","555":"GRUPO 3","556":"GRUPO 3","557":"GRUPO 3","558":"GRUPO 3","559":"GRUPO 3","560":"GRUPO 3","561":"GRUPO 3","562":"GRUPO 3","563":"GRUPO 3","564":"GRUPO 4","565":"GRUPO 4","566":"GRUPO 4","567":"GRUPO 4","568":"GRUPO 4","569":"GRUPO 4","570":"GRUPO 4","571":"GRUPO 4","572":"GRUPO 4","573":"GRUPO 4","574":"GRUPO 4","575":"GRUPO 4","576":"GRUPO 1","577":"GRUPO 1","578":"GRUPO 1","579":"GRUPO 1","580":"GRUPO 1","581":"GRUPO 1","582":"GRUPO 1","583":"GRUPO 1","584":"GRUPO 1","585":"GRUPO 1","586":"GRUPO 1","587":"GRUPO 1","588":"GRUPO 2","589":"GRUPO 2","590":"GRUPO 2","591":"GRUPO 2","592":"GRUPO 2","593":"GRUPO 2","594":"GRUPO 2","595":"GRUPO 2","596":"GRUPO 2","597":"GRUPO 2","598":"GRUPO 2","599":"GRUPO 2","600":"GRUPO 3","601":"GRUPO 3","602":"GRUPO 3","603":"GRUPO 3","604":"GRUPO 3","605":"GRUPO 3","606":"GRUPO 3","607":"GRUPO 3","608":"GRUPO 3","609":"GRUPO 3","610":"GRUPO 3","611":"GRUPO 3","612":"GRUPO 4","613":"GRUPO 4","614":"GRUPO 4","615":"GRUPO 4","616":"GRUPO 4","617":"GRUPO 4","618":"GRUPO 4","619":"GRUPO 4","620":"GRUPO 4","621":"GRUPO 4","622":"GRUPO 4","623":"GRUPO 4","624":"GRUPO 1","625":"GRUPO 1","626":"GRUPO 1","627":"GRUPO 1","628":"GRUPO 1","629":"GRUPO 1","630":"GRUPO 1","631":"GRUPO 1","632":"GRUPO 1","633":"GRUPO 1","634":"GRUPO 1","635":"GRUPO 1","636":"GRUPO 2","637":"GRUPO 2","638":"GRUPO 2","639":"GRUPO 2","640":"GRUPO 2","641":"GRUPO 2","642":"GRUPO 2","643":"GRUPO 2","644":"GRUPO 2","645":"GRUPO 2","646":"GRUPO 2","647":"GRUPO 2","648":"GRUPO 3","649":"GRUPO 3","650":"GRUPO 3","651":"GRUPO 3","652":"GRUPO 3","653":"GRUPO 3","654":"GRUPO 3","655":"GRUPO 3","656":"GRUPO 3","657":"GRUPO 3","658":"GRUPO 3","659":"GRUPO 3","660":"GRUPO 4","661":"GRUPO 4","662":"GRUPO 4","663":"GRUPO 4","664":"GRUPO 4","665":"GRUPO 4","666":"GRUPO 4","667":"GRUPO 4","668":"GRUPO 4","669":"GRUPO 4","670":"GRUPO 4","671":"GRUPO 4","672":"GRUPO 1","673":"GRUPO 1","674":"GRUPO 1","675":"GRUPO 1","676":"GRUPO 1","677":"GRUPO 1","678":"GRUPO 1","679":"GRUPO 1","680":"GRUPO 1","681":"GRUPO 1","682":"GRUPO 1","683":"GRUPO 1","684":"GRUPO 2","685":"GRUPO 2","686":"GRUPO 2","687":"GRUPO 2","688":"GRUPO 2","689":"GRUPO 2","690":"GRUPO 2","691":"GRUPO 2","692":"GRUPO 2","693":"GRUPO 2","694":"GRUPO 2","695":"GRUPO 2","696":"GRUPO 3","697":"GRUPO 3","698":"GRUPO 3","699":"GRUPO 3","700":"GRUPO 3","701":"GRUPO 3","702":"GRUPO 3","703":"GRUPO 3","704":"GRUPO 3","705":"GRUPO 3","706":"GRUPO 3","707":"GRUPO 3","708":"GRUPO 4","709":"GRUPO 4","710":"GRUPO 4","711":"GRUPO 4","712":"GRUPO 4","713":"GRUPO 4","714":"GRUPO 4","715":"GRUPO 4","716":"GRUPO 4","717":"GRUPO 4","718":"GRUPO 4","719":"GRUPO 4","720":"GRUPO 1","721":"GRUPO 1","722":"GRUPO 1","723":"GRUPO 1","724":"GRUPO 1","725":"GRUPO 1","726":"GRUPO 1","727":"GRUPO 1","728":"GRUPO 1","729":"GRUPO 1","730":"GRUPO 1","731":"GRUPO 1","732":"GRUPO 2","733":"GRUPO 2","734":"GRUPO 2","735":"GRUPO 2","736":"GRUPO 2","737":"GRUPO 2","738":"GRUPO 2","739":"GRUPO 2","740":"GRUPO 2","741":"GRUPO 2","742":"GRUPO 2","743":"GRUPO 2","744":"GRUPO 3","745":"GRUPO 3","746":"GRUPO 3","747":"GRUPO 3","748":"GRUPO 3","749":"GRUPO 3","750":"GRUPO 3","751":"GRUPO 3","752":"GRUPO 3","753":"GRUPO 3","754":"GRUPO 3","755":"GRUPO 3","756":"GRUPO 4","757":"GRUPO 4","758":"GRUPO 4","759":"GRUPO 4","760":"GRUPO 4","761":"GRUPO 4","762":"GRUPO 4","763":"GRUPO 4","764":"GRUPO 4","765":"GRUPO 4","766":"GRUPO 4","767":"GRUPO 4","768":"GRUPO 1","769":"GRUPO 1","770":"GRUPO 1","771":"GRUPO 1","772":"GRUPO 1","773":"GRUPO 1","774":"GRUPO 1","775":"GRUPO 1","776":"GRUPO 1","777":"GRUPO 1","778":"GRUPO 1","779":"GRUPO 1","780":"GRUPO 2","781":"GRUPO 2","782":"GRUPO 2","783":"GRUPO 2","784":"GRUPO 2","785":"GRUPO 2","786":"GRUPO 2","787":"GRUPO 2","788":"GRUPO 2","789":"GRUPO 2","790":"GRUPO 2","791":"GRUPO 2","792":"GRUPO 3","793":"GRUPO 3","794":"GRUPO 3","795":"GRUPO 3","796":"GRUPO 3","797":"GRUPO 3","798":"GRUPO 3","799":"GRUPO 3","800":"GRUPO 3","801":"GRUPO 3","802":"GRUPO 3","803":"GRUPO 3","804":"GRUPO 4","805":"GRUPO 4","806":"GRUPO 4","807":"GRUPO 4","808":"GRUPO 4","809":"GRUPO 4","810":"GRUPO 4","811":"GRUPO 4","812":"GRUPO 4","813":"GRUPO 4","814":"GRUPO 4","815":"GRUPO 4","816":"GRUPO 1","817":"GRUPO 1","818":"GRUPO 1","819":"GRUPO 1","820":"GRUPO 1","821":"GRUPO 1","822":"GRUPO 1","823":"GRUPO 1","824":"GRUPO 1","825":"GRUPO 1","826":"GRUPO 1","827":"GRUPO 1","828":"GRUPO 2","829":"GRUPO 2","830":"GRUPO 2","831":"GRUPO 2","832":"GRUPO 2","833":"GRUPO 2","834":"GRUPO 2","835":"GRUPO 2","836":"GRUPO 2","837":"GRUPO 2","838":"GRUPO 2","839":"GRUPO 2","840":"GRUPO 3","841":"GRUPO 3","842":"GRUPO 3","843":"GRUPO 3","844":"GRUPO 3","845":"GRUPO 3","846":"GRUPO 3","847":"GRUPO 3","848":"GRUPO 3","849":"GRUPO 3","850":"GRUPO 3","851":"GRUPO 3","852":"GRUPO 4","853":"GRUPO 4","854":"GRUPO 4","855":"GRUPO 4","856":"GRUPO 4","857":"GRUPO 4","858":"GRUPO 4","859":"GRUPO 4","860":"GRUPO 4","861":"GRUPO 4","862":"GRUPO 4","863":"GRUPO 4","864":"GRUPO 1","865":"GRUPO 1","866":"GRUPO 1","867":"GRUPO 1","868":"GRUPO 1","869":"GRUPO 1","870":"GRUPO 1","871":"GRUPO 1","872":"GRUPO 1","873":"GRUPO 1","874":"GRUPO 1","875":"GRUPO 1","876":"GRUPO 2","877":"GRUPO 2","878":"GRUPO 2","879":"GRUPO 2","880":"GRUPO 2","881":"GRUPO 2","882":"GRUPO 2","883":"GRUPO 2","884":"GRUPO 2","885":"GRUPO 2","886":"GRUPO 2","887":"GRUPO 2","888":"GRUPO 3","889":"GRUPO 3","890":"GRUPO 3","891":"GRUPO 3","892":"GRUPO 3","893":"GRUPO 3","894":"GRUPO 3","895":"GRUPO 3","896":"GRUPO 3","897":"GRUPO 3","898":"GRUPO 3","899":"GRUPO 3","900":"GRUPO 4","901":"GRUPO 4","902":"GRUPO 4","903":"GRUPO 4","904":"GRUPO 4","905":"GRUPO 4","906":"GRUPO 4","907":"GRUPO 4","908":"GRUPO 4","909":"GRUPO 4","910":"GRUPO 4","911":"GRUPO 4","912":"GRUPO 1","913":"GRUPO 1","914":"GRUPO 1","915":"GRUPO 1","916":"GRUPO 1","917":"GRUPO 1","918":"GRUPO 1","919":"GRUPO 1","920":"GRUPO 1","921":"GRUPO 1","922":"GRUPO 1","923":"GRUPO 1","924":"GRUPO 2","925":"GRUPO 2","926":"GRUPO 2","927":"GRUPO 2","928":"GRUPO 2","929":"GRUPO 2","930":"GRUPO 2","931":"GRUPO 2","932":"GRUPO 2","933":"GRUPO 2","934":"GRUPO 2","935":"GRUPO 2","936":"GRUPO 3","937":"GRUPO 3","938":"GRUPO 3","939":"GRUPO 3","940":"GRUPO 3","941":"GRUPO 3","942":"GRUPO 3","943":"GRUPO 3","944":"GRUPO 3","945":"GRUPO 3","946":"GRUPO 3","947":"GRUPO 3","948":"GRUPO 4","949":"GRUPO 4","950":"GRUPO 4","951":"GRUPO 4","952":"GRUPO 4","953":"GRUPO 4","954":"GRUPO 4","955":"GRUPO 4","956":"GRUPO 4","957":"GRUPO 4","958":"GRUPO 4","959":"GRUPO 4","960":"GRUPO 1","961":"GRUPO 1","962":"GRUPO 1","963":"GRUPO 1","964":"GRUPO 1","965":"GRUPO 1","966":"GRUPO 1","967":"GRUPO 1","968":"GRUPO 1","969":"GRUPO 1","970":"GRUPO 1","971":"GRUPO 1","972":"GRUPO 2","973":"GRUPO 2","974":"GRUPO 2","975":"GRUPO 2","976":"GRUPO 2","977":"GRUPO 2","978":"GRUPO 2","979":"GRUPO 2","980":"GRUPO 2","981":"GRUPO 2","982":"GRUPO 2","983":"GRUPO 2","984":"GRUPO 3","985":"GRUPO 3","986":"GRUPO 3","987":"GRUPO 3","988":"GRUPO 3","989":"GRUPO 3","990":"GRUPO 3","991":"GRUPO 3","992":"GRUPO 3","993":"GRUPO 3","994":"GRUPO 3","995":"GRUPO 3","996":"GRUPO 4","997":"GRUPO 4","998":"GRUPO 4","999":"GRUPO 4","1000":"GRUPO 4","1001":"GRUPO 4","1002":"GRUPO 4","1003":"GRUPO 4","1004":"GRUPO 4","1005":"GRUPO 4","1006":"GRUPO 4","1007":"GRUPO 4","1008":"GRUPO 1","1009":"GRUPO 1","1010":"GRUPO 1","1011":"GRUPO 1","1012":"GRUPO 1","1013":"GRUPO 1","1014":"GRUPO 1","1015":"GRUPO 1","1016":"GRUPO 1","1017":"GRUPO 1","1018":"GRUPO 1","1019":"GRUPO 1","1020":"GRUPO 2","1021":"GRUPO 2","1022":"GRUPO 2","1023":"GRUPO 2","1024":"GRUPO 2","1025":"GRUPO 2","1026":"GRUPO 2","1027":"GRUPO 2","1028":"GRUPO 2","1029":"GRUPO 2","1030":"GRUPO 2","1031":"GRUPO 2","1032":"GRUPO 3","1033":"GRUPO 3","1034":"GRUPO 3","1035":"GRUPO 3","1036":"GRUPO 3","1037":"GRUPO 3","1038":"GRUPO 3","1039":"GRUPO 3","1040":"GRUPO 3","1041":"GRUPO 3","1042":"GRUPO 3","1043":"GRUPO 3","1044":"GRUPO 4","1045":"GRUPO 4","1046":"GRUPO 4","1047":"GRUPO 4","1048":"GRUPO 4","1049":"GRUPO 4","1050":"GRUPO 4","1051":"GRUPO 4","1052":"GRUPO 4","1053":"GRUPO 4","1054":"GRUPO 4","1055":"GRUPO 4","1056":"GRUPO 1","1057":"GRUPO 1","1058":"GRUPO 1","1059":"GRUPO 1","1060":"GRUPO 1","1061":"GRUPO 1","1062":"GRUPO 1","1063":"GRUPO 1","1064":"GRUPO 1","1065":"GRUPO 1","1066":"GRUPO 1","1067":"GRUPO 1","1068":"GRUPO 2","1069":"GRUPO 2","1070":"GRUPO 2","1071":"GRUPO 2","1072":"GRUPO 2","1073":"GRUPO 2","1074":"GRUPO 2","1075":"GRUPO 2","1076":"GRUPO 2","1077":"GRUPO 2","1078":"GRUPO 2","1079":"GRUPO 2","1080":"GRUPO 3","1081":"GRUPO 3","1082":"GRUPO 3","1083":"GRUPO 3","1084":"GRUPO 3","1085":"GRUPO 3","1086":"GRUPO 3","1087":"GRUPO 3","1088":"GRUPO 3","1089":"GRUPO 3","1090":"GRUPO 3","1091":"GRUPO 3","1092":"GRUPO 4","1093":"GRUPO 4","1094":"GRUPO 4","1095":"GRUPO 4","1096":"GRUPO 4","1097":"GRUPO 4","1098":"GRUPO 4","1099":"GRUPO 4","1100":"GRUPO 4","1101":"GRUPO 4","1102":"GRUPO 4","1103":"GRUPO 4","1104":"GRUPO 1","1105":"GRUPO 1","1106":"GRUPO 1","1107":"GRUPO 1","1108":"GRUPO 1","1109":"GRUPO 1","1110":"GRUPO 1","1111":"GRUPO 1","1112":"GRUPO 1","1113":"GRUPO 1","1114":"GRUPO 1","1115":"GRUPO 1","1116":"GRUPO 2","1117":"GRUPO 2","1118":"GRUPO 2","1119":"GRUPO 2","1120":"GRUPO 2","1121":"GRUPO 2","1122":"GRUPO 2","1123":"GRUPO 2","1124":"GRUPO 2","1125":"GRUPO 2","1126":"GRUPO 2","1127":"GRUPO 2","1128":"GRUPO 3","1129":"GRUPO 3","1130":"GRUPO 3","1131":"GRUPO 3","1132":"GRUPO 3","1133":"GRUPO 3","1134":"GRUPO 3","1135":"GRUPO 3","1136":"GRUPO 3","1137":"GRUPO 3","1138":"GRUPO 3","1139":"GRUPO 3","1140":"GRUPO 4","1141":"GRUPO 4","1142":"GRUPO 4","1143":"GRUPO 4","1144":"GRUPO 4","1145":"GRUPO 4","1146":"GRUPO 4","1147":"GRUPO 4","1148":"GRUPO 4","1149":"GRUPO 4","1150":"GRUPO 4","1151":"GRUPO 4","1152":"GRUPO 1","1153":"GRUPO 1","1154":"GRUPO 1","1155":"GRUPO 1","1156":"GRUPO 1","1157":"GRUPO 1","1158":"GRUPO 1","1159":"GRUPO 1","1160":"GRUPO 1","1161":"GRUPO 1","1162":"GRUPO 1","1163":"GRUPO 1","1164":"GRUPO 2","1165":"GRUPO 2","1166":"GRUPO 2","1167":"GRUPO 2","1168":"GRUPO 2","1169":"GRUPO 2","1170":"GRUPO 2","1171":"GRUPO 2","1172":"GRUPO 2","1173":"GRUPO 2","1174":"GRUPO 2","1175":"GRUPO 2","1176":"GRUPO 3","1177":"GRUPO 3","1178":"GRUPO 3","1179":"GRUPO 3","1180":"GRUPO 3","1181":"GRUPO 3","1182":"GRUPO 3","1183":"GRUPO 3","1184":"GRUPO 3","1185":"GRUPO 3","1186":"GRUPO 3","1187":"GRUPO 3","1188":"GRUPO 4","1189":"GRUPO 4","1190":"GRUPO 4","1191":"GRUPO 4","1192":"GRUPO 4","1193":"GRUPO 4","1194":"GRUPO 4","1195":"GRUPO 4","1196":"GRUPO 4","1197":"GRUPO 4","1198":"GRUPO 4","1199":"GRUPO 4","1200":"GRUPO 1","1201":"GRUPO 1","1202":"GRUPO 1","1203":"GRUPO 1","1204":"GRUPO 1","1205":"GRUPO 1","1206":"GRUPO 1","1207":"GRUPO 1","1208":"GRUPO 1","1209":"GRUPO 1","1210":"GRUPO 1","1211":"GRUPO 1","1212":"GRUPO 2","1213":"GRUPO 2","1214":"GRUPO 2","1215":"GRUPO 2","1216":"GRUPO 2","1217":"GRUPO 2","1218":"GRUPO 2","1219":"GRUPO 2","1220":"GRUPO 2","1221":"GRUPO 2","1222":"GRUPO 2","1223":"GRUPO 2","1224":"GRUPO 3","1225":"GRUPO 3","1226":"GRUPO 3","1227":"GRUPO 3","1228":"GRUPO 3","1229":"GRUPO 3","1230":"GRUPO 3","1231":"GRUPO 3","1232":"GRUPO 3","1233":"GRUPO 3","1234":"GRUPO 3","1235":"GRUPO 3","1236":"GRUPO 4","1237":"GRUPO 4","1238":"GRUPO 4","1239":"GRUPO 4","1240":"GRUPO 4","1241":"GRUPO 4","1242":"GRUPO 4","1243":"GRUPO 4","1244":"GRUPO 4","1245":"GRUPO 4","1246":"GRUPO 4","1247":"GRUPO 4","1248":"GRUPO 1","1249":"GRUPO 1","1250":"GRUPO 1","1251":"GRUPO 1","1252":"GRUPO 1","1253":"GRUPO 1","1254":"GRUPO 1","1255":"GRUPO 1","1256":"GRUPO 1","1257":"GRUPO 1","1258":"GRUPO 1","1259":"GRUPO 1","1260":"GRUPO 2","1261":"GRUPO 2","1262":"GRUPO 2","1263":"GRUPO 2","1264":"GRUPO 2","1265":"GRUPO 2","1266":"GRUPO 2","1267":"GRUPO 2","1268":"GRUPO 2","1269":"GRUPO 2","1270":"GRUPO 2","1271":"GRUPO 2","1272":"GRUPO 3","1273":"GRUPO 3","1274":"GRUPO 3","1275":"GRUPO 3","1276":"GRUPO 3","1277":"GRUPO 3","1278":"GRUPO 3","1279":"GRUPO 3","1280":"GRUPO 3","1281":"GRUPO 3","1282":"GRUPO 3","1283":"GRUPO 3","1284":"GRUPO 4","1285":"GRUPO 4","1286":"GRUPO 4","1287":"GRUPO 4","1288":"GRUPO 4","1289":"GRUPO 4","1290":"GRUPO 4","1291":"GRUPO 4","1292":"GRUPO 4","1293":"GRUPO 4","1294":"GRUPO 4","1295":"GRUPO 4","1296":"GRUPO 1","1297":"GRUPO 1","1298":"GRUPO 1","1299":"GRUPO 1","1300":"GRUPO 1","1301":"GRUPO 1","1302":"GRUPO 1","1303":"GRUPO 1","1304":"GRUPO 1","1305":"GRUPO 1","1306":"GRUPO 1","1307":"GRUPO 1","1308":"GRUPO 2","1309":"GRUPO 2","1310":"GRUPO 2","1311":"GRUPO 2","1312":"GRUPO 2","1313":"GRUPO 2","1314":"GRUPO 2","1315":"GRUPO 2","1316":"GRUPO 2","1317":"GRUPO 2","1318":"GRUPO 2","1319":"GRUPO 2","1320":"GRUPO 3","1321":"GRUPO 3","1322":"GRUPO 3","1323":"GRUPO 3","1324":"GRUPO 3","1325":"GRUPO 3","1326":"GRUPO 3","1327":"GRUPO 3","1328":"GRUPO 3","1329":"GRUPO 3","1330":"GRUPO 3","1331":"GRUPO 3","1332":"GRUPO 4","1333":"GRUPO 4","1334":"GRUPO 4","1335":"GRUPO 4","1336":"GRUPO 4","1337":"GRUPO 4","1338":"GRUPO 4","1339":"GRUPO 4","1340":"GRUPO 4","1341":"GRUPO 4","1342":"GRUPO 4","1343":"GRUPO 4","1344":"GRUPO 1","1345":"GRUPO 1","1346":"GRUPO 1","1347":"GRUPO 1","1348":"GRUPO 1","1349":"GRUPO 1","1350":"GRUPO 1","1351":"GRUPO 1","1352":"GRUPO 1","1353":"GRUPO 1","1354":"GRUPO 1","1355":"GRUPO 1","1356":"GRUPO 2","1357":"GRUPO 2","1358":"GRUPO 2","1359":"GRUPO 2","1360":"GRUPO 2","1361":"GRUPO 2","1362":"GRUPO 2","1363":"GRUPO 2","1364":"GRUPO 2","1365":"GRUPO 2","1366":"GRUPO 2","1367":"GRUPO 2","1368":"GRUPO 3","1369":"GRUPO 3","1370":"GRUPO 3","1371":"GRUPO 3","1372":"GRUPO 3","1373":"GRUPO 3","1374":"GRUPO 3","1375":"GRUPO 3","1376":"GRUPO 3","1377":"GRUPO 3","1378":"GRUPO 3","1379":"GRUPO 3","1380":"GRUPO 4","1381":"GRUPO 4","1382":"GRUPO 4","1383":"GRUPO 4","1384":"GRUPO 4","1385":"GRUPO 4","1386":"GRUPO 4","1387":"GRUPO 4","1388":"GRUPO 4","1389":"GRUPO 4","1390":"GRUPO 4","1391":"GRUPO 4","1392":"GRUPO 1","1393":"GRUPO 1","1394":"GRUPO 1","1395":"GRUPO 1","1396":"GRUPO 1","1397":"GRUPO 1","1398":"GRUPO 1","1399":"GRUPO 1","1400":"GRUPO 1","1401":"GRUPO 1","1402":"GRUPO 1","1403":"GRUPO 1","1404":"GRUPO 2","1405":"GRUPO 2","1406":"GRUPO 2","1407":"GRUPO 2","1408":"GRUPO 2","1409":"GRUPO 2","1410":"GRUPO 2","1411":"GRUPO 2","1412":"GRUPO 2","1413":"GRUPO 2","1414":"GRUPO 2","1415":"GRUPO 2","1416":"GRUPO 3","1417":"GRUPO 3","1418":"GRUPO 3","1419":"GRUPO 3","1420":"GRUPO 3","1421":"GRUPO 3","1422":"GRUPO 3","1423":"GRUPO 3","1424":"GRUPO 3","1425":"GRUPO 3","1426":"GRUPO 3","1427":"GRUPO 3","1428":"GRUPO 4","1429":"GRUPO 4","1430":"GRUPO 4","1431":"GRUPO 4","1432":"GRUPO 4","1433":"GRUPO 4","1434":"GRUPO 4","1435":"GRUPO 4","1436":"GRUPO 4","1437":"GRUPO 4","1438":"GRUPO 4","1439":"GRUPO 4","1440":"GRUPO 1","1441":"GRUPO 1","1442":"GRUPO 1","1443":"GRUPO 1","1444":"GRUPO 1","1445":"GRUPO 1","1446":"GRUPO 1","1447":"GRUPO 1","1448":"GRUPO 1","1449":"GRUPO 1","1450":"GRUPO 1","1451":"GRUPO 1","1452":"GRUPO 2","1453":"GRUPO 2","1454":"GRUPO 2","1455":"GRUPO 2","1456":"GRUPO 2","1457":"GRUPO 2","1458":"GRUPO 2","1459":"GRUPO 2","1460":"GRUPO 2","1461":"GRUPO 2","1462":"GRUPO 2","1463":"GRUPO 2","1464":"GRUPO 3","1465":"GRUPO 3","1466":"GRUPO 3","1467":"GRUPO 3","1468":"GRUPO 3","1469":"GRUPO 3","1470":"GRUPO 3","1471":"GRUPO 3","1472":"GRUPO 3","1473":"GRUPO 3","1474":"GRUPO 3","1475":"GRUPO 3","1476":"GRUPO 4","1477":"GRUPO 4","1478":"GRUPO 4","1479":"GRUPO 4","1480":"GRUPO 4","1481":"GRUPO 4","1482":"GRUPO 4","1483":"GRUPO 4","1484":"GRUPO 4","1485":"GRUPO 4","1486":"GRUPO 4","1487":"GRUPO 4"},"Empleado":{"0":"BARON HERNANDEZ HAROLD ANTONIO","1":"CASTELLANOS CARVAJAL DEYVITH FABIAN","2":"AROCA TORRES JULIAN EDUARDO","3":"BERMUDEZ PARRA JENNIFER XIOMARA","4":"BERNAL BAQUERO JAMES RICARDO","5":"BURGOS ORTIZ JOSE HORACIO","6":"CANTOR PORRAS JUAN FERNEY","7":"CAPERA CAPERA JOSE GABRIEL","8":"CARDENAS LOTERO RICARDO ANDR\u00c9S","9":"RENDON OSPINA NELSON LEANDRO","10":"SARMIENTO URBINA MOISES DANIEL","11":"VELASCO VELASCO SEBASTI\u00c1N DAVID","12":"DELGADO DELGADO JOHAN DARIO","13":"FLOREZ SAUCESO KENIS ALBERTO","14":"CARDONA GARCIA OSCAR JAVIER","15":"CARVAJAL GARC\u00cdA HOVER MARCK","16":"CEPEDA PIRAQUIVE JUAN DAVID","17":"FAJARDO SAENZ OSCAR FERNANDO","18":"FLOREZ ESPITIA RONY ALBERTO","19":"GARCIA CUERVO EDWIN JAVIER","20":"GONZALEZ OCHOA JUAN CARLOS","21":"XXX1","22":"XXX2","23":"XXX3","24":"FONSECA RAY RICARDO","25":"GOMEZ BETANCUR JAIDER ANDRES","26":"GRANADA PATI\u00d1O CARLOS MARINO","27":"GRASS PLATA MIGUEL SNEIDER","28":"MANZANO CALVO JUAN SEBASTIAN","29":"MENDOZA GOITA MARIANSEL ZENAYDA","30":"MURILLO ARAQUE JAIVER GEOVANY","31":"NI\u00d1O ARENAS HECTOR GONZALO","32":"RAMIREZ CHAVERRA JHON EDISON","33":"XXX4","34":"XXX5","35":"XXX6","36":"RODRIGUEZ MOSQUERA LUIS FERNANDO","37":"PEPITO PEREZ","38":"RAMIREZ VARGAS MARCELA PAOLA","39":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","40":"TORO CISNEROS GARY JOSE","41":"USECHE CALDERON JADID ESTIVEN","42":"VASQUEZ NIETO CAMILO ANDRES","43":"JHONY CASTRO","44":"BERNAL JUAN DAVID","45":"XXX7","46":"XXX8","47":"XXX9","48":"BARON HERNANDEZ HAROLD ANTONIO","49":"CASTELLANOS CARVAJAL DEYVITH FABIAN","50":"AROCA TORRES JULIAN EDUARDO","51":"BERMUDEZ PARRA JENNIFER XIOMARA","52":"BERNAL BAQUERO JAMES RICARDO","53":"BURGOS ORTIZ JOSE HORACIO","54":"CANTOR PORRAS JUAN FERNEY","55":"CAPERA CAPERA JOSE GABRIEL","56":"CARDENAS LOTERO RICARDO ANDR\u00c9S","57":"RENDON OSPINA NELSON LEANDRO","58":"SARMIENTO URBINA MOISES DANIEL","59":"VELASCO VELASCO SEBASTI\u00c1N DAVID","60":"DELGADO DELGADO JOHAN DARIO","61":"FLOREZ SAUCESO KENIS ALBERTO","62":"CARDONA GARCIA OSCAR JAVIER","63":"CARVAJAL GARC\u00cdA HOVER MARCK","64":"CEPEDA PIRAQUIVE JUAN DAVID","65":"FAJARDO SAENZ OSCAR FERNANDO","66":"FLOREZ ESPITIA RONY ALBERTO","67":"GARCIA CUERVO EDWIN JAVIER","68":"GONZALEZ OCHOA JUAN CARLOS","69":"XXX1","70":"XXX2","71":"XXX3","72":"FONSECA RAY RICARDO","73":"GOMEZ BETANCUR JAIDER ANDRES","74":"GRANADA PATI\u00d1O CARLOS MARINO","75":"GRASS PLATA MIGUEL SNEIDER","76":"MANZANO CALVO JUAN SEBASTIAN","77":"MENDOZA GOITA MARIANSEL ZENAYDA","78":"MURILLO ARAQUE JAIVER GEOVANY","79":"NI\u00d1O ARENAS HECTOR GONZALO","80":"RAMIREZ CHAVERRA JHON EDISON","81":"XXX4","82":"XXX5","83":"XXX6","84":"RODRIGUEZ MOSQUERA LUIS FERNANDO","85":"PEPITO PEREZ","86":"RAMIREZ VARGAS MARCELA PAOLA","87":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","88":"TORO CISNEROS GARY JOSE","89":"USECHE CALDERON JADID ESTIVEN","90":"VASQUEZ NIETO CAMILO ANDRES","91":"JHONY CASTRO","92":"BERNAL JUAN DAVID","93":"XXX7","94":"XXX8","95":"XXX9","96":"BARON HERNANDEZ HAROLD ANTONIO","97":"CASTELLANOS CARVAJAL DEYVITH FABIAN","98":"AROCA TORRES JULIAN EDUARDO","99":"BERMUDEZ PARRA JENNIFER XIOMARA","100":"BERNAL BAQUERO JAMES RICARDO","101":"BURGOS ORTIZ JOSE HORACIO","102":"CANTOR PORRAS JUAN FERNEY","103":"CAPERA CAPERA JOSE GABRIEL","104":"CARDENAS LOTERO RICARDO ANDR\u00c9S","105":"RENDON OSPINA NELSON LEANDRO","106":"SARMIENTO URBINA MOISES DANIEL","107":"VELASCO VELASCO SEBASTI\u00c1N DAVID","108":"DELGADO DELGADO JOHAN DARIO","109":"FLOREZ SAUCESO KENIS ALBERTO","110":"CARDONA GARCIA OSCAR JAVIER","111":"CARVAJAL GARC\u00cdA HOVER MARCK","112":"CEPEDA PIRAQUIVE JUAN DAVID","113":"FAJARDO SAENZ OSCAR FERNANDO","114":"FLOREZ ESPITIA RONY ALBERTO","115":"GARCIA CUERVO EDWIN JAVIER","116":"GONZALEZ OCHOA JUAN CARLOS","117":"XXX1","118":"XXX2","119":"XXX3","120":"FONSECA RAY RICARDO","121":"GOMEZ BETANCUR JAIDER ANDRES","122":"GRANADA PATI\u00d1O CARLOS MARINO","123":"GRASS PLATA MIGUEL SNEIDER","124":"MANZANO CALVO JUAN SEBASTIAN","125":"MENDOZA GOITA MARIANSEL ZENAYDA","126":"MURILLO ARAQUE JAIVER GEOVANY","127":"NI\u00d1O ARENAS HECTOR GONZALO","128":"RAMIREZ CHAVERRA JHON EDISON","129":"XXX4","130":"XXX5","131":"XXX6","132":"RODRIGUEZ MOSQUERA LUIS FERNANDO","133":"PEPITO PEREZ","134":"RAMIREZ VARGAS MARCELA PAOLA","135":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","136":"TORO CISNEROS GARY JOSE","137":"USECHE CALDERON JADID ESTIVEN","138":"VASQUEZ NIETO CAMILO ANDRES","139":"JHONY CASTRO","140":"BERNAL JUAN DAVID","141":"XXX7","142":"XXX8","143":"XXX9","144":"BARON HERNANDEZ HAROLD ANTONIO","145":"CASTELLANOS CARVAJAL DEYVITH FABIAN","146":"AROCA TORRES JULIAN EDUARDO","147":"BERMUDEZ PARRA JENNIFER XIOMARA","148":"BERNAL BAQUERO JAMES RICARDO","149":"BURGOS ORTIZ JOSE HORACIO","150":"CANTOR PORRAS JUAN FERNEY","151":"CAPERA CAPERA JOSE GABRIEL","152":"CARDENAS LOTERO RICARDO ANDR\u00c9S","153":"RENDON OSPINA NELSON LEANDRO","154":"SARMIENTO URBINA MOISES DANIEL","155":"VELASCO VELASCO SEBASTI\u00c1N DAVID","156":"DELGADO DELGADO JOHAN DARIO","157":"FLOREZ SAUCESO KENIS ALBERTO","158":"CARDONA GARCIA OSCAR JAVIER","159":"CARVAJAL GARC\u00cdA HOVER MARCK","160":"CEPEDA PIRAQUIVE JUAN DAVID","161":"FAJARDO SAENZ OSCAR FERNANDO","162":"FLOREZ ESPITIA RONY ALBERTO","163":"GARCIA CUERVO EDWIN JAVIER","164":"GONZALEZ OCHOA JUAN CARLOS","165":"XXX1","166":"XXX2","167":"XXX3","168":"FONSECA RAY RICARDO","169":"GOMEZ BETANCUR JAIDER ANDRES","170":"GRANADA PATI\u00d1O CARLOS MARINO","171":"GRASS PLATA MIGUEL SNEIDER","172":"MANZANO CALVO JUAN SEBASTIAN","173":"MENDOZA GOITA MARIANSEL ZENAYDA","174":"MURILLO ARAQUE JAIVER GEOVANY","175":"NI\u00d1O ARENAS HECTOR GONZALO","176":"RAMIREZ CHAVERRA JHON EDISON","177":"XXX4","178":"XXX5","179":"XXX6","180":"RODRIGUEZ MOSQUERA LUIS FERNANDO","181":"PEPITO PEREZ","182":"RAMIREZ VARGAS MARCELA PAOLA","183":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","184":"TORO CISNEROS GARY JOSE","185":"USECHE CALDERON JADID ESTIVEN","186":"VASQUEZ NIETO CAMILO ANDRES","187":"JHONY CASTRO","188":"BERNAL JUAN DAVID","189":"XXX7","190":"XXX8","191":"XXX9","192":"BARON HERNANDEZ HAROLD ANTONIO","193":"CASTELLANOS CARVAJAL DEYVITH FABIAN","194":"AROCA TORRES JULIAN EDUARDO","195":"BERMUDEZ PARRA JENNIFER XIOMARA","196":"BERNAL BAQUERO JAMES RICARDO","197":"BURGOS ORTIZ JOSE HORACIO","198":"CANTOR PORRAS JUAN FERNEY","199":"CAPERA CAPERA JOSE GABRIEL","200":"CARDENAS LOTERO RICARDO ANDR\u00c9S","201":"RENDON OSPINA NELSON LEANDRO","202":"SARMIENTO URBINA MOISES DANIEL","203":"VELASCO VELASCO SEBASTI\u00c1N DAVID","204":"DELGADO DELGADO JOHAN DARIO","205":"FLOREZ SAUCESO KENIS ALBERTO","206":"CARDONA GARCIA OSCAR JAVIER","207":"CARVAJAL GARC\u00cdA HOVER MARCK","208":"CEPEDA PIRAQUIVE JUAN DAVID","209":"FAJARDO SAENZ OSCAR FERNANDO","210":"FLOREZ ESPITIA RONY ALBERTO","211":"GARCIA CUERVO EDWIN JAVIER","212":"GONZALEZ OCHOA JUAN CARLOS","213":"XXX1","214":"XXX2","215":"XXX3","216":"FONSECA RAY RICARDO","217":"GOMEZ BETANCUR JAIDER ANDRES","218":"GRANADA PATI\u00d1O CARLOS MARINO","219":"GRASS PLATA MIGUEL SNEIDER","220":"MANZANO CALVO JUAN SEBASTIAN","221":"MENDOZA GOITA MARIANSEL ZENAYDA","222":"MURILLO ARAQUE JAIVER GEOVANY","223":"NI\u00d1O ARENAS HECTOR GONZALO","224":"RAMIREZ CHAVERRA JHON EDISON","225":"XXX4","226":"XXX5","227":"XXX6","228":"RODRIGUEZ MOSQUERA LUIS FERNANDO","229":"PEPITO PEREZ","230":"RAMIREZ VARGAS MARCELA PAOLA","231":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","232":"TORO CISNEROS GARY JOSE","233":"USECHE CALDERON JADID ESTIVEN","234":"VASQUEZ NIETO CAMILO ANDRES","235":"JHONY CASTRO","236":"BERNAL JUAN DAVID","237":"XXX7","238":"XXX8","239":"XXX9","240":"BARON HERNANDEZ HAROLD ANTONIO","241":"CASTELLANOS CARVAJAL DEYVITH FABIAN","242":"AROCA TORRES JULIAN EDUARDO","243":"BERMUDEZ PARRA JENNIFER XIOMARA","244":"BERNAL BAQUERO JAMES RICARDO","245":"BURGOS ORTIZ JOSE HORACIO","246":"CANTOR PORRAS JUAN FERNEY","247":"CAPERA CAPERA JOSE GABRIEL","248":"CARDENAS LOTERO RICARDO ANDR\u00c9S","249":"RENDON OSPINA NELSON LEANDRO","250":"SARMIENTO URBINA MOISES DANIEL","251":"VELASCO VELASCO SEBASTI\u00c1N DAVID","252":"DELGADO DELGADO JOHAN DARIO","253":"FLOREZ SAUCESO KENIS ALBERTO","254":"CARDONA GARCIA OSCAR JAVIER","255":"CARVAJAL GARC\u00cdA HOVER MARCK","256":"CEPEDA PIRAQUIVE JUAN DAVID","257":"FAJARDO SAENZ OSCAR FERNANDO","258":"FLOREZ ESPITIA RONY ALBERTO","259":"GARCIA CUERVO EDWIN JAVIER","260":"GONZALEZ OCHOA JUAN CARLOS","261":"XXX1","262":"XXX2","263":"XXX3","264":"FONSECA RAY RICARDO","265":"GOMEZ BETANCUR JAIDER ANDRES","266":"GRANADA PATI\u00d1O CARLOS MARINO","267":"GR</t>
   </si>
   <si>
@@ -68,6 +74,9 @@
   </si>
   <si>
     <t>[{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master</t>
+  </si>
+  <si>
+    <t>[{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"01-Sab","Final":"T2","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"01-Sab","Final":"T2","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"01-Sab","Final":"T2","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"01-Sab","Final":"T2","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"01-Sab","Final":"T2","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"01-Sab","Final":"T2","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"01-Sab","Final":"T2","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"01-Sab","Final":"T2","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"01-Sab","Final":"T2","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"01-Sab","Final":"T2","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"01-Sab","Final":"T2","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"01-Sab","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"01-Sab","Final":"T1","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"01-Sab","Final":"T1","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"01-Sab","Final":"T1","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"01-Sab","Final":"T1","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"01-Sab","Final":"T1","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"01-Sab","Final":"T1","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"01-Sab","Final":"T1","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"01-Sab","Final":"T1","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"01-Sab","Final":"T1","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"01-Sab","Final":"T1","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"01-Sab","Final":"T1","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"01-Sab","Final":"T1","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"01-Sab","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"01-Sab","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"01-Sab","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"01-Sab","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"01-Sab","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"01-Sab","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"01-Sab","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"01-Sab","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"01-Sab","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"01-Sab","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"01-Sab","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"01-Sab","Final":"T3","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"01-Sab","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"01-Sab","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"01-Sab","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"01-Sab","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"01-Sab","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"01-Sab","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"01-Sab","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"01-Sab","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"01-Sab","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"01-Sab","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"01-Sab","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"01-Sab","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"02-Dom","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"02-Dom","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"02-Dom","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"02-Dom","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"02-Dom","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"02-Dom","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"02-Dom","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"02-Dom","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"02-Dom","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"02-Dom","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"02-Dom","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"02-Dom","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"02-Dom","Final":"T1","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"02-Dom","Final":"T1","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"02-Dom","Final":"T1","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"02-Dom","Final":"T1","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"02-Dom","Final":"T1","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"02-Dom","Final":"T1","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"02-Dom","Final":"T1","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"02-Dom","Final":"T1","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"02-Dom","Final":"T1","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"02-Dom","Final":"T1","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"02-Dom","Final":"T1","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"02-Dom","Final":"T1","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"02-Dom","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"02-Dom","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"02-Dom","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"02-Dom","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"02-Dom","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"02-Dom","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"02-Dom","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"02-Dom","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"02-Dom","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"02-Dom","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"02-Dom","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"02-Dom","Final":"T3","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"02-Dom","Final":"T2","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"02-Dom","Final":"T2","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"02-Dom","Final":"T2","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"02-Dom","Final":"T2","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"02-Dom","Final":"T2","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"02-Dom","Final":"T2","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"02-Dom","Final":"T2","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"02-Dom","Final":"T2","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"02-Dom","Final":"T2","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"02-Dom","Final":"T2","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"02-Dom","Final":"T2","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"02-Dom","Final":"T2","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"03-Lun","Final":"T1","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"03-Lun","Final":"T1","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"03-Lun","Final":"T1","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"03-Lun","Final":"T1","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"03-Lun","Final":"T1","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"03-Lun","Final":"T1","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"03-Lun","Final":"T1","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"03-Lun","Final":"T1","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"03-Lun","Final":"T1","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"03-Lun","Final":"T1","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"03-Lun","Final":"T1","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"03-Lun","Final":"T1","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"03-Lun","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"03-Lun","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"03-Lun","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"03-Lun","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"03-Lun","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"03-Lun","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"03-Lun","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"03-Lun","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"03-Lun","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"03-Lun","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"03-Lun","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"03-Lun","Final":"T3","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"04-Mar","Final":"T1","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"04-Mar","Final":"T1","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"04-Mar","Final":"T1","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"04-Mar","Final":"T1","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"04-Mar","Final":"T1","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"04-Mar","Final":"T1","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"04-Mar","Final":"T1","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"04-Mar","Final":"T1","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"04-Mar","Final":"T1","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"04-Mar","Final":"T1","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"04-Mar","Final":"T1","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"04-Mar","Final":"T1","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"04-Mar","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"04-Mar","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"04-Mar","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"04-Mar","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"04-Mar","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"04-Mar","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"04-Mar","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"04-Mar","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"04-Mar","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"04-Mar","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"04-Mar","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"04-Mar","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"05-Mie","Final":"T1","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"05-Mie","Final":"T1","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"05-Mie","Final":"T1","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"05-Mie","Final":"T1","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"05-Mie","Final":"T1","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"05-Mie","Final":"T1","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"05-Mie","Final":"T1","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"05-Mie","Final":"T1","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"05-Mie","Final":"T1","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"05-Mie","Final":"T1","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"05-Mie","Final":"T1","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"05-Mie","Final":"T1","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"05-Mie","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"05-Mie","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"05-Mie","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"05-Mie","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"05-Mie","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"05-Mie","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"05-Mie","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"05-Mie","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"05-Mie","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"05-Mie","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"05-Mie","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"05-Mie","Final":"T3","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"06-Jue","Final":"T2","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"06-Jue","Final":"T2","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"06-Jue","Final":"T2","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"06-Jue","Final":"T2","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"06-Jue","Final":"T2","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"06-Jue","Final":"T2","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"06-Jue","Final":"T2","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"06-Jue","Final":"T2","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"06-Jue","Final":"T2","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"06-Jue","Final":"T2","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"06-Jue","Final":"T2","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"06-Jue","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"06-Jue","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"06-Jue","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"06-Jue","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"06-Jue","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"06-Jue","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"06-Jue","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"06-Jue","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"06-Jue","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"06-Jue","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"06-Jue","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"06-Jue","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"06-Jue","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"06-Jue","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"06-Jue","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"06-Jue","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"06-Jue","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"06-Jue","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"06-Jue","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"06-Jue","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"06-Jue","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"06-Jue","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"06-Jue","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"06-Jue","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"06-Jue","Final":"T3","n_dia":6},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"06-Jue","Final":"T2","n_dia":6},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"06-Jue","Final":"T2","n_dia":6},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VA</t>
   </si>
 </sst>
 </file>
@@ -399,7 +408,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -427,13 +436,13 @@
         <v>2026</v>
       </c>
       <c r="C2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -444,13 +453,13 @@
         <v>2026</v>
       </c>
       <c r="C3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -461,13 +470,13 @@
         <v>2026</v>
       </c>
       <c r="C4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E4" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -478,13 +487,30 @@
         <v>2026</v>
       </c>
       <c r="C5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" t="s">
         <v>9</v>
       </c>
-      <c r="D5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E5" t="s">
-        <v>17</v>
+      <c r="B6">
+        <v>2026</v>
+      </c>
+      <c r="C6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" t="s">
+        <v>15</v>
+      </c>
+      <c r="E6" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update historico_mallas.xlsx 2026-04-24 21:35:11.005332
</commit_message>
<xml_diff>
--- a/historico_mallas.xlsx
+++ b/historico_mallas.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="23">
   <si>
     <t>Mes</t>
   </si>
@@ -31,27 +31,27 @@
     <t>Datos_JSON</t>
   </si>
   <si>
+    <t>Alcance</t>
+  </si>
+  <si>
+    <t>Abril</t>
+  </si>
+  <si>
+    <t>Junio</t>
+  </si>
+  <si>
+    <t>Julio</t>
+  </si>
+  <si>
+    <t>Agosto</t>
+  </si>
+  <si>
     <t>Mayo</t>
   </si>
   <si>
-    <t>Abril</t>
-  </si>
-  <si>
-    <t>Junio</t>
-  </si>
-  <si>
-    <t>Julio</t>
-  </si>
-  <si>
-    <t>Agosto</t>
-  </si>
-  <si>
     <t>Técnica</t>
   </si>
   <si>
-    <t>24/04/2026 17:55</t>
-  </si>
-  <si>
     <t>2026-04-24 18:15</t>
   </si>
   <si>
@@ -64,7 +64,7 @@
     <t>2026-04-24 18:28</t>
   </si>
   <si>
-    <t>{"Grupo":{"0":"GRUPO 1","1":"GRUPO 1","2":"GRUPO 1","3":"GRUPO 1","4":"GRUPO 1","5":"GRUPO 1","6":"GRUPO 1","7":"GRUPO 1","8":"GRUPO 1","9":"GRUPO 1","10":"GRUPO 1","11":"GRUPO 1","12":"GRUPO 2","13":"GRUPO 2","14":"GRUPO 2","15":"GRUPO 2","16":"GRUPO 2","17":"GRUPO 2","18":"GRUPO 2","19":"GRUPO 2","20":"GRUPO 2","21":"GRUPO 2","22":"GRUPO 2","23":"GRUPO 2","24":"GRUPO 3","25":"GRUPO 3","26":"GRUPO 3","27":"GRUPO 3","28":"GRUPO 3","29":"GRUPO 3","30":"GRUPO 3","31":"GRUPO 3","32":"GRUPO 3","33":"GRUPO 3","34":"GRUPO 3","35":"GRUPO 3","36":"GRUPO 4","37":"GRUPO 4","38":"GRUPO 4","39":"GRUPO 4","40":"GRUPO 4","41":"GRUPO 4","42":"GRUPO 4","43":"GRUPO 4","44":"GRUPO 4","45":"GRUPO 4","46":"GRUPO 4","47":"GRUPO 4","48":"GRUPO 1","49":"GRUPO 1","50":"GRUPO 1","51":"GRUPO 1","52":"GRUPO 1","53":"GRUPO 1","54":"GRUPO 1","55":"GRUPO 1","56":"GRUPO 1","57":"GRUPO 1","58":"GRUPO 1","59":"GRUPO 1","60":"GRUPO 2","61":"GRUPO 2","62":"GRUPO 2","63":"GRUPO 2","64":"GRUPO 2","65":"GRUPO 2","66":"GRUPO 2","67":"GRUPO 2","68":"GRUPO 2","69":"GRUPO 2","70":"GRUPO 2","71":"GRUPO 2","72":"GRUPO 3","73":"GRUPO 3","74":"GRUPO 3","75":"GRUPO 3","76":"GRUPO 3","77":"GRUPO 3","78":"GRUPO 3","79":"GRUPO 3","80":"GRUPO 3","81":"GRUPO 3","82":"GRUPO 3","83":"GRUPO 3","84":"GRUPO 4","85":"GRUPO 4","86":"GRUPO 4","87":"GRUPO 4","88":"GRUPO 4","89":"GRUPO 4","90":"GRUPO 4","91":"GRUPO 4","92":"GRUPO 4","93":"GRUPO 4","94":"GRUPO 4","95":"GRUPO 4","96":"GRUPO 1","97":"GRUPO 1","98":"GRUPO 1","99":"GRUPO 1","100":"GRUPO 1","101":"GRUPO 1","102":"GRUPO 1","103":"GRUPO 1","104":"GRUPO 1","105":"GRUPO 1","106":"GRUPO 1","107":"GRUPO 1","108":"GRUPO 2","109":"GRUPO 2","110":"GRUPO 2","111":"GRUPO 2","112":"GRUPO 2","113":"GRUPO 2","114":"GRUPO 2","115":"GRUPO 2","116":"GRUPO 2","117":"GRUPO 2","118":"GRUPO 2","119":"GRUPO 2","120":"GRUPO 3","121":"GRUPO 3","122":"GRUPO 3","123":"GRUPO 3","124":"GRUPO 3","125":"GRUPO 3","126":"GRUPO 3","127":"GRUPO 3","128":"GRUPO 3","129":"GRUPO 3","130":"GRUPO 3","131":"GRUPO 3","132":"GRUPO 4","133":"GRUPO 4","134":"GRUPO 4","135":"GRUPO 4","136":"GRUPO 4","137":"GRUPO 4","138":"GRUPO 4","139":"GRUPO 4","140":"GRUPO 4","141":"GRUPO 4","142":"GRUPO 4","143":"GRUPO 4","144":"GRUPO 1","145":"GRUPO 1","146":"GRUPO 1","147":"GRUPO 1","148":"GRUPO 1","149":"GRUPO 1","150":"GRUPO 1","151":"GRUPO 1","152":"GRUPO 1","153":"GRUPO 1","154":"GRUPO 1","155":"GRUPO 1","156":"GRUPO 2","157":"GRUPO 2","158":"GRUPO 2","159":"GRUPO 2","160":"GRUPO 2","161":"GRUPO 2","162":"GRUPO 2","163":"GRUPO 2","164":"GRUPO 2","165":"GRUPO 2","166":"GRUPO 2","167":"GRUPO 2","168":"GRUPO 3","169":"GRUPO 3","170":"GRUPO 3","171":"GRUPO 3","172":"GRUPO 3","173":"GRUPO 3","174":"GRUPO 3","175":"GRUPO 3","176":"GRUPO 3","177":"GRUPO 3","178":"GRUPO 3","179":"GRUPO 3","180":"GRUPO 4","181":"GRUPO 4","182":"GRUPO 4","183":"GRUPO 4","184":"GRUPO 4","185":"GRUPO 4","186":"GRUPO 4","187":"GRUPO 4","188":"GRUPO 4","189":"GRUPO 4","190":"GRUPO 4","191":"GRUPO 4","192":"GRUPO 1","193":"GRUPO 1","194":"GRUPO 1","195":"GRUPO 1","196":"GRUPO 1","197":"GRUPO 1","198":"GRUPO 1","199":"GRUPO 1","200":"GRUPO 1","201":"GRUPO 1","202":"GRUPO 1","203":"GRUPO 1","204":"GRUPO 2","205":"GRUPO 2","206":"GRUPO 2","207":"GRUPO 2","208":"GRUPO 2","209":"GRUPO 2","210":"GRUPO 2","211":"GRUPO 2","212":"GRUPO 2","213":"GRUPO 2","214":"GRUPO 2","215":"GRUPO 2","216":"GRUPO 3","217":"GRUPO 3","218":"GRUPO 3","219":"GRUPO 3","220":"GRUPO 3","221":"GRUPO 3","222":"GRUPO 3","223":"GRUPO 3","224":"GRUPO 3","225":"GRUPO 3","226":"GRUPO 3","227":"GRUPO 3","228":"GRUPO 4","229":"GRUPO 4","230":"GRUPO 4","231":"GRUPO 4","232":"GRUPO 4","233":"GRUPO 4","234":"GRUPO 4","235":"GRUPO 4","236":"GRUPO 4","237":"GRUPO 4","238":"GRUPO 4","239":"GRUPO 4","240":"GRUPO 1","241":"GRUPO 1","242":"GRUPO 1","243":"GRUPO 1","244":"GRUPO 1","245":"GRUPO 1","246":"GRUPO 1","247":"GRUPO 1","248":"GRUPO 1","249":"GRUPO 1","250":"GRUPO 1","251":"GRUPO 1","252":"GRUPO 2","253":"GRUPO 2","254":"GRUPO 2","255":"GRUPO 2","256":"GRUPO 2","257":"GRUPO 2","258":"GRUPO 2","259":"GRUPO 2","260":"GRUPO 2","261":"GRUPO 2","262":"GRUPO 2","263":"GRUPO 2","264":"GRUPO 3","265":"GRUPO 3","266":"GRUPO 3","267":"GRUPO 3","268":"GRUPO 3","269":"GRUPO 3","270":"GRUPO 3","271":"GRUPO 3","272":"GRUPO 3","273":"GRUPO 3","274":"GRUPO 3","275":"GRUPO 3","276":"GRUPO 4","277":"GRUPO 4","278":"GRUPO 4","279":"GRUPO 4","280":"GRUPO 4","281":"GRUPO 4","282":"GRUPO 4","283":"GRUPO 4","284":"GRUPO 4","285":"GRUPO 4","286":"GRUPO 4","287":"GRUPO 4","288":"GRUPO 1","289":"GRUPO 1","290":"GRUPO 1","291":"GRUPO 1","292":"GRUPO 1","293":"GRUPO 1","294":"GRUPO 1","295":"GRUPO 1","296":"GRUPO 1","297":"GRUPO 1","298":"GRUPO 1","299":"GRUPO 1","300":"GRUPO 2","301":"GRUPO 2","302":"GRUPO 2","303":"GRUPO 2","304":"GRUPO 2","305":"GRUPO 2","306":"GRUPO 2","307":"GRUPO 2","308":"GRUPO 2","309":"GRUPO 2","310":"GRUPO 2","311":"GRUPO 2","312":"GRUPO 3","313":"GRUPO 3","314":"GRUPO 3","315":"GRUPO 3","316":"GRUPO 3","317":"GRUPO 3","318":"GRUPO 3","319":"GRUPO 3","320":"GRUPO 3","321":"GRUPO 3","322":"GRUPO 3","323":"GRUPO 3","324":"GRUPO 4","325":"GRUPO 4","326":"GRUPO 4","327":"GRUPO 4","328":"GRUPO 4","329":"GRUPO 4","330":"GRUPO 4","331":"GRUPO 4","332":"GRUPO 4","333":"GRUPO 4","334":"GRUPO 4","335":"GRUPO 4","336":"GRUPO 1","337":"GRUPO 1","338":"GRUPO 1","339":"GRUPO 1","340":"GRUPO 1","341":"GRUPO 1","342":"GRUPO 1","343":"GRUPO 1","344":"GRUPO 1","345":"GRUPO 1","346":"GRUPO 1","347":"GRUPO 1","348":"GRUPO 2","349":"GRUPO 2","350":"GRUPO 2","351":"GRUPO 2","352":"GRUPO 2","353":"GRUPO 2","354":"GRUPO 2","355":"GRUPO 2","356":"GRUPO 2","357":"GRUPO 2","358":"GRUPO 2","359":"GRUPO 2","360":"GRUPO 3","361":"GRUPO 3","362":"GRUPO 3","363":"GRUPO 3","364":"GRUPO 3","365":"GRUPO 3","366":"GRUPO 3","367":"GRUPO 3","368":"GRUPO 3","369":"GRUPO 3","370":"GRUPO 3","371":"GRUPO 3","372":"GRUPO 4","373":"GRUPO 4","374":"GRUPO 4","375":"GRUPO 4","376":"GRUPO 4","377":"GRUPO 4","378":"GRUPO 4","379":"GRUPO 4","380":"GRUPO 4","381":"GRUPO 4","382":"GRUPO 4","383":"GRUPO 4","384":"GRUPO 1","385":"GRUPO 1","386":"GRUPO 1","387":"GRUPO 1","388":"GRUPO 1","389":"GRUPO 1","390":"GRUPO 1","391":"GRUPO 1","392":"GRUPO 1","393":"GRUPO 1","394":"GRUPO 1","395":"GRUPO 1","396":"GRUPO 2","397":"GRUPO 2","398":"GRUPO 2","399":"GRUPO 2","400":"GRUPO 2","401":"GRUPO 2","402":"GRUPO 2","403":"GRUPO 2","404":"GRUPO 2","405":"GRUPO 2","406":"GRUPO 2","407":"GRUPO 2","408":"GRUPO 3","409":"GRUPO 3","410":"GRUPO 3","411":"GRUPO 3","412":"GRUPO 3","413":"GRUPO 3","414":"GRUPO 3","415":"GRUPO 3","416":"GRUPO 3","417":"GRUPO 3","418":"GRUPO 3","419":"GRUPO 3","420":"GRUPO 4","421":"GRUPO 4","422":"GRUPO 4","423":"GRUPO 4","424":"GRUPO 4","425":"GRUPO 4","426":"GRUPO 4","427":"GRUPO 4","428":"GRUPO 4","429":"GRUPO 4","430":"GRUPO 4","431":"GRUPO 4","432":"GRUPO 1","433":"GRUPO 1","434":"GRUPO 1","435":"GRUPO 1","436":"GRUPO 1","437":"GRUPO 1","438":"GRUPO 1","439":"GRUPO 1","440":"GRUPO 1","441":"GRUPO 1","442":"GRUPO 1","443":"GRUPO 1","444":"GRUPO 2","445":"GRUPO 2","446":"GRUPO 2","447":"GRUPO 2","448":"GRUPO 2","449":"GRUPO 2","450":"GRUPO 2","451":"GRUPO 2","452":"GRUPO 2","453":"GRUPO 2","454":"GRUPO 2","455":"GRUPO 2","456":"GRUPO 3","457":"GRUPO 3","458":"GRUPO 3","459":"GRUPO 3","460":"GRUPO 3","461":"GRUPO 3","462":"GRUPO 3","463":"GRUPO 3","464":"GRUPO 3","465":"GRUPO 3","466":"GRUPO 3","467":"GRUPO 3","468":"GRUPO 4","469":"GRUPO 4","470":"GRUPO 4","471":"GRUPO 4","472":"GRUPO 4","473":"GRUPO 4","474":"GRUPO 4","475":"GRUPO 4","476":"GRUPO 4","477":"GRUPO 4","478":"GRUPO 4","479":"GRUPO 4","480":"GRUPO 1","481":"GRUPO 1","482":"GRUPO 1","483":"GRUPO 1","484":"GRUPO 1","485":"GRUPO 1","486":"GRUPO 1","487":"GRUPO 1","488":"GRUPO 1","489":"GRUPO 1","490":"GRUPO 1","491":"GRUPO 1","492":"GRUPO 2","493":"GRUPO 2","494":"GRUPO 2","495":"GRUPO 2","496":"GRUPO 2","497":"GRUPO 2","498":"GRUPO 2","499":"GRUPO 2","500":"GRUPO 2","501":"GRUPO 2","502":"GRUPO 2","503":"GRUPO 2","504":"GRUPO 3","505":"GRUPO 3","506":"GRUPO 3","507":"GRUPO 3","508":"GRUPO 3","509":"GRUPO 3","510":"GRUPO 3","511":"GRUPO 3","512":"GRUPO 3","513":"GRUPO 3","514":"GRUPO 3","515":"GRUPO 3","516":"GRUPO 4","517":"GRUPO 4","518":"GRUPO 4","519":"GRUPO 4","520":"GRUPO 4","521":"GRUPO 4","522":"GRUPO 4","523":"GRUPO 4","524":"GRUPO 4","525":"GRUPO 4","526":"GRUPO 4","527":"GRUPO 4","528":"GRUPO 1","529":"GRUPO 1","530":"GRUPO 1","531":"GRUPO 1","532":"GRUPO 1","533":"GRUPO 1","534":"GRUPO 1","535":"GRUPO 1","536":"GRUPO 1","537":"GRUPO 1","538":"GRUPO 1","539":"GRUPO 1","540":"GRUPO 2","541":"GRUPO 2","542":"GRUPO 2","543":"GRUPO 2","544":"GRUPO 2","545":"GRUPO 2","546":"GRUPO 2","547":"GRUPO 2","548":"GRUPO 2","549":"GRUPO 2","550":"GRUPO 2","551":"GRUPO 2","552":"GRUPO 3","553":"GRUPO 3","554":"GRUPO 3","555":"GRUPO 3","556":"GRUPO 3","557":"GRUPO 3","558":"GRUPO 3","559":"GRUPO 3","560":"GRUPO 3","561":"GRUPO 3","562":"GRUPO 3","563":"GRUPO 3","564":"GRUPO 4","565":"GRUPO 4","566":"GRUPO 4","567":"GRUPO 4","568":"GRUPO 4","569":"GRUPO 4","570":"GRUPO 4","571":"GRUPO 4","572":"GRUPO 4","573":"GRUPO 4","574":"GRUPO 4","575":"GRUPO 4","576":"GRUPO 1","577":"GRUPO 1","578":"GRUPO 1","579":"GRUPO 1","580":"GRUPO 1","581":"GRUPO 1","582":"GRUPO 1","583":"GRUPO 1","584":"GRUPO 1","585":"GRUPO 1","586":"GRUPO 1","587":"GRUPO 1","588":"GRUPO 2","589":"GRUPO 2","590":"GRUPO 2","591":"GRUPO 2","592":"GRUPO 2","593":"GRUPO 2","594":"GRUPO 2","595":"GRUPO 2","596":"GRUPO 2","597":"GRUPO 2","598":"GRUPO 2","599":"GRUPO 2","600":"GRUPO 3","601":"GRUPO 3","602":"GRUPO 3","603":"GRUPO 3","604":"GRUPO 3","605":"GRUPO 3","606":"GRUPO 3","607":"GRUPO 3","608":"GRUPO 3","609":"GRUPO 3","610":"GRUPO 3","611":"GRUPO 3","612":"GRUPO 4","613":"GRUPO 4","614":"GRUPO 4","615":"GRUPO 4","616":"GRUPO 4","617":"GRUPO 4","618":"GRUPO 4","619":"GRUPO 4","620":"GRUPO 4","621":"GRUPO 4","622":"GRUPO 4","623":"GRUPO 4","624":"GRUPO 1","625":"GRUPO 1","626":"GRUPO 1","627":"GRUPO 1","628":"GRUPO 1","629":"GRUPO 1","630":"GRUPO 1","631":"GRUPO 1","632":"GRUPO 1","633":"GRUPO 1","634":"GRUPO 1","635":"GRUPO 1","636":"GRUPO 2","637":"GRUPO 2","638":"GRUPO 2","639":"GRUPO 2","640":"GRUPO 2","641":"GRUPO 2","642":"GRUPO 2","643":"GRUPO 2","644":"GRUPO 2","645":"GRUPO 2","646":"GRUPO 2","647":"GRUPO 2","648":"GRUPO 3","649":"GRUPO 3","650":"GRUPO 3","651":"GRUPO 3","652":"GRUPO 3","653":"GRUPO 3","654":"GRUPO 3","655":"GRUPO 3","656":"GRUPO 3","657":"GRUPO 3","658":"GRUPO 3","659":"GRUPO 3","660":"GRUPO 4","661":"GRUPO 4","662":"GRUPO 4","663":"GRUPO 4","664":"GRUPO 4","665":"GRUPO 4","666":"GRUPO 4","667":"GRUPO 4","668":"GRUPO 4","669":"GRUPO 4","670":"GRUPO 4","671":"GRUPO 4","672":"GRUPO 1","673":"GRUPO 1","674":"GRUPO 1","675":"GRUPO 1","676":"GRUPO 1","677":"GRUPO 1","678":"GRUPO 1","679":"GRUPO 1","680":"GRUPO 1","681":"GRUPO 1","682":"GRUPO 1","683":"GRUPO 1","684":"GRUPO 2","685":"GRUPO 2","686":"GRUPO 2","687":"GRUPO 2","688":"GRUPO 2","689":"GRUPO 2","690":"GRUPO 2","691":"GRUPO 2","692":"GRUPO 2","693":"GRUPO 2","694":"GRUPO 2","695":"GRUPO 2","696":"GRUPO 3","697":"GRUPO 3","698":"GRUPO 3","699":"GRUPO 3","700":"GRUPO 3","701":"GRUPO 3","702":"GRUPO 3","703":"GRUPO 3","704":"GRUPO 3","705":"GRUPO 3","706":"GRUPO 3","707":"GRUPO 3","708":"GRUPO 4","709":"GRUPO 4","710":"GRUPO 4","711":"GRUPO 4","712":"GRUPO 4","713":"GRUPO 4","714":"GRUPO 4","715":"GRUPO 4","716":"GRUPO 4","717":"GRUPO 4","718":"GRUPO 4","719":"GRUPO 4","720":"GRUPO 1","721":"GRUPO 1","722":"GRUPO 1","723":"GRUPO 1","724":"GRUPO 1","725":"GRUPO 1","726":"GRUPO 1","727":"GRUPO 1","728":"GRUPO 1","729":"GRUPO 1","730":"GRUPO 1","731":"GRUPO 1","732":"GRUPO 2","733":"GRUPO 2","734":"GRUPO 2","735":"GRUPO 2","736":"GRUPO 2","737":"GRUPO 2","738":"GRUPO 2","739":"GRUPO 2","740":"GRUPO 2","741":"GRUPO 2","742":"GRUPO 2","743":"GRUPO 2","744":"GRUPO 3","745":"GRUPO 3","746":"GRUPO 3","747":"GRUPO 3","748":"GRUPO 3","749":"GRUPO 3","750":"GRUPO 3","751":"GRUPO 3","752":"GRUPO 3","753":"GRUPO 3","754":"GRUPO 3","755":"GRUPO 3","756":"GRUPO 4","757":"GRUPO 4","758":"GRUPO 4","759":"GRUPO 4","760":"GRUPO 4","761":"GRUPO 4","762":"GRUPO 4","763":"GRUPO 4","764":"GRUPO 4","765":"GRUPO 4","766":"GRUPO 4","767":"GRUPO 4","768":"GRUPO 1","769":"GRUPO 1","770":"GRUPO 1","771":"GRUPO 1","772":"GRUPO 1","773":"GRUPO 1","774":"GRUPO 1","775":"GRUPO 1","776":"GRUPO 1","777":"GRUPO 1","778":"GRUPO 1","779":"GRUPO 1","780":"GRUPO 2","781":"GRUPO 2","782":"GRUPO 2","783":"GRUPO 2","784":"GRUPO 2","785":"GRUPO 2","786":"GRUPO 2","787":"GRUPO 2","788":"GRUPO 2","789":"GRUPO 2","790":"GRUPO 2","791":"GRUPO 2","792":"GRUPO 3","793":"GRUPO 3","794":"GRUPO 3","795":"GRUPO 3","796":"GRUPO 3","797":"GRUPO 3","798":"GRUPO 3","799":"GRUPO 3","800":"GRUPO 3","801":"GRUPO 3","802":"GRUPO 3","803":"GRUPO 3","804":"GRUPO 4","805":"GRUPO 4","806":"GRUPO 4","807":"GRUPO 4","808":"GRUPO 4","809":"GRUPO 4","810":"GRUPO 4","811":"GRUPO 4","812":"GRUPO 4","813":"GRUPO 4","814":"GRUPO 4","815":"GRUPO 4","816":"GRUPO 1","817":"GRUPO 1","818":"GRUPO 1","819":"GRUPO 1","820":"GRUPO 1","821":"GRUPO 1","822":"GRUPO 1","823":"GRUPO 1","824":"GRUPO 1","825":"GRUPO 1","826":"GRUPO 1","827":"GRUPO 1","828":"GRUPO 2","829":"GRUPO 2","830":"GRUPO 2","831":"GRUPO 2","832":"GRUPO 2","833":"GRUPO 2","834":"GRUPO 2","835":"GRUPO 2","836":"GRUPO 2","837":"GRUPO 2","838":"GRUPO 2","839":"GRUPO 2","840":"GRUPO 3","841":"GRUPO 3","842":"GRUPO 3","843":"GRUPO 3","844":"GRUPO 3","845":"GRUPO 3","846":"GRUPO 3","847":"GRUPO 3","848":"GRUPO 3","849":"GRUPO 3","850":"GRUPO 3","851":"GRUPO 3","852":"GRUPO 4","853":"GRUPO 4","854":"GRUPO 4","855":"GRUPO 4","856":"GRUPO 4","857":"GRUPO 4","858":"GRUPO 4","859":"GRUPO 4","860":"GRUPO 4","861":"GRUPO 4","862":"GRUPO 4","863":"GRUPO 4","864":"GRUPO 1","865":"GRUPO 1","866":"GRUPO 1","867":"GRUPO 1","868":"GRUPO 1","869":"GRUPO 1","870":"GRUPO 1","871":"GRUPO 1","872":"GRUPO 1","873":"GRUPO 1","874":"GRUPO 1","875":"GRUPO 1","876":"GRUPO 2","877":"GRUPO 2","878":"GRUPO 2","879":"GRUPO 2","880":"GRUPO 2","881":"GRUPO 2","882":"GRUPO 2","883":"GRUPO 2","884":"GRUPO 2","885":"GRUPO 2","886":"GRUPO 2","887":"GRUPO 2","888":"GRUPO 3","889":"GRUPO 3","890":"GRUPO 3","891":"GRUPO 3","892":"GRUPO 3","893":"GRUPO 3","894":"GRUPO 3","895":"GRUPO 3","896":"GRUPO 3","897":"GRUPO 3","898":"GRUPO 3","899":"GRUPO 3","900":"GRUPO 4","901":"GRUPO 4","902":"GRUPO 4","903":"GRUPO 4","904":"GRUPO 4","905":"GRUPO 4","906":"GRUPO 4","907":"GRUPO 4","908":"GRUPO 4","909":"GRUPO 4","910":"GRUPO 4","911":"GRUPO 4","912":"GRUPO 1","913":"GRUPO 1","914":"GRUPO 1","915":"GRUPO 1","916":"GRUPO 1","917":"GRUPO 1","918":"GRUPO 1","919":"GRUPO 1","920":"GRUPO 1","921":"GRUPO 1","922":"GRUPO 1","923":"GRUPO 1","924":"GRUPO 2","925":"GRUPO 2","926":"GRUPO 2","927":"GRUPO 2","928":"GRUPO 2","929":"GRUPO 2","930":"GRUPO 2","931":"GRUPO 2","932":"GRUPO 2","933":"GRUPO 2","934":"GRUPO 2","935":"GRUPO 2","936":"GRUPO 3","937":"GRUPO 3","938":"GRUPO 3","939":"GRUPO 3","940":"GRUPO 3","941":"GRUPO 3","942":"GRUPO 3","943":"GRUPO 3","944":"GRUPO 3","945":"GRUPO 3","946":"GRUPO 3","947":"GRUPO 3","948":"GRUPO 4","949":"GRUPO 4","950":"GRUPO 4","951":"GRUPO 4","952":"GRUPO 4","953":"GRUPO 4","954":"GRUPO 4","955":"GRUPO 4","956":"GRUPO 4","957":"GRUPO 4","958":"GRUPO 4","959":"GRUPO 4","960":"GRUPO 1","961":"GRUPO 1","962":"GRUPO 1","963":"GRUPO 1","964":"GRUPO 1","965":"GRUPO 1","966":"GRUPO 1","967":"GRUPO 1","968":"GRUPO 1","969":"GRUPO 1","970":"GRUPO 1","971":"GRUPO 1","972":"GRUPO 2","973":"GRUPO 2","974":"GRUPO 2","975":"GRUPO 2","976":"GRUPO 2","977":"GRUPO 2","978":"GRUPO 2","979":"GRUPO 2","980":"GRUPO 2","981":"GRUPO 2","982":"GRUPO 2","983":"GRUPO 2","984":"GRUPO 3","985":"GRUPO 3","986":"GRUPO 3","987":"GRUPO 3","988":"GRUPO 3","989":"GRUPO 3","990":"GRUPO 3","991":"GRUPO 3","992":"GRUPO 3","993":"GRUPO 3","994":"GRUPO 3","995":"GRUPO 3","996":"GRUPO 4","997":"GRUPO 4","998":"GRUPO 4","999":"GRUPO 4","1000":"GRUPO 4","1001":"GRUPO 4","1002":"GRUPO 4","1003":"GRUPO 4","1004":"GRUPO 4","1005":"GRUPO 4","1006":"GRUPO 4","1007":"GRUPO 4","1008":"GRUPO 1","1009":"GRUPO 1","1010":"GRUPO 1","1011":"GRUPO 1","1012":"GRUPO 1","1013":"GRUPO 1","1014":"GRUPO 1","1015":"GRUPO 1","1016":"GRUPO 1","1017":"GRUPO 1","1018":"GRUPO 1","1019":"GRUPO 1","1020":"GRUPO 2","1021":"GRUPO 2","1022":"GRUPO 2","1023":"GRUPO 2","1024":"GRUPO 2","1025":"GRUPO 2","1026":"GRUPO 2","1027":"GRUPO 2","1028":"GRUPO 2","1029":"GRUPO 2","1030":"GRUPO 2","1031":"GRUPO 2","1032":"GRUPO 3","1033":"GRUPO 3","1034":"GRUPO 3","1035":"GRUPO 3","1036":"GRUPO 3","1037":"GRUPO 3","1038":"GRUPO 3","1039":"GRUPO 3","1040":"GRUPO 3","1041":"GRUPO 3","1042":"GRUPO 3","1043":"GRUPO 3","1044":"GRUPO 4","1045":"GRUPO 4","1046":"GRUPO 4","1047":"GRUPO 4","1048":"GRUPO 4","1049":"GRUPO 4","1050":"GRUPO 4","1051":"GRUPO 4","1052":"GRUPO 4","1053":"GRUPO 4","1054":"GRUPO 4","1055":"GRUPO 4","1056":"GRUPO 1","1057":"GRUPO 1","1058":"GRUPO 1","1059":"GRUPO 1","1060":"GRUPO 1","1061":"GRUPO 1","1062":"GRUPO 1","1063":"GRUPO 1","1064":"GRUPO 1","1065":"GRUPO 1","1066":"GRUPO 1","1067":"GRUPO 1","1068":"GRUPO 2","1069":"GRUPO 2","1070":"GRUPO 2","1071":"GRUPO 2","1072":"GRUPO 2","1073":"GRUPO 2","1074":"GRUPO 2","1075":"GRUPO 2","1076":"GRUPO 2","1077":"GRUPO 2","1078":"GRUPO 2","1079":"GRUPO 2","1080":"GRUPO 3","1081":"GRUPO 3","1082":"GRUPO 3","1083":"GRUPO 3","1084":"GRUPO 3","1085":"GRUPO 3","1086":"GRUPO 3","1087":"GRUPO 3","1088":"GRUPO 3","1089":"GRUPO 3","1090":"GRUPO 3","1091":"GRUPO 3","1092":"GRUPO 4","1093":"GRUPO 4","1094":"GRUPO 4","1095":"GRUPO 4","1096":"GRUPO 4","1097":"GRUPO 4","1098":"GRUPO 4","1099":"GRUPO 4","1100":"GRUPO 4","1101":"GRUPO 4","1102":"GRUPO 4","1103":"GRUPO 4","1104":"GRUPO 1","1105":"GRUPO 1","1106":"GRUPO 1","1107":"GRUPO 1","1108":"GRUPO 1","1109":"GRUPO 1","1110":"GRUPO 1","1111":"GRUPO 1","1112":"GRUPO 1","1113":"GRUPO 1","1114":"GRUPO 1","1115":"GRUPO 1","1116":"GRUPO 2","1117":"GRUPO 2","1118":"GRUPO 2","1119":"GRUPO 2","1120":"GRUPO 2","1121":"GRUPO 2","1122":"GRUPO 2","1123":"GRUPO 2","1124":"GRUPO 2","1125":"GRUPO 2","1126":"GRUPO 2","1127":"GRUPO 2","1128":"GRUPO 3","1129":"GRUPO 3","1130":"GRUPO 3","1131":"GRUPO 3","1132":"GRUPO 3","1133":"GRUPO 3","1134":"GRUPO 3","1135":"GRUPO 3","1136":"GRUPO 3","1137":"GRUPO 3","1138":"GRUPO 3","1139":"GRUPO 3","1140":"GRUPO 4","1141":"GRUPO 4","1142":"GRUPO 4","1143":"GRUPO 4","1144":"GRUPO 4","1145":"GRUPO 4","1146":"GRUPO 4","1147":"GRUPO 4","1148":"GRUPO 4","1149":"GRUPO 4","1150":"GRUPO 4","1151":"GRUPO 4","1152":"GRUPO 1","1153":"GRUPO 1","1154":"GRUPO 1","1155":"GRUPO 1","1156":"GRUPO 1","1157":"GRUPO 1","1158":"GRUPO 1","1159":"GRUPO 1","1160":"GRUPO 1","1161":"GRUPO 1","1162":"GRUPO 1","1163":"GRUPO 1","1164":"GRUPO 2","1165":"GRUPO 2","1166":"GRUPO 2","1167":"GRUPO 2","1168":"GRUPO 2","1169":"GRUPO 2","1170":"GRUPO 2","1171":"GRUPO 2","1172":"GRUPO 2","1173":"GRUPO 2","1174":"GRUPO 2","1175":"GRUPO 2","1176":"GRUPO 3","1177":"GRUPO 3","1178":"GRUPO 3","1179":"GRUPO 3","1180":"GRUPO 3","1181":"GRUPO 3","1182":"GRUPO 3","1183":"GRUPO 3","1184":"GRUPO 3","1185":"GRUPO 3","1186":"GRUPO 3","1187":"GRUPO 3","1188":"GRUPO 4","1189":"GRUPO 4","1190":"GRUPO 4","1191":"GRUPO 4","1192":"GRUPO 4","1193":"GRUPO 4","1194":"GRUPO 4","1195":"GRUPO 4","1196":"GRUPO 4","1197":"GRUPO 4","1198":"GRUPO 4","1199":"GRUPO 4","1200":"GRUPO 1","1201":"GRUPO 1","1202":"GRUPO 1","1203":"GRUPO 1","1204":"GRUPO 1","1205":"GRUPO 1","1206":"GRUPO 1","1207":"GRUPO 1","1208":"GRUPO 1","1209":"GRUPO 1","1210":"GRUPO 1","1211":"GRUPO 1","1212":"GRUPO 2","1213":"GRUPO 2","1214":"GRUPO 2","1215":"GRUPO 2","1216":"GRUPO 2","1217":"GRUPO 2","1218":"GRUPO 2","1219":"GRUPO 2","1220":"GRUPO 2","1221":"GRUPO 2","1222":"GRUPO 2","1223":"GRUPO 2","1224":"GRUPO 3","1225":"GRUPO 3","1226":"GRUPO 3","1227":"GRUPO 3","1228":"GRUPO 3","1229":"GRUPO 3","1230":"GRUPO 3","1231":"GRUPO 3","1232":"GRUPO 3","1233":"GRUPO 3","1234":"GRUPO 3","1235":"GRUPO 3","1236":"GRUPO 4","1237":"GRUPO 4","1238":"GRUPO 4","1239":"GRUPO 4","1240":"GRUPO 4","1241":"GRUPO 4","1242":"GRUPO 4","1243":"GRUPO 4","1244":"GRUPO 4","1245":"GRUPO 4","1246":"GRUPO 4","1247":"GRUPO 4","1248":"GRUPO 1","1249":"GRUPO 1","1250":"GRUPO 1","1251":"GRUPO 1","1252":"GRUPO 1","1253":"GRUPO 1","1254":"GRUPO 1","1255":"GRUPO 1","1256":"GRUPO 1","1257":"GRUPO 1","1258":"GRUPO 1","1259":"GRUPO 1","1260":"GRUPO 2","1261":"GRUPO 2","1262":"GRUPO 2","1263":"GRUPO 2","1264":"GRUPO 2","1265":"GRUPO 2","1266":"GRUPO 2","1267":"GRUPO 2","1268":"GRUPO 2","1269":"GRUPO 2","1270":"GRUPO 2","1271":"GRUPO 2","1272":"GRUPO 3","1273":"GRUPO 3","1274":"GRUPO 3","1275":"GRUPO 3","1276":"GRUPO 3","1277":"GRUPO 3","1278":"GRUPO 3","1279":"GRUPO 3","1280":"GRUPO 3","1281":"GRUPO 3","1282":"GRUPO 3","1283":"GRUPO 3","1284":"GRUPO 4","1285":"GRUPO 4","1286":"GRUPO 4","1287":"GRUPO 4","1288":"GRUPO 4","1289":"GRUPO 4","1290":"GRUPO 4","1291":"GRUPO 4","1292":"GRUPO 4","1293":"GRUPO 4","1294":"GRUPO 4","1295":"GRUPO 4","1296":"GRUPO 1","1297":"GRUPO 1","1298":"GRUPO 1","1299":"GRUPO 1","1300":"GRUPO 1","1301":"GRUPO 1","1302":"GRUPO 1","1303":"GRUPO 1","1304":"GRUPO 1","1305":"GRUPO 1","1306":"GRUPO 1","1307":"GRUPO 1","1308":"GRUPO 2","1309":"GRUPO 2","1310":"GRUPO 2","1311":"GRUPO 2","1312":"GRUPO 2","1313":"GRUPO 2","1314":"GRUPO 2","1315":"GRUPO 2","1316":"GRUPO 2","1317":"GRUPO 2","1318":"GRUPO 2","1319":"GRUPO 2","1320":"GRUPO 3","1321":"GRUPO 3","1322":"GRUPO 3","1323":"GRUPO 3","1324":"GRUPO 3","1325":"GRUPO 3","1326":"GRUPO 3","1327":"GRUPO 3","1328":"GRUPO 3","1329":"GRUPO 3","1330":"GRUPO 3","1331":"GRUPO 3","1332":"GRUPO 4","1333":"GRUPO 4","1334":"GRUPO 4","1335":"GRUPO 4","1336":"GRUPO 4","1337":"GRUPO 4","1338":"GRUPO 4","1339":"GRUPO 4","1340":"GRUPO 4","1341":"GRUPO 4","1342":"GRUPO 4","1343":"GRUPO 4","1344":"GRUPO 1","1345":"GRUPO 1","1346":"GRUPO 1","1347":"GRUPO 1","1348":"GRUPO 1","1349":"GRUPO 1","1350":"GRUPO 1","1351":"GRUPO 1","1352":"GRUPO 1","1353":"GRUPO 1","1354":"GRUPO 1","1355":"GRUPO 1","1356":"GRUPO 2","1357":"GRUPO 2","1358":"GRUPO 2","1359":"GRUPO 2","1360":"GRUPO 2","1361":"GRUPO 2","1362":"GRUPO 2","1363":"GRUPO 2","1364":"GRUPO 2","1365":"GRUPO 2","1366":"GRUPO 2","1367":"GRUPO 2","1368":"GRUPO 3","1369":"GRUPO 3","1370":"GRUPO 3","1371":"GRUPO 3","1372":"GRUPO 3","1373":"GRUPO 3","1374":"GRUPO 3","1375":"GRUPO 3","1376":"GRUPO 3","1377":"GRUPO 3","1378":"GRUPO 3","1379":"GRUPO 3","1380":"GRUPO 4","1381":"GRUPO 4","1382":"GRUPO 4","1383":"GRUPO 4","1384":"GRUPO 4","1385":"GRUPO 4","1386":"GRUPO 4","1387":"GRUPO 4","1388":"GRUPO 4","1389":"GRUPO 4","1390":"GRUPO 4","1391":"GRUPO 4","1392":"GRUPO 1","1393":"GRUPO 1","1394":"GRUPO 1","1395":"GRUPO 1","1396":"GRUPO 1","1397":"GRUPO 1","1398":"GRUPO 1","1399":"GRUPO 1","1400":"GRUPO 1","1401":"GRUPO 1","1402":"GRUPO 1","1403":"GRUPO 1","1404":"GRUPO 2","1405":"GRUPO 2","1406":"GRUPO 2","1407":"GRUPO 2","1408":"GRUPO 2","1409":"GRUPO 2","1410":"GRUPO 2","1411":"GRUPO 2","1412":"GRUPO 2","1413":"GRUPO 2","1414":"GRUPO 2","1415":"GRUPO 2","1416":"GRUPO 3","1417":"GRUPO 3","1418":"GRUPO 3","1419":"GRUPO 3","1420":"GRUPO 3","1421":"GRUPO 3","1422":"GRUPO 3","1423":"GRUPO 3","1424":"GRUPO 3","1425":"GRUPO 3","1426":"GRUPO 3","1427":"GRUPO 3","1428":"GRUPO 4","1429":"GRUPO 4","1430":"GRUPO 4","1431":"GRUPO 4","1432":"GRUPO 4","1433":"GRUPO 4","1434":"GRUPO 4","1435":"GRUPO 4","1436":"GRUPO 4","1437":"GRUPO 4","1438":"GRUPO 4","1439":"GRUPO 4","1440":"GRUPO 1","1441":"GRUPO 1","1442":"GRUPO 1","1443":"GRUPO 1","1444":"GRUPO 1","1445":"GRUPO 1","1446":"GRUPO 1","1447":"GRUPO 1","1448":"GRUPO 1","1449":"GRUPO 1","1450":"GRUPO 1","1451":"GRUPO 1","1452":"GRUPO 2","1453":"GRUPO 2","1454":"GRUPO 2","1455":"GRUPO 2","1456":"GRUPO 2","1457":"GRUPO 2","1458":"GRUPO 2","1459":"GRUPO 2","1460":"GRUPO 2","1461":"GRUPO 2","1462":"GRUPO 2","1463":"GRUPO 2","1464":"GRUPO 3","1465":"GRUPO 3","1466":"GRUPO 3","1467":"GRUPO 3","1468":"GRUPO 3","1469":"GRUPO 3","1470":"GRUPO 3","1471":"GRUPO 3","1472":"GRUPO 3","1473":"GRUPO 3","1474":"GRUPO 3","1475":"GRUPO 3","1476":"GRUPO 4","1477":"GRUPO 4","1478":"GRUPO 4","1479":"GRUPO 4","1480":"GRUPO 4","1481":"GRUPO 4","1482":"GRUPO 4","1483":"GRUPO 4","1484":"GRUPO 4","1485":"GRUPO 4","1486":"GRUPO 4","1487":"GRUPO 4"},"Empleado":{"0":"BARON HERNANDEZ HAROLD ANTONIO","1":"CASTELLANOS CARVAJAL DEYVITH FABIAN","2":"AROCA TORRES JULIAN EDUARDO","3":"BERMUDEZ PARRA JENNIFER XIOMARA","4":"BERNAL BAQUERO JAMES RICARDO","5":"BURGOS ORTIZ JOSE HORACIO","6":"CANTOR PORRAS JUAN FERNEY","7":"CAPERA CAPERA JOSE GABRIEL","8":"CARDENAS LOTERO RICARDO ANDR\u00c9S","9":"RENDON OSPINA NELSON LEANDRO","10":"SARMIENTO URBINA MOISES DANIEL","11":"VELASCO VELASCO SEBASTI\u00c1N DAVID","12":"DELGADO DELGADO JOHAN DARIO","13":"FLOREZ SAUCESO KENIS ALBERTO","14":"CARDONA GARCIA OSCAR JAVIER","15":"CARVAJAL GARC\u00cdA HOVER MARCK","16":"CEPEDA PIRAQUIVE JUAN DAVID","17":"FAJARDO SAENZ OSCAR FERNANDO","18":"FLOREZ ESPITIA RONY ALBERTO","19":"GARCIA CUERVO EDWIN JAVIER","20":"GONZALEZ OCHOA JUAN CARLOS","21":"XXX1","22":"XXX2","23":"XXX3","24":"FONSECA RAY RICARDO","25":"GOMEZ BETANCUR JAIDER ANDRES","26":"GRANADA PATI\u00d1O CARLOS MARINO","27":"GRASS PLATA MIGUEL SNEIDER","28":"MANZANO CALVO JUAN SEBASTIAN","29":"MENDOZA GOITA MARIANSEL ZENAYDA","30":"MURILLO ARAQUE JAIVER GEOVANY","31":"NI\u00d1O ARENAS HECTOR GONZALO","32":"RAMIREZ CHAVERRA JHON EDISON","33":"XXX4","34":"XXX5","35":"XXX6","36":"RODRIGUEZ MOSQUERA LUIS FERNANDO","37":"PEPITO PEREZ","38":"RAMIREZ VARGAS MARCELA PAOLA","39":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","40":"TORO CISNEROS GARY JOSE","41":"USECHE CALDERON JADID ESTIVEN","42":"VASQUEZ NIETO CAMILO ANDRES","43":"JHONY CASTRO","44":"BERNAL JUAN DAVID","45":"XXX7","46":"XXX8","47":"XXX9","48":"BARON HERNANDEZ HAROLD ANTONIO","49":"CASTELLANOS CARVAJAL DEYVITH FABIAN","50":"AROCA TORRES JULIAN EDUARDO","51":"BERMUDEZ PARRA JENNIFER XIOMARA","52":"BERNAL BAQUERO JAMES RICARDO","53":"BURGOS ORTIZ JOSE HORACIO","54":"CANTOR PORRAS JUAN FERNEY","55":"CAPERA CAPERA JOSE GABRIEL","56":"CARDENAS LOTERO RICARDO ANDR\u00c9S","57":"RENDON OSPINA NELSON LEANDRO","58":"SARMIENTO URBINA MOISES DANIEL","59":"VELASCO VELASCO SEBASTI\u00c1N DAVID","60":"DELGADO DELGADO JOHAN DARIO","61":"FLOREZ SAUCESO KENIS ALBERTO","62":"CARDONA GARCIA OSCAR JAVIER","63":"CARVAJAL GARC\u00cdA HOVER MARCK","64":"CEPEDA PIRAQUIVE JUAN DAVID","65":"FAJARDO SAENZ OSCAR FERNANDO","66":"FLOREZ ESPITIA RONY ALBERTO","67":"GARCIA CUERVO EDWIN JAVIER","68":"GONZALEZ OCHOA JUAN CARLOS","69":"XXX1","70":"XXX2","71":"XXX3","72":"FONSECA RAY RICARDO","73":"GOMEZ BETANCUR JAIDER ANDRES","74":"GRANADA PATI\u00d1O CARLOS MARINO","75":"GRASS PLATA MIGUEL SNEIDER","76":"MANZANO CALVO JUAN SEBASTIAN","77":"MENDOZA GOITA MARIANSEL ZENAYDA","78":"MURILLO ARAQUE JAIVER GEOVANY","79":"NI\u00d1O ARENAS HECTOR GONZALO","80":"RAMIREZ CHAVERRA JHON EDISON","81":"XXX4","82":"XXX5","83":"XXX6","84":"RODRIGUEZ MOSQUERA LUIS FERNANDO","85":"PEPITO PEREZ","86":"RAMIREZ VARGAS MARCELA PAOLA","87":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","88":"TORO CISNEROS GARY JOSE","89":"USECHE CALDERON JADID ESTIVEN","90":"VASQUEZ NIETO CAMILO ANDRES","91":"JHONY CASTRO","92":"BERNAL JUAN DAVID","93":"XXX7","94":"XXX8","95":"XXX9","96":"BARON HERNANDEZ HAROLD ANTONIO","97":"CASTELLANOS CARVAJAL DEYVITH FABIAN","98":"AROCA TORRES JULIAN EDUARDO","99":"BERMUDEZ PARRA JENNIFER XIOMARA","100":"BERNAL BAQUERO JAMES RICARDO","101":"BURGOS ORTIZ JOSE HORACIO","102":"CANTOR PORRAS JUAN FERNEY","103":"CAPERA CAPERA JOSE GABRIEL","104":"CARDENAS LOTERO RICARDO ANDR\u00c9S","105":"RENDON OSPINA NELSON LEANDRO","106":"SARMIENTO URBINA MOISES DANIEL","107":"VELASCO VELASCO SEBASTI\u00c1N DAVID","108":"DELGADO DELGADO JOHAN DARIO","109":"FLOREZ SAUCESO KENIS ALBERTO","110":"CARDONA GARCIA OSCAR JAVIER","111":"CARVAJAL GARC\u00cdA HOVER MARCK","112":"CEPEDA PIRAQUIVE JUAN DAVID","113":"FAJARDO SAENZ OSCAR FERNANDO","114":"FLOREZ ESPITIA RONY ALBERTO","115":"GARCIA CUERVO EDWIN JAVIER","116":"GONZALEZ OCHOA JUAN CARLOS","117":"XXX1","118":"XXX2","119":"XXX3","120":"FONSECA RAY RICARDO","121":"GOMEZ BETANCUR JAIDER ANDRES","122":"GRANADA PATI\u00d1O CARLOS MARINO","123":"GRASS PLATA MIGUEL SNEIDER","124":"MANZANO CALVO JUAN SEBASTIAN","125":"MENDOZA GOITA MARIANSEL ZENAYDA","126":"MURILLO ARAQUE JAIVER GEOVANY","127":"NI\u00d1O ARENAS HECTOR GONZALO","128":"RAMIREZ CHAVERRA JHON EDISON","129":"XXX4","130":"XXX5","131":"XXX6","132":"RODRIGUEZ MOSQUERA LUIS FERNANDO","133":"PEPITO PEREZ","134":"RAMIREZ VARGAS MARCELA PAOLA","135":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","136":"TORO CISNEROS GARY JOSE","137":"USECHE CALDERON JADID ESTIVEN","138":"VASQUEZ NIETO CAMILO ANDRES","139":"JHONY CASTRO","140":"BERNAL JUAN DAVID","141":"XXX7","142":"XXX8","143":"XXX9","144":"BARON HERNANDEZ HAROLD ANTONIO","145":"CASTELLANOS CARVAJAL DEYVITH FABIAN","146":"AROCA TORRES JULIAN EDUARDO","147":"BERMUDEZ PARRA JENNIFER XIOMARA","148":"BERNAL BAQUERO JAMES RICARDO","149":"BURGOS ORTIZ JOSE HORACIO","150":"CANTOR PORRAS JUAN FERNEY","151":"CAPERA CAPERA JOSE GABRIEL","152":"CARDENAS LOTERO RICARDO ANDR\u00c9S","153":"RENDON OSPINA NELSON LEANDRO","154":"SARMIENTO URBINA MOISES DANIEL","155":"VELASCO VELASCO SEBASTI\u00c1N DAVID","156":"DELGADO DELGADO JOHAN DARIO","157":"FLOREZ SAUCESO KENIS ALBERTO","158":"CARDONA GARCIA OSCAR JAVIER","159":"CARVAJAL GARC\u00cdA HOVER MARCK","160":"CEPEDA PIRAQUIVE JUAN DAVID","161":"FAJARDO SAENZ OSCAR FERNANDO","162":"FLOREZ ESPITIA RONY ALBERTO","163":"GARCIA CUERVO EDWIN JAVIER","164":"GONZALEZ OCHOA JUAN CARLOS","165":"XXX1","166":"XXX2","167":"XXX3","168":"FONSECA RAY RICARDO","169":"GOMEZ BETANCUR JAIDER ANDRES","170":"GRANADA PATI\u00d1O CARLOS MARINO","171":"GRASS PLATA MIGUEL SNEIDER","172":"MANZANO CALVO JUAN SEBASTIAN","173":"MENDOZA GOITA MARIANSEL ZENAYDA","174":"MURILLO ARAQUE JAIVER GEOVANY","175":"NI\u00d1O ARENAS HECTOR GONZALO","176":"RAMIREZ CHAVERRA JHON EDISON","177":"XXX4","178":"XXX5","179":"XXX6","180":"RODRIGUEZ MOSQUERA LUIS FERNANDO","181":"PEPITO PEREZ","182":"RAMIREZ VARGAS MARCELA PAOLA","183":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","184":"TORO CISNEROS GARY JOSE","185":"USECHE CALDERON JADID ESTIVEN","186":"VASQUEZ NIETO CAMILO ANDRES","187":"JHONY CASTRO","188":"BERNAL JUAN DAVID","189":"XXX7","190":"XXX8","191":"XXX9","192":"BARON HERNANDEZ HAROLD ANTONIO","193":"CASTELLANOS CARVAJAL DEYVITH FABIAN","194":"AROCA TORRES JULIAN EDUARDO","195":"BERMUDEZ PARRA JENNIFER XIOMARA","196":"BERNAL BAQUERO JAMES RICARDO","197":"BURGOS ORTIZ JOSE HORACIO","198":"CANTOR PORRAS JUAN FERNEY","199":"CAPERA CAPERA JOSE GABRIEL","200":"CARDENAS LOTERO RICARDO ANDR\u00c9S","201":"RENDON OSPINA NELSON LEANDRO","202":"SARMIENTO URBINA MOISES DANIEL","203":"VELASCO VELASCO SEBASTI\u00c1N DAVID","204":"DELGADO DELGADO JOHAN DARIO","205":"FLOREZ SAUCESO KENIS ALBERTO","206":"CARDONA GARCIA OSCAR JAVIER","207":"CARVAJAL GARC\u00cdA HOVER MARCK","208":"CEPEDA PIRAQUIVE JUAN DAVID","209":"FAJARDO SAENZ OSCAR FERNANDO","210":"FLOREZ ESPITIA RONY ALBERTO","211":"GARCIA CUERVO EDWIN JAVIER","212":"GONZALEZ OCHOA JUAN CARLOS","213":"XXX1","214":"XXX2","215":"XXX3","216":"FONSECA RAY RICARDO","217":"GOMEZ BETANCUR JAIDER ANDRES","218":"GRANADA PATI\u00d1O CARLOS MARINO","219":"GRASS PLATA MIGUEL SNEIDER","220":"MANZANO CALVO JUAN SEBASTIAN","221":"MENDOZA GOITA MARIANSEL ZENAYDA","222":"MURILLO ARAQUE JAIVER GEOVANY","223":"NI\u00d1O ARENAS HECTOR GONZALO","224":"RAMIREZ CHAVERRA JHON EDISON","225":"XXX4","226":"XXX5","227":"XXX6","228":"RODRIGUEZ MOSQUERA LUIS FERNANDO","229":"PEPITO PEREZ","230":"RAMIREZ VARGAS MARCELA PAOLA","231":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","232":"TORO CISNEROS GARY JOSE","233":"USECHE CALDERON JADID ESTIVEN","234":"VASQUEZ NIETO CAMILO ANDRES","235":"JHONY CASTRO","236":"BERNAL JUAN DAVID","237":"XXX7","238":"XXX8","239":"XXX9","240":"BARON HERNANDEZ HAROLD ANTONIO","241":"CASTELLANOS CARVAJAL DEYVITH FABIAN","242":"AROCA TORRES JULIAN EDUARDO","243":"BERMUDEZ PARRA JENNIFER XIOMARA","244":"BERNAL BAQUERO JAMES RICARDO","245":"BURGOS ORTIZ JOSE HORACIO","246":"CANTOR PORRAS JUAN FERNEY","247":"CAPERA CAPERA JOSE GABRIEL","248":"CARDENAS LOTERO RICARDO ANDR\u00c9S","249":"RENDON OSPINA NELSON LEANDRO","250":"SARMIENTO URBINA MOISES DANIEL","251":"VELASCO VELASCO SEBASTI\u00c1N DAVID","252":"DELGADO DELGADO JOHAN DARIO","253":"FLOREZ SAUCESO KENIS ALBERTO","254":"CARDONA GARCIA OSCAR JAVIER","255":"CARVAJAL GARC\u00cdA HOVER MARCK","256":"CEPEDA PIRAQUIVE JUAN DAVID","257":"FAJARDO SAENZ OSCAR FERNANDO","258":"FLOREZ ESPITIA RONY ALBERTO","259":"GARCIA CUERVO EDWIN JAVIER","260":"GONZALEZ OCHOA JUAN CARLOS","261":"XXX1","262":"XXX2","263":"XXX3","264":"FONSECA RAY RICARDO","265":"GOMEZ BETANCUR JAIDER ANDRES","266":"GRANADA PATI\u00d1O CARLOS MARINO","267":"GR</t>
+    <t>24/04/2026 21:35</t>
   </si>
   <si>
     <t>{"Grupo":{"0":"GRUPO 1","1":"GRUPO 1","2":"GRUPO 1","3":"GRUPO 1","4":"GRUPO 1","5":"GRUPO 1","6":"GRUPO 1","7":"GRUPO 1","8":"GRUPO 1","9":"GRUPO 1","10":"GRUPO 1","11":"GRUPO 1","12":"GRUPO 2","13":"GRUPO 2","14":"GRUPO 2","15":"GRUPO 2","16":"GRUPO 2","17":"GRUPO 2","18":"GRUPO 2","19":"GRUPO 2","20":"GRUPO 2","21":"GRUPO 2","22":"GRUPO 2","23":"GRUPO 2","24":"GRUPO 3","25":"GRUPO 3","26":"GRUPO 3","27":"GRUPO 3","28":"GRUPO 3","29":"GRUPO 3","30":"GRUPO 3","31":"GRUPO 3","32":"GRUPO 3","33":"GRUPO 3","34":"GRUPO 3","35":"GRUPO 3","36":"GRUPO 4","37":"GRUPO 4","38":"GRUPO 4","39":"GRUPO 4","40":"GRUPO 4","41":"GRUPO 4","42":"GRUPO 4","43":"GRUPO 4","44":"GRUPO 4","45":"GRUPO 4","46":"GRUPO 4","47":"GRUPO 4","48":"GRUPO 1","49":"GRUPO 1","50":"GRUPO 1","51":"GRUPO 1","52":"GRUPO 1","53":"GRUPO 1","54":"GRUPO 1","55":"GRUPO 1","56":"GRUPO 1","57":"GRUPO 1","58":"GRUPO 1","59":"GRUPO 1","60":"GRUPO 2","61":"GRUPO 2","62":"GRUPO 2","63":"GRUPO 2","64":"GRUPO 2","65":"GRUPO 2","66":"GRUPO 2","67":"GRUPO 2","68":"GRUPO 2","69":"GRUPO 2","70":"GRUPO 2","71":"GRUPO 2","72":"GRUPO 3","73":"GRUPO 3","74":"GRUPO 3","75":"GRUPO 3","76":"GRUPO 3","77":"GRUPO 3","78":"GRUPO 3","79":"GRUPO 3","80":"GRUPO 3","81":"GRUPO 3","82":"GRUPO 3","83":"GRUPO 3","84":"GRUPO 4","85":"GRUPO 4","86":"GRUPO 4","87":"GRUPO 4","88":"GRUPO 4","89":"GRUPO 4","90":"GRUPO 4","91":"GRUPO 4","92":"GRUPO 4","93":"GRUPO 4","94":"GRUPO 4","95":"GRUPO 4","96":"GRUPO 1","97":"GRUPO 1","98":"GRUPO 1","99":"GRUPO 1","100":"GRUPO 1","101":"GRUPO 1","102":"GRUPO 1","103":"GRUPO 1","104":"GRUPO 1","105":"GRUPO 1","106":"GRUPO 1","107":"GRUPO 1","108":"GRUPO 2","109":"GRUPO 2","110":"GRUPO 2","111":"GRUPO 2","112":"GRUPO 2","113":"GRUPO 2","114":"GRUPO 2","115":"GRUPO 2","116":"GRUPO 2","117":"GRUPO 2","118":"GRUPO 2","119":"GRUPO 2","120":"GRUPO 3","121":"GRUPO 3","122":"GRUPO 3","123":"GRUPO 3","124":"GRUPO 3","125":"GRUPO 3","126":"GRUPO 3","127":"GRUPO 3","128":"GRUPO 3","129":"GRUPO 3","130":"GRUPO 3","131":"GRUPO 3","132":"GRUPO 4","133":"GRUPO 4","134":"GRUPO 4","135":"GRUPO 4","136":"GRUPO 4","137":"GRUPO 4","138":"GRUPO 4","139":"GRUPO 4","140":"GRUPO 4","141":"GRUPO 4","142":"GRUPO 4","143":"GRUPO 4","144":"GRUPO 1","145":"GRUPO 1","146":"GRUPO 1","147":"GRUPO 1","148":"GRUPO 1","149":"GRUPO 1","150":"GRUPO 1","151":"GRUPO 1","152":"GRUPO 1","153":"GRUPO 1","154":"GRUPO 1","155":"GRUPO 1","156":"GRUPO 2","157":"GRUPO 2","158":"GRUPO 2","159":"GRUPO 2","160":"GRUPO 2","161":"GRUPO 2","162":"GRUPO 2","163":"GRUPO 2","164":"GRUPO 2","165":"GRUPO 2","166":"GRUPO 2","167":"GRUPO 2","168":"GRUPO 3","169":"GRUPO 3","170":"GRUPO 3","171":"GRUPO 3","172":"GRUPO 3","173":"GRUPO 3","174":"GRUPO 3","175":"GRUPO 3","176":"GRUPO 3","177":"GRUPO 3","178":"GRUPO 3","179":"GRUPO 3","180":"GRUPO 4","181":"GRUPO 4","182":"GRUPO 4","183":"GRUPO 4","184":"GRUPO 4","185":"GRUPO 4","186":"GRUPO 4","187":"GRUPO 4","188":"GRUPO 4","189":"GRUPO 4","190":"GRUPO 4","191":"GRUPO 4","192":"GRUPO 1","193":"GRUPO 1","194":"GRUPO 1","195":"GRUPO 1","196":"GRUPO 1","197":"GRUPO 1","198":"GRUPO 1","199":"GRUPO 1","200":"GRUPO 1","201":"GRUPO 1","202":"GRUPO 1","203":"GRUPO 1","204":"GRUPO 2","205":"GRUPO 2","206":"GRUPO 2","207":"GRUPO 2","208":"GRUPO 2","209":"GRUPO 2","210":"GRUPO 2","211":"GRUPO 2","212":"GRUPO 2","213":"GRUPO 2","214":"GRUPO 2","215":"GRUPO 2","216":"GRUPO 3","217":"GRUPO 3","218":"GRUPO 3","219":"GRUPO 3","220":"GRUPO 3","221":"GRUPO 3","222":"GRUPO 3","223":"GRUPO 3","224":"GRUPO 3","225":"GRUPO 3","226":"GRUPO 3","227":"GRUPO 3","228":"GRUPO 4","229":"GRUPO 4","230":"GRUPO 4","231":"GRUPO 4","232":"GRUPO 4","233":"GRUPO 4","234":"GRUPO 4","235":"GRUPO 4","236":"GRUPO 4","237":"GRUPO 4","238":"GRUPO 4","239":"GRUPO 4","240":"GRUPO 1","241":"GRUPO 1","242":"GRUPO 1","243":"GRUPO 1","244":"GRUPO 1","245":"GRUPO 1","246":"GRUPO 1","247":"GRUPO 1","248":"GRUPO 1","249":"GRUPO 1","250":"GRUPO 1","251":"GRUPO 1","252":"GRUPO 2","253":"GRUPO 2","254":"GRUPO 2","255":"GRUPO 2","256":"GRUPO 2","257":"GRUPO 2","258":"GRUPO 2","259":"GRUPO 2","260":"GRUPO 2","261":"GRUPO 2","262":"GRUPO 2","263":"GRUPO 2","264":"GRUPO 3","265":"GRUPO 3","266":"GRUPO 3","267":"GRUPO 3","268":"GRUPO 3","269":"GRUPO 3","270":"GRUPO 3","271":"GRUPO 3","272":"GRUPO 3","273":"GRUPO 3","274":"GRUPO 3","275":"GRUPO 3","276":"GRUPO 4","277":"GRUPO 4","278":"GRUPO 4","279":"GRUPO 4","280":"GRUPO 4","281":"GRUPO 4","282":"GRUPO 4","283":"GRUPO 4","284":"GRUPO 4","285":"GRUPO 4","286":"GRUPO 4","287":"GRUPO 4","288":"GRUPO 1","289":"GRUPO 1","290":"GRUPO 1","291":"GRUPO 1","292":"GRUPO 1","293":"GRUPO 1","294":"GRUPO 1","295":"GRUPO 1","296":"GRUPO 1","297":"GRUPO 1","298":"GRUPO 1","299":"GRUPO 1","300":"GRUPO 2","301":"GRUPO 2","302":"GRUPO 2","303":"GRUPO 2","304":"GRUPO 2","305":"GRUPO 2","306":"GRUPO 2","307":"GRUPO 2","308":"GRUPO 2","309":"GRUPO 2","310":"GRUPO 2","311":"GRUPO 2","312":"GRUPO 3","313":"GRUPO 3","314":"GRUPO 3","315":"GRUPO 3","316":"GRUPO 3","317":"GRUPO 3","318":"GRUPO 3","319":"GRUPO 3","320":"GRUPO 3","321":"GRUPO 3","322":"GRUPO 3","323":"GRUPO 3","324":"GRUPO 4","325":"GRUPO 4","326":"GRUPO 4","327":"GRUPO 4","328":"GRUPO 4","329":"GRUPO 4","330":"GRUPO 4","331":"GRUPO 4","332":"GRUPO 4","333":"GRUPO 4","334":"GRUPO 4","335":"GRUPO 4","336":"GRUPO 1","337":"GRUPO 1","338":"GRUPO 1","339":"GRUPO 1","340":"GRUPO 1","341":"GRUPO 1","342":"GRUPO 1","343":"GRUPO 1","344":"GRUPO 1","345":"GRUPO 1","346":"GRUPO 1","347":"GRUPO 1","348":"GRUPO 2","349":"GRUPO 2","350":"GRUPO 2","351":"GRUPO 2","352":"GRUPO 2","353":"GRUPO 2","354":"GRUPO 2","355":"GRUPO 2","356":"GRUPO 2","357":"GRUPO 2","358":"GRUPO 2","359":"GRUPO 2","360":"GRUPO 3","361":"GRUPO 3","362":"GRUPO 3","363":"GRUPO 3","364":"GRUPO 3","365":"GRUPO 3","366":"GRUPO 3","367":"GRUPO 3","368":"GRUPO 3","369":"GRUPO 3","370":"GRUPO 3","371":"GRUPO 3","372":"GRUPO 4","373":"GRUPO 4","374":"GRUPO 4","375":"GRUPO 4","376":"GRUPO 4","377":"GRUPO 4","378":"GRUPO 4","379":"GRUPO 4","380":"GRUPO 4","381":"GRUPO 4","382":"GRUPO 4","383":"GRUPO 4","384":"GRUPO 1","385":"GRUPO 1","386":"GRUPO 1","387":"GRUPO 1","388":"GRUPO 1","389":"GRUPO 1","390":"GRUPO 1","391":"GRUPO 1","392":"GRUPO 1","393":"GRUPO 1","394":"GRUPO 1","395":"GRUPO 1","396":"GRUPO 2","397":"GRUPO 2","398":"GRUPO 2","399":"GRUPO 2","400":"GRUPO 2","401":"GRUPO 2","402":"GRUPO 2","403":"GRUPO 2","404":"GRUPO 2","405":"GRUPO 2","406":"GRUPO 2","407":"GRUPO 2","408":"GRUPO 3","409":"GRUPO 3","410":"GRUPO 3","411":"GRUPO 3","412":"GRUPO 3","413":"GRUPO 3","414":"GRUPO 3","415":"GRUPO 3","416":"GRUPO 3","417":"GRUPO 3","418":"GRUPO 3","419":"GRUPO 3","420":"GRUPO 4","421":"GRUPO 4","422":"GRUPO 4","423":"GRUPO 4","424":"GRUPO 4","425":"GRUPO 4","426":"GRUPO 4","427":"GRUPO 4","428":"GRUPO 4","429":"GRUPO 4","430":"GRUPO 4","431":"GRUPO 4","432":"GRUPO 1","433":"GRUPO 1","434":"GRUPO 1","435":"GRUPO 1","436":"GRUPO 1","437":"GRUPO 1","438":"GRUPO 1","439":"GRUPO 1","440":"GRUPO 1","441":"GRUPO 1","442":"GRUPO 1","443":"GRUPO 1","444":"GRUPO 2","445":"GRUPO 2","446":"GRUPO 2","447":"GRUPO 2","448":"GRUPO 2","449":"GRUPO 2","450":"GRUPO 2","451":"GRUPO 2","452":"GRUPO 2","453":"GRUPO 2","454":"GRUPO 2","455":"GRUPO 2","456":"GRUPO 3","457":"GRUPO 3","458":"GRUPO 3","459":"GRUPO 3","460":"GRUPO 3","461":"GRUPO 3","462":"GRUPO 3","463":"GRUPO 3","464":"GRUPO 3","465":"GRUPO 3","466":"GRUPO 3","467":"GRUPO 3","468":"GRUPO 4","469":"GRUPO 4","470":"GRUPO 4","471":"GRUPO 4","472":"GRUPO 4","473":"GRUPO 4","474":"GRUPO 4","475":"GRUPO 4","476":"GRUPO 4","477":"GRUPO 4","478":"GRUPO 4","479":"GRUPO 4","480":"GRUPO 1","481":"GRUPO 1","482":"GRUPO 1","483":"GRUPO 1","484":"GRUPO 1","485":"GRUPO 1","486":"GRUPO 1","487":"GRUPO 1","488":"GRUPO 1","489":"GRUPO 1","490":"GRUPO 1","491":"GRUPO 1","492":"GRUPO 2","493":"GRUPO 2","494":"GRUPO 2","495":"GRUPO 2","496":"GRUPO 2","497":"GRUPO 2","498":"GRUPO 2","499":"GRUPO 2","500":"GRUPO 2","501":"GRUPO 2","502":"GRUPO 2","503":"GRUPO 2","504":"GRUPO 3","505":"GRUPO 3","506":"GRUPO 3","507":"GRUPO 3","508":"GRUPO 3","509":"GRUPO 3","510":"GRUPO 3","511":"GRUPO 3","512":"GRUPO 3","513":"GRUPO 3","514":"GRUPO 3","515":"GRUPO 3","516":"GRUPO 4","517":"GRUPO 4","518":"GRUPO 4","519":"GRUPO 4","520":"GRUPO 4","521":"GRUPO 4","522":"GRUPO 4","523":"GRUPO 4","524":"GRUPO 4","525":"GRUPO 4","526":"GRUPO 4","527":"GRUPO 4","528":"GRUPO 1","529":"GRUPO 1","530":"GRUPO 1","531":"GRUPO 1","532":"GRUPO 1","533":"GRUPO 1","534":"GRUPO 1","535":"GRUPO 1","536":"GRUPO 1","537":"GRUPO 1","538":"GRUPO 1","539":"GRUPO 1","540":"GRUPO 2","541":"GRUPO 2","542":"GRUPO 2","543":"GRUPO 2","544":"GRUPO 2","545":"GRUPO 2","546":"GRUPO 2","547":"GRUPO 2","548":"GRUPO 2","549":"GRUPO 2","550":"GRUPO 2","551":"GRUPO 2","552":"GRUPO 3","553":"GRUPO 3","554":"GRUPO 3","555":"GRUPO 3","556":"GRUPO 3","557":"GRUPO 3","558":"GRUPO 3","559":"GRUPO 3","560":"GRUPO 3","561":"GRUPO 3","562":"GRUPO 3","563":"GRUPO 3","564":"GRUPO 4","565":"GRUPO 4","566":"GRUPO 4","567":"GRUPO 4","568":"GRUPO 4","569":"GRUPO 4","570":"GRUPO 4","571":"GRUPO 4","572":"GRUPO 4","573":"GRUPO 4","574":"GRUPO 4","575":"GRUPO 4","576":"GRUPO 1","577":"GRUPO 1","578":"GRUPO 1","579":"GRUPO 1","580":"GRUPO 1","581":"GRUPO 1","582":"GRUPO 1","583":"GRUPO 1","584":"GRUPO 1","585":"GRUPO 1","586":"GRUPO 1","587":"GRUPO 1","588":"GRUPO 2","589":"GRUPO 2","590":"GRUPO 2","591":"GRUPO 2","592":"GRUPO 2","593":"GRUPO 2","594":"GRUPO 2","595":"GRUPO 2","596":"GRUPO 2","597":"GRUPO 2","598":"GRUPO 2","599":"GRUPO 2","600":"GRUPO 3","601":"GRUPO 3","602":"GRUPO 3","603":"GRUPO 3","604":"GRUPO 3","605":"GRUPO 3","606":"GRUPO 3","607":"GRUPO 3","608":"GRUPO 3","609":"GRUPO 3","610":"GRUPO 3","611":"GRUPO 3","612":"GRUPO 4","613":"GRUPO 4","614":"GRUPO 4","615":"GRUPO 4","616":"GRUPO 4","617":"GRUPO 4","618":"GRUPO 4","619":"GRUPO 4","620":"GRUPO 4","621":"GRUPO 4","622":"GRUPO 4","623":"GRUPO 4","624":"GRUPO 1","625":"GRUPO 1","626":"GRUPO 1","627":"GRUPO 1","628":"GRUPO 1","629":"GRUPO 1","630":"GRUPO 1","631":"GRUPO 1","632":"GRUPO 1","633":"GRUPO 1","634":"GRUPO 1","635":"GRUPO 1","636":"GRUPO 2","637":"GRUPO 2","638":"GRUPO 2","639":"GRUPO 2","640":"GRUPO 2","641":"GRUPO 2","642":"GRUPO 2","643":"GRUPO 2","644":"GRUPO 2","645":"GRUPO 2","646":"GRUPO 2","647":"GRUPO 2","648":"GRUPO 3","649":"GRUPO 3","650":"GRUPO 3","651":"GRUPO 3","652":"GRUPO 3","653":"GRUPO 3","654":"GRUPO 3","655":"GRUPO 3","656":"GRUPO 3","657":"GRUPO 3","658":"GRUPO 3","659":"GRUPO 3","660":"GRUPO 4","661":"GRUPO 4","662":"GRUPO 4","663":"GRUPO 4","664":"GRUPO 4","665":"GRUPO 4","666":"GRUPO 4","667":"GRUPO 4","668":"GRUPO 4","669":"GRUPO 4","670":"GRUPO 4","671":"GRUPO 4","672":"GRUPO 1","673":"GRUPO 1","674":"GRUPO 1","675":"GRUPO 1","676":"GRUPO 1","677":"GRUPO 1","678":"GRUPO 1","679":"GRUPO 1","680":"GRUPO 1","681":"GRUPO 1","682":"GRUPO 1","683":"GRUPO 1","684":"GRUPO 2","685":"GRUPO 2","686":"GRUPO 2","687":"GRUPO 2","688":"GRUPO 2","689":"GRUPO 2","690":"GRUPO 2","691":"GRUPO 2","692":"GRUPO 2","693":"GRUPO 2","694":"GRUPO 2","695":"GRUPO 2","696":"GRUPO 3","697":"GRUPO 3","698":"GRUPO 3","699":"GRUPO 3","700":"GRUPO 3","701":"GRUPO 3","702":"GRUPO 3","703":"GRUPO 3","704":"GRUPO 3","705":"GRUPO 3","706":"GRUPO 3","707":"GRUPO 3","708":"GRUPO 4","709":"GRUPO 4","710":"GRUPO 4","711":"GRUPO 4","712":"GRUPO 4","713":"GRUPO 4","714":"GRUPO 4","715":"GRUPO 4","716":"GRUPO 4","717":"GRUPO 4","718":"GRUPO 4","719":"GRUPO 4","720":"GRUPO 1","721":"GRUPO 1","722":"GRUPO 1","723":"GRUPO 1","724":"GRUPO 1","725":"GRUPO 1","726":"GRUPO 1","727":"GRUPO 1","728":"GRUPO 1","729":"GRUPO 1","730":"GRUPO 1","731":"GRUPO 1","732":"GRUPO 2","733":"GRUPO 2","734":"GRUPO 2","735":"GRUPO 2","736":"GRUPO 2","737":"GRUPO 2","738":"GRUPO 2","739":"GRUPO 2","740":"GRUPO 2","741":"GRUPO 2","742":"GRUPO 2","743":"GRUPO 2","744":"GRUPO 3","745":"GRUPO 3","746":"GRUPO 3","747":"GRUPO 3","748":"GRUPO 3","749":"GRUPO 3","750":"GRUPO 3","751":"GRUPO 3","752":"GRUPO 3","753":"GRUPO 3","754":"GRUPO 3","755":"GRUPO 3","756":"GRUPO 4","757":"GRUPO 4","758":"GRUPO 4","759":"GRUPO 4","760":"GRUPO 4","761":"GRUPO 4","762":"GRUPO 4","763":"GRUPO 4","764":"GRUPO 4","765":"GRUPO 4","766":"GRUPO 4","767":"GRUPO 4","768":"GRUPO 1","769":"GRUPO 1","770":"GRUPO 1","771":"GRUPO 1","772":"GRUPO 1","773":"GRUPO 1","774":"GRUPO 1","775":"GRUPO 1","776":"GRUPO 1","777":"GRUPO 1","778":"GRUPO 1","779":"GRUPO 1","780":"GRUPO 2","781":"GRUPO 2","782":"GRUPO 2","783":"GRUPO 2","784":"GRUPO 2","785":"GRUPO 2","786":"GRUPO 2","787":"GRUPO 2","788":"GRUPO 2","789":"GRUPO 2","790":"GRUPO 2","791":"GRUPO 2","792":"GRUPO 3","793":"GRUPO 3","794":"GRUPO 3","795":"GRUPO 3","796":"GRUPO 3","797":"GRUPO 3","798":"GRUPO 3","799":"GRUPO 3","800":"GRUPO 3","801":"GRUPO 3","802":"GRUPO 3","803":"GRUPO 3","804":"GRUPO 4","805":"GRUPO 4","806":"GRUPO 4","807":"GRUPO 4","808":"GRUPO 4","809":"GRUPO 4","810":"GRUPO 4","811":"GRUPO 4","812":"GRUPO 4","813":"GRUPO 4","814":"GRUPO 4","815":"GRUPO 4","816":"GRUPO 1","817":"GRUPO 1","818":"GRUPO 1","819":"GRUPO 1","820":"GRUPO 1","821":"GRUPO 1","822":"GRUPO 1","823":"GRUPO 1","824":"GRUPO 1","825":"GRUPO 1","826":"GRUPO 1","827":"GRUPO 1","828":"GRUPO 2","829":"GRUPO 2","830":"GRUPO 2","831":"GRUPO 2","832":"GRUPO 2","833":"GRUPO 2","834":"GRUPO 2","835":"GRUPO 2","836":"GRUPO 2","837":"GRUPO 2","838":"GRUPO 2","839":"GRUPO 2","840":"GRUPO 3","841":"GRUPO 3","842":"GRUPO 3","843":"GRUPO 3","844":"GRUPO 3","845":"GRUPO 3","846":"GRUPO 3","847":"GRUPO 3","848":"GRUPO 3","849":"GRUPO 3","850":"GRUPO 3","851":"GRUPO 3","852":"GRUPO 4","853":"GRUPO 4","854":"GRUPO 4","855":"GRUPO 4","856":"GRUPO 4","857":"GRUPO 4","858":"GRUPO 4","859":"GRUPO 4","860":"GRUPO 4","861":"GRUPO 4","862":"GRUPO 4","863":"GRUPO 4","864":"GRUPO 1","865":"GRUPO 1","866":"GRUPO 1","867":"GRUPO 1","868":"GRUPO 1","869":"GRUPO 1","870":"GRUPO 1","871":"GRUPO 1","872":"GRUPO 1","873":"GRUPO 1","874":"GRUPO 1","875":"GRUPO 1","876":"GRUPO 2","877":"GRUPO 2","878":"GRUPO 2","879":"GRUPO 2","880":"GRUPO 2","881":"GRUPO 2","882":"GRUPO 2","883":"GRUPO 2","884":"GRUPO 2","885":"GRUPO 2","886":"GRUPO 2","887":"GRUPO 2","888":"GRUPO 3","889":"GRUPO 3","890":"GRUPO 3","891":"GRUPO 3","892":"GRUPO 3","893":"GRUPO 3","894":"GRUPO 3","895":"GRUPO 3","896":"GRUPO 3","897":"GRUPO 3","898":"GRUPO 3","899":"GRUPO 3","900":"GRUPO 4","901":"GRUPO 4","902":"GRUPO 4","903":"GRUPO 4","904":"GRUPO 4","905":"GRUPO 4","906":"GRUPO 4","907":"GRUPO 4","908":"GRUPO 4","909":"GRUPO 4","910":"GRUPO 4","911":"GRUPO 4","912":"GRUPO 1","913":"GRUPO 1","914":"GRUPO 1","915":"GRUPO 1","916":"GRUPO 1","917":"GRUPO 1","918":"GRUPO 1","919":"GRUPO 1","920":"GRUPO 1","921":"GRUPO 1","922":"GRUPO 1","923":"GRUPO 1","924":"GRUPO 2","925":"GRUPO 2","926":"GRUPO 2","927":"GRUPO 2","928":"GRUPO 2","929":"GRUPO 2","930":"GRUPO 2","931":"GRUPO 2","932":"GRUPO 2","933":"GRUPO 2","934":"GRUPO 2","935":"GRUPO 2","936":"GRUPO 3","937":"GRUPO 3","938":"GRUPO 3","939":"GRUPO 3","940":"GRUPO 3","941":"GRUPO 3","942":"GRUPO 3","943":"GRUPO 3","944":"GRUPO 3","945":"GRUPO 3","946":"GRUPO 3","947":"GRUPO 3","948":"GRUPO 4","949":"GRUPO 4","950":"GRUPO 4","951":"GRUPO 4","952":"GRUPO 4","953":"GRUPO 4","954":"GRUPO 4","955":"GRUPO 4","956":"GRUPO 4","957":"GRUPO 4","958":"GRUPO 4","959":"GRUPO 4","960":"GRUPO 1","961":"GRUPO 1","962":"GRUPO 1","963":"GRUPO 1","964":"GRUPO 1","965":"GRUPO 1","966":"GRUPO 1","967":"GRUPO 1","968":"GRUPO 1","969":"GRUPO 1","970":"GRUPO 1","971":"GRUPO 1","972":"GRUPO 2","973":"GRUPO 2","974":"GRUPO 2","975":"GRUPO 2","976":"GRUPO 2","977":"GRUPO 2","978":"GRUPO 2","979":"GRUPO 2","980":"GRUPO 2","981":"GRUPO 2","982":"GRUPO 2","983":"GRUPO 2","984":"GRUPO 3","985":"GRUPO 3","986":"GRUPO 3","987":"GRUPO 3","988":"GRUPO 3","989":"GRUPO 3","990":"GRUPO 3","991":"GRUPO 3","992":"GRUPO 3","993":"GRUPO 3","994":"GRUPO 3","995":"GRUPO 3","996":"GRUPO 4","997":"GRUPO 4","998":"GRUPO 4","999":"GRUPO 4","1000":"GRUPO 4","1001":"GRUPO 4","1002":"GRUPO 4","1003":"GRUPO 4","1004":"GRUPO 4","1005":"GRUPO 4","1006":"GRUPO 4","1007":"GRUPO 4","1008":"GRUPO 1","1009":"GRUPO 1","1010":"GRUPO 1","1011":"GRUPO 1","1012":"GRUPO 1","1013":"GRUPO 1","1014":"GRUPO 1","1015":"GRUPO 1","1016":"GRUPO 1","1017":"GRUPO 1","1018":"GRUPO 1","1019":"GRUPO 1","1020":"GRUPO 2","1021":"GRUPO 2","1022":"GRUPO 2","1023":"GRUPO 2","1024":"GRUPO 2","1025":"GRUPO 2","1026":"GRUPO 2","1027":"GRUPO 2","1028":"GRUPO 2","1029":"GRUPO 2","1030":"GRUPO 2","1031":"GRUPO 2","1032":"GRUPO 3","1033":"GRUPO 3","1034":"GRUPO 3","1035":"GRUPO 3","1036":"GRUPO 3","1037":"GRUPO 3","1038":"GRUPO 3","1039":"GRUPO 3","1040":"GRUPO 3","1041":"GRUPO 3","1042":"GRUPO 3","1043":"GRUPO 3","1044":"GRUPO 4","1045":"GRUPO 4","1046":"GRUPO 4","1047":"GRUPO 4","1048":"GRUPO 4","1049":"GRUPO 4","1050":"GRUPO 4","1051":"GRUPO 4","1052":"GRUPO 4","1053":"GRUPO 4","1054":"GRUPO 4","1055":"GRUPO 4","1056":"GRUPO 1","1057":"GRUPO 1","1058":"GRUPO 1","1059":"GRUPO 1","1060":"GRUPO 1","1061":"GRUPO 1","1062":"GRUPO 1","1063":"GRUPO 1","1064":"GRUPO 1","1065":"GRUPO 1","1066":"GRUPO 1","1067":"GRUPO 1","1068":"GRUPO 2","1069":"GRUPO 2","1070":"GRUPO 2","1071":"GRUPO 2","1072":"GRUPO 2","1073":"GRUPO 2","1074":"GRUPO 2","1075":"GRUPO 2","1076":"GRUPO 2","1077":"GRUPO 2","1078":"GRUPO 2","1079":"GRUPO 2","1080":"GRUPO 3","1081":"GRUPO 3","1082":"GRUPO 3","1083":"GRUPO 3","1084":"GRUPO 3","1085":"GRUPO 3","1086":"GRUPO 3","1087":"GRUPO 3","1088":"GRUPO 3","1089":"GRUPO 3","1090":"GRUPO 3","1091":"GRUPO 3","1092":"GRUPO 4","1093":"GRUPO 4","1094":"GRUPO 4","1095":"GRUPO 4","1096":"GRUPO 4","1097":"GRUPO 4","1098":"GRUPO 4","1099":"GRUPO 4","1100":"GRUPO 4","1101":"GRUPO 4","1102":"GRUPO 4","1103":"GRUPO 4","1104":"GRUPO 1","1105":"GRUPO 1","1106":"GRUPO 1","1107":"GRUPO 1","1108":"GRUPO 1","1109":"GRUPO 1","1110":"GRUPO 1","1111":"GRUPO 1","1112":"GRUPO 1","1113":"GRUPO 1","1114":"GRUPO 1","1115":"GRUPO 1","1116":"GRUPO 2","1117":"GRUPO 2","1118":"GRUPO 2","1119":"GRUPO 2","1120":"GRUPO 2","1121":"GRUPO 2","1122":"GRUPO 2","1123":"GRUPO 2","1124":"GRUPO 2","1125":"GRUPO 2","1126":"GRUPO 2","1127":"GRUPO 2","1128":"GRUPO 3","1129":"GRUPO 3","1130":"GRUPO 3","1131":"GRUPO 3","1132":"GRUPO 3","1133":"GRUPO 3","1134":"GRUPO 3","1135":"GRUPO 3","1136":"GRUPO 3","1137":"GRUPO 3","1138":"GRUPO 3","1139":"GRUPO 3","1140":"GRUPO 4","1141":"GRUPO 4","1142":"GRUPO 4","1143":"GRUPO 4","1144":"GRUPO 4","1145":"GRUPO 4","1146":"GRUPO 4","1147":"GRUPO 4","1148":"GRUPO 4","1149":"GRUPO 4","1150":"GRUPO 4","1151":"GRUPO 4","1152":"GRUPO 1","1153":"GRUPO 1","1154":"GRUPO 1","1155":"GRUPO 1","1156":"GRUPO 1","1157":"GRUPO 1","1158":"GRUPO 1","1159":"GRUPO 1","1160":"GRUPO 1","1161":"GRUPO 1","1162":"GRUPO 1","1163":"GRUPO 1","1164":"GRUPO 2","1165":"GRUPO 2","1166":"GRUPO 2","1167":"GRUPO 2","1168":"GRUPO 2","1169":"GRUPO 2","1170":"GRUPO 2","1171":"GRUPO 2","1172":"GRUPO 2","1173":"GRUPO 2","1174":"GRUPO 2","1175":"GRUPO 2","1176":"GRUPO 3","1177":"GRUPO 3","1178":"GRUPO 3","1179":"GRUPO 3","1180":"GRUPO 3","1181":"GRUPO 3","1182":"GRUPO 3","1183":"GRUPO 3","1184":"GRUPO 3","1185":"GRUPO 3","1186":"GRUPO 3","1187":"GRUPO 3","1188":"GRUPO 4","1189":"GRUPO 4","1190":"GRUPO 4","1191":"GRUPO 4","1192":"GRUPO 4","1193":"GRUPO 4","1194":"GRUPO 4","1195":"GRUPO 4","1196":"GRUPO 4","1197":"GRUPO 4","1198":"GRUPO 4","1199":"GRUPO 4","1200":"GRUPO 1","1201":"GRUPO 1","1202":"GRUPO 1","1203":"GRUPO 1","1204":"GRUPO 1","1205":"GRUPO 1","1206":"GRUPO 1","1207":"GRUPO 1","1208":"GRUPO 1","1209":"GRUPO 1","1210":"GRUPO 1","1211":"GRUPO 1","1212":"GRUPO 2","1213":"GRUPO 2","1214":"GRUPO 2","1215":"GRUPO 2","1216":"GRUPO 2","1217":"GRUPO 2","1218":"GRUPO 2","1219":"GRUPO 2","1220":"GRUPO 2","1221":"GRUPO 2","1222":"GRUPO 2","1223":"GRUPO 2","1224":"GRUPO 3","1225":"GRUPO 3","1226":"GRUPO 3","1227":"GRUPO 3","1228":"GRUPO 3","1229":"GRUPO 3","1230":"GRUPO 3","1231":"GRUPO 3","1232":"GRUPO 3","1233":"GRUPO 3","1234":"GRUPO 3","1235":"GRUPO 3","1236":"GRUPO 4","1237":"GRUPO 4","1238":"GRUPO 4","1239":"GRUPO 4","1240":"GRUPO 4","1241":"GRUPO 4","1242":"GRUPO 4","1243":"GRUPO 4","1244":"GRUPO 4","1245":"GRUPO 4","1246":"GRUPO 4","1247":"GRUPO 4","1248":"GRUPO 1","1249":"GRUPO 1","1250":"GRUPO 1","1251":"GRUPO 1","1252":"GRUPO 1","1253":"GRUPO 1","1254":"GRUPO 1","1255":"GRUPO 1","1256":"GRUPO 1","1257":"GRUPO 1","1258":"GRUPO 1","1259":"GRUPO 1","1260":"GRUPO 2","1261":"GRUPO 2","1262":"GRUPO 2","1263":"GRUPO 2","1264":"GRUPO 2","1265":"GRUPO 2","1266":"GRUPO 2","1267":"GRUPO 2","1268":"GRUPO 2","1269":"GRUPO 2","1270":"GRUPO 2","1271":"GRUPO 2","1272":"GRUPO 3","1273":"GRUPO 3","1274":"GRUPO 3","1275":"GRUPO 3","1276":"GRUPO 3","1277":"GRUPO 3","1278":"GRUPO 3","1279":"GRUPO 3","1280":"GRUPO 3","1281":"GRUPO 3","1282":"GRUPO 3","1283":"GRUPO 3","1284":"GRUPO 4","1285":"GRUPO 4","1286":"GRUPO 4","1287":"GRUPO 4","1288":"GRUPO 4","1289":"GRUPO 4","1290":"GRUPO 4","1291":"GRUPO 4","1292":"GRUPO 4","1293":"GRUPO 4","1294":"GRUPO 4","1295":"GRUPO 4","1296":"GRUPO 1","1297":"GRUPO 1","1298":"GRUPO 1","1299":"GRUPO 1","1300":"GRUPO 1","1301":"GRUPO 1","1302":"GRUPO 1","1303":"GRUPO 1","1304":"GRUPO 1","1305":"GRUPO 1","1306":"GRUPO 1","1307":"GRUPO 1","1308":"GRUPO 2","1309":"GRUPO 2","1310":"GRUPO 2","1311":"GRUPO 2","1312":"GRUPO 2","1313":"GRUPO 2","1314":"GRUPO 2","1315":"GRUPO 2","1316":"GRUPO 2","1317":"GRUPO 2","1318":"GRUPO 2","1319":"GRUPO 2","1320":"GRUPO 3","1321":"GRUPO 3","1322":"GRUPO 3","1323":"GRUPO 3","1324":"GRUPO 3","1325":"GRUPO 3","1326":"GRUPO 3","1327":"GRUPO 3","1328":"GRUPO 3","1329":"GRUPO 3","1330":"GRUPO 3","1331":"GRUPO 3","1332":"GRUPO 4","1333":"GRUPO 4","1334":"GRUPO 4","1335":"GRUPO 4","1336":"GRUPO 4","1337":"GRUPO 4","1338":"GRUPO 4","1339":"GRUPO 4","1340":"GRUPO 4","1341":"GRUPO 4","1342":"GRUPO 4","1343":"GRUPO 4","1344":"GRUPO 1","1345":"GRUPO 1","1346":"GRUPO 1","1347":"GRUPO 1","1348":"GRUPO 1","1349":"GRUPO 1","1350":"GRUPO 1","1351":"GRUPO 1","1352":"GRUPO 1","1353":"GRUPO 1","1354":"GRUPO 1","1355":"GRUPO 1","1356":"GRUPO 2","1357":"GRUPO 2","1358":"GRUPO 2","1359":"GRUPO 2","1360":"GRUPO 2","1361":"GRUPO 2","1362":"GRUPO 2","1363":"GRUPO 2","1364":"GRUPO 2","1365":"GRUPO 2","1366":"GRUPO 2","1367":"GRUPO 2","1368":"GRUPO 3","1369":"GRUPO 3","1370":"GRUPO 3","1371":"GRUPO 3","1372":"GRUPO 3","1373":"GRUPO 3","1374":"GRUPO 3","1375":"GRUPO 3","1376":"GRUPO 3","1377":"GRUPO 3","1378":"GRUPO 3","1379":"GRUPO 3","1380":"GRUPO 4","1381":"GRUPO 4","1382":"GRUPO 4","1383":"GRUPO 4","1384":"GRUPO 4","1385":"GRUPO 4","1386":"GRUPO 4","1387":"GRUPO 4","1388":"GRUPO 4","1389":"GRUPO 4","1390":"GRUPO 4","1391":"GRUPO 4","1392":"GRUPO 1","1393":"GRUPO 1","1394":"GRUPO 1","1395":"GRUPO 1","1396":"GRUPO 1","1397":"GRUPO 1","1398":"GRUPO 1","1399":"GRUPO 1","1400":"GRUPO 1","1401":"GRUPO 1","1402":"GRUPO 1","1403":"GRUPO 1","1404":"GRUPO 2","1405":"GRUPO 2","1406":"GRUPO 2","1407":"GRUPO 2","1408":"GRUPO 2","1409":"GRUPO 2","1410":"GRUPO 2","1411":"GRUPO 2","1412":"GRUPO 2","1413":"GRUPO 2","1414":"GRUPO 2","1415":"GRUPO 2","1416":"GRUPO 3","1417":"GRUPO 3","1418":"GRUPO 3","1419":"GRUPO 3","1420":"GRUPO 3","1421":"GRUPO 3","1422":"GRUPO 3","1423":"GRUPO 3","1424":"GRUPO 3","1425":"GRUPO 3","1426":"GRUPO 3","1427":"GRUPO 3","1428":"GRUPO 4","1429":"GRUPO 4","1430":"GRUPO 4","1431":"GRUPO 4","1432":"GRUPO 4","1433":"GRUPO 4","1434":"GRUPO 4","1435":"GRUPO 4","1436":"GRUPO 4","1437":"GRUPO 4","1438":"GRUPO 4","1439":"GRUPO 4"},"Empleado":{"0":"BARON HERNANDEZ HAROLD ANTONIO","1":"CASTELLANOS CARVAJAL DEYVITH FABIAN","2":"AROCA TORRES JULIAN EDUARDO","3":"BERMUDEZ PARRA JENNIFER XIOMARA","4":"BERNAL BAQUERO JAMES RICARDO","5":"BURGOS ORTIZ JOSE HORACIO","6":"CANTOR PORRAS JUAN FERNEY","7":"CAPERA CAPERA JOSE GABRIEL","8":"CARDENAS LOTERO RICARDO ANDR\u00c9S","9":"RENDON OSPINA NELSON LEANDRO","10":"SARMIENTO URBINA MOISES DANIEL","11":"VELASCO VELASCO SEBASTI\u00c1N DAVID","12":"DELGADO DELGADO JOHAN DARIO","13":"FLOREZ SAUCESO KENIS ALBERTO","14":"CARDONA GARCIA OSCAR JAVIER","15":"CARVAJAL GARC\u00cdA HOVER MARCK","16":"CEPEDA PIRAQUIVE JUAN DAVID","17":"FAJARDO SAENZ OSCAR FERNANDO","18":"FLOREZ ESPITIA RONY ALBERTO","19":"GARCIA CUERVO EDWIN JAVIER","20":"GONZALEZ OCHOA JUAN CARLOS","21":"XXX1","22":"XXX2","23":"XXX3","24":"FONSECA RAY RICARDO","25":"GOMEZ BETANCUR JAIDER ANDRES","26":"GRANADA PATI\u00d1O CARLOS MARINO","27":"GRASS PLATA MIGUEL SNEIDER","28":"MANZANO CALVO JUAN SEBASTIAN","29":"MENDOZA GOITA MARIANSEL ZENAYDA","30":"MURILLO ARAQUE JAIVER GEOVANY","31":"NI\u00d1O ARENAS HECTOR GONZALO","32":"RAMIREZ CHAVERRA JHON EDISON","33":"XXX4","34":"XXX5","35":"XXX6","36":"RODRIGUEZ MOSQUERA LUIS FERNANDO","37":"PEPITO PEREZ","38":"RAMIREZ VARGAS MARCELA PAOLA","39":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","40":"TORO CISNEROS GARY JOSE","41":"USECHE CALDERON JADID ESTIVEN","42":"VASQUEZ NIETO CAMILO ANDRES","43":"JHONY CASTRO","44":"BERNAL JUAN DAVID","45":"XXX7","46":"XXX8","47":"XXX9","48":"BARON HERNANDEZ HAROLD ANTONIO","49":"CASTELLANOS CARVAJAL DEYVITH FABIAN","50":"AROCA TORRES JULIAN EDUARDO","51":"BERMUDEZ PARRA JENNIFER XIOMARA","52":"BERNAL BAQUERO JAMES RICARDO","53":"BURGOS ORTIZ JOSE HORACIO","54":"CANTOR PORRAS JUAN FERNEY","55":"CAPERA CAPERA JOSE GABRIEL","56":"CARDENAS LOTERO RICARDO ANDR\u00c9S","57":"RENDON OSPINA NELSON LEANDRO","58":"SARMIENTO URBINA MOISES DANIEL","59":"VELASCO VELASCO SEBASTI\u00c1N DAVID","60":"DELGADO DELGADO JOHAN DARIO","61":"FLOREZ SAUCESO KENIS ALBERTO","62":"CARDONA GARCIA OSCAR JAVIER","63":"CARVAJAL GARC\u00cdA HOVER MARCK","64":"CEPEDA PIRAQUIVE JUAN DAVID","65":"FAJARDO SAENZ OSCAR FERNANDO","66":"FLOREZ ESPITIA RONY ALBERTO","67":"GARCIA CUERVO EDWIN JAVIER","68":"GONZALEZ OCHOA JUAN CARLOS","69":"XXX1","70":"XXX2","71":"XXX3","72":"FONSECA RAY RICARDO","73":"GOMEZ BETANCUR JAIDER ANDRES","74":"GRANADA PATI\u00d1O CARLOS MARINO","75":"GRASS PLATA MIGUEL SNEIDER","76":"MANZANO CALVO JUAN SEBASTIAN","77":"MENDOZA GOITA MARIANSEL ZENAYDA","78":"MURILLO ARAQUE JAIVER GEOVANY","79":"NI\u00d1O ARENAS HECTOR GONZALO","80":"RAMIREZ CHAVERRA JHON EDISON","81":"XXX4","82":"XXX5","83":"XXX6","84":"RODRIGUEZ MOSQUERA LUIS FERNANDO","85":"PEPITO PEREZ","86":"RAMIREZ VARGAS MARCELA PAOLA","87":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","88":"TORO CISNEROS GARY JOSE","89":"USECHE CALDERON JADID ESTIVEN","90":"VASQUEZ NIETO CAMILO ANDRES","91":"JHONY CASTRO","92":"BERNAL JUAN DAVID","93":"XXX7","94":"XXX8","95":"XXX9","96":"BARON HERNANDEZ HAROLD ANTONIO","97":"CASTELLANOS CARVAJAL DEYVITH FABIAN","98":"AROCA TORRES JULIAN EDUARDO","99":"BERMUDEZ PARRA JENNIFER XIOMARA","100":"BERNAL BAQUERO JAMES RICARDO","101":"BURGOS ORTIZ JOSE HORACIO","102":"CANTOR PORRAS JUAN FERNEY","103":"CAPERA CAPERA JOSE GABRIEL","104":"CARDENAS LOTERO RICARDO ANDR\u00c9S","105":"RENDON OSPINA NELSON LEANDRO","106":"SARMIENTO URBINA MOISES DANIEL","107":"VELASCO VELASCO SEBASTI\u00c1N DAVID","108":"DELGADO DELGADO JOHAN DARIO","109":"FLOREZ SAUCESO KENIS ALBERTO","110":"CARDONA GARCIA OSCAR JAVIER","111":"CARVAJAL GARC\u00cdA HOVER MARCK","112":"CEPEDA PIRAQUIVE JUAN DAVID","113":"FAJARDO SAENZ OSCAR FERNANDO","114":"FLOREZ ESPITIA RONY ALBERTO","115":"GARCIA CUERVO EDWIN JAVIER","116":"GONZALEZ OCHOA JUAN CARLOS","117":"XXX1","118":"XXX2","119":"XXX3","120":"FONSECA RAY RICARDO","121":"GOMEZ BETANCUR JAIDER ANDRES","122":"GRANADA PATI\u00d1O CARLOS MARINO","123":"GRASS PLATA MIGUEL SNEIDER","124":"MANZANO CALVO JUAN SEBASTIAN","125":"MENDOZA GOITA MARIANSEL ZENAYDA","126":"MURILLO ARAQUE JAIVER GEOVANY","127":"NI\u00d1O ARENAS HECTOR GONZALO","128":"RAMIREZ CHAVERRA JHON EDISON","129":"XXX4","130":"XXX5","131":"XXX6","132":"RODRIGUEZ MOSQUERA LUIS FERNANDO","133":"PEPITO PEREZ","134":"RAMIREZ VARGAS MARCELA PAOLA","135":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","136":"TORO CISNEROS GARY JOSE","137":"USECHE CALDERON JADID ESTIVEN","138":"VASQUEZ NIETO CAMILO ANDRES","139":"JHONY CASTRO","140":"BERNAL JUAN DAVID","141":"XXX7","142":"XXX8","143":"XXX9","144":"BARON HERNANDEZ HAROLD ANTONIO","145":"CASTELLANOS CARVAJAL DEYVITH FABIAN","146":"AROCA TORRES JULIAN EDUARDO","147":"BERMUDEZ PARRA JENNIFER XIOMARA","148":"BERNAL BAQUERO JAMES RICARDO","149":"BURGOS ORTIZ JOSE HORACIO","150":"CANTOR PORRAS JUAN FERNEY","151":"CAPERA CAPERA JOSE GABRIEL","152":"CARDENAS LOTERO RICARDO ANDR\u00c9S","153":"RENDON OSPINA NELSON LEANDRO","154":"SARMIENTO URBINA MOISES DANIEL","155":"VELASCO VELASCO SEBASTI\u00c1N DAVID","156":"DELGADO DELGADO JOHAN DARIO","157":"FLOREZ SAUCESO KENIS ALBERTO","158":"CARDONA GARCIA OSCAR JAVIER","159":"CARVAJAL GARC\u00cdA HOVER MARCK","160":"CEPEDA PIRAQUIVE JUAN DAVID","161":"FAJARDO SAENZ OSCAR FERNANDO","162":"FLOREZ ESPITIA RONY ALBERTO","163":"GARCIA CUERVO EDWIN JAVIER","164":"GONZALEZ OCHOA JUAN CARLOS","165":"XXX1","166":"XXX2","167":"XXX3","168":"FONSECA RAY RICARDO","169":"GOMEZ BETANCUR JAIDER ANDRES","170":"GRANADA PATI\u00d1O CARLOS MARINO","171":"GRASS PLATA MIGUEL SNEIDER","172":"MANZANO CALVO JUAN SEBASTIAN","173":"MENDOZA GOITA MARIANSEL ZENAYDA","174":"MURILLO ARAQUE JAIVER GEOVANY","175":"NI\u00d1O ARENAS HECTOR GONZALO","176":"RAMIREZ CHAVERRA JHON EDISON","177":"XXX4","178":"XXX5","179":"XXX6","180":"RODRIGUEZ MOSQUERA LUIS FERNANDO","181":"PEPITO PEREZ","182":"RAMIREZ VARGAS MARCELA PAOLA","183":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","184":"TORO CISNEROS GARY JOSE","185":"USECHE CALDERON JADID ESTIVEN","186":"VASQUEZ NIETO CAMILO ANDRES","187":"JHONY CASTRO","188":"BERNAL JUAN DAVID","189":"XXX7","190":"XXX8","191":"XXX9","192":"BARON HERNANDEZ HAROLD ANTONIO","193":"CASTELLANOS CARVAJAL DEYVITH FABIAN","194":"AROCA TORRES JULIAN EDUARDO","195":"BERMUDEZ PARRA JENNIFER XIOMARA","196":"BERNAL BAQUERO JAMES RICARDO","197":"BURGOS ORTIZ JOSE HORACIO","198":"CANTOR PORRAS JUAN FERNEY","199":"CAPERA CAPERA JOSE GABRIEL","200":"CARDENAS LOTERO RICARDO ANDR\u00c9S","201":"RENDON OSPINA NELSON LEANDRO","202":"SARMIENTO URBINA MOISES DANIEL","203":"VELASCO VELASCO SEBASTI\u00c1N DAVID","204":"DELGADO DELGADO JOHAN DARIO","205":"FLOREZ SAUCESO KENIS ALBERTO","206":"CARDONA GARCIA OSCAR JAVIER","207":"CARVAJAL GARC\u00cdA HOVER MARCK","208":"CEPEDA PIRAQUIVE JUAN DAVID","209":"FAJARDO SAENZ OSCAR FERNANDO","210":"FLOREZ ESPITIA RONY ALBERTO","211":"GARCIA CUERVO EDWIN JAVIER","212":"GONZALEZ OCHOA JUAN CARLOS","213":"XXX1","214":"XXX2","215":"XXX3","216":"FONSECA RAY RICARDO","217":"GOMEZ BETANCUR JAIDER ANDRES","218":"GRANADA PATI\u00d1O CARLOS MARINO","219":"GRASS PLATA MIGUEL SNEIDER","220":"MANZANO CALVO JUAN SEBASTIAN","221":"MENDOZA GOITA MARIANSEL ZENAYDA","222":"MURILLO ARAQUE JAIVER GEOVANY","223":"NI\u00d1O ARENAS HECTOR GONZALO","224":"RAMIREZ CHAVERRA JHON EDISON","225":"XXX4","226":"XXX5","227":"XXX6","228":"RODRIGUEZ MOSQUERA LUIS FERNANDO","229":"PEPITO PEREZ","230":"RAMIREZ VARGAS MARCELA PAOLA","231":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","232":"TORO CISNEROS GARY JOSE","233":"USECHE CALDERON JADID ESTIVEN","234":"VASQUEZ NIETO CAMILO ANDRES","235":"JHONY CASTRO","236":"BERNAL JUAN DAVID","237":"XXX7","238":"XXX8","239":"XXX9","240":"BARON HERNANDEZ HAROLD ANTONIO","241":"CASTELLANOS CARVAJAL DEYVITH FABIAN","242":"AROCA TORRES JULIAN EDUARDO","243":"BERMUDEZ PARRA JENNIFER XIOMARA","244":"BERNAL BAQUERO JAMES RICARDO","245":"BURGOS ORTIZ JOSE HORACIO","246":"CANTOR PORRAS JUAN FERNEY","247":"CAPERA CAPERA JOSE GABRIEL","248":"CARDENAS LOTERO RICARDO ANDR\u00c9S","249":"RENDON OSPINA NELSON LEANDRO","250":"SARMIENTO URBINA MOISES DANIEL","251":"VELASCO VELASCO SEBASTI\u00c1N DAVID","252":"DELGADO DELGADO JOHAN DARIO","253":"FLOREZ SAUCESO KENIS ALBERTO","254":"CARDONA GARCIA OSCAR JAVIER","255":"CARVAJAL GARC\u00cdA HOVER MARCK","256":"CEPEDA PIRAQUIVE JUAN DAVID","257":"FAJARDO SAENZ OSCAR FERNANDO","258":"FLOREZ ESPITIA RONY ALBERTO","259":"GARCIA CUERVO EDWIN JAVIER","260":"GONZALEZ OCHOA JUAN CARLOS","261":"XXX1","262":"XXX2","263":"XXX3","264":"FONSECA RAY RICARDO","265":"GOMEZ BETANCUR JAIDER ANDRES","266":"GRANADA PATI\u00d1O CARLOS MARINO","267":"GRASS PLATA MIGUEL SNEIDER","268":"MANZANO CALVO JUAN SEBASTIAN","269":"MENDOZA GOITA MARIANSEL ZENAYDA","270":"MURILLO ARAQUE JAIVER GEOVANY","271":"NI\u00d1O ARENAS HECTOR GONZALO","272":"RAMIREZ CHAVERRA JHON EDISON","273":"XXX4","274":"XXX5","275":"XXX6","276":"RODRIGUEZ MOSQUERA LUIS FERNANDO","277":"PEPITO PEREZ","278":"RAMIREZ VARGAS MARCELA PAOLA","279":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","280":"TORO CISNEROS GARY JOSE","281":"USECHE CALDERON JADID ESTIVEN","282":"VASQUEZ NIETO CAMILO ANDRES","283":"JHONY CASTRO","284":"BERNAL JUAN DAVID","285":"XXX7","286":"XXX8","287":"XXX9","288":"BARON HERNANDEZ HAROLD ANTONIO","289":"CASTELLANOS CARVAJAL DEYVITH FABIAN","290":"AROCA TORRES JULIAN EDUARDO","291":"BERMUDEZ PARRA JENNIFER XIOMARA","292":"BERNAL BAQUERO JAMES RICARDO","293":"BURGOS ORTIZ JOSE</t>
@@ -77,6 +77,12 @@
   </si>
   <si>
     <t>[{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"01-Sab","Final":"T2","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"01-Sab","Final":"T2","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"01-Sab","Final":"T2","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"01-Sab","Final":"T2","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"01-Sab","Final":"T2","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"01-Sab","Final":"T2","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"01-Sab","Final":"T2","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"01-Sab","Final":"T2","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"01-Sab","Final":"T2","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"01-Sab","Final":"T2","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"01-Sab","Final":"T2","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"01-Sab","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"01-Sab","Final":"T1","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"01-Sab","Final":"T1","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"01-Sab","Final":"T1","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"01-Sab","Final":"T1","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"01-Sab","Final":"T1","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"01-Sab","Final":"T1","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"01-Sab","Final":"T1","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"01-Sab","Final":"T1","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"01-Sab","Final":"T1","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"01-Sab","Final":"T1","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"01-Sab","Final":"T1","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"01-Sab","Final":"T1","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"01-Sab","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"01-Sab","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"01-Sab","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"01-Sab","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"01-Sab","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"01-Sab","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"01-Sab","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"01-Sab","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"01-Sab","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"01-Sab","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"01-Sab","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"01-Sab","Final":"T3","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"01-Sab","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"01-Sab","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"01-Sab","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"01-Sab","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"01-Sab","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"01-Sab","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"01-Sab","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"01-Sab","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"01-Sab","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"01-Sab","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"01-Sab","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"01-Sab","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"02-Dom","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"02-Dom","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"02-Dom","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"02-Dom","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"02-Dom","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"02-Dom","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"02-Dom","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"02-Dom","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"02-Dom","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"02-Dom","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"02-Dom","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"02-Dom","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"02-Dom","Final":"T1","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"02-Dom","Final":"T1","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"02-Dom","Final":"T1","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"02-Dom","Final":"T1","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"02-Dom","Final":"T1","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"02-Dom","Final":"T1","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"02-Dom","Final":"T1","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"02-Dom","Final":"T1","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"02-Dom","Final":"T1","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"02-Dom","Final":"T1","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"02-Dom","Final":"T1","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"02-Dom","Final":"T1","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"02-Dom","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"02-Dom","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"02-Dom","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"02-Dom","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"02-Dom","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"02-Dom","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"02-Dom","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"02-Dom","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"02-Dom","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"02-Dom","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"02-Dom","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"02-Dom","Final":"T3","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"02-Dom","Final":"T2","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"02-Dom","Final":"T2","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"02-Dom","Final":"T2","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"02-Dom","Final":"T2","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"02-Dom","Final":"T2","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"02-Dom","Final":"T2","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"02-Dom","Final":"T2","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"02-Dom","Final":"T2","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"02-Dom","Final":"T2","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"02-Dom","Final":"T2","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"02-Dom","Final":"T2","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"02-Dom","Final":"T2","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"03-Lun","Final":"T1","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"03-Lun","Final":"T1","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"03-Lun","Final":"T1","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"03-Lun","Final":"T1","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"03-Lun","Final":"T1","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"03-Lun","Final":"T1","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"03-Lun","Final":"T1","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"03-Lun","Final":"T1","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"03-Lun","Final":"T1","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"03-Lun","Final":"T1","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"03-Lun","Final":"T1","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"03-Lun","Final":"T1","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"03-Lun","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"03-Lun","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"03-Lun","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"03-Lun","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"03-Lun","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"03-Lun","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"03-Lun","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"03-Lun","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"03-Lun","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"03-Lun","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"03-Lun","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"03-Lun","Final":"T3","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"03-Lun","Final":"T2","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"04-Mar","Final":"T1","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"04-Mar","Final":"T1","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"04-Mar","Final":"T1","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"04-Mar","Final":"T1","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"04-Mar","Final":"T1","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"04-Mar","Final":"T1","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"04-Mar","Final":"T1","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"04-Mar","Final":"T1","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"04-Mar","Final":"T1","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"04-Mar","Final":"T1","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"04-Mar","Final":"T1","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"04-Mar","Final":"T1","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"04-Mar","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"04-Mar","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"04-Mar","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"04-Mar","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"04-Mar","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"04-Mar","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"04-Mar","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"04-Mar","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"04-Mar","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"04-Mar","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"04-Mar","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"04-Mar","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"04-Mar","Final":"T2","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"05-Mie","Final":"T1","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"05-Mie","Final":"T1","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"05-Mie","Final":"T1","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"05-Mie","Final":"T1","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"05-Mie","Final":"T1","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"05-Mie","Final":"T1","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"05-Mie","Final":"T1","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"05-Mie","Final":"T1","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"05-Mie","Final":"T1","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"05-Mie","Final":"T1","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"05-Mie","Final":"T1","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"05-Mie","Final":"T1","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"05-Mie","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"05-Mie","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"05-Mie","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"05-Mie","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"05-Mie","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"05-Mie","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"05-Mie","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"05-Mie","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"05-Mie","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"05-Mie","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"05-Mie","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"05-Mie","Final":"T3","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"05-Mie","Final":"T2","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"06-Jue","Final":"T2","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"06-Jue","Final":"T2","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"06-Jue","Final":"T2","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"06-Jue","Final":"T2","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"06-Jue","Final":"T2","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"06-Jue","Final":"T2","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"06-Jue","Final":"T2","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"06-Jue","Final":"T2","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"06-Jue","Final":"T2","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"06-Jue","Final":"T2","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"06-Jue","Final":"T2","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"06-Jue","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"06-Jue","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"06-Jue","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"06-Jue","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"06-Jue","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"06-Jue","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"06-Jue","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"06-Jue","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"06-Jue","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"06-Jue","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"06-Jue","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"06-Jue","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"06-Jue","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"06-Jue","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"06-Jue","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"06-Jue","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"06-Jue","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"06-Jue","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"06-Jue","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"06-Jue","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"06-Jue","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"06-Jue","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"06-Jue","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"06-Jue","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"06-Jue","Final":"T3","n_dia":6},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"06-Jue","Final":"T2","n_dia":6},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"06-Jue","Final":"T2","n_dia":6},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VA</t>
+  </si>
+  <si>
+    <t>{"columns":["Grupo","Empleado","Cargo","Label","Final","n_dia"],"index":[0,1,2,3,4,5,6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23,24,25,26,27,28,29,30,31,32,33,34,35,36,37,38,39,40,41,42,43,44,45,46,47,48,49,50,51,52,53,54,55,56,57,58,59,60,61,62,63,64,65,66,67,68,69,70,71,72,73,74,75,76,77,78,79,80,81,82,83,84,85,86,87,88,89,90,91,92,93,94,95,96,97,98,99,100,101,102,103,104,105,106,107,108,109,110,111,112,113,114,115,116,117,118,119,120,121,122,123,124,125,126,127,128,129,130,131,132,133,134,135,136,137,138,139,140,141,142,143,144,145,146,147,148,149,150,151,152,153,154,155,156,157,158,159,160,161,162,163,164,165,166,167,168,169,170,171,172,173,174,175,176,177,178,179,180,181,182,183,184,185,186,187,188,189,190,191,192,193,194,195,196,197,198,199,200,201,202,203,204,205,206,207,208,209,210,211,212,213,214,215,216,217,218,219,220,221,222,223,224,225,226,227,228,229,230,231,232,233,234,235,236,237,238,239,240,241,242,243,244,245,246,247,248,249,250,251,252,253,254,255,256,257,258,259,260,261,262,263,264,265,266,267,268,269,270,271,272,273,274,275,276,277,278,279,280,281,282,283,284,285,286,287,288,289,290,291,292,293,294,295,296,297,298,299,300,301,302,303,304,305,306,307,308,309,310,311,312,313,314,315,316,317,318,319,320,321,322,323,324,325,326,327,328,329,330,331,332,333,334,335,336,337,338,339,340,341,342,343,344,345,346,347,348,349,350,351,352,353,354,355,356,357,358,359,360,361,362,363,364,365,366,367,368,369,370,371,372,373,374,375,376,377,378,379,380,381,382,383,384,385,386,387,388,389,390,391,392,393,394,395,396,397,398,399,400,401,402,403,404,405,406,407,408,409,410,411,412,413,414,415,416,417,418,419,420,421,422,423,424,425,426,427,428,429,430,431,432,433,434,435,436,437,438,439,440,441,442,443,444,445,446,447,448,449,450,451,452,453,454,455,456,457,458,459,460,461,462,463,464,465,466,467,468,469,470,471,472,473,474,475,476,477,478,479,480,481,482,483,484,485,486,487,488,489,490,491,492,493,494,495,496,497,498,499,500,501,502,503,504,505,506,507,508,509,510,511,512,513,514,515,516,517,518,519,520,521,522,523,524,525,526,527,528,529,530,531,532,533,534,535,536,537,538,539,540,541,542,543,544,545,546,547,548,549,550,551,552,553,554,555,556,557,558,559,560,561,562,563,564,565,566,567,568,569,570,571,572,573,574,575,576,577,578,579,580,581,582,583,584,585,586,587,588,589,590,591,592,593,594,595,596,597,598,599,600,601,602,603,604,605,606,607,608,609,610,611,612,613,614,615,616,617,618,619,620,621,622,623,624,625,626,627,628,629,630,631,632,633,634,635,636,637,638,639,640,641,642,643,644,645,646,647,648,649,650,651,652,653,654,655,656,657,658,659,660,661,662,663,664,665,666,667,668,669,670,671,672,673,674,675,676,677,678,679,680,681,682,683,684,685,686,687,688,689,690,691,692,693,694,695,696,697,698,699,700,701,702,703,704,705,706,707,708,709,710,711,712,713,714,715,716,717,718,719,720,721,722,723,724,725,726,727,728,729,730,731,732,733,734,735,736,737,738,739,740,741,742,743,744,745,746,747,748,749,750,751,752,753,754,755,756,757,758,759,760,761,762,763,764,765,766,767,768,769,770,771,772,773,774,775,776,777,778,779,780,781,782,783,784,785,786,787,788,789,790,791,792,793,794,795,796,797,798,799,800,801,802,803,804,805,806,807,808,809,810,811,812,813,814,815,816,817,818,819,820,821,822,823,824,825,826,827,828,829,830,831,832,833,834,835,836,837,838,839,840,841,842,843,844,845,846,847,848,849,850,851,852,853,854,855,856,857,858,859,860,861,862,863,864,865,866,867,868,869,870,871,872,873,874,875,876,877,878,879,880,881,882,883,884,885,886,887,888,889,890,891,892,893,894,895,896,897,898,899,900,901,902,903,904,905,906,907,908,909,910,911,912,913,914,915,916,917,918,919,920,921,922,923,924,925,926,927,928,929,930,931,932,933,934,935,936,937,938,939,940,941,942,943,944,945,946,947,948,949,950,951,952,953,954,955,956,957,958,959,960,961,962,963,964,965,966,967,968,969,970,971,972,973,974,975,976,977,978,979,980,981,982,983,984,985,986,987,988,989,990,991,992,993,994,995,996,997,998,999,1000,1001,1002,1003,1004,1005,1006,1007,1008,1009,1010,1011,1012,1013,1014,1015,1016,1017,1018,1019,1020,1021,1022,1023,1024,1025,1026,1027,1028,1029,1030,1031,1032,1033,1034,1035,1036,1037,1038,1039,1040,1041,1042,1043,1044,1045,1046,1047,1048,1049,1050,1051,1052,1053,1054,1055,1056,1057,1058,1059,1060,1061,1062,1063,1064,1065,1066,1067,1068,1069,1070,1071,1072,1073,1074,1075,1076,1077,1078,1079,1080,1081,1082,1083,1084,1085,1086,1087,1088,1089,1090,1091,1092,1093,1094,1095,1096,1097,1098,1099,1100,1101,1102,1103,1104,1105,1106,1107,1108,1109,1110,1111,1112,1113,1114,1115,1116,1117,1118,1119,1120,1121,1122,1123,1124,1125,1126,1127,1128,1129,1130,1131,1132,1133,1134,1135,1136,1137,1138,1139,1140,1141,1142,1143,1144,1145,1146,1147,1148,1149,1150,1151,1152,1153,1154,1155,1156,1157,1158,1159,1160,1161,1162,1163,1164,1165,1166,1167,1168,1169,1170,1171,1172,1173,1174,1175,1176,1177,1178,1179,1180,1181,1182,1183,1184,1185,1186,1187,1188,1189,1190,1191,1192,1193,1194,1195,1196,1197,1198,1199,1200,1201,1202,1203,1204,1205,1206,1207,1208,1209,1210,1211,1212,1213,1214,1215,1216,1217,1218,1219,1220,1221,1222,1223,1224,1225,1226,1227,1228,1229,1230,1231,1232,1233,1234,1235,1236,1237,1238,1239,1240,1241,1242,1243,1244,1245,1246,1247,1248,1249,1250,1251,1252,1253,1254,1255,1256,1257,1258,1259,1260,1261,1262,1263,1264,1265,1266,1267,1268,1269,1270,1271,1272,1273,1274,1275,1276,1277,1278,1279,1280,1281,1282,1283,1284,1285,1286,1287,1288,1289,1290,1291,1292,1293,1294,1295,1296,1297,1298,1299,1300,1301,1302,1303,1304,1305,1306,1307,1308,1309,1310,1311,1312,1313,1314,1315,1316,1317,1318,1319,1320,1321,1322,1323,1324,1325,1326,1327,1328,1329,1330,1331,1332,1333,1334,1335,1336,1337,1338,1339,1340,1341,1342,1343,1344,1345,1346,1347,1348,1349,1350,1351,1352,1353,1354,1355,1356,1357,1358,1359,1360,1361,1362,1363,1364,1365,1366,1367,1368,1369,1370,1371,1372,1373,1374,1375,1376,1377,1378,1379,1380,1381,1382,1383,1384,1385,1386,1387,1388,1389,1390,1391,1392,1393,1394,1395,1396,1397,1398,1399,1400,1401,1402,1403,1404,1405,1406,1407,1408,1409,1410,1411,1412,1413,1414,1415,1416,1417,1418,1419,1420,1421,1422,1423,1424,1425,1426,1427,1428,1429,1430,1431,1432,1433,1434,1435,1436,1437,1438,1439,1440,1441,1442,1443,1444,1445,1446,1447,1448,1449,1450,1451,1452,1453,1454,1455,1456,1457,1458,1459,1460,1461,1462,1463,1464,1465,1466,1467,1468,1469,1470,1471,1472,1473,1474,1475,1476,1477,1478,1479,1480,1481,1482,1483,1484,1485,1486,1487],"data":[["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","01-Vie","T1",1],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","01-Vie","T1",1],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","01-Vie","T1",1],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","01-Vie","T1",1],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","01-Vie","T1",1],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","01-Vie","T1",1],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","01-Vie","T1",1],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","01-Vie","T1",1],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","01-Vie","T1",1],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","01-Vie","T1",1],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","01-Vie","T1",1],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","01-Vie","T1",1],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","01-Vie","DESC. LEY",1],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","01-Vie","DESC. LEY",1],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","01-Vie","DESC. LEY",1],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","01-Vie","DESC. LEY",1],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","01-Vie","DESC. LEY",1],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","01-Vie","DESC. LEY",1],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","01-Vie","DESC. LEY",1],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","01-Vie","DESC. LEY",1],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","01-Vie","DESC. LEY",1],["GRUPO 2","XXX1","Tecnico B","01-Vie","DESC. LEY",1],["GRUPO 2","XXX2","Tecnico B","01-Vie","DESC. LEY",1],["GRUPO 2","XXX3","Tecnico B","01-Vie","DESC. LEY",1],["GRUPO 3","FONSECA RAY RICARDO","Master","01-Vie","T3",1],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","01-Vie","T3",1],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","01-Vie","T3",1],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","01-Vie","T3",1],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","01-Vie","T3",1],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","01-Vie","T3",1],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","01-Vie","T3",1],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","01-Vie","T3",1],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","01-Vie","T3",1],["GRUPO 3","XXX4","Tecnico B","01-Vie","T3",1],["GRUPO 3","XXX5","Tecnico B","01-Vie","T3",1],["GRUPO 3","XXX6","Tecnico B","01-Vie","T3",1],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","01-Vie","T2",1],["GRUPO 4","PEPITO PEREZ","Master","01-Vie","T2",1],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","01-Vie","T2",1],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","01-Vie","T2",1],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","01-Vie","T2",1],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","01-Vie","T2",1],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","01-Vie","T2",1],["GRUPO 4","JHONY CASTRO","Tecnico A","01-Vie","T2",1],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","01-Vie","T2",1],["GRUPO 4","XXX7","Tecnico B","01-Vie","T2",1],["GRUPO 4","XXX8","Tecnico B","01-Vie","T2",1],["GRUPO 4","XXX9","Tecnico B","01-Vie","T2",1],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","02-Sab","T1",2],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","02-Sab","T1",2],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","02-Sab","T1",2],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","02-Sab","T1",2],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","02-Sab","T1",2],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","02-Sab","T1",2],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","02-Sab","T1",2],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","02-Sab","T1",2],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","02-Sab","T1",2],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","02-Sab","T1",2],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","02-Sab","T1",2],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","02-Sab","T1",2],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","02-Sab","T2",2],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","02-Sab","T2",2],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","02-Sab","T2",2],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","02-Sab","T2",2],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","02-Sab","T2",2],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","02-Sab","T2",2],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","02-Sab","T2",2],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","02-Sab","T2",2],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","02-Sab","T2",2],["GRUPO 2","XXX1","Tecnico B","02-Sab","T2",2],["GRUPO 2","XXX2","Tecnico B","02-Sab","T2",2],["GRUPO 2","XXX3","Tecnico B","02-Sab","T2",2],["GRUPO 3","FONSECA RAY RICARDO","Master","02-Sab","DESC. LEY",2],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","02-Sab","DESC. LEY",2],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","02-Sab","DESC. LEY",2],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","02-Sab","DESC. LEY",2],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","02-Sab","DESC. LEY",2],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","02-Sab","DESC. LEY",2],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","02-Sab","DESC. LEY",2],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","02-Sab","DESC. LEY",2],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","02-Sab","DESC. LEY",2],["GRUPO 3","XXX4","Tecnico B","02-Sab","DESC. LEY",2],["GRUPO 3","XXX5","Tecnico B","02-Sab","DESC. LEY",2],["GRUPO 3","XXX6","Tecnico B","02-Sab","DESC. LEY",2],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","02-Sab","T3",2],["GRUPO 4","PEPITO PEREZ","Master","02-Sab","T3",2],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","02-Sab","T3",2],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","02-Sab","T3",2],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","02-Sab","T3",2],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","02-Sab","T3",2],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","02-Sab","T3",2],["GRUPO 4","JHONY CASTRO","Tecnico A","02-Sab","T3",2],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","02-Sab","T3",2],["GRUPO 4","XXX7","Tecnico B","02-Sab","T3",2],["GRUPO 4","XXX8","Tecnico B","02-Sab","T3",2],["GRUPO 4","XXX9","Tecnico B","02-Sab","T3",2],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","03-Dom","T1",3],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","03-Dom","T1",3],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","03-Dom","T1",3],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","03-Dom","T1",3],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","03-Dom","T1",3],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","03-Dom","T1",3],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","03-Dom","T1",3],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","03-Dom","T1",3],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","03-Dom","T1",3],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","03-Dom","T1",3],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","03-Dom","T1",3],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","03-Dom","T1",3],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","03-Dom","T2",3],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","03-Dom","T2",3],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","03-Dom","T2",3],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","03-Dom","T2",3],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","03-Dom","T2",3],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","03-Dom","T2",3],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","03-Dom","T2",3],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","03-Dom","T2",3],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","03-Dom","T2",3],["GRUPO 2","XXX1","Tecnico B","03-Dom","T2",3],["GRUPO 2","XXX2","Tecnico B","03-Dom","T2",3],["GRUPO 2","XXX3","Tecnico B","03-Dom","T2",3],["GRUPO 3","FONSECA RAY RICARDO","Master","03-Dom","T3",3],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","03-Dom","T3",3],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","03-Dom","T3",3],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","03-Dom","T3",3],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","03-Dom","T3",3],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","03-Dom","T3",3],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","03-Dom","T3",3],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","03-Dom","T3",3],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","03-Dom","T3",3],["GRUPO 3","XXX4","Tecnico B","03-Dom","T3",3],["GRUPO 3","XXX5","Tecnico B","03-Dom","T3",3],["GRUPO 3","XXX6","Tecnico B","03-Dom","T3",3],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","03-Dom","DESC. LEY",3],["GRUPO 4","PEPITO PEREZ","Master","03-Dom","DESC. LEY",3],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","03-Dom","DESC. LEY",3],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","03-Dom","DESC. LEY",3],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","03-Dom","DESC. LEY",3],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","03-Dom","DESC. LEY",3],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","03-Dom","DESC. LEY",3],["GRUPO 4","JHONY CASTRO","Tecnico A","03-Dom","DESC. LEY",3],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","03-Dom","DESC. LEY",3],["GRUPO 4","XXX7","Tecnico B","03-Dom","DESC. LEY",3],["GRUPO 4","XXX8","Tecnico B","03-Dom","DESC. LEY",3],["GRUPO 4","XXX9","Tecnico B","03-Dom","DESC. LEY",3],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","04-Lun","T1",4],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","04-Lun","T1",4],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","04-Lun","T1",4],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","04-Lun","T1",4],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","04-Lun","T1",4],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","04-Lun","T1",4],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","04-Lun","T1",4],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","04-Lun","T1",4],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","04-Lun","T1",4],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","04-Lun","T1",4],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","04-Lun","T1",4],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","04-Lun","T1",4],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","04-Lun","T2",4],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","04-Lun","T2",4],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","04-Lun","T2",4],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","04-Lun","T2",4],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","04-Lun","T2",4],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","04-Lun","T2",4],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","04-Lun","T2",4],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","04-Lun","T2",4],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","04-Lun","T2",4],["GRUPO 2","XXX1","Tecnico B","04-Lun","T2",4],["GRUPO 2","XXX2","Tecnico B","04-Lun","T2",4],["GRUPO 2","XXX3","Tecnico B","04-Lun","T2",4],["GRUPO 3","FONSECA RAY RICARDO","Master","04-Lun","T3",4],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","04-Lun","T3",4],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","04-Lun","T3",4],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","04-Lun","T3",4],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","04-Lun","T3",4],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","04-Lun","T3",4],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","04-Lun","T3",4],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","04-Lun","T3",4],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","04-Lun","T3",4],["GRUPO 3","XXX4","Tecnico B","04-Lun","T3",4],["GRUPO 3","XXX5","Tecnico B","04-Lun","T3",4],["GRUPO 3","XXX6","Tecnico B","04-Lun","T3",4],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","04-Lun","T1",4],["GRUPO 4","PEPITO PEREZ","Master","04-Lun","T1",4],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","04-Lun","T1",4],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","04-Lun","T1",4],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","04-Lun","T1",4],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","04-Lun","T1",4],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","04-Lun","T1",4],["GRUPO 4","JHONY CASTRO","Tecnico A","04-Lun","T1",4],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","04-Lun","T1",4],["GRUPO 4","XXX7","Tecnico B","04-Lun","T1",4],["GRUPO 4","XXX8","Tecnico B","04-Lun","T1",4],["GRUPO 4","XXX9","Tecnico B","04-Lun","T1",4],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","05-Mar","T1",5],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","05-Mar","T1",5],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","05-Mar","T1",5],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","05-Mar","T1",5],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","05-Mar","T1",5],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","05-Mar","T1",5],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","05-Mar","T1",5],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","05-Mar","T1",5],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","05-Mar","T1",5],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","05-Mar","T1",5],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","05-Mar","T1",5],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","05-Mar","T1",5],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","05-Mar","T2",5],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","05-Mar","T2",5],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","05-Mar","T2",5],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","05-Mar","T2",5],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","05-Mar","T2",5],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","05-Mar","T2",5],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","05-Mar","T2",5],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","05-Mar","T2",5],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","05-Mar","T2",5],["GRUPO 2","XXX1","Tecnico B","05-Mar","T2",5],["GRUPO 2","XXX2","Tecnico B","05-Mar","T2",5],["GRUPO 2","XXX3","Tecnico B","05-Mar","T2",5],["GRUPO 3","FONSECA RAY RICARDO","Master","05-Mar","T3",5],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","05-Mar","T3",5],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","05-Mar","T3",5],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","05-Mar","T3",5],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","05-Mar","T3",5],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","05-Mar","T3",5],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","05-Mar","T3",5],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","05-Mar","T3",5],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","05-Mar","T3",5],["GRUPO 3","XXX4","Tecnico B","05-Mar","T3",5],["GRUPO 3","XXX5","Tecnico B","05-Mar","T3",5],["GRUPO 3","XXX6","Tecnico B","05-Mar","T3",5],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","05-Mar","T1",5],["GRUPO 4","PEPITO PEREZ","Master","05-Mar","T1",5],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","05-Mar","T1",5],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","05-Mar","T1",5],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","05-Mar","T1",5],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","05-Mar","T1",5],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","05-Mar","T1",5],["GRUPO 4","JHONY CASTRO","Tecnico A","05-Mar","T1",5],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","05-Mar","T1",5],["GRUPO 4","XXX7","Tecnico B","05-Mar","T1",5],["GRUPO 4","XXX8","Tecnico B","05-Mar","T1",5],["GRUPO 4","XXX9","Tecnico B","05-Mar","T1",5],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","06-Mie","T1",6],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","06-Mie","T1",6],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","06-Mie","T1",6],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","06-Mie","T1",6],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","06-Mie","T1",6],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","06-Mie","T1",6],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","06-Mie","T1",6],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","06-Mie","T1",6],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","06-Mie","T1",6],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","06-Mie","T1",6],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","06-Mie","T1",6],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","06-Mie","T1",6],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","06-Mie","T2",6],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","06-Mie","T2",6],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","06-Mie","T2",6],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","06-Mie","T2",6],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","06-Mie","T2",6],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","06-Mie","T2",6],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","06-Mie","T2",6],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","06-Mie","T2",6],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","06-Mie","T2",6],["GRUPO 2","XXX1","Tecnico B","06-Mie","T2",6],["GRUPO 2","XXX2","Tecnico B","06-Mie","T2",6],["GRUPO 2","XXX3","Tecnico B","06-Mie","T2",6],["GRUPO 3","FONSECA RAY RICARDO","Master","06-Mie","T3",6],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","06-Mie","T3",6],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","06-Mie","T3",6],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","06-Mie","T3",6],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","06-Mie","T3",6],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","06-Mie","T3",6],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","06-Mie","T3",6],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","06-Mie","T3",6],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","06-Mie","T3",6],["GRUPO 3","XXX4","Tecnico B","06-Mie","T3",6],["GRUPO 3","XXX5","Tecnico B","06-Mie","T3",6],["GRUPO 3","XXX6","Tecnico B","06-Mie","T3",6],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","06-Mie","T1",6],["GRUPO 4","PEPITO PEREZ","Master","06-Mie","T1",6],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","06-Mie","T1",6],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","06-Mie","T1",6],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","06-Mie","T1",6],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","06-Mie","T1",6],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","06-Mie","T1",6],["GRUPO 4","JHONY CASTRO","Tecnico A","06-Mie","T1",6],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","06-Mie","T1",6],["GRUPO 4","XXX7","Tecnico B","06-Mie","T1",6],["GRUPO 4","XXX8","Tecnico B","06-Mie","T1",6],["GRUPO 4","XXX9","Tecnico B","06-Mie","T1",6],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","07-Jue","DESC. LEY",7],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","07-Jue","DESC. LEY",7],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","07-Jue","DESC. LEY",7],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","07-Jue","DESC. LEY",7],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","07-Jue","DESC. LEY",7],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","07-Jue","DESC. LEY",7],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","07-Jue","DESC. LEY",7],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","07-Jue","DESC. LEY",7],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","07-Jue","DESC. LEY",7],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","07-Jue","DESC. LEY",7],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","07-Jue","DESC. LEY",7],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","07-Jue","DESC. LEY",7],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","07-Jue","T2",7],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","07-Jue","T2",7],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","07-Jue","T2",7],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","07-Jue","T2",7],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","07-Jue","T2",7],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","07-Jue","T2",7],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","07-Jue","T2",7],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","07-Jue","T2",7],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","07-Jue","T2",7],["GRUPO 2","XXX1","Tecnico B","07-Jue","T2",7],["GRUPO 2","XXX2","Tecnico B","07-Jue","T2",7],["GRUPO 2","XXX3","Tecnico B","07-Jue","T2",7],["GRUPO 3","FONSECA RAY RICARDO","Master","07-Jue","T3",7],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","07-Jue","T3",7],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","07-Jue","T3",7],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","07-Jue","T3",7],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","07-Jue","T3",7],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","07-Jue","T3",7],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","07-Jue","T3",7],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","07-Jue","T3",7],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","07-Jue","T3",7],["GRUPO 3","XXX4","Tecnico B","07-Jue","T3",7],["GRUPO 3","XXX5","Tecnico B","07-Jue","T3",7],["GRUPO 3","XXX6","Tecnico B","07-Jue","T3",7],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","07-Jue","T2",7],["GRUPO 4","PEPITO PEREZ","Master","07-Jue","T2",7],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","07-Jue","T2",7],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","07-Jue","T2",7],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","07-Jue","T2",7],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","07-Jue","T2",7],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","07-Jue","T2",7],["GRUPO 4","JHONY CASTRO","Tecnico A","07-Jue","T2",7],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","07-Jue","T2",7],["GRUPO 4","XXX7","Tecnico B","07-Jue","T2",7],["GRUPO 4","XXX8","Tecnico B","07-Jue","T2",7],["GRUPO 4","XXX9","Tecnico B","07-Jue","T2",7],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","08-Vie","T2",8],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","08-Vie","T2",8],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","08-Vie","T2",8],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","08-Vie","T2",8],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","08-Vie","T2",8],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","08-Vie","T2",8],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","08-Vie","T2",8],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","08-Vie","T2",8],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","08-Vie","T2",8],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","08-Vie","T2",8],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","08-Vie","T2",8],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","08-Vie","T2",8],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","08-Vie","DESC. LEY",8],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","08-Vie","DESC. LEY",8],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","08-Vie","DESC. LEY",8],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","08-Vie","DESC. LEY",8],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","08-Vie","DESC. LEY",8],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","08-Vie","DESC. LEY",8],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","08-Vie","DESC. LEY",8],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","08-Vie","DESC. LEY",8],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","08-Vie","DESC. LEY",8],["GRUPO 2","XXX1","Tecnico B","08-Vie","DESC. LEY",8],["GRUPO 2","XXX2","Tecnico B","08-Vie","DESC. LEY",8],["GRUPO 2","XXX3","Tecnico B","08-Vie","DESC. LEY",8],["GRUPO 3","FONSECA RAY RICARDO","Master","08-Vie","T3",8],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","08-Vie","T3",8],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","08-Vie","T3",8],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","08-Vie","T3",8],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","08-Vie","T3",8],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","08-Vie","T3",8],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","08-Vie","T3",8],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","08-Vie","T3",8],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","08-Vie","T3",8],["GRUPO 3","XXX4","Tecnico B","08-Vie","T3",8],["GRUPO 3","XXX5","Tecnico B","08-Vie","T3",8],["GRUPO 3","XXX6","Tecnico B","08-Vie","T3",8],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","08-Vie","T3",8],["GRUPO 4","PEPITO PEREZ","Master","08-Vie","T3",8],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","08-Vie","T3",8],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","08-Vie","T3",8],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","08-Vie","T3",8],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","08-Vie","T3",8],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","08-Vie","T3",8],["GRUPO 4","JHONY CASTRO","Tecnico A","08-Vie","T3",8],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","08-Vie","T3",8],["GRUPO 4","XXX7","Tecnico B","08-Vie","T3",8],["GRUPO 4","XXX8","Tecnico B","08-Vie","T3",8],["GRUPO 4","XXX9","Tecnico B","08-Vie","T3",8],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","09-Sab","T2",9],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","09-Sab","T2",9],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","09-Sab","T2",9],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","09-Sab","T2",9],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","09-Sab","T2",9],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","09-Sab","T2",9],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","09-Sab","T2",9],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","09-Sab","T2",9],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","09-Sab","T2",9],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","09-Sab","T2",9],["GRU</t>
+  </si>
+  <si>
+    <t>Mes Completo</t>
   </si>
 </sst>
 </file>
@@ -408,10 +414,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:6">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -427,90 +433,108 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B2">
         <v>2026</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E2" t="s">
-        <v>16</v>
+        <v>17</v>
+      </c>
+      <c r="F2" t="s">
+        <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B3">
         <v>2026</v>
       </c>
       <c r="C3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E3" t="s">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="F3" t="s">
+        <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B4">
         <v>2026</v>
       </c>
       <c r="C4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E4" t="s">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="F4" t="s">
+        <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B5">
         <v>2026</v>
       </c>
       <c r="C5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" t="s">
         <v>10</v>
-      </c>
-      <c r="D5" t="s">
-        <v>14</v>
-      </c>
-      <c r="E5" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5">
-      <c r="A6" t="s">
-        <v>9</v>
       </c>
       <c r="B6">
         <v>2026</v>
       </c>
       <c r="C6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E6" t="s">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="F6" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update historico_mallas.xlsx 2026-04-24 21:36:33.652494
</commit_message>
<xml_diff>
--- a/historico_mallas.xlsx
+++ b/historico_mallas.xlsx
@@ -37,27 +37,24 @@
     <t>Abril</t>
   </si>
   <si>
+    <t>Julio</t>
+  </si>
+  <si>
+    <t>Agosto</t>
+  </si>
+  <si>
+    <t>Mayo</t>
+  </si>
+  <si>
     <t>Junio</t>
   </si>
   <si>
-    <t>Julio</t>
-  </si>
-  <si>
-    <t>Agosto</t>
-  </si>
-  <si>
-    <t>Mayo</t>
-  </si>
-  <si>
     <t>Técnica</t>
   </si>
   <si>
     <t>2026-04-24 18:15</t>
   </si>
   <si>
-    <t>2026-04-24 18:24</t>
-  </si>
-  <si>
     <t>2026-04-24 18:27</t>
   </si>
   <si>
@@ -67,12 +64,12 @@
     <t>24/04/2026 21:35</t>
   </si>
   <si>
+    <t>24/04/2026 21:36</t>
+  </si>
+  <si>
     <t>{"Grupo":{"0":"GRUPO 1","1":"GRUPO 1","2":"GRUPO 1","3":"GRUPO 1","4":"GRUPO 1","5":"GRUPO 1","6":"GRUPO 1","7":"GRUPO 1","8":"GRUPO 1","9":"GRUPO 1","10":"GRUPO 1","11":"GRUPO 1","12":"GRUPO 2","13":"GRUPO 2","14":"GRUPO 2","15":"GRUPO 2","16":"GRUPO 2","17":"GRUPO 2","18":"GRUPO 2","19":"GRUPO 2","20":"GRUPO 2","21":"GRUPO 2","22":"GRUPO 2","23":"GRUPO 2","24":"GRUPO 3","25":"GRUPO 3","26":"GRUPO 3","27":"GRUPO 3","28":"GRUPO 3","29":"GRUPO 3","30":"GRUPO 3","31":"GRUPO 3","32":"GRUPO 3","33":"GRUPO 3","34":"GRUPO 3","35":"GRUPO 3","36":"GRUPO 4","37":"GRUPO 4","38":"GRUPO 4","39":"GRUPO 4","40":"GRUPO 4","41":"GRUPO 4","42":"GRUPO 4","43":"GRUPO 4","44":"GRUPO 4","45":"GRUPO 4","46":"GRUPO 4","47":"GRUPO 4","48":"GRUPO 1","49":"GRUPO 1","50":"GRUPO 1","51":"GRUPO 1","52":"GRUPO 1","53":"GRUPO 1","54":"GRUPO 1","55":"GRUPO 1","56":"GRUPO 1","57":"GRUPO 1","58":"GRUPO 1","59":"GRUPO 1","60":"GRUPO 2","61":"GRUPO 2","62":"GRUPO 2","63":"GRUPO 2","64":"GRUPO 2","65":"GRUPO 2","66":"GRUPO 2","67":"GRUPO 2","68":"GRUPO 2","69":"GRUPO 2","70":"GRUPO 2","71":"GRUPO 2","72":"GRUPO 3","73":"GRUPO 3","74":"GRUPO 3","75":"GRUPO 3","76":"GRUPO 3","77":"GRUPO 3","78":"GRUPO 3","79":"GRUPO 3","80":"GRUPO 3","81":"GRUPO 3","82":"GRUPO 3","83":"GRUPO 3","84":"GRUPO 4","85":"GRUPO 4","86":"GRUPO 4","87":"GRUPO 4","88":"GRUPO 4","89":"GRUPO 4","90":"GRUPO 4","91":"GRUPO 4","92":"GRUPO 4","93":"GRUPO 4","94":"GRUPO 4","95":"GRUPO 4","96":"GRUPO 1","97":"GRUPO 1","98":"GRUPO 1","99":"GRUPO 1","100":"GRUPO 1","101":"GRUPO 1","102":"GRUPO 1","103":"GRUPO 1","104":"GRUPO 1","105":"GRUPO 1","106":"GRUPO 1","107":"GRUPO 1","108":"GRUPO 2","109":"GRUPO 2","110":"GRUPO 2","111":"GRUPO 2","112":"GRUPO 2","113":"GRUPO 2","114":"GRUPO 2","115":"GRUPO 2","116":"GRUPO 2","117":"GRUPO 2","118":"GRUPO 2","119":"GRUPO 2","120":"GRUPO 3","121":"GRUPO 3","122":"GRUPO 3","123":"GRUPO 3","124":"GRUPO 3","125":"GRUPO 3","126":"GRUPO 3","127":"GRUPO 3","128":"GRUPO 3","129":"GRUPO 3","130":"GRUPO 3","131":"GRUPO 3","132":"GRUPO 4","133":"GRUPO 4","134":"GRUPO 4","135":"GRUPO 4","136":"GRUPO 4","137":"GRUPO 4","138":"GRUPO 4","139":"GRUPO 4","140":"GRUPO 4","141":"GRUPO 4","142":"GRUPO 4","143":"GRUPO 4","144":"GRUPO 1","145":"GRUPO 1","146":"GRUPO 1","147":"GRUPO 1","148":"GRUPO 1","149":"GRUPO 1","150":"GRUPO 1","151":"GRUPO 1","152":"GRUPO 1","153":"GRUPO 1","154":"GRUPO 1","155":"GRUPO 1","156":"GRUPO 2","157":"GRUPO 2","158":"GRUPO 2","159":"GRUPO 2","160":"GRUPO 2","161":"GRUPO 2","162":"GRUPO 2","163":"GRUPO 2","164":"GRUPO 2","165":"GRUPO 2","166":"GRUPO 2","167":"GRUPO 2","168":"GRUPO 3","169":"GRUPO 3","170":"GRUPO 3","171":"GRUPO 3","172":"GRUPO 3","173":"GRUPO 3","174":"GRUPO 3","175":"GRUPO 3","176":"GRUPO 3","177":"GRUPO 3","178":"GRUPO 3","179":"GRUPO 3","180":"GRUPO 4","181":"GRUPO 4","182":"GRUPO 4","183":"GRUPO 4","184":"GRUPO 4","185":"GRUPO 4","186":"GRUPO 4","187":"GRUPO 4","188":"GRUPO 4","189":"GRUPO 4","190":"GRUPO 4","191":"GRUPO 4","192":"GRUPO 1","193":"GRUPO 1","194":"GRUPO 1","195":"GRUPO 1","196":"GRUPO 1","197":"GRUPO 1","198":"GRUPO 1","199":"GRUPO 1","200":"GRUPO 1","201":"GRUPO 1","202":"GRUPO 1","203":"GRUPO 1","204":"GRUPO 2","205":"GRUPO 2","206":"GRUPO 2","207":"GRUPO 2","208":"GRUPO 2","209":"GRUPO 2","210":"GRUPO 2","211":"GRUPO 2","212":"GRUPO 2","213":"GRUPO 2","214":"GRUPO 2","215":"GRUPO 2","216":"GRUPO 3","217":"GRUPO 3","218":"GRUPO 3","219":"GRUPO 3","220":"GRUPO 3","221":"GRUPO 3","222":"GRUPO 3","223":"GRUPO 3","224":"GRUPO 3","225":"GRUPO 3","226":"GRUPO 3","227":"GRUPO 3","228":"GRUPO 4","229":"GRUPO 4","230":"GRUPO 4","231":"GRUPO 4","232":"GRUPO 4","233":"GRUPO 4","234":"GRUPO 4","235":"GRUPO 4","236":"GRUPO 4","237":"GRUPO 4","238":"GRUPO 4","239":"GRUPO 4","240":"GRUPO 1","241":"GRUPO 1","242":"GRUPO 1","243":"GRUPO 1","244":"GRUPO 1","245":"GRUPO 1","246":"GRUPO 1","247":"GRUPO 1","248":"GRUPO 1","249":"GRUPO 1","250":"GRUPO 1","251":"GRUPO 1","252":"GRUPO 2","253":"GRUPO 2","254":"GRUPO 2","255":"GRUPO 2","256":"GRUPO 2","257":"GRUPO 2","258":"GRUPO 2","259":"GRUPO 2","260":"GRUPO 2","261":"GRUPO 2","262":"GRUPO 2","263":"GRUPO 2","264":"GRUPO 3","265":"GRUPO 3","266":"GRUPO 3","267":"GRUPO 3","268":"GRUPO 3","269":"GRUPO 3","270":"GRUPO 3","271":"GRUPO 3","272":"GRUPO 3","273":"GRUPO 3","274":"GRUPO 3","275":"GRUPO 3","276":"GRUPO 4","277":"GRUPO 4","278":"GRUPO 4","279":"GRUPO 4","280":"GRUPO 4","281":"GRUPO 4","282":"GRUPO 4","283":"GRUPO 4","284":"GRUPO 4","285":"GRUPO 4","286":"GRUPO 4","287":"GRUPO 4","288":"GRUPO 1","289":"GRUPO 1","290":"GRUPO 1","291":"GRUPO 1","292":"GRUPO 1","293":"GRUPO 1","294":"GRUPO 1","295":"GRUPO 1","296":"GRUPO 1","297":"GRUPO 1","298":"GRUPO 1","299":"GRUPO 1","300":"GRUPO 2","301":"GRUPO 2","302":"GRUPO 2","303":"GRUPO 2","304":"GRUPO 2","305":"GRUPO 2","306":"GRUPO 2","307":"GRUPO 2","308":"GRUPO 2","309":"GRUPO 2","310":"GRUPO 2","311":"GRUPO 2","312":"GRUPO 3","313":"GRUPO 3","314":"GRUPO 3","315":"GRUPO 3","316":"GRUPO 3","317":"GRUPO 3","318":"GRUPO 3","319":"GRUPO 3","320":"GRUPO 3","321":"GRUPO 3","322":"GRUPO 3","323":"GRUPO 3","324":"GRUPO 4","325":"GRUPO 4","326":"GRUPO 4","327":"GRUPO 4","328":"GRUPO 4","329":"GRUPO 4","330":"GRUPO 4","331":"GRUPO 4","332":"GRUPO 4","333":"GRUPO 4","334":"GRUPO 4","335":"GRUPO 4","336":"GRUPO 1","337":"GRUPO 1","338":"GRUPO 1","339":"GRUPO 1","340":"GRUPO 1","341":"GRUPO 1","342":"GRUPO 1","343":"GRUPO 1","344":"GRUPO 1","345":"GRUPO 1","346":"GRUPO 1","347":"GRUPO 1","348":"GRUPO 2","349":"GRUPO 2","350":"GRUPO 2","351":"GRUPO 2","352":"GRUPO 2","353":"GRUPO 2","354":"GRUPO 2","355":"GRUPO 2","356":"GRUPO 2","357":"GRUPO 2","358":"GRUPO 2","359":"GRUPO 2","360":"GRUPO 3","361":"GRUPO 3","362":"GRUPO 3","363":"GRUPO 3","364":"GRUPO 3","365":"GRUPO 3","366":"GRUPO 3","367":"GRUPO 3","368":"GRUPO 3","369":"GRUPO 3","370":"GRUPO 3","371":"GRUPO 3","372":"GRUPO 4","373":"GRUPO 4","374":"GRUPO 4","375":"GRUPO 4","376":"GRUPO 4","377":"GRUPO 4","378":"GRUPO 4","379":"GRUPO 4","380":"GRUPO 4","381":"GRUPO 4","382":"GRUPO 4","383":"GRUPO 4","384":"GRUPO 1","385":"GRUPO 1","386":"GRUPO 1","387":"GRUPO 1","388":"GRUPO 1","389":"GRUPO 1","390":"GRUPO 1","391":"GRUPO 1","392":"GRUPO 1","393":"GRUPO 1","394":"GRUPO 1","395":"GRUPO 1","396":"GRUPO 2","397":"GRUPO 2","398":"GRUPO 2","399":"GRUPO 2","400":"GRUPO 2","401":"GRUPO 2","402":"GRUPO 2","403":"GRUPO 2","404":"GRUPO 2","405":"GRUPO 2","406":"GRUPO 2","407":"GRUPO 2","408":"GRUPO 3","409":"GRUPO 3","410":"GRUPO 3","411":"GRUPO 3","412":"GRUPO 3","413":"GRUPO 3","414":"GRUPO 3","415":"GRUPO 3","416":"GRUPO 3","417":"GRUPO 3","418":"GRUPO 3","419":"GRUPO 3","420":"GRUPO 4","421":"GRUPO 4","422":"GRUPO 4","423":"GRUPO 4","424":"GRUPO 4","425":"GRUPO 4","426":"GRUPO 4","427":"GRUPO 4","428":"GRUPO 4","429":"GRUPO 4","430":"GRUPO 4","431":"GRUPO 4","432":"GRUPO 1","433":"GRUPO 1","434":"GRUPO 1","435":"GRUPO 1","436":"GRUPO 1","437":"GRUPO 1","438":"GRUPO 1","439":"GRUPO 1","440":"GRUPO 1","441":"GRUPO 1","442":"GRUPO 1","443":"GRUPO 1","444":"GRUPO 2","445":"GRUPO 2","446":"GRUPO 2","447":"GRUPO 2","448":"GRUPO 2","449":"GRUPO 2","450":"GRUPO 2","451":"GRUPO 2","452":"GRUPO 2","453":"GRUPO 2","454":"GRUPO 2","455":"GRUPO 2","456":"GRUPO 3","457":"GRUPO 3","458":"GRUPO 3","459":"GRUPO 3","460":"GRUPO 3","461":"GRUPO 3","462":"GRUPO 3","463":"GRUPO 3","464":"GRUPO 3","465":"GRUPO 3","466":"GRUPO 3","467":"GRUPO 3","468":"GRUPO 4","469":"GRUPO 4","470":"GRUPO 4","471":"GRUPO 4","472":"GRUPO 4","473":"GRUPO 4","474":"GRUPO 4","475":"GRUPO 4","476":"GRUPO 4","477":"GRUPO 4","478":"GRUPO 4","479":"GRUPO 4","480":"GRUPO 1","481":"GRUPO 1","482":"GRUPO 1","483":"GRUPO 1","484":"GRUPO 1","485":"GRUPO 1","486":"GRUPO 1","487":"GRUPO 1","488":"GRUPO 1","489":"GRUPO 1","490":"GRUPO 1","491":"GRUPO 1","492":"GRUPO 2","493":"GRUPO 2","494":"GRUPO 2","495":"GRUPO 2","496":"GRUPO 2","497":"GRUPO 2","498":"GRUPO 2","499":"GRUPO 2","500":"GRUPO 2","501":"GRUPO 2","502":"GRUPO 2","503":"GRUPO 2","504":"GRUPO 3","505":"GRUPO 3","506":"GRUPO 3","507":"GRUPO 3","508":"GRUPO 3","509":"GRUPO 3","510":"GRUPO 3","511":"GRUPO 3","512":"GRUPO 3","513":"GRUPO 3","514":"GRUPO 3","515":"GRUPO 3","516":"GRUPO 4","517":"GRUPO 4","518":"GRUPO 4","519":"GRUPO 4","520":"GRUPO 4","521":"GRUPO 4","522":"GRUPO 4","523":"GRUPO 4","524":"GRUPO 4","525":"GRUPO 4","526":"GRUPO 4","527":"GRUPO 4","528":"GRUPO 1","529":"GRUPO 1","530":"GRUPO 1","531":"GRUPO 1","532":"GRUPO 1","533":"GRUPO 1","534":"GRUPO 1","535":"GRUPO 1","536":"GRUPO 1","537":"GRUPO 1","538":"GRUPO 1","539":"GRUPO 1","540":"GRUPO 2","541":"GRUPO 2","542":"GRUPO 2","543":"GRUPO 2","544":"GRUPO 2","545":"GRUPO 2","546":"GRUPO 2","547":"GRUPO 2","548":"GRUPO 2","549":"GRUPO 2","550":"GRUPO 2","551":"GRUPO 2","552":"GRUPO 3","553":"GRUPO 3","554":"GRUPO 3","555":"GRUPO 3","556":"GRUPO 3","557":"GRUPO 3","558":"GRUPO 3","559":"GRUPO 3","560":"GRUPO 3","561":"GRUPO 3","562":"GRUPO 3","563":"GRUPO 3","564":"GRUPO 4","565":"GRUPO 4","566":"GRUPO 4","567":"GRUPO 4","568":"GRUPO 4","569":"GRUPO 4","570":"GRUPO 4","571":"GRUPO 4","572":"GRUPO 4","573":"GRUPO 4","574":"GRUPO 4","575":"GRUPO 4","576":"GRUPO 1","577":"GRUPO 1","578":"GRUPO 1","579":"GRUPO 1","580":"GRUPO 1","581":"GRUPO 1","582":"GRUPO 1","583":"GRUPO 1","584":"GRUPO 1","585":"GRUPO 1","586":"GRUPO 1","587":"GRUPO 1","588":"GRUPO 2","589":"GRUPO 2","590":"GRUPO 2","591":"GRUPO 2","592":"GRUPO 2","593":"GRUPO 2","594":"GRUPO 2","595":"GRUPO 2","596":"GRUPO 2","597":"GRUPO 2","598":"GRUPO 2","599":"GRUPO 2","600":"GRUPO 3","601":"GRUPO 3","602":"GRUPO 3","603":"GRUPO 3","604":"GRUPO 3","605":"GRUPO 3","606":"GRUPO 3","607":"GRUPO 3","608":"GRUPO 3","609":"GRUPO 3","610":"GRUPO 3","611":"GRUPO 3","612":"GRUPO 4","613":"GRUPO 4","614":"GRUPO 4","615":"GRUPO 4","616":"GRUPO 4","617":"GRUPO 4","618":"GRUPO 4","619":"GRUPO 4","620":"GRUPO 4","621":"GRUPO 4","622":"GRUPO 4","623":"GRUPO 4","624":"GRUPO 1","625":"GRUPO 1","626":"GRUPO 1","627":"GRUPO 1","628":"GRUPO 1","629":"GRUPO 1","630":"GRUPO 1","631":"GRUPO 1","632":"GRUPO 1","633":"GRUPO 1","634":"GRUPO 1","635":"GRUPO 1","636":"GRUPO 2","637":"GRUPO 2","638":"GRUPO 2","639":"GRUPO 2","640":"GRUPO 2","641":"GRUPO 2","642":"GRUPO 2","643":"GRUPO 2","644":"GRUPO 2","645":"GRUPO 2","646":"GRUPO 2","647":"GRUPO 2","648":"GRUPO 3","649":"GRUPO 3","650":"GRUPO 3","651":"GRUPO 3","652":"GRUPO 3","653":"GRUPO 3","654":"GRUPO 3","655":"GRUPO 3","656":"GRUPO 3","657":"GRUPO 3","658":"GRUPO 3","659":"GRUPO 3","660":"GRUPO 4","661":"GRUPO 4","662":"GRUPO 4","663":"GRUPO 4","664":"GRUPO 4","665":"GRUPO 4","666":"GRUPO 4","667":"GRUPO 4","668":"GRUPO 4","669":"GRUPO 4","670":"GRUPO 4","671":"GRUPO 4","672":"GRUPO 1","673":"GRUPO 1","674":"GRUPO 1","675":"GRUPO 1","676":"GRUPO 1","677":"GRUPO 1","678":"GRUPO 1","679":"GRUPO 1","680":"GRUPO 1","681":"GRUPO 1","682":"GRUPO 1","683":"GRUPO 1","684":"GRUPO 2","685":"GRUPO 2","686":"GRUPO 2","687":"GRUPO 2","688":"GRUPO 2","689":"GRUPO 2","690":"GRUPO 2","691":"GRUPO 2","692":"GRUPO 2","693":"GRUPO 2","694":"GRUPO 2","695":"GRUPO 2","696":"GRUPO 3","697":"GRUPO 3","698":"GRUPO 3","699":"GRUPO 3","700":"GRUPO 3","701":"GRUPO 3","702":"GRUPO 3","703":"GRUPO 3","704":"GRUPO 3","705":"GRUPO 3","706":"GRUPO 3","707":"GRUPO 3","708":"GRUPO 4","709":"GRUPO 4","710":"GRUPO 4","711":"GRUPO 4","712":"GRUPO 4","713":"GRUPO 4","714":"GRUPO 4","715":"GRUPO 4","716":"GRUPO 4","717":"GRUPO 4","718":"GRUPO 4","719":"GRUPO 4","720":"GRUPO 1","721":"GRUPO 1","722":"GRUPO 1","723":"GRUPO 1","724":"GRUPO 1","725":"GRUPO 1","726":"GRUPO 1","727":"GRUPO 1","728":"GRUPO 1","729":"GRUPO 1","730":"GRUPO 1","731":"GRUPO 1","732":"GRUPO 2","733":"GRUPO 2","734":"GRUPO 2","735":"GRUPO 2","736":"GRUPO 2","737":"GRUPO 2","738":"GRUPO 2","739":"GRUPO 2","740":"GRUPO 2","741":"GRUPO 2","742":"GRUPO 2","743":"GRUPO 2","744":"GRUPO 3","745":"GRUPO 3","746":"GRUPO 3","747":"GRUPO 3","748":"GRUPO 3","749":"GRUPO 3","750":"GRUPO 3","751":"GRUPO 3","752":"GRUPO 3","753":"GRUPO 3","754":"GRUPO 3","755":"GRUPO 3","756":"GRUPO 4","757":"GRUPO 4","758":"GRUPO 4","759":"GRUPO 4","760":"GRUPO 4","761":"GRUPO 4","762":"GRUPO 4","763":"GRUPO 4","764":"GRUPO 4","765":"GRUPO 4","766":"GRUPO 4","767":"GRUPO 4","768":"GRUPO 1","769":"GRUPO 1","770":"GRUPO 1","771":"GRUPO 1","772":"GRUPO 1","773":"GRUPO 1","774":"GRUPO 1","775":"GRUPO 1","776":"GRUPO 1","777":"GRUPO 1","778":"GRUPO 1","779":"GRUPO 1","780":"GRUPO 2","781":"GRUPO 2","782":"GRUPO 2","783":"GRUPO 2","784":"GRUPO 2","785":"GRUPO 2","786":"GRUPO 2","787":"GRUPO 2","788":"GRUPO 2","789":"GRUPO 2","790":"GRUPO 2","791":"GRUPO 2","792":"GRUPO 3","793":"GRUPO 3","794":"GRUPO 3","795":"GRUPO 3","796":"GRUPO 3","797":"GRUPO 3","798":"GRUPO 3","799":"GRUPO 3","800":"GRUPO 3","801":"GRUPO 3","802":"GRUPO 3","803":"GRUPO 3","804":"GRUPO 4","805":"GRUPO 4","806":"GRUPO 4","807":"GRUPO 4","808":"GRUPO 4","809":"GRUPO 4","810":"GRUPO 4","811":"GRUPO 4","812":"GRUPO 4","813":"GRUPO 4","814":"GRUPO 4","815":"GRUPO 4","816":"GRUPO 1","817":"GRUPO 1","818":"GRUPO 1","819":"GRUPO 1","820":"GRUPO 1","821":"GRUPO 1","822":"GRUPO 1","823":"GRUPO 1","824":"GRUPO 1","825":"GRUPO 1","826":"GRUPO 1","827":"GRUPO 1","828":"GRUPO 2","829":"GRUPO 2","830":"GRUPO 2","831":"GRUPO 2","832":"GRUPO 2","833":"GRUPO 2","834":"GRUPO 2","835":"GRUPO 2","836":"GRUPO 2","837":"GRUPO 2","838":"GRUPO 2","839":"GRUPO 2","840":"GRUPO 3","841":"GRUPO 3","842":"GRUPO 3","843":"GRUPO 3","844":"GRUPO 3","845":"GRUPO 3","846":"GRUPO 3","847":"GRUPO 3","848":"GRUPO 3","849":"GRUPO 3","850":"GRUPO 3","851":"GRUPO 3","852":"GRUPO 4","853":"GRUPO 4","854":"GRUPO 4","855":"GRUPO 4","856":"GRUPO 4","857":"GRUPO 4","858":"GRUPO 4","859":"GRUPO 4","860":"GRUPO 4","861":"GRUPO 4","862":"GRUPO 4","863":"GRUPO 4","864":"GRUPO 1","865":"GRUPO 1","866":"GRUPO 1","867":"GRUPO 1","868":"GRUPO 1","869":"GRUPO 1","870":"GRUPO 1","871":"GRUPO 1","872":"GRUPO 1","873":"GRUPO 1","874":"GRUPO 1","875":"GRUPO 1","876":"GRUPO 2","877":"GRUPO 2","878":"GRUPO 2","879":"GRUPO 2","880":"GRUPO 2","881":"GRUPO 2","882":"GRUPO 2","883":"GRUPO 2","884":"GRUPO 2","885":"GRUPO 2","886":"GRUPO 2","887":"GRUPO 2","888":"GRUPO 3","889":"GRUPO 3","890":"GRUPO 3","891":"GRUPO 3","892":"GRUPO 3","893":"GRUPO 3","894":"GRUPO 3","895":"GRUPO 3","896":"GRUPO 3","897":"GRUPO 3","898":"GRUPO 3","899":"GRUPO 3","900":"GRUPO 4","901":"GRUPO 4","902":"GRUPO 4","903":"GRUPO 4","904":"GRUPO 4","905":"GRUPO 4","906":"GRUPO 4","907":"GRUPO 4","908":"GRUPO 4","909":"GRUPO 4","910":"GRUPO 4","911":"GRUPO 4","912":"GRUPO 1","913":"GRUPO 1","914":"GRUPO 1","915":"GRUPO 1","916":"GRUPO 1","917":"GRUPO 1","918":"GRUPO 1","919":"GRUPO 1","920":"GRUPO 1","921":"GRUPO 1","922":"GRUPO 1","923":"GRUPO 1","924":"GRUPO 2","925":"GRUPO 2","926":"GRUPO 2","927":"GRUPO 2","928":"GRUPO 2","929":"GRUPO 2","930":"GRUPO 2","931":"GRUPO 2","932":"GRUPO 2","933":"GRUPO 2","934":"GRUPO 2","935":"GRUPO 2","936":"GRUPO 3","937":"GRUPO 3","938":"GRUPO 3","939":"GRUPO 3","940":"GRUPO 3","941":"GRUPO 3","942":"GRUPO 3","943":"GRUPO 3","944":"GRUPO 3","945":"GRUPO 3","946":"GRUPO 3","947":"GRUPO 3","948":"GRUPO 4","949":"GRUPO 4","950":"GRUPO 4","951":"GRUPO 4","952":"GRUPO 4","953":"GRUPO 4","954":"GRUPO 4","955":"GRUPO 4","956":"GRUPO 4","957":"GRUPO 4","958":"GRUPO 4","959":"GRUPO 4","960":"GRUPO 1","961":"GRUPO 1","962":"GRUPO 1","963":"GRUPO 1","964":"GRUPO 1","965":"GRUPO 1","966":"GRUPO 1","967":"GRUPO 1","968":"GRUPO 1","969":"GRUPO 1","970":"GRUPO 1","971":"GRUPO 1","972":"GRUPO 2","973":"GRUPO 2","974":"GRUPO 2","975":"GRUPO 2","976":"GRUPO 2","977":"GRUPO 2","978":"GRUPO 2","979":"GRUPO 2","980":"GRUPO 2","981":"GRUPO 2","982":"GRUPO 2","983":"GRUPO 2","984":"GRUPO 3","985":"GRUPO 3","986":"GRUPO 3","987":"GRUPO 3","988":"GRUPO 3","989":"GRUPO 3","990":"GRUPO 3","991":"GRUPO 3","992":"GRUPO 3","993":"GRUPO 3","994":"GRUPO 3","995":"GRUPO 3","996":"GRUPO 4","997":"GRUPO 4","998":"GRUPO 4","999":"GRUPO 4","1000":"GRUPO 4","1001":"GRUPO 4","1002":"GRUPO 4","1003":"GRUPO 4","1004":"GRUPO 4","1005":"GRUPO 4","1006":"GRUPO 4","1007":"GRUPO 4","1008":"GRUPO 1","1009":"GRUPO 1","1010":"GRUPO 1","1011":"GRUPO 1","1012":"GRUPO 1","1013":"GRUPO 1","1014":"GRUPO 1","1015":"GRUPO 1","1016":"GRUPO 1","1017":"GRUPO 1","1018":"GRUPO 1","1019":"GRUPO 1","1020":"GRUPO 2","1021":"GRUPO 2","1022":"GRUPO 2","1023":"GRUPO 2","1024":"GRUPO 2","1025":"GRUPO 2","1026":"GRUPO 2","1027":"GRUPO 2","1028":"GRUPO 2","1029":"GRUPO 2","1030":"GRUPO 2","1031":"GRUPO 2","1032":"GRUPO 3","1033":"GRUPO 3","1034":"GRUPO 3","1035":"GRUPO 3","1036":"GRUPO 3","1037":"GRUPO 3","1038":"GRUPO 3","1039":"GRUPO 3","1040":"GRUPO 3","1041":"GRUPO 3","1042":"GRUPO 3","1043":"GRUPO 3","1044":"GRUPO 4","1045":"GRUPO 4","1046":"GRUPO 4","1047":"GRUPO 4","1048":"GRUPO 4","1049":"GRUPO 4","1050":"GRUPO 4","1051":"GRUPO 4","1052":"GRUPO 4","1053":"GRUPO 4","1054":"GRUPO 4","1055":"GRUPO 4","1056":"GRUPO 1","1057":"GRUPO 1","1058":"GRUPO 1","1059":"GRUPO 1","1060":"GRUPO 1","1061":"GRUPO 1","1062":"GRUPO 1","1063":"GRUPO 1","1064":"GRUPO 1","1065":"GRUPO 1","1066":"GRUPO 1","1067":"GRUPO 1","1068":"GRUPO 2","1069":"GRUPO 2","1070":"GRUPO 2","1071":"GRUPO 2","1072":"GRUPO 2","1073":"GRUPO 2","1074":"GRUPO 2","1075":"GRUPO 2","1076":"GRUPO 2","1077":"GRUPO 2","1078":"GRUPO 2","1079":"GRUPO 2","1080":"GRUPO 3","1081":"GRUPO 3","1082":"GRUPO 3","1083":"GRUPO 3","1084":"GRUPO 3","1085":"GRUPO 3","1086":"GRUPO 3","1087":"GRUPO 3","1088":"GRUPO 3","1089":"GRUPO 3","1090":"GRUPO 3","1091":"GRUPO 3","1092":"GRUPO 4","1093":"GRUPO 4","1094":"GRUPO 4","1095":"GRUPO 4","1096":"GRUPO 4","1097":"GRUPO 4","1098":"GRUPO 4","1099":"GRUPO 4","1100":"GRUPO 4","1101":"GRUPO 4","1102":"GRUPO 4","1103":"GRUPO 4","1104":"GRUPO 1","1105":"GRUPO 1","1106":"GRUPO 1","1107":"GRUPO 1","1108":"GRUPO 1","1109":"GRUPO 1","1110":"GRUPO 1","1111":"GRUPO 1","1112":"GRUPO 1","1113":"GRUPO 1","1114":"GRUPO 1","1115":"GRUPO 1","1116":"GRUPO 2","1117":"GRUPO 2","1118":"GRUPO 2","1119":"GRUPO 2","1120":"GRUPO 2","1121":"GRUPO 2","1122":"GRUPO 2","1123":"GRUPO 2","1124":"GRUPO 2","1125":"GRUPO 2","1126":"GRUPO 2","1127":"GRUPO 2","1128":"GRUPO 3","1129":"GRUPO 3","1130":"GRUPO 3","1131":"GRUPO 3","1132":"GRUPO 3","1133":"GRUPO 3","1134":"GRUPO 3","1135":"GRUPO 3","1136":"GRUPO 3","1137":"GRUPO 3","1138":"GRUPO 3","1139":"GRUPO 3","1140":"GRUPO 4","1141":"GRUPO 4","1142":"GRUPO 4","1143":"GRUPO 4","1144":"GRUPO 4","1145":"GRUPO 4","1146":"GRUPO 4","1147":"GRUPO 4","1148":"GRUPO 4","1149":"GRUPO 4","1150":"GRUPO 4","1151":"GRUPO 4","1152":"GRUPO 1","1153":"GRUPO 1","1154":"GRUPO 1","1155":"GRUPO 1","1156":"GRUPO 1","1157":"GRUPO 1","1158":"GRUPO 1","1159":"GRUPO 1","1160":"GRUPO 1","1161":"GRUPO 1","1162":"GRUPO 1","1163":"GRUPO 1","1164":"GRUPO 2","1165":"GRUPO 2","1166":"GRUPO 2","1167":"GRUPO 2","1168":"GRUPO 2","1169":"GRUPO 2","1170":"GRUPO 2","1171":"GRUPO 2","1172":"GRUPO 2","1173":"GRUPO 2","1174":"GRUPO 2","1175":"GRUPO 2","1176":"GRUPO 3","1177":"GRUPO 3","1178":"GRUPO 3","1179":"GRUPO 3","1180":"GRUPO 3","1181":"GRUPO 3","1182":"GRUPO 3","1183":"GRUPO 3","1184":"GRUPO 3","1185":"GRUPO 3","1186":"GRUPO 3","1187":"GRUPO 3","1188":"GRUPO 4","1189":"GRUPO 4","1190":"GRUPO 4","1191":"GRUPO 4","1192":"GRUPO 4","1193":"GRUPO 4","1194":"GRUPO 4","1195":"GRUPO 4","1196":"GRUPO 4","1197":"GRUPO 4","1198":"GRUPO 4","1199":"GRUPO 4","1200":"GRUPO 1","1201":"GRUPO 1","1202":"GRUPO 1","1203":"GRUPO 1","1204":"GRUPO 1","1205":"GRUPO 1","1206":"GRUPO 1","1207":"GRUPO 1","1208":"GRUPO 1","1209":"GRUPO 1","1210":"GRUPO 1","1211":"GRUPO 1","1212":"GRUPO 2","1213":"GRUPO 2","1214":"GRUPO 2","1215":"GRUPO 2","1216":"GRUPO 2","1217":"GRUPO 2","1218":"GRUPO 2","1219":"GRUPO 2","1220":"GRUPO 2","1221":"GRUPO 2","1222":"GRUPO 2","1223":"GRUPO 2","1224":"GRUPO 3","1225":"GRUPO 3","1226":"GRUPO 3","1227":"GRUPO 3","1228":"GRUPO 3","1229":"GRUPO 3","1230":"GRUPO 3","1231":"GRUPO 3","1232":"GRUPO 3","1233":"GRUPO 3","1234":"GRUPO 3","1235":"GRUPO 3","1236":"GRUPO 4","1237":"GRUPO 4","1238":"GRUPO 4","1239":"GRUPO 4","1240":"GRUPO 4","1241":"GRUPO 4","1242":"GRUPO 4","1243":"GRUPO 4","1244":"GRUPO 4","1245":"GRUPO 4","1246":"GRUPO 4","1247":"GRUPO 4","1248":"GRUPO 1","1249":"GRUPO 1","1250":"GRUPO 1","1251":"GRUPO 1","1252":"GRUPO 1","1253":"GRUPO 1","1254":"GRUPO 1","1255":"GRUPO 1","1256":"GRUPO 1","1257":"GRUPO 1","1258":"GRUPO 1","1259":"GRUPO 1","1260":"GRUPO 2","1261":"GRUPO 2","1262":"GRUPO 2","1263":"GRUPO 2","1264":"GRUPO 2","1265":"GRUPO 2","1266":"GRUPO 2","1267":"GRUPO 2","1268":"GRUPO 2","1269":"GRUPO 2","1270":"GRUPO 2","1271":"GRUPO 2","1272":"GRUPO 3","1273":"GRUPO 3","1274":"GRUPO 3","1275":"GRUPO 3","1276":"GRUPO 3","1277":"GRUPO 3","1278":"GRUPO 3","1279":"GRUPO 3","1280":"GRUPO 3","1281":"GRUPO 3","1282":"GRUPO 3","1283":"GRUPO 3","1284":"GRUPO 4","1285":"GRUPO 4","1286":"GRUPO 4","1287":"GRUPO 4","1288":"GRUPO 4","1289":"GRUPO 4","1290":"GRUPO 4","1291":"GRUPO 4","1292":"GRUPO 4","1293":"GRUPO 4","1294":"GRUPO 4","1295":"GRUPO 4","1296":"GRUPO 1","1297":"GRUPO 1","1298":"GRUPO 1","1299":"GRUPO 1","1300":"GRUPO 1","1301":"GRUPO 1","1302":"GRUPO 1","1303":"GRUPO 1","1304":"GRUPO 1","1305":"GRUPO 1","1306":"GRUPO 1","1307":"GRUPO 1","1308":"GRUPO 2","1309":"GRUPO 2","1310":"GRUPO 2","1311":"GRUPO 2","1312":"GRUPO 2","1313":"GRUPO 2","1314":"GRUPO 2","1315":"GRUPO 2","1316":"GRUPO 2","1317":"GRUPO 2","1318":"GRUPO 2","1319":"GRUPO 2","1320":"GRUPO 3","1321":"GRUPO 3","1322":"GRUPO 3","1323":"GRUPO 3","1324":"GRUPO 3","1325":"GRUPO 3","1326":"GRUPO 3","1327":"GRUPO 3","1328":"GRUPO 3","1329":"GRUPO 3","1330":"GRUPO 3","1331":"GRUPO 3","1332":"GRUPO 4","1333":"GRUPO 4","1334":"GRUPO 4","1335":"GRUPO 4","1336":"GRUPO 4","1337":"GRUPO 4","1338":"GRUPO 4","1339":"GRUPO 4","1340":"GRUPO 4","1341":"GRUPO 4","1342":"GRUPO 4","1343":"GRUPO 4","1344":"GRUPO 1","1345":"GRUPO 1","1346":"GRUPO 1","1347":"GRUPO 1","1348":"GRUPO 1","1349":"GRUPO 1","1350":"GRUPO 1","1351":"GRUPO 1","1352":"GRUPO 1","1353":"GRUPO 1","1354":"GRUPO 1","1355":"GRUPO 1","1356":"GRUPO 2","1357":"GRUPO 2","1358":"GRUPO 2","1359":"GRUPO 2","1360":"GRUPO 2","1361":"GRUPO 2","1362":"GRUPO 2","1363":"GRUPO 2","1364":"GRUPO 2","1365":"GRUPO 2","1366":"GRUPO 2","1367":"GRUPO 2","1368":"GRUPO 3","1369":"GRUPO 3","1370":"GRUPO 3","1371":"GRUPO 3","1372":"GRUPO 3","1373":"GRUPO 3","1374":"GRUPO 3","1375":"GRUPO 3","1376":"GRUPO 3","1377":"GRUPO 3","1378":"GRUPO 3","1379":"GRUPO 3","1380":"GRUPO 4","1381":"GRUPO 4","1382":"GRUPO 4","1383":"GRUPO 4","1384":"GRUPO 4","1385":"GRUPO 4","1386":"GRUPO 4","1387":"GRUPO 4","1388":"GRUPO 4","1389":"GRUPO 4","1390":"GRUPO 4","1391":"GRUPO 4","1392":"GRUPO 1","1393":"GRUPO 1","1394":"GRUPO 1","1395":"GRUPO 1","1396":"GRUPO 1","1397":"GRUPO 1","1398":"GRUPO 1","1399":"GRUPO 1","1400":"GRUPO 1","1401":"GRUPO 1","1402":"GRUPO 1","1403":"GRUPO 1","1404":"GRUPO 2","1405":"GRUPO 2","1406":"GRUPO 2","1407":"GRUPO 2","1408":"GRUPO 2","1409":"GRUPO 2","1410":"GRUPO 2","1411":"GRUPO 2","1412":"GRUPO 2","1413":"GRUPO 2","1414":"GRUPO 2","1415":"GRUPO 2","1416":"GRUPO 3","1417":"GRUPO 3","1418":"GRUPO 3","1419":"GRUPO 3","1420":"GRUPO 3","1421":"GRUPO 3","1422":"GRUPO 3","1423":"GRUPO 3","1424":"GRUPO 3","1425":"GRUPO 3","1426":"GRUPO 3","1427":"GRUPO 3","1428":"GRUPO 4","1429":"GRUPO 4","1430":"GRUPO 4","1431":"GRUPO 4","1432":"GRUPO 4","1433":"GRUPO 4","1434":"GRUPO 4","1435":"GRUPO 4","1436":"GRUPO 4","1437":"GRUPO 4","1438":"GRUPO 4","1439":"GRUPO 4"},"Empleado":{"0":"BARON HERNANDEZ HAROLD ANTONIO","1":"CASTELLANOS CARVAJAL DEYVITH FABIAN","2":"AROCA TORRES JULIAN EDUARDO","3":"BERMUDEZ PARRA JENNIFER XIOMARA","4":"BERNAL BAQUERO JAMES RICARDO","5":"BURGOS ORTIZ JOSE HORACIO","6":"CANTOR PORRAS JUAN FERNEY","7":"CAPERA CAPERA JOSE GABRIEL","8":"CARDENAS LOTERO RICARDO ANDR\u00c9S","9":"RENDON OSPINA NELSON LEANDRO","10":"SARMIENTO URBINA MOISES DANIEL","11":"VELASCO VELASCO SEBASTI\u00c1N DAVID","12":"DELGADO DELGADO JOHAN DARIO","13":"FLOREZ SAUCESO KENIS ALBERTO","14":"CARDONA GARCIA OSCAR JAVIER","15":"CARVAJAL GARC\u00cdA HOVER MARCK","16":"CEPEDA PIRAQUIVE JUAN DAVID","17":"FAJARDO SAENZ OSCAR FERNANDO","18":"FLOREZ ESPITIA RONY ALBERTO","19":"GARCIA CUERVO EDWIN JAVIER","20":"GONZALEZ OCHOA JUAN CARLOS","21":"XXX1","22":"XXX2","23":"XXX3","24":"FONSECA RAY RICARDO","25":"GOMEZ BETANCUR JAIDER ANDRES","26":"GRANADA PATI\u00d1O CARLOS MARINO","27":"GRASS PLATA MIGUEL SNEIDER","28":"MANZANO CALVO JUAN SEBASTIAN","29":"MENDOZA GOITA MARIANSEL ZENAYDA","30":"MURILLO ARAQUE JAIVER GEOVANY","31":"NI\u00d1O ARENAS HECTOR GONZALO","32":"RAMIREZ CHAVERRA JHON EDISON","33":"XXX4","34":"XXX5","35":"XXX6","36":"RODRIGUEZ MOSQUERA LUIS FERNANDO","37":"PEPITO PEREZ","38":"RAMIREZ VARGAS MARCELA PAOLA","39":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","40":"TORO CISNEROS GARY JOSE","41":"USECHE CALDERON JADID ESTIVEN","42":"VASQUEZ NIETO CAMILO ANDRES","43":"JHONY CASTRO","44":"BERNAL JUAN DAVID","45":"XXX7","46":"XXX8","47":"XXX9","48":"BARON HERNANDEZ HAROLD ANTONIO","49":"CASTELLANOS CARVAJAL DEYVITH FABIAN","50":"AROCA TORRES JULIAN EDUARDO","51":"BERMUDEZ PARRA JENNIFER XIOMARA","52":"BERNAL BAQUERO JAMES RICARDO","53":"BURGOS ORTIZ JOSE HORACIO","54":"CANTOR PORRAS JUAN FERNEY","55":"CAPERA CAPERA JOSE GABRIEL","56":"CARDENAS LOTERO RICARDO ANDR\u00c9S","57":"RENDON OSPINA NELSON LEANDRO","58":"SARMIENTO URBINA MOISES DANIEL","59":"VELASCO VELASCO SEBASTI\u00c1N DAVID","60":"DELGADO DELGADO JOHAN DARIO","61":"FLOREZ SAUCESO KENIS ALBERTO","62":"CARDONA GARCIA OSCAR JAVIER","63":"CARVAJAL GARC\u00cdA HOVER MARCK","64":"CEPEDA PIRAQUIVE JUAN DAVID","65":"FAJARDO SAENZ OSCAR FERNANDO","66":"FLOREZ ESPITIA RONY ALBERTO","67":"GARCIA CUERVO EDWIN JAVIER","68":"GONZALEZ OCHOA JUAN CARLOS","69":"XXX1","70":"XXX2","71":"XXX3","72":"FONSECA RAY RICARDO","73":"GOMEZ BETANCUR JAIDER ANDRES","74":"GRANADA PATI\u00d1O CARLOS MARINO","75":"GRASS PLATA MIGUEL SNEIDER","76":"MANZANO CALVO JUAN SEBASTIAN","77":"MENDOZA GOITA MARIANSEL ZENAYDA","78":"MURILLO ARAQUE JAIVER GEOVANY","79":"NI\u00d1O ARENAS HECTOR GONZALO","80":"RAMIREZ CHAVERRA JHON EDISON","81":"XXX4","82":"XXX5","83":"XXX6","84":"RODRIGUEZ MOSQUERA LUIS FERNANDO","85":"PEPITO PEREZ","86":"RAMIREZ VARGAS MARCELA PAOLA","87":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","88":"TORO CISNEROS GARY JOSE","89":"USECHE CALDERON JADID ESTIVEN","90":"VASQUEZ NIETO CAMILO ANDRES","91":"JHONY CASTRO","92":"BERNAL JUAN DAVID","93":"XXX7","94":"XXX8","95":"XXX9","96":"BARON HERNANDEZ HAROLD ANTONIO","97":"CASTELLANOS CARVAJAL DEYVITH FABIAN","98":"AROCA TORRES JULIAN EDUARDO","99":"BERMUDEZ PARRA JENNIFER XIOMARA","100":"BERNAL BAQUERO JAMES RICARDO","101":"BURGOS ORTIZ JOSE HORACIO","102":"CANTOR PORRAS JUAN FERNEY","103":"CAPERA CAPERA JOSE GABRIEL","104":"CARDENAS LOTERO RICARDO ANDR\u00c9S","105":"RENDON OSPINA NELSON LEANDRO","106":"SARMIENTO URBINA MOISES DANIEL","107":"VELASCO VELASCO SEBASTI\u00c1N DAVID","108":"DELGADO DELGADO JOHAN DARIO","109":"FLOREZ SAUCESO KENIS ALBERTO","110":"CARDONA GARCIA OSCAR JAVIER","111":"CARVAJAL GARC\u00cdA HOVER MARCK","112":"CEPEDA PIRAQUIVE JUAN DAVID","113":"FAJARDO SAENZ OSCAR FERNANDO","114":"FLOREZ ESPITIA RONY ALBERTO","115":"GARCIA CUERVO EDWIN JAVIER","116":"GONZALEZ OCHOA JUAN CARLOS","117":"XXX1","118":"XXX2","119":"XXX3","120":"FONSECA RAY RICARDO","121":"GOMEZ BETANCUR JAIDER ANDRES","122":"GRANADA PATI\u00d1O CARLOS MARINO","123":"GRASS PLATA MIGUEL SNEIDER","124":"MANZANO CALVO JUAN SEBASTIAN","125":"MENDOZA GOITA MARIANSEL ZENAYDA","126":"MURILLO ARAQUE JAIVER GEOVANY","127":"NI\u00d1O ARENAS HECTOR GONZALO","128":"RAMIREZ CHAVERRA JHON EDISON","129":"XXX4","130":"XXX5","131":"XXX6","132":"RODRIGUEZ MOSQUERA LUIS FERNANDO","133":"PEPITO PEREZ","134":"RAMIREZ VARGAS MARCELA PAOLA","135":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","136":"TORO CISNEROS GARY JOSE","137":"USECHE CALDERON JADID ESTIVEN","138":"VASQUEZ NIETO CAMILO ANDRES","139":"JHONY CASTRO","140":"BERNAL JUAN DAVID","141":"XXX7","142":"XXX8","143":"XXX9","144":"BARON HERNANDEZ HAROLD ANTONIO","145":"CASTELLANOS CARVAJAL DEYVITH FABIAN","146":"AROCA TORRES JULIAN EDUARDO","147":"BERMUDEZ PARRA JENNIFER XIOMARA","148":"BERNAL BAQUERO JAMES RICARDO","149":"BURGOS ORTIZ JOSE HORACIO","150":"CANTOR PORRAS JUAN FERNEY","151":"CAPERA CAPERA JOSE GABRIEL","152":"CARDENAS LOTERO RICARDO ANDR\u00c9S","153":"RENDON OSPINA NELSON LEANDRO","154":"SARMIENTO URBINA MOISES DANIEL","155":"VELASCO VELASCO SEBASTI\u00c1N DAVID","156":"DELGADO DELGADO JOHAN DARIO","157":"FLOREZ SAUCESO KENIS ALBERTO","158":"CARDONA GARCIA OSCAR JAVIER","159":"CARVAJAL GARC\u00cdA HOVER MARCK","160":"CEPEDA PIRAQUIVE JUAN DAVID","161":"FAJARDO SAENZ OSCAR FERNANDO","162":"FLOREZ ESPITIA RONY ALBERTO","163":"GARCIA CUERVO EDWIN JAVIER","164":"GONZALEZ OCHOA JUAN CARLOS","165":"XXX1","166":"XXX2","167":"XXX3","168":"FONSECA RAY RICARDO","169":"GOMEZ BETANCUR JAIDER ANDRES","170":"GRANADA PATI\u00d1O CARLOS MARINO","171":"GRASS PLATA MIGUEL SNEIDER","172":"MANZANO CALVO JUAN SEBASTIAN","173":"MENDOZA GOITA MARIANSEL ZENAYDA","174":"MURILLO ARAQUE JAIVER GEOVANY","175":"NI\u00d1O ARENAS HECTOR GONZALO","176":"RAMIREZ CHAVERRA JHON EDISON","177":"XXX4","178":"XXX5","179":"XXX6","180":"RODRIGUEZ MOSQUERA LUIS FERNANDO","181":"PEPITO PEREZ","182":"RAMIREZ VARGAS MARCELA PAOLA","183":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","184":"TORO CISNEROS GARY JOSE","185":"USECHE CALDERON JADID ESTIVEN","186":"VASQUEZ NIETO CAMILO ANDRES","187":"JHONY CASTRO","188":"BERNAL JUAN DAVID","189":"XXX7","190":"XXX8","191":"XXX9","192":"BARON HERNANDEZ HAROLD ANTONIO","193":"CASTELLANOS CARVAJAL DEYVITH FABIAN","194":"AROCA TORRES JULIAN EDUARDO","195":"BERMUDEZ PARRA JENNIFER XIOMARA","196":"BERNAL BAQUERO JAMES RICARDO","197":"BURGOS ORTIZ JOSE HORACIO","198":"CANTOR PORRAS JUAN FERNEY","199":"CAPERA CAPERA JOSE GABRIEL","200":"CARDENAS LOTERO RICARDO ANDR\u00c9S","201":"RENDON OSPINA NELSON LEANDRO","202":"SARMIENTO URBINA MOISES DANIEL","203":"VELASCO VELASCO SEBASTI\u00c1N DAVID","204":"DELGADO DELGADO JOHAN DARIO","205":"FLOREZ SAUCESO KENIS ALBERTO","206":"CARDONA GARCIA OSCAR JAVIER","207":"CARVAJAL GARC\u00cdA HOVER MARCK","208":"CEPEDA PIRAQUIVE JUAN DAVID","209":"FAJARDO SAENZ OSCAR FERNANDO","210":"FLOREZ ESPITIA RONY ALBERTO","211":"GARCIA CUERVO EDWIN JAVIER","212":"GONZALEZ OCHOA JUAN CARLOS","213":"XXX1","214":"XXX2","215":"XXX3","216":"FONSECA RAY RICARDO","217":"GOMEZ BETANCUR JAIDER ANDRES","218":"GRANADA PATI\u00d1O CARLOS MARINO","219":"GRASS PLATA MIGUEL SNEIDER","220":"MANZANO CALVO JUAN SEBASTIAN","221":"MENDOZA GOITA MARIANSEL ZENAYDA","222":"MURILLO ARAQUE JAIVER GEOVANY","223":"NI\u00d1O ARENAS HECTOR GONZALO","224":"RAMIREZ CHAVERRA JHON EDISON","225":"XXX4","226":"XXX5","227":"XXX6","228":"RODRIGUEZ MOSQUERA LUIS FERNANDO","229":"PEPITO PEREZ","230":"RAMIREZ VARGAS MARCELA PAOLA","231":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","232":"TORO CISNEROS GARY JOSE","233":"USECHE CALDERON JADID ESTIVEN","234":"VASQUEZ NIETO CAMILO ANDRES","235":"JHONY CASTRO","236":"BERNAL JUAN DAVID","237":"XXX7","238":"XXX8","239":"XXX9","240":"BARON HERNANDEZ HAROLD ANTONIO","241":"CASTELLANOS CARVAJAL DEYVITH FABIAN","242":"AROCA TORRES JULIAN EDUARDO","243":"BERMUDEZ PARRA JENNIFER XIOMARA","244":"BERNAL BAQUERO JAMES RICARDO","245":"BURGOS ORTIZ JOSE HORACIO","246":"CANTOR PORRAS JUAN FERNEY","247":"CAPERA CAPERA JOSE GABRIEL","248":"CARDENAS LOTERO RICARDO ANDR\u00c9S","249":"RENDON OSPINA NELSON LEANDRO","250":"SARMIENTO URBINA MOISES DANIEL","251":"VELASCO VELASCO SEBASTI\u00c1N DAVID","252":"DELGADO DELGADO JOHAN DARIO","253":"FLOREZ SAUCESO KENIS ALBERTO","254":"CARDONA GARCIA OSCAR JAVIER","255":"CARVAJAL GARC\u00cdA HOVER MARCK","256":"CEPEDA PIRAQUIVE JUAN DAVID","257":"FAJARDO SAENZ OSCAR FERNANDO","258":"FLOREZ ESPITIA RONY ALBERTO","259":"GARCIA CUERVO EDWIN JAVIER","260":"GONZALEZ OCHOA JUAN CARLOS","261":"XXX1","262":"XXX2","263":"XXX3","264":"FONSECA RAY RICARDO","265":"GOMEZ BETANCUR JAIDER ANDRES","266":"GRANADA PATI\u00d1O CARLOS MARINO","267":"GRASS PLATA MIGUEL SNEIDER","268":"MANZANO CALVO JUAN SEBASTIAN","269":"MENDOZA GOITA MARIANSEL ZENAYDA","270":"MURILLO ARAQUE JAIVER GEOVANY","271":"NI\u00d1O ARENAS HECTOR GONZALO","272":"RAMIREZ CHAVERRA JHON EDISON","273":"XXX4","274":"XXX5","275":"XXX6","276":"RODRIGUEZ MOSQUERA LUIS FERNANDO","277":"PEPITO PEREZ","278":"RAMIREZ VARGAS MARCELA PAOLA","279":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","280":"TORO CISNEROS GARY JOSE","281":"USECHE CALDERON JADID ESTIVEN","282":"VASQUEZ NIETO CAMILO ANDRES","283":"JHONY CASTRO","284":"BERNAL JUAN DAVID","285":"XXX7","286":"XXX8","287":"XXX9","288":"BARON HERNANDEZ HAROLD ANTONIO","289":"CASTELLANOS CARVAJAL DEYVITH FABIAN","290":"AROCA TORRES JULIAN EDUARDO","291":"BERMUDEZ PARRA JENNIFER XIOMARA","292":"BERNAL BAQUERO JAMES RICARDO","293":"BURGOS ORTIZ JOSE</t>
   </si>
   <si>
-    <t>[{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"01-Mie","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"01-Mie","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"01-Mie","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"01-Mie","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"01-Mie","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"01-Mie","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"01-Mie","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"01-Mie","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"01-Mie","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"01-Mie","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"01-Mie","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"01-Mie","Final":"DESC. LEY","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"06-Lun","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"06-Lun","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"06-Lun","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"06-Lun","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"06-Lun","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"06-Lun","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"06-Lun","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"06-Lun","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"06-Lun","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"06-Lun","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"06-Lun","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"06-Lun","Final":"DESC. LEY","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VA</t>
-  </si>
-  <si>
     <t>[{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master</t>
   </si>
   <si>
@@ -80,6 +77,9 @@
   </si>
   <si>
     <t>{"columns":["Grupo","Empleado","Cargo","Label","Final","n_dia"],"index":[0,1,2,3,4,5,6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23,24,25,26,27,28,29,30,31,32,33,34,35,36,37,38,39,40,41,42,43,44,45,46,47,48,49,50,51,52,53,54,55,56,57,58,59,60,61,62,63,64,65,66,67,68,69,70,71,72,73,74,75,76,77,78,79,80,81,82,83,84,85,86,87,88,89,90,91,92,93,94,95,96,97,98,99,100,101,102,103,104,105,106,107,108,109,110,111,112,113,114,115,116,117,118,119,120,121,122,123,124,125,126,127,128,129,130,131,132,133,134,135,136,137,138,139,140,141,142,143,144,145,146,147,148,149,150,151,152,153,154,155,156,157,158,159,160,161,162,163,164,165,166,167,168,169,170,171,172,173,174,175,176,177,178,179,180,181,182,183,184,185,186,187,188,189,190,191,192,193,194,195,196,197,198,199,200,201,202,203,204,205,206,207,208,209,210,211,212,213,214,215,216,217,218,219,220,221,222,223,224,225,226,227,228,229,230,231,232,233,234,235,236,237,238,239,240,241,242,243,244,245,246,247,248,249,250,251,252,253,254,255,256,257,258,259,260,261,262,263,264,265,266,267,268,269,270,271,272,273,274,275,276,277,278,279,280,281,282,283,284,285,286,287,288,289,290,291,292,293,294,295,296,297,298,299,300,301,302,303,304,305,306,307,308,309,310,311,312,313,314,315,316,317,318,319,320,321,322,323,324,325,326,327,328,329,330,331,332,333,334,335,336,337,338,339,340,341,342,343,344,345,346,347,348,349,350,351,352,353,354,355,356,357,358,359,360,361,362,363,364,365,366,367,368,369,370,371,372,373,374,375,376,377,378,379,380,381,382,383,384,385,386,387,388,389,390,391,392,393,394,395,396,397,398,399,400,401,402,403,404,405,406,407,408,409,410,411,412,413,414,415,416,417,418,419,420,421,422,423,424,425,426,427,428,429,430,431,432,433,434,435,436,437,438,439,440,441,442,443,444,445,446,447,448,449,450,451,452,453,454,455,456,457,458,459,460,461,462,463,464,465,466,467,468,469,470,471,472,473,474,475,476,477,478,479,480,481,482,483,484,485,486,487,488,489,490,491,492,493,494,495,496,497,498,499,500,501,502,503,504,505,506,507,508,509,510,511,512,513,514,515,516,517,518,519,520,521,522,523,524,525,526,527,528,529,530,531,532,533,534,535,536,537,538,539,540,541,542,543,544,545,546,547,548,549,550,551,552,553,554,555,556,557,558,559,560,561,562,563,564,565,566,567,568,569,570,571,572,573,574,575,576,577,578,579,580,581,582,583,584,585,586,587,588,589,590,591,592,593,594,595,596,597,598,599,600,601,602,603,604,605,606,607,608,609,610,611,612,613,614,615,616,617,618,619,620,621,622,623,624,625,626,627,628,629,630,631,632,633,634,635,636,637,638,639,640,641,642,643,644,645,646,647,648,649,650,651,652,653,654,655,656,657,658,659,660,661,662,663,664,665,666,667,668,669,670,671,672,673,674,675,676,677,678,679,680,681,682,683,684,685,686,687,688,689,690,691,692,693,694,695,696,697,698,699,700,701,702,703,704,705,706,707,708,709,710,711,712,713,714,715,716,717,718,719,720,721,722,723,724,725,726,727,728,729,730,731,732,733,734,735,736,737,738,739,740,741,742,743,744,745,746,747,748,749,750,751,752,753,754,755,756,757,758,759,760,761,762,763,764,765,766,767,768,769,770,771,772,773,774,775,776,777,778,779,780,781,782,783,784,785,786,787,788,789,790,791,792,793,794,795,796,797,798,799,800,801,802,803,804,805,806,807,808,809,810,811,812,813,814,815,816,817,818,819,820,821,822,823,824,825,826,827,828,829,830,831,832,833,834,835,836,837,838,839,840,841,842,843,844,845,846,847,848,849,850,851,852,853,854,855,856,857,858,859,860,861,862,863,864,865,866,867,868,869,870,871,872,873,874,875,876,877,878,879,880,881,882,883,884,885,886,887,888,889,890,891,892,893,894,895,896,897,898,899,900,901,902,903,904,905,906,907,908,909,910,911,912,913,914,915,916,917,918,919,920,921,922,923,924,925,926,927,928,929,930,931,932,933,934,935,936,937,938,939,940,941,942,943,944,945,946,947,948,949,950,951,952,953,954,955,956,957,958,959,960,961,962,963,964,965,966,967,968,969,970,971,972,973,974,975,976,977,978,979,980,981,982,983,984,985,986,987,988,989,990,991,992,993,994,995,996,997,998,999,1000,1001,1002,1003,1004,1005,1006,1007,1008,1009,1010,1011,1012,1013,1014,1015,1016,1017,1018,1019,1020,1021,1022,1023,1024,1025,1026,1027,1028,1029,1030,1031,1032,1033,1034,1035,1036,1037,1038,1039,1040,1041,1042,1043,1044,1045,1046,1047,1048,1049,1050,1051,1052,1053,1054,1055,1056,1057,1058,1059,1060,1061,1062,1063,1064,1065,1066,1067,1068,1069,1070,1071,1072,1073,1074,1075,1076,1077,1078,1079,1080,1081,1082,1083,1084,1085,1086,1087,1088,1089,1090,1091,1092,1093,1094,1095,1096,1097,1098,1099,1100,1101,1102,1103,1104,1105,1106,1107,1108,1109,1110,1111,1112,1113,1114,1115,1116,1117,1118,1119,1120,1121,1122,1123,1124,1125,1126,1127,1128,1129,1130,1131,1132,1133,1134,1135,1136,1137,1138,1139,1140,1141,1142,1143,1144,1145,1146,1147,1148,1149,1150,1151,1152,1153,1154,1155,1156,1157,1158,1159,1160,1161,1162,1163,1164,1165,1166,1167,1168,1169,1170,1171,1172,1173,1174,1175,1176,1177,1178,1179,1180,1181,1182,1183,1184,1185,1186,1187,1188,1189,1190,1191,1192,1193,1194,1195,1196,1197,1198,1199,1200,1201,1202,1203,1204,1205,1206,1207,1208,1209,1210,1211,1212,1213,1214,1215,1216,1217,1218,1219,1220,1221,1222,1223,1224,1225,1226,1227,1228,1229,1230,1231,1232,1233,1234,1235,1236,1237,1238,1239,1240,1241,1242,1243,1244,1245,1246,1247,1248,1249,1250,1251,1252,1253,1254,1255,1256,1257,1258,1259,1260,1261,1262,1263,1264,1265,1266,1267,1268,1269,1270,1271,1272,1273,1274,1275,1276,1277,1278,1279,1280,1281,1282,1283,1284,1285,1286,1287,1288,1289,1290,1291,1292,1293,1294,1295,1296,1297,1298,1299,1300,1301,1302,1303,1304,1305,1306,1307,1308,1309,1310,1311,1312,1313,1314,1315,1316,1317,1318,1319,1320,1321,1322,1323,1324,1325,1326,1327,1328,1329,1330,1331,1332,1333,1334,1335,1336,1337,1338,1339,1340,1341,1342,1343,1344,1345,1346,1347,1348,1349,1350,1351,1352,1353,1354,1355,1356,1357,1358,1359,1360,1361,1362,1363,1364,1365,1366,1367,1368,1369,1370,1371,1372,1373,1374,1375,1376,1377,1378,1379,1380,1381,1382,1383,1384,1385,1386,1387,1388,1389,1390,1391,1392,1393,1394,1395,1396,1397,1398,1399,1400,1401,1402,1403,1404,1405,1406,1407,1408,1409,1410,1411,1412,1413,1414,1415,1416,1417,1418,1419,1420,1421,1422,1423,1424,1425,1426,1427,1428,1429,1430,1431,1432,1433,1434,1435,1436,1437,1438,1439,1440,1441,1442,1443,1444,1445,1446,1447,1448,1449,1450,1451,1452,1453,1454,1455,1456,1457,1458,1459,1460,1461,1462,1463,1464,1465,1466,1467,1468,1469,1470,1471,1472,1473,1474,1475,1476,1477,1478,1479,1480,1481,1482,1483,1484,1485,1486,1487],"data":[["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","01-Vie","T1",1],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","01-Vie","T1",1],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","01-Vie","T1",1],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","01-Vie","T1",1],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","01-Vie","T1",1],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","01-Vie","T1",1],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","01-Vie","T1",1],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","01-Vie","T1",1],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","01-Vie","T1",1],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","01-Vie","T1",1],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","01-Vie","T1",1],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","01-Vie","T1",1],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","01-Vie","DESC. LEY",1],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","01-Vie","DESC. LEY",1],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","01-Vie","DESC. LEY",1],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","01-Vie","DESC. LEY",1],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","01-Vie","DESC. LEY",1],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","01-Vie","DESC. LEY",1],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","01-Vie","DESC. LEY",1],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","01-Vie","DESC. LEY",1],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","01-Vie","DESC. LEY",1],["GRUPO 2","XXX1","Tecnico B","01-Vie","DESC. LEY",1],["GRUPO 2","XXX2","Tecnico B","01-Vie","DESC. LEY",1],["GRUPO 2","XXX3","Tecnico B","01-Vie","DESC. LEY",1],["GRUPO 3","FONSECA RAY RICARDO","Master","01-Vie","T3",1],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","01-Vie","T3",1],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","01-Vie","T3",1],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","01-Vie","T3",1],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","01-Vie","T3",1],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","01-Vie","T3",1],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","01-Vie","T3",1],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","01-Vie","T3",1],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","01-Vie","T3",1],["GRUPO 3","XXX4","Tecnico B","01-Vie","T3",1],["GRUPO 3","XXX5","Tecnico B","01-Vie","T3",1],["GRUPO 3","XXX6","Tecnico B","01-Vie","T3",1],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","01-Vie","T2",1],["GRUPO 4","PEPITO PEREZ","Master","01-Vie","T2",1],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","01-Vie","T2",1],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","01-Vie","T2",1],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","01-Vie","T2",1],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","01-Vie","T2",1],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","01-Vie","T2",1],["GRUPO 4","JHONY CASTRO","Tecnico A","01-Vie","T2",1],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","01-Vie","T2",1],["GRUPO 4","XXX7","Tecnico B","01-Vie","T2",1],["GRUPO 4","XXX8","Tecnico B","01-Vie","T2",1],["GRUPO 4","XXX9","Tecnico B","01-Vie","T2",1],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","02-Sab","T1",2],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","02-Sab","T1",2],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","02-Sab","T1",2],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","02-Sab","T1",2],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","02-Sab","T1",2],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","02-Sab","T1",2],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","02-Sab","T1",2],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","02-Sab","T1",2],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","02-Sab","T1",2],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","02-Sab","T1",2],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","02-Sab","T1",2],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","02-Sab","T1",2],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","02-Sab","T2",2],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","02-Sab","T2",2],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","02-Sab","T2",2],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","02-Sab","T2",2],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","02-Sab","T2",2],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","02-Sab","T2",2],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","02-Sab","T2",2],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","02-Sab","T2",2],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","02-Sab","T2",2],["GRUPO 2","XXX1","Tecnico B","02-Sab","T2",2],["GRUPO 2","XXX2","Tecnico B","02-Sab","T2",2],["GRUPO 2","XXX3","Tecnico B","02-Sab","T2",2],["GRUPO 3","FONSECA RAY RICARDO","Master","02-Sab","DESC. LEY",2],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","02-Sab","DESC. LEY",2],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","02-Sab","DESC. LEY",2],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","02-Sab","DESC. LEY",2],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","02-Sab","DESC. LEY",2],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","02-Sab","DESC. LEY",2],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","02-Sab","DESC. LEY",2],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","02-Sab","DESC. LEY",2],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","02-Sab","DESC. LEY",2],["GRUPO 3","XXX4","Tecnico B","02-Sab","DESC. LEY",2],["GRUPO 3","XXX5","Tecnico B","02-Sab","DESC. LEY",2],["GRUPO 3","XXX6","Tecnico B","02-Sab","DESC. LEY",2],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","02-Sab","T3",2],["GRUPO 4","PEPITO PEREZ","Master","02-Sab","T3",2],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","02-Sab","T3",2],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","02-Sab","T3",2],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","02-Sab","T3",2],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","02-Sab","T3",2],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","02-Sab","T3",2],["GRUPO 4","JHONY CASTRO","Tecnico A","02-Sab","T3",2],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","02-Sab","T3",2],["GRUPO 4","XXX7","Tecnico B","02-Sab","T3",2],["GRUPO 4","XXX8","Tecnico B","02-Sab","T3",2],["GRUPO 4","XXX9","Tecnico B","02-Sab","T3",2],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","03-Dom","T1",3],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","03-Dom","T1",3],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","03-Dom","T1",3],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","03-Dom","T1",3],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","03-Dom","T1",3],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","03-Dom","T1",3],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","03-Dom","T1",3],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","03-Dom","T1",3],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","03-Dom","T1",3],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","03-Dom","T1",3],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","03-Dom","T1",3],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","03-Dom","T1",3],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","03-Dom","T2",3],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","03-Dom","T2",3],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","03-Dom","T2",3],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","03-Dom","T2",3],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","03-Dom","T2",3],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","03-Dom","T2",3],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","03-Dom","T2",3],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","03-Dom","T2",3],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","03-Dom","T2",3],["GRUPO 2","XXX1","Tecnico B","03-Dom","T2",3],["GRUPO 2","XXX2","Tecnico B","03-Dom","T2",3],["GRUPO 2","XXX3","Tecnico B","03-Dom","T2",3],["GRUPO 3","FONSECA RAY RICARDO","Master","03-Dom","T3",3],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","03-Dom","T3",3],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","03-Dom","T3",3],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","03-Dom","T3",3],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","03-Dom","T3",3],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","03-Dom","T3",3],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","03-Dom","T3",3],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","03-Dom","T3",3],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","03-Dom","T3",3],["GRUPO 3","XXX4","Tecnico B","03-Dom","T3",3],["GRUPO 3","XXX5","Tecnico B","03-Dom","T3",3],["GRUPO 3","XXX6","Tecnico B","03-Dom","T3",3],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","03-Dom","DESC. LEY",3],["GRUPO 4","PEPITO PEREZ","Master","03-Dom","DESC. LEY",3],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","03-Dom","DESC. LEY",3],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","03-Dom","DESC. LEY",3],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","03-Dom","DESC. LEY",3],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","03-Dom","DESC. LEY",3],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","03-Dom","DESC. LEY",3],["GRUPO 4","JHONY CASTRO","Tecnico A","03-Dom","DESC. LEY",3],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","03-Dom","DESC. LEY",3],["GRUPO 4","XXX7","Tecnico B","03-Dom","DESC. LEY",3],["GRUPO 4","XXX8","Tecnico B","03-Dom","DESC. LEY",3],["GRUPO 4","XXX9","Tecnico B","03-Dom","DESC. LEY",3],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","04-Lun","T1",4],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","04-Lun","T1",4],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","04-Lun","T1",4],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","04-Lun","T1",4],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","04-Lun","T1",4],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","04-Lun","T1",4],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","04-Lun","T1",4],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","04-Lun","T1",4],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","04-Lun","T1",4],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","04-Lun","T1",4],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","04-Lun","T1",4],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","04-Lun","T1",4],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","04-Lun","T2",4],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","04-Lun","T2",4],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","04-Lun","T2",4],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","04-Lun","T2",4],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","04-Lun","T2",4],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","04-Lun","T2",4],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","04-Lun","T2",4],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","04-Lun","T2",4],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","04-Lun","T2",4],["GRUPO 2","XXX1","Tecnico B","04-Lun","T2",4],["GRUPO 2","XXX2","Tecnico B","04-Lun","T2",4],["GRUPO 2","XXX3","Tecnico B","04-Lun","T2",4],["GRUPO 3","FONSECA RAY RICARDO","Master","04-Lun","T3",4],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","04-Lun","T3",4],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","04-Lun","T3",4],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","04-Lun","T3",4],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","04-Lun","T3",4],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","04-Lun","T3",4],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","04-Lun","T3",4],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","04-Lun","T3",4],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","04-Lun","T3",4],["GRUPO 3","XXX4","Tecnico B","04-Lun","T3",4],["GRUPO 3","XXX5","Tecnico B","04-Lun","T3",4],["GRUPO 3","XXX6","Tecnico B","04-Lun","T3",4],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","04-Lun","T1",4],["GRUPO 4","PEPITO PEREZ","Master","04-Lun","T1",4],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","04-Lun","T1",4],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","04-Lun","T1",4],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","04-Lun","T1",4],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","04-Lun","T1",4],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","04-Lun","T1",4],["GRUPO 4","JHONY CASTRO","Tecnico A","04-Lun","T1",4],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","04-Lun","T1",4],["GRUPO 4","XXX7","Tecnico B","04-Lun","T1",4],["GRUPO 4","XXX8","Tecnico B","04-Lun","T1",4],["GRUPO 4","XXX9","Tecnico B","04-Lun","T1",4],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","05-Mar","T1",5],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","05-Mar","T1",5],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","05-Mar","T1",5],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","05-Mar","T1",5],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","05-Mar","T1",5],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","05-Mar","T1",5],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","05-Mar","T1",5],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","05-Mar","T1",5],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","05-Mar","T1",5],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","05-Mar","T1",5],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","05-Mar","T1",5],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","05-Mar","T1",5],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","05-Mar","T2",5],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","05-Mar","T2",5],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","05-Mar","T2",5],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","05-Mar","T2",5],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","05-Mar","T2",5],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","05-Mar","T2",5],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","05-Mar","T2",5],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","05-Mar","T2",5],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","05-Mar","T2",5],["GRUPO 2","XXX1","Tecnico B","05-Mar","T2",5],["GRUPO 2","XXX2","Tecnico B","05-Mar","T2",5],["GRUPO 2","XXX3","Tecnico B","05-Mar","T2",5],["GRUPO 3","FONSECA RAY RICARDO","Master","05-Mar","T3",5],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","05-Mar","T3",5],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","05-Mar","T3",5],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","05-Mar","T3",5],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","05-Mar","T3",5],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","05-Mar","T3",5],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","05-Mar","T3",5],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","05-Mar","T3",5],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","05-Mar","T3",5],["GRUPO 3","XXX4","Tecnico B","05-Mar","T3",5],["GRUPO 3","XXX5","Tecnico B","05-Mar","T3",5],["GRUPO 3","XXX6","Tecnico B","05-Mar","T3",5],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","05-Mar","T1",5],["GRUPO 4","PEPITO PEREZ","Master","05-Mar","T1",5],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","05-Mar","T1",5],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","05-Mar","T1",5],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","05-Mar","T1",5],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","05-Mar","T1",5],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","05-Mar","T1",5],["GRUPO 4","JHONY CASTRO","Tecnico A","05-Mar","T1",5],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","05-Mar","T1",5],["GRUPO 4","XXX7","Tecnico B","05-Mar","T1",5],["GRUPO 4","XXX8","Tecnico B","05-Mar","T1",5],["GRUPO 4","XXX9","Tecnico B","05-Mar","T1",5],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","06-Mie","T1",6],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","06-Mie","T1",6],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","06-Mie","T1",6],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","06-Mie","T1",6],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","06-Mie","T1",6],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","06-Mie","T1",6],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","06-Mie","T1",6],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","06-Mie","T1",6],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","06-Mie","T1",6],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","06-Mie","T1",6],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","06-Mie","T1",6],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","06-Mie","T1",6],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","06-Mie","T2",6],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","06-Mie","T2",6],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","06-Mie","T2",6],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","06-Mie","T2",6],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","06-Mie","T2",6],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","06-Mie","T2",6],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","06-Mie","T2",6],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","06-Mie","T2",6],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","06-Mie","T2",6],["GRUPO 2","XXX1","Tecnico B","06-Mie","T2",6],["GRUPO 2","XXX2","Tecnico B","06-Mie","T2",6],["GRUPO 2","XXX3","Tecnico B","06-Mie","T2",6],["GRUPO 3","FONSECA RAY RICARDO","Master","06-Mie","T3",6],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","06-Mie","T3",6],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","06-Mie","T3",6],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","06-Mie","T3",6],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","06-Mie","T3",6],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","06-Mie","T3",6],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","06-Mie","T3",6],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","06-Mie","T3",6],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","06-Mie","T3",6],["GRUPO 3","XXX4","Tecnico B","06-Mie","T3",6],["GRUPO 3","XXX5","Tecnico B","06-Mie","T3",6],["GRUPO 3","XXX6","Tecnico B","06-Mie","T3",6],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","06-Mie","T1",6],["GRUPO 4","PEPITO PEREZ","Master","06-Mie","T1",6],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","06-Mie","T1",6],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","06-Mie","T1",6],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","06-Mie","T1",6],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","06-Mie","T1",6],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","06-Mie","T1",6],["GRUPO 4","JHONY CASTRO","Tecnico A","06-Mie","T1",6],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","06-Mie","T1",6],["GRUPO 4","XXX7","Tecnico B","06-Mie","T1",6],["GRUPO 4","XXX8","Tecnico B","06-Mie","T1",6],["GRUPO 4","XXX9","Tecnico B","06-Mie","T1",6],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","07-Jue","DESC. LEY",7],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","07-Jue","DESC. LEY",7],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","07-Jue","DESC. LEY",7],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","07-Jue","DESC. LEY",7],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","07-Jue","DESC. LEY",7],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","07-Jue","DESC. LEY",7],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","07-Jue","DESC. LEY",7],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","07-Jue","DESC. LEY",7],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","07-Jue","DESC. LEY",7],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","07-Jue","DESC. LEY",7],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","07-Jue","DESC. LEY",7],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","07-Jue","DESC. LEY",7],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","07-Jue","T2",7],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","07-Jue","T2",7],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","07-Jue","T2",7],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","07-Jue","T2",7],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","07-Jue","T2",7],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","07-Jue","T2",7],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","07-Jue","T2",7],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","07-Jue","T2",7],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","07-Jue","T2",7],["GRUPO 2","XXX1","Tecnico B","07-Jue","T2",7],["GRUPO 2","XXX2","Tecnico B","07-Jue","T2",7],["GRUPO 2","XXX3","Tecnico B","07-Jue","T2",7],["GRUPO 3","FONSECA RAY RICARDO","Master","07-Jue","T3",7],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","07-Jue","T3",7],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","07-Jue","T3",7],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","07-Jue","T3",7],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","07-Jue","T3",7],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","07-Jue","T3",7],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","07-Jue","T3",7],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","07-Jue","T3",7],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","07-Jue","T3",7],["GRUPO 3","XXX4","Tecnico B","07-Jue","T3",7],["GRUPO 3","XXX5","Tecnico B","07-Jue","T3",7],["GRUPO 3","XXX6","Tecnico B","07-Jue","T3",7],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","07-Jue","T2",7],["GRUPO 4","PEPITO PEREZ","Master","07-Jue","T2",7],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","07-Jue","T2",7],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","07-Jue","T2",7],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","07-Jue","T2",7],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","07-Jue","T2",7],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","07-Jue","T2",7],["GRUPO 4","JHONY CASTRO","Tecnico A","07-Jue","T2",7],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","07-Jue","T2",7],["GRUPO 4","XXX7","Tecnico B","07-Jue","T2",7],["GRUPO 4","XXX8","Tecnico B","07-Jue","T2",7],["GRUPO 4","XXX9","Tecnico B","07-Jue","T2",7],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","08-Vie","T2",8],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","08-Vie","T2",8],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","08-Vie","T2",8],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","08-Vie","T2",8],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","08-Vie","T2",8],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","08-Vie","T2",8],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","08-Vie","T2",8],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","08-Vie","T2",8],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","08-Vie","T2",8],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","08-Vie","T2",8],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","08-Vie","T2",8],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","08-Vie","T2",8],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","08-Vie","DESC. LEY",8],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","08-Vie","DESC. LEY",8],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","08-Vie","DESC. LEY",8],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","08-Vie","DESC. LEY",8],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","08-Vie","DESC. LEY",8],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","08-Vie","DESC. LEY",8],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","08-Vie","DESC. LEY",8],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","08-Vie","DESC. LEY",8],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","08-Vie","DESC. LEY",8],["GRUPO 2","XXX1","Tecnico B","08-Vie","DESC. LEY",8],["GRUPO 2","XXX2","Tecnico B","08-Vie","DESC. LEY",8],["GRUPO 2","XXX3","Tecnico B","08-Vie","DESC. LEY",8],["GRUPO 3","FONSECA RAY RICARDO","Master","08-Vie","T3",8],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","08-Vie","T3",8],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","08-Vie","T3",8],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","08-Vie","T3",8],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","08-Vie","T3",8],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","08-Vie","T3",8],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","08-Vie","T3",8],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","08-Vie","T3",8],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","08-Vie","T3",8],["GRUPO 3","XXX4","Tecnico B","08-Vie","T3",8],["GRUPO 3","XXX5","Tecnico B","08-Vie","T3",8],["GRUPO 3","XXX6","Tecnico B","08-Vie","T3",8],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","08-Vie","T3",8],["GRUPO 4","PEPITO PEREZ","Master","08-Vie","T3",8],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","08-Vie","T3",8],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","08-Vie","T3",8],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","08-Vie","T3",8],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","08-Vie","T3",8],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","08-Vie","T3",8],["GRUPO 4","JHONY CASTRO","Tecnico A","08-Vie","T3",8],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","08-Vie","T3",8],["GRUPO 4","XXX7","Tecnico B","08-Vie","T3",8],["GRUPO 4","XXX8","Tecnico B","08-Vie","T3",8],["GRUPO 4","XXX9","Tecnico B","08-Vie","T3",8],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","09-Sab","T2",9],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","09-Sab","T2",9],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","09-Sab","T2",9],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","09-Sab","T2",9],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","09-Sab","T2",9],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","09-Sab","T2",9],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","09-Sab","T2",9],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","09-Sab","T2",9],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","09-Sab","T2",9],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","09-Sab","T2",9],["GRU</t>
+  </si>
+  <si>
+    <t>{"columns":["Grupo","Empleado","Cargo","Label","Final","n_dia"],"index":[0,1,2,3,4,5,6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23,24,25,26,27,28,29,30,31,32,33,34,35,36,37,38,39,40,41,42,43,44,45,46,47,48,49,50,51,52,53,54,55,56,57,58,59,60,61,62,63,64,65,66,67,68,69,70,71,72,73,74,75,76,77,78,79,80,81,82,83,84,85,86,87,88,89,90,91,92,93,94,95,96,97,98,99,100,101,102,103,104,105,106,107,108,109,110,111,112,113,114,115,116,117,118,119,120,121,122,123,124,125,126,127,128,129,130,131,132,133,134,135,136,137,138,139,140,141,142,143,144,145,146,147,148,149,150,151,152,153,154,155,156,157,158,159,160,161,162,163,164,165,166,167,168,169,170,171,172,173,174,175,176,177,178,179,180,181,182,183,184,185,186,187,188,189,190,191,192,193,194,195,196,197,198,199,200,201,202,203,204,205,206,207,208,209,210,211,212,213,214,215,216,217,218,219,220,221,222,223,224,225,226,227,228,229,230,231,232,233,234,235,236,237,238,239,240,241,242,243,244,245,246,247,248,249,250,251,252,253,254,255,256,257,258,259,260,261,262,263,264,265,266,267,268,269,270,271,272,273,274,275,276,277,278,279,280,281,282,283,284,285,286,287,288,289,290,291,292,293,294,295,296,297,298,299,300,301,302,303,304,305,306,307,308,309,310,311,312,313,314,315,316,317,318,319,320,321,322,323,324,325,326,327,328,329,330,331,332,333,334,335,336,337,338,339,340,341,342,343,344,345,346,347,348,349,350,351,352,353,354,355,356,357,358,359,360,361,362,363,364,365,366,367,368,369,370,371,372,373,374,375,376,377,378,379,380,381,382,383,384,385,386,387,388,389,390,391,392,393,394,395,396,397,398,399,400,401,402,403,404,405,406,407,408,409,410,411,412,413,414,415,416,417,418,419,420,421,422,423,424,425,426,427,428,429,430,431,432,433,434,435,436,437,438,439,440,441,442,443,444,445,446,447,448,449,450,451,452,453,454,455,456,457,458,459,460,461,462,463,464,465,466,467,468,469,470,471,472,473,474,475,476,477,478,479,480,481,482,483,484,485,486,487,488,489,490,491,492,493,494,495,496,497,498,499,500,501,502,503,504,505,506,507,508,509,510,511,512,513,514,515,516,517,518,519,520,521,522,523,524,525,526,527,528,529,530,531,532,533,534,535,536,537,538,539,540,541,542,543,544,545,546,547,548,549,550,551,552,553,554,555,556,557,558,559,560,561,562,563,564,565,566,567,568,569,570,571,572,573,574,575,576,577,578,579,580,581,582,583,584,585,586,587,588,589,590,591,592,593,594,595,596,597,598,599,600,601,602,603,604,605,606,607,608,609,610,611,612,613,614,615,616,617,618,619,620,621,622,623,624,625,626,627,628,629,630,631,632,633,634,635,636,637,638,639,640,641,642,643,644,645,646,647,648,649,650,651,652,653,654,655,656,657,658,659,660,661,662,663,664,665,666,667,668,669,670,671,672,673,674,675,676,677,678,679,680,681,682,683,684,685,686,687,688,689,690,691,692,693,694,695,696,697,698,699,700,701,702,703,704,705,706,707,708,709,710,711,712,713,714,715,716,717,718,719,720,721,722,723,724,725,726,727,728,729,730,731,732,733,734,735,736,737,738,739,740,741,742,743,744,745,746,747,748,749,750,751,752,753,754,755,756,757,758,759,760,761,762,763,764,765,766,767,768,769,770,771,772,773,774,775,776,777,778,779,780,781,782,783,784,785,786,787,788,789,790,791,792,793,794,795,796,797,798,799,800,801,802,803,804,805,806,807,808,809,810,811,812,813,814,815,816,817,818,819,820,821,822,823,824,825,826,827,828,829,830,831,832,833,834,835,836,837,838,839,840,841,842,843,844,845,846,847,848,849,850,851,852,853,854,855,856,857,858,859,860,861,862,863,864,865,866,867,868,869,870,871,872,873,874,875,876,877,878,879,880,881,882,883,884,885,886,887,888,889,890,891,892,893,894,895,896,897,898,899,900,901,902,903,904,905,906,907,908,909,910,911,912,913,914,915,916,917,918,919,920,921,922,923,924,925,926,927,928,929,930,931,932,933,934,935,936,937,938,939,940,941,942,943,944,945,946,947,948,949,950,951,952,953,954,955,956,957,958,959,960,961,962,963,964,965,966,967,968,969,970,971,972,973,974,975,976,977,978,979,980,981,982,983,984,985,986,987,988,989,990,991,992,993,994,995,996,997,998,999,1000,1001,1002,1003,1004,1005,1006,1007,1008,1009,1010,1011,1012,1013,1014,1015,1016,1017,1018,1019,1020,1021,1022,1023,1024,1025,1026,1027,1028,1029,1030,1031,1032,1033,1034,1035,1036,1037,1038,1039,1040,1041,1042,1043,1044,1045,1046,1047,1048,1049,1050,1051,1052,1053,1054,1055,1056,1057,1058,1059,1060,1061,1062,1063,1064,1065,1066,1067,1068,1069,1070,1071,1072,1073,1074,1075,1076,1077,1078,1079,1080,1081,1082,1083,1084,1085,1086,1087,1088,1089,1090,1091,1092,1093,1094,1095,1096,1097,1098,1099,1100,1101,1102,1103,1104,1105,1106,1107,1108,1109,1110,1111,1112,1113,1114,1115,1116,1117,1118,1119,1120,1121,1122,1123,1124,1125,1126,1127,1128,1129,1130,1131,1132,1133,1134,1135,1136,1137,1138,1139,1140,1141,1142,1143,1144,1145,1146,1147,1148,1149,1150,1151,1152,1153,1154,1155,1156,1157,1158,1159,1160,1161,1162,1163,1164,1165,1166,1167,1168,1169,1170,1171,1172,1173,1174,1175,1176,1177,1178,1179,1180,1181,1182,1183,1184,1185,1186,1187,1188,1189,1190,1191,1192,1193,1194,1195,1196,1197,1198,1199,1200,1201,1202,1203,1204,1205,1206,1207,1208,1209,1210,1211,1212,1213,1214,1215,1216,1217,1218,1219,1220,1221,1222,1223,1224,1225,1226,1227,1228,1229,1230,1231,1232,1233,1234,1235,1236,1237,1238,1239,1240,1241,1242,1243,1244,1245,1246,1247,1248,1249,1250,1251,1252,1253,1254,1255,1256,1257,1258,1259,1260,1261,1262,1263,1264,1265,1266,1267,1268,1269,1270,1271,1272,1273,1274,1275,1276,1277,1278,1279,1280,1281,1282,1283,1284,1285,1286,1287,1288,1289,1290,1291,1292,1293,1294,1295,1296,1297,1298,1299,1300,1301,1302,1303,1304,1305,1306,1307,1308,1309,1310,1311,1312,1313,1314,1315,1316,1317,1318,1319,1320,1321,1322,1323,1324,1325,1326,1327,1328,1329,1330,1331,1332,1333,1334,1335,1336,1337,1338,1339,1340,1341,1342,1343,1344,1345,1346,1347,1348,1349,1350,1351,1352,1353,1354,1355,1356,1357,1358,1359,1360,1361,1362,1363,1364,1365,1366,1367,1368,1369,1370,1371,1372,1373,1374,1375,1376,1377,1378,1379,1380,1381,1382,1383,1384,1385,1386,1387,1388,1389,1390,1391,1392,1393,1394,1395,1396,1397,1398,1399,1400,1401,1402,1403,1404,1405,1406,1407,1408,1409,1410,1411,1412,1413,1414,1415,1416,1417,1418,1419,1420,1421,1422,1423,1424,1425,1426,1427,1428,1429,1430,1431,1432,1433,1434,1435,1436,1437,1438,1439],"data":[["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","01-Lun","T1",1],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","01-Lun","T1",1],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","01-Lun","T1",1],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","01-Lun","T1",1],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","01-Lun","T1",1],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","01-Lun","T1",1],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","01-Lun","T1",1],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","01-Lun","T1",1],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","01-Lun","T1",1],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","01-Lun","T1",1],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","01-Lun","T1",1],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","01-Lun","T1",1],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","01-Lun","T2",1],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","01-Lun","T2",1],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","01-Lun","T2",1],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","01-Lun","T2",1],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","01-Lun","T2",1],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","01-Lun","T2",1],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","01-Lun","T2",1],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","01-Lun","T2",1],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","01-Lun","T2",1],["GRUPO 2","XXX1","Tecnico B","01-Lun","T2",1],["GRUPO 2","XXX2","Tecnico B","01-Lun","T2",1],["GRUPO 2","XXX3","Tecnico B","01-Lun","T2",1],["GRUPO 3","FONSECA RAY RICARDO","Master","01-Lun","T3",1],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","01-Lun","T3",1],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","01-Lun","T3",1],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","01-Lun","T3",1],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","01-Lun","T3",1],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","01-Lun","T3",1],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","01-Lun","T3",1],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","01-Lun","T3",1],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","01-Lun","T3",1],["GRUPO 3","XXX4","Tecnico B","01-Lun","T3",1],["GRUPO 3","XXX5","Tecnico B","01-Lun","T3",1],["GRUPO 3","XXX6","Tecnico B","01-Lun","T3",1],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","01-Lun","T1",1],["GRUPO 4","PEPITO PEREZ","Master","01-Lun","T1",1],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","01-Lun","T1",1],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","01-Lun","T1",1],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","01-Lun","T1",1],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","01-Lun","T1",1],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","01-Lun","T1",1],["GRUPO 4","JHONY CASTRO","Tecnico A","01-Lun","T1",1],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","01-Lun","T1",1],["GRUPO 4","XXX7","Tecnico B","01-Lun","T1",1],["GRUPO 4","XXX8","Tecnico B","01-Lun","T1",1],["GRUPO 4","XXX9","Tecnico B","01-Lun","T1",1],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","02-Mar","T1",2],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","02-Mar","T1",2],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","02-Mar","T1",2],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","02-Mar","T1",2],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","02-Mar","T1",2],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","02-Mar","T1",2],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","02-Mar","T1",2],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","02-Mar","T1",2],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","02-Mar","T1",2],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","02-Mar","T1",2],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","02-Mar","T1",2],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","02-Mar","T1",2],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","02-Mar","T2",2],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","02-Mar","T2",2],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","02-Mar","T2",2],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","02-Mar","T2",2],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","02-Mar","T2",2],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","02-Mar","T2",2],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","02-Mar","T2",2],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","02-Mar","T2",2],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","02-Mar","T2",2],["GRUPO 2","XXX1","Tecnico B","02-Mar","T2",2],["GRUPO 2","XXX2","Tecnico B","02-Mar","T2",2],["GRUPO 2","XXX3","Tecnico B","02-Mar","T2",2],["GRUPO 3","FONSECA RAY RICARDO","Master","02-Mar","T3",2],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","02-Mar","T3",2],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","02-Mar","T3",2],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","02-Mar","T3",2],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","02-Mar","T3",2],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","02-Mar","T3",2],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","02-Mar","T3",2],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","02-Mar","T3",2],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","02-Mar","T3",2],["GRUPO 3","XXX4","Tecnico B","02-Mar","T3",2],["GRUPO 3","XXX5","Tecnico B","02-Mar","T3",2],["GRUPO 3","XXX6","Tecnico B","02-Mar","T3",2],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","02-Mar","T1",2],["GRUPO 4","PEPITO PEREZ","Master","02-Mar","T1",2],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","02-Mar","T1",2],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","02-Mar","T1",2],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","02-Mar","T1",2],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","02-Mar","T1",2],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","02-Mar","T1",2],["GRUPO 4","JHONY CASTRO","Tecnico A","02-Mar","T1",2],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","02-Mar","T1",2],["GRUPO 4","XXX7","Tecnico B","02-Mar","T1",2],["GRUPO 4","XXX8","Tecnico B","02-Mar","T1",2],["GRUPO 4","XXX9","Tecnico B","02-Mar","T1",2],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","03-Mie","T1",3],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","03-Mie","T1",3],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","03-Mie","T1",3],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","03-Mie","T1",3],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","03-Mie","T1",3],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","03-Mie","T1",3],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","03-Mie","T1",3],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","03-Mie","T1",3],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","03-Mie","T1",3],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","03-Mie","T1",3],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","03-Mie","T1",3],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","03-Mie","T1",3],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","03-Mie","T2",3],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","03-Mie","T2",3],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","03-Mie","T2",3],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","03-Mie","T2",3],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","03-Mie","T2",3],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","03-Mie","T2",3],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","03-Mie","T2",3],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","03-Mie","T2",3],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","03-Mie","T2",3],["GRUPO 2","XXX1","Tecnico B","03-Mie","T2",3],["GRUPO 2","XXX2","Tecnico B","03-Mie","T2",3],["GRUPO 2","XXX3","Tecnico B","03-Mie","T2",3],["GRUPO 3","FONSECA RAY RICARDO","Master","03-Mie","T3",3],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","03-Mie","T3",3],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","03-Mie","T3",3],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","03-Mie","T3",3],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","03-Mie","T3",3],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","03-Mie","T3",3],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","03-Mie","T3",3],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","03-Mie","T3",3],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","03-Mie","T3",3],["GRUPO 3","XXX4","Tecnico B","03-Mie","T3",3],["GRUPO 3","XXX5","Tecnico B","03-Mie","T3",3],["GRUPO 3","XXX6","Tecnico B","03-Mie","T3",3],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","03-Mie","T1",3],["GRUPO 4","PEPITO PEREZ","Master","03-Mie","T1",3],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","03-Mie","T1",3],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","03-Mie","T1",3],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","03-Mie","T1",3],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","03-Mie","T1",3],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","03-Mie","T1",3],["GRUPO 4","JHONY CASTRO","Tecnico A","03-Mie","T1",3],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","03-Mie","T1",3],["GRUPO 4","XXX7","Tecnico B","03-Mie","T1",3],["GRUPO 4","XXX8","Tecnico B","03-Mie","T1",3],["GRUPO 4","XXX9","Tecnico B","03-Mie","T1",3],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","04-Jue","DESC. LEY",4],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","04-Jue","DESC. LEY",4],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","04-Jue","DESC. LEY",4],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","04-Jue","DESC. LEY",4],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","04-Jue","DESC. LEY",4],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","04-Jue","DESC. LEY",4],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","04-Jue","DESC. LEY",4],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","04-Jue","DESC. LEY",4],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","04-Jue","DESC. LEY",4],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","04-Jue","DESC. LEY",4],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","04-Jue","DESC. LEY",4],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","04-Jue","DESC. LEY",4],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","04-Jue","T2",4],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","04-Jue","T2",4],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","04-Jue","T2",4],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","04-Jue","T2",4],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","04-Jue","T2",4],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","04-Jue","T2",4],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","04-Jue","T2",4],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","04-Jue","T2",4],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","04-Jue","T2",4],["GRUPO 2","XXX1","Tecnico B","04-Jue","T2",4],["GRUPO 2","XXX2","Tecnico B","04-Jue","T2",4],["GRUPO 2","XXX3","Tecnico B","04-Jue","T2",4],["GRUPO 3","FONSECA RAY RICARDO","Master","04-Jue","T3",4],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","04-Jue","T3",4],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","04-Jue","T3",4],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","04-Jue","T3",4],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","04-Jue","T3",4],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","04-Jue","T3",4],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","04-Jue","T3",4],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","04-Jue","T3",4],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","04-Jue","T3",4],["GRUPO 3","XXX4","Tecnico B","04-Jue","T3",4],["GRUPO 3","XXX5","Tecnico B","04-Jue","T3",4],["GRUPO 3","XXX6","Tecnico B","04-Jue","T3",4],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","04-Jue","T1",4],["GRUPO 4","PEPITO PEREZ","Master","04-Jue","T1",4],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","04-Jue","T1",4],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","04-Jue","T1",4],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","04-Jue","T1",4],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","04-Jue","T1",4],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","04-Jue","T1",4],["GRUPO 4","JHONY CASTRO","Tecnico A","04-Jue","T1",4],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","04-Jue","T1",4],["GRUPO 4","XXX7","Tecnico B","04-Jue","T1",4],["GRUPO 4","XXX8","Tecnico B","04-Jue","T1",4],["GRUPO 4","XXX9","Tecnico B","04-Jue","T1",4],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","05-Vie","T1",5],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","05-Vie","T1",5],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","05-Vie","T1",5],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","05-Vie","T1",5],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","05-Vie","T1",5],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","05-Vie","T1",5],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","05-Vie","T1",5],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","05-Vie","T1",5],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","05-Vie","T1",5],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","05-Vie","T1",5],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","05-Vie","T1",5],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","05-Vie","T1",5],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","05-Vie","DESC. LEY",5],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","05-Vie","DESC. LEY",5],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","05-Vie","DESC. LEY",5],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","05-Vie","DESC. LEY",5],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","05-Vie","DESC. LEY",5],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","05-Vie","DESC. LEY",5],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","05-Vie","DESC. LEY",5],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","05-Vie","DESC. LEY",5],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","05-Vie","DESC. LEY",5],["GRUPO 2","XXX1","Tecnico B","05-Vie","DESC. LEY",5],["GRUPO 2","XXX2","Tecnico B","05-Vie","DESC. LEY",5],["GRUPO 2","XXX3","Tecnico B","05-Vie","DESC. LEY",5],["GRUPO 3","FONSECA RAY RICARDO","Master","05-Vie","T3",5],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","05-Vie","T3",5],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","05-Vie","T3",5],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","05-Vie","T3",5],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","05-Vie","T3",5],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","05-Vie","T3",5],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","05-Vie","T3",5],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","05-Vie","T3",5],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","05-Vie","T3",5],["GRUPO 3","XXX4","Tecnico B","05-Vie","T3",5],["GRUPO 3","XXX5","Tecnico B","05-Vie","T3",5],["GRUPO 3","XXX6","Tecnico B","05-Vie","T3",5],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","05-Vie","T2",5],["GRUPO 4","PEPITO PEREZ","Master","05-Vie","T2",5],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","05-Vie","T2",5],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","05-Vie","T2",5],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","05-Vie","T2",5],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","05-Vie","T2",5],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","05-Vie","T2",5],["GRUPO 4","JHONY CASTRO","Tecnico A","05-Vie","T2",5],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","05-Vie","T2",5],["GRUPO 4","XXX7","Tecnico B","05-Vie","T2",5],["GRUPO 4","XXX8","Tecnico B","05-Vie","T2",5],["GRUPO 4","XXX9","Tecnico B","05-Vie","T2",5],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","06-Sab","T1",6],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","06-Sab","T1",6],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","06-Sab","T1",6],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","06-Sab","T1",6],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","06-Sab","T1",6],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","06-Sab","T1",6],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","06-Sab","T1",6],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","06-Sab","T1",6],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","06-Sab","T1",6],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","06-Sab","T1",6],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","06-Sab","T1",6],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","06-Sab","T1",6],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","06-Sab","T2",6],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","06-Sab","T2",6],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","06-Sab","T2",6],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","06-Sab","T2",6],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","06-Sab","T2",6],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","06-Sab","T2",6],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","06-Sab","T2",6],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","06-Sab","T2",6],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","06-Sab","T2",6],["GRUPO 2","XXX1","Tecnico B","06-Sab","T2",6],["GRUPO 2","XXX2","Tecnico B","06-Sab","T2",6],["GRUPO 2","XXX3","Tecnico B","06-Sab","T2",6],["GRUPO 3","FONSECA RAY RICARDO","Master","06-Sab","DESC. LEY",6],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","06-Sab","DESC. LEY",6],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","06-Sab","DESC. LEY",6],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","06-Sab","DESC. LEY",6],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","06-Sab","DESC. LEY",6],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","06-Sab","DESC. LEY",6],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","06-Sab","DESC. LEY",6],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","06-Sab","DESC. LEY",6],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","06-Sab","DESC. LEY",6],["GRUPO 3","XXX4","Tecnico B","06-Sab","DESC. LEY",6],["GRUPO 3","XXX5","Tecnico B","06-Sab","DESC. LEY",6],["GRUPO 3","XXX6","Tecnico B","06-Sab","DESC. LEY",6],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","06-Sab","T3",6],["GRUPO 4","PEPITO PEREZ","Master","06-Sab","T3",6],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","06-Sab","T3",6],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","06-Sab","T3",6],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","06-Sab","T3",6],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","06-Sab","T3",6],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","06-Sab","T3",6],["GRUPO 4","JHONY CASTRO","Tecnico A","06-Sab","T3",6],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","06-Sab","T3",6],["GRUPO 4","XXX7","Tecnico B","06-Sab","T3",6],["GRUPO 4","XXX8","Tecnico B","06-Sab","T3",6],["GRUPO 4","XXX9","Tecnico B","06-Sab","T3",6],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","07-Dom","T1",7],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","07-Dom","T1",7],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","07-Dom","T1",7],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","07-Dom","T1",7],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","07-Dom","T1",7],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","07-Dom","T1",7],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","07-Dom","T1",7],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","07-Dom","T1",7],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","07-Dom","T1",7],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","07-Dom","T1",7],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","07-Dom","T1",7],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","07-Dom","T1",7],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","07-Dom","T2",7],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","07-Dom","T2",7],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","07-Dom","T2",7],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","07-Dom","T2",7],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","07-Dom","T2",7],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","07-Dom","T2",7],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","07-Dom","T2",7],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","07-Dom","T2",7],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","07-Dom","T2",7],["GRUPO 2","XXX1","Tecnico B","07-Dom","T2",7],["GRUPO 2","XXX2","Tecnico B","07-Dom","T2",7],["GRUPO 2","XXX3","Tecnico B","07-Dom","T2",7],["GRUPO 3","FONSECA RAY RICARDO","Master","07-Dom","T3",7],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","07-Dom","T3",7],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","07-Dom","T3",7],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","07-Dom","T3",7],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","07-Dom","T3",7],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","07-Dom","T3",7],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","07-Dom","T3",7],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","07-Dom","T3",7],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","07-Dom","T3",7],["GRUPO 3","XXX4","Tecnico B","07-Dom","T3",7],["GRUPO 3","XXX5","Tecnico B","07-Dom","T3",7],["GRUPO 3","XXX6","Tecnico B","07-Dom","T3",7],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","07-Dom","DESC. LEY",7],["GRUPO 4","PEPITO PEREZ","Master","07-Dom","DESC. LEY",7],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","07-Dom","DESC. LEY",7],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","07-Dom","DESC. LEY",7],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","07-Dom","DESC. LEY",7],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","07-Dom","DESC. LEY",7],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","07-Dom","DESC. LEY",7],["GRUPO 4","JHONY CASTRO","Tecnico A","07-Dom","DESC. LEY",7],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","07-Dom","DESC. LEY",7],["GRUPO 4","XXX7","Tecnico B","07-Dom","DESC. LEY",7],["GRUPO 4","XXX8","Tecnico B","07-Dom","DESC. LEY",7],["GRUPO 4","XXX9","Tecnico B","07-Dom","DESC. LEY",7],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","08-Lun","T1",8],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","08-Lun","T1",8],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","08-Lun","T1",8],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","08-Lun","T1",8],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","08-Lun","T1",8],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","08-Lun","T1",8],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","08-Lun","T1",8],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","08-Lun","T1",8],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","08-Lun","T1",8],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","08-Lun","T1",8],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","08-Lun","T1",8],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","08-Lun","T1",8],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","08-Lun","T2",8],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","08-Lun","T2",8],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","08-Lun","T2",8],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","08-Lun","T2",8],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","08-Lun","T2",8],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","08-Lun","T2",8],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","08-Lun","T2",8],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","08-Lun","T2",8],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","08-Lun","T2",8],["GRUPO 2","XXX1","Tecnico B","08-Lun","T2",8],["GRUPO 2","XXX2","Tecnico B","08-Lun","T2",8],["GRUPO 2","XXX3","Tecnico B","08-Lun","T2",8],["GRUPO 3","FONSECA RAY RICARDO","Master","08-Lun","T3",8],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","08-Lun","T3",8],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","08-Lun","T3",8],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","08-Lun","T3",8],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","08-Lun","T3",8],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","08-Lun","T3",8],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","08-Lun","T3",8],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","08-Lun","T3",8],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","08-Lun","T3",8],["GRUPO 3","XXX4","Tecnico B","08-Lun","T3",8],["GRUPO 3","XXX5","Tecnico B","08-Lun","T3",8],["GRUPO 3","XXX6","Tecnico B","08-Lun","T3",8],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","08-Lun","T1",8],["GRUPO 4","PEPITO PEREZ","Master","08-Lun","T1",8],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","08-Lun","T1",8],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","08-Lun","T1",8],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","08-Lun","T1",8],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","08-Lun","T1",8],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","08-Lun","T1",8],["GRUPO 4","JHONY CASTRO","Tecnico A","08-Lun","T1",8],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","08-Lun","T1",8],["GRUPO 4","XXX7","Tecnico B","08-Lun","T1",8],["GRUPO 4","XXX8","Tecnico B","08-Lun","T1",8],["GRUPO 4","XXX9","Tecnico B","08-Lun","T1",8],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","09-Mar","T1",9],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","09-Mar","T1",9],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","09-Mar","T1",9],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","09-Mar","T1",9],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","09-Mar","T1",9],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","09-Mar","T1",9],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","09-Mar","T1",9],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","09-Mar","T1",9],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","09-Mar","T1",9],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","09-Mar","T1",9],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","09-Mar","T1",9],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","09-Mar","T1",9],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","09-Mar","T2",9],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","09-Mar","T2",9],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","</t>
   </si>
   <si>
     <t>Mes Completo</t>

</xml_diff>

<commit_message>
Update historico_mallas.xlsx 2026-04-27 15:57:23.509280
</commit_message>
<xml_diff>
--- a/historico_mallas.xlsx
+++ b/historico_mallas.xlsx
@@ -34,27 +34,24 @@
     <t>Alcance</t>
   </si>
   <si>
+    <t>Julio</t>
+  </si>
+  <si>
+    <t>Agosto</t>
+  </si>
+  <si>
+    <t>Mayo</t>
+  </si>
+  <si>
+    <t>Junio</t>
+  </si>
+  <si>
     <t>Abril</t>
   </si>
   <si>
-    <t>Julio</t>
-  </si>
-  <si>
-    <t>Agosto</t>
-  </si>
-  <si>
-    <t>Mayo</t>
-  </si>
-  <si>
-    <t>Junio</t>
-  </si>
-  <si>
     <t>Técnica</t>
   </si>
   <si>
-    <t>2026-04-24 18:15</t>
-  </si>
-  <si>
     <t>2026-04-24 18:27</t>
   </si>
   <si>
@@ -67,7 +64,7 @@
     <t>24/04/2026 21:36</t>
   </si>
   <si>
-    <t>{"Grupo":{"0":"GRUPO 1","1":"GRUPO 1","2":"GRUPO 1","3":"GRUPO 1","4":"GRUPO 1","5":"GRUPO 1","6":"GRUPO 1","7":"GRUPO 1","8":"GRUPO 1","9":"GRUPO 1","10":"GRUPO 1","11":"GRUPO 1","12":"GRUPO 2","13":"GRUPO 2","14":"GRUPO 2","15":"GRUPO 2","16":"GRUPO 2","17":"GRUPO 2","18":"GRUPO 2","19":"GRUPO 2","20":"GRUPO 2","21":"GRUPO 2","22":"GRUPO 2","23":"GRUPO 2","24":"GRUPO 3","25":"GRUPO 3","26":"GRUPO 3","27":"GRUPO 3","28":"GRUPO 3","29":"GRUPO 3","30":"GRUPO 3","31":"GRUPO 3","32":"GRUPO 3","33":"GRUPO 3","34":"GRUPO 3","35":"GRUPO 3","36":"GRUPO 4","37":"GRUPO 4","38":"GRUPO 4","39":"GRUPO 4","40":"GRUPO 4","41":"GRUPO 4","42":"GRUPO 4","43":"GRUPO 4","44":"GRUPO 4","45":"GRUPO 4","46":"GRUPO 4","47":"GRUPO 4","48":"GRUPO 1","49":"GRUPO 1","50":"GRUPO 1","51":"GRUPO 1","52":"GRUPO 1","53":"GRUPO 1","54":"GRUPO 1","55":"GRUPO 1","56":"GRUPO 1","57":"GRUPO 1","58":"GRUPO 1","59":"GRUPO 1","60":"GRUPO 2","61":"GRUPO 2","62":"GRUPO 2","63":"GRUPO 2","64":"GRUPO 2","65":"GRUPO 2","66":"GRUPO 2","67":"GRUPO 2","68":"GRUPO 2","69":"GRUPO 2","70":"GRUPO 2","71":"GRUPO 2","72":"GRUPO 3","73":"GRUPO 3","74":"GRUPO 3","75":"GRUPO 3","76":"GRUPO 3","77":"GRUPO 3","78":"GRUPO 3","79":"GRUPO 3","80":"GRUPO 3","81":"GRUPO 3","82":"GRUPO 3","83":"GRUPO 3","84":"GRUPO 4","85":"GRUPO 4","86":"GRUPO 4","87":"GRUPO 4","88":"GRUPO 4","89":"GRUPO 4","90":"GRUPO 4","91":"GRUPO 4","92":"GRUPO 4","93":"GRUPO 4","94":"GRUPO 4","95":"GRUPO 4","96":"GRUPO 1","97":"GRUPO 1","98":"GRUPO 1","99":"GRUPO 1","100":"GRUPO 1","101":"GRUPO 1","102":"GRUPO 1","103":"GRUPO 1","104":"GRUPO 1","105":"GRUPO 1","106":"GRUPO 1","107":"GRUPO 1","108":"GRUPO 2","109":"GRUPO 2","110":"GRUPO 2","111":"GRUPO 2","112":"GRUPO 2","113":"GRUPO 2","114":"GRUPO 2","115":"GRUPO 2","116":"GRUPO 2","117":"GRUPO 2","118":"GRUPO 2","119":"GRUPO 2","120":"GRUPO 3","121":"GRUPO 3","122":"GRUPO 3","123":"GRUPO 3","124":"GRUPO 3","125":"GRUPO 3","126":"GRUPO 3","127":"GRUPO 3","128":"GRUPO 3","129":"GRUPO 3","130":"GRUPO 3","131":"GRUPO 3","132":"GRUPO 4","133":"GRUPO 4","134":"GRUPO 4","135":"GRUPO 4","136":"GRUPO 4","137":"GRUPO 4","138":"GRUPO 4","139":"GRUPO 4","140":"GRUPO 4","141":"GRUPO 4","142":"GRUPO 4","143":"GRUPO 4","144":"GRUPO 1","145":"GRUPO 1","146":"GRUPO 1","147":"GRUPO 1","148":"GRUPO 1","149":"GRUPO 1","150":"GRUPO 1","151":"GRUPO 1","152":"GRUPO 1","153":"GRUPO 1","154":"GRUPO 1","155":"GRUPO 1","156":"GRUPO 2","157":"GRUPO 2","158":"GRUPO 2","159":"GRUPO 2","160":"GRUPO 2","161":"GRUPO 2","162":"GRUPO 2","163":"GRUPO 2","164":"GRUPO 2","165":"GRUPO 2","166":"GRUPO 2","167":"GRUPO 2","168":"GRUPO 3","169":"GRUPO 3","170":"GRUPO 3","171":"GRUPO 3","172":"GRUPO 3","173":"GRUPO 3","174":"GRUPO 3","175":"GRUPO 3","176":"GRUPO 3","177":"GRUPO 3","178":"GRUPO 3","179":"GRUPO 3","180":"GRUPO 4","181":"GRUPO 4","182":"GRUPO 4","183":"GRUPO 4","184":"GRUPO 4","185":"GRUPO 4","186":"GRUPO 4","187":"GRUPO 4","188":"GRUPO 4","189":"GRUPO 4","190":"GRUPO 4","191":"GRUPO 4","192":"GRUPO 1","193":"GRUPO 1","194":"GRUPO 1","195":"GRUPO 1","196":"GRUPO 1","197":"GRUPO 1","198":"GRUPO 1","199":"GRUPO 1","200":"GRUPO 1","201":"GRUPO 1","202":"GRUPO 1","203":"GRUPO 1","204":"GRUPO 2","205":"GRUPO 2","206":"GRUPO 2","207":"GRUPO 2","208":"GRUPO 2","209":"GRUPO 2","210":"GRUPO 2","211":"GRUPO 2","212":"GRUPO 2","213":"GRUPO 2","214":"GRUPO 2","215":"GRUPO 2","216":"GRUPO 3","217":"GRUPO 3","218":"GRUPO 3","219":"GRUPO 3","220":"GRUPO 3","221":"GRUPO 3","222":"GRUPO 3","223":"GRUPO 3","224":"GRUPO 3","225":"GRUPO 3","226":"GRUPO 3","227":"GRUPO 3","228":"GRUPO 4","229":"GRUPO 4","230":"GRUPO 4","231":"GRUPO 4","232":"GRUPO 4","233":"GRUPO 4","234":"GRUPO 4","235":"GRUPO 4","236":"GRUPO 4","237":"GRUPO 4","238":"GRUPO 4","239":"GRUPO 4","240":"GRUPO 1","241":"GRUPO 1","242":"GRUPO 1","243":"GRUPO 1","244":"GRUPO 1","245":"GRUPO 1","246":"GRUPO 1","247":"GRUPO 1","248":"GRUPO 1","249":"GRUPO 1","250":"GRUPO 1","251":"GRUPO 1","252":"GRUPO 2","253":"GRUPO 2","254":"GRUPO 2","255":"GRUPO 2","256":"GRUPO 2","257":"GRUPO 2","258":"GRUPO 2","259":"GRUPO 2","260":"GRUPO 2","261":"GRUPO 2","262":"GRUPO 2","263":"GRUPO 2","264":"GRUPO 3","265":"GRUPO 3","266":"GRUPO 3","267":"GRUPO 3","268":"GRUPO 3","269":"GRUPO 3","270":"GRUPO 3","271":"GRUPO 3","272":"GRUPO 3","273":"GRUPO 3","274":"GRUPO 3","275":"GRUPO 3","276":"GRUPO 4","277":"GRUPO 4","278":"GRUPO 4","279":"GRUPO 4","280":"GRUPO 4","281":"GRUPO 4","282":"GRUPO 4","283":"GRUPO 4","284":"GRUPO 4","285":"GRUPO 4","286":"GRUPO 4","287":"GRUPO 4","288":"GRUPO 1","289":"GRUPO 1","290":"GRUPO 1","291":"GRUPO 1","292":"GRUPO 1","293":"GRUPO 1","294":"GRUPO 1","295":"GRUPO 1","296":"GRUPO 1","297":"GRUPO 1","298":"GRUPO 1","299":"GRUPO 1","300":"GRUPO 2","301":"GRUPO 2","302":"GRUPO 2","303":"GRUPO 2","304":"GRUPO 2","305":"GRUPO 2","306":"GRUPO 2","307":"GRUPO 2","308":"GRUPO 2","309":"GRUPO 2","310":"GRUPO 2","311":"GRUPO 2","312":"GRUPO 3","313":"GRUPO 3","314":"GRUPO 3","315":"GRUPO 3","316":"GRUPO 3","317":"GRUPO 3","318":"GRUPO 3","319":"GRUPO 3","320":"GRUPO 3","321":"GRUPO 3","322":"GRUPO 3","323":"GRUPO 3","324":"GRUPO 4","325":"GRUPO 4","326":"GRUPO 4","327":"GRUPO 4","328":"GRUPO 4","329":"GRUPO 4","330":"GRUPO 4","331":"GRUPO 4","332":"GRUPO 4","333":"GRUPO 4","334":"GRUPO 4","335":"GRUPO 4","336":"GRUPO 1","337":"GRUPO 1","338":"GRUPO 1","339":"GRUPO 1","340":"GRUPO 1","341":"GRUPO 1","342":"GRUPO 1","343":"GRUPO 1","344":"GRUPO 1","345":"GRUPO 1","346":"GRUPO 1","347":"GRUPO 1","348":"GRUPO 2","349":"GRUPO 2","350":"GRUPO 2","351":"GRUPO 2","352":"GRUPO 2","353":"GRUPO 2","354":"GRUPO 2","355":"GRUPO 2","356":"GRUPO 2","357":"GRUPO 2","358":"GRUPO 2","359":"GRUPO 2","360":"GRUPO 3","361":"GRUPO 3","362":"GRUPO 3","363":"GRUPO 3","364":"GRUPO 3","365":"GRUPO 3","366":"GRUPO 3","367":"GRUPO 3","368":"GRUPO 3","369":"GRUPO 3","370":"GRUPO 3","371":"GRUPO 3","372":"GRUPO 4","373":"GRUPO 4","374":"GRUPO 4","375":"GRUPO 4","376":"GRUPO 4","377":"GRUPO 4","378":"GRUPO 4","379":"GRUPO 4","380":"GRUPO 4","381":"GRUPO 4","382":"GRUPO 4","383":"GRUPO 4","384":"GRUPO 1","385":"GRUPO 1","386":"GRUPO 1","387":"GRUPO 1","388":"GRUPO 1","389":"GRUPO 1","390":"GRUPO 1","391":"GRUPO 1","392":"GRUPO 1","393":"GRUPO 1","394":"GRUPO 1","395":"GRUPO 1","396":"GRUPO 2","397":"GRUPO 2","398":"GRUPO 2","399":"GRUPO 2","400":"GRUPO 2","401":"GRUPO 2","402":"GRUPO 2","403":"GRUPO 2","404":"GRUPO 2","405":"GRUPO 2","406":"GRUPO 2","407":"GRUPO 2","408":"GRUPO 3","409":"GRUPO 3","410":"GRUPO 3","411":"GRUPO 3","412":"GRUPO 3","413":"GRUPO 3","414":"GRUPO 3","415":"GRUPO 3","416":"GRUPO 3","417":"GRUPO 3","418":"GRUPO 3","419":"GRUPO 3","420":"GRUPO 4","421":"GRUPO 4","422":"GRUPO 4","423":"GRUPO 4","424":"GRUPO 4","425":"GRUPO 4","426":"GRUPO 4","427":"GRUPO 4","428":"GRUPO 4","429":"GRUPO 4","430":"GRUPO 4","431":"GRUPO 4","432":"GRUPO 1","433":"GRUPO 1","434":"GRUPO 1","435":"GRUPO 1","436":"GRUPO 1","437":"GRUPO 1","438":"GRUPO 1","439":"GRUPO 1","440":"GRUPO 1","441":"GRUPO 1","442":"GRUPO 1","443":"GRUPO 1","444":"GRUPO 2","445":"GRUPO 2","446":"GRUPO 2","447":"GRUPO 2","448":"GRUPO 2","449":"GRUPO 2","450":"GRUPO 2","451":"GRUPO 2","452":"GRUPO 2","453":"GRUPO 2","454":"GRUPO 2","455":"GRUPO 2","456":"GRUPO 3","457":"GRUPO 3","458":"GRUPO 3","459":"GRUPO 3","460":"GRUPO 3","461":"GRUPO 3","462":"GRUPO 3","463":"GRUPO 3","464":"GRUPO 3","465":"GRUPO 3","466":"GRUPO 3","467":"GRUPO 3","468":"GRUPO 4","469":"GRUPO 4","470":"GRUPO 4","471":"GRUPO 4","472":"GRUPO 4","473":"GRUPO 4","474":"GRUPO 4","475":"GRUPO 4","476":"GRUPO 4","477":"GRUPO 4","478":"GRUPO 4","479":"GRUPO 4","480":"GRUPO 1","481":"GRUPO 1","482":"GRUPO 1","483":"GRUPO 1","484":"GRUPO 1","485":"GRUPO 1","486":"GRUPO 1","487":"GRUPO 1","488":"GRUPO 1","489":"GRUPO 1","490":"GRUPO 1","491":"GRUPO 1","492":"GRUPO 2","493":"GRUPO 2","494":"GRUPO 2","495":"GRUPO 2","496":"GRUPO 2","497":"GRUPO 2","498":"GRUPO 2","499":"GRUPO 2","500":"GRUPO 2","501":"GRUPO 2","502":"GRUPO 2","503":"GRUPO 2","504":"GRUPO 3","505":"GRUPO 3","506":"GRUPO 3","507":"GRUPO 3","508":"GRUPO 3","509":"GRUPO 3","510":"GRUPO 3","511":"GRUPO 3","512":"GRUPO 3","513":"GRUPO 3","514":"GRUPO 3","515":"GRUPO 3","516":"GRUPO 4","517":"GRUPO 4","518":"GRUPO 4","519":"GRUPO 4","520":"GRUPO 4","521":"GRUPO 4","522":"GRUPO 4","523":"GRUPO 4","524":"GRUPO 4","525":"GRUPO 4","526":"GRUPO 4","527":"GRUPO 4","528":"GRUPO 1","529":"GRUPO 1","530":"GRUPO 1","531":"GRUPO 1","532":"GRUPO 1","533":"GRUPO 1","534":"GRUPO 1","535":"GRUPO 1","536":"GRUPO 1","537":"GRUPO 1","538":"GRUPO 1","539":"GRUPO 1","540":"GRUPO 2","541":"GRUPO 2","542":"GRUPO 2","543":"GRUPO 2","544":"GRUPO 2","545":"GRUPO 2","546":"GRUPO 2","547":"GRUPO 2","548":"GRUPO 2","549":"GRUPO 2","550":"GRUPO 2","551":"GRUPO 2","552":"GRUPO 3","553":"GRUPO 3","554":"GRUPO 3","555":"GRUPO 3","556":"GRUPO 3","557":"GRUPO 3","558":"GRUPO 3","559":"GRUPO 3","560":"GRUPO 3","561":"GRUPO 3","562":"GRUPO 3","563":"GRUPO 3","564":"GRUPO 4","565":"GRUPO 4","566":"GRUPO 4","567":"GRUPO 4","568":"GRUPO 4","569":"GRUPO 4","570":"GRUPO 4","571":"GRUPO 4","572":"GRUPO 4","573":"GRUPO 4","574":"GRUPO 4","575":"GRUPO 4","576":"GRUPO 1","577":"GRUPO 1","578":"GRUPO 1","579":"GRUPO 1","580":"GRUPO 1","581":"GRUPO 1","582":"GRUPO 1","583":"GRUPO 1","584":"GRUPO 1","585":"GRUPO 1","586":"GRUPO 1","587":"GRUPO 1","588":"GRUPO 2","589":"GRUPO 2","590":"GRUPO 2","591":"GRUPO 2","592":"GRUPO 2","593":"GRUPO 2","594":"GRUPO 2","595":"GRUPO 2","596":"GRUPO 2","597":"GRUPO 2","598":"GRUPO 2","599":"GRUPO 2","600":"GRUPO 3","601":"GRUPO 3","602":"GRUPO 3","603":"GRUPO 3","604":"GRUPO 3","605":"GRUPO 3","606":"GRUPO 3","607":"GRUPO 3","608":"GRUPO 3","609":"GRUPO 3","610":"GRUPO 3","611":"GRUPO 3","612":"GRUPO 4","613":"GRUPO 4","614":"GRUPO 4","615":"GRUPO 4","616":"GRUPO 4","617":"GRUPO 4","618":"GRUPO 4","619":"GRUPO 4","620":"GRUPO 4","621":"GRUPO 4","622":"GRUPO 4","623":"GRUPO 4","624":"GRUPO 1","625":"GRUPO 1","626":"GRUPO 1","627":"GRUPO 1","628":"GRUPO 1","629":"GRUPO 1","630":"GRUPO 1","631":"GRUPO 1","632":"GRUPO 1","633":"GRUPO 1","634":"GRUPO 1","635":"GRUPO 1","636":"GRUPO 2","637":"GRUPO 2","638":"GRUPO 2","639":"GRUPO 2","640":"GRUPO 2","641":"GRUPO 2","642":"GRUPO 2","643":"GRUPO 2","644":"GRUPO 2","645":"GRUPO 2","646":"GRUPO 2","647":"GRUPO 2","648":"GRUPO 3","649":"GRUPO 3","650":"GRUPO 3","651":"GRUPO 3","652":"GRUPO 3","653":"GRUPO 3","654":"GRUPO 3","655":"GRUPO 3","656":"GRUPO 3","657":"GRUPO 3","658":"GRUPO 3","659":"GRUPO 3","660":"GRUPO 4","661":"GRUPO 4","662":"GRUPO 4","663":"GRUPO 4","664":"GRUPO 4","665":"GRUPO 4","666":"GRUPO 4","667":"GRUPO 4","668":"GRUPO 4","669":"GRUPO 4","670":"GRUPO 4","671":"GRUPO 4","672":"GRUPO 1","673":"GRUPO 1","674":"GRUPO 1","675":"GRUPO 1","676":"GRUPO 1","677":"GRUPO 1","678":"GRUPO 1","679":"GRUPO 1","680":"GRUPO 1","681":"GRUPO 1","682":"GRUPO 1","683":"GRUPO 1","684":"GRUPO 2","685":"GRUPO 2","686":"GRUPO 2","687":"GRUPO 2","688":"GRUPO 2","689":"GRUPO 2","690":"GRUPO 2","691":"GRUPO 2","692":"GRUPO 2","693":"GRUPO 2","694":"GRUPO 2","695":"GRUPO 2","696":"GRUPO 3","697":"GRUPO 3","698":"GRUPO 3","699":"GRUPO 3","700":"GRUPO 3","701":"GRUPO 3","702":"GRUPO 3","703":"GRUPO 3","704":"GRUPO 3","705":"GRUPO 3","706":"GRUPO 3","707":"GRUPO 3","708":"GRUPO 4","709":"GRUPO 4","710":"GRUPO 4","711":"GRUPO 4","712":"GRUPO 4","713":"GRUPO 4","714":"GRUPO 4","715":"GRUPO 4","716":"GRUPO 4","717":"GRUPO 4","718":"GRUPO 4","719":"GRUPO 4","720":"GRUPO 1","721":"GRUPO 1","722":"GRUPO 1","723":"GRUPO 1","724":"GRUPO 1","725":"GRUPO 1","726":"GRUPO 1","727":"GRUPO 1","728":"GRUPO 1","729":"GRUPO 1","730":"GRUPO 1","731":"GRUPO 1","732":"GRUPO 2","733":"GRUPO 2","734":"GRUPO 2","735":"GRUPO 2","736":"GRUPO 2","737":"GRUPO 2","738":"GRUPO 2","739":"GRUPO 2","740":"GRUPO 2","741":"GRUPO 2","742":"GRUPO 2","743":"GRUPO 2","744":"GRUPO 3","745":"GRUPO 3","746":"GRUPO 3","747":"GRUPO 3","748":"GRUPO 3","749":"GRUPO 3","750":"GRUPO 3","751":"GRUPO 3","752":"GRUPO 3","753":"GRUPO 3","754":"GRUPO 3","755":"GRUPO 3","756":"GRUPO 4","757":"GRUPO 4","758":"GRUPO 4","759":"GRUPO 4","760":"GRUPO 4","761":"GRUPO 4","762":"GRUPO 4","763":"GRUPO 4","764":"GRUPO 4","765":"GRUPO 4","766":"GRUPO 4","767":"GRUPO 4","768":"GRUPO 1","769":"GRUPO 1","770":"GRUPO 1","771":"GRUPO 1","772":"GRUPO 1","773":"GRUPO 1","774":"GRUPO 1","775":"GRUPO 1","776":"GRUPO 1","777":"GRUPO 1","778":"GRUPO 1","779":"GRUPO 1","780":"GRUPO 2","781":"GRUPO 2","782":"GRUPO 2","783":"GRUPO 2","784":"GRUPO 2","785":"GRUPO 2","786":"GRUPO 2","787":"GRUPO 2","788":"GRUPO 2","789":"GRUPO 2","790":"GRUPO 2","791":"GRUPO 2","792":"GRUPO 3","793":"GRUPO 3","794":"GRUPO 3","795":"GRUPO 3","796":"GRUPO 3","797":"GRUPO 3","798":"GRUPO 3","799":"GRUPO 3","800":"GRUPO 3","801":"GRUPO 3","802":"GRUPO 3","803":"GRUPO 3","804":"GRUPO 4","805":"GRUPO 4","806":"GRUPO 4","807":"GRUPO 4","808":"GRUPO 4","809":"GRUPO 4","810":"GRUPO 4","811":"GRUPO 4","812":"GRUPO 4","813":"GRUPO 4","814":"GRUPO 4","815":"GRUPO 4","816":"GRUPO 1","817":"GRUPO 1","818":"GRUPO 1","819":"GRUPO 1","820":"GRUPO 1","821":"GRUPO 1","822":"GRUPO 1","823":"GRUPO 1","824":"GRUPO 1","825":"GRUPO 1","826":"GRUPO 1","827":"GRUPO 1","828":"GRUPO 2","829":"GRUPO 2","830":"GRUPO 2","831":"GRUPO 2","832":"GRUPO 2","833":"GRUPO 2","834":"GRUPO 2","835":"GRUPO 2","836":"GRUPO 2","837":"GRUPO 2","838":"GRUPO 2","839":"GRUPO 2","840":"GRUPO 3","841":"GRUPO 3","842":"GRUPO 3","843":"GRUPO 3","844":"GRUPO 3","845":"GRUPO 3","846":"GRUPO 3","847":"GRUPO 3","848":"GRUPO 3","849":"GRUPO 3","850":"GRUPO 3","851":"GRUPO 3","852":"GRUPO 4","853":"GRUPO 4","854":"GRUPO 4","855":"GRUPO 4","856":"GRUPO 4","857":"GRUPO 4","858":"GRUPO 4","859":"GRUPO 4","860":"GRUPO 4","861":"GRUPO 4","862":"GRUPO 4","863":"GRUPO 4","864":"GRUPO 1","865":"GRUPO 1","866":"GRUPO 1","867":"GRUPO 1","868":"GRUPO 1","869":"GRUPO 1","870":"GRUPO 1","871":"GRUPO 1","872":"GRUPO 1","873":"GRUPO 1","874":"GRUPO 1","875":"GRUPO 1","876":"GRUPO 2","877":"GRUPO 2","878":"GRUPO 2","879":"GRUPO 2","880":"GRUPO 2","881":"GRUPO 2","882":"GRUPO 2","883":"GRUPO 2","884":"GRUPO 2","885":"GRUPO 2","886":"GRUPO 2","887":"GRUPO 2","888":"GRUPO 3","889":"GRUPO 3","890":"GRUPO 3","891":"GRUPO 3","892":"GRUPO 3","893":"GRUPO 3","894":"GRUPO 3","895":"GRUPO 3","896":"GRUPO 3","897":"GRUPO 3","898":"GRUPO 3","899":"GRUPO 3","900":"GRUPO 4","901":"GRUPO 4","902":"GRUPO 4","903":"GRUPO 4","904":"GRUPO 4","905":"GRUPO 4","906":"GRUPO 4","907":"GRUPO 4","908":"GRUPO 4","909":"GRUPO 4","910":"GRUPO 4","911":"GRUPO 4","912":"GRUPO 1","913":"GRUPO 1","914":"GRUPO 1","915":"GRUPO 1","916":"GRUPO 1","917":"GRUPO 1","918":"GRUPO 1","919":"GRUPO 1","920":"GRUPO 1","921":"GRUPO 1","922":"GRUPO 1","923":"GRUPO 1","924":"GRUPO 2","925":"GRUPO 2","926":"GRUPO 2","927":"GRUPO 2","928":"GRUPO 2","929":"GRUPO 2","930":"GRUPO 2","931":"GRUPO 2","932":"GRUPO 2","933":"GRUPO 2","934":"GRUPO 2","935":"GRUPO 2","936":"GRUPO 3","937":"GRUPO 3","938":"GRUPO 3","939":"GRUPO 3","940":"GRUPO 3","941":"GRUPO 3","942":"GRUPO 3","943":"GRUPO 3","944":"GRUPO 3","945":"GRUPO 3","946":"GRUPO 3","947":"GRUPO 3","948":"GRUPO 4","949":"GRUPO 4","950":"GRUPO 4","951":"GRUPO 4","952":"GRUPO 4","953":"GRUPO 4","954":"GRUPO 4","955":"GRUPO 4","956":"GRUPO 4","957":"GRUPO 4","958":"GRUPO 4","959":"GRUPO 4","960":"GRUPO 1","961":"GRUPO 1","962":"GRUPO 1","963":"GRUPO 1","964":"GRUPO 1","965":"GRUPO 1","966":"GRUPO 1","967":"GRUPO 1","968":"GRUPO 1","969":"GRUPO 1","970":"GRUPO 1","971":"GRUPO 1","972":"GRUPO 2","973":"GRUPO 2","974":"GRUPO 2","975":"GRUPO 2","976":"GRUPO 2","977":"GRUPO 2","978":"GRUPO 2","979":"GRUPO 2","980":"GRUPO 2","981":"GRUPO 2","982":"GRUPO 2","983":"GRUPO 2","984":"GRUPO 3","985":"GRUPO 3","986":"GRUPO 3","987":"GRUPO 3","988":"GRUPO 3","989":"GRUPO 3","990":"GRUPO 3","991":"GRUPO 3","992":"GRUPO 3","993":"GRUPO 3","994":"GRUPO 3","995":"GRUPO 3","996":"GRUPO 4","997":"GRUPO 4","998":"GRUPO 4","999":"GRUPO 4","1000":"GRUPO 4","1001":"GRUPO 4","1002":"GRUPO 4","1003":"GRUPO 4","1004":"GRUPO 4","1005":"GRUPO 4","1006":"GRUPO 4","1007":"GRUPO 4","1008":"GRUPO 1","1009":"GRUPO 1","1010":"GRUPO 1","1011":"GRUPO 1","1012":"GRUPO 1","1013":"GRUPO 1","1014":"GRUPO 1","1015":"GRUPO 1","1016":"GRUPO 1","1017":"GRUPO 1","1018":"GRUPO 1","1019":"GRUPO 1","1020":"GRUPO 2","1021":"GRUPO 2","1022":"GRUPO 2","1023":"GRUPO 2","1024":"GRUPO 2","1025":"GRUPO 2","1026":"GRUPO 2","1027":"GRUPO 2","1028":"GRUPO 2","1029":"GRUPO 2","1030":"GRUPO 2","1031":"GRUPO 2","1032":"GRUPO 3","1033":"GRUPO 3","1034":"GRUPO 3","1035":"GRUPO 3","1036":"GRUPO 3","1037":"GRUPO 3","1038":"GRUPO 3","1039":"GRUPO 3","1040":"GRUPO 3","1041":"GRUPO 3","1042":"GRUPO 3","1043":"GRUPO 3","1044":"GRUPO 4","1045":"GRUPO 4","1046":"GRUPO 4","1047":"GRUPO 4","1048":"GRUPO 4","1049":"GRUPO 4","1050":"GRUPO 4","1051":"GRUPO 4","1052":"GRUPO 4","1053":"GRUPO 4","1054":"GRUPO 4","1055":"GRUPO 4","1056":"GRUPO 1","1057":"GRUPO 1","1058":"GRUPO 1","1059":"GRUPO 1","1060":"GRUPO 1","1061":"GRUPO 1","1062":"GRUPO 1","1063":"GRUPO 1","1064":"GRUPO 1","1065":"GRUPO 1","1066":"GRUPO 1","1067":"GRUPO 1","1068":"GRUPO 2","1069":"GRUPO 2","1070":"GRUPO 2","1071":"GRUPO 2","1072":"GRUPO 2","1073":"GRUPO 2","1074":"GRUPO 2","1075":"GRUPO 2","1076":"GRUPO 2","1077":"GRUPO 2","1078":"GRUPO 2","1079":"GRUPO 2","1080":"GRUPO 3","1081":"GRUPO 3","1082":"GRUPO 3","1083":"GRUPO 3","1084":"GRUPO 3","1085":"GRUPO 3","1086":"GRUPO 3","1087":"GRUPO 3","1088":"GRUPO 3","1089":"GRUPO 3","1090":"GRUPO 3","1091":"GRUPO 3","1092":"GRUPO 4","1093":"GRUPO 4","1094":"GRUPO 4","1095":"GRUPO 4","1096":"GRUPO 4","1097":"GRUPO 4","1098":"GRUPO 4","1099":"GRUPO 4","1100":"GRUPO 4","1101":"GRUPO 4","1102":"GRUPO 4","1103":"GRUPO 4","1104":"GRUPO 1","1105":"GRUPO 1","1106":"GRUPO 1","1107":"GRUPO 1","1108":"GRUPO 1","1109":"GRUPO 1","1110":"GRUPO 1","1111":"GRUPO 1","1112":"GRUPO 1","1113":"GRUPO 1","1114":"GRUPO 1","1115":"GRUPO 1","1116":"GRUPO 2","1117":"GRUPO 2","1118":"GRUPO 2","1119":"GRUPO 2","1120":"GRUPO 2","1121":"GRUPO 2","1122":"GRUPO 2","1123":"GRUPO 2","1124":"GRUPO 2","1125":"GRUPO 2","1126":"GRUPO 2","1127":"GRUPO 2","1128":"GRUPO 3","1129":"GRUPO 3","1130":"GRUPO 3","1131":"GRUPO 3","1132":"GRUPO 3","1133":"GRUPO 3","1134":"GRUPO 3","1135":"GRUPO 3","1136":"GRUPO 3","1137":"GRUPO 3","1138":"GRUPO 3","1139":"GRUPO 3","1140":"GRUPO 4","1141":"GRUPO 4","1142":"GRUPO 4","1143":"GRUPO 4","1144":"GRUPO 4","1145":"GRUPO 4","1146":"GRUPO 4","1147":"GRUPO 4","1148":"GRUPO 4","1149":"GRUPO 4","1150":"GRUPO 4","1151":"GRUPO 4","1152":"GRUPO 1","1153":"GRUPO 1","1154":"GRUPO 1","1155":"GRUPO 1","1156":"GRUPO 1","1157":"GRUPO 1","1158":"GRUPO 1","1159":"GRUPO 1","1160":"GRUPO 1","1161":"GRUPO 1","1162":"GRUPO 1","1163":"GRUPO 1","1164":"GRUPO 2","1165":"GRUPO 2","1166":"GRUPO 2","1167":"GRUPO 2","1168":"GRUPO 2","1169":"GRUPO 2","1170":"GRUPO 2","1171":"GRUPO 2","1172":"GRUPO 2","1173":"GRUPO 2","1174":"GRUPO 2","1175":"GRUPO 2","1176":"GRUPO 3","1177":"GRUPO 3","1178":"GRUPO 3","1179":"GRUPO 3","1180":"GRUPO 3","1181":"GRUPO 3","1182":"GRUPO 3","1183":"GRUPO 3","1184":"GRUPO 3","1185":"GRUPO 3","1186":"GRUPO 3","1187":"GRUPO 3","1188":"GRUPO 4","1189":"GRUPO 4","1190":"GRUPO 4","1191":"GRUPO 4","1192":"GRUPO 4","1193":"GRUPO 4","1194":"GRUPO 4","1195":"GRUPO 4","1196":"GRUPO 4","1197":"GRUPO 4","1198":"GRUPO 4","1199":"GRUPO 4","1200":"GRUPO 1","1201":"GRUPO 1","1202":"GRUPO 1","1203":"GRUPO 1","1204":"GRUPO 1","1205":"GRUPO 1","1206":"GRUPO 1","1207":"GRUPO 1","1208":"GRUPO 1","1209":"GRUPO 1","1210":"GRUPO 1","1211":"GRUPO 1","1212":"GRUPO 2","1213":"GRUPO 2","1214":"GRUPO 2","1215":"GRUPO 2","1216":"GRUPO 2","1217":"GRUPO 2","1218":"GRUPO 2","1219":"GRUPO 2","1220":"GRUPO 2","1221":"GRUPO 2","1222":"GRUPO 2","1223":"GRUPO 2","1224":"GRUPO 3","1225":"GRUPO 3","1226":"GRUPO 3","1227":"GRUPO 3","1228":"GRUPO 3","1229":"GRUPO 3","1230":"GRUPO 3","1231":"GRUPO 3","1232":"GRUPO 3","1233":"GRUPO 3","1234":"GRUPO 3","1235":"GRUPO 3","1236":"GRUPO 4","1237":"GRUPO 4","1238":"GRUPO 4","1239":"GRUPO 4","1240":"GRUPO 4","1241":"GRUPO 4","1242":"GRUPO 4","1243":"GRUPO 4","1244":"GRUPO 4","1245":"GRUPO 4","1246":"GRUPO 4","1247":"GRUPO 4","1248":"GRUPO 1","1249":"GRUPO 1","1250":"GRUPO 1","1251":"GRUPO 1","1252":"GRUPO 1","1253":"GRUPO 1","1254":"GRUPO 1","1255":"GRUPO 1","1256":"GRUPO 1","1257":"GRUPO 1","1258":"GRUPO 1","1259":"GRUPO 1","1260":"GRUPO 2","1261":"GRUPO 2","1262":"GRUPO 2","1263":"GRUPO 2","1264":"GRUPO 2","1265":"GRUPO 2","1266":"GRUPO 2","1267":"GRUPO 2","1268":"GRUPO 2","1269":"GRUPO 2","1270":"GRUPO 2","1271":"GRUPO 2","1272":"GRUPO 3","1273":"GRUPO 3","1274":"GRUPO 3","1275":"GRUPO 3","1276":"GRUPO 3","1277":"GRUPO 3","1278":"GRUPO 3","1279":"GRUPO 3","1280":"GRUPO 3","1281":"GRUPO 3","1282":"GRUPO 3","1283":"GRUPO 3","1284":"GRUPO 4","1285":"GRUPO 4","1286":"GRUPO 4","1287":"GRUPO 4","1288":"GRUPO 4","1289":"GRUPO 4","1290":"GRUPO 4","1291":"GRUPO 4","1292":"GRUPO 4","1293":"GRUPO 4","1294":"GRUPO 4","1295":"GRUPO 4","1296":"GRUPO 1","1297":"GRUPO 1","1298":"GRUPO 1","1299":"GRUPO 1","1300":"GRUPO 1","1301":"GRUPO 1","1302":"GRUPO 1","1303":"GRUPO 1","1304":"GRUPO 1","1305":"GRUPO 1","1306":"GRUPO 1","1307":"GRUPO 1","1308":"GRUPO 2","1309":"GRUPO 2","1310":"GRUPO 2","1311":"GRUPO 2","1312":"GRUPO 2","1313":"GRUPO 2","1314":"GRUPO 2","1315":"GRUPO 2","1316":"GRUPO 2","1317":"GRUPO 2","1318":"GRUPO 2","1319":"GRUPO 2","1320":"GRUPO 3","1321":"GRUPO 3","1322":"GRUPO 3","1323":"GRUPO 3","1324":"GRUPO 3","1325":"GRUPO 3","1326":"GRUPO 3","1327":"GRUPO 3","1328":"GRUPO 3","1329":"GRUPO 3","1330":"GRUPO 3","1331":"GRUPO 3","1332":"GRUPO 4","1333":"GRUPO 4","1334":"GRUPO 4","1335":"GRUPO 4","1336":"GRUPO 4","1337":"GRUPO 4","1338":"GRUPO 4","1339":"GRUPO 4","1340":"GRUPO 4","1341":"GRUPO 4","1342":"GRUPO 4","1343":"GRUPO 4","1344":"GRUPO 1","1345":"GRUPO 1","1346":"GRUPO 1","1347":"GRUPO 1","1348":"GRUPO 1","1349":"GRUPO 1","1350":"GRUPO 1","1351":"GRUPO 1","1352":"GRUPO 1","1353":"GRUPO 1","1354":"GRUPO 1","1355":"GRUPO 1","1356":"GRUPO 2","1357":"GRUPO 2","1358":"GRUPO 2","1359":"GRUPO 2","1360":"GRUPO 2","1361":"GRUPO 2","1362":"GRUPO 2","1363":"GRUPO 2","1364":"GRUPO 2","1365":"GRUPO 2","1366":"GRUPO 2","1367":"GRUPO 2","1368":"GRUPO 3","1369":"GRUPO 3","1370":"GRUPO 3","1371":"GRUPO 3","1372":"GRUPO 3","1373":"GRUPO 3","1374":"GRUPO 3","1375":"GRUPO 3","1376":"GRUPO 3","1377":"GRUPO 3","1378":"GRUPO 3","1379":"GRUPO 3","1380":"GRUPO 4","1381":"GRUPO 4","1382":"GRUPO 4","1383":"GRUPO 4","1384":"GRUPO 4","1385":"GRUPO 4","1386":"GRUPO 4","1387":"GRUPO 4","1388":"GRUPO 4","1389":"GRUPO 4","1390":"GRUPO 4","1391":"GRUPO 4","1392":"GRUPO 1","1393":"GRUPO 1","1394":"GRUPO 1","1395":"GRUPO 1","1396":"GRUPO 1","1397":"GRUPO 1","1398":"GRUPO 1","1399":"GRUPO 1","1400":"GRUPO 1","1401":"GRUPO 1","1402":"GRUPO 1","1403":"GRUPO 1","1404":"GRUPO 2","1405":"GRUPO 2","1406":"GRUPO 2","1407":"GRUPO 2","1408":"GRUPO 2","1409":"GRUPO 2","1410":"GRUPO 2","1411":"GRUPO 2","1412":"GRUPO 2","1413":"GRUPO 2","1414":"GRUPO 2","1415":"GRUPO 2","1416":"GRUPO 3","1417":"GRUPO 3","1418":"GRUPO 3","1419":"GRUPO 3","1420":"GRUPO 3","1421":"GRUPO 3","1422":"GRUPO 3","1423":"GRUPO 3","1424":"GRUPO 3","1425":"GRUPO 3","1426":"GRUPO 3","1427":"GRUPO 3","1428":"GRUPO 4","1429":"GRUPO 4","1430":"GRUPO 4","1431":"GRUPO 4","1432":"GRUPO 4","1433":"GRUPO 4","1434":"GRUPO 4","1435":"GRUPO 4","1436":"GRUPO 4","1437":"GRUPO 4","1438":"GRUPO 4","1439":"GRUPO 4"},"Empleado":{"0":"BARON HERNANDEZ HAROLD ANTONIO","1":"CASTELLANOS CARVAJAL DEYVITH FABIAN","2":"AROCA TORRES JULIAN EDUARDO","3":"BERMUDEZ PARRA JENNIFER XIOMARA","4":"BERNAL BAQUERO JAMES RICARDO","5":"BURGOS ORTIZ JOSE HORACIO","6":"CANTOR PORRAS JUAN FERNEY","7":"CAPERA CAPERA JOSE GABRIEL","8":"CARDENAS LOTERO RICARDO ANDR\u00c9S","9":"RENDON OSPINA NELSON LEANDRO","10":"SARMIENTO URBINA MOISES DANIEL","11":"VELASCO VELASCO SEBASTI\u00c1N DAVID","12":"DELGADO DELGADO JOHAN DARIO","13":"FLOREZ SAUCESO KENIS ALBERTO","14":"CARDONA GARCIA OSCAR JAVIER","15":"CARVAJAL GARC\u00cdA HOVER MARCK","16":"CEPEDA PIRAQUIVE JUAN DAVID","17":"FAJARDO SAENZ OSCAR FERNANDO","18":"FLOREZ ESPITIA RONY ALBERTO","19":"GARCIA CUERVO EDWIN JAVIER","20":"GONZALEZ OCHOA JUAN CARLOS","21":"XXX1","22":"XXX2","23":"XXX3","24":"FONSECA RAY RICARDO","25":"GOMEZ BETANCUR JAIDER ANDRES","26":"GRANADA PATI\u00d1O CARLOS MARINO","27":"GRASS PLATA MIGUEL SNEIDER","28":"MANZANO CALVO JUAN SEBASTIAN","29":"MENDOZA GOITA MARIANSEL ZENAYDA","30":"MURILLO ARAQUE JAIVER GEOVANY","31":"NI\u00d1O ARENAS HECTOR GONZALO","32":"RAMIREZ CHAVERRA JHON EDISON","33":"XXX4","34":"XXX5","35":"XXX6","36":"RODRIGUEZ MOSQUERA LUIS FERNANDO","37":"PEPITO PEREZ","38":"RAMIREZ VARGAS MARCELA PAOLA","39":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","40":"TORO CISNEROS GARY JOSE","41":"USECHE CALDERON JADID ESTIVEN","42":"VASQUEZ NIETO CAMILO ANDRES","43":"JHONY CASTRO","44":"BERNAL JUAN DAVID","45":"XXX7","46":"XXX8","47":"XXX9","48":"BARON HERNANDEZ HAROLD ANTONIO","49":"CASTELLANOS CARVAJAL DEYVITH FABIAN","50":"AROCA TORRES JULIAN EDUARDO","51":"BERMUDEZ PARRA JENNIFER XIOMARA","52":"BERNAL BAQUERO JAMES RICARDO","53":"BURGOS ORTIZ JOSE HORACIO","54":"CANTOR PORRAS JUAN FERNEY","55":"CAPERA CAPERA JOSE GABRIEL","56":"CARDENAS LOTERO RICARDO ANDR\u00c9S","57":"RENDON OSPINA NELSON LEANDRO","58":"SARMIENTO URBINA MOISES DANIEL","59":"VELASCO VELASCO SEBASTI\u00c1N DAVID","60":"DELGADO DELGADO JOHAN DARIO","61":"FLOREZ SAUCESO KENIS ALBERTO","62":"CARDONA GARCIA OSCAR JAVIER","63":"CARVAJAL GARC\u00cdA HOVER MARCK","64":"CEPEDA PIRAQUIVE JUAN DAVID","65":"FAJARDO SAENZ OSCAR FERNANDO","66":"FLOREZ ESPITIA RONY ALBERTO","67":"GARCIA CUERVO EDWIN JAVIER","68":"GONZALEZ OCHOA JUAN CARLOS","69":"XXX1","70":"XXX2","71":"XXX3","72":"FONSECA RAY RICARDO","73":"GOMEZ BETANCUR JAIDER ANDRES","74":"GRANADA PATI\u00d1O CARLOS MARINO","75":"GRASS PLATA MIGUEL SNEIDER","76":"MANZANO CALVO JUAN SEBASTIAN","77":"MENDOZA GOITA MARIANSEL ZENAYDA","78":"MURILLO ARAQUE JAIVER GEOVANY","79":"NI\u00d1O ARENAS HECTOR GONZALO","80":"RAMIREZ CHAVERRA JHON EDISON","81":"XXX4","82":"XXX5","83":"XXX6","84":"RODRIGUEZ MOSQUERA LUIS FERNANDO","85":"PEPITO PEREZ","86":"RAMIREZ VARGAS MARCELA PAOLA","87":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","88":"TORO CISNEROS GARY JOSE","89":"USECHE CALDERON JADID ESTIVEN","90":"VASQUEZ NIETO CAMILO ANDRES","91":"JHONY CASTRO","92":"BERNAL JUAN DAVID","93":"XXX7","94":"XXX8","95":"XXX9","96":"BARON HERNANDEZ HAROLD ANTONIO","97":"CASTELLANOS CARVAJAL DEYVITH FABIAN","98":"AROCA TORRES JULIAN EDUARDO","99":"BERMUDEZ PARRA JENNIFER XIOMARA","100":"BERNAL BAQUERO JAMES RICARDO","101":"BURGOS ORTIZ JOSE HORACIO","102":"CANTOR PORRAS JUAN FERNEY","103":"CAPERA CAPERA JOSE GABRIEL","104":"CARDENAS LOTERO RICARDO ANDR\u00c9S","105":"RENDON OSPINA NELSON LEANDRO","106":"SARMIENTO URBINA MOISES DANIEL","107":"VELASCO VELASCO SEBASTI\u00c1N DAVID","108":"DELGADO DELGADO JOHAN DARIO","109":"FLOREZ SAUCESO KENIS ALBERTO","110":"CARDONA GARCIA OSCAR JAVIER","111":"CARVAJAL GARC\u00cdA HOVER MARCK","112":"CEPEDA PIRAQUIVE JUAN DAVID","113":"FAJARDO SAENZ OSCAR FERNANDO","114":"FLOREZ ESPITIA RONY ALBERTO","115":"GARCIA CUERVO EDWIN JAVIER","116":"GONZALEZ OCHOA JUAN CARLOS","117":"XXX1","118":"XXX2","119":"XXX3","120":"FONSECA RAY RICARDO","121":"GOMEZ BETANCUR JAIDER ANDRES","122":"GRANADA PATI\u00d1O CARLOS MARINO","123":"GRASS PLATA MIGUEL SNEIDER","124":"MANZANO CALVO JUAN SEBASTIAN","125":"MENDOZA GOITA MARIANSEL ZENAYDA","126":"MURILLO ARAQUE JAIVER GEOVANY","127":"NI\u00d1O ARENAS HECTOR GONZALO","128":"RAMIREZ CHAVERRA JHON EDISON","129":"XXX4","130":"XXX5","131":"XXX6","132":"RODRIGUEZ MOSQUERA LUIS FERNANDO","133":"PEPITO PEREZ","134":"RAMIREZ VARGAS MARCELA PAOLA","135":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","136":"TORO CISNEROS GARY JOSE","137":"USECHE CALDERON JADID ESTIVEN","138":"VASQUEZ NIETO CAMILO ANDRES","139":"JHONY CASTRO","140":"BERNAL JUAN DAVID","141":"XXX7","142":"XXX8","143":"XXX9","144":"BARON HERNANDEZ HAROLD ANTONIO","145":"CASTELLANOS CARVAJAL DEYVITH FABIAN","146":"AROCA TORRES JULIAN EDUARDO","147":"BERMUDEZ PARRA JENNIFER XIOMARA","148":"BERNAL BAQUERO JAMES RICARDO","149":"BURGOS ORTIZ JOSE HORACIO","150":"CANTOR PORRAS JUAN FERNEY","151":"CAPERA CAPERA JOSE GABRIEL","152":"CARDENAS LOTERO RICARDO ANDR\u00c9S","153":"RENDON OSPINA NELSON LEANDRO","154":"SARMIENTO URBINA MOISES DANIEL","155":"VELASCO VELASCO SEBASTI\u00c1N DAVID","156":"DELGADO DELGADO JOHAN DARIO","157":"FLOREZ SAUCESO KENIS ALBERTO","158":"CARDONA GARCIA OSCAR JAVIER","159":"CARVAJAL GARC\u00cdA HOVER MARCK","160":"CEPEDA PIRAQUIVE JUAN DAVID","161":"FAJARDO SAENZ OSCAR FERNANDO","162":"FLOREZ ESPITIA RONY ALBERTO","163":"GARCIA CUERVO EDWIN JAVIER","164":"GONZALEZ OCHOA JUAN CARLOS","165":"XXX1","166":"XXX2","167":"XXX3","168":"FONSECA RAY RICARDO","169":"GOMEZ BETANCUR JAIDER ANDRES","170":"GRANADA PATI\u00d1O CARLOS MARINO","171":"GRASS PLATA MIGUEL SNEIDER","172":"MANZANO CALVO JUAN SEBASTIAN","173":"MENDOZA GOITA MARIANSEL ZENAYDA","174":"MURILLO ARAQUE JAIVER GEOVANY","175":"NI\u00d1O ARENAS HECTOR GONZALO","176":"RAMIREZ CHAVERRA JHON EDISON","177":"XXX4","178":"XXX5","179":"XXX6","180":"RODRIGUEZ MOSQUERA LUIS FERNANDO","181":"PEPITO PEREZ","182":"RAMIREZ VARGAS MARCELA PAOLA","183":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","184":"TORO CISNEROS GARY JOSE","185":"USECHE CALDERON JADID ESTIVEN","186":"VASQUEZ NIETO CAMILO ANDRES","187":"JHONY CASTRO","188":"BERNAL JUAN DAVID","189":"XXX7","190":"XXX8","191":"XXX9","192":"BARON HERNANDEZ HAROLD ANTONIO","193":"CASTELLANOS CARVAJAL DEYVITH FABIAN","194":"AROCA TORRES JULIAN EDUARDO","195":"BERMUDEZ PARRA JENNIFER XIOMARA","196":"BERNAL BAQUERO JAMES RICARDO","197":"BURGOS ORTIZ JOSE HORACIO","198":"CANTOR PORRAS JUAN FERNEY","199":"CAPERA CAPERA JOSE GABRIEL","200":"CARDENAS LOTERO RICARDO ANDR\u00c9S","201":"RENDON OSPINA NELSON LEANDRO","202":"SARMIENTO URBINA MOISES DANIEL","203":"VELASCO VELASCO SEBASTI\u00c1N DAVID","204":"DELGADO DELGADO JOHAN DARIO","205":"FLOREZ SAUCESO KENIS ALBERTO","206":"CARDONA GARCIA OSCAR JAVIER","207":"CARVAJAL GARC\u00cdA HOVER MARCK","208":"CEPEDA PIRAQUIVE JUAN DAVID","209":"FAJARDO SAENZ OSCAR FERNANDO","210":"FLOREZ ESPITIA RONY ALBERTO","211":"GARCIA CUERVO EDWIN JAVIER","212":"GONZALEZ OCHOA JUAN CARLOS","213":"XXX1","214":"XXX2","215":"XXX3","216":"FONSECA RAY RICARDO","217":"GOMEZ BETANCUR JAIDER ANDRES","218":"GRANADA PATI\u00d1O CARLOS MARINO","219":"GRASS PLATA MIGUEL SNEIDER","220":"MANZANO CALVO JUAN SEBASTIAN","221":"MENDOZA GOITA MARIANSEL ZENAYDA","222":"MURILLO ARAQUE JAIVER GEOVANY","223":"NI\u00d1O ARENAS HECTOR GONZALO","224":"RAMIREZ CHAVERRA JHON EDISON","225":"XXX4","226":"XXX5","227":"XXX6","228":"RODRIGUEZ MOSQUERA LUIS FERNANDO","229":"PEPITO PEREZ","230":"RAMIREZ VARGAS MARCELA PAOLA","231":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","232":"TORO CISNEROS GARY JOSE","233":"USECHE CALDERON JADID ESTIVEN","234":"VASQUEZ NIETO CAMILO ANDRES","235":"JHONY CASTRO","236":"BERNAL JUAN DAVID","237":"XXX7","238":"XXX8","239":"XXX9","240":"BARON HERNANDEZ HAROLD ANTONIO","241":"CASTELLANOS CARVAJAL DEYVITH FABIAN","242":"AROCA TORRES JULIAN EDUARDO","243":"BERMUDEZ PARRA JENNIFER XIOMARA","244":"BERNAL BAQUERO JAMES RICARDO","245":"BURGOS ORTIZ JOSE HORACIO","246":"CANTOR PORRAS JUAN FERNEY","247":"CAPERA CAPERA JOSE GABRIEL","248":"CARDENAS LOTERO RICARDO ANDR\u00c9S","249":"RENDON OSPINA NELSON LEANDRO","250":"SARMIENTO URBINA MOISES DANIEL","251":"VELASCO VELASCO SEBASTI\u00c1N DAVID","252":"DELGADO DELGADO JOHAN DARIO","253":"FLOREZ SAUCESO KENIS ALBERTO","254":"CARDONA GARCIA OSCAR JAVIER","255":"CARVAJAL GARC\u00cdA HOVER MARCK","256":"CEPEDA PIRAQUIVE JUAN DAVID","257":"FAJARDO SAENZ OSCAR FERNANDO","258":"FLOREZ ESPITIA RONY ALBERTO","259":"GARCIA CUERVO EDWIN JAVIER","260":"GONZALEZ OCHOA JUAN CARLOS","261":"XXX1","262":"XXX2","263":"XXX3","264":"FONSECA RAY RICARDO","265":"GOMEZ BETANCUR JAIDER ANDRES","266":"GRANADA PATI\u00d1O CARLOS MARINO","267":"GRASS PLATA MIGUEL SNEIDER","268":"MANZANO CALVO JUAN SEBASTIAN","269":"MENDOZA GOITA MARIANSEL ZENAYDA","270":"MURILLO ARAQUE JAIVER GEOVANY","271":"NI\u00d1O ARENAS HECTOR GONZALO","272":"RAMIREZ CHAVERRA JHON EDISON","273":"XXX4","274":"XXX5","275":"XXX6","276":"RODRIGUEZ MOSQUERA LUIS FERNANDO","277":"PEPITO PEREZ","278":"RAMIREZ VARGAS MARCELA PAOLA","279":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","280":"TORO CISNEROS GARY JOSE","281":"USECHE CALDERON JADID ESTIVEN","282":"VASQUEZ NIETO CAMILO ANDRES","283":"JHONY CASTRO","284":"BERNAL JUAN DAVID","285":"XXX7","286":"XXX8","287":"XXX9","288":"BARON HERNANDEZ HAROLD ANTONIO","289":"CASTELLANOS CARVAJAL DEYVITH FABIAN","290":"AROCA TORRES JULIAN EDUARDO","291":"BERMUDEZ PARRA JENNIFER XIOMARA","292":"BERNAL BAQUERO JAMES RICARDO","293":"BURGOS ORTIZ JOSE</t>
+    <t>27/04/2026 15:57</t>
   </si>
   <si>
     <t>[{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master</t>
@@ -80,6 +77,9 @@
   </si>
   <si>
     <t>{"columns":["Grupo","Empleado","Cargo","Label","Final","n_dia"],"index":[0,1,2,3,4,5,6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23,24,25,26,27,28,29,30,31,32,33,34,35,36,37,38,39,40,41,42,43,44,45,46,47,48,49,50,51,52,53,54,55,56,57,58,59,60,61,62,63,64,65,66,67,68,69,70,71,72,73,74,75,76,77,78,79,80,81,82,83,84,85,86,87,88,89,90,91,92,93,94,95,96,97,98,99,100,101,102,103,104,105,106,107,108,109,110,111,112,113,114,115,116,117,118,119,120,121,122,123,124,125,126,127,128,129,130,131,132,133,134,135,136,137,138,139,140,141,142,143,144,145,146,147,148,149,150,151,152,153,154,155,156,157,158,159,160,161,162,163,164,165,166,167,168,169,170,171,172,173,174,175,176,177,178,179,180,181,182,183,184,185,186,187,188,189,190,191,192,193,194,195,196,197,198,199,200,201,202,203,204,205,206,207,208,209,210,211,212,213,214,215,216,217,218,219,220,221,222,223,224,225,226,227,228,229,230,231,232,233,234,235,236,237,238,239,240,241,242,243,244,245,246,247,248,249,250,251,252,253,254,255,256,257,258,259,260,261,262,263,264,265,266,267,268,269,270,271,272,273,274,275,276,277,278,279,280,281,282,283,284,285,286,287,288,289,290,291,292,293,294,295,296,297,298,299,300,301,302,303,304,305,306,307,308,309,310,311,312,313,314,315,316,317,318,319,320,321,322,323,324,325,326,327,328,329,330,331,332,333,334,335,336,337,338,339,340,341,342,343,344,345,346,347,348,349,350,351,352,353,354,355,356,357,358,359,360,361,362,363,364,365,366,367,368,369,370,371,372,373,374,375,376,377,378,379,380,381,382,383,384,385,386,387,388,389,390,391,392,393,394,395,396,397,398,399,400,401,402,403,404,405,406,407,408,409,410,411,412,413,414,415,416,417,418,419,420,421,422,423,424,425,426,427,428,429,430,431,432,433,434,435,436,437,438,439,440,441,442,443,444,445,446,447,448,449,450,451,452,453,454,455,456,457,458,459,460,461,462,463,464,465,466,467,468,469,470,471,472,473,474,475,476,477,478,479,480,481,482,483,484,485,486,487,488,489,490,491,492,493,494,495,496,497,498,499,500,501,502,503,504,505,506,507,508,509,510,511,512,513,514,515,516,517,518,519,520,521,522,523,524,525,526,527,528,529,530,531,532,533,534,535,536,537,538,539,540,541,542,543,544,545,546,547,548,549,550,551,552,553,554,555,556,557,558,559,560,561,562,563,564,565,566,567,568,569,570,571,572,573,574,575,576,577,578,579,580,581,582,583,584,585,586,587,588,589,590,591,592,593,594,595,596,597,598,599,600,601,602,603,604,605,606,607,608,609,610,611,612,613,614,615,616,617,618,619,620,621,622,623,624,625,626,627,628,629,630,631,632,633,634,635,636,637,638,639,640,641,642,643,644,645,646,647,648,649,650,651,652,653,654,655,656,657,658,659,660,661,662,663,664,665,666,667,668,669,670,671,672,673,674,675,676,677,678,679,680,681,682,683,684,685,686,687,688,689,690,691,692,693,694,695,696,697,698,699,700,701,702,703,704,705,706,707,708,709,710,711,712,713,714,715,716,717,718,719,720,721,722,723,724,725,726,727,728,729,730,731,732,733,734,735,736,737,738,739,740,741,742,743,744,745,746,747,748,749,750,751,752,753,754,755,756,757,758,759,760,761,762,763,764,765,766,767,768,769,770,771,772,773,774,775,776,777,778,779,780,781,782,783,784,785,786,787,788,789,790,791,792,793,794,795,796,797,798,799,800,801,802,803,804,805,806,807,808,809,810,811,812,813,814,815,816,817,818,819,820,821,822,823,824,825,826,827,828,829,830,831,832,833,834,835,836,837,838,839,840,841,842,843,844,845,846,847,848,849,850,851,852,853,854,855,856,857,858,859,860,861,862,863,864,865,866,867,868,869,870,871,872,873,874,875,876,877,878,879,880,881,882,883,884,885,886,887,888,889,890,891,892,893,894,895,896,897,898,899,900,901,902,903,904,905,906,907,908,909,910,911,912,913,914,915,916,917,918,919,920,921,922,923,924,925,926,927,928,929,930,931,932,933,934,935,936,937,938,939,940,941,942,943,944,945,946,947,948,949,950,951,952,953,954,955,956,957,958,959,960,961,962,963,964,965,966,967,968,969,970,971,972,973,974,975,976,977,978,979,980,981,982,983,984,985,986,987,988,989,990,991,992,993,994,995,996,997,998,999,1000,1001,1002,1003,1004,1005,1006,1007,1008,1009,1010,1011,1012,1013,1014,1015,1016,1017,1018,1019,1020,1021,1022,1023,1024,1025,1026,1027,1028,1029,1030,1031,1032,1033,1034,1035,1036,1037,1038,1039,1040,1041,1042,1043,1044,1045,1046,1047,1048,1049,1050,1051,1052,1053,1054,1055,1056,1057,1058,1059,1060,1061,1062,1063,1064,1065,1066,1067,1068,1069,1070,1071,1072,1073,1074,1075,1076,1077,1078,1079,1080,1081,1082,1083,1084,1085,1086,1087,1088,1089,1090,1091,1092,1093,1094,1095,1096,1097,1098,1099,1100,1101,1102,1103,1104,1105,1106,1107,1108,1109,1110,1111,1112,1113,1114,1115,1116,1117,1118,1119,1120,1121,1122,1123,1124,1125,1126,1127,1128,1129,1130,1131,1132,1133,1134,1135,1136,1137,1138,1139,1140,1141,1142,1143,1144,1145,1146,1147,1148,1149,1150,1151,1152,1153,1154,1155,1156,1157,1158,1159,1160,1161,1162,1163,1164,1165,1166,1167,1168,1169,1170,1171,1172,1173,1174,1175,1176,1177,1178,1179,1180,1181,1182,1183,1184,1185,1186,1187,1188,1189,1190,1191,1192,1193,1194,1195,1196,1197,1198,1199,1200,1201,1202,1203,1204,1205,1206,1207,1208,1209,1210,1211,1212,1213,1214,1215,1216,1217,1218,1219,1220,1221,1222,1223,1224,1225,1226,1227,1228,1229,1230,1231,1232,1233,1234,1235,1236,1237,1238,1239,1240,1241,1242,1243,1244,1245,1246,1247,1248,1249,1250,1251,1252,1253,1254,1255,1256,1257,1258,1259,1260,1261,1262,1263,1264,1265,1266,1267,1268,1269,1270,1271,1272,1273,1274,1275,1276,1277,1278,1279,1280,1281,1282,1283,1284,1285,1286,1287,1288,1289,1290,1291,1292,1293,1294,1295,1296,1297,1298,1299,1300,1301,1302,1303,1304,1305,1306,1307,1308,1309,1310,1311,1312,1313,1314,1315,1316,1317,1318,1319,1320,1321,1322,1323,1324,1325,1326,1327,1328,1329,1330,1331,1332,1333,1334,1335,1336,1337,1338,1339,1340,1341,1342,1343,1344,1345,1346,1347,1348,1349,1350,1351,1352,1353,1354,1355,1356,1357,1358,1359,1360,1361,1362,1363,1364,1365,1366,1367,1368,1369,1370,1371,1372,1373,1374,1375,1376,1377,1378,1379,1380,1381,1382,1383,1384,1385,1386,1387,1388,1389,1390,1391,1392,1393,1394,1395,1396,1397,1398,1399,1400,1401,1402,1403,1404,1405,1406,1407,1408,1409,1410,1411,1412,1413,1414,1415,1416,1417,1418,1419,1420,1421,1422,1423,1424,1425,1426,1427,1428,1429,1430,1431,1432,1433,1434,1435,1436,1437,1438,1439],"data":[["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","01-Lun","T1",1],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","01-Lun","T1",1],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","01-Lun","T1",1],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","01-Lun","T1",1],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","01-Lun","T1",1],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","01-Lun","T1",1],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","01-Lun","T1",1],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","01-Lun","T1",1],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","01-Lun","T1",1],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","01-Lun","T1",1],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","01-Lun","T1",1],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","01-Lun","T1",1],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","01-Lun","T2",1],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","01-Lun","T2",1],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","01-Lun","T2",1],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","01-Lun","T2",1],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","01-Lun","T2",1],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","01-Lun","T2",1],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","01-Lun","T2",1],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","01-Lun","T2",1],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","01-Lun","T2",1],["GRUPO 2","XXX1","Tecnico B","01-Lun","T2",1],["GRUPO 2","XXX2","Tecnico B","01-Lun","T2",1],["GRUPO 2","XXX3","Tecnico B","01-Lun","T2",1],["GRUPO 3","FONSECA RAY RICARDO","Master","01-Lun","T3",1],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","01-Lun","T3",1],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","01-Lun","T3",1],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","01-Lun","T3",1],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","01-Lun","T3",1],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","01-Lun","T3",1],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","01-Lun","T3",1],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","01-Lun","T3",1],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","01-Lun","T3",1],["GRUPO 3","XXX4","Tecnico B","01-Lun","T3",1],["GRUPO 3","XXX5","Tecnico B","01-Lun","T3",1],["GRUPO 3","XXX6","Tecnico B","01-Lun","T3",1],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","01-Lun","T1",1],["GRUPO 4","PEPITO PEREZ","Master","01-Lun","T1",1],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","01-Lun","T1",1],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","01-Lun","T1",1],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","01-Lun","T1",1],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","01-Lun","T1",1],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","01-Lun","T1",1],["GRUPO 4","JHONY CASTRO","Tecnico A","01-Lun","T1",1],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","01-Lun","T1",1],["GRUPO 4","XXX7","Tecnico B","01-Lun","T1",1],["GRUPO 4","XXX8","Tecnico B","01-Lun","T1",1],["GRUPO 4","XXX9","Tecnico B","01-Lun","T1",1],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","02-Mar","T1",2],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","02-Mar","T1",2],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","02-Mar","T1",2],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","02-Mar","T1",2],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","02-Mar","T1",2],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","02-Mar","T1",2],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","02-Mar","T1",2],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","02-Mar","T1",2],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","02-Mar","T1",2],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","02-Mar","T1",2],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","02-Mar","T1",2],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","02-Mar","T1",2],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","02-Mar","T2",2],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","02-Mar","T2",2],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","02-Mar","T2",2],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","02-Mar","T2",2],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","02-Mar","T2",2],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","02-Mar","T2",2],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","02-Mar","T2",2],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","02-Mar","T2",2],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","02-Mar","T2",2],["GRUPO 2","XXX1","Tecnico B","02-Mar","T2",2],["GRUPO 2","XXX2","Tecnico B","02-Mar","T2",2],["GRUPO 2","XXX3","Tecnico B","02-Mar","T2",2],["GRUPO 3","FONSECA RAY RICARDO","Master","02-Mar","T3",2],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","02-Mar","T3",2],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","02-Mar","T3",2],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","02-Mar","T3",2],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","02-Mar","T3",2],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","02-Mar","T3",2],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","02-Mar","T3",2],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","02-Mar","T3",2],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","02-Mar","T3",2],["GRUPO 3","XXX4","Tecnico B","02-Mar","T3",2],["GRUPO 3","XXX5","Tecnico B","02-Mar","T3",2],["GRUPO 3","XXX6","Tecnico B","02-Mar","T3",2],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","02-Mar","T1",2],["GRUPO 4","PEPITO PEREZ","Master","02-Mar","T1",2],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","02-Mar","T1",2],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","02-Mar","T1",2],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","02-Mar","T1",2],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","02-Mar","T1",2],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","02-Mar","T1",2],["GRUPO 4","JHONY CASTRO","Tecnico A","02-Mar","T1",2],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","02-Mar","T1",2],["GRUPO 4","XXX7","Tecnico B","02-Mar","T1",2],["GRUPO 4","XXX8","Tecnico B","02-Mar","T1",2],["GRUPO 4","XXX9","Tecnico B","02-Mar","T1",2],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","03-Mie","T1",3],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","03-Mie","T1",3],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","03-Mie","T1",3],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","03-Mie","T1",3],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","03-Mie","T1",3],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","03-Mie","T1",3],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","03-Mie","T1",3],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","03-Mie","T1",3],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","03-Mie","T1",3],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","03-Mie","T1",3],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","03-Mie","T1",3],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","03-Mie","T1",3],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","03-Mie","T2",3],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","03-Mie","T2",3],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","03-Mie","T2",3],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","03-Mie","T2",3],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","03-Mie","T2",3],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","03-Mie","T2",3],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","03-Mie","T2",3],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","03-Mie","T2",3],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","03-Mie","T2",3],["GRUPO 2","XXX1","Tecnico B","03-Mie","T2",3],["GRUPO 2","XXX2","Tecnico B","03-Mie","T2",3],["GRUPO 2","XXX3","Tecnico B","03-Mie","T2",3],["GRUPO 3","FONSECA RAY RICARDO","Master","03-Mie","T3",3],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","03-Mie","T3",3],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","03-Mie","T3",3],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","03-Mie","T3",3],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","03-Mie","T3",3],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","03-Mie","T3",3],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","03-Mie","T3",3],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","03-Mie","T3",3],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","03-Mie","T3",3],["GRUPO 3","XXX4","Tecnico B","03-Mie","T3",3],["GRUPO 3","XXX5","Tecnico B","03-Mie","T3",3],["GRUPO 3","XXX6","Tecnico B","03-Mie","T3",3],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","03-Mie","T1",3],["GRUPO 4","PEPITO PEREZ","Master","03-Mie","T1",3],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","03-Mie","T1",3],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","03-Mie","T1",3],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","03-Mie","T1",3],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","03-Mie","T1",3],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","03-Mie","T1",3],["GRUPO 4","JHONY CASTRO","Tecnico A","03-Mie","T1",3],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","03-Mie","T1",3],["GRUPO 4","XXX7","Tecnico B","03-Mie","T1",3],["GRUPO 4","XXX8","Tecnico B","03-Mie","T1",3],["GRUPO 4","XXX9","Tecnico B","03-Mie","T1",3],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","04-Jue","DESC. LEY",4],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","04-Jue","DESC. LEY",4],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","04-Jue","DESC. LEY",4],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","04-Jue","DESC. LEY",4],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","04-Jue","DESC. LEY",4],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","04-Jue","DESC. LEY",4],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","04-Jue","DESC. LEY",4],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","04-Jue","DESC. LEY",4],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","04-Jue","DESC. LEY",4],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","04-Jue","DESC. LEY",4],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","04-Jue","DESC. LEY",4],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","04-Jue","DESC. LEY",4],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","04-Jue","T2",4],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","04-Jue","T2",4],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","04-Jue","T2",4],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","04-Jue","T2",4],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","04-Jue","T2",4],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","04-Jue","T2",4],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","04-Jue","T2",4],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","04-Jue","T2",4],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","04-Jue","T2",4],["GRUPO 2","XXX1","Tecnico B","04-Jue","T2",4],["GRUPO 2","XXX2","Tecnico B","04-Jue","T2",4],["GRUPO 2","XXX3","Tecnico B","04-Jue","T2",4],["GRUPO 3","FONSECA RAY RICARDO","Master","04-Jue","T3",4],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","04-Jue","T3",4],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","04-Jue","T3",4],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","04-Jue","T3",4],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","04-Jue","T3",4],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","04-Jue","T3",4],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","04-Jue","T3",4],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","04-Jue","T3",4],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","04-Jue","T3",4],["GRUPO 3","XXX4","Tecnico B","04-Jue","T3",4],["GRUPO 3","XXX5","Tecnico B","04-Jue","T3",4],["GRUPO 3","XXX6","Tecnico B","04-Jue","T3",4],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","04-Jue","T1",4],["GRUPO 4","PEPITO PEREZ","Master","04-Jue","T1",4],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","04-Jue","T1",4],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","04-Jue","T1",4],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","04-Jue","T1",4],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","04-Jue","T1",4],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","04-Jue","T1",4],["GRUPO 4","JHONY CASTRO","Tecnico A","04-Jue","T1",4],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","04-Jue","T1",4],["GRUPO 4","XXX7","Tecnico B","04-Jue","T1",4],["GRUPO 4","XXX8","Tecnico B","04-Jue","T1",4],["GRUPO 4","XXX9","Tecnico B","04-Jue","T1",4],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","05-Vie","T1",5],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","05-Vie","T1",5],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","05-Vie","T1",5],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","05-Vie","T1",5],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","05-Vie","T1",5],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","05-Vie","T1",5],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","05-Vie","T1",5],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","05-Vie","T1",5],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","05-Vie","T1",5],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","05-Vie","T1",5],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","05-Vie","T1",5],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","05-Vie","T1",5],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","05-Vie","DESC. LEY",5],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","05-Vie","DESC. LEY",5],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","05-Vie","DESC. LEY",5],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","05-Vie","DESC. LEY",5],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","05-Vie","DESC. LEY",5],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","05-Vie","DESC. LEY",5],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","05-Vie","DESC. LEY",5],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","05-Vie","DESC. LEY",5],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","05-Vie","DESC. LEY",5],["GRUPO 2","XXX1","Tecnico B","05-Vie","DESC. LEY",5],["GRUPO 2","XXX2","Tecnico B","05-Vie","DESC. LEY",5],["GRUPO 2","XXX3","Tecnico B","05-Vie","DESC. LEY",5],["GRUPO 3","FONSECA RAY RICARDO","Master","05-Vie","T3",5],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","05-Vie","T3",5],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","05-Vie","T3",5],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","05-Vie","T3",5],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","05-Vie","T3",5],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","05-Vie","T3",5],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","05-Vie","T3",5],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","05-Vie","T3",5],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","05-Vie","T3",5],["GRUPO 3","XXX4","Tecnico B","05-Vie","T3",5],["GRUPO 3","XXX5","Tecnico B","05-Vie","T3",5],["GRUPO 3","XXX6","Tecnico B","05-Vie","T3",5],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","05-Vie","T2",5],["GRUPO 4","PEPITO PEREZ","Master","05-Vie","T2",5],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","05-Vie","T2",5],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","05-Vie","T2",5],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","05-Vie","T2",5],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","05-Vie","T2",5],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","05-Vie","T2",5],["GRUPO 4","JHONY CASTRO","Tecnico A","05-Vie","T2",5],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","05-Vie","T2",5],["GRUPO 4","XXX7","Tecnico B","05-Vie","T2",5],["GRUPO 4","XXX8","Tecnico B","05-Vie","T2",5],["GRUPO 4","XXX9","Tecnico B","05-Vie","T2",5],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","06-Sab","T1",6],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","06-Sab","T1",6],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","06-Sab","T1",6],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","06-Sab","T1",6],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","06-Sab","T1",6],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","06-Sab","T1",6],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","06-Sab","T1",6],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","06-Sab","T1",6],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","06-Sab","T1",6],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","06-Sab","T1",6],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","06-Sab","T1",6],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","06-Sab","T1",6],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","06-Sab","T2",6],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","06-Sab","T2",6],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","06-Sab","T2",6],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","06-Sab","T2",6],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","06-Sab","T2",6],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","06-Sab","T2",6],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","06-Sab","T2",6],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","06-Sab","T2",6],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","06-Sab","T2",6],["GRUPO 2","XXX1","Tecnico B","06-Sab","T2",6],["GRUPO 2","XXX2","Tecnico B","06-Sab","T2",6],["GRUPO 2","XXX3","Tecnico B","06-Sab","T2",6],["GRUPO 3","FONSECA RAY RICARDO","Master","06-Sab","DESC. LEY",6],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","06-Sab","DESC. LEY",6],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","06-Sab","DESC. LEY",6],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","06-Sab","DESC. LEY",6],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","06-Sab","DESC. LEY",6],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","06-Sab","DESC. LEY",6],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","06-Sab","DESC. LEY",6],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","06-Sab","DESC. LEY",6],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","06-Sab","DESC. LEY",6],["GRUPO 3","XXX4","Tecnico B","06-Sab","DESC. LEY",6],["GRUPO 3","XXX5","Tecnico B","06-Sab","DESC. LEY",6],["GRUPO 3","XXX6","Tecnico B","06-Sab","DESC. LEY",6],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","06-Sab","T3",6],["GRUPO 4","PEPITO PEREZ","Master","06-Sab","T3",6],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","06-Sab","T3",6],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","06-Sab","T3",6],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","06-Sab","T3",6],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","06-Sab","T3",6],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","06-Sab","T3",6],["GRUPO 4","JHONY CASTRO","Tecnico A","06-Sab","T3",6],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","06-Sab","T3",6],["GRUPO 4","XXX7","Tecnico B","06-Sab","T3",6],["GRUPO 4","XXX8","Tecnico B","06-Sab","T3",6],["GRUPO 4","XXX9","Tecnico B","06-Sab","T3",6],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","07-Dom","T1",7],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","07-Dom","T1",7],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","07-Dom","T1",7],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","07-Dom","T1",7],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","07-Dom","T1",7],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","07-Dom","T1",7],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","07-Dom","T1",7],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","07-Dom","T1",7],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","07-Dom","T1",7],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","07-Dom","T1",7],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","07-Dom","T1",7],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","07-Dom","T1",7],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","07-Dom","T2",7],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","07-Dom","T2",7],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","07-Dom","T2",7],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","07-Dom","T2",7],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","07-Dom","T2",7],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","07-Dom","T2",7],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","07-Dom","T2",7],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","07-Dom","T2",7],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","07-Dom","T2",7],["GRUPO 2","XXX1","Tecnico B","07-Dom","T2",7],["GRUPO 2","XXX2","Tecnico B","07-Dom","T2",7],["GRUPO 2","XXX3","Tecnico B","07-Dom","T2",7],["GRUPO 3","FONSECA RAY RICARDO","Master","07-Dom","T3",7],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","07-Dom","T3",7],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","07-Dom","T3",7],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","07-Dom","T3",7],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","07-Dom","T3",7],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","07-Dom","T3",7],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","07-Dom","T3",7],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","07-Dom","T3",7],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","07-Dom","T3",7],["GRUPO 3","XXX4","Tecnico B","07-Dom","T3",7],["GRUPO 3","XXX5","Tecnico B","07-Dom","T3",7],["GRUPO 3","XXX6","Tecnico B","07-Dom","T3",7],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","07-Dom","DESC. LEY",7],["GRUPO 4","PEPITO PEREZ","Master","07-Dom","DESC. LEY",7],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","07-Dom","DESC. LEY",7],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","07-Dom","DESC. LEY",7],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","07-Dom","DESC. LEY",7],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","07-Dom","DESC. LEY",7],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","07-Dom","DESC. LEY",7],["GRUPO 4","JHONY CASTRO","Tecnico A","07-Dom","DESC. LEY",7],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","07-Dom","DESC. LEY",7],["GRUPO 4","XXX7","Tecnico B","07-Dom","DESC. LEY",7],["GRUPO 4","XXX8","Tecnico B","07-Dom","DESC. LEY",7],["GRUPO 4","XXX9","Tecnico B","07-Dom","DESC. LEY",7],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","08-Lun","T1",8],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","08-Lun","T1",8],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","08-Lun","T1",8],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","08-Lun","T1",8],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","08-Lun","T1",8],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","08-Lun","T1",8],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","08-Lun","T1",8],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","08-Lun","T1",8],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","08-Lun","T1",8],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","08-Lun","T1",8],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","08-Lun","T1",8],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","08-Lun","T1",8],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","08-Lun","T2",8],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","08-Lun","T2",8],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","08-Lun","T2",8],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","08-Lun","T2",8],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","08-Lun","T2",8],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","08-Lun","T2",8],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","08-Lun","T2",8],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","08-Lun","T2",8],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","08-Lun","T2",8],["GRUPO 2","XXX1","Tecnico B","08-Lun","T2",8],["GRUPO 2","XXX2","Tecnico B","08-Lun","T2",8],["GRUPO 2","XXX3","Tecnico B","08-Lun","T2",8],["GRUPO 3","FONSECA RAY RICARDO","Master","08-Lun","T3",8],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","08-Lun","T3",8],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","08-Lun","T3",8],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","08-Lun","T3",8],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","08-Lun","T3",8],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","08-Lun","T3",8],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","08-Lun","T3",8],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","08-Lun","T3",8],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","08-Lun","T3",8],["GRUPO 3","XXX4","Tecnico B","08-Lun","T3",8],["GRUPO 3","XXX5","Tecnico B","08-Lun","T3",8],["GRUPO 3","XXX6","Tecnico B","08-Lun","T3",8],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","08-Lun","T1",8],["GRUPO 4","PEPITO PEREZ","Master","08-Lun","T1",8],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","08-Lun","T1",8],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","08-Lun","T1",8],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","08-Lun","T1",8],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","08-Lun","T1",8],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","08-Lun","T1",8],["GRUPO 4","JHONY CASTRO","Tecnico A","08-Lun","T1",8],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","08-Lun","T1",8],["GRUPO 4","XXX7","Tecnico B","08-Lun","T1",8],["GRUPO 4","XXX8","Tecnico B","08-Lun","T1",8],["GRUPO 4","XXX9","Tecnico B","08-Lun","T1",8],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","09-Mar","T1",9],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","09-Mar","T1",9],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","09-Mar","T1",9],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","09-Mar","T1",9],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","09-Mar","T1",9],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","09-Mar","T1",9],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","09-Mar","T1",9],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","09-Mar","T1",9],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","09-Mar","T1",9],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","09-Mar","T1",9],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","09-Mar","T1",9],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","09-Mar","T1",9],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","09-Mar","T2",9],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","09-Mar","T2",9],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","</t>
+  </si>
+  <si>
+    <t>{"columns":["Grupo","Empleado","Cargo","Label","Final","n_dia"],"index":[0,1,2,3,4,5,6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23,24,25,26,27,28,29,30,31,32,33,34,35,36,37,38,39,40,41,42,43,44,45,46,47,48,49,50,51,52,53,54,55,56,57,58,59,60,61,62,63,64,65,66,67,68,69,70,71,72,73,74,75,76,77,78,79,80,81,82,83,84,85,86,87,88,89,90,91,92,93,94,95,96,97,98,99,100,101,102,103,104,105,106,107,108,109,110,111,112,113,114,115,116,117,118,119,120,121,122,123,124,125,126,127,128,129,130,131,132,133,134,135,136,137,138,139,140,141,142,143,144,145,146,147,148,149,150,151,152,153,154,155,156,157,158,159,160,161,162,163,164,165,166,167,168,169,170,171,172,173,174,175,176,177,178,179,180,181,182,183,184,185,186,187,188,189,190,191,192,193,194,195,196,197,198,199,200,201,202,203,204,205,206,207,208,209,210,211,212,213,214,215,216,217,218,219,220,221,222,223,224,225,226,227,228,229,230,231,232,233,234,235,236,237,238,239,240,241,242,243,244,245,246,247,248,249,250,251,252,253,254,255,256,257,258,259,260,261,262,263,264,265,266,267,268,269,270,271,272,273,274,275,276,277,278,279,280,281,282,283,284,285,286,287,288,289,290,291,292,293,294,295,296,297,298,299,300,301,302,303,304,305,306,307,308,309,310,311,312,313,314,315,316,317,318,319,320,321,322,323,324,325,326,327,328,329,330,331,332,333,334,335,336,337,338,339,340,341,342,343,344,345,346,347,348,349,350,351,352,353,354,355,356,357,358,359,360,361,362,363,364,365,366,367,368,369,370,371,372,373,374,375,376,377,378,379,380,381,382,383,384,385,386,387,388,389,390,391,392,393,394,395,396,397,398,399,400,401,402,403,404,405,406,407,408,409,410,411,412,413,414,415,416,417,418,419,420,421,422,423,424,425,426,427,428,429,430,431,432,433,434,435,436,437,438,439,440,441,442,443,444,445,446,447,448,449,450,451,452,453,454,455,456,457,458,459,460,461,462,463,464,465,466,467,468,469,470,471,472,473,474,475,476,477,478,479,480,481,482,483,484,485,486,487,488,489,490,491,492,493,494,495,496,497,498,499,500,501,502,503,504,505,506,507,508,509,510,511,512,513,514,515,516,517,518,519,520,521,522,523,524,525,526,527,528,529,530,531,532,533,534,535,536,537,538,539,540,541,542,543,544,545,546,547,548,549,550,551,552,553,554,555,556,557,558,559,560,561,562,563,564,565,566,567,568,569,570,571,572,573,574,575,576,577,578,579,580,581,582,583,584,585,586,587,588,589,590,591,592,593,594,595,596,597,598,599,600,601,602,603,604,605,606,607,608,609,610,611,612,613,614,615,616,617,618,619,620,621,622,623,624,625,626,627,628,629,630,631,632,633,634,635,636,637,638,639,640,641,642,643,644,645,646,647,648,649,650,651,652,653,654,655,656,657,658,659,660,661,662,663,664,665,666,667,668,669,670,671,672,673,674,675,676,677,678,679,680,681,682,683,684,685,686,687,688,689,690,691,692,693,694,695,696,697,698,699,700,701,702,703,704,705,706,707,708,709,710,711,712,713,714,715,716,717,718,719,720,721,722,723,724,725,726,727,728,729,730,731,732,733,734,735,736,737,738,739,740,741,742,743,744,745,746,747,748,749,750,751,752,753,754,755,756,757,758,759,760,761,762,763,764,765,766,767,768,769,770,771,772,773,774,775,776,777,778,779,780,781,782,783,784,785,786,787,788,789,790,791,792,793,794,795,796,797,798,799,800,801,802,803,804,805,806,807,808,809,810,811,812,813,814,815,816,817,818,819,820,821,822,823,824,825,826,827,828,829,830,831,832,833,834,835,836,837,838,839,840,841,842,843,844,845,846,847,848,849,850,851,852,853,854,855,856,857,858,859,860,861,862,863,864,865,866,867,868,869,870,871,872,873,874,875,876,877,878,879,880,881,882,883,884,885,886,887,888,889,890,891,892,893,894,895,896,897,898,899,900,901,902,903,904,905,906,907,908,909,910,911,912,913,914,915,916,917,918,919,920,921,922,923,924,925,926,927,928,929,930,931,932,933,934,935,936,937,938,939,940,941,942,943,944,945,946,947,948,949,950,951,952,953,954,955,956,957,958,959,960,961,962,963,964,965,966,967,968,969,970,971,972,973,974,975,976,977,978,979,980,981,982,983,984,985,986,987,988,989,990,991,992,993,994,995,996,997,998,999,1000,1001,1002,1003,1004,1005,1006,1007,1008,1009,1010,1011,1012,1013,1014,1015,1016,1017,1018,1019,1020,1021,1022,1023,1024,1025,1026,1027,1028,1029,1030,1031,1032,1033,1034,1035,1036,1037,1038,1039,1040,1041,1042,1043,1044,1045,1046,1047,1048,1049,1050,1051,1052,1053,1054,1055,1056,1057,1058,1059,1060,1061,1062,1063,1064,1065,1066,1067,1068,1069,1070,1071,1072,1073,1074,1075,1076,1077,1078,1079,1080,1081,1082,1083,1084,1085,1086,1087,1088,1089,1090,1091,1092,1093,1094,1095,1096,1097,1098,1099,1100,1101,1102,1103,1104,1105,1106,1107,1108,1109,1110,1111,1112,1113,1114,1115,1116,1117,1118,1119,1120,1121,1122,1123,1124,1125,1126,1127,1128,1129,1130,1131,1132,1133,1134,1135,1136,1137,1138,1139,1140,1141,1142,1143,1144,1145,1146,1147,1148,1149,1150,1151,1152,1153,1154,1155,1156,1157,1158,1159,1160,1161,1162,1163,1164,1165,1166,1167,1168,1169,1170,1171,1172,1173,1174,1175,1176,1177,1178,1179,1180,1181,1182,1183,1184,1185,1186,1187,1188,1189,1190,1191,1192,1193,1194,1195,1196,1197,1198,1199,1200,1201,1202,1203,1204,1205,1206,1207,1208,1209,1210,1211,1212,1213,1214,1215,1216,1217,1218,1219,1220,1221,1222,1223,1224,1225,1226,1227,1228,1229,1230,1231,1232,1233,1234,1235,1236,1237,1238,1239,1240,1241,1242,1243,1244,1245,1246,1247,1248,1249,1250,1251,1252,1253,1254,1255,1256,1257,1258,1259,1260,1261,1262,1263,1264,1265,1266,1267,1268,1269,1270,1271,1272,1273,1274,1275,1276,1277,1278,1279,1280,1281,1282,1283,1284,1285,1286,1287,1288,1289,1290,1291,1292,1293,1294,1295,1296,1297,1298,1299,1300,1301,1302,1303,1304,1305,1306,1307,1308,1309,1310,1311,1312,1313,1314,1315,1316,1317,1318,1319,1320,1321,1322,1323,1324,1325,1326,1327,1328,1329,1330,1331,1332,1333,1334,1335,1336,1337,1338,1339,1340,1341,1342,1343,1344,1345,1346,1347,1348,1349,1350,1351,1352,1353,1354,1355,1356,1357,1358,1359,1360,1361,1362,1363,1364,1365,1366,1367,1368,1369,1370,1371,1372,1373,1374,1375,1376,1377,1378,1379,1380,1381,1382,1383,1384,1385,1386,1387,1388,1389,1390,1391,1392,1393,1394,1395,1396,1397,1398,1399,1400,1401,1402,1403,1404,1405,1406,1407,1408,1409,1410,1411,1412,1413,1414,1415,1416,1417,1418,1419,1420,1421,1422,1423,1424,1425,1426,1427,1428,1429,1430,1431,1432,1433,1434,1435,1436,1437,1438,1439],"data":[["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","01-Mie","T1",1],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","01-Mie","T1",1],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","01-Mie","T1",1],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","01-Mie","T1",1],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","01-Mie","T1",1],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","01-Mie","T1",1],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","01-Mie","T1",1],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","01-Mie","T1",1],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","01-Mie","T1",1],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","01-Mie","T1",1],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","01-Mie","T1",1],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","01-Mie","T1",1],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","01-Mie","T2",1],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","01-Mie","T2",1],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","01-Mie","T2",1],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","01-Mie","T2",1],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","01-Mie","T2",1],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","01-Mie","T2",1],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","01-Mie","T2",1],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","01-Mie","T2",1],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","01-Mie","T2",1],["GRUPO 2","XXX1","Tecnico B","01-Mie","T2",1],["GRUPO 2","XXX2","Tecnico B","01-Mie","T2",1],["GRUPO 2","XXX3","Tecnico B","01-Mie","T2",1],["GRUPO 3","FONSECA RAY RICARDO","Master","01-Mie","T3",1],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","01-Mie","T3",1],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","01-Mie","T3",1],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","01-Mie","T3",1],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","01-Mie","T3",1],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","01-Mie","T3",1],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","01-Mie","T3",1],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","01-Mie","T3",1],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","01-Mie","T3",1],["GRUPO 3","XXX4","Tecnico B","01-Mie","T3",1],["GRUPO 3","XXX5","Tecnico B","01-Mie","T3",1],["GRUPO 3","XXX6","Tecnico B","01-Mie","T3",1],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","01-Mie","T1",1],["GRUPO 4","PEPITO PEREZ","Master","01-Mie","T1",1],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","01-Mie","T1",1],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","01-Mie","T1",1],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","01-Mie","T1",1],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","01-Mie","T1",1],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","01-Mie","T1",1],["GRUPO 4","JHONY CASTRO","Tecnico A","01-Mie","T1",1],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","01-Mie","T1",1],["GRUPO 4","XXX7","Tecnico B","01-Mie","T1",1],["GRUPO 4","XXX8","Tecnico B","01-Mie","T1",1],["GRUPO 4","XXX9","Tecnico B","01-Mie","T1",1],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","02-Jue","DESC. LEY",2],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","02-Jue","DESC. LEY",2],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","02-Jue","DESC. LEY",2],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","02-Jue","DESC. LEY",2],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","02-Jue","DESC. LEY",2],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","02-Jue","DESC. LEY",2],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","02-Jue","DESC. LEY",2],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","02-Jue","DESC. LEY",2],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","02-Jue","DESC. LEY",2],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","02-Jue","DESC. LEY",2],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","02-Jue","DESC. LEY",2],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","02-Jue","DESC. LEY",2],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","02-Jue","T2",2],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","02-Jue","T2",2],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","02-Jue","T2",2],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","02-Jue","T2",2],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","02-Jue","T2",2],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","02-Jue","T2",2],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","02-Jue","T2",2],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","02-Jue","T2",2],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","02-Jue","T2",2],["GRUPO 2","XXX1","Tecnico B","02-Jue","T2",2],["GRUPO 2","XXX2","Tecnico B","02-Jue","T2",2],["GRUPO 2","XXX3","Tecnico B","02-Jue","T2",2],["GRUPO 3","FONSECA RAY RICARDO","Master","02-Jue","T3",2],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","02-Jue","T3",2],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","02-Jue","T3",2],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","02-Jue","T3",2],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","02-Jue","T3",2],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","02-Jue","T3",2],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","02-Jue","T3",2],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","02-Jue","T3",2],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","02-Jue","T3",2],["GRUPO 3","XXX4","Tecnico B","02-Jue","T3",2],["GRUPO 3","XXX5","Tecnico B","02-Jue","T3",2],["GRUPO 3","XXX6","Tecnico B","02-Jue","T3",2],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","02-Jue","T1",2],["GRUPO 4","PEPITO PEREZ","Master","02-Jue","T1",2],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","02-Jue","T1",2],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","02-Jue","T1",2],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","02-Jue","T1",2],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","02-Jue","T1",2],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","02-Jue","T1",2],["GRUPO 4","JHONY CASTRO","Tecnico A","02-Jue","T1",2],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","02-Jue","T1",2],["GRUPO 4","XXX7","Tecnico B","02-Jue","T1",2],["GRUPO 4","XXX8","Tecnico B","02-Jue","T1",2],["GRUPO 4","XXX9","Tecnico B","02-Jue","T1",2],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","03-Vie","T1",3],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","03-Vie","T1",3],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","03-Vie","T1",3],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","03-Vie","T1",3],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","03-Vie","T1",3],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","03-Vie","T1",3],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","03-Vie","T1",3],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","03-Vie","T1",3],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","03-Vie","T1",3],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","03-Vie","T1",3],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","03-Vie","T1",3],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","03-Vie","T1",3],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","03-Vie","DESC. LEY",3],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","03-Vie","DESC. LEY",3],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","03-Vie","DESC. LEY",3],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","03-Vie","DESC. LEY",3],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","03-Vie","DESC. LEY",3],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","03-Vie","DESC. LEY",3],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","03-Vie","DESC. LEY",3],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","03-Vie","DESC. LEY",3],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","03-Vie","DESC. LEY",3],["GRUPO 2","XXX1","Tecnico B","03-Vie","DESC. LEY",3],["GRUPO 2","XXX2","Tecnico B","03-Vie","DESC. LEY",3],["GRUPO 2","XXX3","Tecnico B","03-Vie","DESC. LEY",3],["GRUPO 3","FONSECA RAY RICARDO","Master","03-Vie","T3",3],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","03-Vie","T3",3],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","03-Vie","T3",3],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","03-Vie","T3",3],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","03-Vie","T3",3],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","03-Vie","T3",3],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","03-Vie","T3",3],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","03-Vie","T3",3],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","03-Vie","T3",3],["GRUPO 3","XXX4","Tecnico B","03-Vie","T3",3],["GRUPO 3","XXX5","Tecnico B","03-Vie","T3",3],["GRUPO 3","XXX6","Tecnico B","03-Vie","T3",3],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","03-Vie","T2",3],["GRUPO 4","PEPITO PEREZ","Master","03-Vie","T2",3],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","03-Vie","T2",3],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","03-Vie","T2",3],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","03-Vie","T2",3],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","03-Vie","T2",3],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","03-Vie","T2",3],["GRUPO 4","JHONY CASTRO","Tecnico A","03-Vie","T2",3],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","03-Vie","T2",3],["GRUPO 4","XXX7","Tecnico B","03-Vie","T2",3],["GRUPO 4","XXX8","Tecnico B","03-Vie","T2",3],["GRUPO 4","XXX9","Tecnico B","03-Vie","T2",3],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","04-Sab","T1",4],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","04-Sab","T1",4],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","04-Sab","T1",4],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","04-Sab","T1",4],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","04-Sab","T1",4],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","04-Sab","T1",4],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","04-Sab","T1",4],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","04-Sab","T1",4],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","04-Sab","T1",4],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","04-Sab","T1",4],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","04-Sab","T1",4],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","04-Sab","T1",4],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","04-Sab","T2",4],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","04-Sab","T2",4],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","04-Sab","T2",4],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","04-Sab","T2",4],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","04-Sab","T2",4],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","04-Sab","T2",4],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","04-Sab","T2",4],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","04-Sab","T2",4],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","04-Sab","T2",4],["GRUPO 2","XXX1","Tecnico B","04-Sab","T2",4],["GRUPO 2","XXX2","Tecnico B","04-Sab","T2",4],["GRUPO 2","XXX3","Tecnico B","04-Sab","T2",4],["GRUPO 3","FONSECA RAY RICARDO","Master","04-Sab","DESC. LEY",4],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","04-Sab","DESC. LEY",4],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","04-Sab","DESC. LEY",4],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","04-Sab","DESC. LEY",4],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","04-Sab","DESC. LEY",4],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","04-Sab","DESC. LEY",4],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","04-Sab","DESC. LEY",4],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","04-Sab","DESC. LEY",4],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","04-Sab","DESC. LEY",4],["GRUPO 3","XXX4","Tecnico B","04-Sab","DESC. LEY",4],["GRUPO 3","XXX5","Tecnico B","04-Sab","DESC. LEY",4],["GRUPO 3","XXX6","Tecnico B","04-Sab","DESC. LEY",4],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","04-Sab","T3",4],["GRUPO 4","PEPITO PEREZ","Master","04-Sab","T3",4],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","04-Sab","T3",4],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","04-Sab","T3",4],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","04-Sab","T3",4],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","04-Sab","T3",4],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","04-Sab","T3",4],["GRUPO 4","JHONY CASTRO","Tecnico A","04-Sab","T3",4],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","04-Sab","T3",4],["GRUPO 4","XXX7","Tecnico B","04-Sab","T3",4],["GRUPO 4","XXX8","Tecnico B","04-Sab","T3",4],["GRUPO 4","XXX9","Tecnico B","04-Sab","T3",4],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","05-Dom","T1",5],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","05-Dom","T1",5],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","05-Dom","T1",5],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","05-Dom","T1",5],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","05-Dom","T1",5],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","05-Dom","T1",5],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","05-Dom","T1",5],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","05-Dom","T1",5],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","05-Dom","T1",5],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","05-Dom","T1",5],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","05-Dom","T1",5],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","05-Dom","T1",5],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","05-Dom","T2",5],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","05-Dom","T2",5],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","05-Dom","T2",5],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","05-Dom","T2",5],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","05-Dom","T2",5],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","05-Dom","T2",5],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","05-Dom","T2",5],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","05-Dom","T2",5],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","05-Dom","T2",5],["GRUPO 2","XXX1","Tecnico B","05-Dom","T2",5],["GRUPO 2","XXX2","Tecnico B","05-Dom","T2",5],["GRUPO 2","XXX3","Tecnico B","05-Dom","T2",5],["GRUPO 3","FONSECA RAY RICARDO","Master","05-Dom","T3",5],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","05-Dom","T3",5],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","05-Dom","T3",5],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","05-Dom","T3",5],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","05-Dom","T3",5],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","05-Dom","T3",5],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","05-Dom","T3",5],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","05-Dom","T3",5],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","05-Dom","T3",5],["GRUPO 3","XXX4","Tecnico B","05-Dom","T3",5],["GRUPO 3","XXX5","Tecnico B","05-Dom","T3",5],["GRUPO 3","XXX6","Tecnico B","05-Dom","T3",5],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","05-Dom","DESC. LEY",5],["GRUPO 4","PEPITO PEREZ","Master","05-Dom","DESC. LEY",5],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","05-Dom","DESC. LEY",5],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","05-Dom","DESC. LEY",5],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","05-Dom","DESC. LEY",5],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","05-Dom","DESC. LEY",5],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","05-Dom","DESC. LEY",5],["GRUPO 4","JHONY CASTRO","Tecnico A","05-Dom","DESC. LEY",5],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","05-Dom","DESC. LEY",5],["GRUPO 4","XXX7","Tecnico B","05-Dom","DESC. LEY",5],["GRUPO 4","XXX8","Tecnico B","05-Dom","DESC. LEY",5],["GRUPO 4","XXX9","Tecnico B","05-Dom","DESC. LEY",5],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","06-Lun","T1",6],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","06-Lun","T1",6],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","06-Lun","T1",6],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","06-Lun","T1",6],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","06-Lun","T1",6],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","06-Lun","T1",6],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","06-Lun","T1",6],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","06-Lun","T1",6],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","06-Lun","T1",6],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","06-Lun","T1",6],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","06-Lun","T1",6],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","06-Lun","T1",6],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","06-Lun","T2",6],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","06-Lun","T2",6],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","06-Lun","T2",6],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","06-Lun","T2",6],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","06-Lun","T2",6],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","06-Lun","T2",6],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","06-Lun","T2",6],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","06-Lun","T2",6],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","06-Lun","T2",6],["GRUPO 2","XXX1","Tecnico B","06-Lun","T2",6],["GRUPO 2","XXX2","Tecnico B","06-Lun","T2",6],["GRUPO 2","XXX3","Tecnico B","06-Lun","T2",6],["GRUPO 3","FONSECA RAY RICARDO","Master","06-Lun","T3",6],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","06-Lun","T3",6],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","06-Lun","T3",6],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","06-Lun","T3",6],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","06-Lun","T3",6],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","06-Lun","T3",6],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","06-Lun","T3",6],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","06-Lun","T3",6],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","06-Lun","T3",6],["GRUPO 3","XXX4","Tecnico B","06-Lun","T3",6],["GRUPO 3","XXX5","Tecnico B","06-Lun","T3",6],["GRUPO 3","XXX6","Tecnico B","06-Lun","T3",6],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","06-Lun","T1",6],["GRUPO 4","PEPITO PEREZ","Master","06-Lun","T1",6],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","06-Lun","T1",6],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","06-Lun","T1",6],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","06-Lun","T1",6],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","06-Lun","T1",6],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","06-Lun","T1",6],["GRUPO 4","JHONY CASTRO","Tecnico A","06-Lun","T1",6],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","06-Lun","T1",6],["GRUPO 4","XXX7","Tecnico B","06-Lun","T1",6],["GRUPO 4","XXX8","Tecnico B","06-Lun","T1",6],["GRUPO 4","XXX9","Tecnico B","06-Lun","T1",6],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","07-Mar","T1",7],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","07-Mar","T1",7],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","07-Mar","T1",7],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","07-Mar","T1",7],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","07-Mar","T1",7],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","07-Mar","T1",7],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","07-Mar","T1",7],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","07-Mar","T1",7],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","07-Mar","T1",7],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","07-Mar","T1",7],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","07-Mar","T1",7],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","07-Mar","T1",7],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","07-Mar","T2",7],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","07-Mar","T2",7],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","07-Mar","T2",7],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","07-Mar","T2",7],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","07-Mar","T2",7],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","07-Mar","T2",7],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","07-Mar","T2",7],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","07-Mar","T2",7],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","07-Mar","T2",7],["GRUPO 2","XXX1","Tecnico B","07-Mar","T2",7],["GRUPO 2","XXX2","Tecnico B","07-Mar","T2",7],["GRUPO 2","XXX3","Tecnico B","07-Mar","T2",7],["GRUPO 3","FONSECA RAY RICARDO","Master","07-Mar","T3",7],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","07-Mar","T3",7],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","07-Mar","T3",7],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","07-Mar","T3",7],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","07-Mar","T3",7],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","07-Mar","T3",7],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","07-Mar","T3",7],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","07-Mar","T3",7],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","07-Mar","T3",7],["GRUPO 3","XXX4","Tecnico B","07-Mar","T3",7],["GRUPO 3","XXX5","Tecnico B","07-Mar","T3",7],["GRUPO 3","XXX6","Tecnico B","07-Mar","T3",7],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","07-Mar","T1",7],["GRUPO 4","PEPITO PEREZ","Master","07-Mar","T1",7],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","07-Mar","T1",7],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","07-Mar","T1",7],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","07-Mar","T1",7],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","07-Mar","T1",7],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","07-Mar","T1",7],["GRUPO 4","JHONY CASTRO","Tecnico A","07-Mar","T1",7],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","07-Mar","T1",7],["GRUPO 4","XXX7","Tecnico B","07-Mar","T1",7],["GRUPO 4","XXX8","Tecnico B","07-Mar","T1",7],["GRUPO 4","XXX9","Tecnico B","07-Mar","T1",7],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","08-Mie","T1",8],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","08-Mie","T1",8],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","08-Mie","T1",8],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","08-Mie","T1",8],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","08-Mie","T1",8],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","08-Mie","T1",8],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","08-Mie","T1",8],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","08-Mie","T1",8],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","08-Mie","T1",8],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","08-Mie","T1",8],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","08-Mie","T1",8],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","08-Mie","T1",8],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","08-Mie","T2",8],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","08-Mie","T2",8],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","08-Mie","T2",8],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","08-Mie","T2",8],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","08-Mie","T2",8],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","08-Mie","T2",8],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","08-Mie","T2",8],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","08-Mie","T2",8],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","08-Mie","T2",8],["GRUPO 2","XXX1","Tecnico B","08-Mie","T2",8],["GRUPO 2","XXX2","Tecnico B","08-Mie","T2",8],["GRUPO 2","XXX3","Tecnico B","08-Mie","T2",8],["GRUPO 3","FONSECA RAY RICARDO","Master","08-Mie","T3",8],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","08-Mie","T3",8],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","08-Mie","T3",8],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","08-Mie","T3",8],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","08-Mie","T3",8],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","08-Mie","T3",8],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","08-Mie","T3",8],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","08-Mie","T3",8],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","08-Mie","T3",8],["GRUPO 3","XXX4","Tecnico B","08-Mie","T3",8],["GRUPO 3","XXX5","Tecnico B","08-Mie","T3",8],["GRUPO 3","XXX6","Tecnico B","08-Mie","T3",8],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","08-Mie","T1",8],["GRUPO 4","PEPITO PEREZ","Master","08-Mie","T1",8],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","08-Mie","T1",8],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","08-Mie","T1",8],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","08-Mie","T1",8],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","08-Mie","T1",8],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","08-Mie","T1",8],["GRUPO 4","JHONY CASTRO","Tecnico A","08-Mie","T1",8],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","08-Mie","T1",8],["GRUPO 4","XXX7","Tecnico B","08-Mie","T1",8],["GRUPO 4","XXX8","Tecnico B","08-Mie","T1",8],["GRUPO 4","XXX9","Tecnico B","08-Mie","T1",8],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","09-Jue","DESC. LEY",9],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","09-Jue","DESC. LEY",9],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","09-Jue","DESC. LEY",9],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","09-Jue","DESC. LEY",9],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","09-Jue","DESC. LEY",9],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","09-Jue","DESC. LEY",9],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","09-Jue","DESC. LEY",9],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","09-Jue","DESC. LEY",9],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","09-Jue","DESC. LEY",9],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","09-Jue","DESC. LEY",9],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","09-Jue","DESC. LEY",9],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","09-Jue","DESC. LEY",9],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","09-Jue","T2",9],["GRUPO 2","FLOREZ SAUCESO</t>
   </si>
   <si>
     <t>Mes Completo</t>

</xml_diff>

<commit_message>
Update historico_mallas.xlsx 2026-04-27 17:08:43.605251
</commit_message>
<xml_diff>
--- a/historico_mallas.xlsx
+++ b/historico_mallas.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="26">
   <si>
     <t>Mes</t>
   </si>
@@ -49,6 +49,9 @@
     <t>Abril</t>
   </si>
   <si>
+    <t>April</t>
+  </si>
+  <si>
     <t>Técnica</t>
   </si>
   <si>
@@ -67,6 +70,9 @@
     <t>27/04/2026 15:57</t>
   </si>
   <si>
+    <t>27/04/2026 17:08</t>
+  </si>
+  <si>
     <t>[{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"01-Mie","Final":"T2","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"01-Mie","Final":"T3","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"01-Mie","Final":"T1","n_dia":1},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"02-Jue","Final":"DESC. LEY","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"02-Jue","Final":"T2","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"02-Jue","Final":"T3","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"02-Jue","Final":"T1","n_dia":2},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"03-Vie","Final":"T1","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"03-Vie","Final":"DESC. LEY","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"03-Vie","Final":"T3","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"03-Vie","Final":"T2","n_dia":3},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"04-Sab","Final":"T1","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"04-Sab","Final":"T2","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"04-Sab","Final":"DESC. LEY","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"04-Sab","Final":"T3","n_dia":4},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"05-Dom","Final":"T1","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"05-Dom","Final":"T2","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"05-Dom","Final":"T3","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"RAMIREZ VARGAS MARCELA PAOLA","Cargo":"Tecnico A","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Cargo":"Tecnico A","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"TORO CISNEROS GARY JOSE","Cargo":"Tecnico A","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"USECHE CALDERON JADID ESTIVEN","Cargo":"Tecnico A","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"VASQUEZ NIETO CAMILO ANDRES","Cargo":"Tecnico A","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"JHONY CASTRO","Cargo":"Tecnico A","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"BERNAL JUAN DAVID","Cargo":"Tecnico A","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"XXX7","Cargo":"Tecnico B","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"XXX8","Cargo":"Tecnico B","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 4","Empleado":"XXX9","Cargo":"Tecnico B","Label":"05-Dom","Final":"DESC. LEY","n_dia":5},{"Grupo":"GRUPO 1","Empleado":"BARON HERNANDEZ HAROLD ANTONIO","Cargo":"Master","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"CASTELLANOS CARVAJAL DEYVITH FABIAN","Cargo":"Master","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"AROCA TORRES JULIAN EDUARDO","Cargo":"Tecnico A","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"BERMUDEZ PARRA JENNIFER XIOMARA","Cargo":"Tecnico A","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"BERNAL BAQUERO JAMES RICARDO","Cargo":"Tecnico A","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"BURGOS ORTIZ JOSE HORACIO","Cargo":"Tecnico A","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"CANTOR PORRAS JUAN FERNEY","Cargo":"Tecnico A","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"CAPERA CAPERA JOSE GABRIEL","Cargo":"Tecnico A","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"CARDENAS LOTERO RICARDO ANDR\u00c9S","Cargo":"Tecnico A","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"RENDON OSPINA NELSON LEANDRO","Cargo":"Tecnico B","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"SARMIENTO URBINA MOISES DANIEL","Cargo":"Tecnico B","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 1","Empleado":"VELASCO VELASCO SEBASTI\u00c1N DAVID","Cargo":"Tecnico B","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"DELGADO DELGADO JOHAN DARIO","Cargo":"Master","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"FLOREZ SAUCESO KENIS ALBERTO","Cargo":"Master","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"CARDONA GARCIA OSCAR JAVIER","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"CARVAJAL GARC\u00cdA HOVER MARCK","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"CEPEDA PIRAQUIVE JUAN DAVID","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"FAJARDO SAENZ OSCAR FERNANDO","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"FLOREZ ESPITIA RONY ALBERTO","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"GARCIA CUERVO EDWIN JAVIER","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"GONZALEZ OCHOA JUAN CARLOS","Cargo":"Tecnico A","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"XXX1","Cargo":"Tecnico B","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"XXX2","Cargo":"Tecnico B","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 2","Empleado":"XXX3","Cargo":"Tecnico B","Label":"06-Lun","Final":"T2","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"FONSECA RAY RICARDO","Cargo":"Master","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"GOMEZ BETANCUR JAIDER ANDRES","Cargo":"Master","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"GRANADA PATI\u00d1O CARLOS MARINO","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"GRASS PLATA MIGUEL SNEIDER","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"MANZANO CALVO JUAN SEBASTIAN","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"MENDOZA GOITA MARIANSEL ZENAYDA","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"MURILLO ARAQUE JAIVER GEOVANY","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"NI\u00d1O ARENAS HECTOR GONZALO","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"RAMIREZ CHAVERRA JHON EDISON","Cargo":"Tecnico A","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"XXX4","Cargo":"Tecnico B","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"XXX5","Cargo":"Tecnico B","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 3","Empleado":"XXX6","Cargo":"Tecnico B","Label":"06-Lun","Final":"T3","n_dia":6},{"Grupo":"GRUPO 4","Empleado":"RODRIGUEZ MOSQUERA LUIS FERNANDO","Cargo":"Master","Label":"06-Lun","Final":"T1","n_dia":6},{"Grupo":"GRUPO 4","Empleado":"PEPITO PEREZ","Cargo":"Master</t>
   </si>
   <si>
@@ -80,6 +86,9 @@
   </si>
   <si>
     <t>{"columns":["Grupo","Empleado","Cargo","Label","Final","n_dia"],"index":[0,1,2,3,4,5,6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23,24,25,26,27,28,29,30,31,32,33,34,35,36,37,38,39,40,41,42,43,44,45,46,47,48,49,50,51,52,53,54,55,56,57,58,59,60,61,62,63,64,65,66,67,68,69,70,71,72,73,74,75,76,77,78,79,80,81,82,83,84,85,86,87,88,89,90,91,92,93,94,95,96,97,98,99,100,101,102,103,104,105,106,107,108,109,110,111,112,113,114,115,116,117,118,119,120,121,122,123,124,125,126,127,128,129,130,131,132,133,134,135,136,137,138,139,140,141,142,143,144,145,146,147,148,149,150,151,152,153,154,155,156,157,158,159,160,161,162,163,164,165,166,167,168,169,170,171,172,173,174,175,176,177,178,179,180,181,182,183,184,185,186,187,188,189,190,191,192,193,194,195,196,197,198,199,200,201,202,203,204,205,206,207,208,209,210,211,212,213,214,215,216,217,218,219,220,221,222,223,224,225,226,227,228,229,230,231,232,233,234,235,236,237,238,239,240,241,242,243,244,245,246,247,248,249,250,251,252,253,254,255,256,257,258,259,260,261,262,263,264,265,266,267,268,269,270,271,272,273,274,275,276,277,278,279,280,281,282,283,284,285,286,287,288,289,290,291,292,293,294,295,296,297,298,299,300,301,302,303,304,305,306,307,308,309,310,311,312,313,314,315,316,317,318,319,320,321,322,323,324,325,326,327,328,329,330,331,332,333,334,335,336,337,338,339,340,341,342,343,344,345,346,347,348,349,350,351,352,353,354,355,356,357,358,359,360,361,362,363,364,365,366,367,368,369,370,371,372,373,374,375,376,377,378,379,380,381,382,383,384,385,386,387,388,389,390,391,392,393,394,395,396,397,398,399,400,401,402,403,404,405,406,407,408,409,410,411,412,413,414,415,416,417,418,419,420,421,422,423,424,425,426,427,428,429,430,431,432,433,434,435,436,437,438,439,440,441,442,443,444,445,446,447,448,449,450,451,452,453,454,455,456,457,458,459,460,461,462,463,464,465,466,467,468,469,470,471,472,473,474,475,476,477,478,479,480,481,482,483,484,485,486,487,488,489,490,491,492,493,494,495,496,497,498,499,500,501,502,503,504,505,506,507,508,509,510,511,512,513,514,515,516,517,518,519,520,521,522,523,524,525,526,527,528,529,530,531,532,533,534,535,536,537,538,539,540,541,542,543,544,545,546,547,548,549,550,551,552,553,554,555,556,557,558,559,560,561,562,563,564,565,566,567,568,569,570,571,572,573,574,575,576,577,578,579,580,581,582,583,584,585,586,587,588,589,590,591,592,593,594,595,596,597,598,599,600,601,602,603,604,605,606,607,608,609,610,611,612,613,614,615,616,617,618,619,620,621,622,623,624,625,626,627,628,629,630,631,632,633,634,635,636,637,638,639,640,641,642,643,644,645,646,647,648,649,650,651,652,653,654,655,656,657,658,659,660,661,662,663,664,665,666,667,668,669,670,671,672,673,674,675,676,677,678,679,680,681,682,683,684,685,686,687,688,689,690,691,692,693,694,695,696,697,698,699,700,701,702,703,704,705,706,707,708,709,710,711,712,713,714,715,716,717,718,719,720,721,722,723,724,725,726,727,728,729,730,731,732,733,734,735,736,737,738,739,740,741,742,743,744,745,746,747,748,749,750,751,752,753,754,755,756,757,758,759,760,761,762,763,764,765,766,767,768,769,770,771,772,773,774,775,776,777,778,779,780,781,782,783,784,785,786,787,788,789,790,791,792,793,794,795,796,797,798,799,800,801,802,803,804,805,806,807,808,809,810,811,812,813,814,815,816,817,818,819,820,821,822,823,824,825,826,827,828,829,830,831,832,833,834,835,836,837,838,839,840,841,842,843,844,845,846,847,848,849,850,851,852,853,854,855,856,857,858,859,860,861,862,863,864,865,866,867,868,869,870,871,872,873,874,875,876,877,878,879,880,881,882,883,884,885,886,887,888,889,890,891,892,893,894,895,896,897,898,899,900,901,902,903,904,905,906,907,908,909,910,911,912,913,914,915,916,917,918,919,920,921,922,923,924,925,926,927,928,929,930,931,932,933,934,935,936,937,938,939,940,941,942,943,944,945,946,947,948,949,950,951,952,953,954,955,956,957,958,959,960,961,962,963,964,965,966,967,968,969,970,971,972,973,974,975,976,977,978,979,980,981,982,983,984,985,986,987,988,989,990,991,992,993,994,995,996,997,998,999,1000,1001,1002,1003,1004,1005,1006,1007,1008,1009,1010,1011,1012,1013,1014,1015,1016,1017,1018,1019,1020,1021,1022,1023,1024,1025,1026,1027,1028,1029,1030,1031,1032,1033,1034,1035,1036,1037,1038,1039,1040,1041,1042,1043,1044,1045,1046,1047,1048,1049,1050,1051,1052,1053,1054,1055,1056,1057,1058,1059,1060,1061,1062,1063,1064,1065,1066,1067,1068,1069,1070,1071,1072,1073,1074,1075,1076,1077,1078,1079,1080,1081,1082,1083,1084,1085,1086,1087,1088,1089,1090,1091,1092,1093,1094,1095,1096,1097,1098,1099,1100,1101,1102,1103,1104,1105,1106,1107,1108,1109,1110,1111,1112,1113,1114,1115,1116,1117,1118,1119,1120,1121,1122,1123,1124,1125,1126,1127,1128,1129,1130,1131,1132,1133,1134,1135,1136,1137,1138,1139,1140,1141,1142,1143,1144,1145,1146,1147,1148,1149,1150,1151,1152,1153,1154,1155,1156,1157,1158,1159,1160,1161,1162,1163,1164,1165,1166,1167,1168,1169,1170,1171,1172,1173,1174,1175,1176,1177,1178,1179,1180,1181,1182,1183,1184,1185,1186,1187,1188,1189,1190,1191,1192,1193,1194,1195,1196,1197,1198,1199,1200,1201,1202,1203,1204,1205,1206,1207,1208,1209,1210,1211,1212,1213,1214,1215,1216,1217,1218,1219,1220,1221,1222,1223,1224,1225,1226,1227,1228,1229,1230,1231,1232,1233,1234,1235,1236,1237,1238,1239,1240,1241,1242,1243,1244,1245,1246,1247,1248,1249,1250,1251,1252,1253,1254,1255,1256,1257,1258,1259,1260,1261,1262,1263,1264,1265,1266,1267,1268,1269,1270,1271,1272,1273,1274,1275,1276,1277,1278,1279,1280,1281,1282,1283,1284,1285,1286,1287,1288,1289,1290,1291,1292,1293,1294,1295,1296,1297,1298,1299,1300,1301,1302,1303,1304,1305,1306,1307,1308,1309,1310,1311,1312,1313,1314,1315,1316,1317,1318,1319,1320,1321,1322,1323,1324,1325,1326,1327,1328,1329,1330,1331,1332,1333,1334,1335,1336,1337,1338,1339,1340,1341,1342,1343,1344,1345,1346,1347,1348,1349,1350,1351,1352,1353,1354,1355,1356,1357,1358,1359,1360,1361,1362,1363,1364,1365,1366,1367,1368,1369,1370,1371,1372,1373,1374,1375,1376,1377,1378,1379,1380,1381,1382,1383,1384,1385,1386,1387,1388,1389,1390,1391,1392,1393,1394,1395,1396,1397,1398,1399,1400,1401,1402,1403,1404,1405,1406,1407,1408,1409,1410,1411,1412,1413,1414,1415,1416,1417,1418,1419,1420,1421,1422,1423,1424,1425,1426,1427,1428,1429,1430,1431,1432,1433,1434,1435,1436,1437,1438,1439],"data":[["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","01-Mie","T1",1],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","01-Mie","T1",1],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","01-Mie","T1",1],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","01-Mie","T1",1],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","01-Mie","T1",1],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","01-Mie","T1",1],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","01-Mie","T1",1],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","01-Mie","T1",1],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","01-Mie","T1",1],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","01-Mie","T1",1],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","01-Mie","T1",1],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","01-Mie","T1",1],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","01-Mie","T2",1],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","01-Mie","T2",1],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","01-Mie","T2",1],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","01-Mie","T2",1],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","01-Mie","T2",1],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","01-Mie","T2",1],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","01-Mie","T2",1],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","01-Mie","T2",1],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","01-Mie","T2",1],["GRUPO 2","XXX1","Tecnico B","01-Mie","T2",1],["GRUPO 2","XXX2","Tecnico B","01-Mie","T2",1],["GRUPO 2","XXX3","Tecnico B","01-Mie","T2",1],["GRUPO 3","FONSECA RAY RICARDO","Master","01-Mie","T3",1],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","01-Mie","T3",1],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","01-Mie","T3",1],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","01-Mie","T3",1],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","01-Mie","T3",1],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","01-Mie","T3",1],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","01-Mie","T3",1],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","01-Mie","T3",1],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","01-Mie","T3",1],["GRUPO 3","XXX4","Tecnico B","01-Mie","T3",1],["GRUPO 3","XXX5","Tecnico B","01-Mie","T3",1],["GRUPO 3","XXX6","Tecnico B","01-Mie","T3",1],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","01-Mie","T1",1],["GRUPO 4","PEPITO PEREZ","Master","01-Mie","T1",1],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","01-Mie","T1",1],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","01-Mie","T1",1],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","01-Mie","T1",1],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","01-Mie","T1",1],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","01-Mie","T1",1],["GRUPO 4","JHONY CASTRO","Tecnico A","01-Mie","T1",1],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","01-Mie","T1",1],["GRUPO 4","XXX7","Tecnico B","01-Mie","T1",1],["GRUPO 4","XXX8","Tecnico B","01-Mie","T1",1],["GRUPO 4","XXX9","Tecnico B","01-Mie","T1",1],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","02-Jue","DESC. LEY",2],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","02-Jue","DESC. LEY",2],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","02-Jue","DESC. LEY",2],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","02-Jue","DESC. LEY",2],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","02-Jue","DESC. LEY",2],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","02-Jue","DESC. LEY",2],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","02-Jue","DESC. LEY",2],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","02-Jue","DESC. LEY",2],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","02-Jue","DESC. LEY",2],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","02-Jue","DESC. LEY",2],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","02-Jue","DESC. LEY",2],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","02-Jue","DESC. LEY",2],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","02-Jue","T2",2],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","02-Jue","T2",2],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","02-Jue","T2",2],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","02-Jue","T2",2],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","02-Jue","T2",2],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","02-Jue","T2",2],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","02-Jue","T2",2],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","02-Jue","T2",2],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","02-Jue","T2",2],["GRUPO 2","XXX1","Tecnico B","02-Jue","T2",2],["GRUPO 2","XXX2","Tecnico B","02-Jue","T2",2],["GRUPO 2","XXX3","Tecnico B","02-Jue","T2",2],["GRUPO 3","FONSECA RAY RICARDO","Master","02-Jue","T3",2],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","02-Jue","T3",2],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","02-Jue","T3",2],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","02-Jue","T3",2],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","02-Jue","T3",2],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","02-Jue","T3",2],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","02-Jue","T3",2],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","02-Jue","T3",2],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","02-Jue","T3",2],["GRUPO 3","XXX4","Tecnico B","02-Jue","T3",2],["GRUPO 3","XXX5","Tecnico B","02-Jue","T3",2],["GRUPO 3","XXX6","Tecnico B","02-Jue","T3",2],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","02-Jue","T1",2],["GRUPO 4","PEPITO PEREZ","Master","02-Jue","T1",2],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","02-Jue","T1",2],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","02-Jue","T1",2],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","02-Jue","T1",2],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","02-Jue","T1",2],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","02-Jue","T1",2],["GRUPO 4","JHONY CASTRO","Tecnico A","02-Jue","T1",2],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","02-Jue","T1",2],["GRUPO 4","XXX7","Tecnico B","02-Jue","T1",2],["GRUPO 4","XXX8","Tecnico B","02-Jue","T1",2],["GRUPO 4","XXX9","Tecnico B","02-Jue","T1",2],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","03-Vie","T1",3],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","03-Vie","T1",3],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","03-Vie","T1",3],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","03-Vie","T1",3],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","03-Vie","T1",3],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","03-Vie","T1",3],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","03-Vie","T1",3],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","03-Vie","T1",3],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","03-Vie","T1",3],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","03-Vie","T1",3],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","03-Vie","T1",3],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","03-Vie","T1",3],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","03-Vie","DESC. LEY",3],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","03-Vie","DESC. LEY",3],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","03-Vie","DESC. LEY",3],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","03-Vie","DESC. LEY",3],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","03-Vie","DESC. LEY",3],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","03-Vie","DESC. LEY",3],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","03-Vie","DESC. LEY",3],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","03-Vie","DESC. LEY",3],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","03-Vie","DESC. LEY",3],["GRUPO 2","XXX1","Tecnico B","03-Vie","DESC. LEY",3],["GRUPO 2","XXX2","Tecnico B","03-Vie","DESC. LEY",3],["GRUPO 2","XXX3","Tecnico B","03-Vie","DESC. LEY",3],["GRUPO 3","FONSECA RAY RICARDO","Master","03-Vie","T3",3],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","03-Vie","T3",3],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","03-Vie","T3",3],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","03-Vie","T3",3],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","03-Vie","T3",3],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","03-Vie","T3",3],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","03-Vie","T3",3],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","03-Vie","T3",3],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","03-Vie","T3",3],["GRUPO 3","XXX4","Tecnico B","03-Vie","T3",3],["GRUPO 3","XXX5","Tecnico B","03-Vie","T3",3],["GRUPO 3","XXX6","Tecnico B","03-Vie","T3",3],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","03-Vie","T2",3],["GRUPO 4","PEPITO PEREZ","Master","03-Vie","T2",3],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","03-Vie","T2",3],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","03-Vie","T2",3],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","03-Vie","T2",3],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","03-Vie","T2",3],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","03-Vie","T2",3],["GRUPO 4","JHONY CASTRO","Tecnico A","03-Vie","T2",3],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","03-Vie","T2",3],["GRUPO 4","XXX7","Tecnico B","03-Vie","T2",3],["GRUPO 4","XXX8","Tecnico B","03-Vie","T2",3],["GRUPO 4","XXX9","Tecnico B","03-Vie","T2",3],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","04-Sab","T1",4],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","04-Sab","T1",4],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","04-Sab","T1",4],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","04-Sab","T1",4],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","04-Sab","T1",4],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","04-Sab","T1",4],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","04-Sab","T1",4],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","04-Sab","T1",4],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","04-Sab","T1",4],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","04-Sab","T1",4],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","04-Sab","T1",4],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","04-Sab","T1",4],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","04-Sab","T2",4],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","04-Sab","T2",4],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","04-Sab","T2",4],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","04-Sab","T2",4],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","04-Sab","T2",4],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","04-Sab","T2",4],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","04-Sab","T2",4],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","04-Sab","T2",4],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","04-Sab","T2",4],["GRUPO 2","XXX1","Tecnico B","04-Sab","T2",4],["GRUPO 2","XXX2","Tecnico B","04-Sab","T2",4],["GRUPO 2","XXX3","Tecnico B","04-Sab","T2",4],["GRUPO 3","FONSECA RAY RICARDO","Master","04-Sab","DESC. LEY",4],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","04-Sab","DESC. LEY",4],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","04-Sab","DESC. LEY",4],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","04-Sab","DESC. LEY",4],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","04-Sab","DESC. LEY",4],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","04-Sab","DESC. LEY",4],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","04-Sab","DESC. LEY",4],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","04-Sab","DESC. LEY",4],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","04-Sab","DESC. LEY",4],["GRUPO 3","XXX4","Tecnico B","04-Sab","DESC. LEY",4],["GRUPO 3","XXX5","Tecnico B","04-Sab","DESC. LEY",4],["GRUPO 3","XXX6","Tecnico B","04-Sab","DESC. LEY",4],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","04-Sab","T3",4],["GRUPO 4","PEPITO PEREZ","Master","04-Sab","T3",4],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","04-Sab","T3",4],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","04-Sab","T3",4],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","04-Sab","T3",4],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","04-Sab","T3",4],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","04-Sab","T3",4],["GRUPO 4","JHONY CASTRO","Tecnico A","04-Sab","T3",4],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","04-Sab","T3",4],["GRUPO 4","XXX7","Tecnico B","04-Sab","T3",4],["GRUPO 4","XXX8","Tecnico B","04-Sab","T3",4],["GRUPO 4","XXX9","Tecnico B","04-Sab","T3",4],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","05-Dom","T1",5],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","05-Dom","T1",5],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","05-Dom","T1",5],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","05-Dom","T1",5],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","05-Dom","T1",5],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","05-Dom","T1",5],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","05-Dom","T1",5],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","05-Dom","T1",5],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","05-Dom","T1",5],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","05-Dom","T1",5],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","05-Dom","T1",5],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","05-Dom","T1",5],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","05-Dom","T2",5],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","05-Dom","T2",5],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","05-Dom","T2",5],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","05-Dom","T2",5],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","05-Dom","T2",5],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","05-Dom","T2",5],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","05-Dom","T2",5],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","05-Dom","T2",5],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","05-Dom","T2",5],["GRUPO 2","XXX1","Tecnico B","05-Dom","T2",5],["GRUPO 2","XXX2","Tecnico B","05-Dom","T2",5],["GRUPO 2","XXX3","Tecnico B","05-Dom","T2",5],["GRUPO 3","FONSECA RAY RICARDO","Master","05-Dom","T3",5],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","05-Dom","T3",5],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","05-Dom","T3",5],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","05-Dom","T3",5],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","05-Dom","T3",5],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","05-Dom","T3",5],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","05-Dom","T3",5],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","05-Dom","T3",5],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","05-Dom","T3",5],["GRUPO 3","XXX4","Tecnico B","05-Dom","T3",5],["GRUPO 3","XXX5","Tecnico B","05-Dom","T3",5],["GRUPO 3","XXX6","Tecnico B","05-Dom","T3",5],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","05-Dom","DESC. LEY",5],["GRUPO 4","PEPITO PEREZ","Master","05-Dom","DESC. LEY",5],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","05-Dom","DESC. LEY",5],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","05-Dom","DESC. LEY",5],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","05-Dom","DESC. LEY",5],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","05-Dom","DESC. LEY",5],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","05-Dom","DESC. LEY",5],["GRUPO 4","JHONY CASTRO","Tecnico A","05-Dom","DESC. LEY",5],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","05-Dom","DESC. LEY",5],["GRUPO 4","XXX7","Tecnico B","05-Dom","DESC. LEY",5],["GRUPO 4","XXX8","Tecnico B","05-Dom","DESC. LEY",5],["GRUPO 4","XXX9","Tecnico B","05-Dom","DESC. LEY",5],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","06-Lun","T1",6],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","06-Lun","T1",6],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","06-Lun","T1",6],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","06-Lun","T1",6],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","06-Lun","T1",6],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","06-Lun","T1",6],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","06-Lun","T1",6],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","06-Lun","T1",6],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","06-Lun","T1",6],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","06-Lun","T1",6],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","06-Lun","T1",6],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","06-Lun","T1",6],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","06-Lun","T2",6],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","06-Lun","T2",6],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","06-Lun","T2",6],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","06-Lun","T2",6],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","06-Lun","T2",6],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","06-Lun","T2",6],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","06-Lun","T2",6],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","06-Lun","T2",6],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","06-Lun","T2",6],["GRUPO 2","XXX1","Tecnico B","06-Lun","T2",6],["GRUPO 2","XXX2","Tecnico B","06-Lun","T2",6],["GRUPO 2","XXX3","Tecnico B","06-Lun","T2",6],["GRUPO 3","FONSECA RAY RICARDO","Master","06-Lun","T3",6],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","06-Lun","T3",6],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","06-Lun","T3",6],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","06-Lun","T3",6],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","06-Lun","T3",6],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","06-Lun","T3",6],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","06-Lun","T3",6],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","06-Lun","T3",6],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","06-Lun","T3",6],["GRUPO 3","XXX4","Tecnico B","06-Lun","T3",6],["GRUPO 3","XXX5","Tecnico B","06-Lun","T3",6],["GRUPO 3","XXX6","Tecnico B","06-Lun","T3",6],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","06-Lun","T1",6],["GRUPO 4","PEPITO PEREZ","Master","06-Lun","T1",6],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","06-Lun","T1",6],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","06-Lun","T1",6],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","06-Lun","T1",6],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","06-Lun","T1",6],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","06-Lun","T1",6],["GRUPO 4","JHONY CASTRO","Tecnico A","06-Lun","T1",6],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","06-Lun","T1",6],["GRUPO 4","XXX7","Tecnico B","06-Lun","T1",6],["GRUPO 4","XXX8","Tecnico B","06-Lun","T1",6],["GRUPO 4","XXX9","Tecnico B","06-Lun","T1",6],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","07-Mar","T1",7],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","07-Mar","T1",7],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","07-Mar","T1",7],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","07-Mar","T1",7],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","07-Mar","T1",7],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","07-Mar","T1",7],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","07-Mar","T1",7],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","07-Mar","T1",7],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","07-Mar","T1",7],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","07-Mar","T1",7],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","07-Mar","T1",7],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","07-Mar","T1",7],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","07-Mar","T2",7],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","07-Mar","T2",7],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","07-Mar","T2",7],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","07-Mar","T2",7],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","07-Mar","T2",7],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","07-Mar","T2",7],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","07-Mar","T2",7],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","07-Mar","T2",7],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","07-Mar","T2",7],["GRUPO 2","XXX1","Tecnico B","07-Mar","T2",7],["GRUPO 2","XXX2","Tecnico B","07-Mar","T2",7],["GRUPO 2","XXX3","Tecnico B","07-Mar","T2",7],["GRUPO 3","FONSECA RAY RICARDO","Master","07-Mar","T3",7],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","07-Mar","T3",7],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","07-Mar","T3",7],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","07-Mar","T3",7],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","07-Mar","T3",7],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","07-Mar","T3",7],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","07-Mar","T3",7],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","07-Mar","T3",7],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","07-Mar","T3",7],["GRUPO 3","XXX4","Tecnico B","07-Mar","T3",7],["GRUPO 3","XXX5","Tecnico B","07-Mar","T3",7],["GRUPO 3","XXX6","Tecnico B","07-Mar","T3",7],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","07-Mar","T1",7],["GRUPO 4","PEPITO PEREZ","Master","07-Mar","T1",7],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","07-Mar","T1",7],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","07-Mar","T1",7],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","07-Mar","T1",7],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","07-Mar","T1",7],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","07-Mar","T1",7],["GRUPO 4","JHONY CASTRO","Tecnico A","07-Mar","T1",7],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","07-Mar","T1",7],["GRUPO 4","XXX7","Tecnico B","07-Mar","T1",7],["GRUPO 4","XXX8","Tecnico B","07-Mar","T1",7],["GRUPO 4","XXX9","Tecnico B","07-Mar","T1",7],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","08-Mie","T1",8],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","08-Mie","T1",8],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","08-Mie","T1",8],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","08-Mie","T1",8],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","08-Mie","T1",8],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","08-Mie","T1",8],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","08-Mie","T1",8],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","08-Mie","T1",8],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","08-Mie","T1",8],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","08-Mie","T1",8],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","08-Mie","T1",8],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","08-Mie","T1",8],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","08-Mie","T2",8],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","08-Mie","T2",8],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","08-Mie","T2",8],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","08-Mie","T2",8],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","08-Mie","T2",8],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","08-Mie","T2",8],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","08-Mie","T2",8],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","08-Mie","T2",8],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","08-Mie","T2",8],["GRUPO 2","XXX1","Tecnico B","08-Mie","T2",8],["GRUPO 2","XXX2","Tecnico B","08-Mie","T2",8],["GRUPO 2","XXX3","Tecnico B","08-Mie","T2",8],["GRUPO 3","FONSECA RAY RICARDO","Master","08-Mie","T3",8],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","08-Mie","T3",8],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","08-Mie","T3",8],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","08-Mie","T3",8],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","08-Mie","T3",8],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","08-Mie","T3",8],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","08-Mie","T3",8],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","08-Mie","T3",8],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","08-Mie","T3",8],["GRUPO 3","XXX4","Tecnico B","08-Mie","T3",8],["GRUPO 3","XXX5","Tecnico B","08-Mie","T3",8],["GRUPO 3","XXX6","Tecnico B","08-Mie","T3",8],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","08-Mie","T1",8],["GRUPO 4","PEPITO PEREZ","Master","08-Mie","T1",8],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","08-Mie","T1",8],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","08-Mie","T1",8],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","08-Mie","T1",8],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","08-Mie","T1",8],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","08-Mie","T1",8],["GRUPO 4","JHONY CASTRO","Tecnico A","08-Mie","T1",8],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","08-Mie","T1",8],["GRUPO 4","XXX7","Tecnico B","08-Mie","T1",8],["GRUPO 4","XXX8","Tecnico B","08-Mie","T1",8],["GRUPO 4","XXX9","Tecnico B","08-Mie","T1",8],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","09-Jue","DESC. LEY",9],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","09-Jue","DESC. LEY",9],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","09-Jue","DESC. LEY",9],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","09-Jue","DESC. LEY",9],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","09-Jue","DESC. LEY",9],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","09-Jue","DESC. LEY",9],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","09-Jue","DESC. LEY",9],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","09-Jue","DESC. LEY",9],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","09-Jue","DESC. LEY",9],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","09-Jue","DESC. LEY",9],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","09-Jue","DESC. LEY",9],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","09-Jue","DESC. LEY",9],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","09-Jue","T2",9],["GRUPO 2","FLOREZ SAUCESO</t>
+  </si>
+  <si>
+    <t>{"columns":["Grupo","Empleado","Cargo","Horario","Label","Final","n_dia","Fecha_DT"],"index":[0,1,2,3,4,5,6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23,24,25,26,27,28,29,30,31,32,33,34,35,36,37,38,39,40,41,42,43,44,45,46,47,48,49,50,51,52,53,54,55,56,57,58,59,60,61,62,63,64,65,66,67,68,69,70,71,72,73,74,75,76,77,78,79,80,81,82,83,84,85,86,87,88,89,90,91,92,93,94,95,96,97,98,99,100,101,102,103,104,105,106,107,108,109,110,111,112,113,114,115,116,117,118,119,120,121,122,123,124,125,126,127,128,129,130,131,132,133,134,135,136,137,138,139,140,141,142,143,144,145,146,147,148,149,150,151,152,153,154,155,156,157,158,159,160,161,162,163,164,165,166,167,168,169,170,171,172,173,174,175,176,177,178,179,180,181,182,183,184,185,186,187,188,189,190,191,192,193,194,195,196,197,198,199,200,201,202,203,204,205,206,207,208,209,210,211,212,213,214,215,216,217,218,219,220,221,222,223,224,225,226,227,228,229,230,231,232,233,234,235,236,237,238,239,240,241,242,243,244,245,246,247,248,249,250,251,252,253,254,255,256,257,258,259,260,261,262,263,264,265,266,267,268,269,270,271,272,273,274,275,276,277,278,279,280,281,282,283,284,285,286,287,288,289,290,291,292,293,294,295,296,297,298,299,300,301,302,303,304,305,306,307,308,309,310,311,312,313,314,315,316,317,318,319,320,321,322,323,324,325,326,327,328,329,330,331,332,333,334,335,336,337,338,339,340,341,342,343,344,345,346,347,348,349,350,351,352,353,354,355,356,357,358,359,360,361,362,363,364,365,366,367,368,369,370,371,372,373,374,375,376,377,378,379,380,381,382,383,384,385,386,387,388,389,390,391,392,393,394,395,396,397,398,399,400,401,402,403,404,405,406,407,408,409,410,411,412,413,414,415,416,417,418,419,420,421,422,423,424,425,426,427,428,429,430,431,432,433,434,435,436,437,438,439,440,441,442,443,444,445,446,447,448,449,450,451,452,453,454,455,456,457,458,459,460,461,462,463,464,465,466,467,468,469,470,471,472,473,474,475,476,477,478,479,480,481,482,483,484,485,486,487,488,489,490,491,492,493,494,495,496,497,498,499,500,501,502,503,504,505,506,507,508,509,510,511,512,513,514,515,516,517,518,519,520,521,522,523,524,525,526,527,528,529,530,531,532,533,534,535,536,537,538,539,540,541,542,543,544,545,546,547,548,549,550,551,552,553,554,555,556,557,558,559,560,561,562,563,564,565,566,567,568,569,570,571,572,573,574,575,576,577,578,579,580,581,582,583,584,585,586,587,588,589,590,591,592,593,594,595,596,597,598,599,600,601,602,603,604,605,606,607,608,609,610,611,612,613,614,615,616,617,618,619,620,621,622,623,624,625,626,627,628,629,630,631,632,633,634,635,636,637,638,639,640,641,642,643,644,645,646,647,648,649,650,651,652,653,654,655,656,657,658,659,660,661,662,663,664,665,666,667,668,669,670,671,672,673,674,675,676,677,678,679,680,681,682,683,684,685,686,687,688,689,690,691,692,693,694,695,696,697,698,699,700,701,702,703,704,705,706,707,708,709,710,711,712,713,714,715,716,717,718,719,720,721,722,723,724,725,726,727,728,729,730,731,732,733,734,735,736,737,738,739,740,741,742,743,744,745,746,747,748,749,750,751,752,753,754,755,756,757,758,759,760,761,762,763,764,765,766,767,768,769,770,771,772,773,774,775,776,777,778,779,780,781,782,783,784,785,786,787,788,789,790,791,792,793,794,795,796,797,798,799,800,801,802,803,804,805,806,807,808,809,810,811,812,813,814,815,816,817,818,819,820,821,822,823,824,825,826,827,828,829,830,831,832,833,834,835,836,837,838,839,840,841,842,843,844,845,846,847,848,849,850,851,852,853,854,855,856,857,858,859,860,861,862,863,864,865,866,867,868,869,870,871,872,873,874,875,876,877,878,879,880,881,882,883,884,885,886,887,888,889,890,891,892,893,894,895,896,897,898,899,900,901,902,903,904,905,906,907,908,909,910,911,912,913,914,915,916,917,918,919,920,921,922,923,924,925,926,927,928,929,930,931,932,933,934,935,936,937,938,939,940,941,942,943,944,945,946,947,948,949,950,951,952,953,954,955,956,957,958,959,960,961,962,963,964,965,966,967,968,969,970,971,972,973,974,975,976,977,978,979,980,981,982,983,984,985,986,987,988,989,990,991,992,993,994,995,996,997,998,999,1000,1001,1002,1003,1004,1005,1006,1007,1008,1009,1010,1011,1012,1013,1014,1015,1016,1017,1018,1019,1020,1021,1022,1023,1024,1025,1026,1027,1028,1029,1030,1031,1032,1033,1034,1035,1036,1037,1038,1039,1040,1041,1042,1043,1044,1045,1046,1047,1048,1049,1050,1051,1052,1053,1054,1055,1056,1057,1058,1059,1060,1061,1062,1063,1064,1065,1066,1067,1068,1069,1070,1071,1072,1073,1074,1075,1076,1077,1078,1079,1080,1081,1082,1083,1084,1085,1086,1087,1088,1089,1090,1091,1092,1093,1094,1095,1096,1097,1098,1099,1100,1101,1102,1103,1104,1105,1106,1107,1108,1109,1110,1111,1112,1113,1114,1115,1116,1117,1118,1119,1120,1121,1122,1123,1124,1125,1126,1127,1128,1129,1130,1131,1132,1133,1134,1135,1136,1137,1138,1139,1140,1141,1142,1143,1144,1145,1146,1147,1148,1149,1150,1151,1152,1153,1154,1155,1156,1157,1158,1159,1160,1161,1162,1163,1164,1165,1166,1167,1168,1169,1170,1171,1172,1173,1174,1175,1176,1177,1178,1179,1180,1181,1182,1183,1184,1185,1186,1187,1188,1189,1190,1191,1192,1193,1194,1195,1196,1197,1198,1199,1200,1201,1202,1203,1204,1205,1206,1207,1208,1209,1210,1211,1212,1213,1214,1215,1216,1217,1218,1219,1220,1221,1222,1223,1224,1225,1226,1227,1228,1229,1230,1231,1232,1233,1234,1235,1236,1237,1238,1239,1240,1241,1242,1243,1244,1245,1246,1247,1248,1249,1250,1251,1252,1253,1254,1255,1256,1257,1258,1259,1260,1261,1262,1263,1264,1265,1266,1267,1268,1269,1270,1271,1272,1273,1274,1275,1276,1277,1278,1279,1280,1281,1282,1283,1284,1285,1286,1287,1288,1289,1290,1291,1292,1293,1294,1295,1296,1297,1298,1299,1300,1301,1302,1303,1304,1305,1306,1307,1308,1309,1310,1311,1312,1313,1314,1315,1316,1317,1318,1319,1320,1321,1322,1323,1324,1325,1326,1327,1328,1329,1330,1331,1332,1333,1334,1335,1336,1337,1338,1339,1340,1341,1342,1343,1344,1345,1346,1347,1348,1349,1350,1351,1352,1353,1354,1355,1356,1357,1358,1359,1360,1361,1362,1363,1364,1365,1366,1367,1368,1369,1370,1371,1372,1373,1374,1375,1376,1377,1378,1379,1380,1381,1382,1383,1384,1385,1386,1387,1388,1389,1390,1391,1392,1393,1394,1395,1396,1397,1398,1399,1400,1401,1402,1403,1404,1405,1406,1407,1408,1409,1410,1411,1412,1413,1414,1415,1416,1417,1418,1419,1420,1421,1422,1423,1424,1425,1426,1427,1428,1429,1430,1431,1432,1433,1434,1435,1436,1437,1438,1439],"data":[["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","06:00 - 14:00","01-Mie","T1",1,1775001600000],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","06:00 - 14:00","01-Mie","T1",1,1775001600000],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","06:00 - 14:00","01-Mie","T1",1,1775001600000],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","06:00 - 14:00","01-Mie","T1",1,1775001600000],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","06:00 - 14:00","01-Mie","T1",1,1775001600000],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","06:00 - 14:00","01-Mie","T1",1,1775001600000],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","06:00 - 14:00","01-Mie","T1",1,1775001600000],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","06:00 - 14:00","01-Mie","T1",1,1775001600000],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","06:00 - 14:00","01-Mie","T1",1,1775001600000],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","06:00 - 14:00","01-Mie","T1",1,1775001600000],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","06:00 - 14:00","01-Mie","T1",1,1775001600000],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","06:00 - 14:00","01-Mie","T1",1,1775001600000],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","14:00 - 22:00","01-Mie","T2",1,1775001600000],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","14:00 - 22:00","01-Mie","T2",1,1775001600000],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","14:00 - 22:00","01-Mie","T2",1,1775001600000],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","14:00 - 22:00","01-Mie","T2",1,1775001600000],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","14:00 - 22:00","01-Mie","T2",1,1775001600000],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","14:00 - 22:00","01-Mie","T2",1,1775001600000],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","14:00 - 22:00","01-Mie","T2",1,1775001600000],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","14:00 - 22:00","01-Mie","T2",1,1775001600000],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","14:00 - 22:00","01-Mie","T2",1,1775001600000],["GRUPO 2","XXX1","Tecnico B","14:00 - 22:00","01-Mie","T2",1,1775001600000],["GRUPO 2","XXX2","Tecnico B","14:00 - 22:00","01-Mie","T2",1,1775001600000],["GRUPO 2","XXX3","Tecnico B","14:00 - 22:00","01-Mie","T2",1,1775001600000],["GRUPO 3","FONSECA RAY RICARDO","Master","22:00 - 06:00","01-Mie","T3",1,1775001600000],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","22:00 - 06:00","01-Mie","T3",1,1775001600000],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","22:00 - 06:00","01-Mie","T3",1,1775001600000],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","22:00 - 06:00","01-Mie","T3",1,1775001600000],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","22:00 - 06:00","01-Mie","T3",1,1775001600000],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","22:00 - 06:00","01-Mie","T3",1,1775001600000],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","22:00 - 06:00","01-Mie","T3",1,1775001600000],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","22:00 - 06:00","01-Mie","T3",1,1775001600000],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","22:00 - 06:00","01-Mie","T3",1,1775001600000],["GRUPO 3","XXX4","Tecnico B","22:00 - 06:00","01-Mie","T3",1,1775001600000],["GRUPO 3","XXX5","Tecnico B","22:00 - 06:00","01-Mie","T3",1,1775001600000],["GRUPO 3","XXX6","Tecnico B","22:00 - 06:00","01-Mie","T3",1,1775001600000],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","06:00 - 14:00","01-Mie","T1",1,1775001600000],["GRUPO 4","PEPITO PEREZ","Master","06:00 - 14:00","01-Mie","T1",1,1775001600000],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","06:00 - 14:00","01-Mie","T1",1,1775001600000],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","06:00 - 14:00","01-Mie","T1",1,1775001600000],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","06:00 - 14:00","01-Mie","T1",1,1775001600000],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","06:00 - 14:00","01-Mie","T1",1,1775001600000],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","06:00 - 14:00","01-Mie","T1",1,1775001600000],["GRUPO 4","JHONY CASTRO","Tecnico A","06:00 - 14:00","01-Mie","T1",1,1775001600000],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","06:00 - 14:00","01-Mie","T1",1,1775001600000],["GRUPO 4","XXX7","Tecnico B","06:00 - 14:00","01-Mie","T1",1,1775001600000],["GRUPO 4","XXX8","Tecnico B","06:00 - 14:00","01-Mie","T1",1,1775001600000],["GRUPO 4","XXX9","Tecnico B","06:00 - 14:00","01-Mie","T1",1,1775001600000],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","","02-Jue","DESC. LEY",2,1775088000000],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","","02-Jue","DESC. LEY",2,1775088000000],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","","02-Jue","DESC. LEY",2,1775088000000],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","","02-Jue","DESC. LEY",2,1775088000000],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","","02-Jue","DESC. LEY",2,1775088000000],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","","02-Jue","DESC. LEY",2,1775088000000],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","","02-Jue","DESC. LEY",2,1775088000000],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","","02-Jue","DESC. LEY",2,1775088000000],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","","02-Jue","DESC. LEY",2,1775088000000],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","","02-Jue","DESC. LEY",2,1775088000000],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","","02-Jue","DESC. LEY",2,1775088000000],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","","02-Jue","DESC. LEY",2,1775088000000],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","14:00 - 22:00","02-Jue","T2",2,1775088000000],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","14:00 - 22:00","02-Jue","T2",2,1775088000000],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","14:00 - 22:00","02-Jue","T2",2,1775088000000],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","14:00 - 22:00","02-Jue","T2",2,1775088000000],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","14:00 - 22:00","02-Jue","T2",2,1775088000000],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","14:00 - 22:00","02-Jue","T2",2,1775088000000],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","14:00 - 22:00","02-Jue","T2",2,1775088000000],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","14:00 - 22:00","02-Jue","T2",2,1775088000000],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","14:00 - 22:00","02-Jue","T2",2,1775088000000],["GRUPO 2","XXX1","Tecnico B","14:00 - 22:00","02-Jue","T2",2,1775088000000],["GRUPO 2","XXX2","Tecnico B","14:00 - 22:00","02-Jue","T2",2,1775088000000],["GRUPO 2","XXX3","Tecnico B","14:00 - 22:00","02-Jue","T2",2,1775088000000],["GRUPO 3","FONSECA RAY RICARDO","Master","22:00 - 06:00","02-Jue","T3",2,1775088000000],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","22:00 - 06:00","02-Jue","T3",2,1775088000000],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","22:00 - 06:00","02-Jue","T3",2,1775088000000],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","22:00 - 06:00","02-Jue","T3",2,1775088000000],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","22:00 - 06:00","02-Jue","T3",2,1775088000000],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","22:00 - 06:00","02-Jue","T3",2,1775088000000],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","22:00 - 06:00","02-Jue","T3",2,1775088000000],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","22:00 - 06:00","02-Jue","T3",2,1775088000000],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","22:00 - 06:00","02-Jue","T3",2,1775088000000],["GRUPO 3","XXX4","Tecnico B","22:00 - 06:00","02-Jue","T3",2,1775088000000],["GRUPO 3","XXX5","Tecnico B","22:00 - 06:00","02-Jue","T3",2,1775088000000],["GRUPO 3","XXX6","Tecnico B","22:00 - 06:00","02-Jue","T3",2,1775088000000],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","06:00 - 14:00","02-Jue","T1",2,1775088000000],["GRUPO 4","PEPITO PEREZ","Master","06:00 - 14:00","02-Jue","T1",2,1775088000000],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","06:00 - 14:00","02-Jue","T1",2,1775088000000],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","06:00 - 14:00","02-Jue","T1",2,1775088000000],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","06:00 - 14:00","02-Jue","T1",2,1775088000000],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","06:00 - 14:00","02-Jue","T1",2,1775088000000],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","06:00 - 14:00","02-Jue","T1",2,1775088000000],["GRUPO 4","JHONY CASTRO","Tecnico A","06:00 - 14:00","02-Jue","T1",2,1775088000000],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","06:00 - 14:00","02-Jue","T1",2,1775088000000],["GRUPO 4","XXX7","Tecnico B","06:00 - 14:00","02-Jue","T1",2,1775088000000],["GRUPO 4","XXX8","Tecnico B","06:00 - 14:00","02-Jue","T1",2,1775088000000],["GRUPO 4","XXX9","Tecnico B","06:00 - 14:00","02-Jue","T1",2,1775088000000],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","06:00 - 14:00","03-Vie","T1",3,1775174400000],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","06:00 - 14:00","03-Vie","T1",3,1775174400000],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","06:00 - 14:00","03-Vie","T1",3,1775174400000],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","06:00 - 14:00","03-Vie","T1",3,1775174400000],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","06:00 - 14:00","03-Vie","T1",3,1775174400000],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","06:00 - 14:00","03-Vie","T1",3,1775174400000],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","06:00 - 14:00","03-Vie","T1",3,1775174400000],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","06:00 - 14:00","03-Vie","T1",3,1775174400000],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","06:00 - 14:00","03-Vie","T1",3,1775174400000],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","06:00 - 14:00","03-Vie","T1",3,1775174400000],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","06:00 - 14:00","03-Vie","T1",3,1775174400000],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","06:00 - 14:00","03-Vie","T1",3,1775174400000],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","","03-Vie","DESC. LEY",3,1775174400000],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","","03-Vie","DESC. LEY",3,1775174400000],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","","03-Vie","DESC. LEY",3,1775174400000],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","","03-Vie","DESC. LEY",3,1775174400000],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","","03-Vie","DESC. LEY",3,1775174400000],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","","03-Vie","DESC. LEY",3,1775174400000],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","","03-Vie","DESC. LEY",3,1775174400000],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","","03-Vie","DESC. LEY",3,1775174400000],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","","03-Vie","DESC. LEY",3,1775174400000],["GRUPO 2","XXX1","Tecnico B","","03-Vie","DESC. LEY",3,1775174400000],["GRUPO 2","XXX2","Tecnico B","","03-Vie","DESC. LEY",3,1775174400000],["GRUPO 2","XXX3","Tecnico B","","03-Vie","DESC. LEY",3,1775174400000],["GRUPO 3","FONSECA RAY RICARDO","Master","22:00 - 06:00","03-Vie","T3",3,1775174400000],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","22:00 - 06:00","03-Vie","T3",3,1775174400000],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","22:00 - 06:00","03-Vie","T3",3,1775174400000],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","22:00 - 06:00","03-Vie","T3",3,1775174400000],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","22:00 - 06:00","03-Vie","T3",3,1775174400000],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","22:00 - 06:00","03-Vie","T3",3,1775174400000],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","22:00 - 06:00","03-Vie","T3",3,1775174400000],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","22:00 - 06:00","03-Vie","T3",3,1775174400000],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","22:00 - 06:00","03-Vie","T3",3,1775174400000],["GRUPO 3","XXX4","Tecnico B","22:00 - 06:00","03-Vie","T3",3,1775174400000],["GRUPO 3","XXX5","Tecnico B","22:00 - 06:00","03-Vie","T3",3,1775174400000],["GRUPO 3","XXX6","Tecnico B","22:00 - 06:00","03-Vie","T3",3,1775174400000],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","14:00 - 22:00","03-Vie","T2",3,1775174400000],["GRUPO 4","PEPITO PEREZ","Master","14:00 - 22:00","03-Vie","T2",3,1775174400000],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","14:00 - 22:00","03-Vie","T2",3,1775174400000],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","14:00 - 22:00","03-Vie","T2",3,1775174400000],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","14:00 - 22:00","03-Vie","T2",3,1775174400000],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","14:00 - 22:00","03-Vie","T2",3,1775174400000],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","14:00 - 22:00","03-Vie","T2",3,1775174400000],["GRUPO 4","JHONY CASTRO","Tecnico A","14:00 - 22:00","03-Vie","T2",3,1775174400000],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","14:00 - 22:00","03-Vie","T2",3,1775174400000],["GRUPO 4","XXX7","Tecnico B","14:00 - 22:00","03-Vie","T2",3,1775174400000],["GRUPO 4","XXX8","Tecnico B","14:00 - 22:00","03-Vie","T2",3,1775174400000],["GRUPO 4","XXX9","Tecnico B","14:00 - 22:00","03-Vie","T2",3,1775174400000],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","06:00 - 14:00","04-Sab","T1",4,1775260800000],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","06:00 - 14:00","04-Sab","T1",4,1775260800000],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","06:00 - 14:00","04-Sab","T1",4,1775260800000],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","06:00 - 14:00","04-Sab","T1",4,1775260800000],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","06:00 - 14:00","04-Sab","T1",4,1775260800000],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","06:00 - 14:00","04-Sab","T1",4,1775260800000],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","06:00 - 14:00","04-Sab","T1",4,1775260800000],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","06:00 - 14:00","04-Sab","T1",4,1775260800000],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","06:00 - 14:00","04-Sab","T1",4,1775260800000],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","06:00 - 14:00","04-Sab","T1",4,1775260800000],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","06:00 - 14:00","04-Sab","T1",4,1775260800000],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","06:00 - 14:00","04-Sab","T1",4,1775260800000],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","14:00 - 22:00","04-Sab","T2",4,1775260800000],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","14:00 - 22:00","04-Sab","T2",4,1775260800000],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","14:00 - 22:00","04-Sab","T2",4,1775260800000],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","14:00 - 22:00","04-Sab","T2",4,1775260800000],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","14:00 - 22:00","04-Sab","T2",4,1775260800000],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","14:00 - 22:00","04-Sab","T2",4,1775260800000],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","14:00 - 22:00","04-Sab","T2",4,1775260800000],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","14:00 - 22:00","04-Sab","T2",4,1775260800000],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","14:00 - 22:00","04-Sab","T2",4,1775260800000],["GRUPO 2","XXX1","Tecnico B","14:00 - 22:00","04-Sab","T2",4,1775260800000],["GRUPO 2","XXX2","Tecnico B","14:00 - 22:00","04-Sab","T2",4,1775260800000],["GRUPO 2","XXX3","Tecnico B","14:00 - 22:00","04-Sab","T2",4,1775260800000],["GRUPO 3","FONSECA RAY RICARDO","Master","","04-Sab","DESC. LEY",4,1775260800000],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","","04-Sab","DESC. LEY",4,1775260800000],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","","04-Sab","DESC. LEY",4,1775260800000],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","","04-Sab","DESC. LEY",4,1775260800000],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","","04-Sab","DESC. LEY",4,1775260800000],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","","04-Sab","DESC. LEY",4,1775260800000],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","","04-Sab","DESC. LEY",4,1775260800000],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","","04-Sab","DESC. LEY",4,1775260800000],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","","04-Sab","DESC. LEY",4,1775260800000],["GRUPO 3","XXX4","Tecnico B","","04-Sab","DESC. LEY",4,1775260800000],["GRUPO 3","XXX5","Tecnico B","","04-Sab","DESC. LEY",4,1775260800000],["GRUPO 3","XXX6","Tecnico B","","04-Sab","DESC. LEY",4,1775260800000],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","22:00 - 06:00","04-Sab","T3",4,1775260800000],["GRUPO 4","PEPITO PEREZ","Master","22:00 - 06:00","04-Sab","T3",4,1775260800000],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","22:00 - 06:00","04-Sab","T3",4,1775260800000],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","22:00 - 06:00","04-Sab","T3",4,1775260800000],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","22:00 - 06:00","04-Sab","T3",4,1775260800000],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","22:00 - 06:00","04-Sab","T3",4,1775260800000],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","22:00 - 06:00","04-Sab","T3",4,1775260800000],["GRUPO 4","JHONY CASTRO","Tecnico A","22:00 - 06:00","04-Sab","T3",4,1775260800000],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","22:00 - 06:00","04-Sab","T3",4,1775260800000],["GRUPO 4","XXX7","Tecnico B","22:00 - 06:00","04-Sab","T3",4,1775260800000],["GRUPO 4","XXX8","Tecnico B","22:00 - 06:00","04-Sab","T3",4,1775260800000],["GRUPO 4","XXX9","Tecnico B","22:00 - 06:00","04-Sab","T3",4,1775260800000],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","06:00 - 14:00","05-Dom","T1",5,1775347200000],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","06:00 - 14:00","05-Dom","T1",5,1775347200000],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","06:00 - 14:00","05-Dom","T1",5,1775347200000],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","06:00 - 14:00","05-Dom","T1",5,1775347200000],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","06:00 - 14:00","05-Dom","T1",5,1775347200000],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","06:00 - 14:00","05-Dom","T1",5,1775347200000],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","06:00 - 14:00","05-Dom","T1",5,1775347200000],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","06:00 - 14:00","05-Dom","T1",5,1775347200000],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","06:00 - 14:00","05-Dom","T1",5,1775347200000],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","06:00 - 14:00","05-Dom","T1",5,1775347200000],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","06:00 - 14:00","05-Dom","T1",5,1775347200000],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","06:00 - 14:00","05-Dom","T1",5,1775347200000],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","14:00 - 22:00","05-Dom","T2",5,1775347200000],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","14:00 - 22:00","05-Dom","T2",5,1775347200000],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","14:00 - 22:00","05-Dom","T2",5,1775347200000],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","14:00 - 22:00","05-Dom","T2",5,1775347200000],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","14:00 - 22:00","05-Dom","T2",5,1775347200000],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","14:00 - 22:00","05-Dom","T2",5,1775347200000],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","14:00 - 22:00","05-Dom","T2",5,1775347200000],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","14:00 - 22:00","05-Dom","T2",5,1775347200000],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","14:00 - 22:00","05-Dom","T2",5,1775347200000],["GRUPO 2","XXX1","Tecnico B","14:00 - 22:00","05-Dom","T2",5,1775347200000],["GRUPO 2","XXX2","Tecnico B","14:00 - 22:00","05-Dom","T2",5,1775347200000],["GRUPO 2","XXX3","Tecnico B","14:00 - 22:00","05-Dom","T2",5,1775347200000],["GRUPO 3","FONSECA RAY RICARDO","Master","22:00 - 06:00","05-Dom","T3",5,1775347200000],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","22:00 - 06:00","05-Dom","T3",5,1775347200000],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","22:00 - 06:00","05-Dom","T3",5,1775347200000],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","22:00 - 06:00","05-Dom","T3",5,1775347200000],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","22:00 - 06:00","05-Dom","T3",5,1775347200000],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","22:00 - 06:00","05-Dom","T3",5,1775347200000],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","22:00 - 06:00","05-Dom","T3",5,1775347200000],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","22:00 - 06:00","05-Dom","T3",5,1775347200000],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","22:00 - 06:00","05-Dom","T3",5,1775347200000],["GRUPO 3","XXX4","Tecnico B","22:00 - 06:00","05-Dom","T3",5,1775347200000],["GRUPO 3","XXX5","Tecnico B","22:00 - 06:00","05-Dom","T3",5,1775347200000],["GRUPO 3","XXX6","Tecnico B","22:00 - 06:00","05-Dom","T3",5,1775347200000],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","","05-Dom","DESC. LEY",5,1775347200000],["GRUPO 4","PEPITO PEREZ","Master","","05-Dom","DESC. LEY",5,1775347200000],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","","05-Dom","DESC. LEY",5,1775347200000],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","","05-Dom","DESC. LEY",5,1775347200000],["GRUPO 4","TORO CISNEROS GARY JOSE","Tecnico A","","05-Dom","DESC. LEY",5,1775347200000],["GRUPO 4","USECHE CALDERON JADID ESTIVEN","Tecnico A","","05-Dom","DESC. LEY",5,1775347200000],["GRUPO 4","VASQUEZ NIETO CAMILO ANDRES","Tecnico A","","05-Dom","DESC. LEY",5,1775347200000],["GRUPO 4","JHONY CASTRO","Tecnico A","","05-Dom","DESC. LEY",5,1775347200000],["GRUPO 4","BERNAL JUAN DAVID","Tecnico A","","05-Dom","DESC. LEY",5,1775347200000],["GRUPO 4","XXX7","Tecnico B","","05-Dom","DESC. LEY",5,1775347200000],["GRUPO 4","XXX8","Tecnico B","","05-Dom","DESC. LEY",5,1775347200000],["GRUPO 4","XXX9","Tecnico B","","05-Dom","DESC. LEY",5,1775347200000],["GRUPO 1","BARON HERNANDEZ HAROLD ANTONIO","Master","06:00 - 14:00","06-Lun","T1",6,1775433600000],["GRUPO 1","CASTELLANOS CARVAJAL DEYVITH FABIAN","Master","06:00 - 14:00","06-Lun","T1",6,1775433600000],["GRUPO 1","AROCA TORRES JULIAN EDUARDO","Tecnico A","06:00 - 14:00","06-Lun","T1",6,1775433600000],["GRUPO 1","BERMUDEZ PARRA JENNIFER XIOMARA","Tecnico A","06:00 - 14:00","06-Lun","T1",6,1775433600000],["GRUPO 1","BERNAL BAQUERO JAMES RICARDO","Tecnico A","06:00 - 14:00","06-Lun","T1",6,1775433600000],["GRUPO 1","BURGOS ORTIZ JOSE HORACIO","Tecnico A","06:00 - 14:00","06-Lun","T1",6,1775433600000],["GRUPO 1","CANTOR PORRAS JUAN FERNEY","Tecnico A","06:00 - 14:00","06-Lun","T1",6,1775433600000],["GRUPO 1","CAPERA CAPERA JOSE GABRIEL","Tecnico A","06:00 - 14:00","06-Lun","T1",6,1775433600000],["GRUPO 1","CARDENAS LOTERO RICARDO ANDR\u00c9S","Tecnico A","06:00 - 14:00","06-Lun","T1",6,1775433600000],["GRUPO 1","RENDON OSPINA NELSON LEANDRO","Tecnico B","06:00 - 14:00","06-Lun","T1",6,1775433600000],["GRUPO 1","SARMIENTO URBINA MOISES DANIEL","Tecnico B","06:00 - 14:00","06-Lun","T1",6,1775433600000],["GRUPO 1","VELASCO VELASCO SEBASTI\u00c1N DAVID","Tecnico B","06:00 - 14:00","06-Lun","T1",6,1775433600000],["GRUPO 2","DELGADO DELGADO JOHAN DARIO","Master","14:00 - 22:00","06-Lun","T2",6,1775433600000],["GRUPO 2","FLOREZ SAUCESO KENIS ALBERTO","Master","14:00 - 22:00","06-Lun","T2",6,1775433600000],["GRUPO 2","CARDONA GARCIA OSCAR JAVIER","Tecnico A","14:00 - 22:00","06-Lun","T2",6,1775433600000],["GRUPO 2","CARVAJAL GARC\u00cdA HOVER MARCK","Tecnico A","14:00 - 22:00","06-Lun","T2",6,1775433600000],["GRUPO 2","CEPEDA PIRAQUIVE JUAN DAVID","Tecnico A","14:00 - 22:00","06-Lun","T2",6,1775433600000],["GRUPO 2","FAJARDO SAENZ OSCAR FERNANDO","Tecnico A","14:00 - 22:00","06-Lun","T2",6,1775433600000],["GRUPO 2","FLOREZ ESPITIA RONY ALBERTO","Tecnico A","14:00 - 22:00","06-Lun","T2",6,1775433600000],["GRUPO 2","GARCIA CUERVO EDWIN JAVIER","Tecnico A","14:00 - 22:00","06-Lun","T2",6,1775433600000],["GRUPO 2","GONZALEZ OCHOA JUAN CARLOS","Tecnico A","14:00 - 22:00","06-Lun","T2",6,1775433600000],["GRUPO 2","XXX1","Tecnico B","14:00 - 22:00","06-Lun","T2",6,1775433600000],["GRUPO 2","XXX2","Tecnico B","14:00 - 22:00","06-Lun","T2",6,1775433600000],["GRUPO 2","XXX3","Tecnico B","14:00 - 22:00","06-Lun","T2",6,1775433600000],["GRUPO 3","FONSECA RAY RICARDO","Master","22:00 - 06:00","06-Lun","T3",6,1775433600000],["GRUPO 3","GOMEZ BETANCUR JAIDER ANDRES","Master","22:00 - 06:00","06-Lun","T3",6,1775433600000],["GRUPO 3","GRANADA PATI\u00d1O CARLOS MARINO","Tecnico A","22:00 - 06:00","06-Lun","T3",6,1775433600000],["GRUPO 3","GRASS PLATA MIGUEL SNEIDER","Tecnico A","22:00 - 06:00","06-Lun","T3",6,1775433600000],["GRUPO 3","MANZANO CALVO JUAN SEBASTIAN","Tecnico A","22:00 - 06:00","06-Lun","T3",6,1775433600000],["GRUPO 3","MENDOZA GOITA MARIANSEL ZENAYDA","Tecnico A","22:00 - 06:00","06-Lun","T3",6,1775433600000],["GRUPO 3","MURILLO ARAQUE JAIVER GEOVANY","Tecnico A","22:00 - 06:00","06-Lun","T3",6,1775433600000],["GRUPO 3","NI\u00d1O ARENAS HECTOR GONZALO","Tecnico A","22:00 - 06:00","06-Lun","T3",6,1775433600000],["GRUPO 3","RAMIREZ CHAVERRA JHON EDISON","Tecnico A","22:00 - 06:00","06-Lun","T3",6,1775433600000],["GRUPO 3","XXX4","Tecnico B","22:00 - 06:00","06-Lun","T3",6,1775433600000],["GRUPO 3","XXX5","Tecnico B","22:00 - 06:00","06-Lun","T3",6,1775433600000],["GRUPO 3","XXX6","Tecnico B","22:00 - 06:00","06-Lun","T3",6,1775433600000],["GRUPO 4","RODRIGUEZ MOSQUERA LUIS FERNANDO","Master","06:00 - 14:00","06-Lun","T1",6,1775433600000],["GRUPO 4","PEPITO PEREZ","Master","06:00 - 14:00","06-Lun","T1",6,1775433600000],["GRUPO 4","RAMIREZ VARGAS MARCELA PAOLA","Tecnico A","06:00 - 14:00","06-Lun","T1",6,1775433600000],["GRUPO 4","SANMARTIN BERR\u00cdO EDUARDO JOS\u00c9","Tecnico A","06:00 - 14:00","06-Lun","T1",6,1775433600000],["GRUPO 4","TO</t>
   </si>
   <si>
     <t>Mes Completo</t>
@@ -414,7 +423,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -445,16 +454,16 @@
         <v>2026</v>
       </c>
       <c r="C2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -465,16 +474,16 @@
         <v>2026</v>
       </c>
       <c r="C3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F3" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -485,16 +494,16 @@
         <v>2026</v>
       </c>
       <c r="C4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E4" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F4" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -505,16 +514,16 @@
         <v>2026</v>
       </c>
       <c r="C5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F5" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -525,16 +534,30 @@
         <v>2026</v>
       </c>
       <c r="C6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" t="s">
+        <v>17</v>
+      </c>
+      <c r="E6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" t="s">
         <v>11</v>
       </c>
-      <c r="D6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E6" t="s">
-        <v>21</v>
-      </c>
-      <c r="F6" t="s">
-        <v>22</v>
+      <c r="B7">
+        <v>2026</v>
+      </c>
+      <c r="D7" t="s">
+        <v>18</v>
+      </c>
+      <c r="E7" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>